<commit_message>
New points - POTEC lab 5
</commit_message>
<xml_diff>
--- a/IoT-points-schedule.xlsx
+++ b/IoT-points-schedule.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\dodo\Desktop\IoT-studies\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7AC26BBE-DE65-4B95-993E-D6F9E9FD051F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A5FE9F87-847C-4430-8D1F-8FEBC4C2A219}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="25440" windowHeight="15390" xr2:uid="{F85F5544-1FE8-4920-A5D4-192A98B113BD}"/>
   </bookViews>
@@ -1018,7 +1018,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="71">
+  <cellXfs count="70">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1121,6 +1121,25 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="19" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1199,16 +1218,6 @@
     <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="19" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="7" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1218,22 +1227,10 @@
     <xf numFmtId="0" fontId="2" fillId="7" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="6" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1620,60 +1617,60 @@
   <sheetData>
     <row r="1" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="2" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B2" s="33" t="s">
+      <c r="B2" s="40" t="s">
         <v>76</v>
       </c>
-      <c r="C2" s="34"/>
-      <c r="D2" s="34"/>
-      <c r="E2" s="34"/>
-      <c r="F2" s="34"/>
-      <c r="G2" s="34"/>
-      <c r="H2" s="34"/>
-      <c r="I2" s="34"/>
-      <c r="J2" s="34"/>
-      <c r="K2" s="34"/>
-      <c r="L2" s="34"/>
-      <c r="M2" s="34"/>
-      <c r="N2" s="34"/>
-      <c r="O2" s="34"/>
-      <c r="P2" s="35"/>
+      <c r="C2" s="41"/>
+      <c r="D2" s="41"/>
+      <c r="E2" s="41"/>
+      <c r="F2" s="41"/>
+      <c r="G2" s="41"/>
+      <c r="H2" s="41"/>
+      <c r="I2" s="41"/>
+      <c r="J2" s="41"/>
+      <c r="K2" s="41"/>
+      <c r="L2" s="41"/>
+      <c r="M2" s="41"/>
+      <c r="N2" s="41"/>
+      <c r="O2" s="41"/>
+      <c r="P2" s="42"/>
     </row>
     <row r="3" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B3" s="36"/>
-      <c r="C3" s="37"/>
-      <c r="D3" s="37"/>
-      <c r="E3" s="37"/>
-      <c r="F3" s="37"/>
-      <c r="G3" s="37"/>
-      <c r="H3" s="37"/>
-      <c r="I3" s="37"/>
-      <c r="J3" s="37"/>
-      <c r="K3" s="37"/>
-      <c r="L3" s="37"/>
-      <c r="M3" s="37"/>
-      <c r="N3" s="37"/>
-      <c r="O3" s="37"/>
-      <c r="P3" s="38"/>
+      <c r="B3" s="43"/>
+      <c r="C3" s="44"/>
+      <c r="D3" s="44"/>
+      <c r="E3" s="44"/>
+      <c r="F3" s="44"/>
+      <c r="G3" s="44"/>
+      <c r="H3" s="44"/>
+      <c r="I3" s="44"/>
+      <c r="J3" s="44"/>
+      <c r="K3" s="44"/>
+      <c r="L3" s="44"/>
+      <c r="M3" s="44"/>
+      <c r="N3" s="44"/>
+      <c r="O3" s="44"/>
+      <c r="P3" s="45"/>
       <c r="R3" s="12"/>
     </row>
     <row r="5" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B5" s="39" t="s">
+      <c r="B5" s="46" t="s">
         <v>83</v>
       </c>
-      <c r="C5" s="40"/>
-      <c r="D5" s="40"/>
-      <c r="E5" s="40"/>
-      <c r="F5" s="41"/>
-      <c r="H5" s="39" t="s">
+      <c r="C5" s="47"/>
+      <c r="D5" s="47"/>
+      <c r="E5" s="47"/>
+      <c r="F5" s="48"/>
+      <c r="H5" s="46" t="s">
         <v>82</v>
       </c>
-      <c r="I5" s="41"/>
-      <c r="K5" s="39" t="s">
+      <c r="I5" s="48"/>
+      <c r="K5" s="46" t="s">
         <v>8</v>
       </c>
-      <c r="L5" s="40"/>
-      <c r="M5" s="40"/>
-      <c r="N5" s="41"/>
+      <c r="L5" s="47"/>
+      <c r="M5" s="47"/>
+      <c r="N5" s="48"/>
       <c r="P5" s="4" t="s">
         <v>74</v>
       </c>
@@ -1733,37 +1730,37 @@
       <c r="P7" s="2"/>
     </row>
     <row r="9" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B9" s="42" t="s">
+      <c r="B9" s="49" t="s">
         <v>22</v>
       </c>
-      <c r="C9" s="42"/>
+      <c r="C9" s="49"/>
       <c r="E9" s="9" t="s">
         <v>67</v>
       </c>
-      <c r="G9" s="42" t="s">
+      <c r="G9" s="49" t="s">
         <v>87</v>
       </c>
-      <c r="H9" s="42"/>
+      <c r="H9" s="49"/>
     </row>
     <row r="10" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B10" s="43">
+      <c r="B10" s="50">
         <f>SUM(B7:F7,H7:I7,K7:N7,P7)</f>
         <v>8.6999999999999993</v>
       </c>
-      <c r="C10" s="43"/>
-      <c r="E10" s="47"/>
-      <c r="G10" s="43">
+      <c r="C10" s="50"/>
+      <c r="E10" s="54"/>
+      <c r="G10" s="50">
         <f>66-SUM(B7:F7,H7:I7,K7:N7,P7)</f>
         <v>57.3</v>
       </c>
-      <c r="H10" s="43"/>
+      <c r="H10" s="50"/>
     </row>
     <row r="11" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B11" s="43"/>
-      <c r="C11" s="43"/>
-      <c r="E11" s="48"/>
-      <c r="G11" s="43"/>
-      <c r="H11" s="43"/>
+      <c r="B11" s="50"/>
+      <c r="C11" s="50"/>
+      <c r="E11" s="55"/>
+      <c r="G11" s="50"/>
+      <c r="H11" s="50"/>
     </row>
     <row r="12" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A12" s="6"/>
@@ -1788,46 +1785,46 @@
     </row>
     <row r="13" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="14" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B14" s="33" t="s">
+      <c r="B14" s="40" t="s">
         <v>77</v>
       </c>
-      <c r="C14" s="34"/>
-      <c r="D14" s="34"/>
-      <c r="E14" s="34"/>
-      <c r="F14" s="34"/>
-      <c r="G14" s="34"/>
-      <c r="H14" s="35"/>
+      <c r="C14" s="41"/>
+      <c r="D14" s="41"/>
+      <c r="E14" s="41"/>
+      <c r="F14" s="41"/>
+      <c r="G14" s="41"/>
+      <c r="H14" s="42"/>
     </row>
     <row r="15" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B15" s="36"/>
-      <c r="C15" s="37"/>
-      <c r="D15" s="37"/>
-      <c r="E15" s="37"/>
-      <c r="F15" s="37"/>
-      <c r="G15" s="37"/>
-      <c r="H15" s="38"/>
+      <c r="B15" s="43"/>
+      <c r="C15" s="44"/>
+      <c r="D15" s="44"/>
+      <c r="E15" s="44"/>
+      <c r="F15" s="44"/>
+      <c r="G15" s="44"/>
+      <c r="H15" s="45"/>
     </row>
     <row r="17" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B17" s="46" t="s">
+      <c r="B17" s="53" t="s">
         <v>91</v>
       </c>
-      <c r="C17" s="46"/>
-      <c r="D17" s="46"/>
-      <c r="E17" s="46"/>
-      <c r="F17" s="46"/>
-      <c r="H17" s="39" t="s">
+      <c r="C17" s="53"/>
+      <c r="D17" s="53"/>
+      <c r="E17" s="53"/>
+      <c r="F17" s="53"/>
+      <c r="H17" s="46" t="s">
         <v>97</v>
       </c>
-      <c r="I17" s="40"/>
-      <c r="J17" s="41"/>
-      <c r="L17" s="42" t="s">
+      <c r="I17" s="47"/>
+      <c r="J17" s="48"/>
+      <c r="L17" s="49" t="s">
         <v>22</v>
       </c>
-      <c r="M17" s="42"/>
-      <c r="O17" s="42" t="s">
+      <c r="M17" s="49"/>
+      <c r="O17" s="49" t="s">
         <v>87</v>
       </c>
-      <c r="P17" s="42"/>
+      <c r="P17" s="49"/>
       <c r="R17" s="9" t="s">
         <v>67</v>
       </c>
@@ -1857,17 +1854,17 @@
       <c r="J18" s="3" t="s">
         <v>95</v>
       </c>
-      <c r="L18" s="43">
+      <c r="L18" s="50">
         <f>SUM(B19:F19,H19:J19)</f>
         <v>29.5</v>
       </c>
-      <c r="M18" s="43"/>
-      <c r="O18" s="43">
+      <c r="M18" s="50"/>
+      <c r="O18" s="50">
         <f>50-SUM(B19:F19,H19:J19)</f>
         <v>20.5</v>
       </c>
-      <c r="P18" s="43"/>
-      <c r="R18" s="32"/>
+      <c r="P18" s="50"/>
+      <c r="R18" s="39"/>
     </row>
     <row r="19" spans="1:19" x14ac:dyDescent="0.25">
       <c r="B19" s="2"/>
@@ -1882,11 +1879,11 @@
         <v>26.5</v>
       </c>
       <c r="J19" s="2"/>
-      <c r="L19" s="43"/>
-      <c r="M19" s="43"/>
-      <c r="O19" s="43"/>
-      <c r="P19" s="43"/>
-      <c r="R19" s="32"/>
+      <c r="L19" s="50"/>
+      <c r="M19" s="50"/>
+      <c r="O19" s="50"/>
+      <c r="P19" s="50"/>
+      <c r="R19" s="39"/>
     </row>
     <row r="21" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A21" s="6"/>
@@ -1911,56 +1908,56 @@
     </row>
     <row r="22" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="23" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B23" s="33" t="s">
+      <c r="B23" s="40" t="s">
         <v>79</v>
       </c>
-      <c r="C23" s="34"/>
-      <c r="D23" s="34"/>
-      <c r="E23" s="34"/>
-      <c r="F23" s="34"/>
-      <c r="G23" s="34"/>
-      <c r="H23" s="34"/>
-      <c r="I23" s="34"/>
-      <c r="J23" s="34"/>
-      <c r="K23" s="34"/>
-      <c r="L23" s="35"/>
-      <c r="N23" s="43" t="s">
+      <c r="C23" s="41"/>
+      <c r="D23" s="41"/>
+      <c r="E23" s="41"/>
+      <c r="F23" s="41"/>
+      <c r="G23" s="41"/>
+      <c r="H23" s="41"/>
+      <c r="I23" s="41"/>
+      <c r="J23" s="41"/>
+      <c r="K23" s="41"/>
+      <c r="L23" s="42"/>
+      <c r="N23" s="50" t="s">
         <v>132</v>
       </c>
-      <c r="O23" s="43"/>
+      <c r="O23" s="50"/>
     </row>
     <row r="24" spans="1:19" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B24" s="36"/>
-      <c r="C24" s="37"/>
-      <c r="D24" s="37"/>
-      <c r="E24" s="37"/>
-      <c r="F24" s="37"/>
-      <c r="G24" s="37"/>
-      <c r="H24" s="37"/>
-      <c r="I24" s="37"/>
-      <c r="J24" s="37"/>
-      <c r="K24" s="37"/>
-      <c r="L24" s="38"/>
-      <c r="N24" s="43"/>
-      <c r="O24" s="43"/>
+      <c r="B24" s="43"/>
+      <c r="C24" s="44"/>
+      <c r="D24" s="44"/>
+      <c r="E24" s="44"/>
+      <c r="F24" s="44"/>
+      <c r="G24" s="44"/>
+      <c r="H24" s="44"/>
+      <c r="I24" s="44"/>
+      <c r="J24" s="44"/>
+      <c r="K24" s="44"/>
+      <c r="L24" s="45"/>
+      <c r="N24" s="50"/>
+      <c r="O24" s="50"/>
     </row>
     <row r="26" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B26" s="46" t="s">
+      <c r="B26" s="53" t="s">
         <v>129</v>
       </c>
-      <c r="C26" s="46"/>
-      <c r="D26" s="46"/>
-      <c r="F26" s="46" t="s">
+      <c r="C26" s="53"/>
+      <c r="D26" s="53"/>
+      <c r="F26" s="53" t="s">
         <v>12</v>
       </c>
-      <c r="G26" s="46"/>
-      <c r="H26" s="46"/>
-      <c r="I26" s="46"/>
+      <c r="G26" s="53"/>
+      <c r="H26" s="53"/>
+      <c r="I26" s="53"/>
       <c r="J26" s="7"/>
-      <c r="K26" s="39" t="s">
+      <c r="K26" s="46" t="s">
         <v>128</v>
       </c>
-      <c r="L26" s="41"/>
+      <c r="L26" s="48"/>
       <c r="N26" s="10" t="s">
         <v>22</v>
       </c>
@@ -1996,11 +1993,11 @@
       <c r="L27" s="2" t="s">
         <v>127</v>
       </c>
-      <c r="N27" s="49">
+      <c r="N27" s="56">
         <f>SUM(B28:D28,F28:I28,K28:L28)</f>
         <v>1</v>
       </c>
-      <c r="O27" s="47"/>
+      <c r="O27" s="54"/>
     </row>
     <row r="28" spans="1:19" x14ac:dyDescent="0.25">
       <c r="B28" s="2"/>
@@ -2014,8 +2011,8 @@
       <c r="I28" s="2"/>
       <c r="K28" s="2"/>
       <c r="L28" s="2"/>
-      <c r="N28" s="50"/>
-      <c r="O28" s="48"/>
+      <c r="N28" s="57"/>
+      <c r="O28" s="55"/>
     </row>
     <row r="30" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A30" s="6"/>
@@ -2040,39 +2037,39 @@
     </row>
     <row r="31" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="32" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B32" s="33" t="s">
+      <c r="B32" s="40" t="s">
         <v>78</v>
       </c>
-      <c r="C32" s="34"/>
-      <c r="D32" s="34"/>
-      <c r="E32" s="34"/>
-      <c r="F32" s="34"/>
-      <c r="G32" s="34"/>
-      <c r="H32" s="34"/>
-      <c r="I32" s="35"/>
+      <c r="C32" s="41"/>
+      <c r="D32" s="41"/>
+      <c r="E32" s="41"/>
+      <c r="F32" s="41"/>
+      <c r="G32" s="41"/>
+      <c r="H32" s="41"/>
+      <c r="I32" s="42"/>
     </row>
     <row r="33" spans="2:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B33" s="36"/>
-      <c r="C33" s="37"/>
-      <c r="D33" s="37"/>
-      <c r="E33" s="37"/>
-      <c r="F33" s="37"/>
-      <c r="G33" s="37"/>
-      <c r="H33" s="37"/>
-      <c r="I33" s="38"/>
+      <c r="B33" s="43"/>
+      <c r="C33" s="44"/>
+      <c r="D33" s="44"/>
+      <c r="E33" s="44"/>
+      <c r="F33" s="44"/>
+      <c r="G33" s="44"/>
+      <c r="H33" s="44"/>
+      <c r="I33" s="45"/>
     </row>
     <row r="35" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B35" s="46" t="s">
+      <c r="B35" s="53" t="s">
         <v>98</v>
       </c>
-      <c r="C35" s="46"/>
+      <c r="C35" s="53"/>
       <c r="D35" s="7"/>
-      <c r="E35" s="39" t="s">
+      <c r="E35" s="46" t="s">
         <v>147</v>
       </c>
-      <c r="F35" s="40"/>
-      <c r="G35" s="40"/>
-      <c r="H35" s="41"/>
+      <c r="F35" s="47"/>
+      <c r="G35" s="47"/>
+      <c r="H35" s="48"/>
     </row>
     <row r="36" spans="2:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B36" s="2" t="s">
@@ -2100,25 +2097,25 @@
       <c r="C37" s="2"/>
       <c r="E37" s="2">
         <f>C56</f>
-        <v>7</v>
+        <v>13</v>
       </c>
       <c r="F37" s="2">
         <f>G51</f>
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="G37" s="2"/>
       <c r="H37" s="2"/>
       <c r="O37" s="7"/>
     </row>
     <row r="40" spans="2:15" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B40" s="44" t="s">
+      <c r="B40" s="51" t="s">
         <v>126</v>
       </c>
-      <c r="C40" s="45"/>
-      <c r="F40" s="43" t="s">
+      <c r="C40" s="52"/>
+      <c r="F40" s="50" t="s">
         <v>102</v>
       </c>
-      <c r="G40" s="43"/>
+      <c r="G40" s="50"/>
       <c r="I40" s="9" t="s">
         <v>22</v>
       </c>
@@ -2135,10 +2132,12 @@
       <c r="F41" s="2" t="s">
         <v>117</v>
       </c>
-      <c r="G41" s="2"/>
+      <c r="G41" s="2">
+        <v>9</v>
+      </c>
       <c r="I41" s="2">
         <f>SUM(B37:C37,E37:H37)</f>
-        <v>7</v>
+        <v>22</v>
       </c>
       <c r="J41" s="7"/>
       <c r="L41" s="7"/>
@@ -2166,7 +2165,7 @@
         <v>119</v>
       </c>
       <c r="G43" s="2"/>
-      <c r="I43" s="42" t="s">
+      <c r="I43" s="49" t="s">
         <v>67</v>
       </c>
     </row>
@@ -2175,19 +2174,21 @@
         <v>106</v>
       </c>
       <c r="C44" s="2">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F44" s="2" t="s">
         <v>120</v>
       </c>
       <c r="G44" s="2"/>
-      <c r="I44" s="42"/>
+      <c r="I44" s="49"/>
     </row>
     <row r="45" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B45" s="2" t="s">
         <v>107</v>
       </c>
-      <c r="C45" s="2"/>
+      <c r="C45" s="2">
+        <v>4</v>
+      </c>
       <c r="F45" s="2" t="s">
         <v>121</v>
       </c>
@@ -2228,7 +2229,7 @@
       <c r="G48" s="2"/>
       <c r="I48" s="2">
         <f>50-SUM(B37:C37,E37:H37)</f>
-        <v>43</v>
+        <v>28</v>
       </c>
     </row>
     <row r="49" spans="1:19" x14ac:dyDescent="0.25">
@@ -2257,7 +2258,7 @@
       </c>
       <c r="G51" s="2">
         <f>SUM(G41:G49)</f>
-        <v>0</v>
+        <v>9</v>
       </c>
     </row>
     <row r="52" spans="1:19" x14ac:dyDescent="0.25">
@@ -2284,7 +2285,7 @@
       </c>
       <c r="C56" s="2">
         <f>SUM(C41:C54)</f>
-        <v>7</v>
+        <v>13</v>
       </c>
     </row>
     <row r="58" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -2310,70 +2311,70 @@
     </row>
     <row r="59" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="60" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B60" s="33" t="s">
+      <c r="B60" s="40" t="s">
         <v>80</v>
       </c>
-      <c r="C60" s="34"/>
-      <c r="D60" s="34"/>
-      <c r="E60" s="34"/>
-      <c r="F60" s="34"/>
-      <c r="G60" s="34"/>
-      <c r="H60" s="34"/>
-      <c r="I60" s="34"/>
-      <c r="J60" s="34"/>
-      <c r="K60" s="34"/>
-      <c r="L60" s="34"/>
-      <c r="M60" s="34"/>
-      <c r="N60" s="34"/>
-      <c r="O60" s="34"/>
-      <c r="P60" s="34"/>
-      <c r="Q60" s="34"/>
-      <c r="R60" s="34"/>
-      <c r="S60" s="35"/>
+      <c r="C60" s="41"/>
+      <c r="D60" s="41"/>
+      <c r="E60" s="41"/>
+      <c r="F60" s="41"/>
+      <c r="G60" s="41"/>
+      <c r="H60" s="41"/>
+      <c r="I60" s="41"/>
+      <c r="J60" s="41"/>
+      <c r="K60" s="41"/>
+      <c r="L60" s="41"/>
+      <c r="M60" s="41"/>
+      <c r="N60" s="41"/>
+      <c r="O60" s="41"/>
+      <c r="P60" s="41"/>
+      <c r="Q60" s="41"/>
+      <c r="R60" s="41"/>
+      <c r="S60" s="42"/>
     </row>
     <row r="61" spans="1:19" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B61" s="36"/>
-      <c r="C61" s="37"/>
-      <c r="D61" s="37"/>
-      <c r="E61" s="37"/>
-      <c r="F61" s="37"/>
-      <c r="G61" s="37"/>
-      <c r="H61" s="37"/>
-      <c r="I61" s="37"/>
-      <c r="J61" s="37"/>
-      <c r="K61" s="37"/>
-      <c r="L61" s="37"/>
-      <c r="M61" s="37"/>
-      <c r="N61" s="37"/>
-      <c r="O61" s="37"/>
-      <c r="P61" s="37"/>
-      <c r="Q61" s="37"/>
-      <c r="R61" s="37"/>
-      <c r="S61" s="38"/>
+      <c r="B61" s="43"/>
+      <c r="C61" s="44"/>
+      <c r="D61" s="44"/>
+      <c r="E61" s="44"/>
+      <c r="F61" s="44"/>
+      <c r="G61" s="44"/>
+      <c r="H61" s="44"/>
+      <c r="I61" s="44"/>
+      <c r="J61" s="44"/>
+      <c r="K61" s="44"/>
+      <c r="L61" s="44"/>
+      <c r="M61" s="44"/>
+      <c r="N61" s="44"/>
+      <c r="O61" s="44"/>
+      <c r="P61" s="44"/>
+      <c r="Q61" s="44"/>
+      <c r="R61" s="44"/>
+      <c r="S61" s="45"/>
     </row>
     <row r="63" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B63" s="46" t="s">
+      <c r="B63" s="53" t="s">
         <v>63</v>
       </c>
-      <c r="C63" s="46"/>
-      <c r="D63" s="46"/>
-      <c r="E63" s="46"/>
-      <c r="F63" s="46"/>
-      <c r="G63" s="46"/>
-      <c r="H63" s="46"/>
-      <c r="I63" s="46"/>
-      <c r="J63" s="46"/>
-      <c r="K63" s="46"/>
-      <c r="M63" s="46" t="s">
+      <c r="C63" s="53"/>
+      <c r="D63" s="53"/>
+      <c r="E63" s="53"/>
+      <c r="F63" s="53"/>
+      <c r="G63" s="53"/>
+      <c r="H63" s="53"/>
+      <c r="I63" s="53"/>
+      <c r="J63" s="53"/>
+      <c r="K63" s="53"/>
+      <c r="M63" s="53" t="s">
         <v>90</v>
       </c>
-      <c r="N63" s="46"/>
-      <c r="O63" s="46"/>
-      <c r="P63" s="46"/>
-      <c r="R63" s="46" t="s">
+      <c r="N63" s="53"/>
+      <c r="O63" s="53"/>
+      <c r="P63" s="53"/>
+      <c r="R63" s="53" t="s">
         <v>64</v>
       </c>
-      <c r="S63" s="46"/>
+      <c r="S63" s="53"/>
     </row>
     <row r="64" spans="1:19" x14ac:dyDescent="0.25">
       <c r="B64" s="2" t="s">
@@ -2462,37 +2463,37 @@
       <c r="S65" s="2"/>
     </row>
     <row r="68" spans="2:19" x14ac:dyDescent="0.25">
-      <c r="B68" s="42" t="s">
+      <c r="B68" s="49" t="s">
         <v>22</v>
       </c>
-      <c r="C68" s="42"/>
+      <c r="C68" s="49"/>
       <c r="E68" s="9" t="s">
         <v>67</v>
       </c>
-      <c r="G68" s="42" t="s">
+      <c r="G68" s="49" t="s">
         <v>87</v>
       </c>
-      <c r="H68" s="42"/>
+      <c r="H68" s="49"/>
     </row>
     <row r="69" spans="2:19" x14ac:dyDescent="0.25">
-      <c r="B69" s="43">
+      <c r="B69" s="50">
         <f>SUM(B65:K65,M65:P65,R65:S65)</f>
         <v>17</v>
       </c>
-      <c r="C69" s="43"/>
-      <c r="E69" s="32"/>
-      <c r="G69" s="43">
+      <c r="C69" s="50"/>
+      <c r="E69" s="39"/>
+      <c r="G69" s="50">
         <f>50-SUM(B65:K65,M65:P65,R65:S65)</f>
         <v>33</v>
       </c>
-      <c r="H69" s="43"/>
+      <c r="H69" s="50"/>
     </row>
     <row r="70" spans="2:19" x14ac:dyDescent="0.25">
-      <c r="B70" s="43"/>
-      <c r="C70" s="43"/>
-      <c r="E70" s="32"/>
-      <c r="G70" s="43"/>
-      <c r="H70" s="43"/>
+      <c r="B70" s="50"/>
+      <c r="C70" s="50"/>
+      <c r="E70" s="39"/>
+      <c r="G70" s="50"/>
+      <c r="H70" s="50"/>
     </row>
   </sheetData>
   <mergeCells count="39">
@@ -2570,60 +2571,60 @@
   <sheetData>
     <row r="1" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="2" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B2" s="51" t="s">
+      <c r="B2" s="58" t="s">
         <v>133</v>
       </c>
-      <c r="C2" s="52"/>
-      <c r="D2" s="52"/>
-      <c r="E2" s="52"/>
-      <c r="F2" s="52"/>
-      <c r="G2" s="52"/>
-      <c r="H2" s="52"/>
-      <c r="I2" s="52"/>
-      <c r="J2" s="52"/>
-      <c r="K2" s="52"/>
-      <c r="L2" s="52"/>
-      <c r="M2" s="52"/>
-      <c r="N2" s="52"/>
-      <c r="O2" s="52"/>
-      <c r="P2" s="53"/>
+      <c r="C2" s="59"/>
+      <c r="D2" s="59"/>
+      <c r="E2" s="59"/>
+      <c r="F2" s="59"/>
+      <c r="G2" s="59"/>
+      <c r="H2" s="59"/>
+      <c r="I2" s="59"/>
+      <c r="J2" s="59"/>
+      <c r="K2" s="59"/>
+      <c r="L2" s="59"/>
+      <c r="M2" s="59"/>
+      <c r="N2" s="59"/>
+      <c r="O2" s="59"/>
+      <c r="P2" s="60"/>
     </row>
     <row r="3" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B3" s="54"/>
-      <c r="C3" s="55"/>
-      <c r="D3" s="55"/>
-      <c r="E3" s="55"/>
-      <c r="F3" s="55"/>
-      <c r="G3" s="55"/>
-      <c r="H3" s="55"/>
-      <c r="I3" s="55"/>
-      <c r="J3" s="55"/>
-      <c r="K3" s="55"/>
-      <c r="L3" s="55"/>
-      <c r="M3" s="55"/>
-      <c r="N3" s="55"/>
-      <c r="O3" s="55"/>
-      <c r="P3" s="56"/>
+      <c r="B3" s="61"/>
+      <c r="C3" s="62"/>
+      <c r="D3" s="62"/>
+      <c r="E3" s="62"/>
+      <c r="F3" s="62"/>
+      <c r="G3" s="62"/>
+      <c r="H3" s="62"/>
+      <c r="I3" s="62"/>
+      <c r="J3" s="62"/>
+      <c r="K3" s="62"/>
+      <c r="L3" s="62"/>
+      <c r="M3" s="62"/>
+      <c r="N3" s="62"/>
+      <c r="O3" s="62"/>
+      <c r="P3" s="63"/>
       <c r="R3" s="12"/>
     </row>
     <row r="5" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B5" s="46" t="s">
+      <c r="B5" s="53" t="s">
         <v>18</v>
       </c>
-      <c r="C5" s="46"/>
-      <c r="D5" s="46"/>
-      <c r="E5" s="46"/>
-      <c r="F5" s="46"/>
-      <c r="G5" s="46"/>
+      <c r="C5" s="53"/>
+      <c r="D5" s="53"/>
+      <c r="E5" s="53"/>
+      <c r="F5" s="53"/>
+      <c r="G5" s="53"/>
       <c r="I5" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="K5" s="39" t="s">
+      <c r="K5" s="46" t="s">
         <v>8</v>
       </c>
-      <c r="L5" s="40"/>
-      <c r="M5" s="40"/>
-      <c r="N5" s="41"/>
+      <c r="L5" s="47"/>
+      <c r="M5" s="47"/>
+      <c r="N5" s="48"/>
       <c r="P5" s="4" t="s">
         <v>74</v>
       </c>
@@ -2705,28 +2706,28 @@
       </c>
     </row>
     <row r="9" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B9" s="42" t="s">
+      <c r="B9" s="49" t="s">
         <v>22</v>
       </c>
-      <c r="C9" s="42"/>
+      <c r="C9" s="49"/>
       <c r="E9" s="9" t="s">
         <v>67</v>
       </c>
     </row>
     <row r="10" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B10" s="43">
+      <c r="B10" s="50">
         <f>_xlfn.CEILING.MATH(SUM(B7:G7,I7,K7:N7,P7),1,1)</f>
         <v>110</v>
       </c>
-      <c r="C10" s="43"/>
-      <c r="E10" s="47">
+      <c r="C10" s="50"/>
+      <c r="E10" s="54">
         <v>4</v>
       </c>
     </row>
     <row r="11" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B11" s="43"/>
-      <c r="C11" s="43"/>
-      <c r="E11" s="48"/>
+      <c r="B11" s="50"/>
+      <c r="C11" s="50"/>
+      <c r="E11" s="55"/>
     </row>
     <row r="12" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A12" s="6"/>
@@ -2751,40 +2752,40 @@
     </row>
     <row r="13" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="14" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B14" s="51" t="s">
+      <c r="B14" s="58" t="s">
         <v>134</v>
       </c>
-      <c r="C14" s="52"/>
-      <c r="D14" s="52"/>
-      <c r="E14" s="52"/>
-      <c r="F14" s="52"/>
-      <c r="G14" s="52"/>
-      <c r="H14" s="53"/>
+      <c r="C14" s="59"/>
+      <c r="D14" s="59"/>
+      <c r="E14" s="59"/>
+      <c r="F14" s="59"/>
+      <c r="G14" s="59"/>
+      <c r="H14" s="60"/>
     </row>
     <row r="15" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B15" s="54"/>
-      <c r="C15" s="55"/>
-      <c r="D15" s="55"/>
-      <c r="E15" s="55"/>
-      <c r="F15" s="55"/>
-      <c r="G15" s="55"/>
-      <c r="H15" s="56"/>
+      <c r="B15" s="61"/>
+      <c r="C15" s="62"/>
+      <c r="D15" s="62"/>
+      <c r="E15" s="62"/>
+      <c r="F15" s="62"/>
+      <c r="G15" s="62"/>
+      <c r="H15" s="63"/>
     </row>
     <row r="17" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B17" s="46" t="s">
+      <c r="B17" s="53" t="s">
         <v>12</v>
       </c>
-      <c r="C17" s="46"/>
-      <c r="D17" s="46"/>
-      <c r="F17" s="46" t="s">
+      <c r="C17" s="53"/>
+      <c r="D17" s="53"/>
+      <c r="F17" s="53" t="s">
         <v>8</v>
       </c>
-      <c r="G17" s="46"/>
-      <c r="H17" s="46"/>
-      <c r="J17" s="42" t="s">
+      <c r="G17" s="53"/>
+      <c r="H17" s="53"/>
+      <c r="J17" s="49" t="s">
         <v>22</v>
       </c>
-      <c r="K17" s="42"/>
+      <c r="K17" s="49"/>
       <c r="M17" s="9" t="s">
         <v>67</v>
       </c>
@@ -2808,12 +2809,12 @@
       <c r="H18" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="J18" s="43">
+      <c r="J18" s="50">
         <f>SUM(B19:D19,F19:H19)</f>
         <v>93</v>
       </c>
-      <c r="K18" s="43"/>
-      <c r="M18" s="32">
+      <c r="K18" s="50"/>
+      <c r="M18" s="39">
         <v>5</v>
       </c>
     </row>
@@ -2836,9 +2837,9 @@
       <c r="H19" s="2">
         <v>4</v>
       </c>
-      <c r="J19" s="43"/>
-      <c r="K19" s="43"/>
-      <c r="M19" s="32"/>
+      <c r="J19" s="50"/>
+      <c r="K19" s="50"/>
+      <c r="M19" s="39"/>
     </row>
     <row r="21" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A21" s="6"/>
@@ -2863,46 +2864,46 @@
     </row>
     <row r="22" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="23" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B23" s="51" t="s">
+      <c r="B23" s="58" t="s">
         <v>135</v>
       </c>
-      <c r="C23" s="52"/>
-      <c r="D23" s="52"/>
-      <c r="E23" s="52"/>
-      <c r="F23" s="52"/>
-      <c r="G23" s="52"/>
-      <c r="H23" s="52"/>
-      <c r="I23" s="52"/>
-      <c r="J23" s="52"/>
-      <c r="K23" s="53"/>
+      <c r="C23" s="59"/>
+      <c r="D23" s="59"/>
+      <c r="E23" s="59"/>
+      <c r="F23" s="59"/>
+      <c r="G23" s="59"/>
+      <c r="H23" s="59"/>
+      <c r="I23" s="59"/>
+      <c r="J23" s="59"/>
+      <c r="K23" s="60"/>
     </row>
     <row r="24" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B24" s="54"/>
-      <c r="C24" s="55"/>
-      <c r="D24" s="55"/>
-      <c r="E24" s="55"/>
-      <c r="F24" s="55"/>
-      <c r="G24" s="55"/>
-      <c r="H24" s="55"/>
-      <c r="I24" s="55"/>
-      <c r="J24" s="55"/>
-      <c r="K24" s="56"/>
+      <c r="B24" s="61"/>
+      <c r="C24" s="62"/>
+      <c r="D24" s="62"/>
+      <c r="E24" s="62"/>
+      <c r="F24" s="62"/>
+      <c r="G24" s="62"/>
+      <c r="H24" s="62"/>
+      <c r="I24" s="62"/>
+      <c r="J24" s="62"/>
+      <c r="K24" s="63"/>
     </row>
     <row r="26" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B26" s="46" t="s">
+      <c r="B26" s="53" t="s">
         <v>17</v>
       </c>
-      <c r="C26" s="46"/>
-      <c r="E26" s="39" t="s">
+      <c r="C26" s="53"/>
+      <c r="E26" s="46" t="s">
         <v>21</v>
       </c>
-      <c r="F26" s="40"/>
-      <c r="G26" s="41"/>
-      <c r="I26" s="46" t="s">
+      <c r="F26" s="47"/>
+      <c r="G26" s="48"/>
+      <c r="I26" s="53" t="s">
         <v>20</v>
       </c>
-      <c r="J26" s="46"/>
-      <c r="K26" s="46"/>
+      <c r="J26" s="53"/>
+      <c r="K26" s="53"/>
       <c r="M26" s="10" t="s">
         <v>22</v>
       </c>
@@ -2937,12 +2938,12 @@
       <c r="K27" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="M27" s="57">
+      <c r="M27" s="64">
         <f>SUM(B28:C28,E28:G28,I28:K28)</f>
         <v>36</v>
       </c>
       <c r="N27" s="7"/>
-      <c r="O27" s="32">
+      <c r="O27" s="39">
         <v>4</v>
       </c>
       <c r="P27" s="8"/>
@@ -2972,9 +2973,9 @@
       <c r="K28" s="2">
         <v>3.2</v>
       </c>
-      <c r="M28" s="57"/>
+      <c r="M28" s="64"/>
       <c r="N28" s="7"/>
-      <c r="O28" s="32"/>
+      <c r="O28" s="39"/>
       <c r="P28" s="8"/>
     </row>
     <row r="30" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -3000,39 +3001,39 @@
     </row>
     <row r="31" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="32" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B32" s="51" t="s">
+      <c r="B32" s="58" t="s">
         <v>136</v>
       </c>
-      <c r="C32" s="52"/>
-      <c r="D32" s="52"/>
-      <c r="E32" s="52"/>
-      <c r="F32" s="52"/>
-      <c r="G32" s="52"/>
-      <c r="H32" s="52"/>
-      <c r="I32" s="53"/>
+      <c r="C32" s="59"/>
+      <c r="D32" s="59"/>
+      <c r="E32" s="59"/>
+      <c r="F32" s="59"/>
+      <c r="G32" s="59"/>
+      <c r="H32" s="59"/>
+      <c r="I32" s="60"/>
     </row>
     <row r="33" spans="2:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B33" s="54"/>
-      <c r="C33" s="55"/>
-      <c r="D33" s="55"/>
-      <c r="E33" s="55"/>
-      <c r="F33" s="55"/>
-      <c r="G33" s="55"/>
-      <c r="H33" s="55"/>
-      <c r="I33" s="56"/>
+      <c r="B33" s="61"/>
+      <c r="C33" s="62"/>
+      <c r="D33" s="62"/>
+      <c r="E33" s="62"/>
+      <c r="F33" s="62"/>
+      <c r="G33" s="62"/>
+      <c r="H33" s="62"/>
+      <c r="I33" s="63"/>
     </row>
     <row r="35" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B35" s="46" t="s">
+      <c r="B35" s="53" t="s">
         <v>31</v>
       </c>
-      <c r="C35" s="46"/>
-      <c r="D35" s="46"/>
-      <c r="F35" s="46" t="s">
+      <c r="C35" s="53"/>
+      <c r="D35" s="53"/>
+      <c r="F35" s="53" t="s">
         <v>12</v>
       </c>
-      <c r="G35" s="46"/>
-      <c r="H35" s="46"/>
-      <c r="I35" s="46"/>
+      <c r="G35" s="53"/>
+      <c r="H35" s="53"/>
+      <c r="I35" s="53"/>
       <c r="N35" s="7"/>
       <c r="O35" s="7"/>
     </row>
@@ -3089,14 +3090,14 @@
       <c r="O37" s="7"/>
     </row>
     <row r="40" spans="2:15" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B40" s="44" t="s">
+      <c r="B40" s="51" t="s">
         <v>35</v>
       </c>
-      <c r="C40" s="45"/>
-      <c r="F40" s="43" t="s">
+      <c r="C40" s="52"/>
+      <c r="F40" s="50" t="s">
         <v>36</v>
       </c>
-      <c r="G40" s="43"/>
+      <c r="G40" s="50"/>
       <c r="I40" s="9" t="s">
         <v>22</v>
       </c>
@@ -3152,7 +3153,7 @@
       <c r="G43" s="2">
         <v>0.44</v>
       </c>
-      <c r="I43" s="42" t="s">
+      <c r="I43" s="49" t="s">
         <v>67</v>
       </c>
     </row>
@@ -3169,7 +3170,7 @@
       <c r="G44" s="2">
         <v>1</v>
       </c>
-      <c r="I44" s="42"/>
+      <c r="I44" s="49"/>
     </row>
     <row r="45" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B45" s="2" t="s">
@@ -3313,67 +3314,67 @@
     </row>
     <row r="57" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="58" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B58" s="51" t="s">
+      <c r="B58" s="58" t="s">
         <v>137</v>
       </c>
-      <c r="C58" s="52"/>
-      <c r="D58" s="52"/>
-      <c r="E58" s="52"/>
-      <c r="F58" s="52"/>
-      <c r="G58" s="52"/>
-      <c r="H58" s="52"/>
-      <c r="I58" s="52"/>
-      <c r="J58" s="52"/>
-      <c r="K58" s="52"/>
-      <c r="L58" s="52"/>
-      <c r="M58" s="52"/>
-      <c r="N58" s="52"/>
-      <c r="O58" s="52"/>
-      <c r="P58" s="52"/>
-      <c r="Q58" s="52"/>
-      <c r="R58" s="53"/>
+      <c r="C58" s="59"/>
+      <c r="D58" s="59"/>
+      <c r="E58" s="59"/>
+      <c r="F58" s="59"/>
+      <c r="G58" s="59"/>
+      <c r="H58" s="59"/>
+      <c r="I58" s="59"/>
+      <c r="J58" s="59"/>
+      <c r="K58" s="59"/>
+      <c r="L58" s="59"/>
+      <c r="M58" s="59"/>
+      <c r="N58" s="59"/>
+      <c r="O58" s="59"/>
+      <c r="P58" s="59"/>
+      <c r="Q58" s="59"/>
+      <c r="R58" s="60"/>
     </row>
     <row r="59" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B59" s="54"/>
-      <c r="C59" s="55"/>
-      <c r="D59" s="55"/>
-      <c r="E59" s="55"/>
-      <c r="F59" s="55"/>
-      <c r="G59" s="55"/>
-      <c r="H59" s="55"/>
-      <c r="I59" s="55"/>
-      <c r="J59" s="55"/>
-      <c r="K59" s="55"/>
-      <c r="L59" s="55"/>
-      <c r="M59" s="55"/>
-      <c r="N59" s="55"/>
-      <c r="O59" s="55"/>
-      <c r="P59" s="55"/>
-      <c r="Q59" s="55"/>
-      <c r="R59" s="56"/>
+      <c r="B59" s="61"/>
+      <c r="C59" s="62"/>
+      <c r="D59" s="62"/>
+      <c r="E59" s="62"/>
+      <c r="F59" s="62"/>
+      <c r="G59" s="62"/>
+      <c r="H59" s="62"/>
+      <c r="I59" s="62"/>
+      <c r="J59" s="62"/>
+      <c r="K59" s="62"/>
+      <c r="L59" s="62"/>
+      <c r="M59" s="62"/>
+      <c r="N59" s="62"/>
+      <c r="O59" s="62"/>
+      <c r="P59" s="62"/>
+      <c r="Q59" s="62"/>
+      <c r="R59" s="63"/>
     </row>
     <row r="61" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B61" s="46" t="s">
+      <c r="B61" s="53" t="s">
         <v>63</v>
       </c>
-      <c r="C61" s="46"/>
-      <c r="D61" s="46"/>
-      <c r="E61" s="46"/>
-      <c r="F61" s="46"/>
-      <c r="G61" s="46"/>
-      <c r="H61" s="46"/>
-      <c r="I61" s="46"/>
-      <c r="J61" s="46"/>
-      <c r="K61" s="46"/>
-      <c r="M61" s="46" t="s">
+      <c r="C61" s="53"/>
+      <c r="D61" s="53"/>
+      <c r="E61" s="53"/>
+      <c r="F61" s="53"/>
+      <c r="G61" s="53"/>
+      <c r="H61" s="53"/>
+      <c r="I61" s="53"/>
+      <c r="J61" s="53"/>
+      <c r="K61" s="53"/>
+      <c r="M61" s="53" t="s">
         <v>68</v>
       </c>
-      <c r="N61" s="46"/>
-      <c r="O61" s="46"/>
-      <c r="Q61" s="46" t="s">
+      <c r="N61" s="53"/>
+      <c r="O61" s="53"/>
+      <c r="Q61" s="53" t="s">
         <v>64</v>
       </c>
-      <c r="R61" s="46"/>
+      <c r="R61" s="53"/>
     </row>
     <row r="62" spans="1:19" x14ac:dyDescent="0.25">
       <c r="B62" s="2" t="s">
@@ -3470,28 +3471,28 @@
       </c>
     </row>
     <row r="66" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B66" s="42" t="s">
+      <c r="B66" s="49" t="s">
         <v>22</v>
       </c>
-      <c r="C66" s="42"/>
+      <c r="C66" s="49"/>
       <c r="E66" s="9" t="s">
         <v>67</v>
       </c>
     </row>
     <row r="67" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B67" s="43">
+      <c r="B67" s="50">
         <f xml:space="preserve"> SUM(B63:K63,M63:O63,Q63:R63)</f>
         <v>85.5</v>
       </c>
-      <c r="C67" s="43"/>
-      <c r="E67" s="32">
+      <c r="C67" s="50"/>
+      <c r="E67" s="39">
         <v>4.5</v>
       </c>
     </row>
     <row r="68" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B68" s="43"/>
-      <c r="C68" s="43"/>
-      <c r="E68" s="32"/>
+      <c r="B68" s="50"/>
+      <c r="C68" s="50"/>
+      <c r="E68" s="39"/>
     </row>
     <row r="70" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A70" s="6"/>
@@ -3516,26 +3517,26 @@
     </row>
     <row r="71" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="72" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B72" s="51" t="s">
+      <c r="B72" s="58" t="s">
         <v>138</v>
       </c>
-      <c r="C72" s="52"/>
-      <c r="D72" s="52"/>
-      <c r="E72" s="52"/>
-      <c r="F72" s="52"/>
-      <c r="G72" s="52"/>
-      <c r="H72" s="52"/>
-      <c r="I72" s="53"/>
+      <c r="C72" s="59"/>
+      <c r="D72" s="59"/>
+      <c r="E72" s="59"/>
+      <c r="F72" s="59"/>
+      <c r="G72" s="59"/>
+      <c r="H72" s="59"/>
+      <c r="I72" s="60"/>
     </row>
     <row r="73" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B73" s="54"/>
-      <c r="C73" s="55"/>
-      <c r="D73" s="55"/>
-      <c r="E73" s="55"/>
-      <c r="F73" s="55"/>
-      <c r="G73" s="55"/>
-      <c r="H73" s="55"/>
-      <c r="I73" s="56"/>
+      <c r="B73" s="61"/>
+      <c r="C73" s="62"/>
+      <c r="D73" s="62"/>
+      <c r="E73" s="62"/>
+      <c r="F73" s="62"/>
+      <c r="G73" s="62"/>
+      <c r="H73" s="62"/>
+      <c r="I73" s="63"/>
     </row>
     <row r="75" spans="1:19" x14ac:dyDescent="0.25">
       <c r="B75" s="4" t="s">
@@ -3562,10 +3563,10 @@
       <c r="I75" s="4" t="s">
         <v>146</v>
       </c>
-      <c r="K75" s="42" t="s">
+      <c r="K75" s="49" t="s">
         <v>22</v>
       </c>
-      <c r="L75" s="42"/>
+      <c r="L75" s="49"/>
       <c r="N75" s="9" t="s">
         <v>67</v>
       </c>
@@ -3595,11 +3596,11 @@
       <c r="I76" s="2">
         <v>5</v>
       </c>
-      <c r="K76" s="43">
+      <c r="K76" s="50">
         <f>SUM(B76:I76)</f>
         <v>96</v>
       </c>
-      <c r="L76" s="43"/>
+      <c r="L76" s="50"/>
       <c r="N76" s="13">
         <v>5</v>
       </c>
@@ -4169,53 +4170,53 @@
   <sheetData>
     <row r="1" spans="2:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="2" spans="2:12" ht="23.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B2" s="62" t="s">
+      <c r="B2" s="65" t="s">
         <v>204</v>
       </c>
-      <c r="C2" s="63"/>
-      <c r="D2" s="64"/>
-      <c r="F2" s="62" t="s">
+      <c r="C2" s="66"/>
+      <c r="D2" s="67"/>
+      <c r="F2" s="65" t="s">
         <v>205</v>
       </c>
-      <c r="G2" s="63"/>
-      <c r="H2" s="64"/>
-      <c r="J2" s="62" t="s">
+      <c r="G2" s="66"/>
+      <c r="H2" s="67"/>
+      <c r="J2" s="65" t="s">
         <v>206</v>
       </c>
-      <c r="K2" s="63"/>
-      <c r="L2" s="64"/>
+      <c r="K2" s="66"/>
+      <c r="L2" s="67"/>
     </row>
     <row r="3" spans="2:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B3" s="65" t="s">
+      <c r="B3" s="34" t="s">
         <v>148</v>
       </c>
-      <c r="C3" s="66" t="s">
+      <c r="C3" s="35" t="s">
         <v>197</v>
       </c>
-      <c r="D3" s="67" t="s">
+      <c r="D3" s="36" t="s">
         <v>196</v>
       </c>
-      <c r="F3" s="65" t="s">
+      <c r="F3" s="34" t="s">
         <v>148</v>
       </c>
-      <c r="G3" s="66" t="s">
+      <c r="G3" s="35" t="s">
         <v>197</v>
       </c>
-      <c r="H3" s="67" t="s">
+      <c r="H3" s="36" t="s">
         <v>196</v>
       </c>
-      <c r="J3" s="65" t="s">
+      <c r="J3" s="34" t="s">
         <v>148</v>
       </c>
-      <c r="K3" s="66" t="s">
+      <c r="K3" s="35" t="s">
         <v>197</v>
       </c>
-      <c r="L3" s="67" t="s">
+      <c r="L3" s="36" t="s">
         <v>196</v>
       </c>
     </row>
     <row r="4" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B4" s="68" t="s">
+      <c r="B4" s="37" t="s">
         <v>133</v>
       </c>
       <c r="C4" s="14">
@@ -4224,14 +4225,14 @@
       <c r="D4" s="14">
         <v>4</v>
       </c>
-      <c r="F4" s="68" t="s">
+      <c r="F4" s="37" t="s">
         <v>76</v>
       </c>
       <c r="G4" s="14">
         <v>5</v>
       </c>
       <c r="H4" s="14"/>
-      <c r="J4" s="68" t="s">
+      <c r="J4" s="37" t="s">
         <v>199</v>
       </c>
       <c r="K4" s="14">
@@ -4240,7 +4241,7 @@
       <c r="L4" s="14"/>
     </row>
     <row r="5" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B5" s="69" t="s">
+      <c r="B5" s="38" t="s">
         <v>134</v>
       </c>
       <c r="C5" s="2">
@@ -4249,14 +4250,14 @@
       <c r="D5" s="2">
         <v>5</v>
       </c>
-      <c r="F5" s="69" t="s">
+      <c r="F5" s="38" t="s">
         <v>79</v>
       </c>
       <c r="G5" s="2">
         <v>4</v>
       </c>
       <c r="H5" s="2"/>
-      <c r="J5" s="69" t="s">
+      <c r="J5" s="38" t="s">
         <v>200</v>
       </c>
       <c r="K5" s="2">
@@ -4265,7 +4266,7 @@
       <c r="L5" s="2"/>
     </row>
     <row r="6" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B6" s="69" t="s">
+      <c r="B6" s="38" t="s">
         <v>135</v>
       </c>
       <c r="C6" s="2">
@@ -4274,14 +4275,14 @@
       <c r="D6" s="2">
         <v>4</v>
       </c>
-      <c r="F6" s="69" t="s">
+      <c r="F6" s="38" t="s">
         <v>77</v>
       </c>
       <c r="G6" s="2">
         <v>5</v>
       </c>
       <c r="H6" s="2"/>
-      <c r="J6" s="69" t="s">
+      <c r="J6" s="38" t="s">
         <v>201</v>
       </c>
       <c r="K6" s="2">
@@ -4290,7 +4291,7 @@
       <c r="L6" s="2"/>
     </row>
     <row r="7" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B7" s="69" t="s">
+      <c r="B7" s="38" t="s">
         <v>136</v>
       </c>
       <c r="C7" s="2">
@@ -4299,14 +4300,14 @@
       <c r="D7" s="2">
         <v>4</v>
       </c>
-      <c r="F7" s="69" t="s">
+      <c r="F7" s="38" t="s">
         <v>78</v>
       </c>
       <c r="G7" s="2">
         <v>5</v>
       </c>
       <c r="H7" s="2"/>
-      <c r="J7" s="69" t="s">
+      <c r="J7" s="38" t="s">
         <v>202</v>
       </c>
       <c r="K7" s="2">
@@ -4315,7 +4316,7 @@
       <c r="L7" s="2"/>
     </row>
     <row r="8" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B8" s="69" t="s">
+      <c r="B8" s="38" t="s">
         <v>137</v>
       </c>
       <c r="C8" s="2">
@@ -4324,14 +4325,14 @@
       <c r="D8" s="2">
         <v>4.5</v>
       </c>
-      <c r="F8" s="69" t="s">
+      <c r="F8" s="38" t="s">
         <v>80</v>
       </c>
       <c r="G8" s="2">
         <v>11</v>
       </c>
       <c r="H8" s="2"/>
-      <c r="J8" s="69" t="s">
+      <c r="J8" s="38" t="s">
         <v>203</v>
       </c>
       <c r="K8" s="2">
@@ -4340,7 +4341,7 @@
       <c r="L8" s="2"/>
     </row>
     <row r="9" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B9" s="69" t="s">
+      <c r="B9" s="38" t="s">
         <v>138</v>
       </c>
       <c r="C9" s="2">
@@ -4349,36 +4350,36 @@
       <c r="D9" s="2">
         <v>5</v>
       </c>
-      <c r="F9" s="58"/>
-      <c r="G9" s="70"/>
-      <c r="H9" s="70"/>
-      <c r="J9" s="58"/>
-      <c r="K9" s="70"/>
-      <c r="L9" s="70"/>
+      <c r="F9" s="32"/>
+      <c r="G9" s="1"/>
+      <c r="H9" s="1"/>
+      <c r="J9" s="32"/>
+      <c r="K9" s="1"/>
+      <c r="L9" s="1"/>
     </row>
     <row r="10" spans="2:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="11" spans="2:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B11" s="59" t="s">
+      <c r="B11" s="68" t="s">
         <v>198</v>
       </c>
-      <c r="C11" s="60"/>
-      <c r="D11" s="61">
+      <c r="C11" s="69"/>
+      <c r="D11" s="33">
         <f>(D4*C4+D5*C5+D6*C6+D7*C7+D8*C8+D9*C9)/30</f>
         <v>4.4333333333333336</v>
       </c>
-      <c r="F11" s="59" t="s">
+      <c r="F11" s="68" t="s">
         <v>198</v>
       </c>
-      <c r="G11" s="60"/>
-      <c r="H11" s="61">
+      <c r="G11" s="69"/>
+      <c r="H11" s="33">
         <f>(H4*G4+H5*G5+H6*G6+H7*G7+H8*G8)/30</f>
         <v>0</v>
       </c>
-      <c r="J11" s="59" t="s">
+      <c r="J11" s="68" t="s">
         <v>198</v>
       </c>
-      <c r="K11" s="60"/>
-      <c r="L11" s="61">
+      <c r="K11" s="69"/>
+      <c r="L11" s="33">
         <f>(L4*K4+L5*K5+L6*K6+L7*K7+L8*K8)/30</f>
         <v>0</v>
       </c>

</xml_diff>

<commit_message>
Points from the colloquium 1 - POTEC
</commit_message>
<xml_diff>
--- a/IoT-points-schedule.xlsx
+++ b/IoT-points-schedule.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\dodo\Desktop\IoT-studies\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B005063B-2C41-45D2-B4E8-5D2F36428623}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A34F131B-8E13-4E22-8B4D-9D282295A033}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="25440" windowHeight="15390" xr2:uid="{F85F5544-1FE8-4920-A5D4-192A98B113BD}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="335" uniqueCount="207">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="334" uniqueCount="211">
   <si>
     <t>1. Krypto</t>
   </si>
@@ -660,6 +660,18 @@
   </si>
   <si>
     <t>III semestr (25Z)</t>
+  </si>
+  <si>
+    <t>LAB1 (γ)</t>
+  </si>
+  <si>
+    <t>LAB3 (Lepkość)</t>
+  </si>
+  <si>
+    <t>LAB2 (Interferencja)</t>
+  </si>
+  <si>
+    <t>LAB4 (Magnetyzm)</t>
   </si>
 </sst>
 </file>
@@ -1018,7 +1030,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="70">
+  <cellXfs count="68">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1165,12 +1177,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1241,6 +1247,10 @@
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <mruColors>
+      <color rgb="FFFF8585"/>
+      <color rgb="FFFDBF8B"/>
+      <color rgb="FFFDAF6F"/>
+      <color rgb="FFFFCC66"/>
       <color rgb="FFDEEDF4"/>
       <color rgb="FFE3EAEF"/>
     </mruColors>
@@ -1599,7 +1609,7 @@
     <col min="4" max="4" width="16" style="1" customWidth="1"/>
     <col min="5" max="5" width="16.28515625" style="1" customWidth="1"/>
     <col min="6" max="6" width="16.85546875" style="1" customWidth="1"/>
-    <col min="7" max="7" width="16.5703125" style="1" customWidth="1"/>
+    <col min="7" max="7" width="17.7109375" style="1" customWidth="1"/>
     <col min="8" max="8" width="16.7109375" style="1" customWidth="1"/>
     <col min="9" max="9" width="17.140625" style="1" customWidth="1"/>
     <col min="10" max="10" width="12.85546875" style="1" customWidth="1"/>
@@ -1654,23 +1664,23 @@
       <c r="R3" s="12"/>
     </row>
     <row r="5" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B5" s="50" t="s">
+      <c r="B5" s="48" t="s">
         <v>83</v>
       </c>
-      <c r="C5" s="52"/>
-      <c r="D5" s="52"/>
-      <c r="E5" s="52"/>
-      <c r="F5" s="51"/>
-      <c r="H5" s="50" t="s">
+      <c r="C5" s="50"/>
+      <c r="D5" s="50"/>
+      <c r="E5" s="50"/>
+      <c r="F5" s="49"/>
+      <c r="H5" s="48" t="s">
         <v>82</v>
       </c>
-      <c r="I5" s="51"/>
-      <c r="K5" s="50" t="s">
+      <c r="I5" s="49"/>
+      <c r="K5" s="48" t="s">
         <v>8</v>
       </c>
-      <c r="L5" s="52"/>
-      <c r="M5" s="52"/>
-      <c r="N5" s="51"/>
+      <c r="L5" s="50"/>
+      <c r="M5" s="50"/>
+      <c r="N5" s="49"/>
       <c r="P5" s="4" t="s">
         <v>74</v>
       </c>
@@ -1730,37 +1740,37 @@
       <c r="P7" s="2"/>
     </row>
     <row r="9" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B9" s="53" t="s">
+      <c r="B9" s="51" t="s">
         <v>22</v>
       </c>
-      <c r="C9" s="53"/>
+      <c r="C9" s="51"/>
       <c r="E9" s="9" t="s">
         <v>67</v>
       </c>
-      <c r="G9" s="53" t="s">
+      <c r="G9" s="51" t="s">
         <v>87</v>
       </c>
-      <c r="H9" s="53"/>
+      <c r="H9" s="51"/>
     </row>
     <row r="10" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B10" s="54">
+      <c r="B10" s="52">
         <f>SUM(B7:F7,H7:I7,K7:N7,P7)</f>
         <v>9.6999999999999993</v>
       </c>
-      <c r="C10" s="54"/>
+      <c r="C10" s="52"/>
       <c r="E10" s="46"/>
-      <c r="G10" s="54">
+      <c r="G10" s="52">
         <f>66-SUM(B7:F7,H7:I7,K7:N7,P7)</f>
         <v>56.3</v>
       </c>
-      <c r="H10" s="54"/>
+      <c r="H10" s="52"/>
     </row>
     <row r="11" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B11" s="54"/>
-      <c r="C11" s="54"/>
+      <c r="B11" s="52"/>
+      <c r="C11" s="52"/>
       <c r="E11" s="47"/>
-      <c r="G11" s="54"/>
-      <c r="H11" s="54"/>
+      <c r="G11" s="52"/>
+      <c r="H11" s="52"/>
     </row>
     <row r="12" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A12" s="6"/>
@@ -1812,19 +1822,19 @@
       <c r="D17" s="39"/>
       <c r="E17" s="39"/>
       <c r="F17" s="39"/>
-      <c r="H17" s="50" t="s">
+      <c r="H17" s="48" t="s">
         <v>97</v>
       </c>
-      <c r="I17" s="52"/>
-      <c r="J17" s="51"/>
-      <c r="L17" s="53" t="s">
+      <c r="I17" s="50"/>
+      <c r="J17" s="49"/>
+      <c r="L17" s="51" t="s">
         <v>22</v>
       </c>
-      <c r="M17" s="53"/>
-      <c r="O17" s="53" t="s">
+      <c r="M17" s="51"/>
+      <c r="O17" s="51" t="s">
         <v>87</v>
       </c>
-      <c r="P17" s="53"/>
+      <c r="P17" s="51"/>
       <c r="R17" s="9" t="s">
         <v>67</v>
       </c>
@@ -1854,17 +1864,17 @@
       <c r="J18" s="3" t="s">
         <v>95</v>
       </c>
-      <c r="L18" s="54">
+      <c r="L18" s="52">
         <f>SUM(B19:F19,H19:J19)</f>
         <v>29.5</v>
       </c>
-      <c r="M18" s="54"/>
-      <c r="O18" s="54">
+      <c r="M18" s="52"/>
+      <c r="O18" s="52">
         <f>50-SUM(B19:F19,H19:J19)</f>
         <v>20.5</v>
       </c>
-      <c r="P18" s="54"/>
-      <c r="R18" s="55"/>
+      <c r="P18" s="52"/>
+      <c r="R18" s="53"/>
     </row>
     <row r="19" spans="1:19" x14ac:dyDescent="0.25">
       <c r="B19" s="2"/>
@@ -1879,11 +1889,11 @@
         <v>26.5</v>
       </c>
       <c r="J19" s="2"/>
-      <c r="L19" s="54"/>
-      <c r="M19" s="54"/>
-      <c r="O19" s="54"/>
-      <c r="P19" s="54"/>
-      <c r="R19" s="55"/>
+      <c r="L19" s="52"/>
+      <c r="M19" s="52"/>
+      <c r="O19" s="52"/>
+      <c r="P19" s="52"/>
+      <c r="R19" s="53"/>
     </row>
     <row r="21" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A21" s="6"/>
@@ -1921,10 +1931,10 @@
       <c r="J23" s="41"/>
       <c r="K23" s="41"/>
       <c r="L23" s="42"/>
-      <c r="N23" s="54" t="s">
+      <c r="N23" s="52" t="s">
         <v>132</v>
       </c>
-      <c r="O23" s="54"/>
+      <c r="O23" s="52"/>
     </row>
     <row r="24" spans="1:19" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B24" s="43"/>
@@ -1938,8 +1948,8 @@
       <c r="J24" s="44"/>
       <c r="K24" s="44"/>
       <c r="L24" s="45"/>
-      <c r="N24" s="54"/>
-      <c r="O24" s="54"/>
+      <c r="N24" s="52"/>
+      <c r="O24" s="52"/>
     </row>
     <row r="26" spans="1:19" x14ac:dyDescent="0.25">
       <c r="B26" s="39" t="s">
@@ -1954,14 +1964,11 @@
       <c r="H26" s="39"/>
       <c r="I26" s="39"/>
       <c r="J26" s="7"/>
-      <c r="K26" s="50" t="s">
+      <c r="K26" s="48" t="s">
         <v>128</v>
       </c>
-      <c r="L26" s="51"/>
-      <c r="N26" s="10" t="s">
-        <v>22</v>
-      </c>
-      <c r="O26" s="9" t="s">
+      <c r="L26" s="49"/>
+      <c r="N26" s="9" t="s">
         <v>67</v>
       </c>
     </row>
@@ -1976,16 +1983,16 @@
         <v>11</v>
       </c>
       <c r="F27" s="2" t="s">
-        <v>103</v>
+        <v>207</v>
       </c>
       <c r="G27" s="2" t="s">
-        <v>104</v>
+        <v>209</v>
       </c>
       <c r="H27" s="2" t="s">
-        <v>105</v>
+        <v>208</v>
       </c>
       <c r="I27" s="2" t="s">
-        <v>106</v>
+        <v>210</v>
       </c>
       <c r="K27" s="14" t="s">
         <v>73</v>
@@ -1993,11 +2000,7 @@
       <c r="L27" s="2" t="s">
         <v>127</v>
       </c>
-      <c r="N27" s="48">
-        <f>SUM(B28:D28,F28:I28,K28:L28)</f>
-        <v>1</v>
-      </c>
-      <c r="O27" s="46"/>
+      <c r="N27" s="46"/>
     </row>
     <row r="28" spans="1:19" x14ac:dyDescent="0.25">
       <c r="B28" s="2"/>
@@ -2006,13 +2009,14 @@
         <v>1</v>
       </c>
       <c r="F28" s="2"/>
-      <c r="G28" s="2"/>
+      <c r="G28" s="2">
+        <v>5</v>
+      </c>
       <c r="H28" s="2"/>
       <c r="I28" s="2"/>
       <c r="K28" s="2"/>
       <c r="L28" s="2"/>
-      <c r="N28" s="49"/>
-      <c r="O28" s="47"/>
+      <c r="N28" s="47"/>
     </row>
     <row r="30" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A30" s="6"/>
@@ -2064,12 +2068,12 @@
       </c>
       <c r="C35" s="39"/>
       <c r="D35" s="7"/>
-      <c r="E35" s="50" t="s">
+      <c r="E35" s="48" t="s">
         <v>147</v>
       </c>
-      <c r="F35" s="52"/>
-      <c r="G35" s="52"/>
-      <c r="H35" s="51"/>
+      <c r="F35" s="50"/>
+      <c r="G35" s="50"/>
+      <c r="H35" s="49"/>
     </row>
     <row r="36" spans="2:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B36" s="2" t="s">
@@ -2093,7 +2097,9 @@
       <c r="O36" s="7"/>
     </row>
     <row r="37" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B37" s="2"/>
+      <c r="B37" s="2">
+        <v>17</v>
+      </c>
       <c r="C37" s="2"/>
       <c r="E37" s="2">
         <f>C56</f>
@@ -2108,14 +2114,14 @@
       <c r="O37" s="7"/>
     </row>
     <row r="40" spans="2:15" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B40" s="56" t="s">
+      <c r="B40" s="54" t="s">
         <v>126</v>
       </c>
-      <c r="C40" s="57"/>
-      <c r="F40" s="54" t="s">
+      <c r="C40" s="55"/>
+      <c r="F40" s="52" t="s">
         <v>102</v>
       </c>
-      <c r="G40" s="54"/>
+      <c r="G40" s="52"/>
       <c r="I40" s="9" t="s">
         <v>22</v>
       </c>
@@ -2137,7 +2143,7 @@
       </c>
       <c r="I41" s="2">
         <f>SUM(B37:C37,E37:H37)</f>
-        <v>22</v>
+        <v>39</v>
       </c>
       <c r="J41" s="7"/>
       <c r="L41" s="7"/>
@@ -2165,7 +2171,7 @@
         <v>119</v>
       </c>
       <c r="G43" s="2"/>
-      <c r="I43" s="53" t="s">
+      <c r="I43" s="51" t="s">
         <v>67</v>
       </c>
     </row>
@@ -2180,7 +2186,7 @@
         <v>120</v>
       </c>
       <c r="G44" s="2"/>
-      <c r="I44" s="53"/>
+      <c r="I44" s="51"/>
     </row>
     <row r="45" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B45" s="2" t="s">
@@ -2229,7 +2235,7 @@
       <c r="G48" s="2"/>
       <c r="I48" s="2">
         <f>50-SUM(B37:C37,E37:H37)</f>
-        <v>28</v>
+        <v>11</v>
       </c>
     </row>
     <row r="49" spans="1:19" x14ac:dyDescent="0.25">
@@ -2463,40 +2469,40 @@
       <c r="S65" s="2"/>
     </row>
     <row r="68" spans="2:19" x14ac:dyDescent="0.25">
-      <c r="B68" s="53" t="s">
+      <c r="B68" s="51" t="s">
         <v>22</v>
       </c>
-      <c r="C68" s="53"/>
+      <c r="C68" s="51"/>
       <c r="E68" s="9" t="s">
         <v>67</v>
       </c>
-      <c r="G68" s="53" t="s">
+      <c r="G68" s="51" t="s">
         <v>87</v>
       </c>
-      <c r="H68" s="53"/>
+      <c r="H68" s="51"/>
     </row>
     <row r="69" spans="2:19" x14ac:dyDescent="0.25">
-      <c r="B69" s="54">
+      <c r="B69" s="52">
         <f>SUM(B65:K65,M65:P65,R65:S65)</f>
         <v>17</v>
       </c>
-      <c r="C69" s="54"/>
-      <c r="E69" s="55"/>
-      <c r="G69" s="54">
+      <c r="C69" s="52"/>
+      <c r="E69" s="53"/>
+      <c r="G69" s="52">
         <f>50-SUM(B65:K65,M65:P65,R65:S65)</f>
         <v>33</v>
       </c>
-      <c r="H69" s="54"/>
+      <c r="H69" s="52"/>
     </row>
     <row r="70" spans="2:19" x14ac:dyDescent="0.25">
-      <c r="B70" s="54"/>
-      <c r="C70" s="54"/>
-      <c r="E70" s="55"/>
-      <c r="G70" s="54"/>
-      <c r="H70" s="54"/>
+      <c r="B70" s="52"/>
+      <c r="C70" s="52"/>
+      <c r="E70" s="53"/>
+      <c r="G70" s="52"/>
+      <c r="H70" s="52"/>
     </row>
   </sheetData>
-  <mergeCells count="39">
+  <mergeCells count="38">
     <mergeCell ref="R18:R19"/>
     <mergeCell ref="B14:H15"/>
     <mergeCell ref="K5:N5"/>
@@ -2525,7 +2531,6 @@
     <mergeCell ref="B10:C11"/>
     <mergeCell ref="L17:M17"/>
     <mergeCell ref="E10:E11"/>
-    <mergeCell ref="O27:O28"/>
     <mergeCell ref="N27:N28"/>
     <mergeCell ref="F26:I26"/>
     <mergeCell ref="K26:L26"/>
@@ -2571,40 +2576,40 @@
   <sheetData>
     <row r="1" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="2" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B2" s="58" t="s">
+      <c r="B2" s="56" t="s">
         <v>133</v>
       </c>
-      <c r="C2" s="59"/>
-      <c r="D2" s="59"/>
-      <c r="E2" s="59"/>
-      <c r="F2" s="59"/>
-      <c r="G2" s="59"/>
-      <c r="H2" s="59"/>
-      <c r="I2" s="59"/>
-      <c r="J2" s="59"/>
-      <c r="K2" s="59"/>
-      <c r="L2" s="59"/>
-      <c r="M2" s="59"/>
-      <c r="N2" s="59"/>
-      <c r="O2" s="59"/>
-      <c r="P2" s="60"/>
+      <c r="C2" s="57"/>
+      <c r="D2" s="57"/>
+      <c r="E2" s="57"/>
+      <c r="F2" s="57"/>
+      <c r="G2" s="57"/>
+      <c r="H2" s="57"/>
+      <c r="I2" s="57"/>
+      <c r="J2" s="57"/>
+      <c r="K2" s="57"/>
+      <c r="L2" s="57"/>
+      <c r="M2" s="57"/>
+      <c r="N2" s="57"/>
+      <c r="O2" s="57"/>
+      <c r="P2" s="58"/>
     </row>
     <row r="3" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B3" s="61"/>
-      <c r="C3" s="62"/>
-      <c r="D3" s="62"/>
-      <c r="E3" s="62"/>
-      <c r="F3" s="62"/>
-      <c r="G3" s="62"/>
-      <c r="H3" s="62"/>
-      <c r="I3" s="62"/>
-      <c r="J3" s="62"/>
-      <c r="K3" s="62"/>
-      <c r="L3" s="62"/>
-      <c r="M3" s="62"/>
-      <c r="N3" s="62"/>
-      <c r="O3" s="62"/>
-      <c r="P3" s="63"/>
+      <c r="B3" s="59"/>
+      <c r="C3" s="60"/>
+      <c r="D3" s="60"/>
+      <c r="E3" s="60"/>
+      <c r="F3" s="60"/>
+      <c r="G3" s="60"/>
+      <c r="H3" s="60"/>
+      <c r="I3" s="60"/>
+      <c r="J3" s="60"/>
+      <c r="K3" s="60"/>
+      <c r="L3" s="60"/>
+      <c r="M3" s="60"/>
+      <c r="N3" s="60"/>
+      <c r="O3" s="60"/>
+      <c r="P3" s="61"/>
       <c r="R3" s="12"/>
     </row>
     <row r="5" spans="1:19" x14ac:dyDescent="0.25">
@@ -2619,12 +2624,12 @@
       <c r="I5" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="K5" s="50" t="s">
+      <c r="K5" s="48" t="s">
         <v>8</v>
       </c>
-      <c r="L5" s="52"/>
-      <c r="M5" s="52"/>
-      <c r="N5" s="51"/>
+      <c r="L5" s="50"/>
+      <c r="M5" s="50"/>
+      <c r="N5" s="49"/>
       <c r="P5" s="4" t="s">
         <v>74</v>
       </c>
@@ -2706,27 +2711,27 @@
       </c>
     </row>
     <row r="9" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B9" s="53" t="s">
+      <c r="B9" s="51" t="s">
         <v>22</v>
       </c>
-      <c r="C9" s="53"/>
+      <c r="C9" s="51"/>
       <c r="E9" s="9" t="s">
         <v>67</v>
       </c>
     </row>
     <row r="10" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B10" s="54">
+      <c r="B10" s="52">
         <f>_xlfn.CEILING.MATH(SUM(B7:G7,I7,K7:N7,P7),1,1)</f>
         <v>110</v>
       </c>
-      <c r="C10" s="54"/>
+      <c r="C10" s="52"/>
       <c r="E10" s="46">
         <v>4</v>
       </c>
     </row>
     <row r="11" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B11" s="54"/>
-      <c r="C11" s="54"/>
+      <c r="B11" s="52"/>
+      <c r="C11" s="52"/>
       <c r="E11" s="47"/>
     </row>
     <row r="12" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -2752,24 +2757,24 @@
     </row>
     <row r="13" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="14" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B14" s="58" t="s">
+      <c r="B14" s="56" t="s">
         <v>134</v>
       </c>
-      <c r="C14" s="59"/>
-      <c r="D14" s="59"/>
-      <c r="E14" s="59"/>
-      <c r="F14" s="59"/>
-      <c r="G14" s="59"/>
-      <c r="H14" s="60"/>
+      <c r="C14" s="57"/>
+      <c r="D14" s="57"/>
+      <c r="E14" s="57"/>
+      <c r="F14" s="57"/>
+      <c r="G14" s="57"/>
+      <c r="H14" s="58"/>
     </row>
     <row r="15" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B15" s="61"/>
-      <c r="C15" s="62"/>
-      <c r="D15" s="62"/>
-      <c r="E15" s="62"/>
-      <c r="F15" s="62"/>
-      <c r="G15" s="62"/>
-      <c r="H15" s="63"/>
+      <c r="B15" s="59"/>
+      <c r="C15" s="60"/>
+      <c r="D15" s="60"/>
+      <c r="E15" s="60"/>
+      <c r="F15" s="60"/>
+      <c r="G15" s="60"/>
+      <c r="H15" s="61"/>
     </row>
     <row r="17" spans="1:19" x14ac:dyDescent="0.25">
       <c r="B17" s="39" t="s">
@@ -2782,10 +2787,10 @@
       </c>
       <c r="G17" s="39"/>
       <c r="H17" s="39"/>
-      <c r="J17" s="53" t="s">
+      <c r="J17" s="51" t="s">
         <v>22</v>
       </c>
-      <c r="K17" s="53"/>
+      <c r="K17" s="51"/>
       <c r="M17" s="9" t="s">
         <v>67</v>
       </c>
@@ -2809,12 +2814,12 @@
       <c r="H18" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="J18" s="54">
+      <c r="J18" s="52">
         <f>SUM(B19:D19,F19:H19)</f>
         <v>93</v>
       </c>
-      <c r="K18" s="54"/>
-      <c r="M18" s="55">
+      <c r="K18" s="52"/>
+      <c r="M18" s="53">
         <v>5</v>
       </c>
     </row>
@@ -2837,9 +2842,9 @@
       <c r="H19" s="2">
         <v>4</v>
       </c>
-      <c r="J19" s="54"/>
-      <c r="K19" s="54"/>
-      <c r="M19" s="55"/>
+      <c r="J19" s="52"/>
+      <c r="K19" s="52"/>
+      <c r="M19" s="53"/>
     </row>
     <row r="21" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A21" s="6"/>
@@ -2864,41 +2869,41 @@
     </row>
     <row r="22" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="23" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B23" s="58" t="s">
+      <c r="B23" s="56" t="s">
         <v>135</v>
       </c>
-      <c r="C23" s="59"/>
-      <c r="D23" s="59"/>
-      <c r="E23" s="59"/>
-      <c r="F23" s="59"/>
-      <c r="G23" s="59"/>
-      <c r="H23" s="59"/>
-      <c r="I23" s="59"/>
-      <c r="J23" s="59"/>
-      <c r="K23" s="60"/>
+      <c r="C23" s="57"/>
+      <c r="D23" s="57"/>
+      <c r="E23" s="57"/>
+      <c r="F23" s="57"/>
+      <c r="G23" s="57"/>
+      <c r="H23" s="57"/>
+      <c r="I23" s="57"/>
+      <c r="J23" s="57"/>
+      <c r="K23" s="58"/>
     </row>
     <row r="24" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B24" s="61"/>
-      <c r="C24" s="62"/>
-      <c r="D24" s="62"/>
-      <c r="E24" s="62"/>
-      <c r="F24" s="62"/>
-      <c r="G24" s="62"/>
-      <c r="H24" s="62"/>
-      <c r="I24" s="62"/>
-      <c r="J24" s="62"/>
-      <c r="K24" s="63"/>
+      <c r="B24" s="59"/>
+      <c r="C24" s="60"/>
+      <c r="D24" s="60"/>
+      <c r="E24" s="60"/>
+      <c r="F24" s="60"/>
+      <c r="G24" s="60"/>
+      <c r="H24" s="60"/>
+      <c r="I24" s="60"/>
+      <c r="J24" s="60"/>
+      <c r="K24" s="61"/>
     </row>
     <row r="26" spans="1:19" x14ac:dyDescent="0.25">
       <c r="B26" s="39" t="s">
         <v>17</v>
       </c>
       <c r="C26" s="39"/>
-      <c r="E26" s="50" t="s">
+      <c r="E26" s="48" t="s">
         <v>21</v>
       </c>
-      <c r="F26" s="52"/>
-      <c r="G26" s="51"/>
+      <c r="F26" s="50"/>
+      <c r="G26" s="49"/>
       <c r="I26" s="39" t="s">
         <v>20</v>
       </c>
@@ -2938,12 +2943,12 @@
       <c r="K27" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="M27" s="64">
+      <c r="M27" s="62">
         <f>SUM(B28:C28,E28:G28,I28:K28)</f>
         <v>36</v>
       </c>
       <c r="N27" s="7"/>
-      <c r="O27" s="55">
+      <c r="O27" s="53">
         <v>4</v>
       </c>
       <c r="P27" s="8"/>
@@ -2973,9 +2978,9 @@
       <c r="K28" s="2">
         <v>3.2</v>
       </c>
-      <c r="M28" s="64"/>
+      <c r="M28" s="62"/>
       <c r="N28" s="7"/>
-      <c r="O28" s="55"/>
+      <c r="O28" s="53"/>
       <c r="P28" s="8"/>
     </row>
     <row r="30" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -3001,26 +3006,26 @@
     </row>
     <row r="31" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="32" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B32" s="58" t="s">
+      <c r="B32" s="56" t="s">
         <v>136</v>
       </c>
-      <c r="C32" s="59"/>
-      <c r="D32" s="59"/>
-      <c r="E32" s="59"/>
-      <c r="F32" s="59"/>
-      <c r="G32" s="59"/>
-      <c r="H32" s="59"/>
-      <c r="I32" s="60"/>
+      <c r="C32" s="57"/>
+      <c r="D32" s="57"/>
+      <c r="E32" s="57"/>
+      <c r="F32" s="57"/>
+      <c r="G32" s="57"/>
+      <c r="H32" s="57"/>
+      <c r="I32" s="58"/>
     </row>
     <row r="33" spans="2:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B33" s="61"/>
-      <c r="C33" s="62"/>
-      <c r="D33" s="62"/>
-      <c r="E33" s="62"/>
-      <c r="F33" s="62"/>
-      <c r="G33" s="62"/>
-      <c r="H33" s="62"/>
-      <c r="I33" s="63"/>
+      <c r="B33" s="59"/>
+      <c r="C33" s="60"/>
+      <c r="D33" s="60"/>
+      <c r="E33" s="60"/>
+      <c r="F33" s="60"/>
+      <c r="G33" s="60"/>
+      <c r="H33" s="60"/>
+      <c r="I33" s="61"/>
     </row>
     <row r="35" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B35" s="39" t="s">
@@ -3090,14 +3095,14 @@
       <c r="O37" s="7"/>
     </row>
     <row r="40" spans="2:15" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B40" s="56" t="s">
+      <c r="B40" s="54" t="s">
         <v>35</v>
       </c>
-      <c r="C40" s="57"/>
-      <c r="F40" s="54" t="s">
+      <c r="C40" s="55"/>
+      <c r="F40" s="52" t="s">
         <v>36</v>
       </c>
-      <c r="G40" s="54"/>
+      <c r="G40" s="52"/>
       <c r="I40" s="9" t="s">
         <v>22</v>
       </c>
@@ -3153,7 +3158,7 @@
       <c r="G43" s="2">
         <v>0.44</v>
       </c>
-      <c r="I43" s="53" t="s">
+      <c r="I43" s="51" t="s">
         <v>67</v>
       </c>
     </row>
@@ -3170,7 +3175,7 @@
       <c r="G44" s="2">
         <v>1</v>
       </c>
-      <c r="I44" s="53"/>
+      <c r="I44" s="51"/>
     </row>
     <row r="45" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B45" s="2" t="s">
@@ -3314,44 +3319,44 @@
     </row>
     <row r="57" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="58" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B58" s="58" t="s">
+      <c r="B58" s="56" t="s">
         <v>137</v>
       </c>
-      <c r="C58" s="59"/>
-      <c r="D58" s="59"/>
-      <c r="E58" s="59"/>
-      <c r="F58" s="59"/>
-      <c r="G58" s="59"/>
-      <c r="H58" s="59"/>
-      <c r="I58" s="59"/>
-      <c r="J58" s="59"/>
-      <c r="K58" s="59"/>
-      <c r="L58" s="59"/>
-      <c r="M58" s="59"/>
-      <c r="N58" s="59"/>
-      <c r="O58" s="59"/>
-      <c r="P58" s="59"/>
-      <c r="Q58" s="59"/>
-      <c r="R58" s="60"/>
+      <c r="C58" s="57"/>
+      <c r="D58" s="57"/>
+      <c r="E58" s="57"/>
+      <c r="F58" s="57"/>
+      <c r="G58" s="57"/>
+      <c r="H58" s="57"/>
+      <c r="I58" s="57"/>
+      <c r="J58" s="57"/>
+      <c r="K58" s="57"/>
+      <c r="L58" s="57"/>
+      <c r="M58" s="57"/>
+      <c r="N58" s="57"/>
+      <c r="O58" s="57"/>
+      <c r="P58" s="57"/>
+      <c r="Q58" s="57"/>
+      <c r="R58" s="58"/>
     </row>
     <row r="59" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B59" s="61"/>
-      <c r="C59" s="62"/>
-      <c r="D59" s="62"/>
-      <c r="E59" s="62"/>
-      <c r="F59" s="62"/>
-      <c r="G59" s="62"/>
-      <c r="H59" s="62"/>
-      <c r="I59" s="62"/>
-      <c r="J59" s="62"/>
-      <c r="K59" s="62"/>
-      <c r="L59" s="62"/>
-      <c r="M59" s="62"/>
-      <c r="N59" s="62"/>
-      <c r="O59" s="62"/>
-      <c r="P59" s="62"/>
-      <c r="Q59" s="62"/>
-      <c r="R59" s="63"/>
+      <c r="B59" s="59"/>
+      <c r="C59" s="60"/>
+      <c r="D59" s="60"/>
+      <c r="E59" s="60"/>
+      <c r="F59" s="60"/>
+      <c r="G59" s="60"/>
+      <c r="H59" s="60"/>
+      <c r="I59" s="60"/>
+      <c r="J59" s="60"/>
+      <c r="K59" s="60"/>
+      <c r="L59" s="60"/>
+      <c r="M59" s="60"/>
+      <c r="N59" s="60"/>
+      <c r="O59" s="60"/>
+      <c r="P59" s="60"/>
+      <c r="Q59" s="60"/>
+      <c r="R59" s="61"/>
     </row>
     <row r="61" spans="1:19" x14ac:dyDescent="0.25">
       <c r="B61" s="39" t="s">
@@ -3471,28 +3476,28 @@
       </c>
     </row>
     <row r="66" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B66" s="53" t="s">
+      <c r="B66" s="51" t="s">
         <v>22</v>
       </c>
-      <c r="C66" s="53"/>
+      <c r="C66" s="51"/>
       <c r="E66" s="9" t="s">
         <v>67</v>
       </c>
     </row>
     <row r="67" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B67" s="54">
+      <c r="B67" s="52">
         <f xml:space="preserve"> SUM(B63:K63,M63:O63,Q63:R63)</f>
         <v>85.5</v>
       </c>
-      <c r="C67" s="54"/>
-      <c r="E67" s="55">
+      <c r="C67" s="52"/>
+      <c r="E67" s="53">
         <v>4.5</v>
       </c>
     </row>
     <row r="68" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B68" s="54"/>
-      <c r="C68" s="54"/>
-      <c r="E68" s="55"/>
+      <c r="B68" s="52"/>
+      <c r="C68" s="52"/>
+      <c r="E68" s="53"/>
     </row>
     <row r="70" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A70" s="6"/>
@@ -3517,26 +3522,26 @@
     </row>
     <row r="71" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="72" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B72" s="58" t="s">
+      <c r="B72" s="56" t="s">
         <v>138</v>
       </c>
-      <c r="C72" s="59"/>
-      <c r="D72" s="59"/>
-      <c r="E72" s="59"/>
-      <c r="F72" s="59"/>
-      <c r="G72" s="59"/>
-      <c r="H72" s="59"/>
-      <c r="I72" s="60"/>
+      <c r="C72" s="57"/>
+      <c r="D72" s="57"/>
+      <c r="E72" s="57"/>
+      <c r="F72" s="57"/>
+      <c r="G72" s="57"/>
+      <c r="H72" s="57"/>
+      <c r="I72" s="58"/>
     </row>
     <row r="73" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B73" s="61"/>
-      <c r="C73" s="62"/>
-      <c r="D73" s="62"/>
-      <c r="E73" s="62"/>
-      <c r="F73" s="62"/>
-      <c r="G73" s="62"/>
-      <c r="H73" s="62"/>
-      <c r="I73" s="63"/>
+      <c r="B73" s="59"/>
+      <c r="C73" s="60"/>
+      <c r="D73" s="60"/>
+      <c r="E73" s="60"/>
+      <c r="F73" s="60"/>
+      <c r="G73" s="60"/>
+      <c r="H73" s="60"/>
+      <c r="I73" s="61"/>
     </row>
     <row r="75" spans="1:19" x14ac:dyDescent="0.25">
       <c r="B75" s="4" t="s">
@@ -3563,10 +3568,10 @@
       <c r="I75" s="4" t="s">
         <v>146</v>
       </c>
-      <c r="K75" s="53" t="s">
+      <c r="K75" s="51" t="s">
         <v>22</v>
       </c>
-      <c r="L75" s="53"/>
+      <c r="L75" s="51"/>
       <c r="N75" s="9" t="s">
         <v>67</v>
       </c>
@@ -3596,11 +3601,11 @@
       <c r="I76" s="2">
         <v>5</v>
       </c>
-      <c r="K76" s="54">
+      <c r="K76" s="52">
         <f>SUM(B76:I76)</f>
         <v>96</v>
       </c>
-      <c r="L76" s="54"/>
+      <c r="L76" s="52"/>
       <c r="N76" s="13">
         <v>5</v>
       </c>
@@ -4170,21 +4175,21 @@
   <sheetData>
     <row r="1" spans="2:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="2" spans="2:12" ht="23.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B2" s="65" t="s">
+      <c r="B2" s="63" t="s">
         <v>204</v>
       </c>
-      <c r="C2" s="66"/>
-      <c r="D2" s="67"/>
-      <c r="F2" s="65" t="s">
+      <c r="C2" s="64"/>
+      <c r="D2" s="65"/>
+      <c r="F2" s="63" t="s">
         <v>205</v>
       </c>
-      <c r="G2" s="66"/>
-      <c r="H2" s="67"/>
-      <c r="J2" s="65" t="s">
+      <c r="G2" s="64"/>
+      <c r="H2" s="65"/>
+      <c r="J2" s="63" t="s">
         <v>206</v>
       </c>
-      <c r="K2" s="66"/>
-      <c r="L2" s="67"/>
+      <c r="K2" s="64"/>
+      <c r="L2" s="65"/>
     </row>
     <row r="3" spans="2:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B3" s="34" t="s">
@@ -4359,26 +4364,26 @@
     </row>
     <row r="10" spans="2:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="11" spans="2:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B11" s="68" t="s">
+      <c r="B11" s="66" t="s">
         <v>198</v>
       </c>
-      <c r="C11" s="69"/>
+      <c r="C11" s="67"/>
       <c r="D11" s="33">
         <f>(D4*C4+D5*C5+D6*C6+D7*C7+D8*C8+D9*C9)/30</f>
         <v>4.4333333333333336</v>
       </c>
-      <c r="F11" s="68" t="s">
+      <c r="F11" s="66" t="s">
         <v>198</v>
       </c>
-      <c r="G11" s="69"/>
+      <c r="G11" s="67"/>
       <c r="H11" s="33">
         <f>(H4*G4+H5*G5+H6*G6+H7*G7+H8*G8)/30</f>
         <v>0</v>
       </c>
-      <c r="J11" s="68" t="s">
+      <c r="J11" s="66" t="s">
         <v>198</v>
       </c>
-      <c r="K11" s="69"/>
+      <c r="K11" s="67"/>
       <c r="L11" s="33">
         <f>(L4*K4+L5*K5+L6*K6+L7*K7+L8*K8)/30</f>
         <v>0</v>

</xml_diff>

<commit_message>
New points - POTEC lab8
</commit_message>
<xml_diff>
--- a/IoT-points-schedule.xlsx
+++ b/IoT-points-schedule.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\dodo\Desktop\IoT-studies\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A34F131B-8E13-4E22-8B4D-9D282295A033}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{34DC516C-F8E4-45B0-9B1F-5B593EB407A1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="25440" windowHeight="15390" xr2:uid="{F85F5544-1FE8-4920-A5D4-192A98B113BD}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="334" uniqueCount="211">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="334" uniqueCount="212">
   <si>
     <t>1. Krypto</t>
   </si>
@@ -672,6 +672,9 @@
   </si>
   <si>
     <t>LAB4 (Magnetyzm)</t>
+  </si>
+  <si>
+    <t>Laboratoria [ocena]</t>
   </si>
 </sst>
 </file>
@@ -1152,56 +1155,56 @@
     <xf numFmtId="0" fontId="6" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1664,23 +1667,23 @@
       <c r="R3" s="12"/>
     </row>
     <row r="5" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B5" s="48" t="s">
+      <c r="B5" s="46" t="s">
         <v>83</v>
       </c>
-      <c r="C5" s="50"/>
-      <c r="D5" s="50"/>
-      <c r="E5" s="50"/>
-      <c r="F5" s="49"/>
-      <c r="H5" s="48" t="s">
+      <c r="C5" s="47"/>
+      <c r="D5" s="47"/>
+      <c r="E5" s="47"/>
+      <c r="F5" s="48"/>
+      <c r="H5" s="46" t="s">
         <v>82</v>
       </c>
-      <c r="I5" s="49"/>
-      <c r="K5" s="48" t="s">
+      <c r="I5" s="48"/>
+      <c r="K5" s="46" t="s">
         <v>8</v>
       </c>
-      <c r="L5" s="50"/>
-      <c r="M5" s="50"/>
-      <c r="N5" s="49"/>
+      <c r="L5" s="47"/>
+      <c r="M5" s="47"/>
+      <c r="N5" s="48"/>
       <c r="P5" s="4" t="s">
         <v>74</v>
       </c>
@@ -1740,37 +1743,37 @@
       <c r="P7" s="2"/>
     </row>
     <row r="9" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B9" s="51" t="s">
+      <c r="B9" s="49" t="s">
         <v>22</v>
       </c>
-      <c r="C9" s="51"/>
+      <c r="C9" s="49"/>
       <c r="E9" s="9" t="s">
         <v>67</v>
       </c>
-      <c r="G9" s="51" t="s">
+      <c r="G9" s="49" t="s">
         <v>87</v>
       </c>
-      <c r="H9" s="51"/>
+      <c r="H9" s="49"/>
     </row>
     <row r="10" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B10" s="52">
+      <c r="B10" s="50">
         <f>SUM(B7:F7,H7:I7,K7:N7,P7)</f>
         <v>9.6999999999999993</v>
       </c>
-      <c r="C10" s="52"/>
-      <c r="E10" s="46"/>
-      <c r="G10" s="52">
+      <c r="C10" s="50"/>
+      <c r="E10" s="54"/>
+      <c r="G10" s="50">
         <f>66-SUM(B7:F7,H7:I7,K7:N7,P7)</f>
         <v>56.3</v>
       </c>
-      <c r="H10" s="52"/>
+      <c r="H10" s="50"/>
     </row>
     <row r="11" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B11" s="52"/>
-      <c r="C11" s="52"/>
-      <c r="E11" s="47"/>
-      <c r="G11" s="52"/>
-      <c r="H11" s="52"/>
+      <c r="B11" s="50"/>
+      <c r="C11" s="50"/>
+      <c r="E11" s="55"/>
+      <c r="G11" s="50"/>
+      <c r="H11" s="50"/>
     </row>
     <row r="12" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A12" s="6"/>
@@ -1815,26 +1818,26 @@
       <c r="H15" s="45"/>
     </row>
     <row r="17" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B17" s="39" t="s">
+      <c r="B17" s="53" t="s">
         <v>91</v>
       </c>
-      <c r="C17" s="39"/>
-      <c r="D17" s="39"/>
-      <c r="E17" s="39"/>
-      <c r="F17" s="39"/>
-      <c r="H17" s="48" t="s">
+      <c r="C17" s="53"/>
+      <c r="D17" s="53"/>
+      <c r="E17" s="53"/>
+      <c r="F17" s="53"/>
+      <c r="H17" s="46" t="s">
         <v>97</v>
       </c>
-      <c r="I17" s="50"/>
-      <c r="J17" s="49"/>
-      <c r="L17" s="51" t="s">
+      <c r="I17" s="47"/>
+      <c r="J17" s="48"/>
+      <c r="L17" s="49" t="s">
         <v>22</v>
       </c>
-      <c r="M17" s="51"/>
-      <c r="O17" s="51" t="s">
+      <c r="M17" s="49"/>
+      <c r="O17" s="49" t="s">
         <v>87</v>
       </c>
-      <c r="P17" s="51"/>
+      <c r="P17" s="49"/>
       <c r="R17" s="9" t="s">
         <v>67</v>
       </c>
@@ -1864,17 +1867,17 @@
       <c r="J18" s="3" t="s">
         <v>95</v>
       </c>
-      <c r="L18" s="52">
+      <c r="L18" s="50">
         <f>SUM(B19:F19,H19:J19)</f>
         <v>29.5</v>
       </c>
-      <c r="M18" s="52"/>
-      <c r="O18" s="52">
+      <c r="M18" s="50"/>
+      <c r="O18" s="50">
         <f>50-SUM(B19:F19,H19:J19)</f>
         <v>20.5</v>
       </c>
-      <c r="P18" s="52"/>
-      <c r="R18" s="53"/>
+      <c r="P18" s="50"/>
+      <c r="R18" s="39"/>
     </row>
     <row r="19" spans="1:19" x14ac:dyDescent="0.25">
       <c r="B19" s="2"/>
@@ -1889,11 +1892,11 @@
         <v>26.5</v>
       </c>
       <c r="J19" s="2"/>
-      <c r="L19" s="52"/>
-      <c r="M19" s="52"/>
-      <c r="O19" s="52"/>
-      <c r="P19" s="52"/>
-      <c r="R19" s="53"/>
+      <c r="L19" s="50"/>
+      <c r="M19" s="50"/>
+      <c r="O19" s="50"/>
+      <c r="P19" s="50"/>
+      <c r="R19" s="39"/>
     </row>
     <row r="21" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A21" s="6"/>
@@ -1931,10 +1934,10 @@
       <c r="J23" s="41"/>
       <c r="K23" s="41"/>
       <c r="L23" s="42"/>
-      <c r="N23" s="52" t="s">
+      <c r="N23" s="50" t="s">
         <v>132</v>
       </c>
-      <c r="O23" s="52"/>
+      <c r="O23" s="50"/>
     </row>
     <row r="24" spans="1:19" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B24" s="43"/>
@@ -1948,26 +1951,26 @@
       <c r="J24" s="44"/>
       <c r="K24" s="44"/>
       <c r="L24" s="45"/>
-      <c r="N24" s="52"/>
-      <c r="O24" s="52"/>
+      <c r="N24" s="50"/>
+      <c r="O24" s="50"/>
     </row>
     <row r="26" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B26" s="39" t="s">
+      <c r="B26" s="53" t="s">
         <v>129</v>
       </c>
-      <c r="C26" s="39"/>
-      <c r="D26" s="39"/>
-      <c r="F26" s="39" t="s">
-        <v>12</v>
-      </c>
-      <c r="G26" s="39"/>
-      <c r="H26" s="39"/>
-      <c r="I26" s="39"/>
+      <c r="C26" s="53"/>
+      <c r="D26" s="53"/>
+      <c r="F26" s="53" t="s">
+        <v>211</v>
+      </c>
+      <c r="G26" s="53"/>
+      <c r="H26" s="53"/>
+      <c r="I26" s="53"/>
       <c r="J26" s="7"/>
-      <c r="K26" s="48" t="s">
+      <c r="K26" s="46" t="s">
         <v>128</v>
       </c>
-      <c r="L26" s="49"/>
+      <c r="L26" s="48"/>
       <c r="N26" s="9" t="s">
         <v>67</v>
       </c>
@@ -2000,7 +2003,7 @@
       <c r="L27" s="2" t="s">
         <v>127</v>
       </c>
-      <c r="N27" s="46"/>
+      <c r="N27" s="54"/>
     </row>
     <row r="28" spans="1:19" x14ac:dyDescent="0.25">
       <c r="B28" s="2"/>
@@ -2016,7 +2019,7 @@
       <c r="I28" s="2"/>
       <c r="K28" s="2"/>
       <c r="L28" s="2"/>
-      <c r="N28" s="47"/>
+      <c r="N28" s="55"/>
     </row>
     <row r="30" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A30" s="6"/>
@@ -2063,17 +2066,17 @@
       <c r="I33" s="45"/>
     </row>
     <row r="35" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B35" s="39" t="s">
+      <c r="B35" s="53" t="s">
         <v>98</v>
       </c>
-      <c r="C35" s="39"/>
+      <c r="C35" s="53"/>
       <c r="D35" s="7"/>
-      <c r="E35" s="48" t="s">
+      <c r="E35" s="46" t="s">
         <v>147</v>
       </c>
-      <c r="F35" s="50"/>
-      <c r="G35" s="50"/>
-      <c r="H35" s="49"/>
+      <c r="F35" s="47"/>
+      <c r="G35" s="47"/>
+      <c r="H35" s="48"/>
     </row>
     <row r="36" spans="2:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B36" s="2" t="s">
@@ -2103,7 +2106,7 @@
       <c r="C37" s="2"/>
       <c r="E37" s="2">
         <f>C56</f>
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="F37" s="2">
         <f>G51</f>
@@ -2114,14 +2117,14 @@
       <c r="O37" s="7"/>
     </row>
     <row r="40" spans="2:15" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B40" s="54" t="s">
+      <c r="B40" s="51" t="s">
         <v>126</v>
       </c>
-      <c r="C40" s="55"/>
-      <c r="F40" s="52" t="s">
+      <c r="C40" s="52"/>
+      <c r="F40" s="50" t="s">
         <v>102</v>
       </c>
-      <c r="G40" s="52"/>
+      <c r="G40" s="50"/>
       <c r="I40" s="9" t="s">
         <v>22</v>
       </c>
@@ -2143,7 +2146,7 @@
       </c>
       <c r="I41" s="2">
         <f>SUM(B37:C37,E37:H37)</f>
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="J41" s="7"/>
       <c r="L41" s="7"/>
@@ -2171,7 +2174,7 @@
         <v>119</v>
       </c>
       <c r="G43" s="2"/>
-      <c r="I43" s="51" t="s">
+      <c r="I43" s="49" t="s">
         <v>67</v>
       </c>
     </row>
@@ -2186,7 +2189,7 @@
         <v>120</v>
       </c>
       <c r="G44" s="2"/>
-      <c r="I44" s="51"/>
+      <c r="I44" s="49"/>
     </row>
     <row r="45" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B45" s="2" t="s">
@@ -2228,14 +2231,16 @@
       <c r="B48" s="2" t="s">
         <v>110</v>
       </c>
-      <c r="C48" s="2"/>
+      <c r="C48" s="2">
+        <v>2</v>
+      </c>
       <c r="F48" s="2" t="s">
         <v>124</v>
       </c>
       <c r="G48" s="2"/>
       <c r="I48" s="2">
         <f>50-SUM(B37:C37,E37:H37)</f>
-        <v>11</v>
+        <v>9</v>
       </c>
     </row>
     <row r="49" spans="1:19" x14ac:dyDescent="0.25">
@@ -2291,7 +2296,7 @@
       </c>
       <c r="C56" s="2">
         <f>SUM(C41:C54)</f>
-        <v>13</v>
+        <v>15</v>
       </c>
     </row>
     <row r="58" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -2359,28 +2364,28 @@
       <c r="S61" s="45"/>
     </row>
     <row r="63" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B63" s="39" t="s">
+      <c r="B63" s="53" t="s">
         <v>63</v>
       </c>
-      <c r="C63" s="39"/>
-      <c r="D63" s="39"/>
-      <c r="E63" s="39"/>
-      <c r="F63" s="39"/>
-      <c r="G63" s="39"/>
-      <c r="H63" s="39"/>
-      <c r="I63" s="39"/>
-      <c r="J63" s="39"/>
-      <c r="K63" s="39"/>
-      <c r="M63" s="39" t="s">
+      <c r="C63" s="53"/>
+      <c r="D63" s="53"/>
+      <c r="E63" s="53"/>
+      <c r="F63" s="53"/>
+      <c r="G63" s="53"/>
+      <c r="H63" s="53"/>
+      <c r="I63" s="53"/>
+      <c r="J63" s="53"/>
+      <c r="K63" s="53"/>
+      <c r="M63" s="53" t="s">
         <v>90</v>
       </c>
-      <c r="N63" s="39"/>
-      <c r="O63" s="39"/>
-      <c r="P63" s="39"/>
-      <c r="R63" s="39" t="s">
+      <c r="N63" s="53"/>
+      <c r="O63" s="53"/>
+      <c r="P63" s="53"/>
+      <c r="R63" s="53" t="s">
         <v>64</v>
       </c>
-      <c r="S63" s="39"/>
+      <c r="S63" s="53"/>
     </row>
     <row r="64" spans="1:19" x14ac:dyDescent="0.25">
       <c r="B64" s="2" t="s">
@@ -2469,40 +2474,62 @@
       <c r="S65" s="2"/>
     </row>
     <row r="68" spans="2:19" x14ac:dyDescent="0.25">
-      <c r="B68" s="51" t="s">
+      <c r="B68" s="49" t="s">
         <v>22</v>
       </c>
-      <c r="C68" s="51"/>
+      <c r="C68" s="49"/>
       <c r="E68" s="9" t="s">
         <v>67</v>
       </c>
-      <c r="G68" s="51" t="s">
+      <c r="G68" s="49" t="s">
         <v>87</v>
       </c>
-      <c r="H68" s="51"/>
+      <c r="H68" s="49"/>
     </row>
     <row r="69" spans="2:19" x14ac:dyDescent="0.25">
-      <c r="B69" s="52">
+      <c r="B69" s="50">
         <f>SUM(B65:K65,M65:P65,R65:S65)</f>
         <v>17</v>
       </c>
-      <c r="C69" s="52"/>
-      <c r="E69" s="53"/>
-      <c r="G69" s="52">
+      <c r="C69" s="50"/>
+      <c r="E69" s="39"/>
+      <c r="G69" s="50">
         <f>50-SUM(B65:K65,M65:P65,R65:S65)</f>
         <v>33</v>
       </c>
-      <c r="H69" s="52"/>
+      <c r="H69" s="50"/>
     </row>
     <row r="70" spans="2:19" x14ac:dyDescent="0.25">
-      <c r="B70" s="52"/>
-      <c r="C70" s="52"/>
-      <c r="E70" s="53"/>
-      <c r="G70" s="52"/>
-      <c r="H70" s="52"/>
+      <c r="B70" s="50"/>
+      <c r="C70" s="50"/>
+      <c r="E70" s="39"/>
+      <c r="G70" s="50"/>
+      <c r="H70" s="50"/>
     </row>
   </sheetData>
   <mergeCells count="38">
+    <mergeCell ref="R63:S63"/>
+    <mergeCell ref="B32:I33"/>
+    <mergeCell ref="B63:K63"/>
+    <mergeCell ref="B60:S61"/>
+    <mergeCell ref="M63:P63"/>
+    <mergeCell ref="N27:N28"/>
+    <mergeCell ref="F26:I26"/>
+    <mergeCell ref="K26:L26"/>
+    <mergeCell ref="B23:L24"/>
+    <mergeCell ref="B26:D26"/>
+    <mergeCell ref="B17:F17"/>
+    <mergeCell ref="H17:J17"/>
+    <mergeCell ref="O17:P17"/>
+    <mergeCell ref="B9:C9"/>
+    <mergeCell ref="B10:C11"/>
+    <mergeCell ref="L17:M17"/>
+    <mergeCell ref="E10:E11"/>
+    <mergeCell ref="E69:E70"/>
+    <mergeCell ref="B68:C68"/>
+    <mergeCell ref="B69:C70"/>
+    <mergeCell ref="G68:H68"/>
+    <mergeCell ref="G69:H70"/>
     <mergeCell ref="R18:R19"/>
     <mergeCell ref="B14:H15"/>
     <mergeCell ref="K5:N5"/>
@@ -2519,28 +2546,6 @@
     <mergeCell ref="E35:H35"/>
     <mergeCell ref="G9:H9"/>
     <mergeCell ref="G10:H11"/>
-    <mergeCell ref="E69:E70"/>
-    <mergeCell ref="B68:C68"/>
-    <mergeCell ref="B69:C70"/>
-    <mergeCell ref="G68:H68"/>
-    <mergeCell ref="G69:H70"/>
-    <mergeCell ref="B17:F17"/>
-    <mergeCell ref="H17:J17"/>
-    <mergeCell ref="O17:P17"/>
-    <mergeCell ref="B9:C9"/>
-    <mergeCell ref="B10:C11"/>
-    <mergeCell ref="L17:M17"/>
-    <mergeCell ref="E10:E11"/>
-    <mergeCell ref="N27:N28"/>
-    <mergeCell ref="F26:I26"/>
-    <mergeCell ref="K26:L26"/>
-    <mergeCell ref="B23:L24"/>
-    <mergeCell ref="B26:D26"/>
-    <mergeCell ref="R63:S63"/>
-    <mergeCell ref="B32:I33"/>
-    <mergeCell ref="B63:K63"/>
-    <mergeCell ref="B60:S61"/>
-    <mergeCell ref="M63:P63"/>
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2613,23 +2618,23 @@
       <c r="R3" s="12"/>
     </row>
     <row r="5" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B5" s="39" t="s">
+      <c r="B5" s="53" t="s">
         <v>18</v>
       </c>
-      <c r="C5" s="39"/>
-      <c r="D5" s="39"/>
-      <c r="E5" s="39"/>
-      <c r="F5" s="39"/>
-      <c r="G5" s="39"/>
+      <c r="C5" s="53"/>
+      <c r="D5" s="53"/>
+      <c r="E5" s="53"/>
+      <c r="F5" s="53"/>
+      <c r="G5" s="53"/>
       <c r="I5" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="K5" s="48" t="s">
+      <c r="K5" s="46" t="s">
         <v>8</v>
       </c>
-      <c r="L5" s="50"/>
-      <c r="M5" s="50"/>
-      <c r="N5" s="49"/>
+      <c r="L5" s="47"/>
+      <c r="M5" s="47"/>
+      <c r="N5" s="48"/>
       <c r="P5" s="4" t="s">
         <v>74</v>
       </c>
@@ -2711,28 +2716,28 @@
       </c>
     </row>
     <row r="9" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B9" s="51" t="s">
+      <c r="B9" s="49" t="s">
         <v>22</v>
       </c>
-      <c r="C9" s="51"/>
+      <c r="C9" s="49"/>
       <c r="E9" s="9" t="s">
         <v>67</v>
       </c>
     </row>
     <row r="10" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B10" s="52">
+      <c r="B10" s="50">
         <f>_xlfn.CEILING.MATH(SUM(B7:G7,I7,K7:N7,P7),1,1)</f>
         <v>110</v>
       </c>
-      <c r="C10" s="52"/>
-      <c r="E10" s="46">
+      <c r="C10" s="50"/>
+      <c r="E10" s="54">
         <v>4</v>
       </c>
     </row>
     <row r="11" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B11" s="52"/>
-      <c r="C11" s="52"/>
-      <c r="E11" s="47"/>
+      <c r="B11" s="50"/>
+      <c r="C11" s="50"/>
+      <c r="E11" s="55"/>
     </row>
     <row r="12" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A12" s="6"/>
@@ -2777,20 +2782,20 @@
       <c r="H15" s="61"/>
     </row>
     <row r="17" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B17" s="39" t="s">
+      <c r="B17" s="53" t="s">
         <v>12</v>
       </c>
-      <c r="C17" s="39"/>
-      <c r="D17" s="39"/>
-      <c r="F17" s="39" t="s">
+      <c r="C17" s="53"/>
+      <c r="D17" s="53"/>
+      <c r="F17" s="53" t="s">
         <v>8</v>
       </c>
-      <c r="G17" s="39"/>
-      <c r="H17" s="39"/>
-      <c r="J17" s="51" t="s">
+      <c r="G17" s="53"/>
+      <c r="H17" s="53"/>
+      <c r="J17" s="49" t="s">
         <v>22</v>
       </c>
-      <c r="K17" s="51"/>
+      <c r="K17" s="49"/>
       <c r="M17" s="9" t="s">
         <v>67</v>
       </c>
@@ -2814,12 +2819,12 @@
       <c r="H18" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="J18" s="52">
+      <c r="J18" s="50">
         <f>SUM(B19:D19,F19:H19)</f>
         <v>93</v>
       </c>
-      <c r="K18" s="52"/>
-      <c r="M18" s="53">
+      <c r="K18" s="50"/>
+      <c r="M18" s="39">
         <v>5</v>
       </c>
     </row>
@@ -2842,9 +2847,9 @@
       <c r="H19" s="2">
         <v>4</v>
       </c>
-      <c r="J19" s="52"/>
-      <c r="K19" s="52"/>
-      <c r="M19" s="53"/>
+      <c r="J19" s="50"/>
+      <c r="K19" s="50"/>
+      <c r="M19" s="39"/>
     </row>
     <row r="21" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A21" s="6"/>
@@ -2895,20 +2900,20 @@
       <c r="K24" s="61"/>
     </row>
     <row r="26" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B26" s="39" t="s">
+      <c r="B26" s="53" t="s">
         <v>17</v>
       </c>
-      <c r="C26" s="39"/>
-      <c r="E26" s="48" t="s">
+      <c r="C26" s="53"/>
+      <c r="E26" s="46" t="s">
         <v>21</v>
       </c>
-      <c r="F26" s="50"/>
-      <c r="G26" s="49"/>
-      <c r="I26" s="39" t="s">
+      <c r="F26" s="47"/>
+      <c r="G26" s="48"/>
+      <c r="I26" s="53" t="s">
         <v>20</v>
       </c>
-      <c r="J26" s="39"/>
-      <c r="K26" s="39"/>
+      <c r="J26" s="53"/>
+      <c r="K26" s="53"/>
       <c r="M26" s="10" t="s">
         <v>22</v>
       </c>
@@ -2948,7 +2953,7 @@
         <v>36</v>
       </c>
       <c r="N27" s="7"/>
-      <c r="O27" s="53">
+      <c r="O27" s="39">
         <v>4</v>
       </c>
       <c r="P27" s="8"/>
@@ -2980,7 +2985,7 @@
       </c>
       <c r="M28" s="62"/>
       <c r="N28" s="7"/>
-      <c r="O28" s="53"/>
+      <c r="O28" s="39"/>
       <c r="P28" s="8"/>
     </row>
     <row r="30" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -3028,17 +3033,17 @@
       <c r="I33" s="61"/>
     </row>
     <row r="35" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B35" s="39" t="s">
+      <c r="B35" s="53" t="s">
         <v>31</v>
       </c>
-      <c r="C35" s="39"/>
-      <c r="D35" s="39"/>
-      <c r="F35" s="39" t="s">
+      <c r="C35" s="53"/>
+      <c r="D35" s="53"/>
+      <c r="F35" s="53" t="s">
         <v>12</v>
       </c>
-      <c r="G35" s="39"/>
-      <c r="H35" s="39"/>
-      <c r="I35" s="39"/>
+      <c r="G35" s="53"/>
+      <c r="H35" s="53"/>
+      <c r="I35" s="53"/>
       <c r="N35" s="7"/>
       <c r="O35" s="7"/>
     </row>
@@ -3095,14 +3100,14 @@
       <c r="O37" s="7"/>
     </row>
     <row r="40" spans="2:15" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B40" s="54" t="s">
+      <c r="B40" s="51" t="s">
         <v>35</v>
       </c>
-      <c r="C40" s="55"/>
-      <c r="F40" s="52" t="s">
+      <c r="C40" s="52"/>
+      <c r="F40" s="50" t="s">
         <v>36</v>
       </c>
-      <c r="G40" s="52"/>
+      <c r="G40" s="50"/>
       <c r="I40" s="9" t="s">
         <v>22</v>
       </c>
@@ -3158,7 +3163,7 @@
       <c r="G43" s="2">
         <v>0.44</v>
       </c>
-      <c r="I43" s="51" t="s">
+      <c r="I43" s="49" t="s">
         <v>67</v>
       </c>
     </row>
@@ -3175,7 +3180,7 @@
       <c r="G44" s="2">
         <v>1</v>
       </c>
-      <c r="I44" s="51"/>
+      <c r="I44" s="49"/>
     </row>
     <row r="45" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B45" s="2" t="s">
@@ -3359,27 +3364,27 @@
       <c r="R59" s="61"/>
     </row>
     <row r="61" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B61" s="39" t="s">
+      <c r="B61" s="53" t="s">
         <v>63</v>
       </c>
-      <c r="C61" s="39"/>
-      <c r="D61" s="39"/>
-      <c r="E61" s="39"/>
-      <c r="F61" s="39"/>
-      <c r="G61" s="39"/>
-      <c r="H61" s="39"/>
-      <c r="I61" s="39"/>
-      <c r="J61" s="39"/>
-      <c r="K61" s="39"/>
-      <c r="M61" s="39" t="s">
+      <c r="C61" s="53"/>
+      <c r="D61" s="53"/>
+      <c r="E61" s="53"/>
+      <c r="F61" s="53"/>
+      <c r="G61" s="53"/>
+      <c r="H61" s="53"/>
+      <c r="I61" s="53"/>
+      <c r="J61" s="53"/>
+      <c r="K61" s="53"/>
+      <c r="M61" s="53" t="s">
         <v>68</v>
       </c>
-      <c r="N61" s="39"/>
-      <c r="O61" s="39"/>
-      <c r="Q61" s="39" t="s">
+      <c r="N61" s="53"/>
+      <c r="O61" s="53"/>
+      <c r="Q61" s="53" t="s">
         <v>64</v>
       </c>
-      <c r="R61" s="39"/>
+      <c r="R61" s="53"/>
     </row>
     <row r="62" spans="1:19" x14ac:dyDescent="0.25">
       <c r="B62" s="2" t="s">
@@ -3476,28 +3481,28 @@
       </c>
     </row>
     <row r="66" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B66" s="51" t="s">
+      <c r="B66" s="49" t="s">
         <v>22</v>
       </c>
-      <c r="C66" s="51"/>
+      <c r="C66" s="49"/>
       <c r="E66" s="9" t="s">
         <v>67</v>
       </c>
     </row>
     <row r="67" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B67" s="52">
+      <c r="B67" s="50">
         <f xml:space="preserve"> SUM(B63:K63,M63:O63,Q63:R63)</f>
         <v>85.5</v>
       </c>
-      <c r="C67" s="52"/>
-      <c r="E67" s="53">
+      <c r="C67" s="50"/>
+      <c r="E67" s="39">
         <v>4.5</v>
       </c>
     </row>
     <row r="68" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B68" s="52"/>
-      <c r="C68" s="52"/>
-      <c r="E68" s="53"/>
+      <c r="B68" s="50"/>
+      <c r="C68" s="50"/>
+      <c r="E68" s="39"/>
     </row>
     <row r="70" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A70" s="6"/>
@@ -3568,10 +3573,10 @@
       <c r="I75" s="4" t="s">
         <v>146</v>
       </c>
-      <c r="K75" s="51" t="s">
+      <c r="K75" s="49" t="s">
         <v>22</v>
       </c>
-      <c r="L75" s="51"/>
+      <c r="L75" s="49"/>
       <c r="N75" s="9" t="s">
         <v>67</v>
       </c>
@@ -3601,11 +3606,11 @@
       <c r="I76" s="2">
         <v>5</v>
       </c>
-      <c r="K76" s="52">
+      <c r="K76" s="50">
         <f>SUM(B76:I76)</f>
         <v>96</v>
       </c>
-      <c r="L76" s="52"/>
+      <c r="L76" s="50"/>
       <c r="N76" s="13">
         <v>5</v>
       </c>
@@ -3633,20 +3638,16 @@
     </row>
   </sheetData>
   <mergeCells count="34">
-    <mergeCell ref="B2:P3"/>
-    <mergeCell ref="B5:G5"/>
-    <mergeCell ref="K5:N5"/>
-    <mergeCell ref="B9:C9"/>
-    <mergeCell ref="B10:C11"/>
-    <mergeCell ref="E10:E11"/>
-    <mergeCell ref="M27:M28"/>
-    <mergeCell ref="O27:O28"/>
-    <mergeCell ref="B14:H15"/>
-    <mergeCell ref="B17:D17"/>
-    <mergeCell ref="F17:H17"/>
-    <mergeCell ref="J17:K17"/>
-    <mergeCell ref="J18:K19"/>
-    <mergeCell ref="M18:M19"/>
+    <mergeCell ref="B72:I73"/>
+    <mergeCell ref="K75:L75"/>
+    <mergeCell ref="K76:L76"/>
+    <mergeCell ref="B58:R59"/>
+    <mergeCell ref="B61:K61"/>
+    <mergeCell ref="M61:O61"/>
+    <mergeCell ref="Q61:R61"/>
+    <mergeCell ref="B66:C66"/>
+    <mergeCell ref="B67:C68"/>
+    <mergeCell ref="E67:E68"/>
     <mergeCell ref="I43:I44"/>
     <mergeCell ref="B23:K24"/>
     <mergeCell ref="B26:C26"/>
@@ -3657,16 +3658,20 @@
     <mergeCell ref="F35:I35"/>
     <mergeCell ref="B40:C40"/>
     <mergeCell ref="F40:G40"/>
-    <mergeCell ref="B72:I73"/>
-    <mergeCell ref="K75:L75"/>
-    <mergeCell ref="K76:L76"/>
-    <mergeCell ref="B58:R59"/>
-    <mergeCell ref="B61:K61"/>
-    <mergeCell ref="M61:O61"/>
-    <mergeCell ref="Q61:R61"/>
-    <mergeCell ref="B66:C66"/>
-    <mergeCell ref="B67:C68"/>
-    <mergeCell ref="E67:E68"/>
+    <mergeCell ref="M27:M28"/>
+    <mergeCell ref="O27:O28"/>
+    <mergeCell ref="B14:H15"/>
+    <mergeCell ref="B17:D17"/>
+    <mergeCell ref="F17:H17"/>
+    <mergeCell ref="J17:K17"/>
+    <mergeCell ref="J18:K19"/>
+    <mergeCell ref="M18:M19"/>
+    <mergeCell ref="B2:P3"/>
+    <mergeCell ref="B5:G5"/>
+    <mergeCell ref="K5:N5"/>
+    <mergeCell ref="B9:C9"/>
+    <mergeCell ref="B10:C11"/>
+    <mergeCell ref="E10:E11"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
New points - POTEC
</commit_message>
<xml_diff>
--- a/IoT-points-schedule.xlsx
+++ b/IoT-points-schedule.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\dodo\Desktop\IoT-studies\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{34DC516C-F8E4-45B0-9B1F-5B593EB407A1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{820C5EFB-E949-48F7-8098-9385FD81E2E4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="25440" windowHeight="15390" xr2:uid="{F85F5544-1FE8-4920-A5D4-192A98B113BD}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="334" uniqueCount="212">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="334" uniqueCount="213">
   <si>
     <t>1. Krypto</t>
   </si>
@@ -675,6 +675,9 @@
   </si>
   <si>
     <t>Laboratoria [ocena]</t>
+  </si>
+  <si>
+    <t>W16</t>
   </si>
 </sst>
 </file>
@@ -1155,56 +1158,56 @@
     <xf numFmtId="0" fontId="6" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1667,23 +1670,23 @@
       <c r="R3" s="12"/>
     </row>
     <row r="5" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B5" s="46" t="s">
+      <c r="B5" s="48" t="s">
         <v>83</v>
       </c>
-      <c r="C5" s="47"/>
-      <c r="D5" s="47"/>
-      <c r="E5" s="47"/>
-      <c r="F5" s="48"/>
-      <c r="H5" s="46" t="s">
+      <c r="C5" s="50"/>
+      <c r="D5" s="50"/>
+      <c r="E5" s="50"/>
+      <c r="F5" s="49"/>
+      <c r="H5" s="48" t="s">
         <v>82</v>
       </c>
-      <c r="I5" s="48"/>
-      <c r="K5" s="46" t="s">
+      <c r="I5" s="49"/>
+      <c r="K5" s="48" t="s">
         <v>8</v>
       </c>
-      <c r="L5" s="47"/>
-      <c r="M5" s="47"/>
-      <c r="N5" s="48"/>
+      <c r="L5" s="50"/>
+      <c r="M5" s="50"/>
+      <c r="N5" s="49"/>
       <c r="P5" s="4" t="s">
         <v>74</v>
       </c>
@@ -1743,37 +1746,37 @@
       <c r="P7" s="2"/>
     </row>
     <row r="9" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B9" s="49" t="s">
+      <c r="B9" s="51" t="s">
         <v>22</v>
       </c>
-      <c r="C9" s="49"/>
+      <c r="C9" s="51"/>
       <c r="E9" s="9" t="s">
         <v>67</v>
       </c>
-      <c r="G9" s="49" t="s">
+      <c r="G9" s="51" t="s">
         <v>87</v>
       </c>
-      <c r="H9" s="49"/>
+      <c r="H9" s="51"/>
     </row>
     <row r="10" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B10" s="50">
+      <c r="B10" s="52">
         <f>SUM(B7:F7,H7:I7,K7:N7,P7)</f>
         <v>9.6999999999999993</v>
       </c>
-      <c r="C10" s="50"/>
-      <c r="E10" s="54"/>
-      <c r="G10" s="50">
+      <c r="C10" s="52"/>
+      <c r="E10" s="46"/>
+      <c r="G10" s="52">
         <f>66-SUM(B7:F7,H7:I7,K7:N7,P7)</f>
         <v>56.3</v>
       </c>
-      <c r="H10" s="50"/>
+      <c r="H10" s="52"/>
     </row>
     <row r="11" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B11" s="50"/>
-      <c r="C11" s="50"/>
-      <c r="E11" s="55"/>
-      <c r="G11" s="50"/>
-      <c r="H11" s="50"/>
+      <c r="B11" s="52"/>
+      <c r="C11" s="52"/>
+      <c r="E11" s="47"/>
+      <c r="G11" s="52"/>
+      <c r="H11" s="52"/>
     </row>
     <row r="12" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A12" s="6"/>
@@ -1818,26 +1821,26 @@
       <c r="H15" s="45"/>
     </row>
     <row r="17" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B17" s="53" t="s">
+      <c r="B17" s="39" t="s">
         <v>91</v>
       </c>
-      <c r="C17" s="53"/>
-      <c r="D17" s="53"/>
-      <c r="E17" s="53"/>
-      <c r="F17" s="53"/>
-      <c r="H17" s="46" t="s">
+      <c r="C17" s="39"/>
+      <c r="D17" s="39"/>
+      <c r="E17" s="39"/>
+      <c r="F17" s="39"/>
+      <c r="H17" s="48" t="s">
         <v>97</v>
       </c>
-      <c r="I17" s="47"/>
-      <c r="J17" s="48"/>
-      <c r="L17" s="49" t="s">
+      <c r="I17" s="50"/>
+      <c r="J17" s="49"/>
+      <c r="L17" s="51" t="s">
         <v>22</v>
       </c>
-      <c r="M17" s="49"/>
-      <c r="O17" s="49" t="s">
+      <c r="M17" s="51"/>
+      <c r="O17" s="51" t="s">
         <v>87</v>
       </c>
-      <c r="P17" s="49"/>
+      <c r="P17" s="51"/>
       <c r="R17" s="9" t="s">
         <v>67</v>
       </c>
@@ -1867,17 +1870,17 @@
       <c r="J18" s="3" t="s">
         <v>95</v>
       </c>
-      <c r="L18" s="50">
+      <c r="L18" s="52">
         <f>SUM(B19:F19,H19:J19)</f>
         <v>29.5</v>
       </c>
-      <c r="M18" s="50"/>
-      <c r="O18" s="50">
+      <c r="M18" s="52"/>
+      <c r="O18" s="52">
         <f>50-SUM(B19:F19,H19:J19)</f>
         <v>20.5</v>
       </c>
-      <c r="P18" s="50"/>
-      <c r="R18" s="39"/>
+      <c r="P18" s="52"/>
+      <c r="R18" s="53"/>
     </row>
     <row r="19" spans="1:19" x14ac:dyDescent="0.25">
       <c r="B19" s="2"/>
@@ -1892,11 +1895,11 @@
         <v>26.5</v>
       </c>
       <c r="J19" s="2"/>
-      <c r="L19" s="50"/>
-      <c r="M19" s="50"/>
-      <c r="O19" s="50"/>
-      <c r="P19" s="50"/>
-      <c r="R19" s="39"/>
+      <c r="L19" s="52"/>
+      <c r="M19" s="52"/>
+      <c r="O19" s="52"/>
+      <c r="P19" s="52"/>
+      <c r="R19" s="53"/>
     </row>
     <row r="21" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A21" s="6"/>
@@ -1934,10 +1937,10 @@
       <c r="J23" s="41"/>
       <c r="K23" s="41"/>
       <c r="L23" s="42"/>
-      <c r="N23" s="50" t="s">
+      <c r="N23" s="52" t="s">
         <v>132</v>
       </c>
-      <c r="O23" s="50"/>
+      <c r="O23" s="52"/>
     </row>
     <row r="24" spans="1:19" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B24" s="43"/>
@@ -1951,26 +1954,26 @@
       <c r="J24" s="44"/>
       <c r="K24" s="44"/>
       <c r="L24" s="45"/>
-      <c r="N24" s="50"/>
-      <c r="O24" s="50"/>
+      <c r="N24" s="52"/>
+      <c r="O24" s="52"/>
     </row>
     <row r="26" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B26" s="53" t="s">
+      <c r="B26" s="39" t="s">
         <v>129</v>
       </c>
-      <c r="C26" s="53"/>
-      <c r="D26" s="53"/>
-      <c r="F26" s="53" t="s">
+      <c r="C26" s="39"/>
+      <c r="D26" s="39"/>
+      <c r="F26" s="39" t="s">
         <v>211</v>
       </c>
-      <c r="G26" s="53"/>
-      <c r="H26" s="53"/>
-      <c r="I26" s="53"/>
+      <c r="G26" s="39"/>
+      <c r="H26" s="39"/>
+      <c r="I26" s="39"/>
       <c r="J26" s="7"/>
-      <c r="K26" s="46" t="s">
+      <c r="K26" s="48" t="s">
         <v>128</v>
       </c>
-      <c r="L26" s="48"/>
+      <c r="L26" s="49"/>
       <c r="N26" s="9" t="s">
         <v>67</v>
       </c>
@@ -2003,7 +2006,7 @@
       <c r="L27" s="2" t="s">
         <v>127</v>
       </c>
-      <c r="N27" s="54"/>
+      <c r="N27" s="46"/>
     </row>
     <row r="28" spans="1:19" x14ac:dyDescent="0.25">
       <c r="B28" s="2"/>
@@ -2019,7 +2022,7 @@
       <c r="I28" s="2"/>
       <c r="K28" s="2"/>
       <c r="L28" s="2"/>
-      <c r="N28" s="55"/>
+      <c r="N28" s="47"/>
     </row>
     <row r="30" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A30" s="6"/>
@@ -2066,17 +2069,17 @@
       <c r="I33" s="45"/>
     </row>
     <row r="35" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B35" s="53" t="s">
+      <c r="B35" s="39" t="s">
         <v>98</v>
       </c>
-      <c r="C35" s="53"/>
+      <c r="C35" s="39"/>
       <c r="D35" s="7"/>
-      <c r="E35" s="46" t="s">
+      <c r="E35" s="48" t="s">
         <v>147</v>
       </c>
-      <c r="F35" s="47"/>
-      <c r="G35" s="47"/>
-      <c r="H35" s="48"/>
+      <c r="F35" s="50"/>
+      <c r="G35" s="50"/>
+      <c r="H35" s="49"/>
     </row>
     <row r="36" spans="2:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B36" s="2" t="s">
@@ -2117,14 +2120,14 @@
       <c r="O37" s="7"/>
     </row>
     <row r="40" spans="2:15" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B40" s="51" t="s">
+      <c r="B40" s="54" t="s">
         <v>126</v>
       </c>
-      <c r="C40" s="52"/>
-      <c r="F40" s="50" t="s">
+      <c r="C40" s="55"/>
+      <c r="F40" s="52" t="s">
         <v>102</v>
       </c>
-      <c r="G40" s="50"/>
+      <c r="G40" s="52"/>
       <c r="I40" s="9" t="s">
         <v>22</v>
       </c>
@@ -2174,7 +2177,7 @@
         <v>119</v>
       </c>
       <c r="G43" s="2"/>
-      <c r="I43" s="49" t="s">
+      <c r="I43" s="51" t="s">
         <v>67</v>
       </c>
     </row>
@@ -2189,7 +2192,7 @@
         <v>120</v>
       </c>
       <c r="G44" s="2"/>
-      <c r="I44" s="49"/>
+      <c r="I44" s="51"/>
     </row>
     <row r="45" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B45" s="2" t="s">
@@ -2364,28 +2367,28 @@
       <c r="S61" s="45"/>
     </row>
     <row r="63" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B63" s="53" t="s">
+      <c r="B63" s="39" t="s">
         <v>63</v>
       </c>
-      <c r="C63" s="53"/>
-      <c r="D63" s="53"/>
-      <c r="E63" s="53"/>
-      <c r="F63" s="53"/>
-      <c r="G63" s="53"/>
-      <c r="H63" s="53"/>
-      <c r="I63" s="53"/>
-      <c r="J63" s="53"/>
-      <c r="K63" s="53"/>
-      <c r="M63" s="53" t="s">
+      <c r="C63" s="39"/>
+      <c r="D63" s="39"/>
+      <c r="E63" s="39"/>
+      <c r="F63" s="39"/>
+      <c r="G63" s="39"/>
+      <c r="H63" s="39"/>
+      <c r="I63" s="39"/>
+      <c r="J63" s="39"/>
+      <c r="K63" s="39"/>
+      <c r="M63" s="39" t="s">
         <v>90</v>
       </c>
-      <c r="N63" s="53"/>
-      <c r="O63" s="53"/>
-      <c r="P63" s="53"/>
-      <c r="R63" s="53" t="s">
+      <c r="N63" s="39"/>
+      <c r="O63" s="39"/>
+      <c r="P63" s="39"/>
+      <c r="R63" s="39" t="s">
         <v>64</v>
       </c>
-      <c r="S63" s="53"/>
+      <c r="S63" s="39"/>
     </row>
     <row r="64" spans="1:19" x14ac:dyDescent="0.25">
       <c r="B64" s="2" t="s">
@@ -2410,10 +2413,10 @@
         <v>56</v>
       </c>
       <c r="I64" s="2" t="s">
-        <v>59</v>
+        <v>81</v>
       </c>
       <c r="J64" s="2" t="s">
-        <v>81</v>
+        <v>212</v>
       </c>
       <c r="K64" s="2" t="s">
         <v>85</v>
@@ -2459,7 +2462,9 @@
       <c r="H65" s="2">
         <v>2</v>
       </c>
-      <c r="I65" s="2"/>
+      <c r="I65" s="2">
+        <v>2</v>
+      </c>
       <c r="J65" s="2">
         <v>2</v>
       </c>
@@ -2474,62 +2479,40 @@
       <c r="S65" s="2"/>
     </row>
     <row r="68" spans="2:19" x14ac:dyDescent="0.25">
-      <c r="B68" s="49" t="s">
+      <c r="B68" s="51" t="s">
         <v>22</v>
       </c>
-      <c r="C68" s="49"/>
+      <c r="C68" s="51"/>
       <c r="E68" s="9" t="s">
         <v>67</v>
       </c>
-      <c r="G68" s="49" t="s">
+      <c r="G68" s="51" t="s">
         <v>87</v>
       </c>
-      <c r="H68" s="49"/>
+      <c r="H68" s="51"/>
     </row>
     <row r="69" spans="2:19" x14ac:dyDescent="0.25">
-      <c r="B69" s="50">
+      <c r="B69" s="52">
         <f>SUM(B65:K65,M65:P65,R65:S65)</f>
-        <v>17</v>
-      </c>
-      <c r="C69" s="50"/>
-      <c r="E69" s="39"/>
-      <c r="G69" s="50">
+        <v>19</v>
+      </c>
+      <c r="C69" s="52"/>
+      <c r="E69" s="53"/>
+      <c r="G69" s="52">
         <f>50-SUM(B65:K65,M65:P65,R65:S65)</f>
-        <v>33</v>
-      </c>
-      <c r="H69" s="50"/>
+        <v>31</v>
+      </c>
+      <c r="H69" s="52"/>
     </row>
     <row r="70" spans="2:19" x14ac:dyDescent="0.25">
-      <c r="B70" s="50"/>
-      <c r="C70" s="50"/>
-      <c r="E70" s="39"/>
-      <c r="G70" s="50"/>
-      <c r="H70" s="50"/>
+      <c r="B70" s="52"/>
+      <c r="C70" s="52"/>
+      <c r="E70" s="53"/>
+      <c r="G70" s="52"/>
+      <c r="H70" s="52"/>
     </row>
   </sheetData>
   <mergeCells count="38">
-    <mergeCell ref="R63:S63"/>
-    <mergeCell ref="B32:I33"/>
-    <mergeCell ref="B63:K63"/>
-    <mergeCell ref="B60:S61"/>
-    <mergeCell ref="M63:P63"/>
-    <mergeCell ref="N27:N28"/>
-    <mergeCell ref="F26:I26"/>
-    <mergeCell ref="K26:L26"/>
-    <mergeCell ref="B23:L24"/>
-    <mergeCell ref="B26:D26"/>
-    <mergeCell ref="B17:F17"/>
-    <mergeCell ref="H17:J17"/>
-    <mergeCell ref="O17:P17"/>
-    <mergeCell ref="B9:C9"/>
-    <mergeCell ref="B10:C11"/>
-    <mergeCell ref="L17:M17"/>
-    <mergeCell ref="E10:E11"/>
-    <mergeCell ref="E69:E70"/>
-    <mergeCell ref="B68:C68"/>
-    <mergeCell ref="B69:C70"/>
-    <mergeCell ref="G68:H68"/>
-    <mergeCell ref="G69:H70"/>
     <mergeCell ref="R18:R19"/>
     <mergeCell ref="B14:H15"/>
     <mergeCell ref="K5:N5"/>
@@ -2546,6 +2529,28 @@
     <mergeCell ref="E35:H35"/>
     <mergeCell ref="G9:H9"/>
     <mergeCell ref="G10:H11"/>
+    <mergeCell ref="E69:E70"/>
+    <mergeCell ref="B68:C68"/>
+    <mergeCell ref="B69:C70"/>
+    <mergeCell ref="G68:H68"/>
+    <mergeCell ref="G69:H70"/>
+    <mergeCell ref="B17:F17"/>
+    <mergeCell ref="H17:J17"/>
+    <mergeCell ref="O17:P17"/>
+    <mergeCell ref="B9:C9"/>
+    <mergeCell ref="B10:C11"/>
+    <mergeCell ref="L17:M17"/>
+    <mergeCell ref="E10:E11"/>
+    <mergeCell ref="N27:N28"/>
+    <mergeCell ref="F26:I26"/>
+    <mergeCell ref="K26:L26"/>
+    <mergeCell ref="B23:L24"/>
+    <mergeCell ref="B26:D26"/>
+    <mergeCell ref="R63:S63"/>
+    <mergeCell ref="B32:I33"/>
+    <mergeCell ref="B63:K63"/>
+    <mergeCell ref="B60:S61"/>
+    <mergeCell ref="M63:P63"/>
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2618,23 +2623,23 @@
       <c r="R3" s="12"/>
     </row>
     <row r="5" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B5" s="53" t="s">
+      <c r="B5" s="39" t="s">
         <v>18</v>
       </c>
-      <c r="C5" s="53"/>
-      <c r="D5" s="53"/>
-      <c r="E5" s="53"/>
-      <c r="F5" s="53"/>
-      <c r="G5" s="53"/>
+      <c r="C5" s="39"/>
+      <c r="D5" s="39"/>
+      <c r="E5" s="39"/>
+      <c r="F5" s="39"/>
+      <c r="G5" s="39"/>
       <c r="I5" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="K5" s="46" t="s">
+      <c r="K5" s="48" t="s">
         <v>8</v>
       </c>
-      <c r="L5" s="47"/>
-      <c r="M5" s="47"/>
-      <c r="N5" s="48"/>
+      <c r="L5" s="50"/>
+      <c r="M5" s="50"/>
+      <c r="N5" s="49"/>
       <c r="P5" s="4" t="s">
         <v>74</v>
       </c>
@@ -2716,28 +2721,28 @@
       </c>
     </row>
     <row r="9" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B9" s="49" t="s">
+      <c r="B9" s="51" t="s">
         <v>22</v>
       </c>
-      <c r="C9" s="49"/>
+      <c r="C9" s="51"/>
       <c r="E9" s="9" t="s">
         <v>67</v>
       </c>
     </row>
     <row r="10" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B10" s="50">
+      <c r="B10" s="52">
         <f>_xlfn.CEILING.MATH(SUM(B7:G7,I7,K7:N7,P7),1,1)</f>
         <v>110</v>
       </c>
-      <c r="C10" s="50"/>
-      <c r="E10" s="54">
+      <c r="C10" s="52"/>
+      <c r="E10" s="46">
         <v>4</v>
       </c>
     </row>
     <row r="11" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B11" s="50"/>
-      <c r="C11" s="50"/>
-      <c r="E11" s="55"/>
+      <c r="B11" s="52"/>
+      <c r="C11" s="52"/>
+      <c r="E11" s="47"/>
     </row>
     <row r="12" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A12" s="6"/>
@@ -2782,20 +2787,20 @@
       <c r="H15" s="61"/>
     </row>
     <row r="17" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B17" s="53" t="s">
+      <c r="B17" s="39" t="s">
         <v>12</v>
       </c>
-      <c r="C17" s="53"/>
-      <c r="D17" s="53"/>
-      <c r="F17" s="53" t="s">
+      <c r="C17" s="39"/>
+      <c r="D17" s="39"/>
+      <c r="F17" s="39" t="s">
         <v>8</v>
       </c>
-      <c r="G17" s="53"/>
-      <c r="H17" s="53"/>
-      <c r="J17" s="49" t="s">
+      <c r="G17" s="39"/>
+      <c r="H17" s="39"/>
+      <c r="J17" s="51" t="s">
         <v>22</v>
       </c>
-      <c r="K17" s="49"/>
+      <c r="K17" s="51"/>
       <c r="M17" s="9" t="s">
         <v>67</v>
       </c>
@@ -2819,12 +2824,12 @@
       <c r="H18" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="J18" s="50">
+      <c r="J18" s="52">
         <f>SUM(B19:D19,F19:H19)</f>
         <v>93</v>
       </c>
-      <c r="K18" s="50"/>
-      <c r="M18" s="39">
+      <c r="K18" s="52"/>
+      <c r="M18" s="53">
         <v>5</v>
       </c>
     </row>
@@ -2847,9 +2852,9 @@
       <c r="H19" s="2">
         <v>4</v>
       </c>
-      <c r="J19" s="50"/>
-      <c r="K19" s="50"/>
-      <c r="M19" s="39"/>
+      <c r="J19" s="52"/>
+      <c r="K19" s="52"/>
+      <c r="M19" s="53"/>
     </row>
     <row r="21" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A21" s="6"/>
@@ -2900,20 +2905,20 @@
       <c r="K24" s="61"/>
     </row>
     <row r="26" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B26" s="53" t="s">
+      <c r="B26" s="39" t="s">
         <v>17</v>
       </c>
-      <c r="C26" s="53"/>
-      <c r="E26" s="46" t="s">
+      <c r="C26" s="39"/>
+      <c r="E26" s="48" t="s">
         <v>21</v>
       </c>
-      <c r="F26" s="47"/>
-      <c r="G26" s="48"/>
-      <c r="I26" s="53" t="s">
+      <c r="F26" s="50"/>
+      <c r="G26" s="49"/>
+      <c r="I26" s="39" t="s">
         <v>20</v>
       </c>
-      <c r="J26" s="53"/>
-      <c r="K26" s="53"/>
+      <c r="J26" s="39"/>
+      <c r="K26" s="39"/>
       <c r="M26" s="10" t="s">
         <v>22</v>
       </c>
@@ -2953,7 +2958,7 @@
         <v>36</v>
       </c>
       <c r="N27" s="7"/>
-      <c r="O27" s="39">
+      <c r="O27" s="53">
         <v>4</v>
       </c>
       <c r="P27" s="8"/>
@@ -2985,7 +2990,7 @@
       </c>
       <c r="M28" s="62"/>
       <c r="N28" s="7"/>
-      <c r="O28" s="39"/>
+      <c r="O28" s="53"/>
       <c r="P28" s="8"/>
     </row>
     <row r="30" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -3033,17 +3038,17 @@
       <c r="I33" s="61"/>
     </row>
     <row r="35" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B35" s="53" t="s">
+      <c r="B35" s="39" t="s">
         <v>31</v>
       </c>
-      <c r="C35" s="53"/>
-      <c r="D35" s="53"/>
-      <c r="F35" s="53" t="s">
+      <c r="C35" s="39"/>
+      <c r="D35" s="39"/>
+      <c r="F35" s="39" t="s">
         <v>12</v>
       </c>
-      <c r="G35" s="53"/>
-      <c r="H35" s="53"/>
-      <c r="I35" s="53"/>
+      <c r="G35" s="39"/>
+      <c r="H35" s="39"/>
+      <c r="I35" s="39"/>
       <c r="N35" s="7"/>
       <c r="O35" s="7"/>
     </row>
@@ -3100,14 +3105,14 @@
       <c r="O37" s="7"/>
     </row>
     <row r="40" spans="2:15" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B40" s="51" t="s">
+      <c r="B40" s="54" t="s">
         <v>35</v>
       </c>
-      <c r="C40" s="52"/>
-      <c r="F40" s="50" t="s">
+      <c r="C40" s="55"/>
+      <c r="F40" s="52" t="s">
         <v>36</v>
       </c>
-      <c r="G40" s="50"/>
+      <c r="G40" s="52"/>
       <c r="I40" s="9" t="s">
         <v>22</v>
       </c>
@@ -3163,7 +3168,7 @@
       <c r="G43" s="2">
         <v>0.44</v>
       </c>
-      <c r="I43" s="49" t="s">
+      <c r="I43" s="51" t="s">
         <v>67</v>
       </c>
     </row>
@@ -3180,7 +3185,7 @@
       <c r="G44" s="2">
         <v>1</v>
       </c>
-      <c r="I44" s="49"/>
+      <c r="I44" s="51"/>
     </row>
     <row r="45" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B45" s="2" t="s">
@@ -3364,27 +3369,27 @@
       <c r="R59" s="61"/>
     </row>
     <row r="61" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B61" s="53" t="s">
+      <c r="B61" s="39" t="s">
         <v>63</v>
       </c>
-      <c r="C61" s="53"/>
-      <c r="D61" s="53"/>
-      <c r="E61" s="53"/>
-      <c r="F61" s="53"/>
-      <c r="G61" s="53"/>
-      <c r="H61" s="53"/>
-      <c r="I61" s="53"/>
-      <c r="J61" s="53"/>
-      <c r="K61" s="53"/>
-      <c r="M61" s="53" t="s">
+      <c r="C61" s="39"/>
+      <c r="D61" s="39"/>
+      <c r="E61" s="39"/>
+      <c r="F61" s="39"/>
+      <c r="G61" s="39"/>
+      <c r="H61" s="39"/>
+      <c r="I61" s="39"/>
+      <c r="J61" s="39"/>
+      <c r="K61" s="39"/>
+      <c r="M61" s="39" t="s">
         <v>68</v>
       </c>
-      <c r="N61" s="53"/>
-      <c r="O61" s="53"/>
-      <c r="Q61" s="53" t="s">
+      <c r="N61" s="39"/>
+      <c r="O61" s="39"/>
+      <c r="Q61" s="39" t="s">
         <v>64</v>
       </c>
-      <c r="R61" s="53"/>
+      <c r="R61" s="39"/>
     </row>
     <row r="62" spans="1:19" x14ac:dyDescent="0.25">
       <c r="B62" s="2" t="s">
@@ -3481,28 +3486,28 @@
       </c>
     </row>
     <row r="66" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B66" s="49" t="s">
+      <c r="B66" s="51" t="s">
         <v>22</v>
       </c>
-      <c r="C66" s="49"/>
+      <c r="C66" s="51"/>
       <c r="E66" s="9" t="s">
         <v>67</v>
       </c>
     </row>
     <row r="67" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B67" s="50">
+      <c r="B67" s="52">
         <f xml:space="preserve"> SUM(B63:K63,M63:O63,Q63:R63)</f>
         <v>85.5</v>
       </c>
-      <c r="C67" s="50"/>
-      <c r="E67" s="39">
+      <c r="C67" s="52"/>
+      <c r="E67" s="53">
         <v>4.5</v>
       </c>
     </row>
     <row r="68" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B68" s="50"/>
-      <c r="C68" s="50"/>
-      <c r="E68" s="39"/>
+      <c r="B68" s="52"/>
+      <c r="C68" s="52"/>
+      <c r="E68" s="53"/>
     </row>
     <row r="70" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A70" s="6"/>
@@ -3573,10 +3578,10 @@
       <c r="I75" s="4" t="s">
         <v>146</v>
       </c>
-      <c r="K75" s="49" t="s">
+      <c r="K75" s="51" t="s">
         <v>22</v>
       </c>
-      <c r="L75" s="49"/>
+      <c r="L75" s="51"/>
       <c r="N75" s="9" t="s">
         <v>67</v>
       </c>
@@ -3606,11 +3611,11 @@
       <c r="I76" s="2">
         <v>5</v>
       </c>
-      <c r="K76" s="50">
+      <c r="K76" s="52">
         <f>SUM(B76:I76)</f>
         <v>96</v>
       </c>
-      <c r="L76" s="50"/>
+      <c r="L76" s="52"/>
       <c r="N76" s="13">
         <v>5</v>
       </c>
@@ -3638,6 +3643,30 @@
     </row>
   </sheetData>
   <mergeCells count="34">
+    <mergeCell ref="B2:P3"/>
+    <mergeCell ref="B5:G5"/>
+    <mergeCell ref="K5:N5"/>
+    <mergeCell ref="B9:C9"/>
+    <mergeCell ref="B10:C11"/>
+    <mergeCell ref="E10:E11"/>
+    <mergeCell ref="M27:M28"/>
+    <mergeCell ref="O27:O28"/>
+    <mergeCell ref="B14:H15"/>
+    <mergeCell ref="B17:D17"/>
+    <mergeCell ref="F17:H17"/>
+    <mergeCell ref="J17:K17"/>
+    <mergeCell ref="J18:K19"/>
+    <mergeCell ref="M18:M19"/>
+    <mergeCell ref="I43:I44"/>
+    <mergeCell ref="B23:K24"/>
+    <mergeCell ref="B26:C26"/>
+    <mergeCell ref="E26:G26"/>
+    <mergeCell ref="I26:K26"/>
+    <mergeCell ref="B32:I33"/>
+    <mergeCell ref="B35:D35"/>
+    <mergeCell ref="F35:I35"/>
+    <mergeCell ref="B40:C40"/>
+    <mergeCell ref="F40:G40"/>
     <mergeCell ref="B72:I73"/>
     <mergeCell ref="K75:L75"/>
     <mergeCell ref="K76:L76"/>
@@ -3648,30 +3677,6 @@
     <mergeCell ref="B66:C66"/>
     <mergeCell ref="B67:C68"/>
     <mergeCell ref="E67:E68"/>
-    <mergeCell ref="I43:I44"/>
-    <mergeCell ref="B23:K24"/>
-    <mergeCell ref="B26:C26"/>
-    <mergeCell ref="E26:G26"/>
-    <mergeCell ref="I26:K26"/>
-    <mergeCell ref="B32:I33"/>
-    <mergeCell ref="B35:D35"/>
-    <mergeCell ref="F35:I35"/>
-    <mergeCell ref="B40:C40"/>
-    <mergeCell ref="F40:G40"/>
-    <mergeCell ref="M27:M28"/>
-    <mergeCell ref="O27:O28"/>
-    <mergeCell ref="B14:H15"/>
-    <mergeCell ref="B17:D17"/>
-    <mergeCell ref="F17:H17"/>
-    <mergeCell ref="J17:K17"/>
-    <mergeCell ref="J18:K19"/>
-    <mergeCell ref="M18:M19"/>
-    <mergeCell ref="B2:P3"/>
-    <mergeCell ref="B5:G5"/>
-    <mergeCell ref="K5:N5"/>
-    <mergeCell ref="B9:C9"/>
-    <mergeCell ref="B10:C11"/>
-    <mergeCell ref="E10:E11"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
New points - MAT3 and FIZ1 + corrections in schedule
</commit_message>
<xml_diff>
--- a/IoT-points-schedule.xlsx
+++ b/IoT-points-schedule.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28623"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28730"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\dodo\Desktop\IoT-studies\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{820C5EFB-E949-48F7-8098-9385FD81E2E4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ECC88167-D2D0-4AC6-BB78-6E55CB9408F0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="25440" windowHeight="15390" xr2:uid="{F85F5544-1FE8-4920-A5D4-192A98B113BD}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="25440" windowHeight="15390" activeTab="2" xr2:uid="{F85F5544-1FE8-4920-A5D4-192A98B113BD}"/>
   </bookViews>
   <sheets>
     <sheet name="II-semestr-25L" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="334" uniqueCount="213">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="340" uniqueCount="218">
   <si>
     <t>1. Krypto</t>
   </si>
@@ -431,9 +431,6 @@
     <t>Ćwiczenia [C = 0,6K+0,4P]</t>
   </si>
   <si>
-    <t>Kolokwium</t>
-  </si>
-  <si>
     <t>Mini-projekt</t>
   </si>
   <si>
@@ -678,6 +675,24 @@
   </si>
   <si>
     <t>W16</t>
+  </si>
+  <si>
+    <t>1. RSA</t>
+  </si>
+  <si>
+    <t>Sieć sortująca</t>
+  </si>
+  <si>
+    <t>Projekt #2</t>
+  </si>
+  <si>
+    <t>6. Zliczanie orbit</t>
+  </si>
+  <si>
+    <t>Kolokwium [15 pkt]</t>
+  </si>
+  <si>
+    <t>Zliczanie orbit</t>
   </si>
 </sst>
 </file>
@@ -1693,22 +1708,26 @@
     </row>
     <row r="6" spans="1:19" ht="29.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B6" s="3" t="s">
+        <v>174</v>
+      </c>
+      <c r="C6" s="3" t="s">
         <v>175</v>
       </c>
-      <c r="C6" s="3" t="s">
+      <c r="D6" s="3" t="s">
         <v>176</v>
       </c>
-      <c r="D6" s="3" t="s">
+      <c r="E6" s="3" t="s">
         <v>177</v>
       </c>
-      <c r="E6" s="3" t="s">
+      <c r="F6" s="3" t="s">
         <v>178</v>
       </c>
-      <c r="F6" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="H6" s="2"/>
-      <c r="I6" s="2"/>
+      <c r="H6" s="2" t="s">
+        <v>212</v>
+      </c>
+      <c r="I6" s="2" t="s">
+        <v>215</v>
+      </c>
       <c r="K6" s="2" t="s">
         <v>24</v>
       </c>
@@ -1732,7 +1751,9 @@
       <c r="C7" s="2">
         <v>2.7</v>
       </c>
-      <c r="D7" s="2"/>
+      <c r="D7" s="2">
+        <v>3</v>
+      </c>
       <c r="E7" s="2"/>
       <c r="F7" s="2"/>
       <c r="H7" s="2"/>
@@ -1761,13 +1782,13 @@
     <row r="10" spans="1:19" x14ac:dyDescent="0.25">
       <c r="B10" s="52">
         <f>SUM(B7:F7,H7:I7,K7:N7,P7)</f>
-        <v>9.6999999999999993</v>
+        <v>12.7</v>
       </c>
       <c r="C10" s="52"/>
       <c r="E10" s="46"/>
       <c r="G10" s="52">
         <f>66-SUM(B7:F7,H7:I7,K7:N7,P7)</f>
-        <v>56.3</v>
+        <v>53.3</v>
       </c>
       <c r="H10" s="52"/>
     </row>
@@ -1847,13 +1868,13 @@
     </row>
     <row r="18" spans="1:19" ht="48.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B18" s="3" t="s">
+        <v>158</v>
+      </c>
+      <c r="C18" s="3" t="s">
         <v>159</v>
       </c>
-      <c r="C18" s="3" t="s">
+      <c r="D18" s="3" t="s">
         <v>160</v>
-      </c>
-      <c r="D18" s="3" t="s">
-        <v>161</v>
       </c>
       <c r="E18" s="3" t="s">
         <v>92</v>
@@ -1938,7 +1959,7 @@
       <c r="K23" s="41"/>
       <c r="L23" s="42"/>
       <c r="N23" s="52" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="O23" s="52"/>
     </row>
@@ -1964,7 +1985,7 @@
       <c r="C26" s="39"/>
       <c r="D26" s="39"/>
       <c r="F26" s="39" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="G26" s="39"/>
       <c r="H26" s="39"/>
@@ -1980,25 +2001,25 @@
     </row>
     <row r="27" spans="1:19" x14ac:dyDescent="0.25">
       <c r="B27" s="14" t="s">
+        <v>216</v>
+      </c>
+      <c r="C27" s="14" t="s">
         <v>130</v>
-      </c>
-      <c r="C27" s="14" t="s">
-        <v>131</v>
       </c>
       <c r="D27" s="2" t="s">
         <v>11</v>
       </c>
       <c r="F27" s="2" t="s">
+        <v>206</v>
+      </c>
+      <c r="G27" s="2" t="s">
+        <v>208</v>
+      </c>
+      <c r="H27" s="2" t="s">
         <v>207</v>
       </c>
-      <c r="G27" s="2" t="s">
+      <c r="I27" s="2" t="s">
         <v>209</v>
-      </c>
-      <c r="H27" s="2" t="s">
-        <v>208</v>
-      </c>
-      <c r="I27" s="2" t="s">
-        <v>210</v>
       </c>
       <c r="K27" s="14" t="s">
         <v>73</v>
@@ -2009,7 +2030,9 @@
       <c r="N27" s="46"/>
     </row>
     <row r="28" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B28" s="2"/>
+      <c r="B28" s="2">
+        <v>6</v>
+      </c>
       <c r="C28" s="2"/>
       <c r="D28" s="2">
         <v>1</v>
@@ -2075,7 +2098,7 @@
       <c r="C35" s="39"/>
       <c r="D35" s="7"/>
       <c r="E35" s="48" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="F35" s="50"/>
       <c r="G35" s="50"/>
@@ -2416,7 +2439,7 @@
         <v>81</v>
       </c>
       <c r="J64" s="2" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="K64" s="2" t="s">
         <v>85</v>
@@ -2454,10 +2477,10 @@
         <v>2</v>
       </c>
       <c r="F65" s="2" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="G65" s="2" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="H65" s="2">
         <v>2</v>
@@ -2472,7 +2495,9 @@
       <c r="M65" s="2">
         <v>5</v>
       </c>
-      <c r="N65" s="2"/>
+      <c r="N65" s="2">
+        <v>5</v>
+      </c>
       <c r="O65" s="2"/>
       <c r="P65" s="2"/>
       <c r="R65" s="2"/>
@@ -2494,13 +2519,13 @@
     <row r="69" spans="2:19" x14ac:dyDescent="0.25">
       <c r="B69" s="52">
         <f>SUM(B65:K65,M65:P65,R65:S65)</f>
-        <v>19</v>
+        <v>24</v>
       </c>
       <c r="C69" s="52"/>
       <c r="E69" s="53"/>
       <c r="G69" s="52">
         <f>50-SUM(B65:K65,M65:P65,R65:S65)</f>
-        <v>31</v>
+        <v>26</v>
       </c>
       <c r="H69" s="52"/>
     </row>
@@ -2587,7 +2612,7 @@
     <row r="1" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="2" spans="1:19" x14ac:dyDescent="0.25">
       <c r="B2" s="56" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="C2" s="57"/>
       <c r="D2" s="57"/>
@@ -2768,7 +2793,7 @@
     <row r="13" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="14" spans="1:19" x14ac:dyDescent="0.25">
       <c r="B14" s="56" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="C14" s="57"/>
       <c r="D14" s="57"/>
@@ -2880,7 +2905,7 @@
     <row r="22" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="23" spans="1:19" x14ac:dyDescent="0.25">
       <c r="B23" s="56" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="C23" s="57"/>
       <c r="D23" s="57"/>
@@ -3017,7 +3042,7 @@
     <row r="31" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="32" spans="1:19" x14ac:dyDescent="0.25">
       <c r="B32" s="56" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="C32" s="57"/>
       <c r="D32" s="57"/>
@@ -3330,7 +3355,7 @@
     <row r="57" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="58" spans="1:19" x14ac:dyDescent="0.25">
       <c r="B58" s="56" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="C58" s="57"/>
       <c r="D58" s="57"/>
@@ -3533,7 +3558,7 @@
     <row r="71" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="72" spans="1:19" x14ac:dyDescent="0.25">
       <c r="B72" s="56" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="C72" s="57"/>
       <c r="D72" s="57"/>
@@ -3555,28 +3580,28 @@
     </row>
     <row r="75" spans="1:19" x14ac:dyDescent="0.25">
       <c r="B75" s="4" t="s">
+        <v>138</v>
+      </c>
+      <c r="C75" s="4" t="s">
         <v>139</v>
       </c>
-      <c r="C75" s="4" t="s">
+      <c r="D75" s="4" t="s">
         <v>140</v>
       </c>
-      <c r="D75" s="4" t="s">
+      <c r="E75" s="4" t="s">
         <v>141</v>
       </c>
-      <c r="E75" s="4" t="s">
+      <c r="F75" s="4" t="s">
         <v>142</v>
       </c>
-      <c r="F75" s="4" t="s">
+      <c r="G75" s="4" t="s">
         <v>143</v>
       </c>
-      <c r="G75" s="4" t="s">
+      <c r="H75" s="4" t="s">
         <v>144</v>
       </c>
-      <c r="H75" s="4" t="s">
+      <c r="I75" s="4" t="s">
         <v>145</v>
-      </c>
-      <c r="I75" s="4" t="s">
-        <v>146</v>
       </c>
       <c r="K75" s="51" t="s">
         <v>22</v>
@@ -3685,7 +3710,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CEAA0BBB-B59A-4C0E-8304-D0FA810EECB4}">
-  <dimension ref="B1:F34"/>
+  <dimension ref="B1:F35"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="3" max="3" width="11.85546875" style="16" customWidth="1"/>
@@ -3697,16 +3722,16 @@
     <row r="1" spans="2:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="2" spans="2:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="C2" s="15" t="s">
+        <v>147</v>
+      </c>
+      <c r="D2" s="15" t="s">
         <v>148</v>
       </c>
-      <c r="D2" s="15" t="s">
-        <v>149</v>
-      </c>
       <c r="E2" s="15" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="F2" s="15" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
     </row>
     <row r="3" spans="2:6" x14ac:dyDescent="0.25">
@@ -3720,10 +3745,10 @@
         <v>45763</v>
       </c>
       <c r="E3" s="26" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="F3" s="24" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
     </row>
     <row r="4" spans="2:6" x14ac:dyDescent="0.25">
@@ -3734,13 +3759,13 @@
         <v>77</v>
       </c>
       <c r="D4" s="20">
-        <v>45810</v>
+        <v>45803</v>
       </c>
       <c r="E4" s="18" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="F4" s="17" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
     </row>
     <row r="5" spans="2:6" x14ac:dyDescent="0.25">
@@ -3754,10 +3779,10 @@
         <v>45817</v>
       </c>
       <c r="E5" s="18" t="s">
+        <v>151</v>
+      </c>
+      <c r="F5" s="17" t="s">
         <v>152</v>
-      </c>
-      <c r="F5" s="17" t="s">
-        <v>153</v>
       </c>
     </row>
     <row r="6" spans="2:6" x14ac:dyDescent="0.25">
@@ -3777,7 +3802,7 @@
         <v>103</v>
       </c>
       <c r="F7" s="27" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
     </row>
     <row r="8" spans="2:6" x14ac:dyDescent="0.25">
@@ -3794,7 +3819,7 @@
         <v>104</v>
       </c>
       <c r="F8" s="27" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
     </row>
     <row r="9" spans="2:6" x14ac:dyDescent="0.25">
@@ -3811,24 +3836,24 @@
         <v>105</v>
       </c>
       <c r="F9" s="27" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="10" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B10" s="23" t="b">
+        <v>1</v>
+      </c>
+      <c r="C10" s="29" t="s">
+        <v>77</v>
+      </c>
+      <c r="D10" s="28">
+        <v>45785</v>
+      </c>
+      <c r="E10" s="27" t="s">
+        <v>106</v>
+      </c>
+      <c r="F10" s="27" t="s">
         <v>156</v>
-      </c>
-    </row>
-    <row r="10" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B10" s="19" t="b">
-        <v>0</v>
-      </c>
-      <c r="C10" s="21" t="s">
-        <v>77</v>
-      </c>
-      <c r="D10" s="20">
-        <v>45785</v>
-      </c>
-      <c r="E10" s="17" t="s">
-        <v>106</v>
-      </c>
-      <c r="F10" s="17" t="s">
-        <v>157</v>
       </c>
     </row>
     <row r="11" spans="2:6" x14ac:dyDescent="0.25">
@@ -3845,7 +3870,7 @@
         <v>107</v>
       </c>
       <c r="F11" s="17" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
     </row>
     <row r="12" spans="2:6" x14ac:dyDescent="0.25">
@@ -3856,7 +3881,7 @@
         <v>1</v>
       </c>
       <c r="C13" s="29" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="D13" s="28">
         <v>45728</v>
@@ -3865,7 +3890,7 @@
         <v>84</v>
       </c>
       <c r="F13" s="27" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
     </row>
     <row r="14" spans="2:6" x14ac:dyDescent="0.25">
@@ -3873,33 +3898,33 @@
         <v>1</v>
       </c>
       <c r="C14" s="29" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="D14" s="28">
         <v>45747</v>
       </c>
       <c r="E14" s="27" t="s">
+        <v>163</v>
+      </c>
+      <c r="F14" s="27" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="15" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B15" s="23" t="b">
+        <v>1</v>
+      </c>
+      <c r="C15" s="29" t="s">
+        <v>161</v>
+      </c>
+      <c r="D15" s="28">
+        <v>45784</v>
+      </c>
+      <c r="E15" s="27" t="s">
         <v>164</v>
       </c>
-      <c r="F14" s="27" t="s">
-        <v>168</v>
-      </c>
-    </row>
-    <row r="15" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B15" s="19" t="b">
-        <v>0</v>
-      </c>
-      <c r="C15" s="21" t="s">
-        <v>162</v>
-      </c>
-      <c r="D15" s="20">
-        <v>45782</v>
-      </c>
-      <c r="E15" s="17" t="s">
+      <c r="F15" s="27" t="s">
         <v>165</v>
-      </c>
-      <c r="F15" s="17" t="s">
-        <v>166</v>
       </c>
     </row>
     <row r="16" spans="2:6" x14ac:dyDescent="0.25">
@@ -3907,7 +3932,7 @@
         <v>0</v>
       </c>
       <c r="C16" s="21" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="D16" s="20">
         <v>45796</v>
@@ -3916,7 +3941,7 @@
         <v>85</v>
       </c>
       <c r="F16" s="17" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
     </row>
     <row r="17" spans="2:6" x14ac:dyDescent="0.25">
@@ -3924,16 +3949,16 @@
         <v>0</v>
       </c>
       <c r="C17" s="21" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="D17" s="20">
         <v>45817</v>
       </c>
       <c r="E17" s="17" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="F17" s="21" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
     </row>
     <row r="18" spans="2:6" x14ac:dyDescent="0.25">
@@ -3941,16 +3966,16 @@
         <v>0</v>
       </c>
       <c r="C18" s="21" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="D18" s="20">
         <v>45819</v>
       </c>
       <c r="E18" s="17" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="F18" s="21" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
     </row>
     <row r="19" spans="2:6" x14ac:dyDescent="0.25">
@@ -3962,13 +3987,13 @@
         <v>0</v>
       </c>
       <c r="C20" s="21" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="D20" s="20">
         <v>45820</v>
       </c>
       <c r="E20" s="17" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
     </row>
     <row r="21" spans="2:6" x14ac:dyDescent="0.25">
@@ -3976,13 +4001,13 @@
         <v>0</v>
       </c>
       <c r="C21" s="21" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="D21" s="20">
         <v>45820</v>
       </c>
       <c r="E21" s="17" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
     </row>
     <row r="22" spans="2:6" x14ac:dyDescent="0.25">
@@ -4000,10 +4025,10 @@
         <v>45728</v>
       </c>
       <c r="E23" s="27" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="F23" s="27" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
     </row>
     <row r="24" spans="2:6" x14ac:dyDescent="0.25">
@@ -4017,10 +4042,10 @@
         <v>45742</v>
       </c>
       <c r="E24" s="27" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="F24" s="27" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
     </row>
     <row r="25" spans="2:6" x14ac:dyDescent="0.25">
@@ -4034,10 +4059,10 @@
         <v>45756</v>
       </c>
       <c r="E25" s="27" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="F25" s="27" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
     </row>
     <row r="26" spans="2:6" x14ac:dyDescent="0.25">
@@ -4051,27 +4076,27 @@
         <v>45770</v>
       </c>
       <c r="E26" s="27" t="s">
+        <v>179</v>
+      </c>
+      <c r="F26" s="29" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="27" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B27" s="23" t="b">
+        <v>1</v>
+      </c>
+      <c r="C27" s="29" t="s">
+        <v>76</v>
+      </c>
+      <c r="D27" s="28">
+        <v>45784</v>
+      </c>
+      <c r="E27" s="27" t="s">
         <v>180</v>
       </c>
-      <c r="F26" s="29" t="s">
-        <v>192</v>
-      </c>
-    </row>
-    <row r="27" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B27" s="19" t="b">
-        <v>0</v>
-      </c>
-      <c r="C27" s="21" t="s">
-        <v>76</v>
-      </c>
-      <c r="D27" s="20">
-        <v>45784</v>
-      </c>
-      <c r="E27" s="17" t="s">
-        <v>181</v>
-      </c>
-      <c r="F27" s="17" t="s">
-        <v>189</v>
+      <c r="F27" s="27" t="s">
+        <v>188</v>
       </c>
     </row>
     <row r="28" spans="2:6" x14ac:dyDescent="0.25">
@@ -4085,10 +4110,10 @@
         <v>45798</v>
       </c>
       <c r="E28" s="17" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="F28" s="17" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
     </row>
     <row r="29" spans="2:6" x14ac:dyDescent="0.25">
@@ -4102,9 +4127,11 @@
         <v>45812</v>
       </c>
       <c r="E29" s="17" t="s">
-        <v>180</v>
-      </c>
-      <c r="F29" s="17"/>
+        <v>179</v>
+      </c>
+      <c r="F29" s="21" t="s">
+        <v>217</v>
+      </c>
     </row>
     <row r="30" spans="2:6" x14ac:dyDescent="0.25">
       <c r="C30" s="31"/>
@@ -4120,10 +4147,10 @@
         <v>45764</v>
       </c>
       <c r="E31" s="27" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="F31" s="27" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
     </row>
     <row r="32" spans="2:6" x14ac:dyDescent="0.25">
@@ -4140,24 +4167,41 @@
         <v>45767</v>
       </c>
       <c r="E33" s="27" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="F33" s="27" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
     </row>
     <row r="34" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B34" s="19" t="b">
+      <c r="B34" s="23" t="b">
+        <v>1</v>
+      </c>
+      <c r="C34" s="29" t="s">
+        <v>78</v>
+      </c>
+      <c r="D34" s="28">
+        <v>45775</v>
+      </c>
+      <c r="E34" s="27" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="35" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B35" s="19" t="b">
         <v>0</v>
       </c>
-      <c r="C34" s="21" t="s">
+      <c r="C35" s="21" t="s">
         <v>78</v>
       </c>
-      <c r="D34" s="20">
-        <v>45775</v>
-      </c>
-      <c r="E34" s="17" t="s">
-        <v>150</v>
+      <c r="D35" s="20">
+        <v>45794</v>
+      </c>
+      <c r="E35" s="17" t="s">
+        <v>214</v>
+      </c>
+      <c r="F35" s="17" t="s">
+        <v>213</v>
       </c>
     </row>
   </sheetData>
@@ -4186,53 +4230,53 @@
     <row r="1" spans="2:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="2" spans="2:12" ht="23.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B2" s="63" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="C2" s="64"/>
       <c r="D2" s="65"/>
       <c r="F2" s="63" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="G2" s="64"/>
       <c r="H2" s="65"/>
       <c r="J2" s="63" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="K2" s="64"/>
       <c r="L2" s="65"/>
     </row>
     <row r="3" spans="2:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B3" s="34" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="C3" s="35" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="D3" s="36" t="s">
+        <v>195</v>
+      </c>
+      <c r="F3" s="34" t="s">
+        <v>147</v>
+      </c>
+      <c r="G3" s="35" t="s">
         <v>196</v>
       </c>
-      <c r="F3" s="34" t="s">
-        <v>148</v>
-      </c>
-      <c r="G3" s="35" t="s">
-        <v>197</v>
-      </c>
       <c r="H3" s="36" t="s">
+        <v>195</v>
+      </c>
+      <c r="J3" s="34" t="s">
+        <v>147</v>
+      </c>
+      <c r="K3" s="35" t="s">
         <v>196</v>
       </c>
-      <c r="J3" s="34" t="s">
-        <v>148</v>
-      </c>
-      <c r="K3" s="35" t="s">
-        <v>197</v>
-      </c>
       <c r="L3" s="36" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
     </row>
     <row r="4" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B4" s="37" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="C4" s="14">
         <v>4</v>
@@ -4248,7 +4292,7 @@
       </c>
       <c r="H4" s="14"/>
       <c r="J4" s="37" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="K4" s="14">
         <v>4</v>
@@ -4257,7 +4301,7 @@
     </row>
     <row r="5" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B5" s="38" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="C5" s="2">
         <v>6</v>
@@ -4273,7 +4317,7 @@
       </c>
       <c r="H5" s="2"/>
       <c r="J5" s="38" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="K5" s="2">
         <v>4</v>
@@ -4282,7 +4326,7 @@
     </row>
     <row r="6" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B6" s="38" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="C6" s="2">
         <v>4</v>
@@ -4298,7 +4342,7 @@
       </c>
       <c r="H6" s="2"/>
       <c r="J6" s="38" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="K6" s="2">
         <v>5</v>
@@ -4307,7 +4351,7 @@
     </row>
     <row r="7" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B7" s="38" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="C7" s="2">
         <v>4</v>
@@ -4323,7 +4367,7 @@
       </c>
       <c r="H7" s="2"/>
       <c r="J7" s="38" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="K7" s="2">
         <v>5</v>
@@ -4332,7 +4376,7 @@
     </row>
     <row r="8" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B8" s="38" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="C8" s="2">
         <v>10</v>
@@ -4348,7 +4392,7 @@
       </c>
       <c r="H8" s="2"/>
       <c r="J8" s="38" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="K8" s="2">
         <v>12</v>
@@ -4357,7 +4401,7 @@
     </row>
     <row r="9" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B9" s="38" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="C9" s="2">
         <v>2</v>
@@ -4375,7 +4419,7 @@
     <row r="10" spans="2:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="11" spans="2:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B11" s="66" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="C11" s="67"/>
       <c r="D11" s="33">
@@ -4383,7 +4427,7 @@
         <v>4.4333333333333336</v>
       </c>
       <c r="F11" s="66" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="G11" s="67"/>
       <c r="H11" s="33">
@@ -4391,7 +4435,7 @@
         <v>0</v>
       </c>
       <c r="J11" s="66" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="K11" s="67"/>
       <c r="L11" s="33">

</xml_diff>

<commit_message>
MAT3 - points from the colloquium and corrections in schedule
</commit_message>
<xml_diff>
--- a/IoT-points-schedule.xlsx
+++ b/IoT-points-schedule.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\dodo\Desktop\IoT-studies\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ECC88167-D2D0-4AC6-BB78-6E55CB9408F0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CF068950-203A-42A1-AF03-542A2F69086C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="25440" windowHeight="15390" activeTab="2" xr2:uid="{F85F5544-1FE8-4920-A5D4-192A98B113BD}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="25440" windowHeight="15390" xr2:uid="{F85F5544-1FE8-4920-A5D4-192A98B113BD}"/>
   </bookViews>
   <sheets>
     <sheet name="II-semestr-25L" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="340" uniqueCount="218">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="348" uniqueCount="223">
   <si>
     <t>1. Krypto</t>
   </si>
@@ -693,6 +693,21 @@
   </si>
   <si>
     <t>Zliczanie orbit</t>
+  </si>
+  <si>
+    <t>Praca domowa</t>
+  </si>
+  <si>
+    <t>Poprawa kolosa</t>
+  </si>
+  <si>
+    <t>Mechanika</t>
+  </si>
+  <si>
+    <t>Wahadło odwrócone</t>
+  </si>
+  <si>
+    <t>Projekt</t>
   </si>
 </sst>
 </file>
@@ -703,7 +718,7 @@
     <numFmt numFmtId="164" formatCode="0.0"/>
     <numFmt numFmtId="165" formatCode="[$-415]d\ mmmm\ yyyy;@"/>
   </numFmts>
-  <fonts count="7" x14ac:knownFonts="1">
+  <fonts count="9" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -751,6 +766,23 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <strike/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <strike/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
@@ -1051,7 +1083,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="68">
+  <cellXfs count="78">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1173,57 +1205,57 @@
     <xf numFmtId="0" fontId="6" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1259,6 +1291,44 @@
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1">
+      <extLst>
+        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
+          <xfpb:xfComplement i="0"/>
+        </ext>
+      </extLst>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1">
+      <extLst>
+        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
+          <xfpb:xfComplement i="0"/>
+        </ext>
+      </extLst>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="7" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="7" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1685,23 +1755,23 @@
       <c r="R3" s="12"/>
     </row>
     <row r="5" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B5" s="48" t="s">
+      <c r="B5" s="46" t="s">
         <v>83</v>
       </c>
-      <c r="C5" s="50"/>
-      <c r="D5" s="50"/>
-      <c r="E5" s="50"/>
-      <c r="F5" s="49"/>
-      <c r="H5" s="48" t="s">
+      <c r="C5" s="47"/>
+      <c r="D5" s="47"/>
+      <c r="E5" s="47"/>
+      <c r="F5" s="48"/>
+      <c r="H5" s="46" t="s">
         <v>82</v>
       </c>
-      <c r="I5" s="49"/>
-      <c r="K5" s="48" t="s">
+      <c r="I5" s="48"/>
+      <c r="K5" s="46" t="s">
         <v>8</v>
       </c>
-      <c r="L5" s="50"/>
-      <c r="M5" s="50"/>
-      <c r="N5" s="49"/>
+      <c r="L5" s="47"/>
+      <c r="M5" s="47"/>
+      <c r="N5" s="48"/>
       <c r="P5" s="4" t="s">
         <v>74</v>
       </c>
@@ -1758,7 +1828,9 @@
       <c r="F7" s="2"/>
       <c r="H7" s="2"/>
       <c r="I7" s="2"/>
-      <c r="K7" s="2"/>
+      <c r="K7" s="2">
+        <v>12</v>
+      </c>
       <c r="L7" s="2"/>
       <c r="M7" s="2"/>
       <c r="N7" s="2">
@@ -1767,37 +1839,37 @@
       <c r="P7" s="2"/>
     </row>
     <row r="9" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B9" s="51" t="s">
+      <c r="B9" s="49" t="s">
         <v>22</v>
       </c>
-      <c r="C9" s="51"/>
+      <c r="C9" s="49"/>
       <c r="E9" s="9" t="s">
         <v>67</v>
       </c>
-      <c r="G9" s="51" t="s">
+      <c r="G9" s="49" t="s">
         <v>87</v>
       </c>
-      <c r="H9" s="51"/>
+      <c r="H9" s="49"/>
     </row>
     <row r="10" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B10" s="52">
+      <c r="B10" s="50">
         <f>SUM(B7:F7,H7:I7,K7:N7,P7)</f>
-        <v>12.7</v>
-      </c>
-      <c r="C10" s="52"/>
-      <c r="E10" s="46"/>
-      <c r="G10" s="52">
+        <v>24.7</v>
+      </c>
+      <c r="C10" s="50"/>
+      <c r="E10" s="54"/>
+      <c r="G10" s="50">
         <f>66-SUM(B7:F7,H7:I7,K7:N7,P7)</f>
-        <v>53.3</v>
-      </c>
-      <c r="H10" s="52"/>
+        <v>41.3</v>
+      </c>
+      <c r="H10" s="50"/>
     </row>
     <row r="11" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B11" s="52"/>
-      <c r="C11" s="52"/>
-      <c r="E11" s="47"/>
-      <c r="G11" s="52"/>
-      <c r="H11" s="52"/>
+      <c r="B11" s="50"/>
+      <c r="C11" s="50"/>
+      <c r="E11" s="55"/>
+      <c r="G11" s="50"/>
+      <c r="H11" s="50"/>
     </row>
     <row r="12" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A12" s="6"/>
@@ -1842,26 +1914,26 @@
       <c r="H15" s="45"/>
     </row>
     <row r="17" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B17" s="39" t="s">
+      <c r="B17" s="53" t="s">
         <v>91</v>
       </c>
-      <c r="C17" s="39"/>
-      <c r="D17" s="39"/>
-      <c r="E17" s="39"/>
-      <c r="F17" s="39"/>
-      <c r="H17" s="48" t="s">
+      <c r="C17" s="53"/>
+      <c r="D17" s="53"/>
+      <c r="E17" s="53"/>
+      <c r="F17" s="53"/>
+      <c r="H17" s="46" t="s">
         <v>97</v>
       </c>
-      <c r="I17" s="50"/>
-      <c r="J17" s="49"/>
-      <c r="L17" s="51" t="s">
+      <c r="I17" s="47"/>
+      <c r="J17" s="48"/>
+      <c r="L17" s="49" t="s">
         <v>22</v>
       </c>
-      <c r="M17" s="51"/>
-      <c r="O17" s="51" t="s">
+      <c r="M17" s="49"/>
+      <c r="O17" s="49" t="s">
         <v>87</v>
       </c>
-      <c r="P17" s="51"/>
+      <c r="P17" s="49"/>
       <c r="R17" s="9" t="s">
         <v>67</v>
       </c>
@@ -1891,17 +1963,17 @@
       <c r="J18" s="3" t="s">
         <v>95</v>
       </c>
-      <c r="L18" s="52">
+      <c r="L18" s="50">
         <f>SUM(B19:F19,H19:J19)</f>
         <v>29.5</v>
       </c>
-      <c r="M18" s="52"/>
-      <c r="O18" s="52">
+      <c r="M18" s="50"/>
+      <c r="O18" s="50">
         <f>50-SUM(B19:F19,H19:J19)</f>
         <v>20.5</v>
       </c>
-      <c r="P18" s="52"/>
-      <c r="R18" s="53"/>
+      <c r="P18" s="50"/>
+      <c r="R18" s="39"/>
     </row>
     <row r="19" spans="1:19" x14ac:dyDescent="0.25">
       <c r="B19" s="2"/>
@@ -1916,11 +1988,11 @@
         <v>26.5</v>
       </c>
       <c r="J19" s="2"/>
-      <c r="L19" s="52"/>
-      <c r="M19" s="52"/>
-      <c r="O19" s="52"/>
-      <c r="P19" s="52"/>
-      <c r="R19" s="53"/>
+      <c r="L19" s="50"/>
+      <c r="M19" s="50"/>
+      <c r="O19" s="50"/>
+      <c r="P19" s="50"/>
+      <c r="R19" s="39"/>
     </row>
     <row r="21" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A21" s="6"/>
@@ -1958,10 +2030,10 @@
       <c r="J23" s="41"/>
       <c r="K23" s="41"/>
       <c r="L23" s="42"/>
-      <c r="N23" s="52" t="s">
+      <c r="N23" s="50" t="s">
         <v>131</v>
       </c>
-      <c r="O23" s="52"/>
+      <c r="O23" s="50"/>
     </row>
     <row r="24" spans="1:19" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B24" s="43"/>
@@ -1975,26 +2047,26 @@
       <c r="J24" s="44"/>
       <c r="K24" s="44"/>
       <c r="L24" s="45"/>
-      <c r="N24" s="52"/>
-      <c r="O24" s="52"/>
+      <c r="N24" s="50"/>
+      <c r="O24" s="50"/>
     </row>
     <row r="26" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B26" s="39" t="s">
+      <c r="B26" s="53" t="s">
         <v>129</v>
       </c>
-      <c r="C26" s="39"/>
-      <c r="D26" s="39"/>
-      <c r="F26" s="39" t="s">
+      <c r="C26" s="53"/>
+      <c r="D26" s="53"/>
+      <c r="F26" s="53" t="s">
         <v>210</v>
       </c>
-      <c r="G26" s="39"/>
-      <c r="H26" s="39"/>
-      <c r="I26" s="39"/>
+      <c r="G26" s="53"/>
+      <c r="H26" s="53"/>
+      <c r="I26" s="53"/>
       <c r="J26" s="7"/>
-      <c r="K26" s="48" t="s">
+      <c r="K26" s="46" t="s">
         <v>128</v>
       </c>
-      <c r="L26" s="49"/>
+      <c r="L26" s="48"/>
       <c r="N26" s="9" t="s">
         <v>67</v>
       </c>
@@ -2027,7 +2099,7 @@
       <c r="L27" s="2" t="s">
         <v>127</v>
       </c>
-      <c r="N27" s="46"/>
+      <c r="N27" s="54"/>
     </row>
     <row r="28" spans="1:19" x14ac:dyDescent="0.25">
       <c r="B28" s="2">
@@ -2045,7 +2117,7 @@
       <c r="I28" s="2"/>
       <c r="K28" s="2"/>
       <c r="L28" s="2"/>
-      <c r="N28" s="47"/>
+      <c r="N28" s="55"/>
     </row>
     <row r="30" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A30" s="6"/>
@@ -2092,17 +2164,17 @@
       <c r="I33" s="45"/>
     </row>
     <row r="35" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B35" s="39" t="s">
+      <c r="B35" s="53" t="s">
         <v>98</v>
       </c>
-      <c r="C35" s="39"/>
+      <c r="C35" s="53"/>
       <c r="D35" s="7"/>
-      <c r="E35" s="48" t="s">
+      <c r="E35" s="46" t="s">
         <v>146</v>
       </c>
-      <c r="F35" s="50"/>
-      <c r="G35" s="50"/>
-      <c r="H35" s="49"/>
+      <c r="F35" s="47"/>
+      <c r="G35" s="47"/>
+      <c r="H35" s="48"/>
     </row>
     <row r="36" spans="2:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B36" s="2" t="s">
@@ -2143,14 +2215,14 @@
       <c r="O37" s="7"/>
     </row>
     <row r="40" spans="2:15" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B40" s="54" t="s">
+      <c r="B40" s="51" t="s">
         <v>126</v>
       </c>
-      <c r="C40" s="55"/>
-      <c r="F40" s="52" t="s">
+      <c r="C40" s="52"/>
+      <c r="F40" s="50" t="s">
         <v>102</v>
       </c>
-      <c r="G40" s="52"/>
+      <c r="G40" s="50"/>
       <c r="I40" s="9" t="s">
         <v>22</v>
       </c>
@@ -2200,7 +2272,7 @@
         <v>119</v>
       </c>
       <c r="G43" s="2"/>
-      <c r="I43" s="51" t="s">
+      <c r="I43" s="49" t="s">
         <v>67</v>
       </c>
     </row>
@@ -2215,7 +2287,7 @@
         <v>120</v>
       </c>
       <c r="G44" s="2"/>
-      <c r="I44" s="51"/>
+      <c r="I44" s="49"/>
     </row>
     <row r="45" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B45" s="2" t="s">
@@ -2390,28 +2462,28 @@
       <c r="S61" s="45"/>
     </row>
     <row r="63" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B63" s="39" t="s">
+      <c r="B63" s="53" t="s">
         <v>63</v>
       </c>
-      <c r="C63" s="39"/>
-      <c r="D63" s="39"/>
-      <c r="E63" s="39"/>
-      <c r="F63" s="39"/>
-      <c r="G63" s="39"/>
-      <c r="H63" s="39"/>
-      <c r="I63" s="39"/>
-      <c r="J63" s="39"/>
-      <c r="K63" s="39"/>
-      <c r="M63" s="39" t="s">
+      <c r="C63" s="53"/>
+      <c r="D63" s="53"/>
+      <c r="E63" s="53"/>
+      <c r="F63" s="53"/>
+      <c r="G63" s="53"/>
+      <c r="H63" s="53"/>
+      <c r="I63" s="53"/>
+      <c r="J63" s="53"/>
+      <c r="K63" s="53"/>
+      <c r="M63" s="53" t="s">
         <v>90</v>
       </c>
-      <c r="N63" s="39"/>
-      <c r="O63" s="39"/>
-      <c r="P63" s="39"/>
-      <c r="R63" s="39" t="s">
+      <c r="N63" s="53"/>
+      <c r="O63" s="53"/>
+      <c r="P63" s="53"/>
+      <c r="R63" s="53" t="s">
         <v>64</v>
       </c>
-      <c r="S63" s="39"/>
+      <c r="S63" s="53"/>
     </row>
     <row r="64" spans="1:19" x14ac:dyDescent="0.25">
       <c r="B64" s="2" t="s">
@@ -2504,40 +2576,62 @@
       <c r="S65" s="2"/>
     </row>
     <row r="68" spans="2:19" x14ac:dyDescent="0.25">
-      <c r="B68" s="51" t="s">
+      <c r="B68" s="49" t="s">
         <v>22</v>
       </c>
-      <c r="C68" s="51"/>
+      <c r="C68" s="49"/>
       <c r="E68" s="9" t="s">
         <v>67</v>
       </c>
-      <c r="G68" s="51" t="s">
+      <c r="G68" s="49" t="s">
         <v>87</v>
       </c>
-      <c r="H68" s="51"/>
+      <c r="H68" s="49"/>
     </row>
     <row r="69" spans="2:19" x14ac:dyDescent="0.25">
-      <c r="B69" s="52">
+      <c r="B69" s="50">
         <f>SUM(B65:K65,M65:P65,R65:S65)</f>
         <v>24</v>
       </c>
-      <c r="C69" s="52"/>
-      <c r="E69" s="53"/>
-      <c r="G69" s="52">
+      <c r="C69" s="50"/>
+      <c r="E69" s="39"/>
+      <c r="G69" s="50">
         <f>50-SUM(B65:K65,M65:P65,R65:S65)</f>
         <v>26</v>
       </c>
-      <c r="H69" s="52"/>
+      <c r="H69" s="50"/>
     </row>
     <row r="70" spans="2:19" x14ac:dyDescent="0.25">
-      <c r="B70" s="52"/>
-      <c r="C70" s="52"/>
-      <c r="E70" s="53"/>
-      <c r="G70" s="52"/>
-      <c r="H70" s="52"/>
+      <c r="B70" s="50"/>
+      <c r="C70" s="50"/>
+      <c r="E70" s="39"/>
+      <c r="G70" s="50"/>
+      <c r="H70" s="50"/>
     </row>
   </sheetData>
   <mergeCells count="38">
+    <mergeCell ref="R63:S63"/>
+    <mergeCell ref="B32:I33"/>
+    <mergeCell ref="B63:K63"/>
+    <mergeCell ref="B60:S61"/>
+    <mergeCell ref="M63:P63"/>
+    <mergeCell ref="N27:N28"/>
+    <mergeCell ref="F26:I26"/>
+    <mergeCell ref="K26:L26"/>
+    <mergeCell ref="B23:L24"/>
+    <mergeCell ref="B26:D26"/>
+    <mergeCell ref="B17:F17"/>
+    <mergeCell ref="H17:J17"/>
+    <mergeCell ref="O17:P17"/>
+    <mergeCell ref="B9:C9"/>
+    <mergeCell ref="B10:C11"/>
+    <mergeCell ref="L17:M17"/>
+    <mergeCell ref="E10:E11"/>
+    <mergeCell ref="E69:E70"/>
+    <mergeCell ref="B68:C68"/>
+    <mergeCell ref="B69:C70"/>
+    <mergeCell ref="G68:H68"/>
+    <mergeCell ref="G69:H70"/>
     <mergeCell ref="R18:R19"/>
     <mergeCell ref="B14:H15"/>
     <mergeCell ref="K5:N5"/>
@@ -2554,28 +2648,6 @@
     <mergeCell ref="E35:H35"/>
     <mergeCell ref="G9:H9"/>
     <mergeCell ref="G10:H11"/>
-    <mergeCell ref="E69:E70"/>
-    <mergeCell ref="B68:C68"/>
-    <mergeCell ref="B69:C70"/>
-    <mergeCell ref="G68:H68"/>
-    <mergeCell ref="G69:H70"/>
-    <mergeCell ref="B17:F17"/>
-    <mergeCell ref="H17:J17"/>
-    <mergeCell ref="O17:P17"/>
-    <mergeCell ref="B9:C9"/>
-    <mergeCell ref="B10:C11"/>
-    <mergeCell ref="L17:M17"/>
-    <mergeCell ref="E10:E11"/>
-    <mergeCell ref="N27:N28"/>
-    <mergeCell ref="F26:I26"/>
-    <mergeCell ref="K26:L26"/>
-    <mergeCell ref="B23:L24"/>
-    <mergeCell ref="B26:D26"/>
-    <mergeCell ref="R63:S63"/>
-    <mergeCell ref="B32:I33"/>
-    <mergeCell ref="B63:K63"/>
-    <mergeCell ref="B60:S61"/>
-    <mergeCell ref="M63:P63"/>
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2648,23 +2720,23 @@
       <c r="R3" s="12"/>
     </row>
     <row r="5" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B5" s="39" t="s">
+      <c r="B5" s="53" t="s">
         <v>18</v>
       </c>
-      <c r="C5" s="39"/>
-      <c r="D5" s="39"/>
-      <c r="E5" s="39"/>
-      <c r="F5" s="39"/>
-      <c r="G5" s="39"/>
+      <c r="C5" s="53"/>
+      <c r="D5" s="53"/>
+      <c r="E5" s="53"/>
+      <c r="F5" s="53"/>
+      <c r="G5" s="53"/>
       <c r="I5" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="K5" s="48" t="s">
+      <c r="K5" s="46" t="s">
         <v>8</v>
       </c>
-      <c r="L5" s="50"/>
-      <c r="M5" s="50"/>
-      <c r="N5" s="49"/>
+      <c r="L5" s="47"/>
+      <c r="M5" s="47"/>
+      <c r="N5" s="48"/>
       <c r="P5" s="4" t="s">
         <v>74</v>
       </c>
@@ -2746,28 +2818,28 @@
       </c>
     </row>
     <row r="9" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B9" s="51" t="s">
+      <c r="B9" s="49" t="s">
         <v>22</v>
       </c>
-      <c r="C9" s="51"/>
+      <c r="C9" s="49"/>
       <c r="E9" s="9" t="s">
         <v>67</v>
       </c>
     </row>
     <row r="10" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B10" s="52">
+      <c r="B10" s="50">
         <f>_xlfn.CEILING.MATH(SUM(B7:G7,I7,K7:N7,P7),1,1)</f>
         <v>110</v>
       </c>
-      <c r="C10" s="52"/>
-      <c r="E10" s="46">
+      <c r="C10" s="50"/>
+      <c r="E10" s="54">
         <v>4</v>
       </c>
     </row>
     <row r="11" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B11" s="52"/>
-      <c r="C11" s="52"/>
-      <c r="E11" s="47"/>
+      <c r="B11" s="50"/>
+      <c r="C11" s="50"/>
+      <c r="E11" s="55"/>
     </row>
     <row r="12" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A12" s="6"/>
@@ -2812,20 +2884,20 @@
       <c r="H15" s="61"/>
     </row>
     <row r="17" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B17" s="39" t="s">
+      <c r="B17" s="53" t="s">
         <v>12</v>
       </c>
-      <c r="C17" s="39"/>
-      <c r="D17" s="39"/>
-      <c r="F17" s="39" t="s">
+      <c r="C17" s="53"/>
+      <c r="D17" s="53"/>
+      <c r="F17" s="53" t="s">
         <v>8</v>
       </c>
-      <c r="G17" s="39"/>
-      <c r="H17" s="39"/>
-      <c r="J17" s="51" t="s">
+      <c r="G17" s="53"/>
+      <c r="H17" s="53"/>
+      <c r="J17" s="49" t="s">
         <v>22</v>
       </c>
-      <c r="K17" s="51"/>
+      <c r="K17" s="49"/>
       <c r="M17" s="9" t="s">
         <v>67</v>
       </c>
@@ -2849,12 +2921,12 @@
       <c r="H18" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="J18" s="52">
+      <c r="J18" s="50">
         <f>SUM(B19:D19,F19:H19)</f>
         <v>93</v>
       </c>
-      <c r="K18" s="52"/>
-      <c r="M18" s="53">
+      <c r="K18" s="50"/>
+      <c r="M18" s="39">
         <v>5</v>
       </c>
     </row>
@@ -2877,9 +2949,9 @@
       <c r="H19" s="2">
         <v>4</v>
       </c>
-      <c r="J19" s="52"/>
-      <c r="K19" s="52"/>
-      <c r="M19" s="53"/>
+      <c r="J19" s="50"/>
+      <c r="K19" s="50"/>
+      <c r="M19" s="39"/>
     </row>
     <row r="21" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A21" s="6"/>
@@ -2930,20 +3002,20 @@
       <c r="K24" s="61"/>
     </row>
     <row r="26" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B26" s="39" t="s">
+      <c r="B26" s="53" t="s">
         <v>17</v>
       </c>
-      <c r="C26" s="39"/>
-      <c r="E26" s="48" t="s">
+      <c r="C26" s="53"/>
+      <c r="E26" s="46" t="s">
         <v>21</v>
       </c>
-      <c r="F26" s="50"/>
-      <c r="G26" s="49"/>
-      <c r="I26" s="39" t="s">
+      <c r="F26" s="47"/>
+      <c r="G26" s="48"/>
+      <c r="I26" s="53" t="s">
         <v>20</v>
       </c>
-      <c r="J26" s="39"/>
-      <c r="K26" s="39"/>
+      <c r="J26" s="53"/>
+      <c r="K26" s="53"/>
       <c r="M26" s="10" t="s">
         <v>22</v>
       </c>
@@ -2983,7 +3055,7 @@
         <v>36</v>
       </c>
       <c r="N27" s="7"/>
-      <c r="O27" s="53">
+      <c r="O27" s="39">
         <v>4</v>
       </c>
       <c r="P27" s="8"/>
@@ -3015,7 +3087,7 @@
       </c>
       <c r="M28" s="62"/>
       <c r="N28" s="7"/>
-      <c r="O28" s="53"/>
+      <c r="O28" s="39"/>
       <c r="P28" s="8"/>
     </row>
     <row r="30" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -3063,17 +3135,17 @@
       <c r="I33" s="61"/>
     </row>
     <row r="35" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B35" s="39" t="s">
+      <c r="B35" s="53" t="s">
         <v>31</v>
       </c>
-      <c r="C35" s="39"/>
-      <c r="D35" s="39"/>
-      <c r="F35" s="39" t="s">
+      <c r="C35" s="53"/>
+      <c r="D35" s="53"/>
+      <c r="F35" s="53" t="s">
         <v>12</v>
       </c>
-      <c r="G35" s="39"/>
-      <c r="H35" s="39"/>
-      <c r="I35" s="39"/>
+      <c r="G35" s="53"/>
+      <c r="H35" s="53"/>
+      <c r="I35" s="53"/>
       <c r="N35" s="7"/>
       <c r="O35" s="7"/>
     </row>
@@ -3130,14 +3202,14 @@
       <c r="O37" s="7"/>
     </row>
     <row r="40" spans="2:15" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B40" s="54" t="s">
+      <c r="B40" s="51" t="s">
         <v>35</v>
       </c>
-      <c r="C40" s="55"/>
-      <c r="F40" s="52" t="s">
+      <c r="C40" s="52"/>
+      <c r="F40" s="50" t="s">
         <v>36</v>
       </c>
-      <c r="G40" s="52"/>
+      <c r="G40" s="50"/>
       <c r="I40" s="9" t="s">
         <v>22</v>
       </c>
@@ -3193,7 +3265,7 @@
       <c r="G43" s="2">
         <v>0.44</v>
       </c>
-      <c r="I43" s="51" t="s">
+      <c r="I43" s="49" t="s">
         <v>67</v>
       </c>
     </row>
@@ -3210,7 +3282,7 @@
       <c r="G44" s="2">
         <v>1</v>
       </c>
-      <c r="I44" s="51"/>
+      <c r="I44" s="49"/>
     </row>
     <row r="45" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B45" s="2" t="s">
@@ -3394,27 +3466,27 @@
       <c r="R59" s="61"/>
     </row>
     <row r="61" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B61" s="39" t="s">
+      <c r="B61" s="53" t="s">
         <v>63</v>
       </c>
-      <c r="C61" s="39"/>
-      <c r="D61" s="39"/>
-      <c r="E61" s="39"/>
-      <c r="F61" s="39"/>
-      <c r="G61" s="39"/>
-      <c r="H61" s="39"/>
-      <c r="I61" s="39"/>
-      <c r="J61" s="39"/>
-      <c r="K61" s="39"/>
-      <c r="M61" s="39" t="s">
+      <c r="C61" s="53"/>
+      <c r="D61" s="53"/>
+      <c r="E61" s="53"/>
+      <c r="F61" s="53"/>
+      <c r="G61" s="53"/>
+      <c r="H61" s="53"/>
+      <c r="I61" s="53"/>
+      <c r="J61" s="53"/>
+      <c r="K61" s="53"/>
+      <c r="M61" s="53" t="s">
         <v>68</v>
       </c>
-      <c r="N61" s="39"/>
-      <c r="O61" s="39"/>
-      <c r="Q61" s="39" t="s">
+      <c r="N61" s="53"/>
+      <c r="O61" s="53"/>
+      <c r="Q61" s="53" t="s">
         <v>64</v>
       </c>
-      <c r="R61" s="39"/>
+      <c r="R61" s="53"/>
     </row>
     <row r="62" spans="1:19" x14ac:dyDescent="0.25">
       <c r="B62" s="2" t="s">
@@ -3511,28 +3583,28 @@
       </c>
     </row>
     <row r="66" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B66" s="51" t="s">
+      <c r="B66" s="49" t="s">
         <v>22</v>
       </c>
-      <c r="C66" s="51"/>
+      <c r="C66" s="49"/>
       <c r="E66" s="9" t="s">
         <v>67</v>
       </c>
     </row>
     <row r="67" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B67" s="52">
+      <c r="B67" s="50">
         <f xml:space="preserve"> SUM(B63:K63,M63:O63,Q63:R63)</f>
         <v>85.5</v>
       </c>
-      <c r="C67" s="52"/>
-      <c r="E67" s="53">
+      <c r="C67" s="50"/>
+      <c r="E67" s="39">
         <v>4.5</v>
       </c>
     </row>
     <row r="68" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B68" s="52"/>
-      <c r="C68" s="52"/>
-      <c r="E68" s="53"/>
+      <c r="B68" s="50"/>
+      <c r="C68" s="50"/>
+      <c r="E68" s="39"/>
     </row>
     <row r="70" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A70" s="6"/>
@@ -3603,10 +3675,10 @@
       <c r="I75" s="4" t="s">
         <v>145</v>
       </c>
-      <c r="K75" s="51" t="s">
+      <c r="K75" s="49" t="s">
         <v>22</v>
       </c>
-      <c r="L75" s="51"/>
+      <c r="L75" s="49"/>
       <c r="N75" s="9" t="s">
         <v>67</v>
       </c>
@@ -3636,11 +3708,11 @@
       <c r="I76" s="2">
         <v>5</v>
       </c>
-      <c r="K76" s="52">
+      <c r="K76" s="50">
         <f>SUM(B76:I76)</f>
         <v>96</v>
       </c>
-      <c r="L76" s="52"/>
+      <c r="L76" s="50"/>
       <c r="N76" s="13">
         <v>5</v>
       </c>
@@ -3668,20 +3740,16 @@
     </row>
   </sheetData>
   <mergeCells count="34">
-    <mergeCell ref="B2:P3"/>
-    <mergeCell ref="B5:G5"/>
-    <mergeCell ref="K5:N5"/>
-    <mergeCell ref="B9:C9"/>
-    <mergeCell ref="B10:C11"/>
-    <mergeCell ref="E10:E11"/>
-    <mergeCell ref="M27:M28"/>
-    <mergeCell ref="O27:O28"/>
-    <mergeCell ref="B14:H15"/>
-    <mergeCell ref="B17:D17"/>
-    <mergeCell ref="F17:H17"/>
-    <mergeCell ref="J17:K17"/>
-    <mergeCell ref="J18:K19"/>
-    <mergeCell ref="M18:M19"/>
+    <mergeCell ref="B72:I73"/>
+    <mergeCell ref="K75:L75"/>
+    <mergeCell ref="K76:L76"/>
+    <mergeCell ref="B58:R59"/>
+    <mergeCell ref="B61:K61"/>
+    <mergeCell ref="M61:O61"/>
+    <mergeCell ref="Q61:R61"/>
+    <mergeCell ref="B66:C66"/>
+    <mergeCell ref="B67:C68"/>
+    <mergeCell ref="E67:E68"/>
     <mergeCell ref="I43:I44"/>
     <mergeCell ref="B23:K24"/>
     <mergeCell ref="B26:C26"/>
@@ -3692,16 +3760,20 @@
     <mergeCell ref="F35:I35"/>
     <mergeCell ref="B40:C40"/>
     <mergeCell ref="F40:G40"/>
-    <mergeCell ref="B72:I73"/>
-    <mergeCell ref="K75:L75"/>
-    <mergeCell ref="K76:L76"/>
-    <mergeCell ref="B58:R59"/>
-    <mergeCell ref="B61:K61"/>
-    <mergeCell ref="M61:O61"/>
-    <mergeCell ref="Q61:R61"/>
-    <mergeCell ref="B66:C66"/>
-    <mergeCell ref="B67:C68"/>
-    <mergeCell ref="E67:E68"/>
+    <mergeCell ref="M27:M28"/>
+    <mergeCell ref="O27:O28"/>
+    <mergeCell ref="B14:H15"/>
+    <mergeCell ref="B17:D17"/>
+    <mergeCell ref="F17:H17"/>
+    <mergeCell ref="J17:K17"/>
+    <mergeCell ref="J18:K19"/>
+    <mergeCell ref="M18:M19"/>
+    <mergeCell ref="B2:P3"/>
+    <mergeCell ref="B5:G5"/>
+    <mergeCell ref="K5:N5"/>
+    <mergeCell ref="B9:C9"/>
+    <mergeCell ref="B10:C11"/>
+    <mergeCell ref="E10:E11"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
@@ -3710,7 +3782,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CEAA0BBB-B59A-4C0E-8304-D0FA810EECB4}">
-  <dimension ref="B1:F35"/>
+  <dimension ref="B1:F39"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="3" max="3" width="11.85546875" style="16" customWidth="1"/>
@@ -3769,19 +3841,19 @@
       </c>
     </row>
     <row r="5" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B5" s="19" t="b">
+      <c r="B5" s="73" t="b">
         <v>0</v>
       </c>
-      <c r="C5" s="21" t="s">
+      <c r="C5" s="74" t="s">
         <v>77</v>
       </c>
-      <c r="D5" s="20">
+      <c r="D5" s="75">
         <v>45817</v>
       </c>
-      <c r="E5" s="18" t="s">
+      <c r="E5" s="76" t="s">
         <v>151</v>
       </c>
-      <c r="F5" s="17" t="s">
+      <c r="F5" s="77" t="s">
         <v>152</v>
       </c>
     </row>
@@ -4154,24 +4226,19 @@
       </c>
     </row>
     <row r="32" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="C32" s="31"/>
-    </row>
-    <row r="33" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B33" s="23" t="b">
-        <v>1</v>
-      </c>
-      <c r="C33" s="29" t="s">
-        <v>78</v>
-      </c>
-      <c r="D33" s="28">
-        <v>45767</v>
-      </c>
-      <c r="E33" s="27" t="s">
-        <v>181</v>
-      </c>
-      <c r="F33" s="27" t="s">
-        <v>190</v>
-      </c>
+      <c r="B32" s="68" t="b">
+        <v>0</v>
+      </c>
+      <c r="C32" s="69" t="s">
+        <v>76</v>
+      </c>
+      <c r="D32" s="70">
+        <v>45815</v>
+      </c>
+      <c r="E32" s="71" t="s">
+        <v>218</v>
+      </c>
+      <c r="F32" s="72"/>
     </row>
     <row r="34" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B34" s="23" t="b">
@@ -4181,27 +4248,78 @@
         <v>78</v>
       </c>
       <c r="D34" s="28">
+        <v>45767</v>
+      </c>
+      <c r="E34" s="27" t="s">
+        <v>181</v>
+      </c>
+      <c r="F34" s="27" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="35" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B35" s="23" t="b">
+        <v>1</v>
+      </c>
+      <c r="C35" s="29" t="s">
+        <v>78</v>
+      </c>
+      <c r="D35" s="28">
         <v>45775</v>
       </c>
-      <c r="E34" s="27" t="s">
+      <c r="E35" s="27" t="s">
         <v>149</v>
       </c>
     </row>
-    <row r="35" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B35" s="19" t="b">
+    <row r="36" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B36" s="19" t="b">
         <v>0</v>
       </c>
-      <c r="C35" s="21" t="s">
+      <c r="C36" s="21" t="s">
         <v>78</v>
       </c>
-      <c r="D35" s="20">
+      <c r="D36" s="20">
         <v>45794</v>
       </c>
-      <c r="E35" s="17" t="s">
+      <c r="E36" s="17" t="s">
         <v>214</v>
       </c>
-      <c r="F35" s="17" t="s">
+      <c r="F36" s="17" t="s">
         <v>213</v>
+      </c>
+    </row>
+    <row r="38" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B38" s="19" t="b">
+        <v>0</v>
+      </c>
+      <c r="C38" s="21" t="s">
+        <v>79</v>
+      </c>
+      <c r="D38" s="20">
+        <v>45797</v>
+      </c>
+      <c r="E38" s="17" t="s">
+        <v>219</v>
+      </c>
+      <c r="F38" s="17" t="s">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="39" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B39" s="19" t="b">
+        <v>0</v>
+      </c>
+      <c r="C39" s="21" t="s">
+        <v>79</v>
+      </c>
+      <c r="D39" s="20">
+        <v>45804</v>
+      </c>
+      <c r="E39" s="17" t="s">
+        <v>222</v>
+      </c>
+      <c r="F39" s="17" t="s">
+        <v>221</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Colloquium 2 (MAT3) added to schedule
</commit_message>
<xml_diff>
--- a/IoT-points-schedule.xlsx
+++ b/IoT-points-schedule.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\dodo\Desktop\IoT-studies\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CF068950-203A-42A1-AF03-542A2F69086C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{166723B2-D992-4CD2-9CCF-90079B51C210}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="25440" windowHeight="15390" xr2:uid="{F85F5544-1FE8-4920-A5D4-192A98B113BD}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="25440" windowHeight="15390" activeTab="2" xr2:uid="{F85F5544-1FE8-4920-A5D4-192A98B113BD}"/>
   </bookViews>
   <sheets>
     <sheet name="II-semestr-25L" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="348" uniqueCount="223">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="351" uniqueCount="224">
   <si>
     <t>1. Krypto</t>
   </si>
@@ -708,6 +708,9 @@
   </si>
   <si>
     <t>Projekt</t>
+  </si>
+  <si>
+    <t>Przekształcenia wektorowe, liniowe, itd..</t>
   </si>
 </sst>
 </file>
@@ -1083,7 +1086,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="78">
+  <cellXfs count="77">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1205,56 +1208,75 @@
     <xf numFmtId="0" fontId="6" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1">
+      <extLst>
+        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
+          <xfpb:xfComplement i="0"/>
+        </ext>
+      </extLst>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="7" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="7" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1306,28 +1328,6 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1">
-      <extLst>
-        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
-          <xfpb:xfComplement i="0"/>
-        </ext>
-      </extLst>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="7" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="7" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -1718,60 +1718,60 @@
   <sheetData>
     <row r="1" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="2" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B2" s="40" t="s">
+      <c r="B2" s="45" t="s">
         <v>76</v>
       </c>
-      <c r="C2" s="41"/>
-      <c r="D2" s="41"/>
-      <c r="E2" s="41"/>
-      <c r="F2" s="41"/>
-      <c r="G2" s="41"/>
-      <c r="H2" s="41"/>
-      <c r="I2" s="41"/>
-      <c r="J2" s="41"/>
-      <c r="K2" s="41"/>
-      <c r="L2" s="41"/>
-      <c r="M2" s="41"/>
-      <c r="N2" s="41"/>
-      <c r="O2" s="41"/>
-      <c r="P2" s="42"/>
+      <c r="C2" s="46"/>
+      <c r="D2" s="46"/>
+      <c r="E2" s="46"/>
+      <c r="F2" s="46"/>
+      <c r="G2" s="46"/>
+      <c r="H2" s="46"/>
+      <c r="I2" s="46"/>
+      <c r="J2" s="46"/>
+      <c r="K2" s="46"/>
+      <c r="L2" s="46"/>
+      <c r="M2" s="46"/>
+      <c r="N2" s="46"/>
+      <c r="O2" s="46"/>
+      <c r="P2" s="47"/>
     </row>
     <row r="3" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B3" s="43"/>
-      <c r="C3" s="44"/>
-      <c r="D3" s="44"/>
-      <c r="E3" s="44"/>
-      <c r="F3" s="44"/>
-      <c r="G3" s="44"/>
-      <c r="H3" s="44"/>
-      <c r="I3" s="44"/>
-      <c r="J3" s="44"/>
-      <c r="K3" s="44"/>
-      <c r="L3" s="44"/>
-      <c r="M3" s="44"/>
-      <c r="N3" s="44"/>
-      <c r="O3" s="44"/>
-      <c r="P3" s="45"/>
+      <c r="B3" s="48"/>
+      <c r="C3" s="49"/>
+      <c r="D3" s="49"/>
+      <c r="E3" s="49"/>
+      <c r="F3" s="49"/>
+      <c r="G3" s="49"/>
+      <c r="H3" s="49"/>
+      <c r="I3" s="49"/>
+      <c r="J3" s="49"/>
+      <c r="K3" s="49"/>
+      <c r="L3" s="49"/>
+      <c r="M3" s="49"/>
+      <c r="N3" s="49"/>
+      <c r="O3" s="49"/>
+      <c r="P3" s="50"/>
       <c r="R3" s="12"/>
     </row>
     <row r="5" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B5" s="46" t="s">
+      <c r="B5" s="53" t="s">
         <v>83</v>
       </c>
-      <c r="C5" s="47"/>
-      <c r="D5" s="47"/>
-      <c r="E5" s="47"/>
-      <c r="F5" s="48"/>
-      <c r="H5" s="46" t="s">
+      <c r="C5" s="55"/>
+      <c r="D5" s="55"/>
+      <c r="E5" s="55"/>
+      <c r="F5" s="54"/>
+      <c r="H5" s="53" t="s">
         <v>82</v>
       </c>
-      <c r="I5" s="48"/>
-      <c r="K5" s="46" t="s">
+      <c r="I5" s="54"/>
+      <c r="K5" s="53" t="s">
         <v>8</v>
       </c>
-      <c r="L5" s="47"/>
-      <c r="M5" s="47"/>
-      <c r="N5" s="48"/>
+      <c r="L5" s="55"/>
+      <c r="M5" s="55"/>
+      <c r="N5" s="54"/>
       <c r="P5" s="4" t="s">
         <v>74</v>
       </c>
@@ -1834,42 +1834,42 @@
       <c r="L7" s="2"/>
       <c r="M7" s="2"/>
       <c r="N7" s="2">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="P7" s="2"/>
     </row>
     <row r="9" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B9" s="49" t="s">
+      <c r="B9" s="56" t="s">
         <v>22</v>
       </c>
-      <c r="C9" s="49"/>
+      <c r="C9" s="56"/>
       <c r="E9" s="9" t="s">
         <v>67</v>
       </c>
-      <c r="G9" s="49" t="s">
+      <c r="G9" s="56" t="s">
         <v>87</v>
       </c>
-      <c r="H9" s="49"/>
+      <c r="H9" s="56"/>
     </row>
     <row r="10" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B10" s="50">
+      <c r="B10" s="57">
         <f>SUM(B7:F7,H7:I7,K7:N7,P7)</f>
-        <v>24.7</v>
-      </c>
-      <c r="C10" s="50"/>
-      <c r="E10" s="54"/>
-      <c r="G10" s="50">
+        <v>25.7</v>
+      </c>
+      <c r="C10" s="57"/>
+      <c r="E10" s="51"/>
+      <c r="G10" s="57">
         <f>66-SUM(B7:F7,H7:I7,K7:N7,P7)</f>
-        <v>41.3</v>
-      </c>
-      <c r="H10" s="50"/>
+        <v>40.299999999999997</v>
+      </c>
+      <c r="H10" s="57"/>
     </row>
     <row r="11" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B11" s="50"/>
-      <c r="C11" s="50"/>
-      <c r="E11" s="55"/>
-      <c r="G11" s="50"/>
-      <c r="H11" s="50"/>
+      <c r="B11" s="57"/>
+      <c r="C11" s="57"/>
+      <c r="E11" s="52"/>
+      <c r="G11" s="57"/>
+      <c r="H11" s="57"/>
     </row>
     <row r="12" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A12" s="6"/>
@@ -1894,46 +1894,46 @@
     </row>
     <row r="13" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="14" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B14" s="40" t="s">
+      <c r="B14" s="45" t="s">
         <v>77</v>
       </c>
-      <c r="C14" s="41"/>
-      <c r="D14" s="41"/>
-      <c r="E14" s="41"/>
-      <c r="F14" s="41"/>
-      <c r="G14" s="41"/>
-      <c r="H14" s="42"/>
+      <c r="C14" s="46"/>
+      <c r="D14" s="46"/>
+      <c r="E14" s="46"/>
+      <c r="F14" s="46"/>
+      <c r="G14" s="46"/>
+      <c r="H14" s="47"/>
     </row>
     <row r="15" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B15" s="43"/>
-      <c r="C15" s="44"/>
-      <c r="D15" s="44"/>
-      <c r="E15" s="44"/>
-      <c r="F15" s="44"/>
-      <c r="G15" s="44"/>
-      <c r="H15" s="45"/>
+      <c r="B15" s="48"/>
+      <c r="C15" s="49"/>
+      <c r="D15" s="49"/>
+      <c r="E15" s="49"/>
+      <c r="F15" s="49"/>
+      <c r="G15" s="49"/>
+      <c r="H15" s="50"/>
     </row>
     <row r="17" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B17" s="53" t="s">
+      <c r="B17" s="44" t="s">
         <v>91</v>
       </c>
-      <c r="C17" s="53"/>
-      <c r="D17" s="53"/>
-      <c r="E17" s="53"/>
-      <c r="F17" s="53"/>
-      <c r="H17" s="46" t="s">
+      <c r="C17" s="44"/>
+      <c r="D17" s="44"/>
+      <c r="E17" s="44"/>
+      <c r="F17" s="44"/>
+      <c r="H17" s="53" t="s">
         <v>97</v>
       </c>
-      <c r="I17" s="47"/>
-      <c r="J17" s="48"/>
-      <c r="L17" s="49" t="s">
+      <c r="I17" s="55"/>
+      <c r="J17" s="54"/>
+      <c r="L17" s="56" t="s">
         <v>22</v>
       </c>
-      <c r="M17" s="49"/>
-      <c r="O17" s="49" t="s">
+      <c r="M17" s="56"/>
+      <c r="O17" s="56" t="s">
         <v>87</v>
       </c>
-      <c r="P17" s="49"/>
+      <c r="P17" s="56"/>
       <c r="R17" s="9" t="s">
         <v>67</v>
       </c>
@@ -1963,17 +1963,17 @@
       <c r="J18" s="3" t="s">
         <v>95</v>
       </c>
-      <c r="L18" s="50">
+      <c r="L18" s="57">
         <f>SUM(B19:F19,H19:J19)</f>
         <v>29.5</v>
       </c>
-      <c r="M18" s="50"/>
-      <c r="O18" s="50">
+      <c r="M18" s="57"/>
+      <c r="O18" s="57">
         <f>50-SUM(B19:F19,H19:J19)</f>
         <v>20.5</v>
       </c>
-      <c r="P18" s="50"/>
-      <c r="R18" s="39"/>
+      <c r="P18" s="57"/>
+      <c r="R18" s="58"/>
     </row>
     <row r="19" spans="1:19" x14ac:dyDescent="0.25">
       <c r="B19" s="2"/>
@@ -1988,11 +1988,11 @@
         <v>26.5</v>
       </c>
       <c r="J19" s="2"/>
-      <c r="L19" s="50"/>
-      <c r="M19" s="50"/>
-      <c r="O19" s="50"/>
-      <c r="P19" s="50"/>
-      <c r="R19" s="39"/>
+      <c r="L19" s="57"/>
+      <c r="M19" s="57"/>
+      <c r="O19" s="57"/>
+      <c r="P19" s="57"/>
+      <c r="R19" s="58"/>
     </row>
     <row r="21" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A21" s="6"/>
@@ -2017,56 +2017,56 @@
     </row>
     <row r="22" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="23" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B23" s="40" t="s">
+      <c r="B23" s="45" t="s">
         <v>79</v>
       </c>
-      <c r="C23" s="41"/>
-      <c r="D23" s="41"/>
-      <c r="E23" s="41"/>
-      <c r="F23" s="41"/>
-      <c r="G23" s="41"/>
-      <c r="H23" s="41"/>
-      <c r="I23" s="41"/>
-      <c r="J23" s="41"/>
-      <c r="K23" s="41"/>
-      <c r="L23" s="42"/>
-      <c r="N23" s="50" t="s">
+      <c r="C23" s="46"/>
+      <c r="D23" s="46"/>
+      <c r="E23" s="46"/>
+      <c r="F23" s="46"/>
+      <c r="G23" s="46"/>
+      <c r="H23" s="46"/>
+      <c r="I23" s="46"/>
+      <c r="J23" s="46"/>
+      <c r="K23" s="46"/>
+      <c r="L23" s="47"/>
+      <c r="N23" s="57" t="s">
         <v>131</v>
       </c>
-      <c r="O23" s="50"/>
+      <c r="O23" s="57"/>
     </row>
     <row r="24" spans="1:19" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B24" s="43"/>
-      <c r="C24" s="44"/>
-      <c r="D24" s="44"/>
-      <c r="E24" s="44"/>
-      <c r="F24" s="44"/>
-      <c r="G24" s="44"/>
-      <c r="H24" s="44"/>
-      <c r="I24" s="44"/>
-      <c r="J24" s="44"/>
-      <c r="K24" s="44"/>
-      <c r="L24" s="45"/>
-      <c r="N24" s="50"/>
-      <c r="O24" s="50"/>
+      <c r="B24" s="48"/>
+      <c r="C24" s="49"/>
+      <c r="D24" s="49"/>
+      <c r="E24" s="49"/>
+      <c r="F24" s="49"/>
+      <c r="G24" s="49"/>
+      <c r="H24" s="49"/>
+      <c r="I24" s="49"/>
+      <c r="J24" s="49"/>
+      <c r="K24" s="49"/>
+      <c r="L24" s="50"/>
+      <c r="N24" s="57"/>
+      <c r="O24" s="57"/>
     </row>
     <row r="26" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B26" s="53" t="s">
+      <c r="B26" s="44" t="s">
         <v>129</v>
       </c>
-      <c r="C26" s="53"/>
-      <c r="D26" s="53"/>
-      <c r="F26" s="53" t="s">
+      <c r="C26" s="44"/>
+      <c r="D26" s="44"/>
+      <c r="F26" s="44" t="s">
         <v>210</v>
       </c>
-      <c r="G26" s="53"/>
-      <c r="H26" s="53"/>
-      <c r="I26" s="53"/>
+      <c r="G26" s="44"/>
+      <c r="H26" s="44"/>
+      <c r="I26" s="44"/>
       <c r="J26" s="7"/>
-      <c r="K26" s="46" t="s">
+      <c r="K26" s="53" t="s">
         <v>128</v>
       </c>
-      <c r="L26" s="48"/>
+      <c r="L26" s="54"/>
       <c r="N26" s="9" t="s">
         <v>67</v>
       </c>
@@ -2099,7 +2099,7 @@
       <c r="L27" s="2" t="s">
         <v>127</v>
       </c>
-      <c r="N27" s="54"/>
+      <c r="N27" s="51"/>
     </row>
     <row r="28" spans="1:19" x14ac:dyDescent="0.25">
       <c r="B28" s="2">
@@ -2117,7 +2117,7 @@
       <c r="I28" s="2"/>
       <c r="K28" s="2"/>
       <c r="L28" s="2"/>
-      <c r="N28" s="55"/>
+      <c r="N28" s="52"/>
     </row>
     <row r="30" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A30" s="6"/>
@@ -2142,39 +2142,39 @@
     </row>
     <row r="31" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="32" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B32" s="40" t="s">
+      <c r="B32" s="45" t="s">
         <v>78</v>
       </c>
-      <c r="C32" s="41"/>
-      <c r="D32" s="41"/>
-      <c r="E32" s="41"/>
-      <c r="F32" s="41"/>
-      <c r="G32" s="41"/>
-      <c r="H32" s="41"/>
-      <c r="I32" s="42"/>
+      <c r="C32" s="46"/>
+      <c r="D32" s="46"/>
+      <c r="E32" s="46"/>
+      <c r="F32" s="46"/>
+      <c r="G32" s="46"/>
+      <c r="H32" s="46"/>
+      <c r="I32" s="47"/>
     </row>
     <row r="33" spans="2:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B33" s="43"/>
-      <c r="C33" s="44"/>
-      <c r="D33" s="44"/>
-      <c r="E33" s="44"/>
-      <c r="F33" s="44"/>
-      <c r="G33" s="44"/>
-      <c r="H33" s="44"/>
-      <c r="I33" s="45"/>
+      <c r="B33" s="48"/>
+      <c r="C33" s="49"/>
+      <c r="D33" s="49"/>
+      <c r="E33" s="49"/>
+      <c r="F33" s="49"/>
+      <c r="G33" s="49"/>
+      <c r="H33" s="49"/>
+      <c r="I33" s="50"/>
     </row>
     <row r="35" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B35" s="53" t="s">
+      <c r="B35" s="44" t="s">
         <v>98</v>
       </c>
-      <c r="C35" s="53"/>
+      <c r="C35" s="44"/>
       <c r="D35" s="7"/>
-      <c r="E35" s="46" t="s">
+      <c r="E35" s="53" t="s">
         <v>146</v>
       </c>
-      <c r="F35" s="47"/>
-      <c r="G35" s="47"/>
-      <c r="H35" s="48"/>
+      <c r="F35" s="55"/>
+      <c r="G35" s="55"/>
+      <c r="H35" s="54"/>
     </row>
     <row r="36" spans="2:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B36" s="2" t="s">
@@ -2215,14 +2215,14 @@
       <c r="O37" s="7"/>
     </row>
     <row r="40" spans="2:15" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B40" s="51" t="s">
+      <c r="B40" s="59" t="s">
         <v>126</v>
       </c>
-      <c r="C40" s="52"/>
-      <c r="F40" s="50" t="s">
+      <c r="C40" s="60"/>
+      <c r="F40" s="57" t="s">
         <v>102</v>
       </c>
-      <c r="G40" s="50"/>
+      <c r="G40" s="57"/>
       <c r="I40" s="9" t="s">
         <v>22</v>
       </c>
@@ -2272,7 +2272,7 @@
         <v>119</v>
       </c>
       <c r="G43" s="2"/>
-      <c r="I43" s="49" t="s">
+      <c r="I43" s="56" t="s">
         <v>67</v>
       </c>
     </row>
@@ -2287,7 +2287,7 @@
         <v>120</v>
       </c>
       <c r="G44" s="2"/>
-      <c r="I44" s="49"/>
+      <c r="I44" s="56"/>
     </row>
     <row r="45" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B45" s="2" t="s">
@@ -2420,70 +2420,70 @@
     </row>
     <row r="59" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="60" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B60" s="40" t="s">
+      <c r="B60" s="45" t="s">
         <v>80</v>
       </c>
-      <c r="C60" s="41"/>
-      <c r="D60" s="41"/>
-      <c r="E60" s="41"/>
-      <c r="F60" s="41"/>
-      <c r="G60" s="41"/>
-      <c r="H60" s="41"/>
-      <c r="I60" s="41"/>
-      <c r="J60" s="41"/>
-      <c r="K60" s="41"/>
-      <c r="L60" s="41"/>
-      <c r="M60" s="41"/>
-      <c r="N60" s="41"/>
-      <c r="O60" s="41"/>
-      <c r="P60" s="41"/>
-      <c r="Q60" s="41"/>
-      <c r="R60" s="41"/>
-      <c r="S60" s="42"/>
+      <c r="C60" s="46"/>
+      <c r="D60" s="46"/>
+      <c r="E60" s="46"/>
+      <c r="F60" s="46"/>
+      <c r="G60" s="46"/>
+      <c r="H60" s="46"/>
+      <c r="I60" s="46"/>
+      <c r="J60" s="46"/>
+      <c r="K60" s="46"/>
+      <c r="L60" s="46"/>
+      <c r="M60" s="46"/>
+      <c r="N60" s="46"/>
+      <c r="O60" s="46"/>
+      <c r="P60" s="46"/>
+      <c r="Q60" s="46"/>
+      <c r="R60" s="46"/>
+      <c r="S60" s="47"/>
     </row>
     <row r="61" spans="1:19" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B61" s="43"/>
-      <c r="C61" s="44"/>
-      <c r="D61" s="44"/>
-      <c r="E61" s="44"/>
-      <c r="F61" s="44"/>
-      <c r="G61" s="44"/>
-      <c r="H61" s="44"/>
-      <c r="I61" s="44"/>
-      <c r="J61" s="44"/>
-      <c r="K61" s="44"/>
-      <c r="L61" s="44"/>
-      <c r="M61" s="44"/>
-      <c r="N61" s="44"/>
-      <c r="O61" s="44"/>
-      <c r="P61" s="44"/>
-      <c r="Q61" s="44"/>
-      <c r="R61" s="44"/>
-      <c r="S61" s="45"/>
+      <c r="B61" s="48"/>
+      <c r="C61" s="49"/>
+      <c r="D61" s="49"/>
+      <c r="E61" s="49"/>
+      <c r="F61" s="49"/>
+      <c r="G61" s="49"/>
+      <c r="H61" s="49"/>
+      <c r="I61" s="49"/>
+      <c r="J61" s="49"/>
+      <c r="K61" s="49"/>
+      <c r="L61" s="49"/>
+      <c r="M61" s="49"/>
+      <c r="N61" s="49"/>
+      <c r="O61" s="49"/>
+      <c r="P61" s="49"/>
+      <c r="Q61" s="49"/>
+      <c r="R61" s="49"/>
+      <c r="S61" s="50"/>
     </row>
     <row r="63" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B63" s="53" t="s">
+      <c r="B63" s="44" t="s">
         <v>63</v>
       </c>
-      <c r="C63" s="53"/>
-      <c r="D63" s="53"/>
-      <c r="E63" s="53"/>
-      <c r="F63" s="53"/>
-      <c r="G63" s="53"/>
-      <c r="H63" s="53"/>
-      <c r="I63" s="53"/>
-      <c r="J63" s="53"/>
-      <c r="K63" s="53"/>
-      <c r="M63" s="53" t="s">
+      <c r="C63" s="44"/>
+      <c r="D63" s="44"/>
+      <c r="E63" s="44"/>
+      <c r="F63" s="44"/>
+      <c r="G63" s="44"/>
+      <c r="H63" s="44"/>
+      <c r="I63" s="44"/>
+      <c r="J63" s="44"/>
+      <c r="K63" s="44"/>
+      <c r="M63" s="44" t="s">
         <v>90</v>
       </c>
-      <c r="N63" s="53"/>
-      <c r="O63" s="53"/>
-      <c r="P63" s="53"/>
-      <c r="R63" s="53" t="s">
+      <c r="N63" s="44"/>
+      <c r="O63" s="44"/>
+      <c r="P63" s="44"/>
+      <c r="R63" s="44" t="s">
         <v>64</v>
       </c>
-      <c r="S63" s="53"/>
+      <c r="S63" s="44"/>
     </row>
     <row r="64" spans="1:19" x14ac:dyDescent="0.25">
       <c r="B64" s="2" t="s">
@@ -2576,62 +2576,40 @@
       <c r="S65" s="2"/>
     </row>
     <row r="68" spans="2:19" x14ac:dyDescent="0.25">
-      <c r="B68" s="49" t="s">
+      <c r="B68" s="56" t="s">
         <v>22</v>
       </c>
-      <c r="C68" s="49"/>
+      <c r="C68" s="56"/>
       <c r="E68" s="9" t="s">
         <v>67</v>
       </c>
-      <c r="G68" s="49" t="s">
+      <c r="G68" s="56" t="s">
         <v>87</v>
       </c>
-      <c r="H68" s="49"/>
+      <c r="H68" s="56"/>
     </row>
     <row r="69" spans="2:19" x14ac:dyDescent="0.25">
-      <c r="B69" s="50">
+      <c r="B69" s="57">
         <f>SUM(B65:K65,M65:P65,R65:S65)</f>
         <v>24</v>
       </c>
-      <c r="C69" s="50"/>
-      <c r="E69" s="39"/>
-      <c r="G69" s="50">
+      <c r="C69" s="57"/>
+      <c r="E69" s="58"/>
+      <c r="G69" s="57">
         <f>50-SUM(B65:K65,M65:P65,R65:S65)</f>
         <v>26</v>
       </c>
-      <c r="H69" s="50"/>
+      <c r="H69" s="57"/>
     </row>
     <row r="70" spans="2:19" x14ac:dyDescent="0.25">
-      <c r="B70" s="50"/>
-      <c r="C70" s="50"/>
-      <c r="E70" s="39"/>
-      <c r="G70" s="50"/>
-      <c r="H70" s="50"/>
+      <c r="B70" s="57"/>
+      <c r="C70" s="57"/>
+      <c r="E70" s="58"/>
+      <c r="G70" s="57"/>
+      <c r="H70" s="57"/>
     </row>
   </sheetData>
   <mergeCells count="38">
-    <mergeCell ref="R63:S63"/>
-    <mergeCell ref="B32:I33"/>
-    <mergeCell ref="B63:K63"/>
-    <mergeCell ref="B60:S61"/>
-    <mergeCell ref="M63:P63"/>
-    <mergeCell ref="N27:N28"/>
-    <mergeCell ref="F26:I26"/>
-    <mergeCell ref="K26:L26"/>
-    <mergeCell ref="B23:L24"/>
-    <mergeCell ref="B26:D26"/>
-    <mergeCell ref="B17:F17"/>
-    <mergeCell ref="H17:J17"/>
-    <mergeCell ref="O17:P17"/>
-    <mergeCell ref="B9:C9"/>
-    <mergeCell ref="B10:C11"/>
-    <mergeCell ref="L17:M17"/>
-    <mergeCell ref="E10:E11"/>
-    <mergeCell ref="E69:E70"/>
-    <mergeCell ref="B68:C68"/>
-    <mergeCell ref="B69:C70"/>
-    <mergeCell ref="G68:H68"/>
-    <mergeCell ref="G69:H70"/>
     <mergeCell ref="R18:R19"/>
     <mergeCell ref="B14:H15"/>
     <mergeCell ref="K5:N5"/>
@@ -2648,6 +2626,28 @@
     <mergeCell ref="E35:H35"/>
     <mergeCell ref="G9:H9"/>
     <mergeCell ref="G10:H11"/>
+    <mergeCell ref="E69:E70"/>
+    <mergeCell ref="B68:C68"/>
+    <mergeCell ref="B69:C70"/>
+    <mergeCell ref="G68:H68"/>
+    <mergeCell ref="G69:H70"/>
+    <mergeCell ref="B17:F17"/>
+    <mergeCell ref="H17:J17"/>
+    <mergeCell ref="O17:P17"/>
+    <mergeCell ref="B9:C9"/>
+    <mergeCell ref="B10:C11"/>
+    <mergeCell ref="L17:M17"/>
+    <mergeCell ref="E10:E11"/>
+    <mergeCell ref="N27:N28"/>
+    <mergeCell ref="F26:I26"/>
+    <mergeCell ref="K26:L26"/>
+    <mergeCell ref="B23:L24"/>
+    <mergeCell ref="B26:D26"/>
+    <mergeCell ref="R63:S63"/>
+    <mergeCell ref="B32:I33"/>
+    <mergeCell ref="B63:K63"/>
+    <mergeCell ref="B60:S61"/>
+    <mergeCell ref="M63:P63"/>
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2683,60 +2683,60 @@
   <sheetData>
     <row r="1" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="2" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B2" s="56" t="s">
+      <c r="B2" s="61" t="s">
         <v>132</v>
       </c>
-      <c r="C2" s="57"/>
-      <c r="D2" s="57"/>
-      <c r="E2" s="57"/>
-      <c r="F2" s="57"/>
-      <c r="G2" s="57"/>
-      <c r="H2" s="57"/>
-      <c r="I2" s="57"/>
-      <c r="J2" s="57"/>
-      <c r="K2" s="57"/>
-      <c r="L2" s="57"/>
-      <c r="M2" s="57"/>
-      <c r="N2" s="57"/>
-      <c r="O2" s="57"/>
-      <c r="P2" s="58"/>
+      <c r="C2" s="62"/>
+      <c r="D2" s="62"/>
+      <c r="E2" s="62"/>
+      <c r="F2" s="62"/>
+      <c r="G2" s="62"/>
+      <c r="H2" s="62"/>
+      <c r="I2" s="62"/>
+      <c r="J2" s="62"/>
+      <c r="K2" s="62"/>
+      <c r="L2" s="62"/>
+      <c r="M2" s="62"/>
+      <c r="N2" s="62"/>
+      <c r="O2" s="62"/>
+      <c r="P2" s="63"/>
     </row>
     <row r="3" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B3" s="59"/>
-      <c r="C3" s="60"/>
-      <c r="D3" s="60"/>
-      <c r="E3" s="60"/>
-      <c r="F3" s="60"/>
-      <c r="G3" s="60"/>
-      <c r="H3" s="60"/>
-      <c r="I3" s="60"/>
-      <c r="J3" s="60"/>
-      <c r="K3" s="60"/>
-      <c r="L3" s="60"/>
-      <c r="M3" s="60"/>
-      <c r="N3" s="60"/>
-      <c r="O3" s="60"/>
-      <c r="P3" s="61"/>
+      <c r="B3" s="64"/>
+      <c r="C3" s="65"/>
+      <c r="D3" s="65"/>
+      <c r="E3" s="65"/>
+      <c r="F3" s="65"/>
+      <c r="G3" s="65"/>
+      <c r="H3" s="65"/>
+      <c r="I3" s="65"/>
+      <c r="J3" s="65"/>
+      <c r="K3" s="65"/>
+      <c r="L3" s="65"/>
+      <c r="M3" s="65"/>
+      <c r="N3" s="65"/>
+      <c r="O3" s="65"/>
+      <c r="P3" s="66"/>
       <c r="R3" s="12"/>
     </row>
     <row r="5" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B5" s="53" t="s">
+      <c r="B5" s="44" t="s">
         <v>18</v>
       </c>
-      <c r="C5" s="53"/>
-      <c r="D5" s="53"/>
-      <c r="E5" s="53"/>
-      <c r="F5" s="53"/>
-      <c r="G5" s="53"/>
+      <c r="C5" s="44"/>
+      <c r="D5" s="44"/>
+      <c r="E5" s="44"/>
+      <c r="F5" s="44"/>
+      <c r="G5" s="44"/>
       <c r="I5" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="K5" s="46" t="s">
+      <c r="K5" s="53" t="s">
         <v>8</v>
       </c>
-      <c r="L5" s="47"/>
-      <c r="M5" s="47"/>
-      <c r="N5" s="48"/>
+      <c r="L5" s="55"/>
+      <c r="M5" s="55"/>
+      <c r="N5" s="54"/>
       <c r="P5" s="4" t="s">
         <v>74</v>
       </c>
@@ -2818,28 +2818,28 @@
       </c>
     </row>
     <row r="9" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B9" s="49" t="s">
+      <c r="B9" s="56" t="s">
         <v>22</v>
       </c>
-      <c r="C9" s="49"/>
+      <c r="C9" s="56"/>
       <c r="E9" s="9" t="s">
         <v>67</v>
       </c>
     </row>
     <row r="10" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B10" s="50">
+      <c r="B10" s="57">
         <f>_xlfn.CEILING.MATH(SUM(B7:G7,I7,K7:N7,P7),1,1)</f>
         <v>110</v>
       </c>
-      <c r="C10" s="50"/>
-      <c r="E10" s="54">
+      <c r="C10" s="57"/>
+      <c r="E10" s="51">
         <v>4</v>
       </c>
     </row>
     <row r="11" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B11" s="50"/>
-      <c r="C11" s="50"/>
-      <c r="E11" s="55"/>
+      <c r="B11" s="57"/>
+      <c r="C11" s="57"/>
+      <c r="E11" s="52"/>
     </row>
     <row r="12" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A12" s="6"/>
@@ -2864,40 +2864,40 @@
     </row>
     <row r="13" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="14" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B14" s="56" t="s">
+      <c r="B14" s="61" t="s">
         <v>133</v>
       </c>
-      <c r="C14" s="57"/>
-      <c r="D14" s="57"/>
-      <c r="E14" s="57"/>
-      <c r="F14" s="57"/>
-      <c r="G14" s="57"/>
-      <c r="H14" s="58"/>
+      <c r="C14" s="62"/>
+      <c r="D14" s="62"/>
+      <c r="E14" s="62"/>
+      <c r="F14" s="62"/>
+      <c r="G14" s="62"/>
+      <c r="H14" s="63"/>
     </row>
     <row r="15" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B15" s="59"/>
-      <c r="C15" s="60"/>
-      <c r="D15" s="60"/>
-      <c r="E15" s="60"/>
-      <c r="F15" s="60"/>
-      <c r="G15" s="60"/>
-      <c r="H15" s="61"/>
+      <c r="B15" s="64"/>
+      <c r="C15" s="65"/>
+      <c r="D15" s="65"/>
+      <c r="E15" s="65"/>
+      <c r="F15" s="65"/>
+      <c r="G15" s="65"/>
+      <c r="H15" s="66"/>
     </row>
     <row r="17" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B17" s="53" t="s">
+      <c r="B17" s="44" t="s">
         <v>12</v>
       </c>
-      <c r="C17" s="53"/>
-      <c r="D17" s="53"/>
-      <c r="F17" s="53" t="s">
+      <c r="C17" s="44"/>
+      <c r="D17" s="44"/>
+      <c r="F17" s="44" t="s">
         <v>8</v>
       </c>
-      <c r="G17" s="53"/>
-      <c r="H17" s="53"/>
-      <c r="J17" s="49" t="s">
+      <c r="G17" s="44"/>
+      <c r="H17" s="44"/>
+      <c r="J17" s="56" t="s">
         <v>22</v>
       </c>
-      <c r="K17" s="49"/>
+      <c r="K17" s="56"/>
       <c r="M17" s="9" t="s">
         <v>67</v>
       </c>
@@ -2921,12 +2921,12 @@
       <c r="H18" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="J18" s="50">
+      <c r="J18" s="57">
         <f>SUM(B19:D19,F19:H19)</f>
         <v>93</v>
       </c>
-      <c r="K18" s="50"/>
-      <c r="M18" s="39">
+      <c r="K18" s="57"/>
+      <c r="M18" s="58">
         <v>5</v>
       </c>
     </row>
@@ -2949,9 +2949,9 @@
       <c r="H19" s="2">
         <v>4</v>
       </c>
-      <c r="J19" s="50"/>
-      <c r="K19" s="50"/>
-      <c r="M19" s="39"/>
+      <c r="J19" s="57"/>
+      <c r="K19" s="57"/>
+      <c r="M19" s="58"/>
     </row>
     <row r="21" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A21" s="6"/>
@@ -2976,46 +2976,46 @@
     </row>
     <row r="22" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="23" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B23" s="56" t="s">
+      <c r="B23" s="61" t="s">
         <v>134</v>
       </c>
-      <c r="C23" s="57"/>
-      <c r="D23" s="57"/>
-      <c r="E23" s="57"/>
-      <c r="F23" s="57"/>
-      <c r="G23" s="57"/>
-      <c r="H23" s="57"/>
-      <c r="I23" s="57"/>
-      <c r="J23" s="57"/>
-      <c r="K23" s="58"/>
+      <c r="C23" s="62"/>
+      <c r="D23" s="62"/>
+      <c r="E23" s="62"/>
+      <c r="F23" s="62"/>
+      <c r="G23" s="62"/>
+      <c r="H23" s="62"/>
+      <c r="I23" s="62"/>
+      <c r="J23" s="62"/>
+      <c r="K23" s="63"/>
     </row>
     <row r="24" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B24" s="59"/>
-      <c r="C24" s="60"/>
-      <c r="D24" s="60"/>
-      <c r="E24" s="60"/>
-      <c r="F24" s="60"/>
-      <c r="G24" s="60"/>
-      <c r="H24" s="60"/>
-      <c r="I24" s="60"/>
-      <c r="J24" s="60"/>
-      <c r="K24" s="61"/>
+      <c r="B24" s="64"/>
+      <c r="C24" s="65"/>
+      <c r="D24" s="65"/>
+      <c r="E24" s="65"/>
+      <c r="F24" s="65"/>
+      <c r="G24" s="65"/>
+      <c r="H24" s="65"/>
+      <c r="I24" s="65"/>
+      <c r="J24" s="65"/>
+      <c r="K24" s="66"/>
     </row>
     <row r="26" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B26" s="53" t="s">
+      <c r="B26" s="44" t="s">
         <v>17</v>
       </c>
-      <c r="C26" s="53"/>
-      <c r="E26" s="46" t="s">
+      <c r="C26" s="44"/>
+      <c r="E26" s="53" t="s">
         <v>21</v>
       </c>
-      <c r="F26" s="47"/>
-      <c r="G26" s="48"/>
-      <c r="I26" s="53" t="s">
+      <c r="F26" s="55"/>
+      <c r="G26" s="54"/>
+      <c r="I26" s="44" t="s">
         <v>20</v>
       </c>
-      <c r="J26" s="53"/>
-      <c r="K26" s="53"/>
+      <c r="J26" s="44"/>
+      <c r="K26" s="44"/>
       <c r="M26" s="10" t="s">
         <v>22</v>
       </c>
@@ -3050,12 +3050,12 @@
       <c r="K27" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="M27" s="62">
+      <c r="M27" s="67">
         <f>SUM(B28:C28,E28:G28,I28:K28)</f>
         <v>36</v>
       </c>
       <c r="N27" s="7"/>
-      <c r="O27" s="39">
+      <c r="O27" s="58">
         <v>4</v>
       </c>
       <c r="P27" s="8"/>
@@ -3085,9 +3085,9 @@
       <c r="K28" s="2">
         <v>3.2</v>
       </c>
-      <c r="M28" s="62"/>
+      <c r="M28" s="67"/>
       <c r="N28" s="7"/>
-      <c r="O28" s="39"/>
+      <c r="O28" s="58"/>
       <c r="P28" s="8"/>
     </row>
     <row r="30" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -3113,39 +3113,39 @@
     </row>
     <row r="31" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="32" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B32" s="56" t="s">
+      <c r="B32" s="61" t="s">
         <v>135</v>
       </c>
-      <c r="C32" s="57"/>
-      <c r="D32" s="57"/>
-      <c r="E32" s="57"/>
-      <c r="F32" s="57"/>
-      <c r="G32" s="57"/>
-      <c r="H32" s="57"/>
-      <c r="I32" s="58"/>
+      <c r="C32" s="62"/>
+      <c r="D32" s="62"/>
+      <c r="E32" s="62"/>
+      <c r="F32" s="62"/>
+      <c r="G32" s="62"/>
+      <c r="H32" s="62"/>
+      <c r="I32" s="63"/>
     </row>
     <row r="33" spans="2:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B33" s="59"/>
-      <c r="C33" s="60"/>
-      <c r="D33" s="60"/>
-      <c r="E33" s="60"/>
-      <c r="F33" s="60"/>
-      <c r="G33" s="60"/>
-      <c r="H33" s="60"/>
-      <c r="I33" s="61"/>
+      <c r="B33" s="64"/>
+      <c r="C33" s="65"/>
+      <c r="D33" s="65"/>
+      <c r="E33" s="65"/>
+      <c r="F33" s="65"/>
+      <c r="G33" s="65"/>
+      <c r="H33" s="65"/>
+      <c r="I33" s="66"/>
     </row>
     <row r="35" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B35" s="53" t="s">
+      <c r="B35" s="44" t="s">
         <v>31</v>
       </c>
-      <c r="C35" s="53"/>
-      <c r="D35" s="53"/>
-      <c r="F35" s="53" t="s">
+      <c r="C35" s="44"/>
+      <c r="D35" s="44"/>
+      <c r="F35" s="44" t="s">
         <v>12</v>
       </c>
-      <c r="G35" s="53"/>
-      <c r="H35" s="53"/>
-      <c r="I35" s="53"/>
+      <c r="G35" s="44"/>
+      <c r="H35" s="44"/>
+      <c r="I35" s="44"/>
       <c r="N35" s="7"/>
       <c r="O35" s="7"/>
     </row>
@@ -3202,14 +3202,14 @@
       <c r="O37" s="7"/>
     </row>
     <row r="40" spans="2:15" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B40" s="51" t="s">
+      <c r="B40" s="59" t="s">
         <v>35</v>
       </c>
-      <c r="C40" s="52"/>
-      <c r="F40" s="50" t="s">
+      <c r="C40" s="60"/>
+      <c r="F40" s="57" t="s">
         <v>36</v>
       </c>
-      <c r="G40" s="50"/>
+      <c r="G40" s="57"/>
       <c r="I40" s="9" t="s">
         <v>22</v>
       </c>
@@ -3265,7 +3265,7 @@
       <c r="G43" s="2">
         <v>0.44</v>
       </c>
-      <c r="I43" s="49" t="s">
+      <c r="I43" s="56" t="s">
         <v>67</v>
       </c>
     </row>
@@ -3282,7 +3282,7 @@
       <c r="G44" s="2">
         <v>1</v>
       </c>
-      <c r="I44" s="49"/>
+      <c r="I44" s="56"/>
     </row>
     <row r="45" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B45" s="2" t="s">
@@ -3426,67 +3426,67 @@
     </row>
     <row r="57" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="58" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B58" s="56" t="s">
+      <c r="B58" s="61" t="s">
         <v>136</v>
       </c>
-      <c r="C58" s="57"/>
-      <c r="D58" s="57"/>
-      <c r="E58" s="57"/>
-      <c r="F58" s="57"/>
-      <c r="G58" s="57"/>
-      <c r="H58" s="57"/>
-      <c r="I58" s="57"/>
-      <c r="J58" s="57"/>
-      <c r="K58" s="57"/>
-      <c r="L58" s="57"/>
-      <c r="M58" s="57"/>
-      <c r="N58" s="57"/>
-      <c r="O58" s="57"/>
-      <c r="P58" s="57"/>
-      <c r="Q58" s="57"/>
-      <c r="R58" s="58"/>
+      <c r="C58" s="62"/>
+      <c r="D58" s="62"/>
+      <c r="E58" s="62"/>
+      <c r="F58" s="62"/>
+      <c r="G58" s="62"/>
+      <c r="H58" s="62"/>
+      <c r="I58" s="62"/>
+      <c r="J58" s="62"/>
+      <c r="K58" s="62"/>
+      <c r="L58" s="62"/>
+      <c r="M58" s="62"/>
+      <c r="N58" s="62"/>
+      <c r="O58" s="62"/>
+      <c r="P58" s="62"/>
+      <c r="Q58" s="62"/>
+      <c r="R58" s="63"/>
     </row>
     <row r="59" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B59" s="59"/>
-      <c r="C59" s="60"/>
-      <c r="D59" s="60"/>
-      <c r="E59" s="60"/>
-      <c r="F59" s="60"/>
-      <c r="G59" s="60"/>
-      <c r="H59" s="60"/>
-      <c r="I59" s="60"/>
-      <c r="J59" s="60"/>
-      <c r="K59" s="60"/>
-      <c r="L59" s="60"/>
-      <c r="M59" s="60"/>
-      <c r="N59" s="60"/>
-      <c r="O59" s="60"/>
-      <c r="P59" s="60"/>
-      <c r="Q59" s="60"/>
-      <c r="R59" s="61"/>
+      <c r="B59" s="64"/>
+      <c r="C59" s="65"/>
+      <c r="D59" s="65"/>
+      <c r="E59" s="65"/>
+      <c r="F59" s="65"/>
+      <c r="G59" s="65"/>
+      <c r="H59" s="65"/>
+      <c r="I59" s="65"/>
+      <c r="J59" s="65"/>
+      <c r="K59" s="65"/>
+      <c r="L59" s="65"/>
+      <c r="M59" s="65"/>
+      <c r="N59" s="65"/>
+      <c r="O59" s="65"/>
+      <c r="P59" s="65"/>
+      <c r="Q59" s="65"/>
+      <c r="R59" s="66"/>
     </row>
     <row r="61" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B61" s="53" t="s">
+      <c r="B61" s="44" t="s">
         <v>63</v>
       </c>
-      <c r="C61" s="53"/>
-      <c r="D61" s="53"/>
-      <c r="E61" s="53"/>
-      <c r="F61" s="53"/>
-      <c r="G61" s="53"/>
-      <c r="H61" s="53"/>
-      <c r="I61" s="53"/>
-      <c r="J61" s="53"/>
-      <c r="K61" s="53"/>
-      <c r="M61" s="53" t="s">
+      <c r="C61" s="44"/>
+      <c r="D61" s="44"/>
+      <c r="E61" s="44"/>
+      <c r="F61" s="44"/>
+      <c r="G61" s="44"/>
+      <c r="H61" s="44"/>
+      <c r="I61" s="44"/>
+      <c r="J61" s="44"/>
+      <c r="K61" s="44"/>
+      <c r="M61" s="44" t="s">
         <v>68</v>
       </c>
-      <c r="N61" s="53"/>
-      <c r="O61" s="53"/>
-      <c r="Q61" s="53" t="s">
+      <c r="N61" s="44"/>
+      <c r="O61" s="44"/>
+      <c r="Q61" s="44" t="s">
         <v>64</v>
       </c>
-      <c r="R61" s="53"/>
+      <c r="R61" s="44"/>
     </row>
     <row r="62" spans="1:19" x14ac:dyDescent="0.25">
       <c r="B62" s="2" t="s">
@@ -3583,28 +3583,28 @@
       </c>
     </row>
     <row r="66" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B66" s="49" t="s">
+      <c r="B66" s="56" t="s">
         <v>22</v>
       </c>
-      <c r="C66" s="49"/>
+      <c r="C66" s="56"/>
       <c r="E66" s="9" t="s">
         <v>67</v>
       </c>
     </row>
     <row r="67" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B67" s="50">
+      <c r="B67" s="57">
         <f xml:space="preserve"> SUM(B63:K63,M63:O63,Q63:R63)</f>
         <v>85.5</v>
       </c>
-      <c r="C67" s="50"/>
-      <c r="E67" s="39">
+      <c r="C67" s="57"/>
+      <c r="E67" s="58">
         <v>4.5</v>
       </c>
     </row>
     <row r="68" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B68" s="50"/>
-      <c r="C68" s="50"/>
-      <c r="E68" s="39"/>
+      <c r="B68" s="57"/>
+      <c r="C68" s="57"/>
+      <c r="E68" s="58"/>
     </row>
     <row r="70" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A70" s="6"/>
@@ -3629,26 +3629,26 @@
     </row>
     <row r="71" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="72" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B72" s="56" t="s">
+      <c r="B72" s="61" t="s">
         <v>137</v>
       </c>
-      <c r="C72" s="57"/>
-      <c r="D72" s="57"/>
-      <c r="E72" s="57"/>
-      <c r="F72" s="57"/>
-      <c r="G72" s="57"/>
-      <c r="H72" s="57"/>
-      <c r="I72" s="58"/>
+      <c r="C72" s="62"/>
+      <c r="D72" s="62"/>
+      <c r="E72" s="62"/>
+      <c r="F72" s="62"/>
+      <c r="G72" s="62"/>
+      <c r="H72" s="62"/>
+      <c r="I72" s="63"/>
     </row>
     <row r="73" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B73" s="59"/>
-      <c r="C73" s="60"/>
-      <c r="D73" s="60"/>
-      <c r="E73" s="60"/>
-      <c r="F73" s="60"/>
-      <c r="G73" s="60"/>
-      <c r="H73" s="60"/>
-      <c r="I73" s="61"/>
+      <c r="B73" s="64"/>
+      <c r="C73" s="65"/>
+      <c r="D73" s="65"/>
+      <c r="E73" s="65"/>
+      <c r="F73" s="65"/>
+      <c r="G73" s="65"/>
+      <c r="H73" s="65"/>
+      <c r="I73" s="66"/>
     </row>
     <row r="75" spans="1:19" x14ac:dyDescent="0.25">
       <c r="B75" s="4" t="s">
@@ -3675,10 +3675,10 @@
       <c r="I75" s="4" t="s">
         <v>145</v>
       </c>
-      <c r="K75" s="49" t="s">
+      <c r="K75" s="56" t="s">
         <v>22</v>
       </c>
-      <c r="L75" s="49"/>
+      <c r="L75" s="56"/>
       <c r="N75" s="9" t="s">
         <v>67</v>
       </c>
@@ -3708,11 +3708,11 @@
       <c r="I76" s="2">
         <v>5</v>
       </c>
-      <c r="K76" s="50">
+      <c r="K76" s="57">
         <f>SUM(B76:I76)</f>
         <v>96</v>
       </c>
-      <c r="L76" s="50"/>
+      <c r="L76" s="57"/>
       <c r="N76" s="13">
         <v>5</v>
       </c>
@@ -3740,6 +3740,30 @@
     </row>
   </sheetData>
   <mergeCells count="34">
+    <mergeCell ref="B2:P3"/>
+    <mergeCell ref="B5:G5"/>
+    <mergeCell ref="K5:N5"/>
+    <mergeCell ref="B9:C9"/>
+    <mergeCell ref="B10:C11"/>
+    <mergeCell ref="E10:E11"/>
+    <mergeCell ref="M27:M28"/>
+    <mergeCell ref="O27:O28"/>
+    <mergeCell ref="B14:H15"/>
+    <mergeCell ref="B17:D17"/>
+    <mergeCell ref="F17:H17"/>
+    <mergeCell ref="J17:K17"/>
+    <mergeCell ref="J18:K19"/>
+    <mergeCell ref="M18:M19"/>
+    <mergeCell ref="I43:I44"/>
+    <mergeCell ref="B23:K24"/>
+    <mergeCell ref="B26:C26"/>
+    <mergeCell ref="E26:G26"/>
+    <mergeCell ref="I26:K26"/>
+    <mergeCell ref="B32:I33"/>
+    <mergeCell ref="B35:D35"/>
+    <mergeCell ref="F35:I35"/>
+    <mergeCell ref="B40:C40"/>
+    <mergeCell ref="F40:G40"/>
     <mergeCell ref="B72:I73"/>
     <mergeCell ref="K75:L75"/>
     <mergeCell ref="K76:L76"/>
@@ -3750,30 +3774,6 @@
     <mergeCell ref="B66:C66"/>
     <mergeCell ref="B67:C68"/>
     <mergeCell ref="E67:E68"/>
-    <mergeCell ref="I43:I44"/>
-    <mergeCell ref="B23:K24"/>
-    <mergeCell ref="B26:C26"/>
-    <mergeCell ref="E26:G26"/>
-    <mergeCell ref="I26:K26"/>
-    <mergeCell ref="B32:I33"/>
-    <mergeCell ref="B35:D35"/>
-    <mergeCell ref="F35:I35"/>
-    <mergeCell ref="B40:C40"/>
-    <mergeCell ref="F40:G40"/>
-    <mergeCell ref="M27:M28"/>
-    <mergeCell ref="O27:O28"/>
-    <mergeCell ref="B14:H15"/>
-    <mergeCell ref="B17:D17"/>
-    <mergeCell ref="F17:H17"/>
-    <mergeCell ref="J17:K17"/>
-    <mergeCell ref="J18:K19"/>
-    <mergeCell ref="M18:M19"/>
-    <mergeCell ref="B2:P3"/>
-    <mergeCell ref="B5:G5"/>
-    <mergeCell ref="K5:N5"/>
-    <mergeCell ref="B9:C9"/>
-    <mergeCell ref="B10:C11"/>
-    <mergeCell ref="E10:E11"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
@@ -3782,7 +3782,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CEAA0BBB-B59A-4C0E-8304-D0FA810EECB4}">
-  <dimension ref="B1:F39"/>
+  <dimension ref="B1:F40"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="3" max="3" width="11.85546875" style="16" customWidth="1"/>
@@ -3841,19 +3841,19 @@
       </c>
     </row>
     <row r="5" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B5" s="73" t="b">
+      <c r="B5" s="39" t="b">
         <v>0</v>
       </c>
-      <c r="C5" s="74" t="s">
+      <c r="C5" s="40" t="s">
         <v>77</v>
       </c>
-      <c r="D5" s="75">
+      <c r="D5" s="41">
         <v>45817</v>
       </c>
-      <c r="E5" s="76" t="s">
+      <c r="E5" s="42" t="s">
         <v>151</v>
       </c>
-      <c r="F5" s="77" t="s">
+      <c r="F5" s="43" t="s">
         <v>152</v>
       </c>
     </row>
@@ -4226,35 +4226,34 @@
       </c>
     </row>
     <row r="32" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B32" s="68" t="b">
+      <c r="B32" s="19" t="b">
         <v>0</v>
       </c>
-      <c r="C32" s="69" t="s">
+      <c r="C32" s="21" t="s">
         <v>76</v>
       </c>
-      <c r="D32" s="70">
+      <c r="D32" s="20">
         <v>45815</v>
       </c>
-      <c r="E32" s="71" t="s">
+      <c r="E32" s="17" t="s">
         <v>218</v>
       </c>
-      <c r="F32" s="72"/>
-    </row>
-    <row r="34" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B34" s="23" t="b">
-        <v>1</v>
-      </c>
-      <c r="C34" s="29" t="s">
-        <v>78</v>
-      </c>
-      <c r="D34" s="28">
-        <v>45767</v>
-      </c>
-      <c r="E34" s="27" t="s">
-        <v>181</v>
-      </c>
-      <c r="F34" s="27" t="s">
-        <v>190</v>
+    </row>
+    <row r="33" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B33" s="73" t="b">
+        <v>0</v>
+      </c>
+      <c r="C33" s="74" t="s">
+        <v>76</v>
+      </c>
+      <c r="D33" s="75">
+        <v>45764</v>
+      </c>
+      <c r="E33" s="76" t="s">
+        <v>150</v>
+      </c>
+      <c r="F33" s="76" t="s">
+        <v>223</v>
       </c>
     </row>
     <row r="35" spans="2:6" x14ac:dyDescent="0.25">
@@ -4265,44 +4264,44 @@
         <v>78</v>
       </c>
       <c r="D35" s="28">
+        <v>45767</v>
+      </c>
+      <c r="E35" s="27" t="s">
+        <v>181</v>
+      </c>
+      <c r="F35" s="27" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="36" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B36" s="23" t="b">
+        <v>1</v>
+      </c>
+      <c r="C36" s="29" t="s">
+        <v>78</v>
+      </c>
+      <c r="D36" s="28">
         <v>45775</v>
       </c>
-      <c r="E35" s="27" t="s">
+      <c r="E36" s="27" t="s">
         <v>149</v>
       </c>
     </row>
-    <row r="36" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B36" s="19" t="b">
-        <v>0</v>
-      </c>
-      <c r="C36" s="21" t="s">
+    <row r="37" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B37" s="23" t="b">
+        <v>1</v>
+      </c>
+      <c r="C37" s="29" t="s">
         <v>78</v>
       </c>
-      <c r="D36" s="20">
+      <c r="D37" s="28">
         <v>45794</v>
       </c>
-      <c r="E36" s="17" t="s">
+      <c r="E37" s="27" t="s">
         <v>214</v>
       </c>
-      <c r="F36" s="17" t="s">
+      <c r="F37" s="27" t="s">
         <v>213</v>
-      </c>
-    </row>
-    <row r="38" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B38" s="19" t="b">
-        <v>0</v>
-      </c>
-      <c r="C38" s="21" t="s">
-        <v>79</v>
-      </c>
-      <c r="D38" s="20">
-        <v>45797</v>
-      </c>
-      <c r="E38" s="17" t="s">
-        <v>219</v>
-      </c>
-      <c r="F38" s="17" t="s">
-        <v>220</v>
       </c>
     </row>
     <row r="39" spans="2:6" x14ac:dyDescent="0.25">
@@ -4313,12 +4312,29 @@
         <v>79</v>
       </c>
       <c r="D39" s="20">
+        <v>45797</v>
+      </c>
+      <c r="E39" s="17" t="s">
+        <v>219</v>
+      </c>
+      <c r="F39" s="17" t="s">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="40" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B40" s="19" t="b">
+        <v>0</v>
+      </c>
+      <c r="C40" s="21" t="s">
+        <v>79</v>
+      </c>
+      <c r="D40" s="20">
         <v>45804</v>
       </c>
-      <c r="E39" s="17" t="s">
+      <c r="E40" s="17" t="s">
         <v>222</v>
       </c>
-      <c r="F39" s="17" t="s">
+      <c r="F40" s="17" t="s">
         <v>221</v>
       </c>
     </row>
@@ -4347,21 +4363,21 @@
   <sheetData>
     <row r="1" spans="2:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="2" spans="2:12" ht="23.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B2" s="63" t="s">
+      <c r="B2" s="68" t="s">
         <v>203</v>
       </c>
-      <c r="C2" s="64"/>
-      <c r="D2" s="65"/>
-      <c r="F2" s="63" t="s">
+      <c r="C2" s="69"/>
+      <c r="D2" s="70"/>
+      <c r="F2" s="68" t="s">
         <v>204</v>
       </c>
-      <c r="G2" s="64"/>
-      <c r="H2" s="65"/>
-      <c r="J2" s="63" t="s">
+      <c r="G2" s="69"/>
+      <c r="H2" s="70"/>
+      <c r="J2" s="68" t="s">
         <v>205</v>
       </c>
-      <c r="K2" s="64"/>
-      <c r="L2" s="65"/>
+      <c r="K2" s="69"/>
+      <c r="L2" s="70"/>
     </row>
     <row r="3" spans="2:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B3" s="34" t="s">
@@ -4536,26 +4552,26 @@
     </row>
     <row r="10" spans="2:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="11" spans="2:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B11" s="66" t="s">
+      <c r="B11" s="71" t="s">
         <v>197</v>
       </c>
-      <c r="C11" s="67"/>
+      <c r="C11" s="72"/>
       <c r="D11" s="33">
         <f>(D4*C4+D5*C5+D6*C6+D7*C7+D8*C8+D9*C9)/30</f>
         <v>4.4333333333333336</v>
       </c>
-      <c r="F11" s="66" t="s">
+      <c r="F11" s="71" t="s">
         <v>197</v>
       </c>
-      <c r="G11" s="67"/>
+      <c r="G11" s="72"/>
       <c r="H11" s="33">
         <f>(H4*G4+H5*G5+H6*G6+H7*G7+H8*G8)/30</f>
         <v>0</v>
       </c>
-      <c r="J11" s="66" t="s">
+      <c r="J11" s="71" t="s">
         <v>197</v>
       </c>
-      <c r="K11" s="67"/>
+      <c r="K11" s="72"/>
       <c r="L11" s="33">
         <f>(L4*K4+L5*K5+L6*K6+L7*K7+L8*K8)/30</f>
         <v>0</v>

</xml_diff>

<commit_message>
New points - PBL2 - and new grade - labs FIZ1
</commit_message>
<xml_diff>
--- a/IoT-points-schedule.xlsx
+++ b/IoT-points-schedule.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\dodo\Desktop\IoT-studies\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F6A26558-A96B-4669-95AE-8FBBB8B239D1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5FF09843-948A-4068-B4D0-581168967817}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="25440" windowHeight="15390" xr2:uid="{F85F5544-1FE8-4920-A5D4-192A98B113BD}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="354" uniqueCount="225">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="355" uniqueCount="226">
   <si>
     <t>1. Krypto</t>
   </si>
@@ -714,6 +714,9 @@
   </si>
   <si>
     <t>Kolos</t>
+  </si>
+  <si>
+    <t>Extra</t>
   </si>
 </sst>
 </file>
@@ -796,7 +799,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="8">
+  <fills count="10">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -839,6 +842,18 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0" tint="-4.9989318521683403E-2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="2" tint="-9.9978637043366805E-2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="20">
     <border>
@@ -1089,7 +1104,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="73">
+  <cellXfs count="76">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1230,6 +1245,12 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1315,6 +1336,9 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1678,7 +1702,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{03C86BD6-21E5-4E44-BF61-9A65607E6D85}">
-  <dimension ref="A1:S70"/>
+  <dimension ref="A1:S71"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="3.85546875" style="1" customWidth="1"/>
@@ -1696,7 +1720,7 @@
     <col min="13" max="13" width="15.28515625" style="1" customWidth="1"/>
     <col min="14" max="14" width="15.7109375" style="1" customWidth="1"/>
     <col min="15" max="15" width="14.28515625" style="1" customWidth="1"/>
-    <col min="16" max="16" width="15.85546875" style="1" customWidth="1"/>
+    <col min="16" max="16" width="15.140625" style="1" customWidth="1"/>
     <col min="17" max="17" width="12.28515625" style="1" customWidth="1"/>
     <col min="18" max="18" width="13.85546875" style="1" customWidth="1"/>
     <col min="19" max="19" width="14.28515625" style="1" customWidth="1"/>
@@ -1705,60 +1729,60 @@
   <sheetData>
     <row r="1" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="2" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B2" s="45" t="s">
+      <c r="B2" s="47" t="s">
         <v>76</v>
       </c>
-      <c r="C2" s="46"/>
-      <c r="D2" s="46"/>
-      <c r="E2" s="46"/>
-      <c r="F2" s="46"/>
-      <c r="G2" s="46"/>
-      <c r="H2" s="46"/>
-      <c r="I2" s="46"/>
-      <c r="J2" s="46"/>
-      <c r="K2" s="46"/>
-      <c r="L2" s="46"/>
-      <c r="M2" s="46"/>
-      <c r="N2" s="46"/>
-      <c r="O2" s="46"/>
-      <c r="P2" s="47"/>
+      <c r="C2" s="48"/>
+      <c r="D2" s="48"/>
+      <c r="E2" s="48"/>
+      <c r="F2" s="48"/>
+      <c r="G2" s="48"/>
+      <c r="H2" s="48"/>
+      <c r="I2" s="48"/>
+      <c r="J2" s="48"/>
+      <c r="K2" s="48"/>
+      <c r="L2" s="48"/>
+      <c r="M2" s="48"/>
+      <c r="N2" s="48"/>
+      <c r="O2" s="48"/>
+      <c r="P2" s="49"/>
     </row>
     <row r="3" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B3" s="48"/>
-      <c r="C3" s="49"/>
-      <c r="D3" s="49"/>
-      <c r="E3" s="49"/>
-      <c r="F3" s="49"/>
-      <c r="G3" s="49"/>
-      <c r="H3" s="49"/>
-      <c r="I3" s="49"/>
-      <c r="J3" s="49"/>
-      <c r="K3" s="49"/>
-      <c r="L3" s="49"/>
-      <c r="M3" s="49"/>
-      <c r="N3" s="49"/>
-      <c r="O3" s="49"/>
-      <c r="P3" s="50"/>
+      <c r="B3" s="50"/>
+      <c r="C3" s="51"/>
+      <c r="D3" s="51"/>
+      <c r="E3" s="51"/>
+      <c r="F3" s="51"/>
+      <c r="G3" s="51"/>
+      <c r="H3" s="51"/>
+      <c r="I3" s="51"/>
+      <c r="J3" s="51"/>
+      <c r="K3" s="51"/>
+      <c r="L3" s="51"/>
+      <c r="M3" s="51"/>
+      <c r="N3" s="51"/>
+      <c r="O3" s="51"/>
+      <c r="P3" s="52"/>
       <c r="R3" s="12"/>
     </row>
     <row r="5" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B5" s="53" t="s">
+      <c r="B5" s="55" t="s">
         <v>83</v>
       </c>
-      <c r="C5" s="55"/>
-      <c r="D5" s="55"/>
-      <c r="E5" s="55"/>
-      <c r="F5" s="54"/>
-      <c r="H5" s="53" t="s">
+      <c r="C5" s="57"/>
+      <c r="D5" s="57"/>
+      <c r="E5" s="57"/>
+      <c r="F5" s="56"/>
+      <c r="H5" s="55" t="s">
         <v>82</v>
       </c>
-      <c r="I5" s="54"/>
-      <c r="K5" s="53" t="s">
+      <c r="I5" s="56"/>
+      <c r="K5" s="55" t="s">
         <v>8</v>
       </c>
-      <c r="L5" s="55"/>
-      <c r="M5" s="55"/>
-      <c r="N5" s="54"/>
+      <c r="L5" s="57"/>
+      <c r="M5" s="57"/>
+      <c r="N5" s="56"/>
       <c r="P5" s="4" t="s">
         <v>74</v>
       </c>
@@ -1826,37 +1850,37 @@
       <c r="P7" s="2"/>
     </row>
     <row r="9" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B9" s="56" t="s">
+      <c r="B9" s="58" t="s">
         <v>22</v>
       </c>
-      <c r="C9" s="56"/>
+      <c r="C9" s="58"/>
       <c r="E9" s="9" t="s">
         <v>67</v>
       </c>
-      <c r="G9" s="56" t="s">
+      <c r="G9" s="58" t="s">
         <v>87</v>
       </c>
-      <c r="H9" s="56"/>
+      <c r="H9" s="58"/>
     </row>
     <row r="10" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B10" s="57">
+      <c r="B10" s="59">
         <f>SUM(B7:F7,H7:I7,K7:N7,P7)</f>
         <v>25.7</v>
       </c>
-      <c r="C10" s="57"/>
-      <c r="E10" s="51"/>
-      <c r="G10" s="57">
+      <c r="C10" s="59"/>
+      <c r="E10" s="53"/>
+      <c r="G10" s="59">
         <f>66-SUM(B7:F7,H7:I7,K7:N7,P7)</f>
         <v>40.299999999999997</v>
       </c>
-      <c r="H10" s="57"/>
+      <c r="H10" s="59"/>
     </row>
     <row r="11" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B11" s="57"/>
-      <c r="C11" s="57"/>
-      <c r="E11" s="52"/>
-      <c r="G11" s="57"/>
-      <c r="H11" s="57"/>
+      <c r="B11" s="59"/>
+      <c r="C11" s="59"/>
+      <c r="E11" s="54"/>
+      <c r="G11" s="59"/>
+      <c r="H11" s="59"/>
     </row>
     <row r="12" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A12" s="6"/>
@@ -1881,46 +1905,46 @@
     </row>
     <row r="13" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="14" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B14" s="45" t="s">
+      <c r="B14" s="47" t="s">
         <v>77</v>
       </c>
-      <c r="C14" s="46"/>
-      <c r="D14" s="46"/>
-      <c r="E14" s="46"/>
-      <c r="F14" s="46"/>
-      <c r="G14" s="46"/>
-      <c r="H14" s="47"/>
+      <c r="C14" s="48"/>
+      <c r="D14" s="48"/>
+      <c r="E14" s="48"/>
+      <c r="F14" s="48"/>
+      <c r="G14" s="48"/>
+      <c r="H14" s="49"/>
     </row>
     <row r="15" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B15" s="48"/>
-      <c r="C15" s="49"/>
-      <c r="D15" s="49"/>
-      <c r="E15" s="49"/>
-      <c r="F15" s="49"/>
-      <c r="G15" s="49"/>
-      <c r="H15" s="50"/>
+      <c r="B15" s="50"/>
+      <c r="C15" s="51"/>
+      <c r="D15" s="51"/>
+      <c r="E15" s="51"/>
+      <c r="F15" s="51"/>
+      <c r="G15" s="51"/>
+      <c r="H15" s="52"/>
     </row>
     <row r="17" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B17" s="44" t="s">
+      <c r="B17" s="46" t="s">
         <v>91</v>
       </c>
-      <c r="C17" s="44"/>
-      <c r="D17" s="44"/>
-      <c r="E17" s="44"/>
-      <c r="F17" s="44"/>
-      <c r="H17" s="53" t="s">
+      <c r="C17" s="46"/>
+      <c r="D17" s="46"/>
+      <c r="E17" s="46"/>
+      <c r="F17" s="46"/>
+      <c r="H17" s="55" t="s">
         <v>97</v>
       </c>
-      <c r="I17" s="55"/>
-      <c r="J17" s="54"/>
-      <c r="L17" s="56" t="s">
+      <c r="I17" s="57"/>
+      <c r="J17" s="56"/>
+      <c r="L17" s="58" t="s">
         <v>22</v>
       </c>
-      <c r="M17" s="56"/>
-      <c r="O17" s="56" t="s">
+      <c r="M17" s="58"/>
+      <c r="O17" s="58" t="s">
         <v>87</v>
       </c>
-      <c r="P17" s="56"/>
+      <c r="P17" s="58"/>
       <c r="R17" s="9" t="s">
         <v>67</v>
       </c>
@@ -1950,17 +1974,17 @@
       <c r="J18" s="3" t="s">
         <v>95</v>
       </c>
-      <c r="L18" s="57">
+      <c r="L18" s="59">
         <f>SUM(B19:F19,H19:J19)</f>
         <v>29.5</v>
       </c>
-      <c r="M18" s="57"/>
-      <c r="O18" s="57">
+      <c r="M18" s="59"/>
+      <c r="O18" s="59">
         <f>50-SUM(B19:F19,H19:J19)</f>
         <v>20.5</v>
       </c>
-      <c r="P18" s="57"/>
-      <c r="R18" s="58"/>
+      <c r="P18" s="59"/>
+      <c r="R18" s="60"/>
     </row>
     <row r="19" spans="1:19" x14ac:dyDescent="0.25">
       <c r="B19" s="2"/>
@@ -1975,11 +1999,11 @@
         <v>26.5</v>
       </c>
       <c r="J19" s="2"/>
-      <c r="L19" s="57"/>
-      <c r="M19" s="57"/>
-      <c r="O19" s="57"/>
-      <c r="P19" s="57"/>
-      <c r="R19" s="58"/>
+      <c r="L19" s="59"/>
+      <c r="M19" s="59"/>
+      <c r="O19" s="59"/>
+      <c r="P19" s="59"/>
+      <c r="R19" s="60"/>
     </row>
     <row r="21" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A21" s="6"/>
@@ -2004,56 +2028,56 @@
     </row>
     <row r="22" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="23" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B23" s="45" t="s">
+      <c r="B23" s="47" t="s">
         <v>79</v>
       </c>
-      <c r="C23" s="46"/>
-      <c r="D23" s="46"/>
-      <c r="E23" s="46"/>
-      <c r="F23" s="46"/>
-      <c r="G23" s="46"/>
-      <c r="H23" s="46"/>
-      <c r="I23" s="46"/>
-      <c r="J23" s="46"/>
-      <c r="K23" s="46"/>
-      <c r="L23" s="47"/>
-      <c r="N23" s="57" t="s">
+      <c r="C23" s="48"/>
+      <c r="D23" s="48"/>
+      <c r="E23" s="48"/>
+      <c r="F23" s="48"/>
+      <c r="G23" s="48"/>
+      <c r="H23" s="48"/>
+      <c r="I23" s="48"/>
+      <c r="J23" s="48"/>
+      <c r="K23" s="48"/>
+      <c r="L23" s="49"/>
+      <c r="N23" s="59" t="s">
         <v>131</v>
       </c>
-      <c r="O23" s="57"/>
+      <c r="O23" s="59"/>
     </row>
     <row r="24" spans="1:19" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B24" s="48"/>
-      <c r="C24" s="49"/>
-      <c r="D24" s="49"/>
-      <c r="E24" s="49"/>
-      <c r="F24" s="49"/>
-      <c r="G24" s="49"/>
-      <c r="H24" s="49"/>
-      <c r="I24" s="49"/>
-      <c r="J24" s="49"/>
-      <c r="K24" s="49"/>
-      <c r="L24" s="50"/>
-      <c r="N24" s="57"/>
-      <c r="O24" s="57"/>
+      <c r="B24" s="50"/>
+      <c r="C24" s="51"/>
+      <c r="D24" s="51"/>
+      <c r="E24" s="51"/>
+      <c r="F24" s="51"/>
+      <c r="G24" s="51"/>
+      <c r="H24" s="51"/>
+      <c r="I24" s="51"/>
+      <c r="J24" s="51"/>
+      <c r="K24" s="51"/>
+      <c r="L24" s="52"/>
+      <c r="N24" s="59"/>
+      <c r="O24" s="59"/>
     </row>
     <row r="26" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B26" s="44" t="s">
+      <c r="B26" s="46" t="s">
         <v>129</v>
       </c>
-      <c r="C26" s="44"/>
-      <c r="D26" s="44"/>
-      <c r="F26" s="44" t="s">
+      <c r="C26" s="46"/>
+      <c r="D26" s="46"/>
+      <c r="F26" s="46" t="s">
         <v>210</v>
       </c>
-      <c r="G26" s="44"/>
-      <c r="H26" s="44"/>
-      <c r="I26" s="44"/>
+      <c r="G26" s="46"/>
+      <c r="H26" s="46"/>
+      <c r="I26" s="46"/>
       <c r="J26" s="7"/>
-      <c r="K26" s="53" t="s">
+      <c r="K26" s="55" t="s">
         <v>128</v>
       </c>
-      <c r="L26" s="54"/>
+      <c r="L26" s="56"/>
       <c r="N26" s="9" t="s">
         <v>67</v>
       </c>
@@ -2086,7 +2110,7 @@
       <c r="L27" s="2" t="s">
         <v>127</v>
       </c>
-      <c r="N27" s="51"/>
+      <c r="N27" s="53"/>
     </row>
     <row r="28" spans="1:19" x14ac:dyDescent="0.25">
       <c r="B28" s="2">
@@ -2102,526 +2126,550 @@
       <c r="G28" s="2">
         <v>5</v>
       </c>
-      <c r="H28" s="2"/>
+      <c r="H28" s="2">
+        <v>4.5</v>
+      </c>
       <c r="I28" s="2">
         <v>5</v>
       </c>
       <c r="K28" s="2"/>
       <c r="L28" s="2"/>
-      <c r="N28" s="52"/>
-    </row>
-    <row r="30" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A30" s="6"/>
-      <c r="B30" s="6"/>
-      <c r="C30" s="6"/>
-      <c r="D30" s="6"/>
-      <c r="E30" s="6"/>
-      <c r="F30" s="6"/>
-      <c r="G30" s="6"/>
-      <c r="H30" s="6"/>
-      <c r="I30" s="6"/>
-      <c r="J30" s="6"/>
-      <c r="K30" s="6"/>
-      <c r="L30" s="6"/>
-      <c r="M30" s="6"/>
-      <c r="N30" s="6"/>
-      <c r="O30" s="6"/>
-      <c r="P30" s="6"/>
-      <c r="Q30" s="6"/>
-      <c r="R30" s="6"/>
-      <c r="S30" s="6"/>
-    </row>
-    <row r="31" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
-    <row r="32" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B32" s="45" t="s">
+      <c r="N28" s="54"/>
+    </row>
+    <row r="29" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="B29" s="45"/>
+      <c r="C29" s="45"/>
+      <c r="D29" s="45"/>
+      <c r="F29" s="45">
+        <v>5</v>
+      </c>
+      <c r="G29" s="45"/>
+      <c r="H29" s="45"/>
+      <c r="I29" s="45"/>
+      <c r="K29" s="45"/>
+      <c r="L29" s="45"/>
+      <c r="N29" s="44"/>
+    </row>
+    <row r="31" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A31" s="6"/>
+      <c r="B31" s="6"/>
+      <c r="C31" s="6"/>
+      <c r="D31" s="6"/>
+      <c r="E31" s="6"/>
+      <c r="F31" s="6"/>
+      <c r="G31" s="6"/>
+      <c r="H31" s="6"/>
+      <c r="I31" s="6"/>
+      <c r="J31" s="6"/>
+      <c r="K31" s="6"/>
+      <c r="L31" s="6"/>
+      <c r="M31" s="6"/>
+      <c r="N31" s="6"/>
+      <c r="O31" s="6"/>
+      <c r="P31" s="6"/>
+      <c r="Q31" s="6"/>
+      <c r="R31" s="6"/>
+      <c r="S31" s="6"/>
+    </row>
+    <row r="32" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="33" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B33" s="47" t="s">
         <v>78</v>
       </c>
-      <c r="C32" s="46"/>
-      <c r="D32" s="46"/>
-      <c r="E32" s="46"/>
-      <c r="F32" s="46"/>
-      <c r="G32" s="46"/>
-      <c r="H32" s="46"/>
-      <c r="I32" s="47"/>
-    </row>
-    <row r="33" spans="2:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B33" s="48"/>
-      <c r="C33" s="49"/>
-      <c r="D33" s="49"/>
-      <c r="E33" s="49"/>
-      <c r="F33" s="49"/>
-      <c r="G33" s="49"/>
-      <c r="H33" s="49"/>
-      <c r="I33" s="50"/>
-    </row>
-    <row r="35" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B35" s="44" t="s">
+      <c r="C33" s="48"/>
+      <c r="D33" s="48"/>
+      <c r="E33" s="48"/>
+      <c r="F33" s="48"/>
+      <c r="G33" s="48"/>
+      <c r="H33" s="48"/>
+      <c r="I33" s="49"/>
+    </row>
+    <row r="34" spans="2:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B34" s="50"/>
+      <c r="C34" s="51"/>
+      <c r="D34" s="51"/>
+      <c r="E34" s="51"/>
+      <c r="F34" s="51"/>
+      <c r="G34" s="51"/>
+      <c r="H34" s="51"/>
+      <c r="I34" s="52"/>
+    </row>
+    <row r="36" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B36" s="46" t="s">
         <v>98</v>
       </c>
-      <c r="C35" s="44"/>
-      <c r="D35" s="7"/>
-      <c r="E35" s="53" t="s">
+      <c r="C36" s="46"/>
+      <c r="D36" s="7"/>
+      <c r="E36" s="55" t="s">
         <v>146</v>
       </c>
-      <c r="F35" s="55"/>
-      <c r="G35" s="55"/>
-      <c r="H35" s="54"/>
-    </row>
-    <row r="36" spans="2:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B36" s="2" t="s">
+      <c r="F36" s="57"/>
+      <c r="G36" s="57"/>
+      <c r="H36" s="56"/>
+    </row>
+    <row r="37" spans="2:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B37" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="C36" s="2" t="s">
+      <c r="C37" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="E36" s="3" t="s">
+      <c r="E37" s="3" t="s">
         <v>101</v>
       </c>
-      <c r="F36" s="3" t="s">
+      <c r="F37" s="3" t="s">
         <v>102</v>
       </c>
-      <c r="G36" s="2" t="s">
+      <c r="G37" s="2" t="s">
         <v>99</v>
       </c>
-      <c r="H36" s="2" t="s">
+      <c r="H37" s="2" t="s">
         <v>100</v>
       </c>
-      <c r="O36" s="7"/>
-    </row>
-    <row r="37" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B37" s="2">
+      <c r="O37" s="7"/>
+    </row>
+    <row r="38" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B38" s="2">
         <v>17</v>
       </c>
-      <c r="C37" s="2"/>
-      <c r="E37" s="2">
-        <f>C56</f>
+      <c r="C38" s="2"/>
+      <c r="E38" s="2">
+        <f>C57</f>
         <v>15</v>
       </c>
-      <c r="F37" s="2">
-        <f>G51</f>
+      <c r="F38" s="2">
+        <f>G52</f>
         <v>9</v>
       </c>
-      <c r="G37" s="2"/>
-      <c r="H37" s="2"/>
-      <c r="O37" s="7"/>
-    </row>
-    <row r="40" spans="2:15" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B40" s="59" t="s">
+      <c r="G38" s="2"/>
+      <c r="H38" s="2"/>
+      <c r="O38" s="7"/>
+    </row>
+    <row r="41" spans="2:15" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B41" s="61" t="s">
         <v>126</v>
       </c>
-      <c r="C40" s="60"/>
-      <c r="F40" s="57" t="s">
+      <c r="C41" s="62"/>
+      <c r="F41" s="59" t="s">
         <v>102</v>
       </c>
-      <c r="G40" s="57"/>
-      <c r="I40" s="9" t="s">
+      <c r="G41" s="59"/>
+      <c r="I41" s="9" t="s">
         <v>22</v>
       </c>
-      <c r="J40" s="11"/>
-      <c r="L40" s="11"/>
-    </row>
-    <row r="41" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B41" s="2" t="s">
-        <v>103</v>
-      </c>
-      <c r="C41" s="2">
-        <v>2</v>
-      </c>
-      <c r="F41" s="2" t="s">
-        <v>117</v>
-      </c>
-      <c r="G41" s="2">
-        <v>9</v>
-      </c>
-      <c r="I41" s="2">
-        <f>SUM(B37:C37,E37:H37)</f>
-        <v>41</v>
-      </c>
-      <c r="J41" s="7"/>
-      <c r="L41" s="7"/>
+      <c r="J41" s="11"/>
+      <c r="L41" s="11"/>
     </row>
     <row r="42" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B42" s="2" t="s">
-        <v>104</v>
-      </c>
-      <c r="C42" s="2"/>
+        <v>103</v>
+      </c>
+      <c r="C42" s="2">
+        <v>2</v>
+      </c>
       <c r="F42" s="2" t="s">
-        <v>118</v>
-      </c>
-      <c r="G42" s="2"/>
-      <c r="I42" s="7"/>
+        <v>117</v>
+      </c>
+      <c r="G42" s="2">
+        <v>9</v>
+      </c>
+      <c r="I42" s="2">
+        <f>SUM(B38:C38,E38:H38)</f>
+        <v>41</v>
+      </c>
       <c r="J42" s="7"/>
+      <c r="L42" s="7"/>
     </row>
     <row r="43" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B43" s="2" t="s">
-        <v>105</v>
-      </c>
-      <c r="C43" s="2">
-        <v>3</v>
-      </c>
+        <v>104</v>
+      </c>
+      <c r="C43" s="2"/>
       <c r="F43" s="2" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="G43" s="2"/>
-      <c r="I43" s="56" t="s">
-        <v>67</v>
-      </c>
+      <c r="I43" s="7"/>
+      <c r="J43" s="7"/>
     </row>
     <row r="44" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B44" s="2" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="C44" s="2">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F44" s="2" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="G44" s="2"/>
-      <c r="I44" s="56"/>
+      <c r="I44" s="58" t="s">
+        <v>67</v>
+      </c>
     </row>
     <row r="45" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B45" s="2" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="C45" s="2">
         <v>4</v>
       </c>
       <c r="F45" s="2" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="G45" s="2"/>
-      <c r="I45" s="13"/>
+      <c r="I45" s="58"/>
     </row>
     <row r="46" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B46" s="2" t="s">
-        <v>108</v>
-      </c>
-      <c r="C46" s="2"/>
+        <v>107</v>
+      </c>
+      <c r="C46" s="2">
+        <v>4</v>
+      </c>
       <c r="F46" s="2" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="G46" s="2"/>
+      <c r="I46" s="13"/>
     </row>
     <row r="47" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B47" s="2" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="C47" s="2"/>
       <c r="F47" s="2" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="G47" s="2"/>
-      <c r="I47" s="9" t="s">
-        <v>87</v>
-      </c>
     </row>
     <row r="48" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B48" s="2" t="s">
-        <v>110</v>
-      </c>
-      <c r="C48" s="2">
-        <v>2</v>
-      </c>
+        <v>109</v>
+      </c>
+      <c r="C48" s="2"/>
       <c r="F48" s="2" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="G48" s="2"/>
-      <c r="I48" s="2">
-        <f>50-SUM(B37:C37,E37:H37)</f>
-        <v>9</v>
+      <c r="I48" s="9" t="s">
+        <v>87</v>
       </c>
     </row>
     <row r="49" spans="1:19" x14ac:dyDescent="0.25">
       <c r="B49" s="2" t="s">
-        <v>111</v>
-      </c>
-      <c r="C49" s="2"/>
+        <v>110</v>
+      </c>
+      <c r="C49" s="2">
+        <v>2</v>
+      </c>
       <c r="F49" s="2" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="G49" s="2"/>
+      <c r="I49" s="2">
+        <f>50-SUM(B38:C38,E38:H38)</f>
+        <v>9</v>
+      </c>
     </row>
     <row r="50" spans="1:19" x14ac:dyDescent="0.25">
       <c r="B50" s="2" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="C50" s="2"/>
+      <c r="F50" s="2" t="s">
+        <v>125</v>
+      </c>
+      <c r="G50" s="2"/>
     </row>
     <row r="51" spans="1:19" x14ac:dyDescent="0.25">
       <c r="B51" s="2" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="C51" s="2"/>
-      <c r="F51" s="2" t="s">
-        <v>48</v>
-      </c>
-      <c r="G51" s="2">
-        <f>SUM(G41:G49)</f>
-        <v>9</v>
-      </c>
     </row>
     <row r="52" spans="1:19" x14ac:dyDescent="0.25">
       <c r="B52" s="2" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="C52" s="2"/>
+      <c r="F52" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="G52" s="2">
+        <f>SUM(G42:G50)</f>
+        <v>9</v>
+      </c>
     </row>
     <row r="53" spans="1:19" x14ac:dyDescent="0.25">
       <c r="B53" s="2" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="C53" s="2"/>
     </row>
     <row r="54" spans="1:19" x14ac:dyDescent="0.25">
       <c r="B54" s="2" t="s">
+        <v>115</v>
+      </c>
+      <c r="C54" s="2"/>
+    </row>
+    <row r="55" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="B55" s="2" t="s">
         <v>116</v>
       </c>
-      <c r="C54" s="2"/>
-    </row>
-    <row r="56" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B56" s="2" t="s">
+      <c r="C55" s="2"/>
+    </row>
+    <row r="57" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="B57" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="C56" s="2">
-        <f>SUM(C41:C54)</f>
+      <c r="C57" s="2">
+        <f>SUM(C42:C55)</f>
         <v>15</v>
       </c>
     </row>
-    <row r="58" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A58" s="6"/>
-      <c r="B58" s="6"/>
-      <c r="C58" s="6"/>
-      <c r="D58" s="6"/>
-      <c r="E58" s="6"/>
-      <c r="F58" s="6"/>
-      <c r="G58" s="6"/>
-      <c r="H58" s="6"/>
-      <c r="I58" s="6"/>
-      <c r="J58" s="6"/>
-      <c r="K58" s="6"/>
-      <c r="L58" s="6"/>
-      <c r="M58" s="6"/>
-      <c r="N58" s="6"/>
-      <c r="O58" s="6"/>
-      <c r="P58" s="6"/>
-      <c r="Q58" s="6"/>
-      <c r="R58" s="6"/>
-      <c r="S58" s="6"/>
-    </row>
-    <row r="59" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
-    <row r="60" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B60" s="45" t="s">
+    <row r="59" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A59" s="6"/>
+      <c r="B59" s="6"/>
+      <c r="C59" s="6"/>
+      <c r="D59" s="6"/>
+      <c r="E59" s="6"/>
+      <c r="F59" s="6"/>
+      <c r="G59" s="6"/>
+      <c r="H59" s="6"/>
+      <c r="I59" s="6"/>
+      <c r="J59" s="6"/>
+      <c r="K59" s="6"/>
+      <c r="L59" s="6"/>
+      <c r="M59" s="6"/>
+      <c r="N59" s="6"/>
+      <c r="O59" s="6"/>
+      <c r="P59" s="6"/>
+      <c r="Q59" s="6"/>
+      <c r="R59" s="6"/>
+      <c r="S59" s="6"/>
+    </row>
+    <row r="60" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="61" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B61" s="47" t="s">
         <v>80</v>
       </c>
-      <c r="C60" s="46"/>
-      <c r="D60" s="46"/>
-      <c r="E60" s="46"/>
-      <c r="F60" s="46"/>
-      <c r="G60" s="46"/>
-      <c r="H60" s="46"/>
-      <c r="I60" s="46"/>
-      <c r="J60" s="46"/>
-      <c r="K60" s="46"/>
-      <c r="L60" s="46"/>
-      <c r="M60" s="46"/>
-      <c r="N60" s="46"/>
-      <c r="O60" s="46"/>
-      <c r="P60" s="46"/>
-      <c r="Q60" s="46"/>
-      <c r="R60" s="46"/>
-      <c r="S60" s="47"/>
-    </row>
-    <row r="61" spans="1:19" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B61" s="48"/>
-      <c r="C61" s="49"/>
-      <c r="D61" s="49"/>
-      <c r="E61" s="49"/>
-      <c r="F61" s="49"/>
-      <c r="G61" s="49"/>
-      <c r="H61" s="49"/>
-      <c r="I61" s="49"/>
-      <c r="J61" s="49"/>
-      <c r="K61" s="49"/>
-      <c r="L61" s="49"/>
-      <c r="M61" s="49"/>
-      <c r="N61" s="49"/>
-      <c r="O61" s="49"/>
-      <c r="P61" s="49"/>
-      <c r="Q61" s="49"/>
-      <c r="R61" s="49"/>
-      <c r="S61" s="50"/>
-    </row>
-    <row r="63" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B63" s="44" t="s">
+      <c r="C61" s="48"/>
+      <c r="D61" s="48"/>
+      <c r="E61" s="48"/>
+      <c r="F61" s="48"/>
+      <c r="G61" s="48"/>
+      <c r="H61" s="48"/>
+      <c r="I61" s="48"/>
+      <c r="J61" s="48"/>
+      <c r="K61" s="48"/>
+      <c r="L61" s="48"/>
+      <c r="M61" s="48"/>
+      <c r="N61" s="48"/>
+      <c r="O61" s="48"/>
+      <c r="P61" s="48"/>
+      <c r="Q61" s="48"/>
+      <c r="R61" s="48"/>
+      <c r="S61" s="49"/>
+    </row>
+    <row r="62" spans="1:19" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B62" s="50"/>
+      <c r="C62" s="51"/>
+      <c r="D62" s="51"/>
+      <c r="E62" s="51"/>
+      <c r="F62" s="51"/>
+      <c r="G62" s="51"/>
+      <c r="H62" s="51"/>
+      <c r="I62" s="51"/>
+      <c r="J62" s="51"/>
+      <c r="K62" s="51"/>
+      <c r="L62" s="51"/>
+      <c r="M62" s="51"/>
+      <c r="N62" s="51"/>
+      <c r="O62" s="51"/>
+      <c r="P62" s="51"/>
+      <c r="Q62" s="51"/>
+      <c r="R62" s="51"/>
+      <c r="S62" s="52"/>
+    </row>
+    <row r="64" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="B64" s="46" t="s">
         <v>63</v>
       </c>
-      <c r="C63" s="44"/>
-      <c r="D63" s="44"/>
-      <c r="E63" s="44"/>
-      <c r="F63" s="44"/>
-      <c r="G63" s="44"/>
-      <c r="H63" s="44"/>
-      <c r="I63" s="44"/>
-      <c r="J63" s="44"/>
-      <c r="K63" s="44"/>
-      <c r="M63" s="44" t="s">
+      <c r="C64" s="46"/>
+      <c r="D64" s="46"/>
+      <c r="E64" s="46"/>
+      <c r="F64" s="46"/>
+      <c r="G64" s="46"/>
+      <c r="H64" s="46"/>
+      <c r="I64" s="46"/>
+      <c r="J64" s="46"/>
+      <c r="K64" s="46"/>
+      <c r="M64" s="46" t="s">
         <v>90</v>
       </c>
-      <c r="N63" s="44"/>
-      <c r="O63" s="44"/>
-      <c r="P63" s="44"/>
-      <c r="R63" s="44" t="s">
+      <c r="N64" s="46"/>
+      <c r="O64" s="46"/>
+      <c r="P64" s="46"/>
+      <c r="R64" s="46" t="s">
         <v>64</v>
       </c>
-      <c r="S63" s="44"/>
-    </row>
-    <row r="64" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B64" s="2" t="s">
+      <c r="S64" s="46"/>
+    </row>
+    <row r="65" spans="2:19" x14ac:dyDescent="0.25">
+      <c r="B65" s="2" t="s">
         <v>49</v>
       </c>
-      <c r="C64" s="2" t="s">
+      <c r="C65" s="2" t="s">
         <v>51</v>
       </c>
-      <c r="D64" s="2" t="s">
+      <c r="D65" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="E64" s="2" t="s">
+      <c r="E65" s="2" t="s">
         <v>84</v>
       </c>
-      <c r="F64" s="2" t="s">
+      <c r="F65" s="2" t="s">
         <v>62</v>
       </c>
-      <c r="G64" s="2" t="s">
+      <c r="G65" s="2" t="s">
         <v>55</v>
       </c>
-      <c r="H64" s="2" t="s">
+      <c r="H65" s="2" t="s">
         <v>56</v>
       </c>
-      <c r="I64" s="2" t="s">
+      <c r="I65" s="2" t="s">
         <v>81</v>
       </c>
-      <c r="J64" s="2" t="s">
+      <c r="J65" s="2" t="s">
         <v>211</v>
       </c>
-      <c r="K64" s="2" t="s">
+      <c r="K65" s="2" t="s">
         <v>85</v>
       </c>
-      <c r="M64" s="2" t="s">
+      <c r="M65" s="2" t="s">
         <v>69</v>
       </c>
-      <c r="N64" s="2" t="s">
+      <c r="N65" s="2" t="s">
         <v>70</v>
       </c>
-      <c r="O64" s="2" t="s">
+      <c r="O65" s="2" t="s">
         <v>86</v>
       </c>
-      <c r="P64" s="2" t="s">
+      <c r="P65" s="2" t="s">
         <v>71</v>
       </c>
-      <c r="R64" s="2" t="s">
+      <c r="R65" s="2" t="s">
         <v>88</v>
       </c>
-      <c r="S64" s="2" t="s">
+      <c r="S65" s="2" t="s">
         <v>89</v>
       </c>
     </row>
-    <row r="65" spans="2:19" x14ac:dyDescent="0.25">
-      <c r="B65" s="2">
+    <row r="66" spans="2:19" x14ac:dyDescent="0.25">
+      <c r="B66" s="2">
         <v>2</v>
       </c>
-      <c r="C65" s="2">
+      <c r="C66" s="2">
         <v>2</v>
       </c>
-      <c r="D65" s="2">
+      <c r="D66" s="2">
         <v>2</v>
       </c>
-      <c r="E65" s="2">
+      <c r="E66" s="2">
         <v>2</v>
       </c>
-      <c r="F65" s="2" t="s">
+      <c r="F66" s="2" t="s">
         <v>193</v>
       </c>
-      <c r="G65" s="2" t="s">
+      <c r="G66" s="2" t="s">
         <v>193</v>
       </c>
-      <c r="H65" s="2">
+      <c r="H66" s="2">
         <v>2</v>
       </c>
-      <c r="I65" s="2">
+      <c r="I66" s="2">
         <v>2</v>
       </c>
-      <c r="J65" s="2">
+      <c r="J66" s="2">
         <v>2</v>
       </c>
-      <c r="K65" s="2"/>
-      <c r="M65" s="2">
+      <c r="K66" s="2"/>
+      <c r="M66" s="2">
         <v>5</v>
       </c>
-      <c r="N65" s="2">
+      <c r="N66" s="2">
         <v>5</v>
       </c>
-      <c r="O65" s="2"/>
-      <c r="P65" s="2"/>
-      <c r="R65" s="2"/>
-      <c r="S65" s="2"/>
-    </row>
-    <row r="68" spans="2:19" x14ac:dyDescent="0.25">
-      <c r="B68" s="56" t="s">
+      <c r="O66" s="2"/>
+      <c r="P66" s="2"/>
+      <c r="R66" s="2"/>
+      <c r="S66" s="2"/>
+    </row>
+    <row r="69" spans="2:19" x14ac:dyDescent="0.25">
+      <c r="B69" s="58" t="s">
         <v>22</v>
       </c>
-      <c r="C68" s="56"/>
-      <c r="E68" s="9" t="s">
+      <c r="C69" s="58"/>
+      <c r="E69" s="9" t="s">
         <v>67</v>
       </c>
-      <c r="G68" s="56" t="s">
+      <c r="G69" s="58" t="s">
         <v>87</v>
       </c>
-      <c r="H68" s="56"/>
-    </row>
-    <row r="69" spans="2:19" x14ac:dyDescent="0.25">
-      <c r="B69" s="57">
-        <f>SUM(B65:K65,M65:P65,R65:S65)</f>
-        <v>24</v>
-      </c>
-      <c r="C69" s="57"/>
-      <c r="E69" s="58"/>
-      <c r="G69" s="57">
-        <f>50-SUM(B65:K65,M65:P65,R65:S65)</f>
-        <v>26</v>
-      </c>
-      <c r="H69" s="57"/>
+      <c r="H69" s="58"/>
+      <c r="K69" s="75" t="s">
+        <v>225</v>
+      </c>
     </row>
     <row r="70" spans="2:19" x14ac:dyDescent="0.25">
-      <c r="B70" s="57"/>
-      <c r="C70" s="57"/>
-      <c r="E70" s="58"/>
-      <c r="G70" s="57"/>
-      <c r="H70" s="57"/>
+      <c r="B70" s="59">
+        <f>SUM(B66:K66,M66:P66,R66:S66,K70)</f>
+        <v>27</v>
+      </c>
+      <c r="C70" s="59"/>
+      <c r="E70" s="60"/>
+      <c r="G70" s="59">
+        <f>50-SUM(B66:K66,M66:P66,R66:S66,K70)</f>
+        <v>23</v>
+      </c>
+      <c r="H70" s="59"/>
+      <c r="K70" s="59">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="71" spans="2:19" x14ac:dyDescent="0.25">
+      <c r="B71" s="59"/>
+      <c r="C71" s="59"/>
+      <c r="E71" s="60"/>
+      <c r="G71" s="59"/>
+      <c r="H71" s="59"/>
+      <c r="K71" s="59"/>
     </row>
   </sheetData>
-  <mergeCells count="38">
+  <mergeCells count="42">
+    <mergeCell ref="K70:K71"/>
     <mergeCell ref="R18:R19"/>
     <mergeCell ref="B14:H15"/>
     <mergeCell ref="K5:N5"/>
     <mergeCell ref="B2:P3"/>
-    <mergeCell ref="I43:I44"/>
-    <mergeCell ref="F40:G40"/>
-    <mergeCell ref="B40:C40"/>
+    <mergeCell ref="I44:I45"/>
+    <mergeCell ref="F41:G41"/>
+    <mergeCell ref="B41:C41"/>
     <mergeCell ref="L18:M19"/>
     <mergeCell ref="B5:F5"/>
     <mergeCell ref="H5:I5"/>
     <mergeCell ref="N23:O24"/>
     <mergeCell ref="O18:P19"/>
-    <mergeCell ref="B35:C35"/>
-    <mergeCell ref="E35:H35"/>
+    <mergeCell ref="B36:C36"/>
+    <mergeCell ref="E36:H36"/>
     <mergeCell ref="G9:H9"/>
     <mergeCell ref="G10:H11"/>
-    <mergeCell ref="E69:E70"/>
-    <mergeCell ref="B68:C68"/>
-    <mergeCell ref="B69:C70"/>
-    <mergeCell ref="G68:H68"/>
-    <mergeCell ref="G69:H70"/>
+    <mergeCell ref="E70:E71"/>
+    <mergeCell ref="B69:C69"/>
+    <mergeCell ref="B70:C71"/>
+    <mergeCell ref="G69:H69"/>
+    <mergeCell ref="G70:H71"/>
     <mergeCell ref="B17:F17"/>
     <mergeCell ref="H17:J17"/>
     <mergeCell ref="O17:P17"/>
@@ -2634,11 +2682,14 @@
     <mergeCell ref="K26:L26"/>
     <mergeCell ref="B23:L24"/>
     <mergeCell ref="B26:D26"/>
-    <mergeCell ref="R63:S63"/>
-    <mergeCell ref="B32:I33"/>
-    <mergeCell ref="B63:K63"/>
-    <mergeCell ref="B60:S61"/>
-    <mergeCell ref="M63:P63"/>
+    <mergeCell ref="F29:I29"/>
+    <mergeCell ref="B29:D29"/>
+    <mergeCell ref="K29:L29"/>
+    <mergeCell ref="R64:S64"/>
+    <mergeCell ref="B33:I34"/>
+    <mergeCell ref="B64:K64"/>
+    <mergeCell ref="B61:S62"/>
+    <mergeCell ref="M64:P64"/>
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2674,60 +2725,60 @@
   <sheetData>
     <row r="1" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="2" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B2" s="61" t="s">
+      <c r="B2" s="63" t="s">
         <v>132</v>
       </c>
-      <c r="C2" s="62"/>
-      <c r="D2" s="62"/>
-      <c r="E2" s="62"/>
-      <c r="F2" s="62"/>
-      <c r="G2" s="62"/>
-      <c r="H2" s="62"/>
-      <c r="I2" s="62"/>
-      <c r="J2" s="62"/>
-      <c r="K2" s="62"/>
-      <c r="L2" s="62"/>
-      <c r="M2" s="62"/>
-      <c r="N2" s="62"/>
-      <c r="O2" s="62"/>
-      <c r="P2" s="63"/>
+      <c r="C2" s="64"/>
+      <c r="D2" s="64"/>
+      <c r="E2" s="64"/>
+      <c r="F2" s="64"/>
+      <c r="G2" s="64"/>
+      <c r="H2" s="64"/>
+      <c r="I2" s="64"/>
+      <c r="J2" s="64"/>
+      <c r="K2" s="64"/>
+      <c r="L2" s="64"/>
+      <c r="M2" s="64"/>
+      <c r="N2" s="64"/>
+      <c r="O2" s="64"/>
+      <c r="P2" s="65"/>
     </row>
     <row r="3" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B3" s="64"/>
-      <c r="C3" s="65"/>
-      <c r="D3" s="65"/>
-      <c r="E3" s="65"/>
-      <c r="F3" s="65"/>
-      <c r="G3" s="65"/>
-      <c r="H3" s="65"/>
-      <c r="I3" s="65"/>
-      <c r="J3" s="65"/>
-      <c r="K3" s="65"/>
-      <c r="L3" s="65"/>
-      <c r="M3" s="65"/>
-      <c r="N3" s="65"/>
-      <c r="O3" s="65"/>
-      <c r="P3" s="66"/>
+      <c r="B3" s="66"/>
+      <c r="C3" s="67"/>
+      <c r="D3" s="67"/>
+      <c r="E3" s="67"/>
+      <c r="F3" s="67"/>
+      <c r="G3" s="67"/>
+      <c r="H3" s="67"/>
+      <c r="I3" s="67"/>
+      <c r="J3" s="67"/>
+      <c r="K3" s="67"/>
+      <c r="L3" s="67"/>
+      <c r="M3" s="67"/>
+      <c r="N3" s="67"/>
+      <c r="O3" s="67"/>
+      <c r="P3" s="68"/>
       <c r="R3" s="12"/>
     </row>
     <row r="5" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B5" s="44" t="s">
+      <c r="B5" s="46" t="s">
         <v>18</v>
       </c>
-      <c r="C5" s="44"/>
-      <c r="D5" s="44"/>
-      <c r="E5" s="44"/>
-      <c r="F5" s="44"/>
-      <c r="G5" s="44"/>
+      <c r="C5" s="46"/>
+      <c r="D5" s="46"/>
+      <c r="E5" s="46"/>
+      <c r="F5" s="46"/>
+      <c r="G5" s="46"/>
       <c r="I5" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="K5" s="53" t="s">
+      <c r="K5" s="55" t="s">
         <v>8</v>
       </c>
-      <c r="L5" s="55"/>
-      <c r="M5" s="55"/>
-      <c r="N5" s="54"/>
+      <c r="L5" s="57"/>
+      <c r="M5" s="57"/>
+      <c r="N5" s="56"/>
       <c r="P5" s="4" t="s">
         <v>74</v>
       </c>
@@ -2809,28 +2860,28 @@
       </c>
     </row>
     <row r="9" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B9" s="56" t="s">
+      <c r="B9" s="58" t="s">
         <v>22</v>
       </c>
-      <c r="C9" s="56"/>
+      <c r="C9" s="58"/>
       <c r="E9" s="9" t="s">
         <v>67</v>
       </c>
     </row>
     <row r="10" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B10" s="57">
+      <c r="B10" s="59">
         <f>_xlfn.CEILING.MATH(SUM(B7:G7,I7,K7:N7,P7),1,1)</f>
         <v>110</v>
       </c>
-      <c r="C10" s="57"/>
-      <c r="E10" s="51">
+      <c r="C10" s="59"/>
+      <c r="E10" s="53">
         <v>4</v>
       </c>
     </row>
     <row r="11" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B11" s="57"/>
-      <c r="C11" s="57"/>
-      <c r="E11" s="52"/>
+      <c r="B11" s="59"/>
+      <c r="C11" s="59"/>
+      <c r="E11" s="54"/>
     </row>
     <row r="12" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A12" s="6"/>
@@ -2855,40 +2906,40 @@
     </row>
     <row r="13" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="14" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B14" s="61" t="s">
+      <c r="B14" s="63" t="s">
         <v>133</v>
       </c>
-      <c r="C14" s="62"/>
-      <c r="D14" s="62"/>
-      <c r="E14" s="62"/>
-      <c r="F14" s="62"/>
-      <c r="G14" s="62"/>
-      <c r="H14" s="63"/>
+      <c r="C14" s="64"/>
+      <c r="D14" s="64"/>
+      <c r="E14" s="64"/>
+      <c r="F14" s="64"/>
+      <c r="G14" s="64"/>
+      <c r="H14" s="65"/>
     </row>
     <row r="15" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B15" s="64"/>
-      <c r="C15" s="65"/>
-      <c r="D15" s="65"/>
-      <c r="E15" s="65"/>
-      <c r="F15" s="65"/>
-      <c r="G15" s="65"/>
-      <c r="H15" s="66"/>
+      <c r="B15" s="66"/>
+      <c r="C15" s="67"/>
+      <c r="D15" s="67"/>
+      <c r="E15" s="67"/>
+      <c r="F15" s="67"/>
+      <c r="G15" s="67"/>
+      <c r="H15" s="68"/>
     </row>
     <row r="17" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B17" s="44" t="s">
+      <c r="B17" s="46" t="s">
         <v>12</v>
       </c>
-      <c r="C17" s="44"/>
-      <c r="D17" s="44"/>
-      <c r="F17" s="44" t="s">
+      <c r="C17" s="46"/>
+      <c r="D17" s="46"/>
+      <c r="F17" s="46" t="s">
         <v>8</v>
       </c>
-      <c r="G17" s="44"/>
-      <c r="H17" s="44"/>
-      <c r="J17" s="56" t="s">
+      <c r="G17" s="46"/>
+      <c r="H17" s="46"/>
+      <c r="J17" s="58" t="s">
         <v>22</v>
       </c>
-      <c r="K17" s="56"/>
+      <c r="K17" s="58"/>
       <c r="M17" s="9" t="s">
         <v>67</v>
       </c>
@@ -2912,12 +2963,12 @@
       <c r="H18" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="J18" s="57">
+      <c r="J18" s="59">
         <f>SUM(B19:D19,F19:H19)</f>
         <v>93</v>
       </c>
-      <c r="K18" s="57"/>
-      <c r="M18" s="58">
+      <c r="K18" s="59"/>
+      <c r="M18" s="60">
         <v>5</v>
       </c>
     </row>
@@ -2940,9 +2991,9 @@
       <c r="H19" s="2">
         <v>4</v>
       </c>
-      <c r="J19" s="57"/>
-      <c r="K19" s="57"/>
-      <c r="M19" s="58"/>
+      <c r="J19" s="59"/>
+      <c r="K19" s="59"/>
+      <c r="M19" s="60"/>
     </row>
     <row r="21" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A21" s="6"/>
@@ -2967,46 +3018,46 @@
     </row>
     <row r="22" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="23" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B23" s="61" t="s">
+      <c r="B23" s="63" t="s">
         <v>134</v>
       </c>
-      <c r="C23" s="62"/>
-      <c r="D23" s="62"/>
-      <c r="E23" s="62"/>
-      <c r="F23" s="62"/>
-      <c r="G23" s="62"/>
-      <c r="H23" s="62"/>
-      <c r="I23" s="62"/>
-      <c r="J23" s="62"/>
-      <c r="K23" s="63"/>
+      <c r="C23" s="64"/>
+      <c r="D23" s="64"/>
+      <c r="E23" s="64"/>
+      <c r="F23" s="64"/>
+      <c r="G23" s="64"/>
+      <c r="H23" s="64"/>
+      <c r="I23" s="64"/>
+      <c r="J23" s="64"/>
+      <c r="K23" s="65"/>
     </row>
     <row r="24" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B24" s="64"/>
-      <c r="C24" s="65"/>
-      <c r="D24" s="65"/>
-      <c r="E24" s="65"/>
-      <c r="F24" s="65"/>
-      <c r="G24" s="65"/>
-      <c r="H24" s="65"/>
-      <c r="I24" s="65"/>
-      <c r="J24" s="65"/>
-      <c r="K24" s="66"/>
+      <c r="B24" s="66"/>
+      <c r="C24" s="67"/>
+      <c r="D24" s="67"/>
+      <c r="E24" s="67"/>
+      <c r="F24" s="67"/>
+      <c r="G24" s="67"/>
+      <c r="H24" s="67"/>
+      <c r="I24" s="67"/>
+      <c r="J24" s="67"/>
+      <c r="K24" s="68"/>
     </row>
     <row r="26" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B26" s="44" t="s">
+      <c r="B26" s="46" t="s">
         <v>17</v>
       </c>
-      <c r="C26" s="44"/>
-      <c r="E26" s="53" t="s">
+      <c r="C26" s="46"/>
+      <c r="E26" s="55" t="s">
         <v>21</v>
       </c>
-      <c r="F26" s="55"/>
-      <c r="G26" s="54"/>
-      <c r="I26" s="44" t="s">
+      <c r="F26" s="57"/>
+      <c r="G26" s="56"/>
+      <c r="I26" s="46" t="s">
         <v>20</v>
       </c>
-      <c r="J26" s="44"/>
-      <c r="K26" s="44"/>
+      <c r="J26" s="46"/>
+      <c r="K26" s="46"/>
       <c r="M26" s="10" t="s">
         <v>22</v>
       </c>
@@ -3041,12 +3092,12 @@
       <c r="K27" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="M27" s="67">
+      <c r="M27" s="69">
         <f>SUM(B28:C28,E28:G28,I28:K28)</f>
         <v>36</v>
       </c>
       <c r="N27" s="7"/>
-      <c r="O27" s="58">
+      <c r="O27" s="60">
         <v>4</v>
       </c>
       <c r="P27" s="8"/>
@@ -3076,9 +3127,9 @@
       <c r="K28" s="2">
         <v>3.2</v>
       </c>
-      <c r="M28" s="67"/>
+      <c r="M28" s="69"/>
       <c r="N28" s="7"/>
-      <c r="O28" s="58"/>
+      <c r="O28" s="60"/>
       <c r="P28" s="8"/>
     </row>
     <row r="30" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -3104,39 +3155,39 @@
     </row>
     <row r="31" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="32" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B32" s="61" t="s">
+      <c r="B32" s="63" t="s">
         <v>135</v>
       </c>
-      <c r="C32" s="62"/>
-      <c r="D32" s="62"/>
-      <c r="E32" s="62"/>
-      <c r="F32" s="62"/>
-      <c r="G32" s="62"/>
-      <c r="H32" s="62"/>
-      <c r="I32" s="63"/>
+      <c r="C32" s="64"/>
+      <c r="D32" s="64"/>
+      <c r="E32" s="64"/>
+      <c r="F32" s="64"/>
+      <c r="G32" s="64"/>
+      <c r="H32" s="64"/>
+      <c r="I32" s="65"/>
     </row>
     <row r="33" spans="2:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B33" s="64"/>
-      <c r="C33" s="65"/>
-      <c r="D33" s="65"/>
-      <c r="E33" s="65"/>
-      <c r="F33" s="65"/>
-      <c r="G33" s="65"/>
-      <c r="H33" s="65"/>
-      <c r="I33" s="66"/>
+      <c r="B33" s="66"/>
+      <c r="C33" s="67"/>
+      <c r="D33" s="67"/>
+      <c r="E33" s="67"/>
+      <c r="F33" s="67"/>
+      <c r="G33" s="67"/>
+      <c r="H33" s="67"/>
+      <c r="I33" s="68"/>
     </row>
     <row r="35" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B35" s="44" t="s">
+      <c r="B35" s="46" t="s">
         <v>31</v>
       </c>
-      <c r="C35" s="44"/>
-      <c r="D35" s="44"/>
-      <c r="F35" s="44" t="s">
+      <c r="C35" s="46"/>
+      <c r="D35" s="46"/>
+      <c r="F35" s="46" t="s">
         <v>12</v>
       </c>
-      <c r="G35" s="44"/>
-      <c r="H35" s="44"/>
-      <c r="I35" s="44"/>
+      <c r="G35" s="46"/>
+      <c r="H35" s="46"/>
+      <c r="I35" s="46"/>
       <c r="N35" s="7"/>
       <c r="O35" s="7"/>
     </row>
@@ -3193,14 +3244,14 @@
       <c r="O37" s="7"/>
     </row>
     <row r="40" spans="2:15" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B40" s="59" t="s">
+      <c r="B40" s="61" t="s">
         <v>35</v>
       </c>
-      <c r="C40" s="60"/>
-      <c r="F40" s="57" t="s">
+      <c r="C40" s="62"/>
+      <c r="F40" s="59" t="s">
         <v>36</v>
       </c>
-      <c r="G40" s="57"/>
+      <c r="G40" s="59"/>
       <c r="I40" s="9" t="s">
         <v>22</v>
       </c>
@@ -3256,7 +3307,7 @@
       <c r="G43" s="2">
         <v>0.44</v>
       </c>
-      <c r="I43" s="56" t="s">
+      <c r="I43" s="58" t="s">
         <v>67</v>
       </c>
     </row>
@@ -3273,7 +3324,7 @@
       <c r="G44" s="2">
         <v>1</v>
       </c>
-      <c r="I44" s="56"/>
+      <c r="I44" s="58"/>
     </row>
     <row r="45" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B45" s="2" t="s">
@@ -3417,67 +3468,67 @@
     </row>
     <row r="57" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="58" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B58" s="61" t="s">
+      <c r="B58" s="63" t="s">
         <v>136</v>
       </c>
-      <c r="C58" s="62"/>
-      <c r="D58" s="62"/>
-      <c r="E58" s="62"/>
-      <c r="F58" s="62"/>
-      <c r="G58" s="62"/>
-      <c r="H58" s="62"/>
-      <c r="I58" s="62"/>
-      <c r="J58" s="62"/>
-      <c r="K58" s="62"/>
-      <c r="L58" s="62"/>
-      <c r="M58" s="62"/>
-      <c r="N58" s="62"/>
-      <c r="O58" s="62"/>
-      <c r="P58" s="62"/>
-      <c r="Q58" s="62"/>
-      <c r="R58" s="63"/>
+      <c r="C58" s="64"/>
+      <c r="D58" s="64"/>
+      <c r="E58" s="64"/>
+      <c r="F58" s="64"/>
+      <c r="G58" s="64"/>
+      <c r="H58" s="64"/>
+      <c r="I58" s="64"/>
+      <c r="J58" s="64"/>
+      <c r="K58" s="64"/>
+      <c r="L58" s="64"/>
+      <c r="M58" s="64"/>
+      <c r="N58" s="64"/>
+      <c r="O58" s="64"/>
+      <c r="P58" s="64"/>
+      <c r="Q58" s="64"/>
+      <c r="R58" s="65"/>
     </row>
     <row r="59" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B59" s="64"/>
-      <c r="C59" s="65"/>
-      <c r="D59" s="65"/>
-      <c r="E59" s="65"/>
-      <c r="F59" s="65"/>
-      <c r="G59" s="65"/>
-      <c r="H59" s="65"/>
-      <c r="I59" s="65"/>
-      <c r="J59" s="65"/>
-      <c r="K59" s="65"/>
-      <c r="L59" s="65"/>
-      <c r="M59" s="65"/>
-      <c r="N59" s="65"/>
-      <c r="O59" s="65"/>
-      <c r="P59" s="65"/>
-      <c r="Q59" s="65"/>
-      <c r="R59" s="66"/>
+      <c r="B59" s="66"/>
+      <c r="C59" s="67"/>
+      <c r="D59" s="67"/>
+      <c r="E59" s="67"/>
+      <c r="F59" s="67"/>
+      <c r="G59" s="67"/>
+      <c r="H59" s="67"/>
+      <c r="I59" s="67"/>
+      <c r="J59" s="67"/>
+      <c r="K59" s="67"/>
+      <c r="L59" s="67"/>
+      <c r="M59" s="67"/>
+      <c r="N59" s="67"/>
+      <c r="O59" s="67"/>
+      <c r="P59" s="67"/>
+      <c r="Q59" s="67"/>
+      <c r="R59" s="68"/>
     </row>
     <row r="61" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B61" s="44" t="s">
+      <c r="B61" s="46" t="s">
         <v>63</v>
       </c>
-      <c r="C61" s="44"/>
-      <c r="D61" s="44"/>
-      <c r="E61" s="44"/>
-      <c r="F61" s="44"/>
-      <c r="G61" s="44"/>
-      <c r="H61" s="44"/>
-      <c r="I61" s="44"/>
-      <c r="J61" s="44"/>
-      <c r="K61" s="44"/>
-      <c r="M61" s="44" t="s">
+      <c r="C61" s="46"/>
+      <c r="D61" s="46"/>
+      <c r="E61" s="46"/>
+      <c r="F61" s="46"/>
+      <c r="G61" s="46"/>
+      <c r="H61" s="46"/>
+      <c r="I61" s="46"/>
+      <c r="J61" s="46"/>
+      <c r="K61" s="46"/>
+      <c r="M61" s="46" t="s">
         <v>68</v>
       </c>
-      <c r="N61" s="44"/>
-      <c r="O61" s="44"/>
-      <c r="Q61" s="44" t="s">
+      <c r="N61" s="46"/>
+      <c r="O61" s="46"/>
+      <c r="Q61" s="46" t="s">
         <v>64</v>
       </c>
-      <c r="R61" s="44"/>
+      <c r="R61" s="46"/>
     </row>
     <row r="62" spans="1:19" x14ac:dyDescent="0.25">
       <c r="B62" s="2" t="s">
@@ -3574,28 +3625,28 @@
       </c>
     </row>
     <row r="66" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B66" s="56" t="s">
+      <c r="B66" s="58" t="s">
         <v>22</v>
       </c>
-      <c r="C66" s="56"/>
+      <c r="C66" s="58"/>
       <c r="E66" s="9" t="s">
         <v>67</v>
       </c>
     </row>
     <row r="67" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B67" s="57">
+      <c r="B67" s="59">
         <f xml:space="preserve"> SUM(B63:K63,M63:O63,Q63:R63)</f>
         <v>85.5</v>
       </c>
-      <c r="C67" s="57"/>
-      <c r="E67" s="58">
+      <c r="C67" s="59"/>
+      <c r="E67" s="60">
         <v>4.5</v>
       </c>
     </row>
     <row r="68" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B68" s="57"/>
-      <c r="C68" s="57"/>
-      <c r="E68" s="58"/>
+      <c r="B68" s="59"/>
+      <c r="C68" s="59"/>
+      <c r="E68" s="60"/>
     </row>
     <row r="70" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A70" s="6"/>
@@ -3620,26 +3671,26 @@
     </row>
     <row r="71" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="72" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B72" s="61" t="s">
+      <c r="B72" s="63" t="s">
         <v>137</v>
       </c>
-      <c r="C72" s="62"/>
-      <c r="D72" s="62"/>
-      <c r="E72" s="62"/>
-      <c r="F72" s="62"/>
-      <c r="G72" s="62"/>
-      <c r="H72" s="62"/>
-      <c r="I72" s="63"/>
+      <c r="C72" s="64"/>
+      <c r="D72" s="64"/>
+      <c r="E72" s="64"/>
+      <c r="F72" s="64"/>
+      <c r="G72" s="64"/>
+      <c r="H72" s="64"/>
+      <c r="I72" s="65"/>
     </row>
     <row r="73" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B73" s="64"/>
-      <c r="C73" s="65"/>
-      <c r="D73" s="65"/>
-      <c r="E73" s="65"/>
-      <c r="F73" s="65"/>
-      <c r="G73" s="65"/>
-      <c r="H73" s="65"/>
-      <c r="I73" s="66"/>
+      <c r="B73" s="66"/>
+      <c r="C73" s="67"/>
+      <c r="D73" s="67"/>
+      <c r="E73" s="67"/>
+      <c r="F73" s="67"/>
+      <c r="G73" s="67"/>
+      <c r="H73" s="67"/>
+      <c r="I73" s="68"/>
     </row>
     <row r="75" spans="1:19" x14ac:dyDescent="0.25">
       <c r="B75" s="4" t="s">
@@ -3666,10 +3717,10 @@
       <c r="I75" s="4" t="s">
         <v>145</v>
       </c>
-      <c r="K75" s="56" t="s">
+      <c r="K75" s="58" t="s">
         <v>22</v>
       </c>
-      <c r="L75" s="56"/>
+      <c r="L75" s="58"/>
       <c r="N75" s="9" t="s">
         <v>67</v>
       </c>
@@ -3699,11 +3750,11 @@
       <c r="I76" s="2">
         <v>5</v>
       </c>
-      <c r="K76" s="57">
+      <c r="K76" s="59">
         <f>SUM(B76:I76)</f>
         <v>96</v>
       </c>
-      <c r="L76" s="57"/>
+      <c r="L76" s="59"/>
       <c r="N76" s="13">
         <v>5</v>
       </c>
@@ -4371,21 +4422,21 @@
   <sheetData>
     <row r="1" spans="2:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="2" spans="2:12" ht="23.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B2" s="68" t="s">
+      <c r="B2" s="70" t="s">
         <v>203</v>
       </c>
-      <c r="C2" s="69"/>
-      <c r="D2" s="70"/>
-      <c r="F2" s="68" t="s">
+      <c r="C2" s="71"/>
+      <c r="D2" s="72"/>
+      <c r="F2" s="70" t="s">
         <v>204</v>
       </c>
-      <c r="G2" s="69"/>
-      <c r="H2" s="70"/>
-      <c r="J2" s="68" t="s">
+      <c r="G2" s="71"/>
+      <c r="H2" s="72"/>
+      <c r="J2" s="70" t="s">
         <v>205</v>
       </c>
-      <c r="K2" s="69"/>
-      <c r="L2" s="70"/>
+      <c r="K2" s="71"/>
+      <c r="L2" s="72"/>
     </row>
     <row r="3" spans="2:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B3" s="34" t="s">
@@ -4560,26 +4611,26 @@
     </row>
     <row r="10" spans="2:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="11" spans="2:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B11" s="71" t="s">
+      <c r="B11" s="73" t="s">
         <v>197</v>
       </c>
-      <c r="C11" s="72"/>
+      <c r="C11" s="74"/>
       <c r="D11" s="33">
         <f>(D4*C4+D5*C5+D6*C6+D7*C7+D8*C8+D9*C9)/30</f>
         <v>4.4333333333333336</v>
       </c>
-      <c r="F11" s="71" t="s">
+      <c r="F11" s="73" t="s">
         <v>197</v>
       </c>
-      <c r="G11" s="72"/>
+      <c r="G11" s="74"/>
       <c r="H11" s="33">
         <f>(H4*G4+H5*G5+H6*G6+H7*G7+H8*G8)/30</f>
         <v>0</v>
       </c>
-      <c r="J11" s="71" t="s">
+      <c r="J11" s="73" t="s">
         <v>197</v>
       </c>
-      <c r="K11" s="72"/>
+      <c r="K11" s="74"/>
       <c r="L11" s="33">
         <f>(L4*K4+L5*K5+L6*K6+L7*K7+L8*K8)/30</f>
         <v>0</v>

</xml_diff>

<commit_message>
POTEC - new points -> passed
</commit_message>
<xml_diff>
--- a/IoT-points-schedule.xlsx
+++ b/IoT-points-schedule.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\dodo\Desktop\IoT-studies\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5FF09843-948A-4068-B4D0-581168967817}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A6B41023-C553-44AC-BF28-ADE8015752C5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="25440" windowHeight="15390" xr2:uid="{F85F5544-1FE8-4920-A5D4-192A98B113BD}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="355" uniqueCount="226">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="354" uniqueCount="226">
   <si>
     <t>1. Krypto</t>
   </si>
@@ -1104,7 +1104,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="76">
+  <cellXfs count="84">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1248,10 +1248,13 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1272,28 +1275,16 @@
     <xf numFmtId="0" fontId="5" fillId="5" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
@@ -1302,6 +1293,18 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1338,7 +1341,28 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="7" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="7" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="7" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="7" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="7" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="7" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1729,59 +1753,59 @@
   <sheetData>
     <row r="1" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="2" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B2" s="47" t="s">
+      <c r="B2" s="48" t="s">
         <v>76</v>
       </c>
-      <c r="C2" s="48"/>
-      <c r="D2" s="48"/>
-      <c r="E2" s="48"/>
-      <c r="F2" s="48"/>
-      <c r="G2" s="48"/>
-      <c r="H2" s="48"/>
-      <c r="I2" s="48"/>
-      <c r="J2" s="48"/>
-      <c r="K2" s="48"/>
-      <c r="L2" s="48"/>
-      <c r="M2" s="48"/>
-      <c r="N2" s="48"/>
-      <c r="O2" s="48"/>
-      <c r="P2" s="49"/>
+      <c r="C2" s="49"/>
+      <c r="D2" s="49"/>
+      <c r="E2" s="49"/>
+      <c r="F2" s="49"/>
+      <c r="G2" s="49"/>
+      <c r="H2" s="49"/>
+      <c r="I2" s="49"/>
+      <c r="J2" s="49"/>
+      <c r="K2" s="49"/>
+      <c r="L2" s="49"/>
+      <c r="M2" s="49"/>
+      <c r="N2" s="49"/>
+      <c r="O2" s="49"/>
+      <c r="P2" s="50"/>
     </row>
     <row r="3" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B3" s="50"/>
-      <c r="C3" s="51"/>
-      <c r="D3" s="51"/>
-      <c r="E3" s="51"/>
-      <c r="F3" s="51"/>
-      <c r="G3" s="51"/>
-      <c r="H3" s="51"/>
-      <c r="I3" s="51"/>
-      <c r="J3" s="51"/>
-      <c r="K3" s="51"/>
-      <c r="L3" s="51"/>
-      <c r="M3" s="51"/>
-      <c r="N3" s="51"/>
-      <c r="O3" s="51"/>
-      <c r="P3" s="52"/>
+      <c r="B3" s="51"/>
+      <c r="C3" s="52"/>
+      <c r="D3" s="52"/>
+      <c r="E3" s="52"/>
+      <c r="F3" s="52"/>
+      <c r="G3" s="52"/>
+      <c r="H3" s="52"/>
+      <c r="I3" s="52"/>
+      <c r="J3" s="52"/>
+      <c r="K3" s="52"/>
+      <c r="L3" s="52"/>
+      <c r="M3" s="52"/>
+      <c r="N3" s="52"/>
+      <c r="O3" s="52"/>
+      <c r="P3" s="53"/>
       <c r="R3" s="12"/>
     </row>
     <row r="5" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B5" s="55" t="s">
+      <c r="B5" s="54" t="s">
         <v>83</v>
       </c>
-      <c r="C5" s="57"/>
-      <c r="D5" s="57"/>
-      <c r="E5" s="57"/>
+      <c r="C5" s="55"/>
+      <c r="D5" s="55"/>
+      <c r="E5" s="55"/>
       <c r="F5" s="56"/>
-      <c r="H5" s="55" t="s">
+      <c r="H5" s="54" t="s">
         <v>82</v>
       </c>
       <c r="I5" s="56"/>
-      <c r="K5" s="55" t="s">
+      <c r="K5" s="54" t="s">
         <v>8</v>
       </c>
-      <c r="L5" s="57"/>
-      <c r="M5" s="57"/>
+      <c r="L5" s="55"/>
+      <c r="M5" s="55"/>
       <c r="N5" s="56"/>
       <c r="P5" s="4" t="s">
         <v>74</v>
@@ -1850,37 +1874,37 @@
       <c r="P7" s="2"/>
     </row>
     <row r="9" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B9" s="58" t="s">
+      <c r="B9" s="57" t="s">
         <v>22</v>
       </c>
-      <c r="C9" s="58"/>
+      <c r="C9" s="57"/>
       <c r="E9" s="9" t="s">
         <v>67</v>
       </c>
-      <c r="G9" s="58" t="s">
+      <c r="G9" s="57" t="s">
         <v>87</v>
       </c>
-      <c r="H9" s="58"/>
+      <c r="H9" s="57"/>
     </row>
     <row r="10" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B10" s="59">
+      <c r="B10" s="46">
         <f>SUM(B7:F7,H7:I7,K7:N7,P7)</f>
         <v>25.7</v>
       </c>
-      <c r="C10" s="59"/>
-      <c r="E10" s="53"/>
-      <c r="G10" s="59">
+      <c r="C10" s="46"/>
+      <c r="E10" s="61"/>
+      <c r="G10" s="46">
         <f>66-SUM(B7:F7,H7:I7,K7:N7,P7)</f>
         <v>40.299999999999997</v>
       </c>
-      <c r="H10" s="59"/>
+      <c r="H10" s="46"/>
     </row>
     <row r="11" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B11" s="59"/>
-      <c r="C11" s="59"/>
-      <c r="E11" s="54"/>
-      <c r="G11" s="59"/>
-      <c r="H11" s="59"/>
+      <c r="B11" s="46"/>
+      <c r="C11" s="46"/>
+      <c r="E11" s="62"/>
+      <c r="G11" s="46"/>
+      <c r="H11" s="46"/>
     </row>
     <row r="12" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A12" s="6"/>
@@ -1905,46 +1929,46 @@
     </row>
     <row r="13" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="14" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B14" s="47" t="s">
+      <c r="B14" s="48" t="s">
         <v>77</v>
       </c>
-      <c r="C14" s="48"/>
-      <c r="D14" s="48"/>
-      <c r="E14" s="48"/>
-      <c r="F14" s="48"/>
-      <c r="G14" s="48"/>
-      <c r="H14" s="49"/>
+      <c r="C14" s="49"/>
+      <c r="D14" s="49"/>
+      <c r="E14" s="49"/>
+      <c r="F14" s="49"/>
+      <c r="G14" s="49"/>
+      <c r="H14" s="50"/>
     </row>
     <row r="15" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B15" s="50"/>
-      <c r="C15" s="51"/>
-      <c r="D15" s="51"/>
-      <c r="E15" s="51"/>
-      <c r="F15" s="51"/>
-      <c r="G15" s="51"/>
-      <c r="H15" s="52"/>
+      <c r="B15" s="51"/>
+      <c r="C15" s="52"/>
+      <c r="D15" s="52"/>
+      <c r="E15" s="52"/>
+      <c r="F15" s="52"/>
+      <c r="G15" s="52"/>
+      <c r="H15" s="53"/>
     </row>
     <row r="17" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B17" s="46" t="s">
+      <c r="B17" s="60" t="s">
         <v>91</v>
       </c>
-      <c r="C17" s="46"/>
-      <c r="D17" s="46"/>
-      <c r="E17" s="46"/>
-      <c r="F17" s="46"/>
-      <c r="H17" s="55" t="s">
+      <c r="C17" s="60"/>
+      <c r="D17" s="60"/>
+      <c r="E17" s="60"/>
+      <c r="F17" s="60"/>
+      <c r="H17" s="54" t="s">
         <v>97</v>
       </c>
-      <c r="I17" s="57"/>
+      <c r="I17" s="55"/>
       <c r="J17" s="56"/>
-      <c r="L17" s="58" t="s">
+      <c r="L17" s="57" t="s">
         <v>22</v>
       </c>
-      <c r="M17" s="58"/>
-      <c r="O17" s="58" t="s">
+      <c r="M17" s="57"/>
+      <c r="O17" s="57" t="s">
         <v>87</v>
       </c>
-      <c r="P17" s="58"/>
+      <c r="P17" s="57"/>
       <c r="R17" s="9" t="s">
         <v>67</v>
       </c>
@@ -1974,17 +1998,17 @@
       <c r="J18" s="3" t="s">
         <v>95</v>
       </c>
-      <c r="L18" s="59">
+      <c r="L18" s="46">
         <f>SUM(B19:F19,H19:J19)</f>
         <v>29.5</v>
       </c>
-      <c r="M18" s="59"/>
-      <c r="O18" s="59">
+      <c r="M18" s="46"/>
+      <c r="O18" s="46">
         <f>50-SUM(B19:F19,H19:J19)</f>
         <v>20.5</v>
       </c>
-      <c r="P18" s="59"/>
-      <c r="R18" s="60"/>
+      <c r="P18" s="46"/>
+      <c r="R18" s="47"/>
     </row>
     <row r="19" spans="1:19" x14ac:dyDescent="0.25">
       <c r="B19" s="2"/>
@@ -1999,11 +2023,11 @@
         <v>26.5</v>
       </c>
       <c r="J19" s="2"/>
-      <c r="L19" s="59"/>
-      <c r="M19" s="59"/>
-      <c r="O19" s="59"/>
-      <c r="P19" s="59"/>
-      <c r="R19" s="60"/>
+      <c r="L19" s="46"/>
+      <c r="M19" s="46"/>
+      <c r="O19" s="46"/>
+      <c r="P19" s="46"/>
+      <c r="R19" s="47"/>
     </row>
     <row r="21" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A21" s="6"/>
@@ -2028,53 +2052,53 @@
     </row>
     <row r="22" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="23" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B23" s="47" t="s">
+      <c r="B23" s="48" t="s">
         <v>79</v>
       </c>
-      <c r="C23" s="48"/>
-      <c r="D23" s="48"/>
-      <c r="E23" s="48"/>
-      <c r="F23" s="48"/>
-      <c r="G23" s="48"/>
-      <c r="H23" s="48"/>
-      <c r="I23" s="48"/>
-      <c r="J23" s="48"/>
-      <c r="K23" s="48"/>
-      <c r="L23" s="49"/>
-      <c r="N23" s="59" t="s">
+      <c r="C23" s="49"/>
+      <c r="D23" s="49"/>
+      <c r="E23" s="49"/>
+      <c r="F23" s="49"/>
+      <c r="G23" s="49"/>
+      <c r="H23" s="49"/>
+      <c r="I23" s="49"/>
+      <c r="J23" s="49"/>
+      <c r="K23" s="49"/>
+      <c r="L23" s="50"/>
+      <c r="N23" s="46" t="s">
         <v>131</v>
       </c>
-      <c r="O23" s="59"/>
+      <c r="O23" s="46"/>
     </row>
     <row r="24" spans="1:19" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B24" s="50"/>
-      <c r="C24" s="51"/>
-      <c r="D24" s="51"/>
-      <c r="E24" s="51"/>
-      <c r="F24" s="51"/>
-      <c r="G24" s="51"/>
-      <c r="H24" s="51"/>
-      <c r="I24" s="51"/>
-      <c r="J24" s="51"/>
-      <c r="K24" s="51"/>
-      <c r="L24" s="52"/>
-      <c r="N24" s="59"/>
-      <c r="O24" s="59"/>
+      <c r="B24" s="51"/>
+      <c r="C24" s="52"/>
+      <c r="D24" s="52"/>
+      <c r="E24" s="52"/>
+      <c r="F24" s="52"/>
+      <c r="G24" s="52"/>
+      <c r="H24" s="52"/>
+      <c r="I24" s="52"/>
+      <c r="J24" s="52"/>
+      <c r="K24" s="52"/>
+      <c r="L24" s="53"/>
+      <c r="N24" s="46"/>
+      <c r="O24" s="46"/>
     </row>
     <row r="26" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B26" s="46" t="s">
+      <c r="B26" s="60" t="s">
         <v>129</v>
       </c>
-      <c r="C26" s="46"/>
-      <c r="D26" s="46"/>
-      <c r="F26" s="46" t="s">
+      <c r="C26" s="60"/>
+      <c r="D26" s="60"/>
+      <c r="F26" s="60" t="s">
         <v>210</v>
       </c>
-      <c r="G26" s="46"/>
-      <c r="H26" s="46"/>
-      <c r="I26" s="46"/>
+      <c r="G26" s="60"/>
+      <c r="H26" s="60"/>
+      <c r="I26" s="60"/>
       <c r="J26" s="7"/>
-      <c r="K26" s="55" t="s">
+      <c r="K26" s="54" t="s">
         <v>128</v>
       </c>
       <c r="L26" s="56"/>
@@ -2110,7 +2134,7 @@
       <c r="L27" s="2" t="s">
         <v>127</v>
       </c>
-      <c r="N27" s="53"/>
+      <c r="N27" s="61"/>
     </row>
     <row r="28" spans="1:19" x14ac:dyDescent="0.25">
       <c r="B28" s="2">
@@ -2134,20 +2158,20 @@
       </c>
       <c r="K28" s="2"/>
       <c r="L28" s="2"/>
-      <c r="N28" s="54"/>
+      <c r="N28" s="62"/>
     </row>
     <row r="29" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B29" s="45"/>
-      <c r="C29" s="45"/>
-      <c r="D29" s="45"/>
-      <c r="F29" s="45">
+      <c r="B29" s="63"/>
+      <c r="C29" s="63"/>
+      <c r="D29" s="63"/>
+      <c r="F29" s="63">
         <v>5</v>
       </c>
-      <c r="G29" s="45"/>
-      <c r="H29" s="45"/>
-      <c r="I29" s="45"/>
-      <c r="K29" s="45"/>
-      <c r="L29" s="45"/>
+      <c r="G29" s="63"/>
+      <c r="H29" s="63"/>
+      <c r="I29" s="63"/>
+      <c r="K29" s="63"/>
+      <c r="L29" s="63"/>
       <c r="N29" s="44"/>
     </row>
     <row r="31" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -2173,38 +2197,38 @@
     </row>
     <row r="32" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="33" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B33" s="47" t="s">
+      <c r="B33" s="76" t="s">
         <v>78</v>
       </c>
-      <c r="C33" s="48"/>
-      <c r="D33" s="48"/>
-      <c r="E33" s="48"/>
-      <c r="F33" s="48"/>
-      <c r="G33" s="48"/>
-      <c r="H33" s="48"/>
-      <c r="I33" s="49"/>
+      <c r="C33" s="77"/>
+      <c r="D33" s="77"/>
+      <c r="E33" s="77"/>
+      <c r="F33" s="77"/>
+      <c r="G33" s="77"/>
+      <c r="H33" s="77"/>
+      <c r="I33" s="78"/>
     </row>
     <row r="34" spans="2:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B34" s="50"/>
-      <c r="C34" s="51"/>
-      <c r="D34" s="51"/>
-      <c r="E34" s="51"/>
-      <c r="F34" s="51"/>
-      <c r="G34" s="51"/>
-      <c r="H34" s="51"/>
-      <c r="I34" s="52"/>
+      <c r="B34" s="79"/>
+      <c r="C34" s="80"/>
+      <c r="D34" s="80"/>
+      <c r="E34" s="80"/>
+      <c r="F34" s="80"/>
+      <c r="G34" s="80"/>
+      <c r="H34" s="80"/>
+      <c r="I34" s="81"/>
     </row>
     <row r="36" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B36" s="46" t="s">
+      <c r="B36" s="60" t="s">
         <v>98</v>
       </c>
-      <c r="C36" s="46"/>
+      <c r="C36" s="60"/>
       <c r="D36" s="7"/>
-      <c r="E36" s="55" t="s">
+      <c r="E36" s="54" t="s">
         <v>146</v>
       </c>
-      <c r="F36" s="57"/>
-      <c r="G36" s="57"/>
+      <c r="F36" s="55"/>
+      <c r="G36" s="55"/>
       <c r="H36" s="56"/>
     </row>
     <row r="37" spans="2:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -2235,25 +2259,25 @@
       <c r="C38" s="2"/>
       <c r="E38" s="2">
         <f>C57</f>
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="F38" s="2">
         <f>G52</f>
-        <v>9</v>
+        <v>19</v>
       </c>
       <c r="G38" s="2"/>
       <c r="H38" s="2"/>
       <c r="O38" s="7"/>
     </row>
     <row r="41" spans="2:15" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B41" s="61" t="s">
+      <c r="B41" s="58" t="s">
         <v>126</v>
       </c>
-      <c r="C41" s="62"/>
-      <c r="F41" s="59" t="s">
+      <c r="C41" s="59"/>
+      <c r="F41" s="46" t="s">
         <v>102</v>
       </c>
-      <c r="G41" s="59"/>
+      <c r="G41" s="46"/>
       <c r="I41" s="9" t="s">
         <v>22</v>
       </c>
@@ -2275,7 +2299,7 @@
       </c>
       <c r="I42" s="2">
         <f>SUM(B38:C38,E38:H38)</f>
-        <v>41</v>
+        <v>53</v>
       </c>
       <c r="J42" s="7"/>
       <c r="L42" s="7"/>
@@ -2288,7 +2312,9 @@
       <c r="F43" s="2" t="s">
         <v>118</v>
       </c>
-      <c r="G43" s="2"/>
+      <c r="G43" s="2">
+        <v>10</v>
+      </c>
       <c r="I43" s="7"/>
       <c r="J43" s="7"/>
     </row>
@@ -2303,7 +2329,7 @@
         <v>119</v>
       </c>
       <c r="G44" s="2"/>
-      <c r="I44" s="58" t="s">
+      <c r="I44" s="57" t="s">
         <v>67</v>
       </c>
     </row>
@@ -2318,7 +2344,7 @@
         <v>120</v>
       </c>
       <c r="G45" s="2"/>
-      <c r="I45" s="58"/>
+      <c r="I45" s="57"/>
     </row>
     <row r="46" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B46" s="2" t="s">
@@ -2331,7 +2357,9 @@
         <v>121</v>
       </c>
       <c r="G46" s="2"/>
-      <c r="I46" s="13"/>
+      <c r="I46" s="13">
+        <v>3</v>
+      </c>
     </row>
     <row r="47" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B47" s="2" t="s">
@@ -2352,9 +2380,7 @@
         <v>123</v>
       </c>
       <c r="G48" s="2"/>
-      <c r="I48" s="9" t="s">
-        <v>87</v>
-      </c>
+      <c r="I48" s="82"/>
     </row>
     <row r="49" spans="1:19" x14ac:dyDescent="0.25">
       <c r="B49" s="2" t="s">
@@ -2367,10 +2393,7 @@
         <v>124</v>
       </c>
       <c r="G49" s="2"/>
-      <c r="I49" s="2">
-        <f>50-SUM(B38:C38,E38:H38)</f>
-        <v>9</v>
-      </c>
+      <c r="I49" s="83"/>
     </row>
     <row r="50" spans="1:19" x14ac:dyDescent="0.25">
       <c r="B50" s="2" t="s">
@@ -2386,7 +2409,9 @@
       <c r="B51" s="2" t="s">
         <v>112</v>
       </c>
-      <c r="C51" s="2"/>
+      <c r="C51" s="2">
+        <v>2</v>
+      </c>
     </row>
     <row r="52" spans="1:19" x14ac:dyDescent="0.25">
       <c r="B52" s="2" t="s">
@@ -2398,7 +2423,7 @@
       </c>
       <c r="G52" s="2">
         <f>SUM(G42:G50)</f>
-        <v>9</v>
+        <v>19</v>
       </c>
     </row>
     <row r="53" spans="1:19" x14ac:dyDescent="0.25">
@@ -2425,7 +2450,7 @@
       </c>
       <c r="C57" s="2">
         <f>SUM(C42:C55)</f>
-        <v>15</v>
+        <v>17</v>
       </c>
     </row>
     <row r="59" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -2451,70 +2476,70 @@
     </row>
     <row r="60" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="61" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B61" s="47" t="s">
+      <c r="B61" s="48" t="s">
         <v>80</v>
       </c>
-      <c r="C61" s="48"/>
-      <c r="D61" s="48"/>
-      <c r="E61" s="48"/>
-      <c r="F61" s="48"/>
-      <c r="G61" s="48"/>
-      <c r="H61" s="48"/>
-      <c r="I61" s="48"/>
-      <c r="J61" s="48"/>
-      <c r="K61" s="48"/>
-      <c r="L61" s="48"/>
-      <c r="M61" s="48"/>
-      <c r="N61" s="48"/>
-      <c r="O61" s="48"/>
-      <c r="P61" s="48"/>
-      <c r="Q61" s="48"/>
-      <c r="R61" s="48"/>
-      <c r="S61" s="49"/>
+      <c r="C61" s="49"/>
+      <c r="D61" s="49"/>
+      <c r="E61" s="49"/>
+      <c r="F61" s="49"/>
+      <c r="G61" s="49"/>
+      <c r="H61" s="49"/>
+      <c r="I61" s="49"/>
+      <c r="J61" s="49"/>
+      <c r="K61" s="49"/>
+      <c r="L61" s="49"/>
+      <c r="M61" s="49"/>
+      <c r="N61" s="49"/>
+      <c r="O61" s="49"/>
+      <c r="P61" s="49"/>
+      <c r="Q61" s="49"/>
+      <c r="R61" s="49"/>
+      <c r="S61" s="50"/>
     </row>
     <row r="62" spans="1:19" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B62" s="50"/>
-      <c r="C62" s="51"/>
-      <c r="D62" s="51"/>
-      <c r="E62" s="51"/>
-      <c r="F62" s="51"/>
-      <c r="G62" s="51"/>
-      <c r="H62" s="51"/>
-      <c r="I62" s="51"/>
-      <c r="J62" s="51"/>
-      <c r="K62" s="51"/>
-      <c r="L62" s="51"/>
-      <c r="M62" s="51"/>
-      <c r="N62" s="51"/>
-      <c r="O62" s="51"/>
-      <c r="P62" s="51"/>
-      <c r="Q62" s="51"/>
-      <c r="R62" s="51"/>
-      <c r="S62" s="52"/>
+      <c r="B62" s="51"/>
+      <c r="C62" s="52"/>
+      <c r="D62" s="52"/>
+      <c r="E62" s="52"/>
+      <c r="F62" s="52"/>
+      <c r="G62" s="52"/>
+      <c r="H62" s="52"/>
+      <c r="I62" s="52"/>
+      <c r="J62" s="52"/>
+      <c r="K62" s="52"/>
+      <c r="L62" s="52"/>
+      <c r="M62" s="52"/>
+      <c r="N62" s="52"/>
+      <c r="O62" s="52"/>
+      <c r="P62" s="52"/>
+      <c r="Q62" s="52"/>
+      <c r="R62" s="52"/>
+      <c r="S62" s="53"/>
     </row>
     <row r="64" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B64" s="46" t="s">
+      <c r="B64" s="60" t="s">
         <v>63</v>
       </c>
-      <c r="C64" s="46"/>
-      <c r="D64" s="46"/>
-      <c r="E64" s="46"/>
-      <c r="F64" s="46"/>
-      <c r="G64" s="46"/>
-      <c r="H64" s="46"/>
-      <c r="I64" s="46"/>
-      <c r="J64" s="46"/>
-      <c r="K64" s="46"/>
-      <c r="M64" s="46" t="s">
+      <c r="C64" s="60"/>
+      <c r="D64" s="60"/>
+      <c r="E64" s="60"/>
+      <c r="F64" s="60"/>
+      <c r="G64" s="60"/>
+      <c r="H64" s="60"/>
+      <c r="I64" s="60"/>
+      <c r="J64" s="60"/>
+      <c r="K64" s="60"/>
+      <c r="M64" s="60" t="s">
         <v>90</v>
       </c>
-      <c r="N64" s="46"/>
-      <c r="O64" s="46"/>
-      <c r="P64" s="46"/>
-      <c r="R64" s="46" t="s">
+      <c r="N64" s="60"/>
+      <c r="O64" s="60"/>
+      <c r="P64" s="60"/>
+      <c r="R64" s="60" t="s">
         <v>64</v>
       </c>
-      <c r="S64" s="46"/>
+      <c r="S64" s="60"/>
     </row>
     <row r="65" spans="2:19" x14ac:dyDescent="0.25">
       <c r="B65" s="2" t="s">
@@ -2607,47 +2632,73 @@
       <c r="S66" s="2"/>
     </row>
     <row r="69" spans="2:19" x14ac:dyDescent="0.25">
-      <c r="B69" s="58" t="s">
+      <c r="B69" s="57" t="s">
         <v>22</v>
       </c>
-      <c r="C69" s="58"/>
+      <c r="C69" s="57"/>
       <c r="E69" s="9" t="s">
         <v>67</v>
       </c>
-      <c r="G69" s="58" t="s">
+      <c r="G69" s="57" t="s">
         <v>87</v>
       </c>
-      <c r="H69" s="58"/>
-      <c r="K69" s="75" t="s">
+      <c r="H69" s="57"/>
+      <c r="K69" s="45" t="s">
         <v>225</v>
       </c>
     </row>
     <row r="70" spans="2:19" x14ac:dyDescent="0.25">
-      <c r="B70" s="59">
+      <c r="B70" s="46">
         <f>SUM(B66:K66,M66:P66,R66:S66,K70)</f>
         <v>27</v>
       </c>
-      <c r="C70" s="59"/>
-      <c r="E70" s="60"/>
-      <c r="G70" s="59">
+      <c r="C70" s="46"/>
+      <c r="E70" s="47"/>
+      <c r="G70" s="46">
         <f>50-SUM(B66:K66,M66:P66,R66:S66,K70)</f>
         <v>23</v>
       </c>
-      <c r="H70" s="59"/>
-      <c r="K70" s="59">
+      <c r="H70" s="46"/>
+      <c r="K70" s="46">
         <v>3</v>
       </c>
     </row>
     <row r="71" spans="2:19" x14ac:dyDescent="0.25">
-      <c r="B71" s="59"/>
-      <c r="C71" s="59"/>
-      <c r="E71" s="60"/>
-      <c r="G71" s="59"/>
-      <c r="H71" s="59"/>
-      <c r="K71" s="59"/>
+      <c r="B71" s="46"/>
+      <c r="C71" s="46"/>
+      <c r="E71" s="47"/>
+      <c r="G71" s="46"/>
+      <c r="H71" s="46"/>
+      <c r="K71" s="46"/>
     </row>
   </sheetData>
   <mergeCells count="42">
+    <mergeCell ref="K29:L29"/>
+    <mergeCell ref="R64:S64"/>
+    <mergeCell ref="B33:I34"/>
+    <mergeCell ref="B64:K64"/>
+    <mergeCell ref="B61:S62"/>
+    <mergeCell ref="M64:P64"/>
+    <mergeCell ref="N27:N28"/>
+    <mergeCell ref="F26:I26"/>
+    <mergeCell ref="K26:L26"/>
+    <mergeCell ref="B23:L24"/>
+    <mergeCell ref="B26:D26"/>
+    <mergeCell ref="O17:P17"/>
+    <mergeCell ref="B9:C9"/>
+    <mergeCell ref="B10:C11"/>
+    <mergeCell ref="L17:M17"/>
+    <mergeCell ref="E10:E11"/>
+    <mergeCell ref="G10:H11"/>
+    <mergeCell ref="E70:E71"/>
+    <mergeCell ref="B69:C69"/>
+    <mergeCell ref="B70:C71"/>
+    <mergeCell ref="G69:H69"/>
+    <mergeCell ref="G70:H71"/>
+    <mergeCell ref="B17:F17"/>
+    <mergeCell ref="H17:J17"/>
+    <mergeCell ref="F29:I29"/>
+    <mergeCell ref="B29:D29"/>
     <mergeCell ref="K70:K71"/>
     <mergeCell ref="R18:R19"/>
     <mergeCell ref="B14:H15"/>
@@ -2664,32 +2715,6 @@
     <mergeCell ref="B36:C36"/>
     <mergeCell ref="E36:H36"/>
     <mergeCell ref="G9:H9"/>
-    <mergeCell ref="G10:H11"/>
-    <mergeCell ref="E70:E71"/>
-    <mergeCell ref="B69:C69"/>
-    <mergeCell ref="B70:C71"/>
-    <mergeCell ref="G69:H69"/>
-    <mergeCell ref="G70:H71"/>
-    <mergeCell ref="B17:F17"/>
-    <mergeCell ref="H17:J17"/>
-    <mergeCell ref="O17:P17"/>
-    <mergeCell ref="B9:C9"/>
-    <mergeCell ref="B10:C11"/>
-    <mergeCell ref="L17:M17"/>
-    <mergeCell ref="E10:E11"/>
-    <mergeCell ref="N27:N28"/>
-    <mergeCell ref="F26:I26"/>
-    <mergeCell ref="K26:L26"/>
-    <mergeCell ref="B23:L24"/>
-    <mergeCell ref="B26:D26"/>
-    <mergeCell ref="F29:I29"/>
-    <mergeCell ref="B29:D29"/>
-    <mergeCell ref="K29:L29"/>
-    <mergeCell ref="R64:S64"/>
-    <mergeCell ref="B33:I34"/>
-    <mergeCell ref="B64:K64"/>
-    <mergeCell ref="B61:S62"/>
-    <mergeCell ref="M64:P64"/>
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2725,59 +2750,59 @@
   <sheetData>
     <row r="1" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="2" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B2" s="63" t="s">
+      <c r="B2" s="64" t="s">
         <v>132</v>
       </c>
-      <c r="C2" s="64"/>
-      <c r="D2" s="64"/>
-      <c r="E2" s="64"/>
-      <c r="F2" s="64"/>
-      <c r="G2" s="64"/>
-      <c r="H2" s="64"/>
-      <c r="I2" s="64"/>
-      <c r="J2" s="64"/>
-      <c r="K2" s="64"/>
-      <c r="L2" s="64"/>
-      <c r="M2" s="64"/>
-      <c r="N2" s="64"/>
-      <c r="O2" s="64"/>
-      <c r="P2" s="65"/>
+      <c r="C2" s="65"/>
+      <c r="D2" s="65"/>
+      <c r="E2" s="65"/>
+      <c r="F2" s="65"/>
+      <c r="G2" s="65"/>
+      <c r="H2" s="65"/>
+      <c r="I2" s="65"/>
+      <c r="J2" s="65"/>
+      <c r="K2" s="65"/>
+      <c r="L2" s="65"/>
+      <c r="M2" s="65"/>
+      <c r="N2" s="65"/>
+      <c r="O2" s="65"/>
+      <c r="P2" s="66"/>
     </row>
     <row r="3" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B3" s="66"/>
-      <c r="C3" s="67"/>
-      <c r="D3" s="67"/>
-      <c r="E3" s="67"/>
-      <c r="F3" s="67"/>
-      <c r="G3" s="67"/>
-      <c r="H3" s="67"/>
-      <c r="I3" s="67"/>
-      <c r="J3" s="67"/>
-      <c r="K3" s="67"/>
-      <c r="L3" s="67"/>
-      <c r="M3" s="67"/>
-      <c r="N3" s="67"/>
-      <c r="O3" s="67"/>
-      <c r="P3" s="68"/>
+      <c r="B3" s="67"/>
+      <c r="C3" s="68"/>
+      <c r="D3" s="68"/>
+      <c r="E3" s="68"/>
+      <c r="F3" s="68"/>
+      <c r="G3" s="68"/>
+      <c r="H3" s="68"/>
+      <c r="I3" s="68"/>
+      <c r="J3" s="68"/>
+      <c r="K3" s="68"/>
+      <c r="L3" s="68"/>
+      <c r="M3" s="68"/>
+      <c r="N3" s="68"/>
+      <c r="O3" s="68"/>
+      <c r="P3" s="69"/>
       <c r="R3" s="12"/>
     </row>
     <row r="5" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B5" s="46" t="s">
+      <c r="B5" s="60" t="s">
         <v>18</v>
       </c>
-      <c r="C5" s="46"/>
-      <c r="D5" s="46"/>
-      <c r="E5" s="46"/>
-      <c r="F5" s="46"/>
-      <c r="G5" s="46"/>
+      <c r="C5" s="60"/>
+      <c r="D5" s="60"/>
+      <c r="E5" s="60"/>
+      <c r="F5" s="60"/>
+      <c r="G5" s="60"/>
       <c r="I5" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="K5" s="55" t="s">
+      <c r="K5" s="54" t="s">
         <v>8</v>
       </c>
-      <c r="L5" s="57"/>
-      <c r="M5" s="57"/>
+      <c r="L5" s="55"/>
+      <c r="M5" s="55"/>
       <c r="N5" s="56"/>
       <c r="P5" s="4" t="s">
         <v>74</v>
@@ -2860,28 +2885,28 @@
       </c>
     </row>
     <row r="9" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B9" s="58" t="s">
+      <c r="B9" s="57" t="s">
         <v>22</v>
       </c>
-      <c r="C9" s="58"/>
+      <c r="C9" s="57"/>
       <c r="E9" s="9" t="s">
         <v>67</v>
       </c>
     </row>
     <row r="10" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B10" s="59">
+      <c r="B10" s="46">
         <f>_xlfn.CEILING.MATH(SUM(B7:G7,I7,K7:N7,P7),1,1)</f>
         <v>110</v>
       </c>
-      <c r="C10" s="59"/>
-      <c r="E10" s="53">
+      <c r="C10" s="46"/>
+      <c r="E10" s="61">
         <v>4</v>
       </c>
     </row>
     <row r="11" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B11" s="59"/>
-      <c r="C11" s="59"/>
-      <c r="E11" s="54"/>
+      <c r="B11" s="46"/>
+      <c r="C11" s="46"/>
+      <c r="E11" s="62"/>
     </row>
     <row r="12" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A12" s="6"/>
@@ -2906,40 +2931,40 @@
     </row>
     <row r="13" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="14" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B14" s="63" t="s">
+      <c r="B14" s="64" t="s">
         <v>133</v>
       </c>
-      <c r="C14" s="64"/>
-      <c r="D14" s="64"/>
-      <c r="E14" s="64"/>
-      <c r="F14" s="64"/>
-      <c r="G14" s="64"/>
-      <c r="H14" s="65"/>
+      <c r="C14" s="65"/>
+      <c r="D14" s="65"/>
+      <c r="E14" s="65"/>
+      <c r="F14" s="65"/>
+      <c r="G14" s="65"/>
+      <c r="H14" s="66"/>
     </row>
     <row r="15" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B15" s="66"/>
-      <c r="C15" s="67"/>
-      <c r="D15" s="67"/>
-      <c r="E15" s="67"/>
-      <c r="F15" s="67"/>
-      <c r="G15" s="67"/>
-      <c r="H15" s="68"/>
+      <c r="B15" s="67"/>
+      <c r="C15" s="68"/>
+      <c r="D15" s="68"/>
+      <c r="E15" s="68"/>
+      <c r="F15" s="68"/>
+      <c r="G15" s="68"/>
+      <c r="H15" s="69"/>
     </row>
     <row r="17" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B17" s="46" t="s">
+      <c r="B17" s="60" t="s">
         <v>12</v>
       </c>
-      <c r="C17" s="46"/>
-      <c r="D17" s="46"/>
-      <c r="F17" s="46" t="s">
+      <c r="C17" s="60"/>
+      <c r="D17" s="60"/>
+      <c r="F17" s="60" t="s">
         <v>8</v>
       </c>
-      <c r="G17" s="46"/>
-      <c r="H17" s="46"/>
-      <c r="J17" s="58" t="s">
+      <c r="G17" s="60"/>
+      <c r="H17" s="60"/>
+      <c r="J17" s="57" t="s">
         <v>22</v>
       </c>
-      <c r="K17" s="58"/>
+      <c r="K17" s="57"/>
       <c r="M17" s="9" t="s">
         <v>67</v>
       </c>
@@ -2963,12 +2988,12 @@
       <c r="H18" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="J18" s="59">
+      <c r="J18" s="46">
         <f>SUM(B19:D19,F19:H19)</f>
         <v>93</v>
       </c>
-      <c r="K18" s="59"/>
-      <c r="M18" s="60">
+      <c r="K18" s="46"/>
+      <c r="M18" s="47">
         <v>5</v>
       </c>
     </row>
@@ -2991,9 +3016,9 @@
       <c r="H19" s="2">
         <v>4</v>
       </c>
-      <c r="J19" s="59"/>
-      <c r="K19" s="59"/>
-      <c r="M19" s="60"/>
+      <c r="J19" s="46"/>
+      <c r="K19" s="46"/>
+      <c r="M19" s="47"/>
     </row>
     <row r="21" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A21" s="6"/>
@@ -3018,46 +3043,46 @@
     </row>
     <row r="22" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="23" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B23" s="63" t="s">
+      <c r="B23" s="64" t="s">
         <v>134</v>
       </c>
-      <c r="C23" s="64"/>
-      <c r="D23" s="64"/>
-      <c r="E23" s="64"/>
-      <c r="F23" s="64"/>
-      <c r="G23" s="64"/>
-      <c r="H23" s="64"/>
-      <c r="I23" s="64"/>
-      <c r="J23" s="64"/>
-      <c r="K23" s="65"/>
+      <c r="C23" s="65"/>
+      <c r="D23" s="65"/>
+      <c r="E23" s="65"/>
+      <c r="F23" s="65"/>
+      <c r="G23" s="65"/>
+      <c r="H23" s="65"/>
+      <c r="I23" s="65"/>
+      <c r="J23" s="65"/>
+      <c r="K23" s="66"/>
     </row>
     <row r="24" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B24" s="66"/>
-      <c r="C24" s="67"/>
-      <c r="D24" s="67"/>
-      <c r="E24" s="67"/>
-      <c r="F24" s="67"/>
-      <c r="G24" s="67"/>
-      <c r="H24" s="67"/>
-      <c r="I24" s="67"/>
-      <c r="J24" s="67"/>
-      <c r="K24" s="68"/>
+      <c r="B24" s="67"/>
+      <c r="C24" s="68"/>
+      <c r="D24" s="68"/>
+      <c r="E24" s="68"/>
+      <c r="F24" s="68"/>
+      <c r="G24" s="68"/>
+      <c r="H24" s="68"/>
+      <c r="I24" s="68"/>
+      <c r="J24" s="68"/>
+      <c r="K24" s="69"/>
     </row>
     <row r="26" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B26" s="46" t="s">
+      <c r="B26" s="60" t="s">
         <v>17</v>
       </c>
-      <c r="C26" s="46"/>
-      <c r="E26" s="55" t="s">
+      <c r="C26" s="60"/>
+      <c r="E26" s="54" t="s">
         <v>21</v>
       </c>
-      <c r="F26" s="57"/>
+      <c r="F26" s="55"/>
       <c r="G26" s="56"/>
-      <c r="I26" s="46" t="s">
+      <c r="I26" s="60" t="s">
         <v>20</v>
       </c>
-      <c r="J26" s="46"/>
-      <c r="K26" s="46"/>
+      <c r="J26" s="60"/>
+      <c r="K26" s="60"/>
       <c r="M26" s="10" t="s">
         <v>22</v>
       </c>
@@ -3092,12 +3117,12 @@
       <c r="K27" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="M27" s="69">
+      <c r="M27" s="70">
         <f>SUM(B28:C28,E28:G28,I28:K28)</f>
         <v>36</v>
       </c>
       <c r="N27" s="7"/>
-      <c r="O27" s="60">
+      <c r="O27" s="47">
         <v>4</v>
       </c>
       <c r="P27" s="8"/>
@@ -3127,9 +3152,9 @@
       <c r="K28" s="2">
         <v>3.2</v>
       </c>
-      <c r="M28" s="69"/>
+      <c r="M28" s="70"/>
       <c r="N28" s="7"/>
-      <c r="O28" s="60"/>
+      <c r="O28" s="47"/>
       <c r="P28" s="8"/>
     </row>
     <row r="30" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -3155,39 +3180,39 @@
     </row>
     <row r="31" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="32" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B32" s="63" t="s">
+      <c r="B32" s="64" t="s">
         <v>135</v>
       </c>
-      <c r="C32" s="64"/>
-      <c r="D32" s="64"/>
-      <c r="E32" s="64"/>
-      <c r="F32" s="64"/>
-      <c r="G32" s="64"/>
-      <c r="H32" s="64"/>
-      <c r="I32" s="65"/>
+      <c r="C32" s="65"/>
+      <c r="D32" s="65"/>
+      <c r="E32" s="65"/>
+      <c r="F32" s="65"/>
+      <c r="G32" s="65"/>
+      <c r="H32" s="65"/>
+      <c r="I32" s="66"/>
     </row>
     <row r="33" spans="2:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B33" s="66"/>
-      <c r="C33" s="67"/>
-      <c r="D33" s="67"/>
-      <c r="E33" s="67"/>
-      <c r="F33" s="67"/>
-      <c r="G33" s="67"/>
-      <c r="H33" s="67"/>
-      <c r="I33" s="68"/>
+      <c r="B33" s="67"/>
+      <c r="C33" s="68"/>
+      <c r="D33" s="68"/>
+      <c r="E33" s="68"/>
+      <c r="F33" s="68"/>
+      <c r="G33" s="68"/>
+      <c r="H33" s="68"/>
+      <c r="I33" s="69"/>
     </row>
     <row r="35" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B35" s="46" t="s">
+      <c r="B35" s="60" t="s">
         <v>31</v>
       </c>
-      <c r="C35" s="46"/>
-      <c r="D35" s="46"/>
-      <c r="F35" s="46" t="s">
+      <c r="C35" s="60"/>
+      <c r="D35" s="60"/>
+      <c r="F35" s="60" t="s">
         <v>12</v>
       </c>
-      <c r="G35" s="46"/>
-      <c r="H35" s="46"/>
-      <c r="I35" s="46"/>
+      <c r="G35" s="60"/>
+      <c r="H35" s="60"/>
+      <c r="I35" s="60"/>
       <c r="N35" s="7"/>
       <c r="O35" s="7"/>
     </row>
@@ -3244,14 +3269,14 @@
       <c r="O37" s="7"/>
     </row>
     <row r="40" spans="2:15" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B40" s="61" t="s">
+      <c r="B40" s="58" t="s">
         <v>35</v>
       </c>
-      <c r="C40" s="62"/>
-      <c r="F40" s="59" t="s">
+      <c r="C40" s="59"/>
+      <c r="F40" s="46" t="s">
         <v>36</v>
       </c>
-      <c r="G40" s="59"/>
+      <c r="G40" s="46"/>
       <c r="I40" s="9" t="s">
         <v>22</v>
       </c>
@@ -3307,7 +3332,7 @@
       <c r="G43" s="2">
         <v>0.44</v>
       </c>
-      <c r="I43" s="58" t="s">
+      <c r="I43" s="57" t="s">
         <v>67</v>
       </c>
     </row>
@@ -3324,7 +3349,7 @@
       <c r="G44" s="2">
         <v>1</v>
       </c>
-      <c r="I44" s="58"/>
+      <c r="I44" s="57"/>
     </row>
     <row r="45" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B45" s="2" t="s">
@@ -3468,67 +3493,67 @@
     </row>
     <row r="57" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="58" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B58" s="63" t="s">
+      <c r="B58" s="64" t="s">
         <v>136</v>
       </c>
-      <c r="C58" s="64"/>
-      <c r="D58" s="64"/>
-      <c r="E58" s="64"/>
-      <c r="F58" s="64"/>
-      <c r="G58" s="64"/>
-      <c r="H58" s="64"/>
-      <c r="I58" s="64"/>
-      <c r="J58" s="64"/>
-      <c r="K58" s="64"/>
-      <c r="L58" s="64"/>
-      <c r="M58" s="64"/>
-      <c r="N58" s="64"/>
-      <c r="O58" s="64"/>
-      <c r="P58" s="64"/>
-      <c r="Q58" s="64"/>
-      <c r="R58" s="65"/>
+      <c r="C58" s="65"/>
+      <c r="D58" s="65"/>
+      <c r="E58" s="65"/>
+      <c r="F58" s="65"/>
+      <c r="G58" s="65"/>
+      <c r="H58" s="65"/>
+      <c r="I58" s="65"/>
+      <c r="J58" s="65"/>
+      <c r="K58" s="65"/>
+      <c r="L58" s="65"/>
+      <c r="M58" s="65"/>
+      <c r="N58" s="65"/>
+      <c r="O58" s="65"/>
+      <c r="P58" s="65"/>
+      <c r="Q58" s="65"/>
+      <c r="R58" s="66"/>
     </row>
     <row r="59" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B59" s="66"/>
-      <c r="C59" s="67"/>
-      <c r="D59" s="67"/>
-      <c r="E59" s="67"/>
-      <c r="F59" s="67"/>
-      <c r="G59" s="67"/>
-      <c r="H59" s="67"/>
-      <c r="I59" s="67"/>
-      <c r="J59" s="67"/>
-      <c r="K59" s="67"/>
-      <c r="L59" s="67"/>
-      <c r="M59" s="67"/>
-      <c r="N59" s="67"/>
-      <c r="O59" s="67"/>
-      <c r="P59" s="67"/>
-      <c r="Q59" s="67"/>
-      <c r="R59" s="68"/>
+      <c r="B59" s="67"/>
+      <c r="C59" s="68"/>
+      <c r="D59" s="68"/>
+      <c r="E59" s="68"/>
+      <c r="F59" s="68"/>
+      <c r="G59" s="68"/>
+      <c r="H59" s="68"/>
+      <c r="I59" s="68"/>
+      <c r="J59" s="68"/>
+      <c r="K59" s="68"/>
+      <c r="L59" s="68"/>
+      <c r="M59" s="68"/>
+      <c r="N59" s="68"/>
+      <c r="O59" s="68"/>
+      <c r="P59" s="68"/>
+      <c r="Q59" s="68"/>
+      <c r="R59" s="69"/>
     </row>
     <row r="61" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B61" s="46" t="s">
+      <c r="B61" s="60" t="s">
         <v>63</v>
       </c>
-      <c r="C61" s="46"/>
-      <c r="D61" s="46"/>
-      <c r="E61" s="46"/>
-      <c r="F61" s="46"/>
-      <c r="G61" s="46"/>
-      <c r="H61" s="46"/>
-      <c r="I61" s="46"/>
-      <c r="J61" s="46"/>
-      <c r="K61" s="46"/>
-      <c r="M61" s="46" t="s">
+      <c r="C61" s="60"/>
+      <c r="D61" s="60"/>
+      <c r="E61" s="60"/>
+      <c r="F61" s="60"/>
+      <c r="G61" s="60"/>
+      <c r="H61" s="60"/>
+      <c r="I61" s="60"/>
+      <c r="J61" s="60"/>
+      <c r="K61" s="60"/>
+      <c r="M61" s="60" t="s">
         <v>68</v>
       </c>
-      <c r="N61" s="46"/>
-      <c r="O61" s="46"/>
-      <c r="Q61" s="46" t="s">
+      <c r="N61" s="60"/>
+      <c r="O61" s="60"/>
+      <c r="Q61" s="60" t="s">
         <v>64</v>
       </c>
-      <c r="R61" s="46"/>
+      <c r="R61" s="60"/>
     </row>
     <row r="62" spans="1:19" x14ac:dyDescent="0.25">
       <c r="B62" s="2" t="s">
@@ -3625,28 +3650,28 @@
       </c>
     </row>
     <row r="66" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B66" s="58" t="s">
+      <c r="B66" s="57" t="s">
         <v>22</v>
       </c>
-      <c r="C66" s="58"/>
+      <c r="C66" s="57"/>
       <c r="E66" s="9" t="s">
         <v>67</v>
       </c>
     </row>
     <row r="67" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B67" s="59">
+      <c r="B67" s="46">
         <f xml:space="preserve"> SUM(B63:K63,M63:O63,Q63:R63)</f>
         <v>85.5</v>
       </c>
-      <c r="C67" s="59"/>
-      <c r="E67" s="60">
+      <c r="C67" s="46"/>
+      <c r="E67" s="47">
         <v>4.5</v>
       </c>
     </row>
     <row r="68" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B68" s="59"/>
-      <c r="C68" s="59"/>
-      <c r="E68" s="60"/>
+      <c r="B68" s="46"/>
+      <c r="C68" s="46"/>
+      <c r="E68" s="47"/>
     </row>
     <row r="70" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A70" s="6"/>
@@ -3671,26 +3696,26 @@
     </row>
     <row r="71" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="72" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B72" s="63" t="s">
+      <c r="B72" s="64" t="s">
         <v>137</v>
       </c>
-      <c r="C72" s="64"/>
-      <c r="D72" s="64"/>
-      <c r="E72" s="64"/>
-      <c r="F72" s="64"/>
-      <c r="G72" s="64"/>
-      <c r="H72" s="64"/>
-      <c r="I72" s="65"/>
+      <c r="C72" s="65"/>
+      <c r="D72" s="65"/>
+      <c r="E72" s="65"/>
+      <c r="F72" s="65"/>
+      <c r="G72" s="65"/>
+      <c r="H72" s="65"/>
+      <c r="I72" s="66"/>
     </row>
     <row r="73" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B73" s="66"/>
-      <c r="C73" s="67"/>
-      <c r="D73" s="67"/>
-      <c r="E73" s="67"/>
-      <c r="F73" s="67"/>
-      <c r="G73" s="67"/>
-      <c r="H73" s="67"/>
-      <c r="I73" s="68"/>
+      <c r="B73" s="67"/>
+      <c r="C73" s="68"/>
+      <c r="D73" s="68"/>
+      <c r="E73" s="68"/>
+      <c r="F73" s="68"/>
+      <c r="G73" s="68"/>
+      <c r="H73" s="68"/>
+      <c r="I73" s="69"/>
     </row>
     <row r="75" spans="1:19" x14ac:dyDescent="0.25">
       <c r="B75" s="4" t="s">
@@ -3717,10 +3742,10 @@
       <c r="I75" s="4" t="s">
         <v>145</v>
       </c>
-      <c r="K75" s="58" t="s">
+      <c r="K75" s="57" t="s">
         <v>22</v>
       </c>
-      <c r="L75" s="58"/>
+      <c r="L75" s="57"/>
       <c r="N75" s="9" t="s">
         <v>67</v>
       </c>
@@ -3750,11 +3775,11 @@
       <c r="I76" s="2">
         <v>5</v>
       </c>
-      <c r="K76" s="59">
+      <c r="K76" s="46">
         <f>SUM(B76:I76)</f>
         <v>96</v>
       </c>
-      <c r="L76" s="59"/>
+      <c r="L76" s="46"/>
       <c r="N76" s="13">
         <v>5</v>
       </c>
@@ -3782,20 +3807,16 @@
     </row>
   </sheetData>
   <mergeCells count="34">
-    <mergeCell ref="B2:P3"/>
-    <mergeCell ref="B5:G5"/>
-    <mergeCell ref="K5:N5"/>
-    <mergeCell ref="B9:C9"/>
-    <mergeCell ref="B10:C11"/>
-    <mergeCell ref="E10:E11"/>
-    <mergeCell ref="M27:M28"/>
-    <mergeCell ref="O27:O28"/>
-    <mergeCell ref="B14:H15"/>
-    <mergeCell ref="B17:D17"/>
-    <mergeCell ref="F17:H17"/>
-    <mergeCell ref="J17:K17"/>
-    <mergeCell ref="J18:K19"/>
-    <mergeCell ref="M18:M19"/>
+    <mergeCell ref="B72:I73"/>
+    <mergeCell ref="K75:L75"/>
+    <mergeCell ref="K76:L76"/>
+    <mergeCell ref="B58:R59"/>
+    <mergeCell ref="B61:K61"/>
+    <mergeCell ref="M61:O61"/>
+    <mergeCell ref="Q61:R61"/>
+    <mergeCell ref="B66:C66"/>
+    <mergeCell ref="B67:C68"/>
+    <mergeCell ref="E67:E68"/>
     <mergeCell ref="I43:I44"/>
     <mergeCell ref="B23:K24"/>
     <mergeCell ref="B26:C26"/>
@@ -3806,16 +3827,20 @@
     <mergeCell ref="F35:I35"/>
     <mergeCell ref="B40:C40"/>
     <mergeCell ref="F40:G40"/>
-    <mergeCell ref="B72:I73"/>
-    <mergeCell ref="K75:L75"/>
-    <mergeCell ref="K76:L76"/>
-    <mergeCell ref="B58:R59"/>
-    <mergeCell ref="B61:K61"/>
-    <mergeCell ref="M61:O61"/>
-    <mergeCell ref="Q61:R61"/>
-    <mergeCell ref="B66:C66"/>
-    <mergeCell ref="B67:C68"/>
-    <mergeCell ref="E67:E68"/>
+    <mergeCell ref="M27:M28"/>
+    <mergeCell ref="O27:O28"/>
+    <mergeCell ref="B14:H15"/>
+    <mergeCell ref="B17:D17"/>
+    <mergeCell ref="F17:H17"/>
+    <mergeCell ref="J17:K17"/>
+    <mergeCell ref="J18:K19"/>
+    <mergeCell ref="M18:M19"/>
+    <mergeCell ref="B2:P3"/>
+    <mergeCell ref="B5:G5"/>
+    <mergeCell ref="K5:N5"/>
+    <mergeCell ref="B9:C9"/>
+    <mergeCell ref="B10:C11"/>
+    <mergeCell ref="E10:E11"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
@@ -4422,21 +4447,21 @@
   <sheetData>
     <row r="1" spans="2:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="2" spans="2:12" ht="23.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B2" s="70" t="s">
+      <c r="B2" s="71" t="s">
         <v>203</v>
       </c>
-      <c r="C2" s="71"/>
-      <c r="D2" s="72"/>
-      <c r="F2" s="70" t="s">
+      <c r="C2" s="72"/>
+      <c r="D2" s="73"/>
+      <c r="F2" s="71" t="s">
         <v>204</v>
       </c>
-      <c r="G2" s="71"/>
-      <c r="H2" s="72"/>
-      <c r="J2" s="70" t="s">
+      <c r="G2" s="72"/>
+      <c r="H2" s="73"/>
+      <c r="J2" s="71" t="s">
         <v>205</v>
       </c>
-      <c r="K2" s="71"/>
-      <c r="L2" s="72"/>
+      <c r="K2" s="72"/>
+      <c r="L2" s="73"/>
     </row>
     <row r="3" spans="2:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B3" s="34" t="s">
@@ -4611,26 +4636,26 @@
     </row>
     <row r="10" spans="2:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="11" spans="2:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B11" s="73" t="s">
+      <c r="B11" s="74" t="s">
         <v>197</v>
       </c>
-      <c r="C11" s="74"/>
+      <c r="C11" s="75"/>
       <c r="D11" s="33">
         <f>(D4*C4+D5*C5+D6*C6+D7*C7+D8*C8+D9*C9)/30</f>
         <v>4.4333333333333336</v>
       </c>
-      <c r="F11" s="73" t="s">
+      <c r="F11" s="74" t="s">
         <v>197</v>
       </c>
-      <c r="G11" s="74"/>
+      <c r="G11" s="75"/>
       <c r="H11" s="33">
         <f>(H4*G4+H5*G5+H6*G6+H7*G7+H8*G8)/30</f>
         <v>0</v>
       </c>
-      <c r="J11" s="73" t="s">
+      <c r="J11" s="74" t="s">
         <v>197</v>
       </c>
-      <c r="K11" s="74"/>
+      <c r="K11" s="75"/>
       <c r="L11" s="33">
         <f>(L4*K4+L5*K5+L6*K6+L7*K7+L8*K8)/30</f>
         <v>0</v>

</xml_diff>

<commit_message>
New points - FIZ1 passed!
</commit_message>
<xml_diff>
--- a/IoT-points-schedule.xlsx
+++ b/IoT-points-schedule.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\dodo\Desktop\IoT-studies\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A6B41023-C553-44AC-BF28-ADE8015752C5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5374CC67-EA74-4F6A-AC75-6B427581DCEA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="25440" windowHeight="15390" xr2:uid="{F85F5544-1FE8-4920-A5D4-192A98B113BD}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="354" uniqueCount="226">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="354" uniqueCount="225">
   <si>
     <t>1. Krypto</t>
   </si>
@@ -428,12 +428,6 @@
     <t>Egzamin [20+10 pkt]</t>
   </si>
   <si>
-    <t>Ćwiczenia [C = 0,6K+0,4P]</t>
-  </si>
-  <si>
-    <t>Mini-projekt</t>
-  </si>
-  <si>
     <t>W = 0,4E + 0,3C + 0,3L</t>
   </si>
   <si>
@@ -717,6 +711,9 @@
   </si>
   <si>
     <t>Extra</t>
+  </si>
+  <si>
+    <t>Mini-projekt [10 pkt]</t>
   </si>
 </sst>
 </file>
@@ -1104,7 +1101,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="84">
+  <cellXfs count="82">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1305,6 +1302,24 @@
     <xf numFmtId="0" fontId="0" fillId="8" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="7" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="7" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="7" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="7" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="7" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="7" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1339,30 +1354,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="7" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="7" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="7" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="7" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="7" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="7" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1731,7 +1722,7 @@
   <cols>
     <col min="1" max="1" width="3.85546875" style="1" customWidth="1"/>
     <col min="2" max="2" width="16" style="1" customWidth="1"/>
-    <col min="3" max="3" width="16.5703125" style="1" customWidth="1"/>
+    <col min="3" max="3" width="17.28515625" style="1" customWidth="1"/>
     <col min="4" max="4" width="16" style="1" customWidth="1"/>
     <col min="5" max="5" width="16.28515625" style="1" customWidth="1"/>
     <col min="6" max="6" width="16.85546875" style="1" customWidth="1"/>
@@ -1813,25 +1804,25 @@
     </row>
     <row r="6" spans="1:19" ht="29.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B6" s="3" t="s">
+        <v>172</v>
+      </c>
+      <c r="C6" s="3" t="s">
+        <v>173</v>
+      </c>
+      <c r="D6" s="3" t="s">
         <v>174</v>
       </c>
-      <c r="C6" s="3" t="s">
+      <c r="E6" s="3" t="s">
         <v>175</v>
       </c>
-      <c r="D6" s="3" t="s">
+      <c r="F6" s="3" t="s">
         <v>176</v>
       </c>
-      <c r="E6" s="3" t="s">
-        <v>177</v>
-      </c>
-      <c r="F6" s="3" t="s">
-        <v>178</v>
-      </c>
       <c r="H6" s="2" t="s">
-        <v>212</v>
+        <v>210</v>
       </c>
       <c r="I6" s="2" t="s">
-        <v>215</v>
+        <v>213</v>
       </c>
       <c r="K6" s="2" t="s">
         <v>24</v>
@@ -1975,13 +1966,13 @@
     </row>
     <row r="18" spans="1:19" ht="48.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B18" s="3" t="s">
+        <v>156</v>
+      </c>
+      <c r="C18" s="3" t="s">
+        <v>157</v>
+      </c>
+      <c r="D18" s="3" t="s">
         <v>158</v>
-      </c>
-      <c r="C18" s="3" t="s">
-        <v>159</v>
-      </c>
-      <c r="D18" s="3" t="s">
-        <v>160</v>
       </c>
       <c r="E18" s="3" t="s">
         <v>92</v>
@@ -2052,47 +2043,53 @@
     </row>
     <row r="22" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="23" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B23" s="48" t="s">
+      <c r="B23" s="64" t="s">
         <v>79</v>
       </c>
-      <c r="C23" s="49"/>
-      <c r="D23" s="49"/>
-      <c r="E23" s="49"/>
-      <c r="F23" s="49"/>
-      <c r="G23" s="49"/>
-      <c r="H23" s="49"/>
-      <c r="I23" s="49"/>
-      <c r="J23" s="49"/>
-      <c r="K23" s="49"/>
-      <c r="L23" s="50"/>
+      <c r="C23" s="65"/>
+      <c r="D23" s="65"/>
+      <c r="E23" s="65"/>
+      <c r="F23" s="65"/>
+      <c r="G23" s="65"/>
+      <c r="H23" s="65"/>
+      <c r="I23" s="65"/>
+      <c r="J23" s="65"/>
+      <c r="K23" s="65"/>
+      <c r="L23" s="66"/>
       <c r="N23" s="46" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="O23" s="46"/>
+      <c r="Q23" s="7"/>
+      <c r="R23" s="7"/>
+      <c r="S23" s="7"/>
     </row>
     <row r="24" spans="1:19" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B24" s="51"/>
-      <c r="C24" s="52"/>
-      <c r="D24" s="52"/>
-      <c r="E24" s="52"/>
-      <c r="F24" s="52"/>
-      <c r="G24" s="52"/>
-      <c r="H24" s="52"/>
-      <c r="I24" s="52"/>
-      <c r="J24" s="52"/>
-      <c r="K24" s="52"/>
-      <c r="L24" s="53"/>
+      <c r="B24" s="67"/>
+      <c r="C24" s="68"/>
+      <c r="D24" s="68"/>
+      <c r="E24" s="68"/>
+      <c r="F24" s="68"/>
+      <c r="G24" s="68"/>
+      <c r="H24" s="68"/>
+      <c r="I24" s="68"/>
+      <c r="J24" s="68"/>
+      <c r="K24" s="68"/>
+      <c r="L24" s="69"/>
       <c r="N24" s="46"/>
       <c r="O24" s="46"/>
+      <c r="Q24" s="7"/>
+      <c r="R24" s="7"/>
+      <c r="S24" s="7"/>
     </row>
     <row r="26" spans="1:19" x14ac:dyDescent="0.25">
       <c r="B26" s="60" t="s">
-        <v>129</v>
+        <v>8</v>
       </c>
       <c r="C26" s="60"/>
       <c r="D26" s="60"/>
       <c r="F26" s="60" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="G26" s="60"/>
       <c r="H26" s="60"/>
@@ -2108,25 +2105,25 @@
     </row>
     <row r="27" spans="1:19" x14ac:dyDescent="0.25">
       <c r="B27" s="14" t="s">
-        <v>216</v>
+        <v>214</v>
       </c>
       <c r="C27" s="14" t="s">
-        <v>130</v>
+        <v>224</v>
       </c>
       <c r="D27" s="2" t="s">
         <v>11</v>
       </c>
       <c r="F27" s="2" t="s">
+        <v>204</v>
+      </c>
+      <c r="G27" s="2" t="s">
         <v>206</v>
       </c>
-      <c r="G27" s="2" t="s">
-        <v>208</v>
-      </c>
       <c r="H27" s="2" t="s">
+        <v>205</v>
+      </c>
+      <c r="I27" s="2" t="s">
         <v>207</v>
-      </c>
-      <c r="I27" s="2" t="s">
-        <v>209</v>
       </c>
       <c r="K27" s="14" t="s">
         <v>73</v>
@@ -2134,13 +2131,18 @@
       <c r="L27" s="2" t="s">
         <v>127</v>
       </c>
-      <c r="N27" s="61"/>
+      <c r="N27" s="61">
+        <f>(K29/30*0.4*5)+(B29/25*0.3*5)+(0.3*F29)</f>
+        <v>4.2133333333333329</v>
+      </c>
     </row>
     <row r="28" spans="1:19" x14ac:dyDescent="0.25">
       <c r="B28" s="2">
         <v>13</v>
       </c>
-      <c r="C28" s="2"/>
+      <c r="C28" s="2">
+        <v>10</v>
+      </c>
       <c r="D28" s="2">
         <v>1</v>
       </c>
@@ -2156,12 +2158,17 @@
       <c r="I28" s="2">
         <v>5</v>
       </c>
-      <c r="K28" s="2"/>
+      <c r="K28" s="2">
+        <v>20</v>
+      </c>
       <c r="L28" s="2"/>
       <c r="N28" s="62"/>
     </row>
     <row r="29" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B29" s="63"/>
+      <c r="B29" s="63">
+        <f>SUM(B28:C28)</f>
+        <v>23</v>
+      </c>
       <c r="C29" s="63"/>
       <c r="D29" s="63"/>
       <c r="F29" s="63">
@@ -2170,7 +2177,10 @@
       <c r="G29" s="63"/>
       <c r="H29" s="63"/>
       <c r="I29" s="63"/>
-      <c r="K29" s="63"/>
+      <c r="K29" s="63">
+        <f>SUM(K28:L28)</f>
+        <v>20</v>
+      </c>
       <c r="L29" s="63"/>
       <c r="N29" s="44"/>
     </row>
@@ -2197,26 +2207,26 @@
     </row>
     <row r="32" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="33" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B33" s="76" t="s">
+      <c r="B33" s="64" t="s">
         <v>78</v>
       </c>
-      <c r="C33" s="77"/>
-      <c r="D33" s="77"/>
-      <c r="E33" s="77"/>
-      <c r="F33" s="77"/>
-      <c r="G33" s="77"/>
-      <c r="H33" s="77"/>
-      <c r="I33" s="78"/>
+      <c r="C33" s="65"/>
+      <c r="D33" s="65"/>
+      <c r="E33" s="65"/>
+      <c r="F33" s="65"/>
+      <c r="G33" s="65"/>
+      <c r="H33" s="65"/>
+      <c r="I33" s="66"/>
     </row>
     <row r="34" spans="2:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B34" s="79"/>
-      <c r="C34" s="80"/>
-      <c r="D34" s="80"/>
-      <c r="E34" s="80"/>
-      <c r="F34" s="80"/>
-      <c r="G34" s="80"/>
-      <c r="H34" s="80"/>
-      <c r="I34" s="81"/>
+      <c r="B34" s="67"/>
+      <c r="C34" s="68"/>
+      <c r="D34" s="68"/>
+      <c r="E34" s="68"/>
+      <c r="F34" s="68"/>
+      <c r="G34" s="68"/>
+      <c r="H34" s="68"/>
+      <c r="I34" s="69"/>
     </row>
     <row r="36" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B36" s="60" t="s">
@@ -2225,7 +2235,7 @@
       <c r="C36" s="60"/>
       <c r="D36" s="7"/>
       <c r="E36" s="54" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="F36" s="55"/>
       <c r="G36" s="55"/>
@@ -2380,7 +2390,7 @@
         <v>123</v>
       </c>
       <c r="G48" s="2"/>
-      <c r="I48" s="82"/>
+      <c r="I48" s="44"/>
     </row>
     <row r="49" spans="1:19" x14ac:dyDescent="0.25">
       <c r="B49" s="2" t="s">
@@ -2393,7 +2403,6 @@
         <v>124</v>
       </c>
       <c r="G49" s="2"/>
-      <c r="I49" s="83"/>
     </row>
     <row r="50" spans="1:19" x14ac:dyDescent="0.25">
       <c r="B50" s="2" t="s">
@@ -2567,7 +2576,7 @@
         <v>81</v>
       </c>
       <c r="J65" s="2" t="s">
-        <v>211</v>
+        <v>209</v>
       </c>
       <c r="K65" s="2" t="s">
         <v>85</v>
@@ -2605,10 +2614,10 @@
         <v>2</v>
       </c>
       <c r="F66" s="2" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
       <c r="G66" s="2" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
       <c r="H66" s="2">
         <v>2</v>
@@ -2619,7 +2628,9 @@
       <c r="J66" s="2">
         <v>2</v>
       </c>
-      <c r="K66" s="2"/>
+      <c r="K66" s="2">
+        <v>2</v>
+      </c>
       <c r="M66" s="2">
         <v>5</v>
       </c>
@@ -2644,19 +2655,19 @@
       </c>
       <c r="H69" s="57"/>
       <c r="K69" s="45" t="s">
-        <v>225</v>
+        <v>223</v>
       </c>
     </row>
     <row r="70" spans="2:19" x14ac:dyDescent="0.25">
       <c r="B70" s="46">
         <f>SUM(B66:K66,M66:P66,R66:S66,K70)</f>
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="C70" s="46"/>
       <c r="E70" s="47"/>
       <c r="G70" s="46">
         <f>50-SUM(B66:K66,M66:P66,R66:S66,K70)</f>
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="H70" s="46"/>
       <c r="K70" s="46">
@@ -2679,6 +2690,8 @@
     <mergeCell ref="B64:K64"/>
     <mergeCell ref="B61:S62"/>
     <mergeCell ref="M64:P64"/>
+    <mergeCell ref="F29:I29"/>
+    <mergeCell ref="B29:D29"/>
     <mergeCell ref="N27:N28"/>
     <mergeCell ref="F26:I26"/>
     <mergeCell ref="K26:L26"/>
@@ -2690,15 +2703,13 @@
     <mergeCell ref="L17:M17"/>
     <mergeCell ref="E10:E11"/>
     <mergeCell ref="G10:H11"/>
+    <mergeCell ref="B17:F17"/>
+    <mergeCell ref="H17:J17"/>
     <mergeCell ref="E70:E71"/>
     <mergeCell ref="B69:C69"/>
     <mergeCell ref="B70:C71"/>
     <mergeCell ref="G69:H69"/>
     <mergeCell ref="G70:H71"/>
-    <mergeCell ref="B17:F17"/>
-    <mergeCell ref="H17:J17"/>
-    <mergeCell ref="F29:I29"/>
-    <mergeCell ref="B29:D29"/>
     <mergeCell ref="K70:K71"/>
     <mergeCell ref="R18:R19"/>
     <mergeCell ref="B14:H15"/>
@@ -2750,40 +2761,40 @@
   <sheetData>
     <row r="1" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="2" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B2" s="64" t="s">
-        <v>132</v>
-      </c>
-      <c r="C2" s="65"/>
-      <c r="D2" s="65"/>
-      <c r="E2" s="65"/>
-      <c r="F2" s="65"/>
-      <c r="G2" s="65"/>
-      <c r="H2" s="65"/>
-      <c r="I2" s="65"/>
-      <c r="J2" s="65"/>
-      <c r="K2" s="65"/>
-      <c r="L2" s="65"/>
-      <c r="M2" s="65"/>
-      <c r="N2" s="65"/>
-      <c r="O2" s="65"/>
-      <c r="P2" s="66"/>
+      <c r="B2" s="70" t="s">
+        <v>130</v>
+      </c>
+      <c r="C2" s="71"/>
+      <c r="D2" s="71"/>
+      <c r="E2" s="71"/>
+      <c r="F2" s="71"/>
+      <c r="G2" s="71"/>
+      <c r="H2" s="71"/>
+      <c r="I2" s="71"/>
+      <c r="J2" s="71"/>
+      <c r="K2" s="71"/>
+      <c r="L2" s="71"/>
+      <c r="M2" s="71"/>
+      <c r="N2" s="71"/>
+      <c r="O2" s="71"/>
+      <c r="P2" s="72"/>
     </row>
     <row r="3" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B3" s="67"/>
-      <c r="C3" s="68"/>
-      <c r="D3" s="68"/>
-      <c r="E3" s="68"/>
-      <c r="F3" s="68"/>
-      <c r="G3" s="68"/>
-      <c r="H3" s="68"/>
-      <c r="I3" s="68"/>
-      <c r="J3" s="68"/>
-      <c r="K3" s="68"/>
-      <c r="L3" s="68"/>
-      <c r="M3" s="68"/>
-      <c r="N3" s="68"/>
-      <c r="O3" s="68"/>
-      <c r="P3" s="69"/>
+      <c r="B3" s="73"/>
+      <c r="C3" s="74"/>
+      <c r="D3" s="74"/>
+      <c r="E3" s="74"/>
+      <c r="F3" s="74"/>
+      <c r="G3" s="74"/>
+      <c r="H3" s="74"/>
+      <c r="I3" s="74"/>
+      <c r="J3" s="74"/>
+      <c r="K3" s="74"/>
+      <c r="L3" s="74"/>
+      <c r="M3" s="74"/>
+      <c r="N3" s="74"/>
+      <c r="O3" s="74"/>
+      <c r="P3" s="75"/>
       <c r="R3" s="12"/>
     </row>
     <row r="5" spans="1:19" x14ac:dyDescent="0.25">
@@ -2931,24 +2942,24 @@
     </row>
     <row r="13" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="14" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B14" s="64" t="s">
-        <v>133</v>
-      </c>
-      <c r="C14" s="65"/>
-      <c r="D14" s="65"/>
-      <c r="E14" s="65"/>
-      <c r="F14" s="65"/>
-      <c r="G14" s="65"/>
-      <c r="H14" s="66"/>
+      <c r="B14" s="70" t="s">
+        <v>131</v>
+      </c>
+      <c r="C14" s="71"/>
+      <c r="D14" s="71"/>
+      <c r="E14" s="71"/>
+      <c r="F14" s="71"/>
+      <c r="G14" s="71"/>
+      <c r="H14" s="72"/>
     </row>
     <row r="15" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B15" s="67"/>
-      <c r="C15" s="68"/>
-      <c r="D15" s="68"/>
-      <c r="E15" s="68"/>
-      <c r="F15" s="68"/>
-      <c r="G15" s="68"/>
-      <c r="H15" s="69"/>
+      <c r="B15" s="73"/>
+      <c r="C15" s="74"/>
+      <c r="D15" s="74"/>
+      <c r="E15" s="74"/>
+      <c r="F15" s="74"/>
+      <c r="G15" s="74"/>
+      <c r="H15" s="75"/>
     </row>
     <row r="17" spans="1:19" x14ac:dyDescent="0.25">
       <c r="B17" s="60" t="s">
@@ -3043,30 +3054,30 @@
     </row>
     <row r="22" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="23" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B23" s="64" t="s">
-        <v>134</v>
-      </c>
-      <c r="C23" s="65"/>
-      <c r="D23" s="65"/>
-      <c r="E23" s="65"/>
-      <c r="F23" s="65"/>
-      <c r="G23" s="65"/>
-      <c r="H23" s="65"/>
-      <c r="I23" s="65"/>
-      <c r="J23" s="65"/>
-      <c r="K23" s="66"/>
+      <c r="B23" s="70" t="s">
+        <v>132</v>
+      </c>
+      <c r="C23" s="71"/>
+      <c r="D23" s="71"/>
+      <c r="E23" s="71"/>
+      <c r="F23" s="71"/>
+      <c r="G23" s="71"/>
+      <c r="H23" s="71"/>
+      <c r="I23" s="71"/>
+      <c r="J23" s="71"/>
+      <c r="K23" s="72"/>
     </row>
     <row r="24" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B24" s="67"/>
-      <c r="C24" s="68"/>
-      <c r="D24" s="68"/>
-      <c r="E24" s="68"/>
-      <c r="F24" s="68"/>
-      <c r="G24" s="68"/>
-      <c r="H24" s="68"/>
-      <c r="I24" s="68"/>
-      <c r="J24" s="68"/>
-      <c r="K24" s="69"/>
+      <c r="B24" s="73"/>
+      <c r="C24" s="74"/>
+      <c r="D24" s="74"/>
+      <c r="E24" s="74"/>
+      <c r="F24" s="74"/>
+      <c r="G24" s="74"/>
+      <c r="H24" s="74"/>
+      <c r="I24" s="74"/>
+      <c r="J24" s="74"/>
+      <c r="K24" s="75"/>
     </row>
     <row r="26" spans="1:19" x14ac:dyDescent="0.25">
       <c r="B26" s="60" t="s">
@@ -3117,7 +3128,7 @@
       <c r="K27" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="M27" s="70">
+      <c r="M27" s="76">
         <f>SUM(B28:C28,E28:G28,I28:K28)</f>
         <v>36</v>
       </c>
@@ -3152,7 +3163,7 @@
       <c r="K28" s="2">
         <v>3.2</v>
       </c>
-      <c r="M28" s="70"/>
+      <c r="M28" s="76"/>
       <c r="N28" s="7"/>
       <c r="O28" s="47"/>
       <c r="P28" s="8"/>
@@ -3180,26 +3191,26 @@
     </row>
     <row r="31" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="32" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B32" s="64" t="s">
-        <v>135</v>
-      </c>
-      <c r="C32" s="65"/>
-      <c r="D32" s="65"/>
-      <c r="E32" s="65"/>
-      <c r="F32" s="65"/>
-      <c r="G32" s="65"/>
-      <c r="H32" s="65"/>
-      <c r="I32" s="66"/>
+      <c r="B32" s="70" t="s">
+        <v>133</v>
+      </c>
+      <c r="C32" s="71"/>
+      <c r="D32" s="71"/>
+      <c r="E32" s="71"/>
+      <c r="F32" s="71"/>
+      <c r="G32" s="71"/>
+      <c r="H32" s="71"/>
+      <c r="I32" s="72"/>
     </row>
     <row r="33" spans="2:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B33" s="67"/>
-      <c r="C33" s="68"/>
-      <c r="D33" s="68"/>
-      <c r="E33" s="68"/>
-      <c r="F33" s="68"/>
-      <c r="G33" s="68"/>
-      <c r="H33" s="68"/>
-      <c r="I33" s="69"/>
+      <c r="B33" s="73"/>
+      <c r="C33" s="74"/>
+      <c r="D33" s="74"/>
+      <c r="E33" s="74"/>
+      <c r="F33" s="74"/>
+      <c r="G33" s="74"/>
+      <c r="H33" s="74"/>
+      <c r="I33" s="75"/>
     </row>
     <row r="35" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B35" s="60" t="s">
@@ -3493,44 +3504,44 @@
     </row>
     <row r="57" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="58" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B58" s="64" t="s">
-        <v>136</v>
-      </c>
-      <c r="C58" s="65"/>
-      <c r="D58" s="65"/>
-      <c r="E58" s="65"/>
-      <c r="F58" s="65"/>
-      <c r="G58" s="65"/>
-      <c r="H58" s="65"/>
-      <c r="I58" s="65"/>
-      <c r="J58" s="65"/>
-      <c r="K58" s="65"/>
-      <c r="L58" s="65"/>
-      <c r="M58" s="65"/>
-      <c r="N58" s="65"/>
-      <c r="O58" s="65"/>
-      <c r="P58" s="65"/>
-      <c r="Q58" s="65"/>
-      <c r="R58" s="66"/>
+      <c r="B58" s="70" t="s">
+        <v>134</v>
+      </c>
+      <c r="C58" s="71"/>
+      <c r="D58" s="71"/>
+      <c r="E58" s="71"/>
+      <c r="F58" s="71"/>
+      <c r="G58" s="71"/>
+      <c r="H58" s="71"/>
+      <c r="I58" s="71"/>
+      <c r="J58" s="71"/>
+      <c r="K58" s="71"/>
+      <c r="L58" s="71"/>
+      <c r="M58" s="71"/>
+      <c r="N58" s="71"/>
+      <c r="O58" s="71"/>
+      <c r="P58" s="71"/>
+      <c r="Q58" s="71"/>
+      <c r="R58" s="72"/>
     </row>
     <row r="59" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B59" s="67"/>
-      <c r="C59" s="68"/>
-      <c r="D59" s="68"/>
-      <c r="E59" s="68"/>
-      <c r="F59" s="68"/>
-      <c r="G59" s="68"/>
-      <c r="H59" s="68"/>
-      <c r="I59" s="68"/>
-      <c r="J59" s="68"/>
-      <c r="K59" s="68"/>
-      <c r="L59" s="68"/>
-      <c r="M59" s="68"/>
-      <c r="N59" s="68"/>
-      <c r="O59" s="68"/>
-      <c r="P59" s="68"/>
-      <c r="Q59" s="68"/>
-      <c r="R59" s="69"/>
+      <c r="B59" s="73"/>
+      <c r="C59" s="74"/>
+      <c r="D59" s="74"/>
+      <c r="E59" s="74"/>
+      <c r="F59" s="74"/>
+      <c r="G59" s="74"/>
+      <c r="H59" s="74"/>
+      <c r="I59" s="74"/>
+      <c r="J59" s="74"/>
+      <c r="K59" s="74"/>
+      <c r="L59" s="74"/>
+      <c r="M59" s="74"/>
+      <c r="N59" s="74"/>
+      <c r="O59" s="74"/>
+      <c r="P59" s="74"/>
+      <c r="Q59" s="74"/>
+      <c r="R59" s="75"/>
     </row>
     <row r="61" spans="1:19" x14ac:dyDescent="0.25">
       <c r="B61" s="60" t="s">
@@ -3696,51 +3707,51 @@
     </row>
     <row r="71" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="72" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B72" s="64" t="s">
-        <v>137</v>
-      </c>
-      <c r="C72" s="65"/>
-      <c r="D72" s="65"/>
-      <c r="E72" s="65"/>
-      <c r="F72" s="65"/>
-      <c r="G72" s="65"/>
-      <c r="H72" s="65"/>
-      <c r="I72" s="66"/>
+      <c r="B72" s="70" t="s">
+        <v>135</v>
+      </c>
+      <c r="C72" s="71"/>
+      <c r="D72" s="71"/>
+      <c r="E72" s="71"/>
+      <c r="F72" s="71"/>
+      <c r="G72" s="71"/>
+      <c r="H72" s="71"/>
+      <c r="I72" s="72"/>
     </row>
     <row r="73" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B73" s="67"/>
-      <c r="C73" s="68"/>
-      <c r="D73" s="68"/>
-      <c r="E73" s="68"/>
-      <c r="F73" s="68"/>
-      <c r="G73" s="68"/>
-      <c r="H73" s="68"/>
-      <c r="I73" s="69"/>
+      <c r="B73" s="73"/>
+      <c r="C73" s="74"/>
+      <c r="D73" s="74"/>
+      <c r="E73" s="74"/>
+      <c r="F73" s="74"/>
+      <c r="G73" s="74"/>
+      <c r="H73" s="74"/>
+      <c r="I73" s="75"/>
     </row>
     <row r="75" spans="1:19" x14ac:dyDescent="0.25">
       <c r="B75" s="4" t="s">
+        <v>136</v>
+      </c>
+      <c r="C75" s="4" t="s">
+        <v>137</v>
+      </c>
+      <c r="D75" s="4" t="s">
         <v>138</v>
       </c>
-      <c r="C75" s="4" t="s">
+      <c r="E75" s="4" t="s">
         <v>139</v>
       </c>
-      <c r="D75" s="4" t="s">
+      <c r="F75" s="4" t="s">
         <v>140</v>
       </c>
-      <c r="E75" s="4" t="s">
+      <c r="G75" s="4" t="s">
         <v>141</v>
       </c>
-      <c r="F75" s="4" t="s">
+      <c r="H75" s="4" t="s">
         <v>142</v>
       </c>
-      <c r="G75" s="4" t="s">
+      <c r="I75" s="4" t="s">
         <v>143</v>
-      </c>
-      <c r="H75" s="4" t="s">
-        <v>144</v>
-      </c>
-      <c r="I75" s="4" t="s">
-        <v>145</v>
       </c>
       <c r="K75" s="57" t="s">
         <v>22</v>
@@ -3861,16 +3872,16 @@
     <row r="1" spans="2:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="2" spans="2:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="C2" s="15" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="D2" s="15" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="E2" s="15" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="F2" s="15" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
     </row>
     <row r="3" spans="2:6" x14ac:dyDescent="0.25">
@@ -3884,10 +3895,10 @@
         <v>45763</v>
       </c>
       <c r="E3" s="26" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="F3" s="24" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
     </row>
     <row r="4" spans="2:6" x14ac:dyDescent="0.25">
@@ -3901,10 +3912,10 @@
         <v>45803</v>
       </c>
       <c r="E4" s="18" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="F4" s="17" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
     </row>
     <row r="5" spans="2:6" x14ac:dyDescent="0.25">
@@ -3918,10 +3929,10 @@
         <v>45817</v>
       </c>
       <c r="E5" s="42" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="F5" s="43" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
     </row>
     <row r="6" spans="2:6" x14ac:dyDescent="0.25">
@@ -3941,7 +3952,7 @@
         <v>103</v>
       </c>
       <c r="F7" s="27" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
     </row>
     <row r="8" spans="2:6" x14ac:dyDescent="0.25">
@@ -3958,7 +3969,7 @@
         <v>104</v>
       </c>
       <c r="F8" s="27" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
     </row>
     <row r="9" spans="2:6" x14ac:dyDescent="0.25">
@@ -3975,7 +3986,7 @@
         <v>105</v>
       </c>
       <c r="F9" s="27" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
     </row>
     <row r="10" spans="2:6" x14ac:dyDescent="0.25">
@@ -3992,7 +4003,7 @@
         <v>106</v>
       </c>
       <c r="F10" s="27" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
     </row>
     <row r="11" spans="2:6" x14ac:dyDescent="0.25">
@@ -4009,7 +4020,7 @@
         <v>107</v>
       </c>
       <c r="F11" s="27" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
     </row>
     <row r="12" spans="2:6" x14ac:dyDescent="0.25">
@@ -4020,7 +4031,7 @@
         <v>1</v>
       </c>
       <c r="C13" s="29" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="D13" s="28">
         <v>45728</v>
@@ -4029,7 +4040,7 @@
         <v>84</v>
       </c>
       <c r="F13" s="27" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
     </row>
     <row r="14" spans="2:6" x14ac:dyDescent="0.25">
@@ -4037,16 +4048,16 @@
         <v>1</v>
       </c>
       <c r="C14" s="29" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="D14" s="28">
         <v>45747</v>
       </c>
       <c r="E14" s="27" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="F14" s="27" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
     </row>
     <row r="15" spans="2:6" x14ac:dyDescent="0.25">
@@ -4054,16 +4065,16 @@
         <v>1</v>
       </c>
       <c r="C15" s="29" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="D15" s="28">
         <v>45784</v>
       </c>
       <c r="E15" s="27" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
       <c r="F15" s="27" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
     </row>
     <row r="16" spans="2:6" x14ac:dyDescent="0.25">
@@ -4071,7 +4082,7 @@
         <v>0</v>
       </c>
       <c r="C16" s="21" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="D16" s="20">
         <v>45806</v>
@@ -4080,7 +4091,7 @@
         <v>85</v>
       </c>
       <c r="F16" s="17" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
     </row>
     <row r="17" spans="2:6" x14ac:dyDescent="0.25">
@@ -4088,16 +4099,16 @@
         <v>0</v>
       </c>
       <c r="C17" s="21" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="D17" s="20">
         <v>45817</v>
       </c>
       <c r="E17" s="17" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
       <c r="F17" s="21" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
     </row>
     <row r="18" spans="2:6" x14ac:dyDescent="0.25">
@@ -4105,16 +4116,16 @@
         <v>0</v>
       </c>
       <c r="C18" s="21" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="D18" s="20">
         <v>45819</v>
       </c>
       <c r="E18" s="17" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
       <c r="F18" s="21" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
     </row>
     <row r="19" spans="2:6" x14ac:dyDescent="0.25">
@@ -4126,13 +4137,13 @@
         <v>0</v>
       </c>
       <c r="C20" s="21" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="D20" s="20">
         <v>45820</v>
       </c>
       <c r="E20" s="17" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
     </row>
     <row r="21" spans="2:6" x14ac:dyDescent="0.25">
@@ -4140,13 +4151,13 @@
         <v>0</v>
       </c>
       <c r="C21" s="21" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="D21" s="20">
         <v>45820</v>
       </c>
       <c r="E21" s="17" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
     </row>
     <row r="22" spans="2:6" x14ac:dyDescent="0.25">
@@ -4164,10 +4175,10 @@
         <v>45728</v>
       </c>
       <c r="E23" s="27" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
       <c r="F23" s="27" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
     </row>
     <row r="24" spans="2:6" x14ac:dyDescent="0.25">
@@ -4181,10 +4192,10 @@
         <v>45742</v>
       </c>
       <c r="E24" s="27" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
       <c r="F24" s="27" t="s">
-        <v>186</v>
+        <v>184</v>
       </c>
     </row>
     <row r="25" spans="2:6" x14ac:dyDescent="0.25">
@@ -4198,10 +4209,10 @@
         <v>45756</v>
       </c>
       <c r="E25" s="27" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
       <c r="F25" s="27" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
     </row>
     <row r="26" spans="2:6" x14ac:dyDescent="0.25">
@@ -4215,10 +4226,10 @@
         <v>45770</v>
       </c>
       <c r="E26" s="27" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="F26" s="29" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
     </row>
     <row r="27" spans="2:6" x14ac:dyDescent="0.25">
@@ -4232,10 +4243,10 @@
         <v>45784</v>
       </c>
       <c r="E27" s="27" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
       <c r="F27" s="27" t="s">
-        <v>188</v>
+        <v>186</v>
       </c>
     </row>
     <row r="28" spans="2:6" x14ac:dyDescent="0.25">
@@ -4249,10 +4260,10 @@
         <v>45798</v>
       </c>
       <c r="E28" s="27" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
       <c r="F28" s="27" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
     </row>
     <row r="29" spans="2:6" x14ac:dyDescent="0.25">
@@ -4266,10 +4277,10 @@
         <v>45812</v>
       </c>
       <c r="E29" s="17" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="F29" s="21" t="s">
-        <v>217</v>
+        <v>215</v>
       </c>
     </row>
     <row r="30" spans="2:6" x14ac:dyDescent="0.25">
@@ -4286,10 +4297,10 @@
         <v>45764</v>
       </c>
       <c r="E31" s="27" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="F31" s="27" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
     </row>
     <row r="32" spans="2:6" x14ac:dyDescent="0.25">
@@ -4303,7 +4314,7 @@
         <v>45815</v>
       </c>
       <c r="E32" s="27" t="s">
-        <v>218</v>
+        <v>216</v>
       </c>
     </row>
     <row r="33" spans="2:6" x14ac:dyDescent="0.25">
@@ -4317,10 +4328,10 @@
         <v>45814</v>
       </c>
       <c r="E33" s="17" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="F33" s="17" t="s">
-        <v>223</v>
+        <v>221</v>
       </c>
     </row>
     <row r="35" spans="2:6" x14ac:dyDescent="0.25">
@@ -4334,10 +4345,10 @@
         <v>45767</v>
       </c>
       <c r="E35" s="27" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
       <c r="F35" s="27" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
     </row>
     <row r="36" spans="2:6" x14ac:dyDescent="0.25">
@@ -4351,7 +4362,7 @@
         <v>45775</v>
       </c>
       <c r="E36" s="27" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
     </row>
     <row r="37" spans="2:6" x14ac:dyDescent="0.25">
@@ -4365,10 +4376,10 @@
         <v>45794</v>
       </c>
       <c r="E37" s="27" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="F37" s="27" t="s">
-        <v>213</v>
+        <v>211</v>
       </c>
     </row>
     <row r="39" spans="2:6" x14ac:dyDescent="0.25">
@@ -4382,10 +4393,10 @@
         <v>45784</v>
       </c>
       <c r="E39" s="27" t="s">
-        <v>224</v>
+        <v>222</v>
       </c>
       <c r="F39" s="27" t="s">
-        <v>220</v>
+        <v>218</v>
       </c>
     </row>
     <row r="40" spans="2:6" x14ac:dyDescent="0.25">
@@ -4399,10 +4410,10 @@
         <v>45798</v>
       </c>
       <c r="E40" s="27" t="s">
-        <v>219</v>
+        <v>217</v>
       </c>
       <c r="F40" s="27" t="s">
-        <v>220</v>
+        <v>218</v>
       </c>
     </row>
     <row r="41" spans="2:6" x14ac:dyDescent="0.25">
@@ -4416,10 +4427,10 @@
         <v>45805</v>
       </c>
       <c r="E41" s="17" t="s">
-        <v>222</v>
+        <v>220</v>
       </c>
       <c r="F41" s="17" t="s">
-        <v>221</v>
+        <v>219</v>
       </c>
     </row>
   </sheetData>
@@ -4447,54 +4458,54 @@
   <sheetData>
     <row r="1" spans="2:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="2" spans="2:12" ht="23.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B2" s="71" t="s">
+      <c r="B2" s="77" t="s">
+        <v>201</v>
+      </c>
+      <c r="C2" s="78"/>
+      <c r="D2" s="79"/>
+      <c r="F2" s="77" t="s">
+        <v>202</v>
+      </c>
+      <c r="G2" s="78"/>
+      <c r="H2" s="79"/>
+      <c r="J2" s="77" t="s">
         <v>203</v>
       </c>
-      <c r="C2" s="72"/>
-      <c r="D2" s="73"/>
-      <c r="F2" s="71" t="s">
-        <v>204</v>
-      </c>
-      <c r="G2" s="72"/>
-      <c r="H2" s="73"/>
-      <c r="J2" s="71" t="s">
-        <v>205</v>
-      </c>
-      <c r="K2" s="72"/>
-      <c r="L2" s="73"/>
+      <c r="K2" s="78"/>
+      <c r="L2" s="79"/>
     </row>
     <row r="3" spans="2:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B3" s="34" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="C3" s="35" t="s">
-        <v>196</v>
+        <v>194</v>
       </c>
       <c r="D3" s="36" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
       <c r="F3" s="34" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="G3" s="35" t="s">
-        <v>196</v>
+        <v>194</v>
       </c>
       <c r="H3" s="36" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
       <c r="J3" s="34" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="K3" s="35" t="s">
-        <v>196</v>
+        <v>194</v>
       </c>
       <c r="L3" s="36" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
     </row>
     <row r="4" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B4" s="37" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="C4" s="14">
         <v>4</v>
@@ -4510,7 +4521,7 @@
       </c>
       <c r="H4" s="14"/>
       <c r="J4" s="37" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
       <c r="K4" s="14">
         <v>4</v>
@@ -4519,7 +4530,7 @@
     </row>
     <row r="5" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B5" s="38" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="C5" s="2">
         <v>6</v>
@@ -4535,7 +4546,7 @@
       </c>
       <c r="H5" s="2"/>
       <c r="J5" s="38" t="s">
-        <v>199</v>
+        <v>197</v>
       </c>
       <c r="K5" s="2">
         <v>4</v>
@@ -4544,7 +4555,7 @@
     </row>
     <row r="6" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B6" s="38" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="C6" s="2">
         <v>4</v>
@@ -4560,7 +4571,7 @@
       </c>
       <c r="H6" s="2"/>
       <c r="J6" s="38" t="s">
-        <v>200</v>
+        <v>198</v>
       </c>
       <c r="K6" s="2">
         <v>5</v>
@@ -4569,7 +4580,7 @@
     </row>
     <row r="7" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B7" s="38" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="C7" s="2">
         <v>4</v>
@@ -4585,7 +4596,7 @@
       </c>
       <c r="H7" s="2"/>
       <c r="J7" s="38" t="s">
-        <v>201</v>
+        <v>199</v>
       </c>
       <c r="K7" s="2">
         <v>5</v>
@@ -4594,7 +4605,7 @@
     </row>
     <row r="8" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B8" s="38" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="C8" s="2">
         <v>10</v>
@@ -4610,7 +4621,7 @@
       </c>
       <c r="H8" s="2"/>
       <c r="J8" s="38" t="s">
-        <v>202</v>
+        <v>200</v>
       </c>
       <c r="K8" s="2">
         <v>12</v>
@@ -4619,7 +4630,7 @@
     </row>
     <row r="9" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B9" s="38" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="C9" s="2">
         <v>2</v>
@@ -4636,26 +4647,26 @@
     </row>
     <row r="10" spans="2:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="11" spans="2:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B11" s="74" t="s">
-        <v>197</v>
-      </c>
-      <c r="C11" s="75"/>
+      <c r="B11" s="80" t="s">
+        <v>195</v>
+      </c>
+      <c r="C11" s="81"/>
       <c r="D11" s="33">
         <f>(D4*C4+D5*C5+D6*C6+D7*C7+D8*C8+D9*C9)/30</f>
         <v>4.4333333333333336</v>
       </c>
-      <c r="F11" s="74" t="s">
-        <v>197</v>
-      </c>
-      <c r="G11" s="75"/>
+      <c r="F11" s="80" t="s">
+        <v>195</v>
+      </c>
+      <c r="G11" s="81"/>
       <c r="H11" s="33">
         <f>(H4*G4+H5*G5+H6*G6+H7*G7+H8*G8)/30</f>
         <v>0</v>
       </c>
-      <c r="J11" s="74" t="s">
-        <v>197</v>
-      </c>
-      <c r="K11" s="75"/>
+      <c r="J11" s="80" t="s">
+        <v>195</v>
+      </c>
+      <c r="K11" s="81"/>
       <c r="L11" s="33">
         <f>(L4*K4+L5*K5+L6*K6+L7*K7+L8*K8)/30</f>
         <v>0</v>

</xml_diff>

<commit_message>
New points - POTEC - project and labs
</commit_message>
<xml_diff>
--- a/IoT-points-schedule.xlsx
+++ b/IoT-points-schedule.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\dodo\Desktop\IoT-studies\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5374CC67-EA74-4F6A-AC75-6B427581DCEA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{60543D3C-71EE-4D16-9EE0-C3329DDD987C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="25440" windowHeight="15390" xr2:uid="{F85F5544-1FE8-4920-A5D4-192A98B113BD}"/>
   </bookViews>
@@ -1101,7 +1101,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="82">
+  <cellXfs count="84">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1299,25 +1299,31 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="2" fontId="2" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="2" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="7" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="7" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="7" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="7" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="7" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="7" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="7" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="7" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="7" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="7" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="7" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="7" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -2043,19 +2049,19 @@
     </row>
     <row r="22" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="23" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B23" s="64" t="s">
+      <c r="B23" s="65" t="s">
         <v>79</v>
       </c>
-      <c r="C23" s="65"/>
-      <c r="D23" s="65"/>
-      <c r="E23" s="65"/>
-      <c r="F23" s="65"/>
-      <c r="G23" s="65"/>
-      <c r="H23" s="65"/>
-      <c r="I23" s="65"/>
-      <c r="J23" s="65"/>
-      <c r="K23" s="65"/>
-      <c r="L23" s="66"/>
+      <c r="C23" s="66"/>
+      <c r="D23" s="66"/>
+      <c r="E23" s="66"/>
+      <c r="F23" s="66"/>
+      <c r="G23" s="66"/>
+      <c r="H23" s="66"/>
+      <c r="I23" s="66"/>
+      <c r="J23" s="66"/>
+      <c r="K23" s="66"/>
+      <c r="L23" s="67"/>
       <c r="N23" s="46" t="s">
         <v>129</v>
       </c>
@@ -2065,17 +2071,17 @@
       <c r="S23" s="7"/>
     </row>
     <row r="24" spans="1:19" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B24" s="67"/>
-      <c r="C24" s="68"/>
-      <c r="D24" s="68"/>
-      <c r="E24" s="68"/>
-      <c r="F24" s="68"/>
-      <c r="G24" s="68"/>
-      <c r="H24" s="68"/>
-      <c r="I24" s="68"/>
-      <c r="J24" s="68"/>
-      <c r="K24" s="68"/>
-      <c r="L24" s="69"/>
+      <c r="B24" s="68"/>
+      <c r="C24" s="69"/>
+      <c r="D24" s="69"/>
+      <c r="E24" s="69"/>
+      <c r="F24" s="69"/>
+      <c r="G24" s="69"/>
+      <c r="H24" s="69"/>
+      <c r="I24" s="69"/>
+      <c r="J24" s="69"/>
+      <c r="K24" s="69"/>
+      <c r="L24" s="70"/>
       <c r="N24" s="46"/>
       <c r="O24" s="46"/>
       <c r="Q24" s="7"/>
@@ -2131,7 +2137,7 @@
       <c r="L27" s="2" t="s">
         <v>127</v>
       </c>
-      <c r="N27" s="61">
+      <c r="N27" s="63">
         <f>(K29/30*0.4*5)+(B29/25*0.3*5)+(0.3*F29)</f>
         <v>4.2133333333333329</v>
       </c>
@@ -2162,26 +2168,26 @@
         <v>20</v>
       </c>
       <c r="L28" s="2"/>
-      <c r="N28" s="62"/>
+      <c r="N28" s="64"/>
     </row>
     <row r="29" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B29" s="63">
+      <c r="B29" s="71">
         <f>SUM(B28:C28)</f>
         <v>23</v>
       </c>
-      <c r="C29" s="63"/>
-      <c r="D29" s="63"/>
-      <c r="F29" s="63">
+      <c r="C29" s="71"/>
+      <c r="D29" s="71"/>
+      <c r="F29" s="71">
         <v>5</v>
       </c>
-      <c r="G29" s="63"/>
-      <c r="H29" s="63"/>
-      <c r="I29" s="63"/>
-      <c r="K29" s="63">
+      <c r="G29" s="71"/>
+      <c r="H29" s="71"/>
+      <c r="I29" s="71"/>
+      <c r="K29" s="71">
         <f>SUM(K28:L28)</f>
         <v>20</v>
       </c>
-      <c r="L29" s="63"/>
+      <c r="L29" s="71"/>
       <c r="N29" s="44"/>
     </row>
     <row r="31" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -2207,26 +2213,26 @@
     </row>
     <row r="32" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="33" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B33" s="64" t="s">
+      <c r="B33" s="65" t="s">
         <v>78</v>
       </c>
-      <c r="C33" s="65"/>
-      <c r="D33" s="65"/>
-      <c r="E33" s="65"/>
-      <c r="F33" s="65"/>
-      <c r="G33" s="65"/>
-      <c r="H33" s="65"/>
-      <c r="I33" s="66"/>
+      <c r="C33" s="66"/>
+      <c r="D33" s="66"/>
+      <c r="E33" s="66"/>
+      <c r="F33" s="66"/>
+      <c r="G33" s="66"/>
+      <c r="H33" s="66"/>
+      <c r="I33" s="67"/>
     </row>
     <row r="34" spans="2:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B34" s="67"/>
-      <c r="C34" s="68"/>
-      <c r="D34" s="68"/>
-      <c r="E34" s="68"/>
-      <c r="F34" s="68"/>
-      <c r="G34" s="68"/>
-      <c r="H34" s="68"/>
-      <c r="I34" s="69"/>
+      <c r="B34" s="68"/>
+      <c r="C34" s="69"/>
+      <c r="D34" s="69"/>
+      <c r="E34" s="69"/>
+      <c r="F34" s="69"/>
+      <c r="G34" s="69"/>
+      <c r="H34" s="69"/>
+      <c r="I34" s="70"/>
     </row>
     <row r="36" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B36" s="60" t="s">
@@ -2266,10 +2272,12 @@
       <c r="B38" s="2">
         <v>17</v>
       </c>
-      <c r="C38" s="2"/>
+      <c r="C38" s="2">
+        <v>20</v>
+      </c>
       <c r="E38" s="2">
         <f>C57</f>
-        <v>17</v>
+        <v>25</v>
       </c>
       <c r="F38" s="2">
         <f>G52</f>
@@ -2309,7 +2317,7 @@
       </c>
       <c r="I42" s="2">
         <f>SUM(B38:C38,E38:H38)</f>
-        <v>53</v>
+        <v>81</v>
       </c>
       <c r="J42" s="7"/>
       <c r="L42" s="7"/>
@@ -2318,7 +2326,9 @@
       <c r="B43" s="2" t="s">
         <v>104</v>
       </c>
-      <c r="C43" s="2"/>
+      <c r="C43" s="2">
+        <v>2</v>
+      </c>
       <c r="F43" s="2" t="s">
         <v>118</v>
       </c>
@@ -2368,7 +2378,7 @@
       </c>
       <c r="G46" s="2"/>
       <c r="I46" s="13">
-        <v>3</v>
+        <v>4.5</v>
       </c>
     </row>
     <row r="47" spans="2:15" x14ac:dyDescent="0.25">
@@ -2426,7 +2436,9 @@
       <c r="B52" s="2" t="s">
         <v>113</v>
       </c>
-      <c r="C52" s="2"/>
+      <c r="C52" s="2">
+        <v>2</v>
+      </c>
       <c r="F52" s="2" t="s">
         <v>48</v>
       </c>
@@ -2439,7 +2451,9 @@
       <c r="B53" s="2" t="s">
         <v>114</v>
       </c>
-      <c r="C53" s="2"/>
+      <c r="C53" s="2">
+        <v>4</v>
+      </c>
     </row>
     <row r="54" spans="1:19" x14ac:dyDescent="0.25">
       <c r="B54" s="2" t="s">
@@ -2459,7 +2473,7 @@
       </c>
       <c r="C57" s="2">
         <f>SUM(C42:C55)</f>
-        <v>17</v>
+        <v>25</v>
       </c>
     </row>
     <row r="59" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -2761,40 +2775,40 @@
   <sheetData>
     <row r="1" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="2" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B2" s="70" t="s">
+      <c r="B2" s="72" t="s">
         <v>130</v>
       </c>
-      <c r="C2" s="71"/>
-      <c r="D2" s="71"/>
-      <c r="E2" s="71"/>
-      <c r="F2" s="71"/>
-      <c r="G2" s="71"/>
-      <c r="H2" s="71"/>
-      <c r="I2" s="71"/>
-      <c r="J2" s="71"/>
-      <c r="K2" s="71"/>
-      <c r="L2" s="71"/>
-      <c r="M2" s="71"/>
-      <c r="N2" s="71"/>
-      <c r="O2" s="71"/>
-      <c r="P2" s="72"/>
+      <c r="C2" s="73"/>
+      <c r="D2" s="73"/>
+      <c r="E2" s="73"/>
+      <c r="F2" s="73"/>
+      <c r="G2" s="73"/>
+      <c r="H2" s="73"/>
+      <c r="I2" s="73"/>
+      <c r="J2" s="73"/>
+      <c r="K2" s="73"/>
+      <c r="L2" s="73"/>
+      <c r="M2" s="73"/>
+      <c r="N2" s="73"/>
+      <c r="O2" s="73"/>
+      <c r="P2" s="74"/>
     </row>
     <row r="3" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B3" s="73"/>
-      <c r="C3" s="74"/>
-      <c r="D3" s="74"/>
-      <c r="E3" s="74"/>
-      <c r="F3" s="74"/>
-      <c r="G3" s="74"/>
-      <c r="H3" s="74"/>
-      <c r="I3" s="74"/>
-      <c r="J3" s="74"/>
-      <c r="K3" s="74"/>
-      <c r="L3" s="74"/>
-      <c r="M3" s="74"/>
-      <c r="N3" s="74"/>
-      <c r="O3" s="74"/>
-      <c r="P3" s="75"/>
+      <c r="B3" s="75"/>
+      <c r="C3" s="76"/>
+      <c r="D3" s="76"/>
+      <c r="E3" s="76"/>
+      <c r="F3" s="76"/>
+      <c r="G3" s="76"/>
+      <c r="H3" s="76"/>
+      <c r="I3" s="76"/>
+      <c r="J3" s="76"/>
+      <c r="K3" s="76"/>
+      <c r="L3" s="76"/>
+      <c r="M3" s="76"/>
+      <c r="N3" s="76"/>
+      <c r="O3" s="76"/>
+      <c r="P3" s="77"/>
       <c r="R3" s="12"/>
     </row>
     <row r="5" spans="1:19" x14ac:dyDescent="0.25">
@@ -2942,24 +2956,24 @@
     </row>
     <row r="13" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="14" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B14" s="70" t="s">
+      <c r="B14" s="72" t="s">
         <v>131</v>
       </c>
-      <c r="C14" s="71"/>
-      <c r="D14" s="71"/>
-      <c r="E14" s="71"/>
-      <c r="F14" s="71"/>
-      <c r="G14" s="71"/>
-      <c r="H14" s="72"/>
+      <c r="C14" s="73"/>
+      <c r="D14" s="73"/>
+      <c r="E14" s="73"/>
+      <c r="F14" s="73"/>
+      <c r="G14" s="73"/>
+      <c r="H14" s="74"/>
     </row>
     <row r="15" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B15" s="73"/>
-      <c r="C15" s="74"/>
-      <c r="D15" s="74"/>
-      <c r="E15" s="74"/>
-      <c r="F15" s="74"/>
-      <c r="G15" s="74"/>
-      <c r="H15" s="75"/>
+      <c r="B15" s="75"/>
+      <c r="C15" s="76"/>
+      <c r="D15" s="76"/>
+      <c r="E15" s="76"/>
+      <c r="F15" s="76"/>
+      <c r="G15" s="76"/>
+      <c r="H15" s="77"/>
     </row>
     <row r="17" spans="1:19" x14ac:dyDescent="0.25">
       <c r="B17" s="60" t="s">
@@ -3054,30 +3068,30 @@
     </row>
     <row r="22" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="23" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B23" s="70" t="s">
+      <c r="B23" s="72" t="s">
         <v>132</v>
       </c>
-      <c r="C23" s="71"/>
-      <c r="D23" s="71"/>
-      <c r="E23" s="71"/>
-      <c r="F23" s="71"/>
-      <c r="G23" s="71"/>
-      <c r="H23" s="71"/>
-      <c r="I23" s="71"/>
-      <c r="J23" s="71"/>
-      <c r="K23" s="72"/>
+      <c r="C23" s="73"/>
+      <c r="D23" s="73"/>
+      <c r="E23" s="73"/>
+      <c r="F23" s="73"/>
+      <c r="G23" s="73"/>
+      <c r="H23" s="73"/>
+      <c r="I23" s="73"/>
+      <c r="J23" s="73"/>
+      <c r="K23" s="74"/>
     </row>
     <row r="24" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B24" s="73"/>
-      <c r="C24" s="74"/>
-      <c r="D24" s="74"/>
-      <c r="E24" s="74"/>
-      <c r="F24" s="74"/>
-      <c r="G24" s="74"/>
-      <c r="H24" s="74"/>
-      <c r="I24" s="74"/>
-      <c r="J24" s="74"/>
-      <c r="K24" s="75"/>
+      <c r="B24" s="75"/>
+      <c r="C24" s="76"/>
+      <c r="D24" s="76"/>
+      <c r="E24" s="76"/>
+      <c r="F24" s="76"/>
+      <c r="G24" s="76"/>
+      <c r="H24" s="76"/>
+      <c r="I24" s="76"/>
+      <c r="J24" s="76"/>
+      <c r="K24" s="77"/>
     </row>
     <row r="26" spans="1:19" x14ac:dyDescent="0.25">
       <c r="B26" s="60" t="s">
@@ -3128,7 +3142,7 @@
       <c r="K27" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="M27" s="76">
+      <c r="M27" s="78">
         <f>SUM(B28:C28,E28:G28,I28:K28)</f>
         <v>36</v>
       </c>
@@ -3163,7 +3177,7 @@
       <c r="K28" s="2">
         <v>3.2</v>
       </c>
-      <c r="M28" s="76"/>
+      <c r="M28" s="78"/>
       <c r="N28" s="7"/>
       <c r="O28" s="47"/>
       <c r="P28" s="8"/>
@@ -3191,26 +3205,26 @@
     </row>
     <row r="31" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="32" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B32" s="70" t="s">
+      <c r="B32" s="72" t="s">
         <v>133</v>
       </c>
-      <c r="C32" s="71"/>
-      <c r="D32" s="71"/>
-      <c r="E32" s="71"/>
-      <c r="F32" s="71"/>
-      <c r="G32" s="71"/>
-      <c r="H32" s="71"/>
-      <c r="I32" s="72"/>
+      <c r="C32" s="73"/>
+      <c r="D32" s="73"/>
+      <c r="E32" s="73"/>
+      <c r="F32" s="73"/>
+      <c r="G32" s="73"/>
+      <c r="H32" s="73"/>
+      <c r="I32" s="74"/>
     </row>
     <row r="33" spans="2:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B33" s="73"/>
-      <c r="C33" s="74"/>
-      <c r="D33" s="74"/>
-      <c r="E33" s="74"/>
-      <c r="F33" s="74"/>
-      <c r="G33" s="74"/>
-      <c r="H33" s="74"/>
-      <c r="I33" s="75"/>
+      <c r="B33" s="75"/>
+      <c r="C33" s="76"/>
+      <c r="D33" s="76"/>
+      <c r="E33" s="76"/>
+      <c r="F33" s="76"/>
+      <c r="G33" s="76"/>
+      <c r="H33" s="76"/>
+      <c r="I33" s="77"/>
     </row>
     <row r="35" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B35" s="60" t="s">
@@ -3504,44 +3518,44 @@
     </row>
     <row r="57" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="58" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B58" s="70" t="s">
+      <c r="B58" s="72" t="s">
         <v>134</v>
       </c>
-      <c r="C58" s="71"/>
-      <c r="D58" s="71"/>
-      <c r="E58" s="71"/>
-      <c r="F58" s="71"/>
-      <c r="G58" s="71"/>
-      <c r="H58" s="71"/>
-      <c r="I58" s="71"/>
-      <c r="J58" s="71"/>
-      <c r="K58" s="71"/>
-      <c r="L58" s="71"/>
-      <c r="M58" s="71"/>
-      <c r="N58" s="71"/>
-      <c r="O58" s="71"/>
-      <c r="P58" s="71"/>
-      <c r="Q58" s="71"/>
-      <c r="R58" s="72"/>
+      <c r="C58" s="73"/>
+      <c r="D58" s="73"/>
+      <c r="E58" s="73"/>
+      <c r="F58" s="73"/>
+      <c r="G58" s="73"/>
+      <c r="H58" s="73"/>
+      <c r="I58" s="73"/>
+      <c r="J58" s="73"/>
+      <c r="K58" s="73"/>
+      <c r="L58" s="73"/>
+      <c r="M58" s="73"/>
+      <c r="N58" s="73"/>
+      <c r="O58" s="73"/>
+      <c r="P58" s="73"/>
+      <c r="Q58" s="73"/>
+      <c r="R58" s="74"/>
     </row>
     <row r="59" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B59" s="73"/>
-      <c r="C59" s="74"/>
-      <c r="D59" s="74"/>
-      <c r="E59" s="74"/>
-      <c r="F59" s="74"/>
-      <c r="G59" s="74"/>
-      <c r="H59" s="74"/>
-      <c r="I59" s="74"/>
-      <c r="J59" s="74"/>
-      <c r="K59" s="74"/>
-      <c r="L59" s="74"/>
-      <c r="M59" s="74"/>
-      <c r="N59" s="74"/>
-      <c r="O59" s="74"/>
-      <c r="P59" s="74"/>
-      <c r="Q59" s="74"/>
-      <c r="R59" s="75"/>
+      <c r="B59" s="75"/>
+      <c r="C59" s="76"/>
+      <c r="D59" s="76"/>
+      <c r="E59" s="76"/>
+      <c r="F59" s="76"/>
+      <c r="G59" s="76"/>
+      <c r="H59" s="76"/>
+      <c r="I59" s="76"/>
+      <c r="J59" s="76"/>
+      <c r="K59" s="76"/>
+      <c r="L59" s="76"/>
+      <c r="M59" s="76"/>
+      <c r="N59" s="76"/>
+      <c r="O59" s="76"/>
+      <c r="P59" s="76"/>
+      <c r="Q59" s="76"/>
+      <c r="R59" s="77"/>
     </row>
     <row r="61" spans="1:19" x14ac:dyDescent="0.25">
       <c r="B61" s="60" t="s">
@@ -3707,26 +3721,26 @@
     </row>
     <row r="71" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="72" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B72" s="70" t="s">
+      <c r="B72" s="72" t="s">
         <v>135</v>
       </c>
-      <c r="C72" s="71"/>
-      <c r="D72" s="71"/>
-      <c r="E72" s="71"/>
-      <c r="F72" s="71"/>
-      <c r="G72" s="71"/>
-      <c r="H72" s="71"/>
-      <c r="I72" s="72"/>
+      <c r="C72" s="73"/>
+      <c r="D72" s="73"/>
+      <c r="E72" s="73"/>
+      <c r="F72" s="73"/>
+      <c r="G72" s="73"/>
+      <c r="H72" s="73"/>
+      <c r="I72" s="74"/>
     </row>
     <row r="73" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B73" s="73"/>
-      <c r="C73" s="74"/>
-      <c r="D73" s="74"/>
-      <c r="E73" s="74"/>
-      <c r="F73" s="74"/>
-      <c r="G73" s="74"/>
-      <c r="H73" s="74"/>
-      <c r="I73" s="75"/>
+      <c r="B73" s="75"/>
+      <c r="C73" s="76"/>
+      <c r="D73" s="76"/>
+      <c r="E73" s="76"/>
+      <c r="F73" s="76"/>
+      <c r="G73" s="76"/>
+      <c r="H73" s="76"/>
+      <c r="I73" s="77"/>
     </row>
     <row r="75" spans="1:19" x14ac:dyDescent="0.25">
       <c r="B75" s="4" t="s">
@@ -4078,19 +4092,19 @@
       </c>
     </row>
     <row r="16" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B16" s="19" t="b">
-        <v>0</v>
-      </c>
-      <c r="C16" s="21" t="s">
+      <c r="B16" s="23" t="b">
+        <v>1</v>
+      </c>
+      <c r="C16" s="29" t="s">
         <v>159</v>
       </c>
-      <c r="D16" s="20">
+      <c r="D16" s="28">
         <v>45806</v>
       </c>
-      <c r="E16" s="17" t="s">
+      <c r="E16" s="27" t="s">
         <v>85</v>
       </c>
-      <c r="F16" s="17" t="s">
+      <c r="F16" s="27" t="s">
         <v>164</v>
       </c>
     </row>
@@ -4417,19 +4431,19 @@
       </c>
     </row>
     <row r="41" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B41" s="19" t="b">
-        <v>0</v>
-      </c>
-      <c r="C41" s="21" t="s">
+      <c r="B41" s="23" t="b">
+        <v>1</v>
+      </c>
+      <c r="C41" s="29" t="s">
         <v>79</v>
       </c>
-      <c r="D41" s="20">
+      <c r="D41" s="28">
         <v>45805</v>
       </c>
-      <c r="E41" s="17" t="s">
+      <c r="E41" s="27" t="s">
         <v>220</v>
       </c>
-      <c r="F41" s="17" t="s">
+      <c r="F41" s="27" t="s">
         <v>219</v>
       </c>
     </row>
@@ -4458,21 +4472,21 @@
   <sheetData>
     <row r="1" spans="2:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="2" spans="2:12" ht="23.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B2" s="77" t="s">
+      <c r="B2" s="79" t="s">
         <v>201</v>
       </c>
-      <c r="C2" s="78"/>
-      <c r="D2" s="79"/>
-      <c r="F2" s="77" t="s">
+      <c r="C2" s="80"/>
+      <c r="D2" s="81"/>
+      <c r="F2" s="79" t="s">
         <v>202</v>
       </c>
-      <c r="G2" s="78"/>
-      <c r="H2" s="79"/>
-      <c r="J2" s="77" t="s">
+      <c r="G2" s="80"/>
+      <c r="H2" s="81"/>
+      <c r="J2" s="79" t="s">
         <v>203</v>
       </c>
-      <c r="K2" s="78"/>
-      <c r="L2" s="79"/>
+      <c r="K2" s="80"/>
+      <c r="L2" s="81"/>
     </row>
     <row r="3" spans="2:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B3" s="34" t="s">
@@ -4647,26 +4661,26 @@
     </row>
     <row r="10" spans="2:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="11" spans="2:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B11" s="80" t="s">
+      <c r="B11" s="82" t="s">
         <v>195</v>
       </c>
-      <c r="C11" s="81"/>
+      <c r="C11" s="83"/>
       <c r="D11" s="33">
         <f>(D4*C4+D5*C5+D6*C6+D7*C7+D8*C8+D9*C9)/30</f>
         <v>4.4333333333333336</v>
       </c>
-      <c r="F11" s="80" t="s">
+      <c r="F11" s="82" t="s">
         <v>195</v>
       </c>
-      <c r="G11" s="81"/>
+      <c r="G11" s="83"/>
       <c r="H11" s="33">
         <f>(H4*G4+H5*G5+H6*G6+H7*G7+H8*G8)/30</f>
         <v>0</v>
       </c>
-      <c r="J11" s="80" t="s">
+      <c r="J11" s="82" t="s">
         <v>195</v>
       </c>
-      <c r="K11" s="81"/>
+      <c r="K11" s="83"/>
       <c r="L11" s="33">
         <f>(L4*K4+L5*K5+L6*K6+L7*K7+L8*K8)/30</f>
         <v>0</v>

</xml_diff>

<commit_message>
New points - SYSY - labs 2 and 5
</commit_message>
<xml_diff>
--- a/IoT-points-schedule.xlsx
+++ b/IoT-points-schedule.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28730"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28827"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\dodo\Desktop\IoT-studies\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{60543D3C-71EE-4D16-9EE0-C3329DDD987C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F8793264-63DB-413E-9767-49B253B37FF2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="25440" windowHeight="15390" xr2:uid="{F85F5544-1FE8-4920-A5D4-192A98B113BD}"/>
   </bookViews>
@@ -1856,10 +1856,18 @@
       <c r="D7" s="2">
         <v>3</v>
       </c>
-      <c r="E7" s="2"/>
-      <c r="F7" s="2"/>
-      <c r="H7" s="2"/>
-      <c r="I7" s="2"/>
+      <c r="E7" s="2">
+        <v>3</v>
+      </c>
+      <c r="F7" s="2">
+        <v>3</v>
+      </c>
+      <c r="H7" s="2">
+        <v>5</v>
+      </c>
+      <c r="I7" s="2">
+        <v>4.9000000000000004</v>
+      </c>
       <c r="K7" s="2">
         <v>12</v>
       </c>
@@ -1886,13 +1894,13 @@
     <row r="10" spans="1:19" x14ac:dyDescent="0.25">
       <c r="B10" s="46">
         <f>SUM(B7:F7,H7:I7,K7:N7,P7)</f>
-        <v>25.7</v>
+        <v>41.6</v>
       </c>
       <c r="C10" s="46"/>
       <c r="E10" s="61"/>
       <c r="G10" s="46">
         <f>66-SUM(B7:F7,H7:I7,K7:N7,P7)</f>
-        <v>40.299999999999997</v>
+        <v>24.4</v>
       </c>
       <c r="H10" s="46"/>
     </row>
@@ -1997,22 +2005,26 @@
       </c>
       <c r="L18" s="46">
         <f>SUM(B19:F19,H19:J19)</f>
-        <v>29.5</v>
+        <v>42.5</v>
       </c>
       <c r="M18" s="46"/>
       <c r="O18" s="46">
         <f>50-SUM(B19:F19,H19:J19)</f>
-        <v>20.5</v>
+        <v>7.5</v>
       </c>
       <c r="P18" s="46"/>
       <c r="R18" s="47"/>
     </row>
     <row r="19" spans="1:19" x14ac:dyDescent="0.25">
       <c r="B19" s="2"/>
-      <c r="C19" s="2"/>
+      <c r="C19" s="2">
+        <v>6.5</v>
+      </c>
       <c r="D19" s="2"/>
       <c r="E19" s="2"/>
-      <c r="F19" s="2"/>
+      <c r="F19" s="2">
+        <v>6.5</v>
+      </c>
       <c r="H19" s="2">
         <v>3</v>
       </c>

</xml_diff>

<commit_message>
SYSY - labs 1, 3 and 4
</commit_message>
<xml_diff>
--- a/IoT-points-schedule.xlsx
+++ b/IoT-points-schedule.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\dodo\Desktop\IoT-studies\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C52DF30C-32C7-42D6-AF27-D65884F59E0D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D13BF28C-868C-4D50-B8BC-1F66635A2391}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="25440" windowHeight="15390" xr2:uid="{F85F5544-1FE8-4920-A5D4-192A98B113BD}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="25440" windowHeight="15390" activeTab="3" xr2:uid="{F85F5544-1FE8-4920-A5D4-192A98B113BD}"/>
   </bookViews>
   <sheets>
     <sheet name="II-semestr-25L" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="354" uniqueCount="225">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="353" uniqueCount="225">
   <si>
     <t>1. Krypto</t>
   </si>
@@ -1101,7 +1101,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="84">
+  <cellXfs count="86">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1152,9 +1152,6 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1">
@@ -1223,37 +1220,67 @@
     <xf numFmtId="0" fontId="6" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
       <extLst>
         <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
           <xfpb:xfComplement i="0"/>
         </ext>
       </extLst>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="165" fontId="7" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="7" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="14" fontId="7" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="14" fontId="7" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="7" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="7" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="7" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="7" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="7" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="7" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1270,15 +1297,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="5" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1305,24 +1323,6 @@
     <xf numFmtId="2" fontId="2" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="7" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="7" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="7" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="7" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="7" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="7" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1360,6 +1360,12 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1750,40 +1756,40 @@
   <sheetData>
     <row r="1" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="2" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B2" s="48" t="s">
+      <c r="B2" s="57" t="s">
         <v>76</v>
       </c>
-      <c r="C2" s="49"/>
-      <c r="D2" s="49"/>
-      <c r="E2" s="49"/>
-      <c r="F2" s="49"/>
-      <c r="G2" s="49"/>
-      <c r="H2" s="49"/>
-      <c r="I2" s="49"/>
-      <c r="J2" s="49"/>
-      <c r="K2" s="49"/>
-      <c r="L2" s="49"/>
-      <c r="M2" s="49"/>
-      <c r="N2" s="49"/>
-      <c r="O2" s="49"/>
-      <c r="P2" s="50"/>
+      <c r="C2" s="58"/>
+      <c r="D2" s="58"/>
+      <c r="E2" s="58"/>
+      <c r="F2" s="58"/>
+      <c r="G2" s="58"/>
+      <c r="H2" s="58"/>
+      <c r="I2" s="58"/>
+      <c r="J2" s="58"/>
+      <c r="K2" s="58"/>
+      <c r="L2" s="58"/>
+      <c r="M2" s="58"/>
+      <c r="N2" s="58"/>
+      <c r="O2" s="58"/>
+      <c r="P2" s="59"/>
     </row>
     <row r="3" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B3" s="51"/>
-      <c r="C3" s="52"/>
-      <c r="D3" s="52"/>
-      <c r="E3" s="52"/>
-      <c r="F3" s="52"/>
-      <c r="G3" s="52"/>
-      <c r="H3" s="52"/>
-      <c r="I3" s="52"/>
-      <c r="J3" s="52"/>
-      <c r="K3" s="52"/>
-      <c r="L3" s="52"/>
-      <c r="M3" s="52"/>
-      <c r="N3" s="52"/>
-      <c r="O3" s="52"/>
-      <c r="P3" s="53"/>
+      <c r="B3" s="60"/>
+      <c r="C3" s="61"/>
+      <c r="D3" s="61"/>
+      <c r="E3" s="61"/>
+      <c r="F3" s="61"/>
+      <c r="G3" s="61"/>
+      <c r="H3" s="61"/>
+      <c r="I3" s="61"/>
+      <c r="J3" s="61"/>
+      <c r="K3" s="61"/>
+      <c r="L3" s="61"/>
+      <c r="M3" s="61"/>
+      <c r="N3" s="61"/>
+      <c r="O3" s="61"/>
+      <c r="P3" s="62"/>
       <c r="R3" s="12"/>
     </row>
     <row r="5" spans="1:19" x14ac:dyDescent="0.25">
@@ -1879,17 +1885,17 @@
       <c r="P7" s="2"/>
     </row>
     <row r="9" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B9" s="57" t="s">
+      <c r="B9" s="63" t="s">
         <v>22</v>
       </c>
-      <c r="C9" s="57"/>
+      <c r="C9" s="63"/>
       <c r="E9" s="9" t="s">
         <v>67</v>
       </c>
-      <c r="G9" s="57" t="s">
+      <c r="G9" s="63" t="s">
         <v>87</v>
       </c>
-      <c r="H9" s="57"/>
+      <c r="H9" s="63"/>
     </row>
     <row r="10" spans="1:19" x14ac:dyDescent="0.25">
       <c r="B10" s="46">
@@ -1897,7 +1903,7 @@
         <v>41.6</v>
       </c>
       <c r="C10" s="46"/>
-      <c r="E10" s="61"/>
+      <c r="E10" s="67"/>
       <c r="G10" s="46">
         <f>66-SUM(B7:F7,H7:I7,K7:N7,P7)</f>
         <v>24.4</v>
@@ -1907,7 +1913,7 @@
     <row r="11" spans="1:19" x14ac:dyDescent="0.25">
       <c r="B11" s="46"/>
       <c r="C11" s="46"/>
-      <c r="E11" s="62"/>
+      <c r="E11" s="68"/>
       <c r="G11" s="46"/>
       <c r="H11" s="46"/>
     </row>
@@ -1934,49 +1940,46 @@
     </row>
     <row r="13" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="14" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B14" s="65" t="s">
+      <c r="B14" s="48" t="s">
         <v>77</v>
       </c>
-      <c r="C14" s="66"/>
-      <c r="D14" s="66"/>
-      <c r="E14" s="66"/>
-      <c r="F14" s="66"/>
-      <c r="G14" s="66"/>
-      <c r="H14" s="67"/>
+      <c r="C14" s="49"/>
+      <c r="D14" s="49"/>
+      <c r="E14" s="49"/>
+      <c r="F14" s="49"/>
+      <c r="G14" s="49"/>
+      <c r="H14" s="50"/>
     </row>
     <row r="15" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B15" s="68"/>
-      <c r="C15" s="69"/>
-      <c r="D15" s="69"/>
-      <c r="E15" s="69"/>
-      <c r="F15" s="69"/>
-      <c r="G15" s="69"/>
-      <c r="H15" s="70"/>
+      <c r="B15" s="51"/>
+      <c r="C15" s="52"/>
+      <c r="D15" s="52"/>
+      <c r="E15" s="52"/>
+      <c r="F15" s="52"/>
+      <c r="G15" s="52"/>
+      <c r="H15" s="53"/>
     </row>
     <row r="17" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B17" s="60" t="s">
+      <c r="B17" s="66" t="s">
         <v>91</v>
       </c>
-      <c r="C17" s="60"/>
-      <c r="D17" s="60"/>
-      <c r="E17" s="60"/>
-      <c r="F17" s="60"/>
+      <c r="C17" s="66"/>
+      <c r="D17" s="66"/>
+      <c r="E17" s="66"/>
+      <c r="F17" s="66"/>
       <c r="H17" s="54" t="s">
         <v>97</v>
       </c>
       <c r="I17" s="55"/>
       <c r="J17" s="56"/>
-      <c r="L17" s="57" t="s">
+      <c r="L17" s="63" t="s">
         <v>22</v>
       </c>
-      <c r="M17" s="57"/>
-      <c r="O17" s="57" t="s">
-        <v>87</v>
-      </c>
-      <c r="P17" s="57"/>
-      <c r="R17" s="9" t="s">
+      <c r="M17" s="63"/>
+      <c r="O17" s="9" t="s">
         <v>67</v>
       </c>
+      <c r="P17" s="85"/>
     </row>
     <row r="18" spans="1:19" ht="48.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B18" s="3" t="s">
@@ -2005,23 +2008,27 @@
       </c>
       <c r="L18" s="46">
         <f>SUM(B19:F19,H19:J19)</f>
-        <v>62</v>
+        <v>85</v>
       </c>
       <c r="M18" s="46"/>
-      <c r="O18" s="46">
-        <f>50-SUM(B19:F19,H19:J19)</f>
-        <v>-12</v>
-      </c>
-      <c r="P18" s="46"/>
-      <c r="R18" s="47"/>
+      <c r="O18" s="47">
+        <v>4.5</v>
+      </c>
+      <c r="P18" s="84"/>
     </row>
     <row r="19" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B19" s="2"/>
+      <c r="B19" s="2">
+        <v>7</v>
+      </c>
       <c r="C19" s="2">
         <v>6.5</v>
       </c>
-      <c r="D19" s="2"/>
-      <c r="E19" s="2"/>
+      <c r="D19" s="2">
+        <v>8</v>
+      </c>
+      <c r="E19" s="2">
+        <v>8</v>
+      </c>
       <c r="F19" s="2">
         <v>6.5</v>
       </c>
@@ -2036,9 +2043,8 @@
       </c>
       <c r="L19" s="46"/>
       <c r="M19" s="46"/>
-      <c r="O19" s="46"/>
-      <c r="P19" s="46"/>
-      <c r="R19" s="47"/>
+      <c r="O19" s="47"/>
+      <c r="P19" s="84"/>
     </row>
     <row r="21" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A21" s="6"/>
@@ -2063,19 +2069,19 @@
     </row>
     <row r="22" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="23" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B23" s="65" t="s">
+      <c r="B23" s="48" t="s">
         <v>79</v>
       </c>
-      <c r="C23" s="66"/>
-      <c r="D23" s="66"/>
-      <c r="E23" s="66"/>
-      <c r="F23" s="66"/>
-      <c r="G23" s="66"/>
-      <c r="H23" s="66"/>
-      <c r="I23" s="66"/>
-      <c r="J23" s="66"/>
-      <c r="K23" s="66"/>
-      <c r="L23" s="67"/>
+      <c r="C23" s="49"/>
+      <c r="D23" s="49"/>
+      <c r="E23" s="49"/>
+      <c r="F23" s="49"/>
+      <c r="G23" s="49"/>
+      <c r="H23" s="49"/>
+      <c r="I23" s="49"/>
+      <c r="J23" s="49"/>
+      <c r="K23" s="49"/>
+      <c r="L23" s="50"/>
       <c r="N23" s="46" t="s">
         <v>129</v>
       </c>
@@ -2085,17 +2091,17 @@
       <c r="S23" s="7"/>
     </row>
     <row r="24" spans="1:19" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B24" s="68"/>
-      <c r="C24" s="69"/>
-      <c r="D24" s="69"/>
-      <c r="E24" s="69"/>
-      <c r="F24" s="69"/>
-      <c r="G24" s="69"/>
-      <c r="H24" s="69"/>
-      <c r="I24" s="69"/>
-      <c r="J24" s="69"/>
-      <c r="K24" s="69"/>
-      <c r="L24" s="70"/>
+      <c r="B24" s="51"/>
+      <c r="C24" s="52"/>
+      <c r="D24" s="52"/>
+      <c r="E24" s="52"/>
+      <c r="F24" s="52"/>
+      <c r="G24" s="52"/>
+      <c r="H24" s="52"/>
+      <c r="I24" s="52"/>
+      <c r="J24" s="52"/>
+      <c r="K24" s="52"/>
+      <c r="L24" s="53"/>
       <c r="N24" s="46"/>
       <c r="O24" s="46"/>
       <c r="Q24" s="7"/>
@@ -2103,17 +2109,17 @@
       <c r="S24" s="7"/>
     </row>
     <row r="26" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B26" s="60" t="s">
+      <c r="B26" s="66" t="s">
         <v>8</v>
       </c>
-      <c r="C26" s="60"/>
-      <c r="D26" s="60"/>
-      <c r="F26" s="60" t="s">
+      <c r="C26" s="66"/>
+      <c r="D26" s="66"/>
+      <c r="F26" s="66" t="s">
         <v>208</v>
       </c>
-      <c r="G26" s="60"/>
-      <c r="H26" s="60"/>
-      <c r="I26" s="60"/>
+      <c r="G26" s="66"/>
+      <c r="H26" s="66"/>
+      <c r="I26" s="66"/>
       <c r="J26" s="7"/>
       <c r="K26" s="54" t="s">
         <v>128</v>
@@ -2151,7 +2157,7 @@
       <c r="L27" s="2" t="s">
         <v>127</v>
       </c>
-      <c r="N27" s="63">
+      <c r="N27" s="69">
         <f>(K29/30*0.4*5)+(B29/25*0.3*5)+(0.3*F29)</f>
         <v>4.2133333333333329</v>
       </c>
@@ -2182,7 +2188,7 @@
         <v>20</v>
       </c>
       <c r="L28" s="2"/>
-      <c r="N28" s="64"/>
+      <c r="N28" s="70"/>
     </row>
     <row r="29" spans="1:19" x14ac:dyDescent="0.25">
       <c r="B29" s="71">
@@ -2202,7 +2208,7 @@
         <v>20</v>
       </c>
       <c r="L29" s="71"/>
-      <c r="N29" s="44"/>
+      <c r="N29" s="38"/>
     </row>
     <row r="31" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A31" s="6"/>
@@ -2227,32 +2233,32 @@
     </row>
     <row r="32" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="33" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B33" s="65" t="s">
+      <c r="B33" s="48" t="s">
         <v>78</v>
       </c>
-      <c r="C33" s="66"/>
-      <c r="D33" s="66"/>
-      <c r="E33" s="66"/>
-      <c r="F33" s="66"/>
-      <c r="G33" s="66"/>
-      <c r="H33" s="66"/>
-      <c r="I33" s="67"/>
+      <c r="C33" s="49"/>
+      <c r="D33" s="49"/>
+      <c r="E33" s="49"/>
+      <c r="F33" s="49"/>
+      <c r="G33" s="49"/>
+      <c r="H33" s="49"/>
+      <c r="I33" s="50"/>
     </row>
     <row r="34" spans="2:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B34" s="68"/>
-      <c r="C34" s="69"/>
-      <c r="D34" s="69"/>
-      <c r="E34" s="69"/>
-      <c r="F34" s="69"/>
-      <c r="G34" s="69"/>
-      <c r="H34" s="69"/>
-      <c r="I34" s="70"/>
+      <c r="B34" s="51"/>
+      <c r="C34" s="52"/>
+      <c r="D34" s="52"/>
+      <c r="E34" s="52"/>
+      <c r="F34" s="52"/>
+      <c r="G34" s="52"/>
+      <c r="H34" s="52"/>
+      <c r="I34" s="53"/>
     </row>
     <row r="36" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B36" s="60" t="s">
+      <c r="B36" s="66" t="s">
         <v>98</v>
       </c>
-      <c r="C36" s="60"/>
+      <c r="C36" s="66"/>
       <c r="D36" s="7"/>
       <c r="E36" s="54" t="s">
         <v>144</v>
@@ -2302,10 +2308,10 @@
       <c r="O38" s="7"/>
     </row>
     <row r="41" spans="2:15" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B41" s="58" t="s">
+      <c r="B41" s="64" t="s">
         <v>126</v>
       </c>
-      <c r="C41" s="59"/>
+      <c r="C41" s="65"/>
       <c r="F41" s="46" t="s">
         <v>102</v>
       </c>
@@ -2363,7 +2369,7 @@
         <v>119</v>
       </c>
       <c r="G44" s="2"/>
-      <c r="I44" s="57" t="s">
+      <c r="I44" s="63" t="s">
         <v>67</v>
       </c>
     </row>
@@ -2378,7 +2384,7 @@
         <v>120</v>
       </c>
       <c r="G45" s="2"/>
-      <c r="I45" s="57"/>
+      <c r="I45" s="63"/>
     </row>
     <row r="46" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B46" s="2" t="s">
@@ -2414,7 +2420,7 @@
         <v>123</v>
       </c>
       <c r="G48" s="2"/>
-      <c r="I48" s="44"/>
+      <c r="I48" s="38"/>
     </row>
     <row r="49" spans="1:19" x14ac:dyDescent="0.25">
       <c r="B49" s="2" t="s">
@@ -2513,70 +2519,70 @@
     </row>
     <row r="60" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="61" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B61" s="48" t="s">
+      <c r="B61" s="57" t="s">
         <v>80</v>
       </c>
-      <c r="C61" s="49"/>
-      <c r="D61" s="49"/>
-      <c r="E61" s="49"/>
-      <c r="F61" s="49"/>
-      <c r="G61" s="49"/>
-      <c r="H61" s="49"/>
-      <c r="I61" s="49"/>
-      <c r="J61" s="49"/>
-      <c r="K61" s="49"/>
-      <c r="L61" s="49"/>
-      <c r="M61" s="49"/>
-      <c r="N61" s="49"/>
-      <c r="O61" s="49"/>
-      <c r="P61" s="49"/>
-      <c r="Q61" s="49"/>
-      <c r="R61" s="49"/>
-      <c r="S61" s="50"/>
+      <c r="C61" s="58"/>
+      <c r="D61" s="58"/>
+      <c r="E61" s="58"/>
+      <c r="F61" s="58"/>
+      <c r="G61" s="58"/>
+      <c r="H61" s="58"/>
+      <c r="I61" s="58"/>
+      <c r="J61" s="58"/>
+      <c r="K61" s="58"/>
+      <c r="L61" s="58"/>
+      <c r="M61" s="58"/>
+      <c r="N61" s="58"/>
+      <c r="O61" s="58"/>
+      <c r="P61" s="58"/>
+      <c r="Q61" s="58"/>
+      <c r="R61" s="58"/>
+      <c r="S61" s="59"/>
     </row>
     <row r="62" spans="1:19" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B62" s="51"/>
-      <c r="C62" s="52"/>
-      <c r="D62" s="52"/>
-      <c r="E62" s="52"/>
-      <c r="F62" s="52"/>
-      <c r="G62" s="52"/>
-      <c r="H62" s="52"/>
-      <c r="I62" s="52"/>
-      <c r="J62" s="52"/>
-      <c r="K62" s="52"/>
-      <c r="L62" s="52"/>
-      <c r="M62" s="52"/>
-      <c r="N62" s="52"/>
-      <c r="O62" s="52"/>
-      <c r="P62" s="52"/>
-      <c r="Q62" s="52"/>
-      <c r="R62" s="52"/>
-      <c r="S62" s="53"/>
+      <c r="B62" s="60"/>
+      <c r="C62" s="61"/>
+      <c r="D62" s="61"/>
+      <c r="E62" s="61"/>
+      <c r="F62" s="61"/>
+      <c r="G62" s="61"/>
+      <c r="H62" s="61"/>
+      <c r="I62" s="61"/>
+      <c r="J62" s="61"/>
+      <c r="K62" s="61"/>
+      <c r="L62" s="61"/>
+      <c r="M62" s="61"/>
+      <c r="N62" s="61"/>
+      <c r="O62" s="61"/>
+      <c r="P62" s="61"/>
+      <c r="Q62" s="61"/>
+      <c r="R62" s="61"/>
+      <c r="S62" s="62"/>
     </row>
     <row r="64" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B64" s="60" t="s">
+      <c r="B64" s="66" t="s">
         <v>63</v>
       </c>
-      <c r="C64" s="60"/>
-      <c r="D64" s="60"/>
-      <c r="E64" s="60"/>
-      <c r="F64" s="60"/>
-      <c r="G64" s="60"/>
-      <c r="H64" s="60"/>
-      <c r="I64" s="60"/>
-      <c r="J64" s="60"/>
-      <c r="K64" s="60"/>
-      <c r="M64" s="60" t="s">
+      <c r="C64" s="66"/>
+      <c r="D64" s="66"/>
+      <c r="E64" s="66"/>
+      <c r="F64" s="66"/>
+      <c r="G64" s="66"/>
+      <c r="H64" s="66"/>
+      <c r="I64" s="66"/>
+      <c r="J64" s="66"/>
+      <c r="K64" s="66"/>
+      <c r="M64" s="66" t="s">
         <v>90</v>
       </c>
-      <c r="N64" s="60"/>
-      <c r="O64" s="60"/>
-      <c r="P64" s="60"/>
-      <c r="R64" s="60" t="s">
+      <c r="N64" s="66"/>
+      <c r="O64" s="66"/>
+      <c r="P64" s="66"/>
+      <c r="R64" s="66" t="s">
         <v>64</v>
       </c>
-      <c r="S64" s="60"/>
+      <c r="S64" s="66"/>
     </row>
     <row r="65" spans="2:19" x14ac:dyDescent="0.25">
       <c r="B65" s="2" t="s">
@@ -2671,18 +2677,18 @@
       <c r="S66" s="2"/>
     </row>
     <row r="69" spans="2:19" x14ac:dyDescent="0.25">
-      <c r="B69" s="57" t="s">
+      <c r="B69" s="63" t="s">
         <v>22</v>
       </c>
-      <c r="C69" s="57"/>
+      <c r="C69" s="63"/>
       <c r="E69" s="9" t="s">
         <v>67</v>
       </c>
-      <c r="G69" s="57" t="s">
+      <c r="G69" s="63" t="s">
         <v>87</v>
       </c>
-      <c r="H69" s="57"/>
-      <c r="K69" s="45" t="s">
+      <c r="H69" s="63"/>
+      <c r="K69" s="39" t="s">
         <v>223</v>
       </c>
     </row>
@@ -2711,7 +2717,7 @@
       <c r="K71" s="46"/>
     </row>
   </sheetData>
-  <mergeCells count="42">
+  <mergeCells count="40">
     <mergeCell ref="K29:L29"/>
     <mergeCell ref="R64:S64"/>
     <mergeCell ref="B33:I34"/>
@@ -2725,7 +2731,6 @@
     <mergeCell ref="K26:L26"/>
     <mergeCell ref="B23:L24"/>
     <mergeCell ref="B26:D26"/>
-    <mergeCell ref="O17:P17"/>
     <mergeCell ref="B9:C9"/>
     <mergeCell ref="B10:C11"/>
     <mergeCell ref="L17:M17"/>
@@ -2739,7 +2744,7 @@
     <mergeCell ref="G69:H69"/>
     <mergeCell ref="G70:H71"/>
     <mergeCell ref="K70:K71"/>
-    <mergeCell ref="R18:R19"/>
+    <mergeCell ref="O18:O19"/>
     <mergeCell ref="B14:H15"/>
     <mergeCell ref="K5:N5"/>
     <mergeCell ref="B2:P3"/>
@@ -2750,7 +2755,6 @@
     <mergeCell ref="B5:F5"/>
     <mergeCell ref="H5:I5"/>
     <mergeCell ref="N23:O24"/>
-    <mergeCell ref="O18:P19"/>
     <mergeCell ref="B36:C36"/>
     <mergeCell ref="E36:H36"/>
     <mergeCell ref="G9:H9"/>
@@ -2826,14 +2830,14 @@
       <c r="R3" s="12"/>
     </row>
     <row r="5" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B5" s="60" t="s">
+      <c r="B5" s="66" t="s">
         <v>18</v>
       </c>
-      <c r="C5" s="60"/>
-      <c r="D5" s="60"/>
-      <c r="E5" s="60"/>
-      <c r="F5" s="60"/>
-      <c r="G5" s="60"/>
+      <c r="C5" s="66"/>
+      <c r="D5" s="66"/>
+      <c r="E5" s="66"/>
+      <c r="F5" s="66"/>
+      <c r="G5" s="66"/>
       <c r="I5" s="4" t="s">
         <v>28</v>
       </c>
@@ -2924,10 +2928,10 @@
       </c>
     </row>
     <row r="9" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B9" s="57" t="s">
+      <c r="B9" s="63" t="s">
         <v>22</v>
       </c>
-      <c r="C9" s="57"/>
+      <c r="C9" s="63"/>
       <c r="E9" s="9" t="s">
         <v>67</v>
       </c>
@@ -2938,14 +2942,14 @@
         <v>110</v>
       </c>
       <c r="C10" s="46"/>
-      <c r="E10" s="61">
+      <c r="E10" s="67">
         <v>4</v>
       </c>
     </row>
     <row r="11" spans="1:19" x14ac:dyDescent="0.25">
       <c r="B11" s="46"/>
       <c r="C11" s="46"/>
-      <c r="E11" s="62"/>
+      <c r="E11" s="68"/>
     </row>
     <row r="12" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A12" s="6"/>
@@ -2990,20 +2994,20 @@
       <c r="H15" s="77"/>
     </row>
     <row r="17" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B17" s="60" t="s">
+      <c r="B17" s="66" t="s">
         <v>12</v>
       </c>
-      <c r="C17" s="60"/>
-      <c r="D17" s="60"/>
-      <c r="F17" s="60" t="s">
+      <c r="C17" s="66"/>
+      <c r="D17" s="66"/>
+      <c r="F17" s="66" t="s">
         <v>8</v>
       </c>
-      <c r="G17" s="60"/>
-      <c r="H17" s="60"/>
-      <c r="J17" s="57" t="s">
+      <c r="G17" s="66"/>
+      <c r="H17" s="66"/>
+      <c r="J17" s="63" t="s">
         <v>22</v>
       </c>
-      <c r="K17" s="57"/>
+      <c r="K17" s="63"/>
       <c r="M17" s="9" t="s">
         <v>67</v>
       </c>
@@ -3108,20 +3112,20 @@
       <c r="K24" s="77"/>
     </row>
     <row r="26" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B26" s="60" t="s">
+      <c r="B26" s="66" t="s">
         <v>17</v>
       </c>
-      <c r="C26" s="60"/>
+      <c r="C26" s="66"/>
       <c r="E26" s="54" t="s">
         <v>21</v>
       </c>
       <c r="F26" s="55"/>
       <c r="G26" s="56"/>
-      <c r="I26" s="60" t="s">
+      <c r="I26" s="66" t="s">
         <v>20</v>
       </c>
-      <c r="J26" s="60"/>
-      <c r="K26" s="60"/>
+      <c r="J26" s="66"/>
+      <c r="K26" s="66"/>
       <c r="M26" s="10" t="s">
         <v>22</v>
       </c>
@@ -3241,17 +3245,17 @@
       <c r="I33" s="77"/>
     </row>
     <row r="35" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B35" s="60" t="s">
+      <c r="B35" s="66" t="s">
         <v>31</v>
       </c>
-      <c r="C35" s="60"/>
-      <c r="D35" s="60"/>
-      <c r="F35" s="60" t="s">
+      <c r="C35" s="66"/>
+      <c r="D35" s="66"/>
+      <c r="F35" s="66" t="s">
         <v>12</v>
       </c>
-      <c r="G35" s="60"/>
-      <c r="H35" s="60"/>
-      <c r="I35" s="60"/>
+      <c r="G35" s="66"/>
+      <c r="H35" s="66"/>
+      <c r="I35" s="66"/>
       <c r="N35" s="7"/>
       <c r="O35" s="7"/>
     </row>
@@ -3308,10 +3312,10 @@
       <c r="O37" s="7"/>
     </row>
     <row r="40" spans="2:15" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B40" s="58" t="s">
+      <c r="B40" s="64" t="s">
         <v>35</v>
       </c>
-      <c r="C40" s="59"/>
+      <c r="C40" s="65"/>
       <c r="F40" s="46" t="s">
         <v>36</v>
       </c>
@@ -3371,7 +3375,7 @@
       <c r="G43" s="2">
         <v>0.44</v>
       </c>
-      <c r="I43" s="57" t="s">
+      <c r="I43" s="63" t="s">
         <v>67</v>
       </c>
     </row>
@@ -3388,7 +3392,7 @@
       <c r="G44" s="2">
         <v>1</v>
       </c>
-      <c r="I44" s="57"/>
+      <c r="I44" s="63"/>
     </row>
     <row r="45" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B45" s="2" t="s">
@@ -3572,27 +3576,27 @@
       <c r="R59" s="77"/>
     </row>
     <row r="61" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B61" s="60" t="s">
+      <c r="B61" s="66" t="s">
         <v>63</v>
       </c>
-      <c r="C61" s="60"/>
-      <c r="D61" s="60"/>
-      <c r="E61" s="60"/>
-      <c r="F61" s="60"/>
-      <c r="G61" s="60"/>
-      <c r="H61" s="60"/>
-      <c r="I61" s="60"/>
-      <c r="J61" s="60"/>
-      <c r="K61" s="60"/>
-      <c r="M61" s="60" t="s">
+      <c r="C61" s="66"/>
+      <c r="D61" s="66"/>
+      <c r="E61" s="66"/>
+      <c r="F61" s="66"/>
+      <c r="G61" s="66"/>
+      <c r="H61" s="66"/>
+      <c r="I61" s="66"/>
+      <c r="J61" s="66"/>
+      <c r="K61" s="66"/>
+      <c r="M61" s="66" t="s">
         <v>68</v>
       </c>
-      <c r="N61" s="60"/>
-      <c r="O61" s="60"/>
-      <c r="Q61" s="60" t="s">
+      <c r="N61" s="66"/>
+      <c r="O61" s="66"/>
+      <c r="Q61" s="66" t="s">
         <v>64</v>
       </c>
-      <c r="R61" s="60"/>
+      <c r="R61" s="66"/>
     </row>
     <row r="62" spans="1:19" x14ac:dyDescent="0.25">
       <c r="B62" s="2" t="s">
@@ -3689,10 +3693,10 @@
       </c>
     </row>
     <row r="66" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B66" s="57" t="s">
+      <c r="B66" s="63" t="s">
         <v>22</v>
       </c>
-      <c r="C66" s="57"/>
+      <c r="C66" s="63"/>
       <c r="E66" s="9" t="s">
         <v>67</v>
       </c>
@@ -3781,10 +3785,10 @@
       <c r="I75" s="4" t="s">
         <v>143</v>
       </c>
-      <c r="K75" s="57" t="s">
+      <c r="K75" s="63" t="s">
         <v>22</v>
       </c>
-      <c r="L75" s="57"/>
+      <c r="L75" s="63"/>
       <c r="N75" s="9" t="s">
         <v>67</v>
       </c>
@@ -3913,261 +3917,261 @@
       </c>
     </row>
     <row r="3" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B3" s="23" t="b">
+      <c r="B3" s="22" t="b">
         <v>1</v>
       </c>
-      <c r="C3" s="30" t="s">
+      <c r="C3" s="29" t="s">
         <v>77</v>
       </c>
-      <c r="D3" s="25">
+      <c r="D3" s="24">
         <v>45763</v>
       </c>
-      <c r="E3" s="26" t="s">
+      <c r="E3" s="25" t="s">
         <v>147</v>
       </c>
-      <c r="F3" s="24" t="s">
+      <c r="F3" s="23" t="s">
         <v>181</v>
       </c>
     </row>
     <row r="4" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B4" s="19" t="b">
+      <c r="B4" s="22" t="b">
+        <v>1</v>
+      </c>
+      <c r="C4" s="28" t="s">
+        <v>77</v>
+      </c>
+      <c r="D4" s="27">
+        <v>45812</v>
+      </c>
+      <c r="E4" s="40" t="s">
+        <v>148</v>
+      </c>
+      <c r="F4" s="26" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="5" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B5" s="41" t="b">
         <v>0</v>
       </c>
-      <c r="C4" s="21" t="s">
+      <c r="C5" s="42" t="s">
         <v>77</v>
       </c>
-      <c r="D4" s="20">
-        <v>45803</v>
-      </c>
-      <c r="E4" s="18" t="s">
-        <v>148</v>
-      </c>
-      <c r="F4" s="17" t="s">
-        <v>182</v>
-      </c>
-    </row>
-    <row r="5" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B5" s="39" t="b">
+      <c r="D5" s="43">
+        <v>45817</v>
+      </c>
+      <c r="E5" s="44" t="s">
+        <v>149</v>
+      </c>
+      <c r="F5" s="45" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="6" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="C6" s="30"/>
+    </row>
+    <row r="7" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B7" s="22" t="b">
+        <v>1</v>
+      </c>
+      <c r="C7" s="28" t="s">
+        <v>77</v>
+      </c>
+      <c r="D7" s="27">
+        <v>45729</v>
+      </c>
+      <c r="E7" s="26" t="s">
+        <v>103</v>
+      </c>
+      <c r="F7" s="26" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="8" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B8" s="22" t="b">
+        <v>1</v>
+      </c>
+      <c r="C8" s="28" t="s">
+        <v>77</v>
+      </c>
+      <c r="D8" s="27">
+        <v>45743</v>
+      </c>
+      <c r="E8" s="26" t="s">
+        <v>104</v>
+      </c>
+      <c r="F8" s="26" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="9" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B9" s="22" t="b">
+        <v>1</v>
+      </c>
+      <c r="C9" s="28" t="s">
+        <v>77</v>
+      </c>
+      <c r="D9" s="27">
+        <v>45757</v>
+      </c>
+      <c r="E9" s="26" t="s">
+        <v>105</v>
+      </c>
+      <c r="F9" s="26" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="10" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B10" s="22" t="b">
+        <v>1</v>
+      </c>
+      <c r="C10" s="28" t="s">
+        <v>77</v>
+      </c>
+      <c r="D10" s="27">
+        <v>45785</v>
+      </c>
+      <c r="E10" s="26" t="s">
+        <v>106</v>
+      </c>
+      <c r="F10" s="26" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="11" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B11" s="22" t="b">
+        <v>1</v>
+      </c>
+      <c r="C11" s="28" t="s">
+        <v>77</v>
+      </c>
+      <c r="D11" s="27">
+        <v>45799</v>
+      </c>
+      <c r="E11" s="26" t="s">
+        <v>107</v>
+      </c>
+      <c r="F11" s="26" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="12" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="C12" s="30"/>
+    </row>
+    <row r="13" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B13" s="22" t="b">
+        <v>1</v>
+      </c>
+      <c r="C13" s="28" t="s">
+        <v>159</v>
+      </c>
+      <c r="D13" s="27">
+        <v>45728</v>
+      </c>
+      <c r="E13" s="26" t="s">
+        <v>84</v>
+      </c>
+      <c r="F13" s="26" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="14" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B14" s="22" t="b">
+        <v>1</v>
+      </c>
+      <c r="C14" s="28" t="s">
+        <v>159</v>
+      </c>
+      <c r="D14" s="27">
+        <v>45747</v>
+      </c>
+      <c r="E14" s="26" t="s">
+        <v>161</v>
+      </c>
+      <c r="F14" s="26" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="15" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B15" s="22" t="b">
+        <v>1</v>
+      </c>
+      <c r="C15" s="28" t="s">
+        <v>159</v>
+      </c>
+      <c r="D15" s="27">
+        <v>45784</v>
+      </c>
+      <c r="E15" s="26" t="s">
+        <v>162</v>
+      </c>
+      <c r="F15" s="26" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="16" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B16" s="22" t="b">
+        <v>1</v>
+      </c>
+      <c r="C16" s="28" t="s">
+        <v>159</v>
+      </c>
+      <c r="D16" s="27">
+        <v>45806</v>
+      </c>
+      <c r="E16" s="26" t="s">
+        <v>85</v>
+      </c>
+      <c r="F16" s="26" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="17" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B17" s="18" t="b">
         <v>0</v>
       </c>
-      <c r="C5" s="40" t="s">
-        <v>77</v>
-      </c>
-      <c r="D5" s="41">
-        <v>45817</v>
-      </c>
-      <c r="E5" s="42" t="s">
-        <v>149</v>
-      </c>
-      <c r="F5" s="43" t="s">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="6" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="C6" s="31"/>
-    </row>
-    <row r="7" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B7" s="23" t="b">
-        <v>1</v>
-      </c>
-      <c r="C7" s="29" t="s">
-        <v>77</v>
-      </c>
-      <c r="D7" s="28">
-        <v>45729</v>
-      </c>
-      <c r="E7" s="27" t="s">
-        <v>103</v>
-      </c>
-      <c r="F7" s="27" t="s">
-        <v>151</v>
-      </c>
-    </row>
-    <row r="8" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B8" s="23" t="b">
-        <v>1</v>
-      </c>
-      <c r="C8" s="29" t="s">
-        <v>77</v>
-      </c>
-      <c r="D8" s="28">
-        <v>45743</v>
-      </c>
-      <c r="E8" s="27" t="s">
-        <v>104</v>
-      </c>
-      <c r="F8" s="27" t="s">
-        <v>152</v>
-      </c>
-    </row>
-    <row r="9" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B9" s="23" t="b">
-        <v>1</v>
-      </c>
-      <c r="C9" s="29" t="s">
-        <v>77</v>
-      </c>
-      <c r="D9" s="28">
-        <v>45757</v>
-      </c>
-      <c r="E9" s="27" t="s">
-        <v>105</v>
-      </c>
-      <c r="F9" s="27" t="s">
-        <v>153</v>
-      </c>
-    </row>
-    <row r="10" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B10" s="23" t="b">
-        <v>1</v>
-      </c>
-      <c r="C10" s="29" t="s">
-        <v>77</v>
-      </c>
-      <c r="D10" s="28">
-        <v>45785</v>
-      </c>
-      <c r="E10" s="27" t="s">
-        <v>106</v>
-      </c>
-      <c r="F10" s="27" t="s">
-        <v>154</v>
-      </c>
-    </row>
-    <row r="11" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B11" s="23" t="b">
-        <v>1</v>
-      </c>
-      <c r="C11" s="29" t="s">
-        <v>77</v>
-      </c>
-      <c r="D11" s="28">
-        <v>45799</v>
-      </c>
-      <c r="E11" s="27" t="s">
-        <v>107</v>
-      </c>
-      <c r="F11" s="27" t="s">
-        <v>155</v>
-      </c>
-    </row>
-    <row r="12" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="C12" s="31"/>
-    </row>
-    <row r="13" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B13" s="23" t="b">
-        <v>1</v>
-      </c>
-      <c r="C13" s="29" t="s">
+      <c r="C17" s="20" t="s">
         <v>159</v>
       </c>
-      <c r="D13" s="28">
-        <v>45728</v>
-      </c>
-      <c r="E13" s="27" t="s">
-        <v>84</v>
-      </c>
-      <c r="F13" s="27" t="s">
-        <v>160</v>
-      </c>
-    </row>
-    <row r="14" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B14" s="23" t="b">
-        <v>1</v>
-      </c>
-      <c r="C14" s="29" t="s">
-        <v>159</v>
-      </c>
-      <c r="D14" s="28">
-        <v>45747</v>
-      </c>
-      <c r="E14" s="27" t="s">
-        <v>161</v>
-      </c>
-      <c r="F14" s="27" t="s">
-        <v>165</v>
-      </c>
-    </row>
-    <row r="15" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B15" s="23" t="b">
-        <v>1</v>
-      </c>
-      <c r="C15" s="29" t="s">
-        <v>159</v>
-      </c>
-      <c r="D15" s="28">
-        <v>45784</v>
-      </c>
-      <c r="E15" s="27" t="s">
-        <v>162</v>
-      </c>
-      <c r="F15" s="27" t="s">
-        <v>163</v>
-      </c>
-    </row>
-    <row r="16" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B16" s="23" t="b">
-        <v>1</v>
-      </c>
-      <c r="C16" s="29" t="s">
-        <v>159</v>
-      </c>
-      <c r="D16" s="28">
-        <v>45806</v>
-      </c>
-      <c r="E16" s="27" t="s">
-        <v>85</v>
-      </c>
-      <c r="F16" s="27" t="s">
-        <v>164</v>
-      </c>
-    </row>
-    <row r="17" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B17" s="19" t="b">
-        <v>0</v>
-      </c>
-      <c r="C17" s="21" t="s">
-        <v>159</v>
-      </c>
-      <c r="D17" s="20">
+      <c r="D17" s="19">
         <v>45817</v>
       </c>
       <c r="E17" s="17" t="s">
         <v>167</v>
       </c>
-      <c r="F17" s="21" t="s">
+      <c r="F17" s="20" t="s">
         <v>166</v>
       </c>
     </row>
     <row r="18" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B18" s="19" t="b">
+      <c r="B18" s="18" t="b">
         <v>0</v>
       </c>
-      <c r="C18" s="21" t="s">
+      <c r="C18" s="20" t="s">
         <v>159</v>
       </c>
-      <c r="D18" s="20">
+      <c r="D18" s="19">
         <v>45819</v>
       </c>
       <c r="E18" s="17" t="s">
         <v>169</v>
       </c>
-      <c r="F18" s="21" t="s">
+      <c r="F18" s="20" t="s">
         <v>168</v>
       </c>
     </row>
     <row r="19" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="C19" s="31"/>
-      <c r="D19" s="22"/>
+      <c r="C19" s="30"/>
+      <c r="D19" s="21"/>
     </row>
     <row r="20" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B20" s="19" t="b">
+      <c r="B20" s="18" t="b">
         <v>0</v>
       </c>
-      <c r="C20" s="21" t="s">
+      <c r="C20" s="20" t="s">
         <v>159</v>
       </c>
-      <c r="D20" s="20">
+      <c r="D20" s="19">
         <v>45820</v>
       </c>
       <c r="E20" s="17" t="s">
@@ -4175,13 +4179,13 @@
       </c>
     </row>
     <row r="21" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B21" s="19" t="b">
+      <c r="B21" s="18" t="b">
         <v>0</v>
       </c>
-      <c r="C21" s="21" t="s">
+      <c r="C21" s="20" t="s">
         <v>159</v>
       </c>
-      <c r="D21" s="20">
+      <c r="D21" s="19">
         <v>45820</v>
       </c>
       <c r="E21" s="17" t="s">
@@ -4189,170 +4193,170 @@
       </c>
     </row>
     <row r="22" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="C22" s="31"/>
-      <c r="D22" s="22"/>
+      <c r="C22" s="30"/>
+      <c r="D22" s="21"/>
     </row>
     <row r="23" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B23" s="23" t="b">
+      <c r="B23" s="22" t="b">
         <v>1</v>
       </c>
-      <c r="C23" s="29" t="s">
+      <c r="C23" s="28" t="s">
         <v>76</v>
       </c>
-      <c r="D23" s="28">
+      <c r="D23" s="27">
         <v>45728</v>
       </c>
-      <c r="E23" s="27" t="s">
+      <c r="E23" s="26" t="s">
         <v>178</v>
       </c>
-      <c r="F23" s="27" t="s">
+      <c r="F23" s="26" t="s">
         <v>183</v>
       </c>
     </row>
     <row r="24" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B24" s="23" t="b">
+      <c r="B24" s="22" t="b">
         <v>1</v>
       </c>
-      <c r="C24" s="29" t="s">
+      <c r="C24" s="28" t="s">
         <v>76</v>
       </c>
-      <c r="D24" s="28">
+      <c r="D24" s="27">
         <v>45742</v>
       </c>
-      <c r="E24" s="27" t="s">
+      <c r="E24" s="26" t="s">
         <v>178</v>
       </c>
-      <c r="F24" s="27" t="s">
+      <c r="F24" s="26" t="s">
         <v>184</v>
       </c>
     </row>
     <row r="25" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B25" s="23" t="b">
+      <c r="B25" s="22" t="b">
         <v>1</v>
       </c>
-      <c r="C25" s="29" t="s">
+      <c r="C25" s="28" t="s">
         <v>76</v>
       </c>
-      <c r="D25" s="28">
+      <c r="D25" s="27">
         <v>45756</v>
       </c>
-      <c r="E25" s="27" t="s">
+      <c r="E25" s="26" t="s">
         <v>178</v>
       </c>
-      <c r="F25" s="27" t="s">
+      <c r="F25" s="26" t="s">
         <v>185</v>
       </c>
     </row>
     <row r="26" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B26" s="23" t="b">
+      <c r="B26" s="22" t="b">
         <v>1</v>
       </c>
-      <c r="C26" s="29" t="s">
+      <c r="C26" s="28" t="s">
         <v>76</v>
       </c>
-      <c r="D26" s="28">
+      <c r="D26" s="27">
         <v>45770</v>
       </c>
-      <c r="E26" s="27" t="s">
+      <c r="E26" s="26" t="s">
         <v>177</v>
       </c>
-      <c r="F26" s="29" t="s">
+      <c r="F26" s="28" t="s">
         <v>189</v>
       </c>
     </row>
     <row r="27" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B27" s="23" t="b">
+      <c r="B27" s="22" t="b">
         <v>1</v>
       </c>
-      <c r="C27" s="29" t="s">
+      <c r="C27" s="28" t="s">
         <v>76</v>
       </c>
-      <c r="D27" s="28">
+      <c r="D27" s="27">
         <v>45784</v>
       </c>
-      <c r="E27" s="27" t="s">
+      <c r="E27" s="26" t="s">
         <v>178</v>
       </c>
-      <c r="F27" s="27" t="s">
+      <c r="F27" s="26" t="s">
         <v>186</v>
       </c>
     </row>
     <row r="28" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B28" s="23" t="b">
+      <c r="B28" s="22" t="b">
         <v>1</v>
       </c>
-      <c r="C28" s="29" t="s">
+      <c r="C28" s="28" t="s">
         <v>76</v>
       </c>
-      <c r="D28" s="28">
+      <c r="D28" s="27">
         <v>45798</v>
       </c>
-      <c r="E28" s="27" t="s">
+      <c r="E28" s="26" t="s">
         <v>178</v>
       </c>
-      <c r="F28" s="27" t="s">
+      <c r="F28" s="26" t="s">
         <v>187</v>
       </c>
     </row>
     <row r="29" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B29" s="19" t="b">
+      <c r="B29" s="22" t="b">
+        <v>1</v>
+      </c>
+      <c r="C29" s="28" t="s">
+        <v>76</v>
+      </c>
+      <c r="D29" s="27">
+        <v>45812</v>
+      </c>
+      <c r="E29" s="26" t="s">
+        <v>177</v>
+      </c>
+      <c r="F29" s="28" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="30" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="C30" s="30"/>
+    </row>
+    <row r="31" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B31" s="22" t="b">
+        <v>1</v>
+      </c>
+      <c r="C31" s="28" t="s">
+        <v>76</v>
+      </c>
+      <c r="D31" s="27">
+        <v>45764</v>
+      </c>
+      <c r="E31" s="26" t="s">
+        <v>147</v>
+      </c>
+      <c r="F31" s="26" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="32" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B32" s="22" t="b">
+        <v>1</v>
+      </c>
+      <c r="C32" s="28" t="s">
+        <v>76</v>
+      </c>
+      <c r="D32" s="27">
+        <v>45815</v>
+      </c>
+      <c r="E32" s="26" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="33" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B33" s="18" t="b">
         <v>0</v>
       </c>
-      <c r="C29" s="21" t="s">
+      <c r="C33" s="20" t="s">
         <v>76</v>
       </c>
-      <c r="D29" s="20">
-        <v>45812</v>
-      </c>
-      <c r="E29" s="17" t="s">
-        <v>177</v>
-      </c>
-      <c r="F29" s="21" t="s">
-        <v>215</v>
-      </c>
-    </row>
-    <row r="30" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="C30" s="31"/>
-    </row>
-    <row r="31" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B31" s="23" t="b">
-        <v>1</v>
-      </c>
-      <c r="C31" s="29" t="s">
-        <v>76</v>
-      </c>
-      <c r="D31" s="28">
-        <v>45764</v>
-      </c>
-      <c r="E31" s="27" t="s">
-        <v>147</v>
-      </c>
-      <c r="F31" s="27" t="s">
-        <v>190</v>
-      </c>
-    </row>
-    <row r="32" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B32" s="23" t="b">
-        <v>1</v>
-      </c>
-      <c r="C32" s="29" t="s">
-        <v>76</v>
-      </c>
-      <c r="D32" s="28">
-        <v>45815</v>
-      </c>
-      <c r="E32" s="27" t="s">
-        <v>216</v>
-      </c>
-    </row>
-    <row r="33" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B33" s="19" t="b">
-        <v>0</v>
-      </c>
-      <c r="C33" s="21" t="s">
-        <v>76</v>
-      </c>
-      <c r="D33" s="20">
+      <c r="D33" s="19">
         <v>45814</v>
       </c>
       <c r="E33" s="17" t="s">
@@ -4363,101 +4367,101 @@
       </c>
     </row>
     <row r="35" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B35" s="23" t="b">
+      <c r="B35" s="22" t="b">
         <v>1</v>
       </c>
-      <c r="C35" s="29" t="s">
+      <c r="C35" s="28" t="s">
         <v>78</v>
       </c>
-      <c r="D35" s="28">
+      <c r="D35" s="27">
         <v>45767</v>
       </c>
-      <c r="E35" s="27" t="s">
+      <c r="E35" s="26" t="s">
         <v>179</v>
       </c>
-      <c r="F35" s="27" t="s">
+      <c r="F35" s="26" t="s">
         <v>188</v>
       </c>
     </row>
     <row r="36" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B36" s="23" t="b">
+      <c r="B36" s="22" t="b">
         <v>1</v>
       </c>
-      <c r="C36" s="29" t="s">
+      <c r="C36" s="28" t="s">
         <v>78</v>
       </c>
-      <c r="D36" s="28">
+      <c r="D36" s="27">
         <v>45775</v>
       </c>
-      <c r="E36" s="27" t="s">
+      <c r="E36" s="26" t="s">
         <v>147</v>
       </c>
     </row>
     <row r="37" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B37" s="23" t="b">
+      <c r="B37" s="22" t="b">
         <v>1</v>
       </c>
-      <c r="C37" s="29" t="s">
+      <c r="C37" s="28" t="s">
         <v>78</v>
       </c>
-      <c r="D37" s="28">
+      <c r="D37" s="27">
         <v>45794</v>
       </c>
-      <c r="E37" s="27" t="s">
+      <c r="E37" s="26" t="s">
         <v>212</v>
       </c>
-      <c r="F37" s="27" t="s">
+      <c r="F37" s="26" t="s">
         <v>211</v>
       </c>
     </row>
     <row r="39" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B39" s="23" t="b">
+      <c r="B39" s="22" t="b">
         <v>1</v>
       </c>
-      <c r="C39" s="29" t="s">
+      <c r="C39" s="28" t="s">
         <v>79</v>
       </c>
-      <c r="D39" s="28">
+      <c r="D39" s="27">
         <v>45784</v>
       </c>
-      <c r="E39" s="27" t="s">
+      <c r="E39" s="26" t="s">
         <v>222</v>
       </c>
-      <c r="F39" s="27" t="s">
+      <c r="F39" s="26" t="s">
         <v>218</v>
       </c>
     </row>
     <row r="40" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B40" s="23" t="b">
+      <c r="B40" s="22" t="b">
         <v>1</v>
       </c>
-      <c r="C40" s="29" t="s">
+      <c r="C40" s="28" t="s">
         <v>79</v>
       </c>
-      <c r="D40" s="28">
+      <c r="D40" s="27">
         <v>45798</v>
       </c>
-      <c r="E40" s="27" t="s">
+      <c r="E40" s="26" t="s">
         <v>217</v>
       </c>
-      <c r="F40" s="27" t="s">
+      <c r="F40" s="26" t="s">
         <v>218</v>
       </c>
     </row>
     <row r="41" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B41" s="23" t="b">
+      <c r="B41" s="22" t="b">
         <v>1</v>
       </c>
-      <c r="C41" s="29" t="s">
+      <c r="C41" s="28" t="s">
         <v>79</v>
       </c>
-      <c r="D41" s="28">
+      <c r="D41" s="27">
         <v>45805</v>
       </c>
-      <c r="E41" s="27" t="s">
+      <c r="E41" s="26" t="s">
         <v>220</v>
       </c>
-      <c r="F41" s="27" t="s">
+      <c r="F41" s="26" t="s">
         <v>219</v>
       </c>
     </row>
@@ -4503,36 +4507,36 @@
       <c r="L2" s="81"/>
     </row>
     <row r="3" spans="2:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B3" s="34" t="s">
+      <c r="B3" s="33" t="s">
         <v>145</v>
       </c>
-      <c r="C3" s="35" t="s">
+      <c r="C3" s="34" t="s">
         <v>194</v>
       </c>
-      <c r="D3" s="36" t="s">
+      <c r="D3" s="35" t="s">
         <v>193</v>
       </c>
-      <c r="F3" s="34" t="s">
+      <c r="F3" s="33" t="s">
         <v>145</v>
       </c>
-      <c r="G3" s="35" t="s">
+      <c r="G3" s="34" t="s">
         <v>194</v>
       </c>
-      <c r="H3" s="36" t="s">
+      <c r="H3" s="35" t="s">
         <v>193</v>
       </c>
-      <c r="J3" s="34" t="s">
+      <c r="J3" s="33" t="s">
         <v>145</v>
       </c>
-      <c r="K3" s="35" t="s">
+      <c r="K3" s="34" t="s">
         <v>194</v>
       </c>
-      <c r="L3" s="36" t="s">
+      <c r="L3" s="35" t="s">
         <v>193</v>
       </c>
     </row>
     <row r="4" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B4" s="37" t="s">
+      <c r="B4" s="36" t="s">
         <v>130</v>
       </c>
       <c r="C4" s="14">
@@ -4541,14 +4545,14 @@
       <c r="D4" s="14">
         <v>4</v>
       </c>
-      <c r="F4" s="37" t="s">
+      <c r="F4" s="36" t="s">
         <v>76</v>
       </c>
       <c r="G4" s="14">
         <v>5</v>
       </c>
       <c r="H4" s="14"/>
-      <c r="J4" s="37" t="s">
+      <c r="J4" s="36" t="s">
         <v>196</v>
       </c>
       <c r="K4" s="14">
@@ -4557,7 +4561,7 @@
       <c r="L4" s="14"/>
     </row>
     <row r="5" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B5" s="38" t="s">
+      <c r="B5" s="37" t="s">
         <v>131</v>
       </c>
       <c r="C5" s="2">
@@ -4566,14 +4570,14 @@
       <c r="D5" s="2">
         <v>5</v>
       </c>
-      <c r="F5" s="38" t="s">
+      <c r="F5" s="37" t="s">
         <v>79</v>
       </c>
       <c r="G5" s="2">
         <v>4</v>
       </c>
       <c r="H5" s="2"/>
-      <c r="J5" s="38" t="s">
+      <c r="J5" s="37" t="s">
         <v>197</v>
       </c>
       <c r="K5" s="2">
@@ -4582,7 +4586,7 @@
       <c r="L5" s="2"/>
     </row>
     <row r="6" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B6" s="38" t="s">
+      <c r="B6" s="37" t="s">
         <v>132</v>
       </c>
       <c r="C6" s="2">
@@ -4591,14 +4595,16 @@
       <c r="D6" s="2">
         <v>4</v>
       </c>
-      <c r="F6" s="38" t="s">
+      <c r="F6" s="37" t="s">
         <v>77</v>
       </c>
       <c r="G6" s="2">
         <v>5</v>
       </c>
-      <c r="H6" s="2"/>
-      <c r="J6" s="38" t="s">
+      <c r="H6" s="2">
+        <v>4.5</v>
+      </c>
+      <c r="J6" s="37" t="s">
         <v>198</v>
       </c>
       <c r="K6" s="2">
@@ -4607,7 +4613,7 @@
       <c r="L6" s="2"/>
     </row>
     <row r="7" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B7" s="38" t="s">
+      <c r="B7" s="37" t="s">
         <v>133</v>
       </c>
       <c r="C7" s="2">
@@ -4616,14 +4622,14 @@
       <c r="D7" s="2">
         <v>4</v>
       </c>
-      <c r="F7" s="38" t="s">
+      <c r="F7" s="37" t="s">
         <v>78</v>
       </c>
       <c r="G7" s="2">
         <v>5</v>
       </c>
       <c r="H7" s="2"/>
-      <c r="J7" s="38" t="s">
+      <c r="J7" s="37" t="s">
         <v>199</v>
       </c>
       <c r="K7" s="2">
@@ -4632,7 +4638,7 @@
       <c r="L7" s="2"/>
     </row>
     <row r="8" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B8" s="38" t="s">
+      <c r="B8" s="37" t="s">
         <v>134</v>
       </c>
       <c r="C8" s="2">
@@ -4641,14 +4647,14 @@
       <c r="D8" s="2">
         <v>4.5</v>
       </c>
-      <c r="F8" s="38" t="s">
+      <c r="F8" s="37" t="s">
         <v>80</v>
       </c>
       <c r="G8" s="2">
         <v>11</v>
       </c>
       <c r="H8" s="2"/>
-      <c r="J8" s="38" t="s">
+      <c r="J8" s="37" t="s">
         <v>200</v>
       </c>
       <c r="K8" s="2">
@@ -4657,7 +4663,7 @@
       <c r="L8" s="2"/>
     </row>
     <row r="9" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B9" s="38" t="s">
+      <c r="B9" s="37" t="s">
         <v>135</v>
       </c>
       <c r="C9" s="2">
@@ -4666,10 +4672,10 @@
       <c r="D9" s="2">
         <v>5</v>
       </c>
-      <c r="F9" s="32"/>
+      <c r="F9" s="31"/>
       <c r="G9" s="1"/>
       <c r="H9" s="1"/>
-      <c r="J9" s="32"/>
+      <c r="J9" s="31"/>
       <c r="K9" s="1"/>
       <c r="L9" s="1"/>
     </row>
@@ -4679,7 +4685,7 @@
         <v>195</v>
       </c>
       <c r="C11" s="83"/>
-      <c r="D11" s="33">
+      <c r="D11" s="32">
         <f>(D4*C4+D5*C5+D6*C6+D7*C7+D8*C8+D9*C9)/30</f>
         <v>4.4333333333333336</v>
       </c>
@@ -4687,15 +4693,15 @@
         <v>195</v>
       </c>
       <c r="G11" s="83"/>
-      <c r="H11" s="33">
+      <c r="H11" s="32">
         <f>(H4*G4+H5*G5+H6*G6+H7*G7+H8*G8)/30</f>
-        <v>0</v>
+        <v>0.75</v>
       </c>
       <c r="J11" s="82" t="s">
         <v>195</v>
       </c>
       <c r="K11" s="83"/>
-      <c r="L11" s="33">
+      <c r="L11" s="32">
         <f>(L4*K4+L5*K5+L6*K6+L7*K7+L8*K8)/30</f>
         <v>0</v>
       </c>

</xml_diff>

<commit_message>
New points - 3rd project - POTEC
</commit_message>
<xml_diff>
--- a/IoT-points-schedule.xlsx
+++ b/IoT-points-schedule.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\dodo\Desktop\IoT-studies\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D13BF28C-868C-4D50-B8BC-1F66635A2391}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FC233770-1B09-40FE-8A9D-14C357B2668A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="25440" windowHeight="15390" activeTab="3" xr2:uid="{F85F5544-1FE8-4920-A5D4-192A98B113BD}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="25440" windowHeight="15390" activeTab="2" xr2:uid="{F85F5544-1FE8-4920-A5D4-192A98B113BD}"/>
   </bookViews>
   <sheets>
     <sheet name="II-semestr-25L" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="353" uniqueCount="225">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="344" uniqueCount="216">
   <si>
     <t>1. Krypto</t>
   </si>
@@ -365,18 +365,12 @@
     <t>LAB5</t>
   </si>
   <si>
-    <t>LAB6</t>
-  </si>
-  <si>
     <t>LAB7</t>
   </si>
   <si>
     <t>LAB8</t>
   </si>
   <si>
-    <t>LAB9</t>
-  </si>
-  <si>
     <t>LAB10</t>
   </si>
   <si>
@@ -386,9 +380,6 @@
     <t>LAB12</t>
   </si>
   <si>
-    <t>LAB13</t>
-  </si>
-  <si>
     <t>LAB14</t>
   </si>
   <si>
@@ -399,24 +390,6 @@
   </si>
   <si>
     <t>PROJ3</t>
-  </si>
-  <si>
-    <t>PROJ4</t>
-  </si>
-  <si>
-    <t>PROJ5</t>
-  </si>
-  <si>
-    <t>PROJ6</t>
-  </si>
-  <si>
-    <t>PROJ7</t>
-  </si>
-  <si>
-    <t>BONUS1</t>
-  </si>
-  <si>
-    <t>BONUS2</t>
   </si>
   <si>
     <t>Laby [14*2 pkt]</t>
@@ -1101,7 +1074,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="86">
+  <cellXfs count="85">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1248,58 +1221,76 @@
     <xf numFmtId="0" fontId="7" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="7" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="7" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="7" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="7" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="7" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="7" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="2" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="2" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="7" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="7" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="7" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="7" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="7" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="7" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
@@ -1308,24 +1299,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="2" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="2" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1363,9 +1336,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1729,7 +1699,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{03C86BD6-21E5-4E44-BF61-9A65607E6D85}">
-  <dimension ref="A1:S71"/>
+  <dimension ref="A1:S68"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="3.85546875" style="1" customWidth="1"/>
@@ -1756,85 +1726,85 @@
   <sheetData>
     <row r="1" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="2" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B2" s="57" t="s">
+      <c r="B2" s="54" t="s">
         <v>76</v>
       </c>
-      <c r="C2" s="58"/>
-      <c r="D2" s="58"/>
-      <c r="E2" s="58"/>
-      <c r="F2" s="58"/>
-      <c r="G2" s="58"/>
-      <c r="H2" s="58"/>
-      <c r="I2" s="58"/>
-      <c r="J2" s="58"/>
-      <c r="K2" s="58"/>
-      <c r="L2" s="58"/>
-      <c r="M2" s="58"/>
-      <c r="N2" s="58"/>
-      <c r="O2" s="58"/>
-      <c r="P2" s="59"/>
+      <c r="C2" s="55"/>
+      <c r="D2" s="55"/>
+      <c r="E2" s="55"/>
+      <c r="F2" s="55"/>
+      <c r="G2" s="55"/>
+      <c r="H2" s="55"/>
+      <c r="I2" s="55"/>
+      <c r="J2" s="55"/>
+      <c r="K2" s="55"/>
+      <c r="L2" s="55"/>
+      <c r="M2" s="55"/>
+      <c r="N2" s="55"/>
+      <c r="O2" s="55"/>
+      <c r="P2" s="56"/>
     </row>
     <row r="3" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B3" s="60"/>
-      <c r="C3" s="61"/>
-      <c r="D3" s="61"/>
-      <c r="E3" s="61"/>
-      <c r="F3" s="61"/>
-      <c r="G3" s="61"/>
-      <c r="H3" s="61"/>
-      <c r="I3" s="61"/>
-      <c r="J3" s="61"/>
-      <c r="K3" s="61"/>
-      <c r="L3" s="61"/>
-      <c r="M3" s="61"/>
-      <c r="N3" s="61"/>
-      <c r="O3" s="61"/>
-      <c r="P3" s="62"/>
+      <c r="B3" s="57"/>
+      <c r="C3" s="58"/>
+      <c r="D3" s="58"/>
+      <c r="E3" s="58"/>
+      <c r="F3" s="58"/>
+      <c r="G3" s="58"/>
+      <c r="H3" s="58"/>
+      <c r="I3" s="58"/>
+      <c r="J3" s="58"/>
+      <c r="K3" s="58"/>
+      <c r="L3" s="58"/>
+      <c r="M3" s="58"/>
+      <c r="N3" s="58"/>
+      <c r="O3" s="58"/>
+      <c r="P3" s="59"/>
       <c r="R3" s="12"/>
     </row>
     <row r="5" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B5" s="54" t="s">
+      <c r="B5" s="62" t="s">
         <v>83</v>
       </c>
-      <c r="C5" s="55"/>
-      <c r="D5" s="55"/>
-      <c r="E5" s="55"/>
-      <c r="F5" s="56"/>
-      <c r="H5" s="54" t="s">
+      <c r="C5" s="68"/>
+      <c r="D5" s="68"/>
+      <c r="E5" s="68"/>
+      <c r="F5" s="63"/>
+      <c r="H5" s="62" t="s">
         <v>82</v>
       </c>
-      <c r="I5" s="56"/>
-      <c r="K5" s="54" t="s">
+      <c r="I5" s="63"/>
+      <c r="K5" s="62" t="s">
         <v>8</v>
       </c>
-      <c r="L5" s="55"/>
-      <c r="M5" s="55"/>
-      <c r="N5" s="56"/>
+      <c r="L5" s="68"/>
+      <c r="M5" s="68"/>
+      <c r="N5" s="63"/>
       <c r="P5" s="4" t="s">
         <v>74</v>
       </c>
     </row>
     <row r="6" spans="1:19" ht="29.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B6" s="3" t="s">
-        <v>172</v>
+        <v>163</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>173</v>
+        <v>164</v>
       </c>
       <c r="D6" s="3" t="s">
-        <v>174</v>
+        <v>165</v>
       </c>
       <c r="E6" s="3" t="s">
-        <v>175</v>
+        <v>166</v>
       </c>
       <c r="F6" s="3" t="s">
-        <v>176</v>
+        <v>167</v>
       </c>
       <c r="H6" s="2" t="s">
-        <v>210</v>
+        <v>201</v>
       </c>
       <c r="I6" s="2" t="s">
-        <v>213</v>
+        <v>204</v>
       </c>
       <c r="K6" s="2" t="s">
         <v>24</v>
@@ -1885,37 +1855,37 @@
       <c r="P7" s="2"/>
     </row>
     <row r="9" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B9" s="63" t="s">
+      <c r="B9" s="64" t="s">
         <v>22</v>
       </c>
-      <c r="C9" s="63"/>
+      <c r="C9" s="64"/>
       <c r="E9" s="9" t="s">
         <v>67</v>
       </c>
-      <c r="G9" s="63" t="s">
+      <c r="G9" s="64" t="s">
         <v>87</v>
       </c>
-      <c r="H9" s="63"/>
+      <c r="H9" s="64"/>
     </row>
     <row r="10" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B10" s="46">
+      <c r="B10" s="65">
         <f>SUM(B7:F7,H7:I7,K7:N7,P7)</f>
         <v>41.6</v>
       </c>
-      <c r="C10" s="46"/>
-      <c r="E10" s="67"/>
-      <c r="G10" s="46">
+      <c r="C10" s="65"/>
+      <c r="E10" s="66"/>
+      <c r="G10" s="65">
         <f>66-SUM(B7:F7,H7:I7,K7:N7,P7)</f>
         <v>24.4</v>
       </c>
-      <c r="H10" s="46"/>
+      <c r="H10" s="65"/>
     </row>
     <row r="11" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B11" s="46"/>
-      <c r="C11" s="46"/>
-      <c r="E11" s="68"/>
-      <c r="G11" s="46"/>
-      <c r="H11" s="46"/>
+      <c r="B11" s="65"/>
+      <c r="C11" s="65"/>
+      <c r="E11" s="67"/>
+      <c r="G11" s="65"/>
+      <c r="H11" s="65"/>
     </row>
     <row r="12" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A12" s="6"/>
@@ -1960,36 +1930,36 @@
       <c r="H15" s="53"/>
     </row>
     <row r="17" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B17" s="66" t="s">
+      <c r="B17" s="47" t="s">
         <v>91</v>
       </c>
-      <c r="C17" s="66"/>
-      <c r="D17" s="66"/>
-      <c r="E17" s="66"/>
-      <c r="F17" s="66"/>
-      <c r="H17" s="54" t="s">
+      <c r="C17" s="47"/>
+      <c r="D17" s="47"/>
+      <c r="E17" s="47"/>
+      <c r="F17" s="47"/>
+      <c r="H17" s="62" t="s">
         <v>97</v>
       </c>
-      <c r="I17" s="55"/>
-      <c r="J17" s="56"/>
-      <c r="L17" s="63" t="s">
+      <c r="I17" s="68"/>
+      <c r="J17" s="63"/>
+      <c r="L17" s="64" t="s">
         <v>22</v>
       </c>
-      <c r="M17" s="63"/>
+      <c r="M17" s="64"/>
       <c r="O17" s="9" t="s">
         <v>67</v>
       </c>
-      <c r="P17" s="85"/>
+      <c r="P17" s="38"/>
     </row>
     <row r="18" spans="1:19" ht="48.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B18" s="3" t="s">
-        <v>156</v>
+        <v>147</v>
       </c>
       <c r="C18" s="3" t="s">
-        <v>157</v>
+        <v>148</v>
       </c>
       <c r="D18" s="3" t="s">
-        <v>158</v>
+        <v>149</v>
       </c>
       <c r="E18" s="3" t="s">
         <v>92</v>
@@ -2006,15 +1976,14 @@
       <c r="J18" s="3" t="s">
         <v>95</v>
       </c>
-      <c r="L18" s="46">
+      <c r="L18" s="65">
         <f>SUM(B19:F19,H19:J19)</f>
         <v>85</v>
       </c>
-      <c r="M18" s="46"/>
-      <c r="O18" s="47">
+      <c r="M18" s="65"/>
+      <c r="O18" s="69">
         <v>4.5</v>
       </c>
-      <c r="P18" s="84"/>
     </row>
     <row r="19" spans="1:19" x14ac:dyDescent="0.25">
       <c r="B19" s="2">
@@ -2041,10 +2010,9 @@
       <c r="J19" s="2">
         <v>19.5</v>
       </c>
-      <c r="L19" s="46"/>
-      <c r="M19" s="46"/>
-      <c r="O19" s="47"/>
-      <c r="P19" s="84"/>
+      <c r="L19" s="65"/>
+      <c r="M19" s="65"/>
+      <c r="O19" s="69"/>
     </row>
     <row r="21" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A21" s="6"/>
@@ -2082,10 +2050,10 @@
       <c r="J23" s="49"/>
       <c r="K23" s="49"/>
       <c r="L23" s="50"/>
-      <c r="N23" s="46" t="s">
-        <v>129</v>
-      </c>
-      <c r="O23" s="46"/>
+      <c r="N23" s="65" t="s">
+        <v>120</v>
+      </c>
+      <c r="O23" s="65"/>
       <c r="Q23" s="7"/>
       <c r="R23" s="7"/>
       <c r="S23" s="7"/>
@@ -2102,62 +2070,62 @@
       <c r="J24" s="52"/>
       <c r="K24" s="52"/>
       <c r="L24" s="53"/>
-      <c r="N24" s="46"/>
-      <c r="O24" s="46"/>
+      <c r="N24" s="65"/>
+      <c r="O24" s="65"/>
       <c r="Q24" s="7"/>
       <c r="R24" s="7"/>
       <c r="S24" s="7"/>
     </row>
     <row r="26" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B26" s="66" t="s">
+      <c r="B26" s="47" t="s">
         <v>8</v>
       </c>
-      <c r="C26" s="66"/>
-      <c r="D26" s="66"/>
-      <c r="F26" s="66" t="s">
-        <v>208</v>
-      </c>
-      <c r="G26" s="66"/>
-      <c r="H26" s="66"/>
-      <c r="I26" s="66"/>
+      <c r="C26" s="47"/>
+      <c r="D26" s="47"/>
+      <c r="F26" s="47" t="s">
+        <v>199</v>
+      </c>
+      <c r="G26" s="47"/>
+      <c r="H26" s="47"/>
+      <c r="I26" s="47"/>
       <c r="J26" s="7"/>
-      <c r="K26" s="54" t="s">
-        <v>128</v>
-      </c>
-      <c r="L26" s="56"/>
+      <c r="K26" s="62" t="s">
+        <v>119</v>
+      </c>
+      <c r="L26" s="63"/>
       <c r="N26" s="9" t="s">
         <v>67</v>
       </c>
     </row>
     <row r="27" spans="1:19" x14ac:dyDescent="0.25">
       <c r="B27" s="14" t="s">
-        <v>214</v>
+        <v>205</v>
       </c>
       <c r="C27" s="14" t="s">
-        <v>224</v>
+        <v>215</v>
       </c>
       <c r="D27" s="2" t="s">
         <v>11</v>
       </c>
       <c r="F27" s="2" t="s">
-        <v>204</v>
+        <v>195</v>
       </c>
       <c r="G27" s="2" t="s">
-        <v>206</v>
+        <v>197</v>
       </c>
       <c r="H27" s="2" t="s">
-        <v>205</v>
+        <v>196</v>
       </c>
       <c r="I27" s="2" t="s">
-        <v>207</v>
+        <v>198</v>
       </c>
       <c r="K27" s="14" t="s">
         <v>73</v>
       </c>
       <c r="L27" s="2" t="s">
-        <v>127</v>
-      </c>
-      <c r="N27" s="69">
+        <v>118</v>
+      </c>
+      <c r="N27" s="60">
         <f>(K29/30*0.4*5)+(B29/25*0.3*5)+(0.3*F29)</f>
         <v>4.2133333333333329</v>
       </c>
@@ -2188,26 +2156,26 @@
         <v>20</v>
       </c>
       <c r="L28" s="2"/>
-      <c r="N28" s="70"/>
+      <c r="N28" s="61"/>
     </row>
     <row r="29" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B29" s="71">
+      <c r="B29" s="46">
         <f>SUM(B28:C28)</f>
         <v>23</v>
       </c>
-      <c r="C29" s="71"/>
-      <c r="D29" s="71"/>
-      <c r="F29" s="71">
+      <c r="C29" s="46"/>
+      <c r="D29" s="46"/>
+      <c r="F29" s="46">
         <v>5</v>
       </c>
-      <c r="G29" s="71"/>
-      <c r="H29" s="71"/>
-      <c r="I29" s="71"/>
-      <c r="K29" s="71">
+      <c r="G29" s="46"/>
+      <c r="H29" s="46"/>
+      <c r="I29" s="46"/>
+      <c r="K29" s="46">
         <f>SUM(K28:L28)</f>
         <v>20</v>
       </c>
-      <c r="L29" s="71"/>
+      <c r="L29" s="46"/>
       <c r="N29" s="38"/>
     </row>
     <row r="31" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -2255,17 +2223,17 @@
       <c r="I34" s="53"/>
     </row>
     <row r="36" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B36" s="66" t="s">
+      <c r="B36" s="47" t="s">
         <v>98</v>
       </c>
-      <c r="C36" s="66"/>
+      <c r="C36" s="47"/>
       <c r="D36" s="7"/>
-      <c r="E36" s="54" t="s">
-        <v>144</v>
-      </c>
-      <c r="F36" s="55"/>
-      <c r="G36" s="55"/>
-      <c r="H36" s="56"/>
+      <c r="E36" s="62" t="s">
+        <v>135</v>
+      </c>
+      <c r="F36" s="68"/>
+      <c r="G36" s="68"/>
+      <c r="H36" s="63"/>
     </row>
     <row r="37" spans="2:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B37" s="2" t="s">
@@ -2296,26 +2264,26 @@
         <v>20</v>
       </c>
       <c r="E38" s="2">
-        <f>C57</f>
+        <f>C54</f>
         <v>25</v>
       </c>
       <c r="F38" s="2">
-        <f>G52</f>
-        <v>19</v>
+        <f>G46</f>
+        <v>29</v>
       </c>
       <c r="G38" s="2"/>
       <c r="H38" s="2"/>
       <c r="O38" s="7"/>
     </row>
     <row r="41" spans="2:15" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B41" s="64" t="s">
-        <v>126</v>
-      </c>
-      <c r="C41" s="65"/>
-      <c r="F41" s="46" t="s">
+      <c r="B41" s="70" t="s">
+        <v>117</v>
+      </c>
+      <c r="C41" s="71"/>
+      <c r="F41" s="65" t="s">
         <v>102</v>
       </c>
-      <c r="G41" s="46"/>
+      <c r="G41" s="65"/>
       <c r="I41" s="9" t="s">
         <v>22</v>
       </c>
@@ -2330,14 +2298,14 @@
         <v>2</v>
       </c>
       <c r="F42" s="2" t="s">
-        <v>117</v>
+        <v>114</v>
       </c>
       <c r="G42" s="2">
         <v>9</v>
       </c>
       <c r="I42" s="2">
         <f>SUM(B38:C38,E38:H38)</f>
-        <v>81</v>
+        <v>91</v>
       </c>
       <c r="J42" s="7"/>
       <c r="L42" s="7"/>
@@ -2350,7 +2318,7 @@
         <v>2</v>
       </c>
       <c r="F43" s="2" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="G43" s="2">
         <v>10</v>
@@ -2366,10 +2334,12 @@
         <v>3</v>
       </c>
       <c r="F44" s="2" t="s">
-        <v>119</v>
-      </c>
-      <c r="G44" s="2"/>
-      <c r="I44" s="63" t="s">
+        <v>116</v>
+      </c>
+      <c r="G44" s="2">
+        <v>10</v>
+      </c>
+      <c r="I44" s="64" t="s">
         <v>67</v>
       </c>
     </row>
@@ -2380,11 +2350,9 @@
       <c r="C45" s="2">
         <v>4</v>
       </c>
-      <c r="F45" s="2" t="s">
-        <v>120</v>
-      </c>
-      <c r="G45" s="2"/>
-      <c r="I45" s="63"/>
+      <c r="F45" s="84"/>
+      <c r="G45" s="84"/>
+      <c r="I45" s="64"/>
     </row>
     <row r="46" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B46" s="2" t="s">
@@ -2394,11 +2362,14 @@
         <v>4</v>
       </c>
       <c r="F46" s="2" t="s">
-        <v>121</v>
-      </c>
-      <c r="G46" s="2"/>
+        <v>48</v>
+      </c>
+      <c r="G46" s="2">
+        <f>SUM(G42:G44)</f>
+        <v>29</v>
+      </c>
       <c r="I46" s="13">
-        <v>4.5</v>
+        <v>5</v>
       </c>
     </row>
     <row r="47" spans="2:15" x14ac:dyDescent="0.25">
@@ -2406,20 +2377,18 @@
         <v>108</v>
       </c>
       <c r="C47" s="2"/>
-      <c r="F47" s="2" t="s">
-        <v>122</v>
-      </c>
-      <c r="G47" s="2"/>
+      <c r="F47" s="84"/>
+      <c r="G47" s="84"/>
     </row>
     <row r="48" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B48" s="2" t="s">
         <v>109</v>
       </c>
-      <c r="C48" s="2"/>
-      <c r="F48" s="2" t="s">
-        <v>123</v>
-      </c>
-      <c r="G48" s="2"/>
+      <c r="C48" s="2">
+        <v>2</v>
+      </c>
+      <c r="F48" s="84"/>
+      <c r="G48" s="84"/>
       <c r="I48" s="38"/>
     </row>
     <row r="49" spans="1:19" x14ac:dyDescent="0.25">
@@ -2429,321 +2398,265 @@
       <c r="C49" s="2">
         <v>2</v>
       </c>
-      <c r="F49" s="2" t="s">
-        <v>124</v>
-      </c>
-      <c r="G49" s="2"/>
+      <c r="F49" s="84"/>
+      <c r="G49" s="84"/>
     </row>
     <row r="50" spans="1:19" x14ac:dyDescent="0.25">
       <c r="B50" s="2" t="s">
         <v>111</v>
       </c>
-      <c r="C50" s="2"/>
-      <c r="F50" s="2" t="s">
-        <v>125</v>
-      </c>
-      <c r="G50" s="2"/>
+      <c r="C50" s="2">
+        <v>2</v>
+      </c>
+      <c r="F50" s="84"/>
+      <c r="G50" s="84"/>
     </row>
     <row r="51" spans="1:19" x14ac:dyDescent="0.25">
       <c r="B51" s="2" t="s">
         <v>112</v>
       </c>
       <c r="C51" s="2">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="52" spans="1:19" x14ac:dyDescent="0.25">
       <c r="B52" s="2" t="s">
         <v>113</v>
       </c>
-      <c r="C52" s="2">
-        <v>2</v>
-      </c>
-      <c r="F52" s="2" t="s">
-        <v>48</v>
-      </c>
-      <c r="G52" s="2">
-        <f>SUM(G42:G50)</f>
-        <v>19</v>
-      </c>
-    </row>
-    <row r="53" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B53" s="2" t="s">
-        <v>114</v>
-      </c>
-      <c r="C53" s="2">
-        <v>4</v>
-      </c>
+      <c r="C52" s="2"/>
     </row>
     <row r="54" spans="1:19" x14ac:dyDescent="0.25">
       <c r="B54" s="2" t="s">
-        <v>115</v>
-      </c>
-      <c r="C54" s="2"/>
-    </row>
-    <row r="55" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B55" s="2" t="s">
-        <v>116</v>
-      </c>
-      <c r="C55" s="2"/>
-    </row>
-    <row r="57" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B57" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="C57" s="2">
-        <f>SUM(C42:C55)</f>
+      <c r="C54" s="2">
+        <f>SUM(C42:C52)</f>
         <v>25</v>
       </c>
     </row>
-    <row r="59" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A59" s="6"/>
-      <c r="B59" s="6"/>
-      <c r="C59" s="6"/>
-      <c r="D59" s="6"/>
-      <c r="E59" s="6"/>
-      <c r="F59" s="6"/>
-      <c r="G59" s="6"/>
-      <c r="H59" s="6"/>
-      <c r="I59" s="6"/>
-      <c r="J59" s="6"/>
-      <c r="K59" s="6"/>
-      <c r="L59" s="6"/>
-      <c r="M59" s="6"/>
-      <c r="N59" s="6"/>
-      <c r="O59" s="6"/>
-      <c r="P59" s="6"/>
-      <c r="Q59" s="6"/>
-      <c r="R59" s="6"/>
-      <c r="S59" s="6"/>
-    </row>
-    <row r="60" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
-    <row r="61" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B61" s="57" t="s">
+    <row r="56" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A56" s="6"/>
+      <c r="B56" s="6"/>
+      <c r="C56" s="6"/>
+      <c r="D56" s="6"/>
+      <c r="E56" s="6"/>
+      <c r="F56" s="6"/>
+      <c r="G56" s="6"/>
+      <c r="H56" s="6"/>
+      <c r="I56" s="6"/>
+      <c r="J56" s="6"/>
+      <c r="K56" s="6"/>
+      <c r="L56" s="6"/>
+      <c r="M56" s="6"/>
+      <c r="N56" s="6"/>
+      <c r="O56" s="6"/>
+      <c r="P56" s="6"/>
+      <c r="Q56" s="6"/>
+      <c r="R56" s="6"/>
+      <c r="S56" s="6"/>
+    </row>
+    <row r="57" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="58" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B58" s="54" t="s">
         <v>80</v>
       </c>
-      <c r="C61" s="58"/>
-      <c r="D61" s="58"/>
-      <c r="E61" s="58"/>
-      <c r="F61" s="58"/>
-      <c r="G61" s="58"/>
-      <c r="H61" s="58"/>
-      <c r="I61" s="58"/>
-      <c r="J61" s="58"/>
-      <c r="K61" s="58"/>
-      <c r="L61" s="58"/>
-      <c r="M61" s="58"/>
-      <c r="N61" s="58"/>
-      <c r="O61" s="58"/>
-      <c r="P61" s="58"/>
-      <c r="Q61" s="58"/>
-      <c r="R61" s="58"/>
-      <c r="S61" s="59"/>
-    </row>
-    <row r="62" spans="1:19" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B62" s="60"/>
-      <c r="C62" s="61"/>
-      <c r="D62" s="61"/>
-      <c r="E62" s="61"/>
-      <c r="F62" s="61"/>
-      <c r="G62" s="61"/>
-      <c r="H62" s="61"/>
-      <c r="I62" s="61"/>
-      <c r="J62" s="61"/>
-      <c r="K62" s="61"/>
-      <c r="L62" s="61"/>
-      <c r="M62" s="61"/>
-      <c r="N62" s="61"/>
-      <c r="O62" s="61"/>
-      <c r="P62" s="61"/>
-      <c r="Q62" s="61"/>
-      <c r="R62" s="61"/>
-      <c r="S62" s="62"/>
-    </row>
-    <row r="64" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B64" s="66" t="s">
+      <c r="C58" s="55"/>
+      <c r="D58" s="55"/>
+      <c r="E58" s="55"/>
+      <c r="F58" s="55"/>
+      <c r="G58" s="55"/>
+      <c r="H58" s="55"/>
+      <c r="I58" s="55"/>
+      <c r="J58" s="55"/>
+      <c r="K58" s="55"/>
+      <c r="L58" s="55"/>
+      <c r="M58" s="55"/>
+      <c r="N58" s="55"/>
+      <c r="O58" s="55"/>
+      <c r="P58" s="55"/>
+      <c r="Q58" s="55"/>
+      <c r="R58" s="55"/>
+      <c r="S58" s="56"/>
+    </row>
+    <row r="59" spans="1:19" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B59" s="57"/>
+      <c r="C59" s="58"/>
+      <c r="D59" s="58"/>
+      <c r="E59" s="58"/>
+      <c r="F59" s="58"/>
+      <c r="G59" s="58"/>
+      <c r="H59" s="58"/>
+      <c r="I59" s="58"/>
+      <c r="J59" s="58"/>
+      <c r="K59" s="58"/>
+      <c r="L59" s="58"/>
+      <c r="M59" s="58"/>
+      <c r="N59" s="58"/>
+      <c r="O59" s="58"/>
+      <c r="P59" s="58"/>
+      <c r="Q59" s="58"/>
+      <c r="R59" s="58"/>
+      <c r="S59" s="59"/>
+    </row>
+    <row r="61" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="B61" s="47" t="s">
         <v>63</v>
       </c>
-      <c r="C64" s="66"/>
-      <c r="D64" s="66"/>
-      <c r="E64" s="66"/>
-      <c r="F64" s="66"/>
-      <c r="G64" s="66"/>
-      <c r="H64" s="66"/>
-      <c r="I64" s="66"/>
-      <c r="J64" s="66"/>
-      <c r="K64" s="66"/>
-      <c r="M64" s="66" t="s">
+      <c r="C61" s="47"/>
+      <c r="D61" s="47"/>
+      <c r="E61" s="47"/>
+      <c r="F61" s="47"/>
+      <c r="G61" s="47"/>
+      <c r="H61" s="47"/>
+      <c r="I61" s="47"/>
+      <c r="J61" s="47"/>
+      <c r="K61" s="47"/>
+      <c r="M61" s="47" t="s">
         <v>90</v>
       </c>
-      <c r="N64" s="66"/>
-      <c r="O64" s="66"/>
-      <c r="P64" s="66"/>
-      <c r="R64" s="66" t="s">
+      <c r="N61" s="47"/>
+      <c r="O61" s="47"/>
+      <c r="P61" s="47"/>
+      <c r="R61" s="47" t="s">
         <v>64</v>
       </c>
-      <c r="S64" s="66"/>
-    </row>
-    <row r="65" spans="2:19" x14ac:dyDescent="0.25">
-      <c r="B65" s="2" t="s">
+      <c r="S61" s="47"/>
+    </row>
+    <row r="62" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="B62" s="2" t="s">
         <v>49</v>
       </c>
-      <c r="C65" s="2" t="s">
+      <c r="C62" s="2" t="s">
         <v>51</v>
       </c>
-      <c r="D65" s="2" t="s">
+      <c r="D62" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="E65" s="2" t="s">
+      <c r="E62" s="2" t="s">
         <v>84</v>
       </c>
-      <c r="F65" s="2" t="s">
+      <c r="F62" s="2" t="s">
         <v>62</v>
       </c>
-      <c r="G65" s="2" t="s">
+      <c r="G62" s="2" t="s">
         <v>55</v>
       </c>
-      <c r="H65" s="2" t="s">
+      <c r="H62" s="2" t="s">
         <v>56</v>
       </c>
-      <c r="I65" s="2" t="s">
+      <c r="I62" s="2" t="s">
         <v>81</v>
       </c>
-      <c r="J65" s="2" t="s">
-        <v>209</v>
-      </c>
-      <c r="K65" s="2" t="s">
+      <c r="J62" s="2" t="s">
+        <v>200</v>
+      </c>
+      <c r="K62" s="2" t="s">
         <v>85</v>
       </c>
-      <c r="M65" s="2" t="s">
+      <c r="M62" s="2" t="s">
         <v>69</v>
       </c>
-      <c r="N65" s="2" t="s">
+      <c r="N62" s="2" t="s">
         <v>70</v>
       </c>
-      <c r="O65" s="2" t="s">
+      <c r="O62" s="2" t="s">
         <v>86</v>
       </c>
-      <c r="P65" s="2" t="s">
+      <c r="P62" s="2" t="s">
         <v>71</v>
       </c>
-      <c r="R65" s="2" t="s">
+      <c r="R62" s="2" t="s">
         <v>88</v>
       </c>
-      <c r="S65" s="2" t="s">
+      <c r="S62" s="2" t="s">
         <v>89</v>
       </c>
     </row>
-    <row r="66" spans="2:19" x14ac:dyDescent="0.25">
-      <c r="B66" s="2">
+    <row r="63" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="B63" s="2">
         <v>2</v>
       </c>
-      <c r="C66" s="2">
+      <c r="C63" s="2">
         <v>2</v>
       </c>
-      <c r="D66" s="2">
+      <c r="D63" s="2">
         <v>2</v>
       </c>
-      <c r="E66" s="2">
+      <c r="E63" s="2">
         <v>2</v>
       </c>
-      <c r="F66" s="2" t="s">
-        <v>191</v>
-      </c>
-      <c r="G66" s="2" t="s">
-        <v>191</v>
-      </c>
-      <c r="H66" s="2">
+      <c r="F63" s="2" t="s">
+        <v>182</v>
+      </c>
+      <c r="G63" s="2" t="s">
+        <v>182</v>
+      </c>
+      <c r="H63" s="2">
         <v>2</v>
       </c>
-      <c r="I66" s="2">
+      <c r="I63" s="2">
         <v>2</v>
       </c>
-      <c r="J66" s="2">
+      <c r="J63" s="2">
         <v>2</v>
       </c>
-      <c r="K66" s="2">
+      <c r="K63" s="2">
         <v>2</v>
       </c>
-      <c r="M66" s="2">
+      <c r="M63" s="2">
         <v>5</v>
       </c>
-      <c r="N66" s="2">
+      <c r="N63" s="2">
         <v>5</v>
       </c>
-      <c r="O66" s="2"/>
-      <c r="P66" s="2"/>
-      <c r="R66" s="2"/>
-      <c r="S66" s="2"/>
-    </row>
-    <row r="69" spans="2:19" x14ac:dyDescent="0.25">
-      <c r="B69" s="63" t="s">
+      <c r="O63" s="2"/>
+      <c r="P63" s="2"/>
+      <c r="R63" s="2"/>
+      <c r="S63" s="2"/>
+    </row>
+    <row r="66" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B66" s="64" t="s">
         <v>22</v>
       </c>
-      <c r="C69" s="63"/>
-      <c r="E69" s="9" t="s">
+      <c r="C66" s="64"/>
+      <c r="E66" s="9" t="s">
         <v>67</v>
       </c>
-      <c r="G69" s="63" t="s">
+      <c r="G66" s="64" t="s">
         <v>87</v>
       </c>
-      <c r="H69" s="63"/>
-      <c r="K69" s="39" t="s">
-        <v>223</v>
-      </c>
-    </row>
-    <row r="70" spans="2:19" x14ac:dyDescent="0.25">
-      <c r="B70" s="46">
-        <f>SUM(B66:K66,M66:P66,R66:S66,K70)</f>
+      <c r="H66" s="64"/>
+      <c r="K66" s="39" t="s">
+        <v>214</v>
+      </c>
+    </row>
+    <row r="67" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B67" s="65">
+        <f>SUM(B63:K63,M63:P63,R63:S63,K67)</f>
         <v>29</v>
       </c>
-      <c r="C70" s="46"/>
-      <c r="E70" s="47"/>
-      <c r="G70" s="46">
-        <f>50-SUM(B66:K66,M66:P66,R66:S66,K70)</f>
+      <c r="C67" s="65"/>
+      <c r="E67" s="69"/>
+      <c r="G67" s="65">
+        <f>50-SUM(B63:K63,M63:P63,R63:S63,K67)</f>
         <v>21</v>
       </c>
-      <c r="H70" s="46"/>
-      <c r="K70" s="46">
+      <c r="H67" s="65"/>
+      <c r="K67" s="65">
         <v>3</v>
       </c>
     </row>
-    <row r="71" spans="2:19" x14ac:dyDescent="0.25">
-      <c r="B71" s="46"/>
-      <c r="C71" s="46"/>
-      <c r="E71" s="47"/>
-      <c r="G71" s="46"/>
-      <c r="H71" s="46"/>
-      <c r="K71" s="46"/>
+    <row r="68" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B68" s="65"/>
+      <c r="C68" s="65"/>
+      <c r="E68" s="69"/>
+      <c r="G68" s="65"/>
+      <c r="H68" s="65"/>
+      <c r="K68" s="65"/>
     </row>
   </sheetData>
   <mergeCells count="40">
-    <mergeCell ref="K29:L29"/>
-    <mergeCell ref="R64:S64"/>
-    <mergeCell ref="B33:I34"/>
-    <mergeCell ref="B64:K64"/>
-    <mergeCell ref="B61:S62"/>
-    <mergeCell ref="M64:P64"/>
-    <mergeCell ref="F29:I29"/>
-    <mergeCell ref="B29:D29"/>
-    <mergeCell ref="N27:N28"/>
-    <mergeCell ref="F26:I26"/>
-    <mergeCell ref="K26:L26"/>
-    <mergeCell ref="B23:L24"/>
-    <mergeCell ref="B26:D26"/>
-    <mergeCell ref="B9:C9"/>
-    <mergeCell ref="B10:C11"/>
-    <mergeCell ref="L17:M17"/>
-    <mergeCell ref="E10:E11"/>
-    <mergeCell ref="G10:H11"/>
-    <mergeCell ref="B17:F17"/>
-    <mergeCell ref="H17:J17"/>
-    <mergeCell ref="E70:E71"/>
-    <mergeCell ref="B69:C69"/>
-    <mergeCell ref="B70:C71"/>
-    <mergeCell ref="G69:H69"/>
-    <mergeCell ref="G70:H71"/>
-    <mergeCell ref="K70:K71"/>
+    <mergeCell ref="K67:K68"/>
     <mergeCell ref="O18:O19"/>
     <mergeCell ref="B14:H15"/>
     <mergeCell ref="K5:N5"/>
@@ -2758,6 +2671,31 @@
     <mergeCell ref="B36:C36"/>
     <mergeCell ref="E36:H36"/>
     <mergeCell ref="G9:H9"/>
+    <mergeCell ref="E67:E68"/>
+    <mergeCell ref="B66:C66"/>
+    <mergeCell ref="B67:C68"/>
+    <mergeCell ref="G66:H66"/>
+    <mergeCell ref="G67:H68"/>
+    <mergeCell ref="B9:C9"/>
+    <mergeCell ref="B10:C11"/>
+    <mergeCell ref="L17:M17"/>
+    <mergeCell ref="E10:E11"/>
+    <mergeCell ref="G10:H11"/>
+    <mergeCell ref="B17:F17"/>
+    <mergeCell ref="H17:J17"/>
+    <mergeCell ref="N27:N28"/>
+    <mergeCell ref="F26:I26"/>
+    <mergeCell ref="K26:L26"/>
+    <mergeCell ref="B23:L24"/>
+    <mergeCell ref="B26:D26"/>
+    <mergeCell ref="K29:L29"/>
+    <mergeCell ref="R61:S61"/>
+    <mergeCell ref="B33:I34"/>
+    <mergeCell ref="B61:K61"/>
+    <mergeCell ref="B58:S59"/>
+    <mergeCell ref="M61:P61"/>
+    <mergeCell ref="F29:I29"/>
+    <mergeCell ref="B29:D29"/>
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2794,7 +2732,7 @@
     <row r="1" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="2" spans="1:19" x14ac:dyDescent="0.25">
       <c r="B2" s="72" t="s">
-        <v>130</v>
+        <v>121</v>
       </c>
       <c r="C2" s="73"/>
       <c r="D2" s="73"/>
@@ -2830,23 +2768,23 @@
       <c r="R3" s="12"/>
     </row>
     <row r="5" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B5" s="66" t="s">
+      <c r="B5" s="47" t="s">
         <v>18</v>
       </c>
-      <c r="C5" s="66"/>
-      <c r="D5" s="66"/>
-      <c r="E5" s="66"/>
-      <c r="F5" s="66"/>
-      <c r="G5" s="66"/>
+      <c r="C5" s="47"/>
+      <c r="D5" s="47"/>
+      <c r="E5" s="47"/>
+      <c r="F5" s="47"/>
+      <c r="G5" s="47"/>
       <c r="I5" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="K5" s="54" t="s">
+      <c r="K5" s="62" t="s">
         <v>8</v>
       </c>
-      <c r="L5" s="55"/>
-      <c r="M5" s="55"/>
-      <c r="N5" s="56"/>
+      <c r="L5" s="68"/>
+      <c r="M5" s="68"/>
+      <c r="N5" s="63"/>
       <c r="P5" s="4" t="s">
         <v>74</v>
       </c>
@@ -2928,28 +2866,28 @@
       </c>
     </row>
     <row r="9" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B9" s="63" t="s">
+      <c r="B9" s="64" t="s">
         <v>22</v>
       </c>
-      <c r="C9" s="63"/>
+      <c r="C9" s="64"/>
       <c r="E9" s="9" t="s">
         <v>67</v>
       </c>
     </row>
     <row r="10" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B10" s="46">
+      <c r="B10" s="65">
         <f>_xlfn.CEILING.MATH(SUM(B7:G7,I7,K7:N7,P7),1,1)</f>
         <v>110</v>
       </c>
-      <c r="C10" s="46"/>
-      <c r="E10" s="67">
+      <c r="C10" s="65"/>
+      <c r="E10" s="66">
         <v>4</v>
       </c>
     </row>
     <row r="11" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B11" s="46"/>
-      <c r="C11" s="46"/>
-      <c r="E11" s="68"/>
+      <c r="B11" s="65"/>
+      <c r="C11" s="65"/>
+      <c r="E11" s="67"/>
     </row>
     <row r="12" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A12" s="6"/>
@@ -2975,7 +2913,7 @@
     <row r="13" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="14" spans="1:19" x14ac:dyDescent="0.25">
       <c r="B14" s="72" t="s">
-        <v>131</v>
+        <v>122</v>
       </c>
       <c r="C14" s="73"/>
       <c r="D14" s="73"/>
@@ -2994,20 +2932,20 @@
       <c r="H15" s="77"/>
     </row>
     <row r="17" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B17" s="66" t="s">
+      <c r="B17" s="47" t="s">
         <v>12</v>
       </c>
-      <c r="C17" s="66"/>
-      <c r="D17" s="66"/>
-      <c r="F17" s="66" t="s">
+      <c r="C17" s="47"/>
+      <c r="D17" s="47"/>
+      <c r="F17" s="47" t="s">
         <v>8</v>
       </c>
-      <c r="G17" s="66"/>
-      <c r="H17" s="66"/>
-      <c r="J17" s="63" t="s">
+      <c r="G17" s="47"/>
+      <c r="H17" s="47"/>
+      <c r="J17" s="64" t="s">
         <v>22</v>
       </c>
-      <c r="K17" s="63"/>
+      <c r="K17" s="64"/>
       <c r="M17" s="9" t="s">
         <v>67</v>
       </c>
@@ -3031,12 +2969,12 @@
       <c r="H18" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="J18" s="46">
+      <c r="J18" s="65">
         <f>SUM(B19:D19,F19:H19)</f>
         <v>93</v>
       </c>
-      <c r="K18" s="46"/>
-      <c r="M18" s="47">
+      <c r="K18" s="65"/>
+      <c r="M18" s="69">
         <v>5</v>
       </c>
     </row>
@@ -3059,9 +2997,9 @@
       <c r="H19" s="2">
         <v>4</v>
       </c>
-      <c r="J19" s="46"/>
-      <c r="K19" s="46"/>
-      <c r="M19" s="47"/>
+      <c r="J19" s="65"/>
+      <c r="K19" s="65"/>
+      <c r="M19" s="69"/>
     </row>
     <row r="21" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A21" s="6"/>
@@ -3087,7 +3025,7 @@
     <row r="22" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="23" spans="1:19" x14ac:dyDescent="0.25">
       <c r="B23" s="72" t="s">
-        <v>132</v>
+        <v>123</v>
       </c>
       <c r="C23" s="73"/>
       <c r="D23" s="73"/>
@@ -3112,20 +3050,20 @@
       <c r="K24" s="77"/>
     </row>
     <row r="26" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B26" s="66" t="s">
+      <c r="B26" s="47" t="s">
         <v>17</v>
       </c>
-      <c r="C26" s="66"/>
-      <c r="E26" s="54" t="s">
+      <c r="C26" s="47"/>
+      <c r="E26" s="62" t="s">
         <v>21</v>
       </c>
-      <c r="F26" s="55"/>
-      <c r="G26" s="56"/>
-      <c r="I26" s="66" t="s">
+      <c r="F26" s="68"/>
+      <c r="G26" s="63"/>
+      <c r="I26" s="47" t="s">
         <v>20</v>
       </c>
-      <c r="J26" s="66"/>
-      <c r="K26" s="66"/>
+      <c r="J26" s="47"/>
+      <c r="K26" s="47"/>
       <c r="M26" s="10" t="s">
         <v>22</v>
       </c>
@@ -3165,7 +3103,7 @@
         <v>36</v>
       </c>
       <c r="N27" s="7"/>
-      <c r="O27" s="47">
+      <c r="O27" s="69">
         <v>4</v>
       </c>
       <c r="P27" s="8"/>
@@ -3197,7 +3135,7 @@
       </c>
       <c r="M28" s="78"/>
       <c r="N28" s="7"/>
-      <c r="O28" s="47"/>
+      <c r="O28" s="69"/>
       <c r="P28" s="8"/>
     </row>
     <row r="30" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -3224,7 +3162,7 @@
     <row r="31" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="32" spans="1:19" x14ac:dyDescent="0.25">
       <c r="B32" s="72" t="s">
-        <v>133</v>
+        <v>124</v>
       </c>
       <c r="C32" s="73"/>
       <c r="D32" s="73"/>
@@ -3245,17 +3183,17 @@
       <c r="I33" s="77"/>
     </row>
     <row r="35" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B35" s="66" t="s">
+      <c r="B35" s="47" t="s">
         <v>31</v>
       </c>
-      <c r="C35" s="66"/>
-      <c r="D35" s="66"/>
-      <c r="F35" s="66" t="s">
+      <c r="C35" s="47"/>
+      <c r="D35" s="47"/>
+      <c r="F35" s="47" t="s">
         <v>12</v>
       </c>
-      <c r="G35" s="66"/>
-      <c r="H35" s="66"/>
-      <c r="I35" s="66"/>
+      <c r="G35" s="47"/>
+      <c r="H35" s="47"/>
+      <c r="I35" s="47"/>
       <c r="N35" s="7"/>
       <c r="O35" s="7"/>
     </row>
@@ -3312,14 +3250,14 @@
       <c r="O37" s="7"/>
     </row>
     <row r="40" spans="2:15" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B40" s="64" t="s">
+      <c r="B40" s="70" t="s">
         <v>35</v>
       </c>
-      <c r="C40" s="65"/>
-      <c r="F40" s="46" t="s">
+      <c r="C40" s="71"/>
+      <c r="F40" s="65" t="s">
         <v>36</v>
       </c>
-      <c r="G40" s="46"/>
+      <c r="G40" s="65"/>
       <c r="I40" s="9" t="s">
         <v>22</v>
       </c>
@@ -3375,7 +3313,7 @@
       <c r="G43" s="2">
         <v>0.44</v>
       </c>
-      <c r="I43" s="63" t="s">
+      <c r="I43" s="64" t="s">
         <v>67</v>
       </c>
     </row>
@@ -3392,7 +3330,7 @@
       <c r="G44" s="2">
         <v>1</v>
       </c>
-      <c r="I44" s="63"/>
+      <c r="I44" s="64"/>
     </row>
     <row r="45" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B45" s="2" t="s">
@@ -3537,7 +3475,7 @@
     <row r="57" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="58" spans="1:19" x14ac:dyDescent="0.25">
       <c r="B58" s="72" t="s">
-        <v>134</v>
+        <v>125</v>
       </c>
       <c r="C58" s="73"/>
       <c r="D58" s="73"/>
@@ -3576,27 +3514,27 @@
       <c r="R59" s="77"/>
     </row>
     <row r="61" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B61" s="66" t="s">
+      <c r="B61" s="47" t="s">
         <v>63</v>
       </c>
-      <c r="C61" s="66"/>
-      <c r="D61" s="66"/>
-      <c r="E61" s="66"/>
-      <c r="F61" s="66"/>
-      <c r="G61" s="66"/>
-      <c r="H61" s="66"/>
-      <c r="I61" s="66"/>
-      <c r="J61" s="66"/>
-      <c r="K61" s="66"/>
-      <c r="M61" s="66" t="s">
+      <c r="C61" s="47"/>
+      <c r="D61" s="47"/>
+      <c r="E61" s="47"/>
+      <c r="F61" s="47"/>
+      <c r="G61" s="47"/>
+      <c r="H61" s="47"/>
+      <c r="I61" s="47"/>
+      <c r="J61" s="47"/>
+      <c r="K61" s="47"/>
+      <c r="M61" s="47" t="s">
         <v>68</v>
       </c>
-      <c r="N61" s="66"/>
-      <c r="O61" s="66"/>
-      <c r="Q61" s="66" t="s">
+      <c r="N61" s="47"/>
+      <c r="O61" s="47"/>
+      <c r="Q61" s="47" t="s">
         <v>64</v>
       </c>
-      <c r="R61" s="66"/>
+      <c r="R61" s="47"/>
     </row>
     <row r="62" spans="1:19" x14ac:dyDescent="0.25">
       <c r="B62" s="2" t="s">
@@ -3693,28 +3631,28 @@
       </c>
     </row>
     <row r="66" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B66" s="63" t="s">
+      <c r="B66" s="64" t="s">
         <v>22</v>
       </c>
-      <c r="C66" s="63"/>
+      <c r="C66" s="64"/>
       <c r="E66" s="9" t="s">
         <v>67</v>
       </c>
     </row>
     <row r="67" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B67" s="46">
+      <c r="B67" s="65">
         <f xml:space="preserve"> SUM(B63:K63,M63:O63,Q63:R63)</f>
         <v>85.5</v>
       </c>
-      <c r="C67" s="46"/>
-      <c r="E67" s="47">
+      <c r="C67" s="65"/>
+      <c r="E67" s="69">
         <v>4.5</v>
       </c>
     </row>
     <row r="68" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B68" s="46"/>
-      <c r="C68" s="46"/>
-      <c r="E68" s="47"/>
+      <c r="B68" s="65"/>
+      <c r="C68" s="65"/>
+      <c r="E68" s="69"/>
     </row>
     <row r="70" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A70" s="6"/>
@@ -3740,7 +3678,7 @@
     <row r="71" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="72" spans="1:19" x14ac:dyDescent="0.25">
       <c r="B72" s="72" t="s">
-        <v>135</v>
+        <v>126</v>
       </c>
       <c r="C72" s="73"/>
       <c r="D72" s="73"/>
@@ -3762,33 +3700,33 @@
     </row>
     <row r="75" spans="1:19" x14ac:dyDescent="0.25">
       <c r="B75" s="4" t="s">
-        <v>136</v>
+        <v>127</v>
       </c>
       <c r="C75" s="4" t="s">
-        <v>137</v>
+        <v>128</v>
       </c>
       <c r="D75" s="4" t="s">
-        <v>138</v>
+        <v>129</v>
       </c>
       <c r="E75" s="4" t="s">
-        <v>139</v>
+        <v>130</v>
       </c>
       <c r="F75" s="4" t="s">
-        <v>140</v>
+        <v>131</v>
       </c>
       <c r="G75" s="4" t="s">
-        <v>141</v>
+        <v>132</v>
       </c>
       <c r="H75" s="4" t="s">
-        <v>142</v>
+        <v>133</v>
       </c>
       <c r="I75" s="4" t="s">
-        <v>143</v>
-      </c>
-      <c r="K75" s="63" t="s">
+        <v>134</v>
+      </c>
+      <c r="K75" s="64" t="s">
         <v>22</v>
       </c>
-      <c r="L75" s="63"/>
+      <c r="L75" s="64"/>
       <c r="N75" s="9" t="s">
         <v>67</v>
       </c>
@@ -3818,11 +3756,11 @@
       <c r="I76" s="2">
         <v>5</v>
       </c>
-      <c r="K76" s="46">
+      <c r="K76" s="65">
         <f>SUM(B76:I76)</f>
         <v>96</v>
       </c>
-      <c r="L76" s="46"/>
+      <c r="L76" s="65"/>
       <c r="N76" s="13">
         <v>5</v>
       </c>
@@ -3850,6 +3788,30 @@
     </row>
   </sheetData>
   <mergeCells count="34">
+    <mergeCell ref="B2:P3"/>
+    <mergeCell ref="B5:G5"/>
+    <mergeCell ref="K5:N5"/>
+    <mergeCell ref="B9:C9"/>
+    <mergeCell ref="B10:C11"/>
+    <mergeCell ref="E10:E11"/>
+    <mergeCell ref="M27:M28"/>
+    <mergeCell ref="O27:O28"/>
+    <mergeCell ref="B14:H15"/>
+    <mergeCell ref="B17:D17"/>
+    <mergeCell ref="F17:H17"/>
+    <mergeCell ref="J17:K17"/>
+    <mergeCell ref="J18:K19"/>
+    <mergeCell ref="M18:M19"/>
+    <mergeCell ref="I43:I44"/>
+    <mergeCell ref="B23:K24"/>
+    <mergeCell ref="B26:C26"/>
+    <mergeCell ref="E26:G26"/>
+    <mergeCell ref="I26:K26"/>
+    <mergeCell ref="B32:I33"/>
+    <mergeCell ref="B35:D35"/>
+    <mergeCell ref="F35:I35"/>
+    <mergeCell ref="B40:C40"/>
+    <mergeCell ref="F40:G40"/>
     <mergeCell ref="B72:I73"/>
     <mergeCell ref="K75:L75"/>
     <mergeCell ref="K76:L76"/>
@@ -3860,30 +3822,6 @@
     <mergeCell ref="B66:C66"/>
     <mergeCell ref="B67:C68"/>
     <mergeCell ref="E67:E68"/>
-    <mergeCell ref="I43:I44"/>
-    <mergeCell ref="B23:K24"/>
-    <mergeCell ref="B26:C26"/>
-    <mergeCell ref="E26:G26"/>
-    <mergeCell ref="I26:K26"/>
-    <mergeCell ref="B32:I33"/>
-    <mergeCell ref="B35:D35"/>
-    <mergeCell ref="F35:I35"/>
-    <mergeCell ref="B40:C40"/>
-    <mergeCell ref="F40:G40"/>
-    <mergeCell ref="M27:M28"/>
-    <mergeCell ref="O27:O28"/>
-    <mergeCell ref="B14:H15"/>
-    <mergeCell ref="B17:D17"/>
-    <mergeCell ref="F17:H17"/>
-    <mergeCell ref="J17:K17"/>
-    <mergeCell ref="J18:K19"/>
-    <mergeCell ref="M18:M19"/>
-    <mergeCell ref="B2:P3"/>
-    <mergeCell ref="B5:G5"/>
-    <mergeCell ref="K5:N5"/>
-    <mergeCell ref="B9:C9"/>
-    <mergeCell ref="B10:C11"/>
-    <mergeCell ref="E10:E11"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
@@ -3904,16 +3842,16 @@
     <row r="1" spans="2:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="2" spans="2:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="C2" s="15" t="s">
-        <v>145</v>
+        <v>136</v>
       </c>
       <c r="D2" s="15" t="s">
-        <v>146</v>
+        <v>137</v>
       </c>
       <c r="E2" s="15" t="s">
-        <v>180</v>
+        <v>171</v>
       </c>
       <c r="F2" s="15" t="s">
-        <v>192</v>
+        <v>183</v>
       </c>
     </row>
     <row r="3" spans="2:6" x14ac:dyDescent="0.25">
@@ -3927,10 +3865,10 @@
         <v>45763</v>
       </c>
       <c r="E3" s="25" t="s">
-        <v>147</v>
+        <v>138</v>
       </c>
       <c r="F3" s="23" t="s">
-        <v>181</v>
+        <v>172</v>
       </c>
     </row>
     <row r="4" spans="2:6" x14ac:dyDescent="0.25">
@@ -3944,10 +3882,10 @@
         <v>45812</v>
       </c>
       <c r="E4" s="40" t="s">
-        <v>148</v>
+        <v>139</v>
       </c>
       <c r="F4" s="26" t="s">
-        <v>182</v>
+        <v>173</v>
       </c>
     </row>
     <row r="5" spans="2:6" x14ac:dyDescent="0.25">
@@ -3961,10 +3899,10 @@
         <v>45817</v>
       </c>
       <c r="E5" s="44" t="s">
-        <v>149</v>
+        <v>140</v>
       </c>
       <c r="F5" s="45" t="s">
-        <v>150</v>
+        <v>141</v>
       </c>
     </row>
     <row r="6" spans="2:6" x14ac:dyDescent="0.25">
@@ -3984,7 +3922,7 @@
         <v>103</v>
       </c>
       <c r="F7" s="26" t="s">
-        <v>151</v>
+        <v>142</v>
       </c>
     </row>
     <row r="8" spans="2:6" x14ac:dyDescent="0.25">
@@ -4001,7 +3939,7 @@
         <v>104</v>
       </c>
       <c r="F8" s="26" t="s">
-        <v>152</v>
+        <v>143</v>
       </c>
     </row>
     <row r="9" spans="2:6" x14ac:dyDescent="0.25">
@@ -4018,7 +3956,7 @@
         <v>105</v>
       </c>
       <c r="F9" s="26" t="s">
-        <v>153</v>
+        <v>144</v>
       </c>
     </row>
     <row r="10" spans="2:6" x14ac:dyDescent="0.25">
@@ -4035,7 +3973,7 @@
         <v>106</v>
       </c>
       <c r="F10" s="26" t="s">
-        <v>154</v>
+        <v>145</v>
       </c>
     </row>
     <row r="11" spans="2:6" x14ac:dyDescent="0.25">
@@ -4052,7 +3990,7 @@
         <v>107</v>
       </c>
       <c r="F11" s="26" t="s">
-        <v>155</v>
+        <v>146</v>
       </c>
     </row>
     <row r="12" spans="2:6" x14ac:dyDescent="0.25">
@@ -4063,7 +4001,7 @@
         <v>1</v>
       </c>
       <c r="C13" s="28" t="s">
-        <v>159</v>
+        <v>150</v>
       </c>
       <c r="D13" s="27">
         <v>45728</v>
@@ -4072,7 +4010,7 @@
         <v>84</v>
       </c>
       <c r="F13" s="26" t="s">
-        <v>160</v>
+        <v>151</v>
       </c>
     </row>
     <row r="14" spans="2:6" x14ac:dyDescent="0.25">
@@ -4080,16 +4018,16 @@
         <v>1</v>
       </c>
       <c r="C14" s="28" t="s">
-        <v>159</v>
+        <v>150</v>
       </c>
       <c r="D14" s="27">
         <v>45747</v>
       </c>
       <c r="E14" s="26" t="s">
-        <v>161</v>
+        <v>152</v>
       </c>
       <c r="F14" s="26" t="s">
-        <v>165</v>
+        <v>156</v>
       </c>
     </row>
     <row r="15" spans="2:6" x14ac:dyDescent="0.25">
@@ -4097,16 +4035,16 @@
         <v>1</v>
       </c>
       <c r="C15" s="28" t="s">
-        <v>159</v>
+        <v>150</v>
       </c>
       <c r="D15" s="27">
         <v>45784</v>
       </c>
       <c r="E15" s="26" t="s">
-        <v>162</v>
+        <v>153</v>
       </c>
       <c r="F15" s="26" t="s">
-        <v>163</v>
+        <v>154</v>
       </c>
     </row>
     <row r="16" spans="2:6" x14ac:dyDescent="0.25">
@@ -4114,7 +4052,7 @@
         <v>1</v>
       </c>
       <c r="C16" s="28" t="s">
-        <v>159</v>
+        <v>150</v>
       </c>
       <c r="D16" s="27">
         <v>45806</v>
@@ -4123,24 +4061,24 @@
         <v>85</v>
       </c>
       <c r="F16" s="26" t="s">
-        <v>164</v>
+        <v>155</v>
       </c>
     </row>
     <row r="17" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B17" s="18" t="b">
-        <v>0</v>
-      </c>
-      <c r="C17" s="20" t="s">
-        <v>159</v>
-      </c>
-      <c r="D17" s="19">
+      <c r="B17" s="22" t="b">
+        <v>1</v>
+      </c>
+      <c r="C17" s="28" t="s">
+        <v>150</v>
+      </c>
+      <c r="D17" s="27">
         <v>45817</v>
       </c>
-      <c r="E17" s="17" t="s">
-        <v>167</v>
-      </c>
-      <c r="F17" s="20" t="s">
-        <v>166</v>
+      <c r="E17" s="26" t="s">
+        <v>158</v>
+      </c>
+      <c r="F17" s="28" t="s">
+        <v>157</v>
       </c>
     </row>
     <row r="18" spans="2:6" x14ac:dyDescent="0.25">
@@ -4148,16 +4086,16 @@
         <v>0</v>
       </c>
       <c r="C18" s="20" t="s">
-        <v>159</v>
+        <v>150</v>
       </c>
       <c r="D18" s="19">
         <v>45819</v>
       </c>
       <c r="E18" s="17" t="s">
-        <v>169</v>
+        <v>160</v>
       </c>
       <c r="F18" s="20" t="s">
-        <v>168</v>
+        <v>159</v>
       </c>
     </row>
     <row r="19" spans="2:6" x14ac:dyDescent="0.25">
@@ -4169,13 +4107,13 @@
         <v>0</v>
       </c>
       <c r="C20" s="20" t="s">
-        <v>159</v>
+        <v>150</v>
       </c>
       <c r="D20" s="19">
         <v>45820</v>
       </c>
       <c r="E20" s="17" t="s">
-        <v>170</v>
+        <v>161</v>
       </c>
     </row>
     <row r="21" spans="2:6" x14ac:dyDescent="0.25">
@@ -4183,13 +4121,13 @@
         <v>0</v>
       </c>
       <c r="C21" s="20" t="s">
-        <v>159</v>
+        <v>150</v>
       </c>
       <c r="D21" s="19">
         <v>45820</v>
       </c>
       <c r="E21" s="17" t="s">
-        <v>171</v>
+        <v>162</v>
       </c>
     </row>
     <row r="22" spans="2:6" x14ac:dyDescent="0.25">
@@ -4207,10 +4145,10 @@
         <v>45728</v>
       </c>
       <c r="E23" s="26" t="s">
-        <v>178</v>
+        <v>169</v>
       </c>
       <c r="F23" s="26" t="s">
-        <v>183</v>
+        <v>174</v>
       </c>
     </row>
     <row r="24" spans="2:6" x14ac:dyDescent="0.25">
@@ -4224,10 +4162,10 @@
         <v>45742</v>
       </c>
       <c r="E24" s="26" t="s">
-        <v>178</v>
+        <v>169</v>
       </c>
       <c r="F24" s="26" t="s">
-        <v>184</v>
+        <v>175</v>
       </c>
     </row>
     <row r="25" spans="2:6" x14ac:dyDescent="0.25">
@@ -4241,10 +4179,10 @@
         <v>45756</v>
       </c>
       <c r="E25" s="26" t="s">
-        <v>178</v>
+        <v>169</v>
       </c>
       <c r="F25" s="26" t="s">
-        <v>185</v>
+        <v>176</v>
       </c>
     </row>
     <row r="26" spans="2:6" x14ac:dyDescent="0.25">
@@ -4258,10 +4196,10 @@
         <v>45770</v>
       </c>
       <c r="E26" s="26" t="s">
-        <v>177</v>
+        <v>168</v>
       </c>
       <c r="F26" s="28" t="s">
-        <v>189</v>
+        <v>180</v>
       </c>
     </row>
     <row r="27" spans="2:6" x14ac:dyDescent="0.25">
@@ -4275,10 +4213,10 @@
         <v>45784</v>
       </c>
       <c r="E27" s="26" t="s">
-        <v>178</v>
+        <v>169</v>
       </c>
       <c r="F27" s="26" t="s">
-        <v>186</v>
+        <v>177</v>
       </c>
     </row>
     <row r="28" spans="2:6" x14ac:dyDescent="0.25">
@@ -4292,10 +4230,10 @@
         <v>45798</v>
       </c>
       <c r="E28" s="26" t="s">
+        <v>169</v>
+      </c>
+      <c r="F28" s="26" t="s">
         <v>178</v>
-      </c>
-      <c r="F28" s="26" t="s">
-        <v>187</v>
       </c>
     </row>
     <row r="29" spans="2:6" x14ac:dyDescent="0.25">
@@ -4309,10 +4247,10 @@
         <v>45812</v>
       </c>
       <c r="E29" s="26" t="s">
-        <v>177</v>
+        <v>168</v>
       </c>
       <c r="F29" s="28" t="s">
-        <v>215</v>
+        <v>206</v>
       </c>
     </row>
     <row r="30" spans="2:6" x14ac:dyDescent="0.25">
@@ -4329,10 +4267,10 @@
         <v>45764</v>
       </c>
       <c r="E31" s="26" t="s">
-        <v>147</v>
+        <v>138</v>
       </c>
       <c r="F31" s="26" t="s">
-        <v>190</v>
+        <v>181</v>
       </c>
     </row>
     <row r="32" spans="2:6" x14ac:dyDescent="0.25">
@@ -4346,24 +4284,24 @@
         <v>45815</v>
       </c>
       <c r="E32" s="26" t="s">
-        <v>216</v>
+        <v>207</v>
       </c>
     </row>
     <row r="33" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B33" s="18" t="b">
-        <v>0</v>
-      </c>
-      <c r="C33" s="20" t="s">
+      <c r="B33" s="22" t="b">
+        <v>1</v>
+      </c>
+      <c r="C33" s="28" t="s">
         <v>76</v>
       </c>
-      <c r="D33" s="19">
+      <c r="D33" s="27">
         <v>45814</v>
       </c>
-      <c r="E33" s="17" t="s">
-        <v>148</v>
-      </c>
-      <c r="F33" s="17" t="s">
-        <v>221</v>
+      <c r="E33" s="26" t="s">
+        <v>139</v>
+      </c>
+      <c r="F33" s="26" t="s">
+        <v>212</v>
       </c>
     </row>
     <row r="35" spans="2:6" x14ac:dyDescent="0.25">
@@ -4377,10 +4315,10 @@
         <v>45767</v>
       </c>
       <c r="E35" s="26" t="s">
+        <v>170</v>
+      </c>
+      <c r="F35" s="26" t="s">
         <v>179</v>
-      </c>
-      <c r="F35" s="26" t="s">
-        <v>188</v>
       </c>
     </row>
     <row r="36" spans="2:6" x14ac:dyDescent="0.25">
@@ -4394,7 +4332,7 @@
         <v>45775</v>
       </c>
       <c r="E36" s="26" t="s">
-        <v>147</v>
+        <v>138</v>
       </c>
     </row>
     <row r="37" spans="2:6" x14ac:dyDescent="0.25">
@@ -4408,10 +4346,10 @@
         <v>45794</v>
       </c>
       <c r="E37" s="26" t="s">
-        <v>212</v>
+        <v>203</v>
       </c>
       <c r="F37" s="26" t="s">
-        <v>211</v>
+        <v>202</v>
       </c>
     </row>
     <row r="39" spans="2:6" x14ac:dyDescent="0.25">
@@ -4425,10 +4363,10 @@
         <v>45784</v>
       </c>
       <c r="E39" s="26" t="s">
-        <v>222</v>
+        <v>213</v>
       </c>
       <c r="F39" s="26" t="s">
-        <v>218</v>
+        <v>209</v>
       </c>
     </row>
     <row r="40" spans="2:6" x14ac:dyDescent="0.25">
@@ -4442,10 +4380,10 @@
         <v>45798</v>
       </c>
       <c r="E40" s="26" t="s">
-        <v>217</v>
+        <v>208</v>
       </c>
       <c r="F40" s="26" t="s">
-        <v>218</v>
+        <v>209</v>
       </c>
     </row>
     <row r="41" spans="2:6" x14ac:dyDescent="0.25">
@@ -4459,10 +4397,10 @@
         <v>45805</v>
       </c>
       <c r="E41" s="26" t="s">
-        <v>220</v>
+        <v>211</v>
       </c>
       <c r="F41" s="26" t="s">
-        <v>219</v>
+        <v>210</v>
       </c>
     </row>
   </sheetData>
@@ -4491,53 +4429,53 @@
     <row r="1" spans="2:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="2" spans="2:12" ht="23.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B2" s="79" t="s">
-        <v>201</v>
+        <v>192</v>
       </c>
       <c r="C2" s="80"/>
       <c r="D2" s="81"/>
       <c r="F2" s="79" t="s">
-        <v>202</v>
+        <v>193</v>
       </c>
       <c r="G2" s="80"/>
       <c r="H2" s="81"/>
       <c r="J2" s="79" t="s">
-        <v>203</v>
+        <v>194</v>
       </c>
       <c r="K2" s="80"/>
       <c r="L2" s="81"/>
     </row>
     <row r="3" spans="2:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B3" s="33" t="s">
-        <v>145</v>
+        <v>136</v>
       </c>
       <c r="C3" s="34" t="s">
-        <v>194</v>
+        <v>185</v>
       </c>
       <c r="D3" s="35" t="s">
-        <v>193</v>
+        <v>184</v>
       </c>
       <c r="F3" s="33" t="s">
-        <v>145</v>
+        <v>136</v>
       </c>
       <c r="G3" s="34" t="s">
-        <v>194</v>
+        <v>185</v>
       </c>
       <c r="H3" s="35" t="s">
-        <v>193</v>
+        <v>184</v>
       </c>
       <c r="J3" s="33" t="s">
-        <v>145</v>
+        <v>136</v>
       </c>
       <c r="K3" s="34" t="s">
-        <v>194</v>
+        <v>185</v>
       </c>
       <c r="L3" s="35" t="s">
-        <v>193</v>
+        <v>184</v>
       </c>
     </row>
     <row r="4" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B4" s="36" t="s">
-        <v>130</v>
+        <v>121</v>
       </c>
       <c r="C4" s="14">
         <v>4</v>
@@ -4553,7 +4491,7 @@
       </c>
       <c r="H4" s="14"/>
       <c r="J4" s="36" t="s">
-        <v>196</v>
+        <v>187</v>
       </c>
       <c r="K4" s="14">
         <v>4</v>
@@ -4562,7 +4500,7 @@
     </row>
     <row r="5" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B5" s="37" t="s">
-        <v>131</v>
+        <v>122</v>
       </c>
       <c r="C5" s="2">
         <v>6</v>
@@ -4578,7 +4516,7 @@
       </c>
       <c r="H5" s="2"/>
       <c r="J5" s="37" t="s">
-        <v>197</v>
+        <v>188</v>
       </c>
       <c r="K5" s="2">
         <v>4</v>
@@ -4587,7 +4525,7 @@
     </row>
     <row r="6" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B6" s="37" t="s">
-        <v>132</v>
+        <v>123</v>
       </c>
       <c r="C6" s="2">
         <v>4</v>
@@ -4605,7 +4543,7 @@
         <v>4.5</v>
       </c>
       <c r="J6" s="37" t="s">
-        <v>198</v>
+        <v>189</v>
       </c>
       <c r="K6" s="2">
         <v>5</v>
@@ -4614,7 +4552,7 @@
     </row>
     <row r="7" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B7" s="37" t="s">
-        <v>133</v>
+        <v>124</v>
       </c>
       <c r="C7" s="2">
         <v>4</v>
@@ -4628,9 +4566,11 @@
       <c r="G7" s="2">
         <v>5</v>
       </c>
-      <c r="H7" s="2"/>
+      <c r="H7" s="2">
+        <v>5</v>
+      </c>
       <c r="J7" s="37" t="s">
-        <v>199</v>
+        <v>190</v>
       </c>
       <c r="K7" s="2">
         <v>5</v>
@@ -4639,7 +4579,7 @@
     </row>
     <row r="8" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B8" s="37" t="s">
-        <v>134</v>
+        <v>125</v>
       </c>
       <c r="C8" s="2">
         <v>10</v>
@@ -4655,7 +4595,7 @@
       </c>
       <c r="H8" s="2"/>
       <c r="J8" s="37" t="s">
-        <v>200</v>
+        <v>191</v>
       </c>
       <c r="K8" s="2">
         <v>12</v>
@@ -4664,7 +4604,7 @@
     </row>
     <row r="9" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B9" s="37" t="s">
-        <v>135</v>
+        <v>126</v>
       </c>
       <c r="C9" s="2">
         <v>2</v>
@@ -4682,7 +4622,7 @@
     <row r="10" spans="2:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="11" spans="2:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B11" s="82" t="s">
-        <v>195</v>
+        <v>186</v>
       </c>
       <c r="C11" s="83"/>
       <c r="D11" s="32">
@@ -4690,15 +4630,15 @@
         <v>4.4333333333333336</v>
       </c>
       <c r="F11" s="82" t="s">
-        <v>195</v>
+        <v>186</v>
       </c>
       <c r="G11" s="83"/>
       <c r="H11" s="32">
         <f>(H4*G4+H5*G5+H6*G6+H7*G7+H8*G8)/30</f>
-        <v>0.75</v>
+        <v>1.5833333333333333</v>
       </c>
       <c r="J11" s="82" t="s">
-        <v>195</v>
+        <v>186</v>
       </c>
       <c r="K11" s="83"/>
       <c r="L11" s="32">

</xml_diff>

<commit_message>
New points - PBL2 -> passed
</commit_message>
<xml_diff>
--- a/IoT-points-schedule.xlsx
+++ b/IoT-points-schedule.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\dodo\Desktop\IoT-studies\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FC233770-1B09-40FE-8A9D-14C357B2668A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BF0EE2A9-3B2E-4037-8903-BB049E272633}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="25440" windowHeight="15390" activeTab="2" xr2:uid="{F85F5544-1FE8-4920-A5D4-192A98B113BD}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="25440" windowHeight="15390" xr2:uid="{F85F5544-1FE8-4920-A5D4-192A98B113BD}"/>
   </bookViews>
   <sheets>
     <sheet name="II-semestr-25L" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="344" uniqueCount="216">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="343" uniqueCount="216">
   <si>
     <t>1. Krypto</t>
   </si>
@@ -769,7 +769,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="10">
+  <fills count="9">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -785,12 +785,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="3" tint="0.89999084444715716"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.59999389629810485"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1074,7 +1068,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="85">
+  <cellXfs count="80">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1143,32 +1137,32 @@
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFill="1" applyBorder="1">
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1">
       <extLst>
         <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
           <xfpb:xfComplement i="0"/>
         </ext>
       </extLst>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="6" borderId="12" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="0" fillId="5" borderId="12" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="14" fontId="0" fillId="6" borderId="12" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="14" fontId="0" fillId="5" borderId="12" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="0" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -1178,89 +1172,116 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="19" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="6" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="14" fontId="0" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="14" fontId="0" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
       <extLst>
         <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
           <xfpb:xfComplement i="0"/>
         </ext>
       </extLst>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="165" fontId="7" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="7" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="14" fontId="7" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="14" fontId="7" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="7" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="7" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="7" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="7" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="7" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="7" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="2" fontId="2" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1269,64 +1290,19 @@
     <xf numFmtId="2" fontId="2" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="7" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="7" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="7" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1335,8 +1311,11 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1726,60 +1705,60 @@
   <sheetData>
     <row r="1" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="2" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B2" s="54" t="s">
+      <c r="B2" s="57" t="s">
         <v>76</v>
       </c>
-      <c r="C2" s="55"/>
-      <c r="D2" s="55"/>
-      <c r="E2" s="55"/>
-      <c r="F2" s="55"/>
-      <c r="G2" s="55"/>
-      <c r="H2" s="55"/>
-      <c r="I2" s="55"/>
-      <c r="J2" s="55"/>
-      <c r="K2" s="55"/>
-      <c r="L2" s="55"/>
-      <c r="M2" s="55"/>
-      <c r="N2" s="55"/>
-      <c r="O2" s="55"/>
-      <c r="P2" s="56"/>
+      <c r="C2" s="58"/>
+      <c r="D2" s="58"/>
+      <c r="E2" s="58"/>
+      <c r="F2" s="58"/>
+      <c r="G2" s="58"/>
+      <c r="H2" s="58"/>
+      <c r="I2" s="58"/>
+      <c r="J2" s="58"/>
+      <c r="K2" s="58"/>
+      <c r="L2" s="58"/>
+      <c r="M2" s="58"/>
+      <c r="N2" s="58"/>
+      <c r="O2" s="58"/>
+      <c r="P2" s="59"/>
     </row>
     <row r="3" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B3" s="57"/>
-      <c r="C3" s="58"/>
-      <c r="D3" s="58"/>
-      <c r="E3" s="58"/>
-      <c r="F3" s="58"/>
-      <c r="G3" s="58"/>
-      <c r="H3" s="58"/>
-      <c r="I3" s="58"/>
-      <c r="J3" s="58"/>
-      <c r="K3" s="58"/>
-      <c r="L3" s="58"/>
-      <c r="M3" s="58"/>
-      <c r="N3" s="58"/>
-      <c r="O3" s="58"/>
-      <c r="P3" s="59"/>
+      <c r="B3" s="60"/>
+      <c r="C3" s="61"/>
+      <c r="D3" s="61"/>
+      <c r="E3" s="61"/>
+      <c r="F3" s="61"/>
+      <c r="G3" s="61"/>
+      <c r="H3" s="61"/>
+      <c r="I3" s="61"/>
+      <c r="J3" s="61"/>
+      <c r="K3" s="61"/>
+      <c r="L3" s="61"/>
+      <c r="M3" s="61"/>
+      <c r="N3" s="61"/>
+      <c r="O3" s="61"/>
+      <c r="P3" s="62"/>
       <c r="R3" s="12"/>
     </row>
     <row r="5" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B5" s="62" t="s">
+      <c r="B5" s="54" t="s">
         <v>83</v>
       </c>
-      <c r="C5" s="68"/>
-      <c r="D5" s="68"/>
-      <c r="E5" s="68"/>
-      <c r="F5" s="63"/>
-      <c r="H5" s="62" t="s">
+      <c r="C5" s="55"/>
+      <c r="D5" s="55"/>
+      <c r="E5" s="55"/>
+      <c r="F5" s="56"/>
+      <c r="H5" s="54" t="s">
         <v>82</v>
       </c>
-      <c r="I5" s="63"/>
-      <c r="K5" s="62" t="s">
+      <c r="I5" s="56"/>
+      <c r="K5" s="54" t="s">
         <v>8</v>
       </c>
-      <c r="L5" s="68"/>
-      <c r="M5" s="68"/>
-      <c r="N5" s="63"/>
+      <c r="L5" s="55"/>
+      <c r="M5" s="55"/>
+      <c r="N5" s="56"/>
       <c r="P5" s="4" t="s">
         <v>74</v>
       </c>
@@ -1855,37 +1834,37 @@
       <c r="P7" s="2"/>
     </row>
     <row r="9" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B9" s="64" t="s">
+      <c r="B9" s="63" t="s">
         <v>22</v>
       </c>
-      <c r="C9" s="64"/>
+      <c r="C9" s="63"/>
       <c r="E9" s="9" t="s">
         <v>67</v>
       </c>
-      <c r="G9" s="64" t="s">
+      <c r="G9" s="63" t="s">
         <v>87</v>
       </c>
-      <c r="H9" s="64"/>
+      <c r="H9" s="63"/>
     </row>
     <row r="10" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B10" s="65">
+      <c r="B10" s="46">
         <f>SUM(B7:F7,H7:I7,K7:N7,P7)</f>
         <v>41.6</v>
       </c>
-      <c r="C10" s="65"/>
-      <c r="E10" s="66"/>
-      <c r="G10" s="65">
+      <c r="C10" s="46"/>
+      <c r="E10" s="67"/>
+      <c r="G10" s="46">
         <f>66-SUM(B7:F7,H7:I7,K7:N7,P7)</f>
         <v>24.4</v>
       </c>
-      <c r="H10" s="65"/>
+      <c r="H10" s="46"/>
     </row>
     <row r="11" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B11" s="65"/>
-      <c r="C11" s="65"/>
-      <c r="E11" s="67"/>
-      <c r="G11" s="65"/>
-      <c r="H11" s="65"/>
+      <c r="B11" s="46"/>
+      <c r="C11" s="46"/>
+      <c r="E11" s="68"/>
+      <c r="G11" s="46"/>
+      <c r="H11" s="46"/>
     </row>
     <row r="12" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A12" s="6"/>
@@ -1930,22 +1909,22 @@
       <c r="H15" s="53"/>
     </row>
     <row r="17" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B17" s="47" t="s">
+      <c r="B17" s="66" t="s">
         <v>91</v>
       </c>
-      <c r="C17" s="47"/>
-      <c r="D17" s="47"/>
-      <c r="E17" s="47"/>
-      <c r="F17" s="47"/>
-      <c r="H17" s="62" t="s">
+      <c r="C17" s="66"/>
+      <c r="D17" s="66"/>
+      <c r="E17" s="66"/>
+      <c r="F17" s="66"/>
+      <c r="H17" s="54" t="s">
         <v>97</v>
       </c>
-      <c r="I17" s="68"/>
-      <c r="J17" s="63"/>
-      <c r="L17" s="64" t="s">
+      <c r="I17" s="55"/>
+      <c r="J17" s="56"/>
+      <c r="L17" s="63" t="s">
         <v>22</v>
       </c>
-      <c r="M17" s="64"/>
+      <c r="M17" s="63"/>
       <c r="O17" s="9" t="s">
         <v>67</v>
       </c>
@@ -1976,12 +1955,12 @@
       <c r="J18" s="3" t="s">
         <v>95</v>
       </c>
-      <c r="L18" s="65">
+      <c r="L18" s="46">
         <f>SUM(B19:F19,H19:J19)</f>
         <v>85</v>
       </c>
-      <c r="M18" s="65"/>
-      <c r="O18" s="69">
+      <c r="M18" s="46"/>
+      <c r="O18" s="47">
         <v>4.5</v>
       </c>
     </row>
@@ -2010,9 +1989,9 @@
       <c r="J19" s="2">
         <v>19.5</v>
       </c>
-      <c r="L19" s="65"/>
-      <c r="M19" s="65"/>
-      <c r="O19" s="69"/>
+      <c r="L19" s="46"/>
+      <c r="M19" s="46"/>
+      <c r="O19" s="47"/>
     </row>
     <row r="21" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A21" s="6"/>
@@ -2050,10 +2029,10 @@
       <c r="J23" s="49"/>
       <c r="K23" s="49"/>
       <c r="L23" s="50"/>
-      <c r="N23" s="65" t="s">
+      <c r="N23" s="46" t="s">
         <v>120</v>
       </c>
-      <c r="O23" s="65"/>
+      <c r="O23" s="46"/>
       <c r="Q23" s="7"/>
       <c r="R23" s="7"/>
       <c r="S23" s="7"/>
@@ -2070,29 +2049,29 @@
       <c r="J24" s="52"/>
       <c r="K24" s="52"/>
       <c r="L24" s="53"/>
-      <c r="N24" s="65"/>
-      <c r="O24" s="65"/>
+      <c r="N24" s="46"/>
+      <c r="O24" s="46"/>
       <c r="Q24" s="7"/>
       <c r="R24" s="7"/>
       <c r="S24" s="7"/>
     </row>
     <row r="26" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B26" s="47" t="s">
+      <c r="B26" s="66" t="s">
         <v>8</v>
       </c>
-      <c r="C26" s="47"/>
-      <c r="D26" s="47"/>
-      <c r="F26" s="47" t="s">
+      <c r="C26" s="66"/>
+      <c r="D26" s="66"/>
+      <c r="F26" s="66" t="s">
         <v>199</v>
       </c>
-      <c r="G26" s="47"/>
-      <c r="H26" s="47"/>
-      <c r="I26" s="47"/>
+      <c r="G26" s="66"/>
+      <c r="H26" s="66"/>
+      <c r="I26" s="66"/>
       <c r="J26" s="7"/>
-      <c r="K26" s="62" t="s">
+      <c r="K26" s="54" t="s">
         <v>119</v>
       </c>
-      <c r="L26" s="63"/>
+      <c r="L26" s="56"/>
       <c r="N26" s="9" t="s">
         <v>67</v>
       </c>
@@ -2125,7 +2104,7 @@
       <c r="L27" s="2" t="s">
         <v>118</v>
       </c>
-      <c r="N27" s="60">
+      <c r="N27" s="69">
         <f>(K29/30*0.4*5)+(B29/25*0.3*5)+(0.3*F29)</f>
         <v>4.2133333333333329</v>
       </c>
@@ -2156,26 +2135,26 @@
         <v>20</v>
       </c>
       <c r="L28" s="2"/>
-      <c r="N28" s="61"/>
+      <c r="N28" s="70"/>
     </row>
     <row r="29" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B29" s="46">
+      <c r="B29" s="71">
         <f>SUM(B28:C28)</f>
         <v>23</v>
       </c>
-      <c r="C29" s="46"/>
-      <c r="D29" s="46"/>
-      <c r="F29" s="46">
+      <c r="C29" s="71"/>
+      <c r="D29" s="71"/>
+      <c r="F29" s="71">
         <v>5</v>
       </c>
-      <c r="G29" s="46"/>
-      <c r="H29" s="46"/>
-      <c r="I29" s="46"/>
-      <c r="K29" s="46">
+      <c r="G29" s="71"/>
+      <c r="H29" s="71"/>
+      <c r="I29" s="71"/>
+      <c r="K29" s="71">
         <f>SUM(K28:L28)</f>
         <v>20</v>
       </c>
-      <c r="L29" s="46"/>
+      <c r="L29" s="71"/>
       <c r="N29" s="38"/>
     </row>
     <row r="31" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -2223,17 +2202,17 @@
       <c r="I34" s="53"/>
     </row>
     <row r="36" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B36" s="47" t="s">
+      <c r="B36" s="66" t="s">
         <v>98</v>
       </c>
-      <c r="C36" s="47"/>
+      <c r="C36" s="66"/>
       <c r="D36" s="7"/>
-      <c r="E36" s="62" t="s">
+      <c r="E36" s="54" t="s">
         <v>135</v>
       </c>
-      <c r="F36" s="68"/>
-      <c r="G36" s="68"/>
-      <c r="H36" s="63"/>
+      <c r="F36" s="55"/>
+      <c r="G36" s="55"/>
+      <c r="H36" s="56"/>
     </row>
     <row r="37" spans="2:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B37" s="2" t="s">
@@ -2276,14 +2255,14 @@
       <c r="O38" s="7"/>
     </row>
     <row r="41" spans="2:15" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B41" s="70" t="s">
+      <c r="B41" s="64" t="s">
         <v>117</v>
       </c>
-      <c r="C41" s="71"/>
-      <c r="F41" s="65" t="s">
+      <c r="C41" s="65"/>
+      <c r="F41" s="46" t="s">
         <v>102</v>
       </c>
-      <c r="G41" s="65"/>
+      <c r="G41" s="46"/>
       <c r="I41" s="9" t="s">
         <v>22</v>
       </c>
@@ -2339,7 +2318,7 @@
       <c r="G44" s="2">
         <v>10</v>
       </c>
-      <c r="I44" s="64" t="s">
+      <c r="I44" s="63" t="s">
         <v>67</v>
       </c>
     </row>
@@ -2350,9 +2329,7 @@
       <c r="C45" s="2">
         <v>4</v>
       </c>
-      <c r="F45" s="84"/>
-      <c r="G45" s="84"/>
-      <c r="I45" s="64"/>
+      <c r="I45" s="63"/>
     </row>
     <row r="46" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B46" s="2" t="s">
@@ -2377,8 +2354,6 @@
         <v>108</v>
       </c>
       <c r="C47" s="2"/>
-      <c r="F47" s="84"/>
-      <c r="G47" s="84"/>
     </row>
     <row r="48" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B48" s="2" t="s">
@@ -2387,8 +2362,6 @@
       <c r="C48" s="2">
         <v>2</v>
       </c>
-      <c r="F48" s="84"/>
-      <c r="G48" s="84"/>
       <c r="I48" s="38"/>
     </row>
     <row r="49" spans="1:19" x14ac:dyDescent="0.25">
@@ -2398,8 +2371,6 @@
       <c r="C49" s="2">
         <v>2</v>
       </c>
-      <c r="F49" s="84"/>
-      <c r="G49" s="84"/>
     </row>
     <row r="50" spans="1:19" x14ac:dyDescent="0.25">
       <c r="B50" s="2" t="s">
@@ -2408,8 +2379,6 @@
       <c r="C50" s="2">
         <v>2</v>
       </c>
-      <c r="F50" s="84"/>
-      <c r="G50" s="84"/>
     </row>
     <row r="51" spans="1:19" x14ac:dyDescent="0.25">
       <c r="B51" s="2" t="s">
@@ -2457,70 +2426,70 @@
     </row>
     <row r="57" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="58" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B58" s="54" t="s">
+      <c r="B58" s="48" t="s">
         <v>80</v>
       </c>
-      <c r="C58" s="55"/>
-      <c r="D58" s="55"/>
-      <c r="E58" s="55"/>
-      <c r="F58" s="55"/>
-      <c r="G58" s="55"/>
-      <c r="H58" s="55"/>
-      <c r="I58" s="55"/>
-      <c r="J58" s="55"/>
-      <c r="K58" s="55"/>
-      <c r="L58" s="55"/>
-      <c r="M58" s="55"/>
-      <c r="N58" s="55"/>
-      <c r="O58" s="55"/>
-      <c r="P58" s="55"/>
-      <c r="Q58" s="55"/>
-      <c r="R58" s="55"/>
-      <c r="S58" s="56"/>
+      <c r="C58" s="49"/>
+      <c r="D58" s="49"/>
+      <c r="E58" s="49"/>
+      <c r="F58" s="49"/>
+      <c r="G58" s="49"/>
+      <c r="H58" s="49"/>
+      <c r="I58" s="49"/>
+      <c r="J58" s="49"/>
+      <c r="K58" s="49"/>
+      <c r="L58" s="49"/>
+      <c r="M58" s="49"/>
+      <c r="N58" s="49"/>
+      <c r="O58" s="49"/>
+      <c r="P58" s="49"/>
+      <c r="Q58" s="49"/>
+      <c r="R58" s="49"/>
+      <c r="S58" s="50"/>
     </row>
     <row r="59" spans="1:19" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B59" s="57"/>
-      <c r="C59" s="58"/>
-      <c r="D59" s="58"/>
-      <c r="E59" s="58"/>
-      <c r="F59" s="58"/>
-      <c r="G59" s="58"/>
-      <c r="H59" s="58"/>
-      <c r="I59" s="58"/>
-      <c r="J59" s="58"/>
-      <c r="K59" s="58"/>
-      <c r="L59" s="58"/>
-      <c r="M59" s="58"/>
-      <c r="N59" s="58"/>
-      <c r="O59" s="58"/>
-      <c r="P59" s="58"/>
-      <c r="Q59" s="58"/>
-      <c r="R59" s="58"/>
-      <c r="S59" s="59"/>
+      <c r="B59" s="51"/>
+      <c r="C59" s="52"/>
+      <c r="D59" s="52"/>
+      <c r="E59" s="52"/>
+      <c r="F59" s="52"/>
+      <c r="G59" s="52"/>
+      <c r="H59" s="52"/>
+      <c r="I59" s="52"/>
+      <c r="J59" s="52"/>
+      <c r="K59" s="52"/>
+      <c r="L59" s="52"/>
+      <c r="M59" s="52"/>
+      <c r="N59" s="52"/>
+      <c r="O59" s="52"/>
+      <c r="P59" s="52"/>
+      <c r="Q59" s="52"/>
+      <c r="R59" s="52"/>
+      <c r="S59" s="53"/>
     </row>
     <row r="61" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B61" s="47" t="s">
+      <c r="B61" s="66" t="s">
         <v>63</v>
       </c>
-      <c r="C61" s="47"/>
-      <c r="D61" s="47"/>
-      <c r="E61" s="47"/>
-      <c r="F61" s="47"/>
-      <c r="G61" s="47"/>
-      <c r="H61" s="47"/>
-      <c r="I61" s="47"/>
-      <c r="J61" s="47"/>
-      <c r="K61" s="47"/>
-      <c r="M61" s="47" t="s">
+      <c r="C61" s="66"/>
+      <c r="D61" s="66"/>
+      <c r="E61" s="66"/>
+      <c r="F61" s="66"/>
+      <c r="G61" s="66"/>
+      <c r="H61" s="66"/>
+      <c r="I61" s="66"/>
+      <c r="J61" s="66"/>
+      <c r="K61" s="66"/>
+      <c r="M61" s="66" t="s">
         <v>90</v>
       </c>
-      <c r="N61" s="47"/>
-      <c r="O61" s="47"/>
-      <c r="P61" s="47"/>
-      <c r="R61" s="47" t="s">
+      <c r="N61" s="66"/>
+      <c r="O61" s="66"/>
+      <c r="P61" s="66"/>
+      <c r="R61" s="66" t="s">
         <v>64</v>
       </c>
-      <c r="S61" s="47"/>
+      <c r="S61" s="66"/>
     </row>
     <row r="62" spans="1:19" x14ac:dyDescent="0.25">
       <c r="B62" s="2" t="s">
@@ -2609,54 +2578,72 @@
       <c r="N63" s="2">
         <v>5</v>
       </c>
-      <c r="O63" s="2"/>
-      <c r="P63" s="2"/>
+      <c r="O63" s="2">
+        <v>10</v>
+      </c>
+      <c r="P63" s="2">
+        <v>20</v>
+      </c>
       <c r="R63" s="2"/>
       <c r="S63" s="2"/>
     </row>
-    <row r="66" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B66" s="64" t="s">
+    <row r="66" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B66" s="63" t="s">
         <v>22</v>
       </c>
-      <c r="C66" s="64"/>
+      <c r="C66" s="63"/>
       <c r="E66" s="9" t="s">
         <v>67</v>
       </c>
-      <c r="G66" s="64" t="s">
-        <v>87</v>
-      </c>
-      <c r="H66" s="64"/>
-      <c r="K66" s="39" t="s">
+      <c r="G66" s="39" t="s">
         <v>214</v>
       </c>
-    </row>
-    <row r="67" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B67" s="65">
-        <f>SUM(B63:K63,M63:P63,R63:S63,K67)</f>
-        <v>29</v>
-      </c>
-      <c r="C67" s="65"/>
-      <c r="E67" s="69"/>
-      <c r="G67" s="65">
-        <f>50-SUM(B63:K63,M63:P63,R63:S63,K67)</f>
-        <v>21</v>
-      </c>
-      <c r="H67" s="65"/>
-      <c r="K67" s="65">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="68" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B68" s="65"/>
-      <c r="C68" s="65"/>
-      <c r="E68" s="69"/>
-      <c r="G68" s="65"/>
-      <c r="H68" s="65"/>
-      <c r="K68" s="65"/>
+      <c r="H66" s="78"/>
+    </row>
+    <row r="67" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B67" s="46">
+        <f>SUM(B63:K63,M63:P63,R63:S63,G67)</f>
+        <v>65</v>
+      </c>
+      <c r="C67" s="46"/>
+      <c r="E67" s="47"/>
+      <c r="G67" s="46">
+        <v>9</v>
+      </c>
+      <c r="H67" s="79"/>
+    </row>
+    <row r="68" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B68" s="46"/>
+      <c r="C68" s="46"/>
+      <c r="E68" s="47"/>
+      <c r="G68" s="46"/>
+      <c r="H68" s="79"/>
     </row>
   </sheetData>
-  <mergeCells count="40">
-    <mergeCell ref="K67:K68"/>
+  <mergeCells count="38">
+    <mergeCell ref="K29:L29"/>
+    <mergeCell ref="R61:S61"/>
+    <mergeCell ref="B33:I34"/>
+    <mergeCell ref="B61:K61"/>
+    <mergeCell ref="B58:S59"/>
+    <mergeCell ref="M61:P61"/>
+    <mergeCell ref="F29:I29"/>
+    <mergeCell ref="B29:D29"/>
+    <mergeCell ref="N27:N28"/>
+    <mergeCell ref="F26:I26"/>
+    <mergeCell ref="K26:L26"/>
+    <mergeCell ref="B23:L24"/>
+    <mergeCell ref="B26:D26"/>
+    <mergeCell ref="L17:M17"/>
+    <mergeCell ref="E10:E11"/>
+    <mergeCell ref="G10:H11"/>
+    <mergeCell ref="B17:F17"/>
+    <mergeCell ref="H17:J17"/>
+    <mergeCell ref="B66:C66"/>
+    <mergeCell ref="B67:C68"/>
+    <mergeCell ref="B9:C9"/>
+    <mergeCell ref="B10:C11"/>
+    <mergeCell ref="G67:G68"/>
     <mergeCell ref="O18:O19"/>
     <mergeCell ref="B14:H15"/>
     <mergeCell ref="K5:N5"/>
@@ -2672,30 +2659,6 @@
     <mergeCell ref="E36:H36"/>
     <mergeCell ref="G9:H9"/>
     <mergeCell ref="E67:E68"/>
-    <mergeCell ref="B66:C66"/>
-    <mergeCell ref="B67:C68"/>
-    <mergeCell ref="G66:H66"/>
-    <mergeCell ref="G67:H68"/>
-    <mergeCell ref="B9:C9"/>
-    <mergeCell ref="B10:C11"/>
-    <mergeCell ref="L17:M17"/>
-    <mergeCell ref="E10:E11"/>
-    <mergeCell ref="G10:H11"/>
-    <mergeCell ref="B17:F17"/>
-    <mergeCell ref="H17:J17"/>
-    <mergeCell ref="N27:N28"/>
-    <mergeCell ref="F26:I26"/>
-    <mergeCell ref="K26:L26"/>
-    <mergeCell ref="B23:L24"/>
-    <mergeCell ref="B26:D26"/>
-    <mergeCell ref="K29:L29"/>
-    <mergeCell ref="R61:S61"/>
-    <mergeCell ref="B33:I34"/>
-    <mergeCell ref="B61:K61"/>
-    <mergeCell ref="B58:S59"/>
-    <mergeCell ref="M61:P61"/>
-    <mergeCell ref="F29:I29"/>
-    <mergeCell ref="B29:D29"/>
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2731,60 +2694,60 @@
   <sheetData>
     <row r="1" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="2" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B2" s="72" t="s">
+      <c r="B2" s="48" t="s">
         <v>121</v>
       </c>
-      <c r="C2" s="73"/>
-      <c r="D2" s="73"/>
-      <c r="E2" s="73"/>
-      <c r="F2" s="73"/>
-      <c r="G2" s="73"/>
-      <c r="H2" s="73"/>
-      <c r="I2" s="73"/>
-      <c r="J2" s="73"/>
-      <c r="K2" s="73"/>
-      <c r="L2" s="73"/>
-      <c r="M2" s="73"/>
-      <c r="N2" s="73"/>
-      <c r="O2" s="73"/>
-      <c r="P2" s="74"/>
+      <c r="C2" s="49"/>
+      <c r="D2" s="49"/>
+      <c r="E2" s="49"/>
+      <c r="F2" s="49"/>
+      <c r="G2" s="49"/>
+      <c r="H2" s="49"/>
+      <c r="I2" s="49"/>
+      <c r="J2" s="49"/>
+      <c r="K2" s="49"/>
+      <c r="L2" s="49"/>
+      <c r="M2" s="49"/>
+      <c r="N2" s="49"/>
+      <c r="O2" s="49"/>
+      <c r="P2" s="50"/>
     </row>
     <row r="3" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B3" s="75"/>
-      <c r="C3" s="76"/>
-      <c r="D3" s="76"/>
-      <c r="E3" s="76"/>
-      <c r="F3" s="76"/>
-      <c r="G3" s="76"/>
-      <c r="H3" s="76"/>
-      <c r="I3" s="76"/>
-      <c r="J3" s="76"/>
-      <c r="K3" s="76"/>
-      <c r="L3" s="76"/>
-      <c r="M3" s="76"/>
-      <c r="N3" s="76"/>
-      <c r="O3" s="76"/>
-      <c r="P3" s="77"/>
+      <c r="B3" s="51"/>
+      <c r="C3" s="52"/>
+      <c r="D3" s="52"/>
+      <c r="E3" s="52"/>
+      <c r="F3" s="52"/>
+      <c r="G3" s="52"/>
+      <c r="H3" s="52"/>
+      <c r="I3" s="52"/>
+      <c r="J3" s="52"/>
+      <c r="K3" s="52"/>
+      <c r="L3" s="52"/>
+      <c r="M3" s="52"/>
+      <c r="N3" s="52"/>
+      <c r="O3" s="52"/>
+      <c r="P3" s="53"/>
       <c r="R3" s="12"/>
     </row>
     <row r="5" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B5" s="47" t="s">
+      <c r="B5" s="66" t="s">
         <v>18</v>
       </c>
-      <c r="C5" s="47"/>
-      <c r="D5" s="47"/>
-      <c r="E5" s="47"/>
-      <c r="F5" s="47"/>
-      <c r="G5" s="47"/>
+      <c r="C5" s="66"/>
+      <c r="D5" s="66"/>
+      <c r="E5" s="66"/>
+      <c r="F5" s="66"/>
+      <c r="G5" s="66"/>
       <c r="I5" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="K5" s="62" t="s">
+      <c r="K5" s="54" t="s">
         <v>8</v>
       </c>
-      <c r="L5" s="68"/>
-      <c r="M5" s="68"/>
-      <c r="N5" s="63"/>
+      <c r="L5" s="55"/>
+      <c r="M5" s="55"/>
+      <c r="N5" s="56"/>
       <c r="P5" s="4" t="s">
         <v>74</v>
       </c>
@@ -2866,28 +2829,28 @@
       </c>
     </row>
     <row r="9" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B9" s="64" t="s">
+      <c r="B9" s="63" t="s">
         <v>22</v>
       </c>
-      <c r="C9" s="64"/>
+      <c r="C9" s="63"/>
       <c r="E9" s="9" t="s">
         <v>67</v>
       </c>
     </row>
     <row r="10" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B10" s="65">
+      <c r="B10" s="46">
         <f>_xlfn.CEILING.MATH(SUM(B7:G7,I7,K7:N7,P7),1,1)</f>
         <v>110</v>
       </c>
-      <c r="C10" s="65"/>
-      <c r="E10" s="66">
+      <c r="C10" s="46"/>
+      <c r="E10" s="67">
         <v>4</v>
       </c>
     </row>
     <row r="11" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B11" s="65"/>
-      <c r="C11" s="65"/>
-      <c r="E11" s="67"/>
+      <c r="B11" s="46"/>
+      <c r="C11" s="46"/>
+      <c r="E11" s="68"/>
     </row>
     <row r="12" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A12" s="6"/>
@@ -2912,40 +2875,40 @@
     </row>
     <row r="13" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="14" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B14" s="72" t="s">
+      <c r="B14" s="48" t="s">
         <v>122</v>
       </c>
-      <c r="C14" s="73"/>
-      <c r="D14" s="73"/>
-      <c r="E14" s="73"/>
-      <c r="F14" s="73"/>
-      <c r="G14" s="73"/>
-      <c r="H14" s="74"/>
+      <c r="C14" s="49"/>
+      <c r="D14" s="49"/>
+      <c r="E14" s="49"/>
+      <c r="F14" s="49"/>
+      <c r="G14" s="49"/>
+      <c r="H14" s="50"/>
     </row>
     <row r="15" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B15" s="75"/>
-      <c r="C15" s="76"/>
-      <c r="D15" s="76"/>
-      <c r="E15" s="76"/>
-      <c r="F15" s="76"/>
-      <c r="G15" s="76"/>
-      <c r="H15" s="77"/>
+      <c r="B15" s="51"/>
+      <c r="C15" s="52"/>
+      <c r="D15" s="52"/>
+      <c r="E15" s="52"/>
+      <c r="F15" s="52"/>
+      <c r="G15" s="52"/>
+      <c r="H15" s="53"/>
     </row>
     <row r="17" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B17" s="47" t="s">
+      <c r="B17" s="66" t="s">
         <v>12</v>
       </c>
-      <c r="C17" s="47"/>
-      <c r="D17" s="47"/>
-      <c r="F17" s="47" t="s">
+      <c r="C17" s="66"/>
+      <c r="D17" s="66"/>
+      <c r="F17" s="66" t="s">
         <v>8</v>
       </c>
-      <c r="G17" s="47"/>
-      <c r="H17" s="47"/>
-      <c r="J17" s="64" t="s">
+      <c r="G17" s="66"/>
+      <c r="H17" s="66"/>
+      <c r="J17" s="63" t="s">
         <v>22</v>
       </c>
-      <c r="K17" s="64"/>
+      <c r="K17" s="63"/>
       <c r="M17" s="9" t="s">
         <v>67</v>
       </c>
@@ -2969,12 +2932,12 @@
       <c r="H18" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="J18" s="65">
+      <c r="J18" s="46">
         <f>SUM(B19:D19,F19:H19)</f>
         <v>93</v>
       </c>
-      <c r="K18" s="65"/>
-      <c r="M18" s="69">
+      <c r="K18" s="46"/>
+      <c r="M18" s="47">
         <v>5</v>
       </c>
     </row>
@@ -2997,9 +2960,9 @@
       <c r="H19" s="2">
         <v>4</v>
       </c>
-      <c r="J19" s="65"/>
-      <c r="K19" s="65"/>
-      <c r="M19" s="69"/>
+      <c r="J19" s="46"/>
+      <c r="K19" s="46"/>
+      <c r="M19" s="47"/>
     </row>
     <row r="21" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A21" s="6"/>
@@ -3024,46 +2987,46 @@
     </row>
     <row r="22" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="23" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B23" s="72" t="s">
+      <c r="B23" s="48" t="s">
         <v>123</v>
       </c>
-      <c r="C23" s="73"/>
-      <c r="D23" s="73"/>
-      <c r="E23" s="73"/>
-      <c r="F23" s="73"/>
-      <c r="G23" s="73"/>
-      <c r="H23" s="73"/>
-      <c r="I23" s="73"/>
-      <c r="J23" s="73"/>
-      <c r="K23" s="74"/>
+      <c r="C23" s="49"/>
+      <c r="D23" s="49"/>
+      <c r="E23" s="49"/>
+      <c r="F23" s="49"/>
+      <c r="G23" s="49"/>
+      <c r="H23" s="49"/>
+      <c r="I23" s="49"/>
+      <c r="J23" s="49"/>
+      <c r="K23" s="50"/>
     </row>
     <row r="24" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B24" s="75"/>
-      <c r="C24" s="76"/>
-      <c r="D24" s="76"/>
-      <c r="E24" s="76"/>
-      <c r="F24" s="76"/>
-      <c r="G24" s="76"/>
-      <c r="H24" s="76"/>
-      <c r="I24" s="76"/>
-      <c r="J24" s="76"/>
-      <c r="K24" s="77"/>
+      <c r="B24" s="51"/>
+      <c r="C24" s="52"/>
+      <c r="D24" s="52"/>
+      <c r="E24" s="52"/>
+      <c r="F24" s="52"/>
+      <c r="G24" s="52"/>
+      <c r="H24" s="52"/>
+      <c r="I24" s="52"/>
+      <c r="J24" s="52"/>
+      <c r="K24" s="53"/>
     </row>
     <row r="26" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B26" s="47" t="s">
+      <c r="B26" s="66" t="s">
         <v>17</v>
       </c>
-      <c r="C26" s="47"/>
-      <c r="E26" s="62" t="s">
+      <c r="C26" s="66"/>
+      <c r="E26" s="54" t="s">
         <v>21</v>
       </c>
-      <c r="F26" s="68"/>
-      <c r="G26" s="63"/>
-      <c r="I26" s="47" t="s">
+      <c r="F26" s="55"/>
+      <c r="G26" s="56"/>
+      <c r="I26" s="66" t="s">
         <v>20</v>
       </c>
-      <c r="J26" s="47"/>
-      <c r="K26" s="47"/>
+      <c r="J26" s="66"/>
+      <c r="K26" s="66"/>
       <c r="M26" s="10" t="s">
         <v>22</v>
       </c>
@@ -3098,12 +3061,12 @@
       <c r="K27" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="M27" s="78">
+      <c r="M27" s="72">
         <f>SUM(B28:C28,E28:G28,I28:K28)</f>
         <v>36</v>
       </c>
       <c r="N27" s="7"/>
-      <c r="O27" s="69">
+      <c r="O27" s="47">
         <v>4</v>
       </c>
       <c r="P27" s="8"/>
@@ -3133,9 +3096,9 @@
       <c r="K28" s="2">
         <v>3.2</v>
       </c>
-      <c r="M28" s="78"/>
+      <c r="M28" s="72"/>
       <c r="N28" s="7"/>
-      <c r="O28" s="69"/>
+      <c r="O28" s="47"/>
       <c r="P28" s="8"/>
     </row>
     <row r="30" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -3161,39 +3124,39 @@
     </row>
     <row r="31" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="32" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B32" s="72" t="s">
+      <c r="B32" s="48" t="s">
         <v>124</v>
       </c>
-      <c r="C32" s="73"/>
-      <c r="D32" s="73"/>
-      <c r="E32" s="73"/>
-      <c r="F32" s="73"/>
-      <c r="G32" s="73"/>
-      <c r="H32" s="73"/>
-      <c r="I32" s="74"/>
+      <c r="C32" s="49"/>
+      <c r="D32" s="49"/>
+      <c r="E32" s="49"/>
+      <c r="F32" s="49"/>
+      <c r="G32" s="49"/>
+      <c r="H32" s="49"/>
+      <c r="I32" s="50"/>
     </row>
     <row r="33" spans="2:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B33" s="75"/>
-      <c r="C33" s="76"/>
-      <c r="D33" s="76"/>
-      <c r="E33" s="76"/>
-      <c r="F33" s="76"/>
-      <c r="G33" s="76"/>
-      <c r="H33" s="76"/>
-      <c r="I33" s="77"/>
+      <c r="B33" s="51"/>
+      <c r="C33" s="52"/>
+      <c r="D33" s="52"/>
+      <c r="E33" s="52"/>
+      <c r="F33" s="52"/>
+      <c r="G33" s="52"/>
+      <c r="H33" s="52"/>
+      <c r="I33" s="53"/>
     </row>
     <row r="35" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B35" s="47" t="s">
+      <c r="B35" s="66" t="s">
         <v>31</v>
       </c>
-      <c r="C35" s="47"/>
-      <c r="D35" s="47"/>
-      <c r="F35" s="47" t="s">
+      <c r="C35" s="66"/>
+      <c r="D35" s="66"/>
+      <c r="F35" s="66" t="s">
         <v>12</v>
       </c>
-      <c r="G35" s="47"/>
-      <c r="H35" s="47"/>
-      <c r="I35" s="47"/>
+      <c r="G35" s="66"/>
+      <c r="H35" s="66"/>
+      <c r="I35" s="66"/>
       <c r="N35" s="7"/>
       <c r="O35" s="7"/>
     </row>
@@ -3250,14 +3213,14 @@
       <c r="O37" s="7"/>
     </row>
     <row r="40" spans="2:15" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B40" s="70" t="s">
+      <c r="B40" s="64" t="s">
         <v>35</v>
       </c>
-      <c r="C40" s="71"/>
-      <c r="F40" s="65" t="s">
+      <c r="C40" s="65"/>
+      <c r="F40" s="46" t="s">
         <v>36</v>
       </c>
-      <c r="G40" s="65"/>
+      <c r="G40" s="46"/>
       <c r="I40" s="9" t="s">
         <v>22</v>
       </c>
@@ -3313,7 +3276,7 @@
       <c r="G43" s="2">
         <v>0.44</v>
       </c>
-      <c r="I43" s="64" t="s">
+      <c r="I43" s="63" t="s">
         <v>67</v>
       </c>
     </row>
@@ -3330,7 +3293,7 @@
       <c r="G44" s="2">
         <v>1</v>
       </c>
-      <c r="I44" s="64"/>
+      <c r="I44" s="63"/>
     </row>
     <row r="45" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B45" s="2" t="s">
@@ -3474,67 +3437,67 @@
     </row>
     <row r="57" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="58" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B58" s="72" t="s">
+      <c r="B58" s="48" t="s">
         <v>125</v>
       </c>
-      <c r="C58" s="73"/>
-      <c r="D58" s="73"/>
-      <c r="E58" s="73"/>
-      <c r="F58" s="73"/>
-      <c r="G58" s="73"/>
-      <c r="H58" s="73"/>
-      <c r="I58" s="73"/>
-      <c r="J58" s="73"/>
-      <c r="K58" s="73"/>
-      <c r="L58" s="73"/>
-      <c r="M58" s="73"/>
-      <c r="N58" s="73"/>
-      <c r="O58" s="73"/>
-      <c r="P58" s="73"/>
-      <c r="Q58" s="73"/>
-      <c r="R58" s="74"/>
+      <c r="C58" s="49"/>
+      <c r="D58" s="49"/>
+      <c r="E58" s="49"/>
+      <c r="F58" s="49"/>
+      <c r="G58" s="49"/>
+      <c r="H58" s="49"/>
+      <c r="I58" s="49"/>
+      <c r="J58" s="49"/>
+      <c r="K58" s="49"/>
+      <c r="L58" s="49"/>
+      <c r="M58" s="49"/>
+      <c r="N58" s="49"/>
+      <c r="O58" s="49"/>
+      <c r="P58" s="49"/>
+      <c r="Q58" s="49"/>
+      <c r="R58" s="50"/>
     </row>
     <row r="59" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B59" s="75"/>
-      <c r="C59" s="76"/>
-      <c r="D59" s="76"/>
-      <c r="E59" s="76"/>
-      <c r="F59" s="76"/>
-      <c r="G59" s="76"/>
-      <c r="H59" s="76"/>
-      <c r="I59" s="76"/>
-      <c r="J59" s="76"/>
-      <c r="K59" s="76"/>
-      <c r="L59" s="76"/>
-      <c r="M59" s="76"/>
-      <c r="N59" s="76"/>
-      <c r="O59" s="76"/>
-      <c r="P59" s="76"/>
-      <c r="Q59" s="76"/>
-      <c r="R59" s="77"/>
+      <c r="B59" s="51"/>
+      <c r="C59" s="52"/>
+      <c r="D59" s="52"/>
+      <c r="E59" s="52"/>
+      <c r="F59" s="52"/>
+      <c r="G59" s="52"/>
+      <c r="H59" s="52"/>
+      <c r="I59" s="52"/>
+      <c r="J59" s="52"/>
+      <c r="K59" s="52"/>
+      <c r="L59" s="52"/>
+      <c r="M59" s="52"/>
+      <c r="N59" s="52"/>
+      <c r="O59" s="52"/>
+      <c r="P59" s="52"/>
+      <c r="Q59" s="52"/>
+      <c r="R59" s="53"/>
     </row>
     <row r="61" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B61" s="47" t="s">
+      <c r="B61" s="66" t="s">
         <v>63</v>
       </c>
-      <c r="C61" s="47"/>
-      <c r="D61" s="47"/>
-      <c r="E61" s="47"/>
-      <c r="F61" s="47"/>
-      <c r="G61" s="47"/>
-      <c r="H61" s="47"/>
-      <c r="I61" s="47"/>
-      <c r="J61" s="47"/>
-      <c r="K61" s="47"/>
-      <c r="M61" s="47" t="s">
+      <c r="C61" s="66"/>
+      <c r="D61" s="66"/>
+      <c r="E61" s="66"/>
+      <c r="F61" s="66"/>
+      <c r="G61" s="66"/>
+      <c r="H61" s="66"/>
+      <c r="I61" s="66"/>
+      <c r="J61" s="66"/>
+      <c r="K61" s="66"/>
+      <c r="M61" s="66" t="s">
         <v>68</v>
       </c>
-      <c r="N61" s="47"/>
-      <c r="O61" s="47"/>
-      <c r="Q61" s="47" t="s">
+      <c r="N61" s="66"/>
+      <c r="O61" s="66"/>
+      <c r="Q61" s="66" t="s">
         <v>64</v>
       </c>
-      <c r="R61" s="47"/>
+      <c r="R61" s="66"/>
     </row>
     <row r="62" spans="1:19" x14ac:dyDescent="0.25">
       <c r="B62" s="2" t="s">
@@ -3631,28 +3594,28 @@
       </c>
     </row>
     <row r="66" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B66" s="64" t="s">
+      <c r="B66" s="63" t="s">
         <v>22</v>
       </c>
-      <c r="C66" s="64"/>
+      <c r="C66" s="63"/>
       <c r="E66" s="9" t="s">
         <v>67</v>
       </c>
     </row>
     <row r="67" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B67" s="65">
+      <c r="B67" s="46">
         <f xml:space="preserve"> SUM(B63:K63,M63:O63,Q63:R63)</f>
         <v>85.5</v>
       </c>
-      <c r="C67" s="65"/>
-      <c r="E67" s="69">
+      <c r="C67" s="46"/>
+      <c r="E67" s="47">
         <v>4.5</v>
       </c>
     </row>
     <row r="68" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B68" s="65"/>
-      <c r="C68" s="65"/>
-      <c r="E68" s="69"/>
+      <c r="B68" s="46"/>
+      <c r="C68" s="46"/>
+      <c r="E68" s="47"/>
     </row>
     <row r="70" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A70" s="6"/>
@@ -3677,26 +3640,26 @@
     </row>
     <row r="71" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="72" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B72" s="72" t="s">
+      <c r="B72" s="48" t="s">
         <v>126</v>
       </c>
-      <c r="C72" s="73"/>
-      <c r="D72" s="73"/>
-      <c r="E72" s="73"/>
-      <c r="F72" s="73"/>
-      <c r="G72" s="73"/>
-      <c r="H72" s="73"/>
-      <c r="I72" s="74"/>
+      <c r="C72" s="49"/>
+      <c r="D72" s="49"/>
+      <c r="E72" s="49"/>
+      <c r="F72" s="49"/>
+      <c r="G72" s="49"/>
+      <c r="H72" s="49"/>
+      <c r="I72" s="50"/>
     </row>
     <row r="73" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B73" s="75"/>
-      <c r="C73" s="76"/>
-      <c r="D73" s="76"/>
-      <c r="E73" s="76"/>
-      <c r="F73" s="76"/>
-      <c r="G73" s="76"/>
-      <c r="H73" s="76"/>
-      <c r="I73" s="77"/>
+      <c r="B73" s="51"/>
+      <c r="C73" s="52"/>
+      <c r="D73" s="52"/>
+      <c r="E73" s="52"/>
+      <c r="F73" s="52"/>
+      <c r="G73" s="52"/>
+      <c r="H73" s="52"/>
+      <c r="I73" s="53"/>
     </row>
     <row r="75" spans="1:19" x14ac:dyDescent="0.25">
       <c r="B75" s="4" t="s">
@@ -3723,10 +3686,10 @@
       <c r="I75" s="4" t="s">
         <v>134</v>
       </c>
-      <c r="K75" s="64" t="s">
+      <c r="K75" s="63" t="s">
         <v>22</v>
       </c>
-      <c r="L75" s="64"/>
+      <c r="L75" s="63"/>
       <c r="N75" s="9" t="s">
         <v>67</v>
       </c>
@@ -3756,11 +3719,11 @@
       <c r="I76" s="2">
         <v>5</v>
       </c>
-      <c r="K76" s="65">
+      <c r="K76" s="46">
         <f>SUM(B76:I76)</f>
         <v>96</v>
       </c>
-      <c r="L76" s="65"/>
+      <c r="L76" s="46"/>
       <c r="N76" s="13">
         <v>5</v>
       </c>
@@ -3788,20 +3751,16 @@
     </row>
   </sheetData>
   <mergeCells count="34">
-    <mergeCell ref="B2:P3"/>
-    <mergeCell ref="B5:G5"/>
-    <mergeCell ref="K5:N5"/>
-    <mergeCell ref="B9:C9"/>
-    <mergeCell ref="B10:C11"/>
-    <mergeCell ref="E10:E11"/>
-    <mergeCell ref="M27:M28"/>
-    <mergeCell ref="O27:O28"/>
-    <mergeCell ref="B14:H15"/>
-    <mergeCell ref="B17:D17"/>
-    <mergeCell ref="F17:H17"/>
-    <mergeCell ref="J17:K17"/>
-    <mergeCell ref="J18:K19"/>
-    <mergeCell ref="M18:M19"/>
+    <mergeCell ref="B72:I73"/>
+    <mergeCell ref="K75:L75"/>
+    <mergeCell ref="K76:L76"/>
+    <mergeCell ref="B58:R59"/>
+    <mergeCell ref="B61:K61"/>
+    <mergeCell ref="M61:O61"/>
+    <mergeCell ref="Q61:R61"/>
+    <mergeCell ref="B66:C66"/>
+    <mergeCell ref="B67:C68"/>
+    <mergeCell ref="E67:E68"/>
     <mergeCell ref="I43:I44"/>
     <mergeCell ref="B23:K24"/>
     <mergeCell ref="B26:C26"/>
@@ -3812,16 +3771,20 @@
     <mergeCell ref="F35:I35"/>
     <mergeCell ref="B40:C40"/>
     <mergeCell ref="F40:G40"/>
-    <mergeCell ref="B72:I73"/>
-    <mergeCell ref="K75:L75"/>
-    <mergeCell ref="K76:L76"/>
-    <mergeCell ref="B58:R59"/>
-    <mergeCell ref="B61:K61"/>
-    <mergeCell ref="M61:O61"/>
-    <mergeCell ref="Q61:R61"/>
-    <mergeCell ref="B66:C66"/>
-    <mergeCell ref="B67:C68"/>
-    <mergeCell ref="E67:E68"/>
+    <mergeCell ref="M27:M28"/>
+    <mergeCell ref="O27:O28"/>
+    <mergeCell ref="B14:H15"/>
+    <mergeCell ref="B17:D17"/>
+    <mergeCell ref="F17:H17"/>
+    <mergeCell ref="J17:K17"/>
+    <mergeCell ref="J18:K19"/>
+    <mergeCell ref="M18:M19"/>
+    <mergeCell ref="B2:P3"/>
+    <mergeCell ref="B5:G5"/>
+    <mergeCell ref="K5:N5"/>
+    <mergeCell ref="B9:C9"/>
+    <mergeCell ref="B10:C11"/>
+    <mergeCell ref="E10:E11"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
@@ -4082,19 +4045,19 @@
       </c>
     </row>
     <row r="18" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B18" s="18" t="b">
-        <v>0</v>
-      </c>
-      <c r="C18" s="20" t="s">
+      <c r="B18" s="22" t="b">
+        <v>1</v>
+      </c>
+      <c r="C18" s="28" t="s">
         <v>150</v>
       </c>
-      <c r="D18" s="19">
+      <c r="D18" s="27">
         <v>45819</v>
       </c>
-      <c r="E18" s="17" t="s">
+      <c r="E18" s="26" t="s">
         <v>160</v>
       </c>
-      <c r="F18" s="20" t="s">
+      <c r="F18" s="28" t="s">
         <v>159</v>
       </c>
     </row>
@@ -4428,21 +4391,21 @@
   <sheetData>
     <row r="1" spans="2:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="2" spans="2:12" ht="23.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B2" s="79" t="s">
+      <c r="B2" s="73" t="s">
         <v>192</v>
       </c>
-      <c r="C2" s="80"/>
-      <c r="D2" s="81"/>
-      <c r="F2" s="79" t="s">
+      <c r="C2" s="74"/>
+      <c r="D2" s="75"/>
+      <c r="F2" s="73" t="s">
         <v>193</v>
       </c>
-      <c r="G2" s="80"/>
-      <c r="H2" s="81"/>
-      <c r="J2" s="79" t="s">
+      <c r="G2" s="74"/>
+      <c r="H2" s="75"/>
+      <c r="J2" s="73" t="s">
         <v>194</v>
       </c>
-      <c r="K2" s="80"/>
-      <c r="L2" s="81"/>
+      <c r="K2" s="74"/>
+      <c r="L2" s="75"/>
     </row>
     <row r="3" spans="2:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B3" s="33" t="s">
@@ -4621,26 +4584,26 @@
     </row>
     <row r="10" spans="2:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="11" spans="2:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B11" s="82" t="s">
+      <c r="B11" s="76" t="s">
         <v>186</v>
       </c>
-      <c r="C11" s="83"/>
+      <c r="C11" s="77"/>
       <c r="D11" s="32">
         <f>(D4*C4+D5*C5+D6*C6+D7*C7+D8*C8+D9*C9)/30</f>
         <v>4.4333333333333336</v>
       </c>
-      <c r="F11" s="82" t="s">
+      <c r="F11" s="76" t="s">
         <v>186</v>
       </c>
-      <c r="G11" s="83"/>
+      <c r="G11" s="77"/>
       <c r="H11" s="32">
         <f>(H4*G4+H5*G5+H6*G6+H7*G7+H8*G8)/30</f>
         <v>1.5833333333333333</v>
       </c>
-      <c r="J11" s="82" t="s">
+      <c r="J11" s="76" t="s">
         <v>186</v>
       </c>
-      <c r="K11" s="83"/>
+      <c r="K11" s="77"/>
       <c r="L11" s="32">
         <f>(L4*K4+L5*K5+L6*K6+L7*K7+L8*K8)/30</f>
         <v>0</v>

</xml_diff>

<commit_message>
New points - final exam PBL2
</commit_message>
<xml_diff>
--- a/IoT-points-schedule.xlsx
+++ b/IoT-points-schedule.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\dodo\Desktop\IoT-studies\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BF0EE2A9-3B2E-4037-8903-BB049E272633}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{69F574BF-2489-4E09-8598-D6F07679B0E8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="25440" windowHeight="15390" xr2:uid="{F85F5544-1FE8-4920-A5D4-192A98B113BD}"/>
   </bookViews>
@@ -1068,7 +1068,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="80">
+  <cellXfs count="74">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1116,22 +1116,6 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1">
-      <extLst>
-        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
-          <xfpb:xfComplement i="0"/>
-        </ext>
-      </extLst>
-    </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
@@ -1215,39 +1199,54 @@
     <xf numFmtId="0" fontId="7" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="6" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="6" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="6" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="6" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="6" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="6" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1266,33 +1265,18 @@
     <xf numFmtId="0" fontId="5" fillId="4" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="2" fontId="2" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="2" fontId="2" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1310,12 +1294,6 @@
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1705,60 +1683,60 @@
   <sheetData>
     <row r="1" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="2" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B2" s="57" t="s">
+      <c r="B2" s="58" t="s">
         <v>76</v>
       </c>
-      <c r="C2" s="58"/>
-      <c r="D2" s="58"/>
-      <c r="E2" s="58"/>
-      <c r="F2" s="58"/>
-      <c r="G2" s="58"/>
-      <c r="H2" s="58"/>
-      <c r="I2" s="58"/>
-      <c r="J2" s="58"/>
-      <c r="K2" s="58"/>
-      <c r="L2" s="58"/>
-      <c r="M2" s="58"/>
-      <c r="N2" s="58"/>
-      <c r="O2" s="58"/>
-      <c r="P2" s="59"/>
+      <c r="C2" s="59"/>
+      <c r="D2" s="59"/>
+      <c r="E2" s="59"/>
+      <c r="F2" s="59"/>
+      <c r="G2" s="59"/>
+      <c r="H2" s="59"/>
+      <c r="I2" s="59"/>
+      <c r="J2" s="59"/>
+      <c r="K2" s="59"/>
+      <c r="L2" s="59"/>
+      <c r="M2" s="59"/>
+      <c r="N2" s="59"/>
+      <c r="O2" s="59"/>
+      <c r="P2" s="60"/>
     </row>
     <row r="3" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B3" s="60"/>
-      <c r="C3" s="61"/>
-      <c r="D3" s="61"/>
-      <c r="E3" s="61"/>
-      <c r="F3" s="61"/>
-      <c r="G3" s="61"/>
-      <c r="H3" s="61"/>
-      <c r="I3" s="61"/>
-      <c r="J3" s="61"/>
-      <c r="K3" s="61"/>
-      <c r="L3" s="61"/>
-      <c r="M3" s="61"/>
-      <c r="N3" s="61"/>
-      <c r="O3" s="61"/>
-      <c r="P3" s="62"/>
+      <c r="B3" s="61"/>
+      <c r="C3" s="62"/>
+      <c r="D3" s="62"/>
+      <c r="E3" s="62"/>
+      <c r="F3" s="62"/>
+      <c r="G3" s="62"/>
+      <c r="H3" s="62"/>
+      <c r="I3" s="62"/>
+      <c r="J3" s="62"/>
+      <c r="K3" s="62"/>
+      <c r="L3" s="62"/>
+      <c r="M3" s="62"/>
+      <c r="N3" s="62"/>
+      <c r="O3" s="62"/>
+      <c r="P3" s="63"/>
       <c r="R3" s="12"/>
     </row>
     <row r="5" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B5" s="54" t="s">
+      <c r="B5" s="42" t="s">
         <v>83</v>
       </c>
-      <c r="C5" s="55"/>
-      <c r="D5" s="55"/>
-      <c r="E5" s="55"/>
-      <c r="F5" s="56"/>
-      <c r="H5" s="54" t="s">
+      <c r="C5" s="57"/>
+      <c r="D5" s="57"/>
+      <c r="E5" s="57"/>
+      <c r="F5" s="43"/>
+      <c r="H5" s="42" t="s">
         <v>82</v>
       </c>
-      <c r="I5" s="56"/>
-      <c r="K5" s="54" t="s">
+      <c r="I5" s="43"/>
+      <c r="K5" s="42" t="s">
         <v>8</v>
       </c>
-      <c r="L5" s="55"/>
-      <c r="M5" s="55"/>
-      <c r="N5" s="56"/>
+      <c r="L5" s="57"/>
+      <c r="M5" s="57"/>
+      <c r="N5" s="43"/>
       <c r="P5" s="4" t="s">
         <v>74</v>
       </c>
@@ -1826,7 +1804,9 @@
       <c r="K7" s="2">
         <v>12</v>
       </c>
-      <c r="L7" s="2"/>
+      <c r="L7" s="2">
+        <v>13.5</v>
+      </c>
       <c r="M7" s="2"/>
       <c r="N7" s="2">
         <v>6</v>
@@ -1834,37 +1814,37 @@
       <c r="P7" s="2"/>
     </row>
     <row r="9" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B9" s="63" t="s">
+      <c r="B9" s="52" t="s">
         <v>22</v>
       </c>
-      <c r="C9" s="63"/>
+      <c r="C9" s="52"/>
       <c r="E9" s="9" t="s">
         <v>67</v>
       </c>
-      <c r="G9" s="63" t="s">
+      <c r="G9" s="52" t="s">
         <v>87</v>
       </c>
-      <c r="H9" s="63"/>
+      <c r="H9" s="52"/>
     </row>
     <row r="10" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B10" s="46">
+      <c r="B10" s="53">
         <f>SUM(B7:F7,H7:I7,K7:N7,P7)</f>
-        <v>41.6</v>
-      </c>
-      <c r="C10" s="46"/>
-      <c r="E10" s="67"/>
-      <c r="G10" s="46">
+        <v>55.1</v>
+      </c>
+      <c r="C10" s="53"/>
+      <c r="E10" s="55"/>
+      <c r="G10" s="53">
         <f>66-SUM(B7:F7,H7:I7,K7:N7,P7)</f>
-        <v>24.4</v>
-      </c>
-      <c r="H10" s="46"/>
+        <v>10.899999999999999</v>
+      </c>
+      <c r="H10" s="53"/>
     </row>
     <row r="11" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B11" s="46"/>
-      <c r="C11" s="46"/>
-      <c r="E11" s="68"/>
-      <c r="G11" s="46"/>
-      <c r="H11" s="46"/>
+      <c r="B11" s="53"/>
+      <c r="C11" s="53"/>
+      <c r="E11" s="56"/>
+      <c r="G11" s="53"/>
+      <c r="H11" s="53"/>
     </row>
     <row r="12" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A12" s="6"/>
@@ -1889,46 +1869,46 @@
     </row>
     <row r="13" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="14" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B14" s="48" t="s">
+      <c r="B14" s="44" t="s">
         <v>77</v>
       </c>
-      <c r="C14" s="49"/>
-      <c r="D14" s="49"/>
-      <c r="E14" s="49"/>
-      <c r="F14" s="49"/>
-      <c r="G14" s="49"/>
-      <c r="H14" s="50"/>
+      <c r="C14" s="45"/>
+      <c r="D14" s="45"/>
+      <c r="E14" s="45"/>
+      <c r="F14" s="45"/>
+      <c r="G14" s="45"/>
+      <c r="H14" s="46"/>
     </row>
     <row r="15" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B15" s="51"/>
-      <c r="C15" s="52"/>
-      <c r="D15" s="52"/>
-      <c r="E15" s="52"/>
-      <c r="F15" s="52"/>
-      <c r="G15" s="52"/>
-      <c r="H15" s="53"/>
+      <c r="B15" s="47"/>
+      <c r="C15" s="48"/>
+      <c r="D15" s="48"/>
+      <c r="E15" s="48"/>
+      <c r="F15" s="48"/>
+      <c r="G15" s="48"/>
+      <c r="H15" s="49"/>
     </row>
     <row r="17" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B17" s="66" t="s">
+      <c r="B17" s="50" t="s">
         <v>91</v>
       </c>
-      <c r="C17" s="66"/>
-      <c r="D17" s="66"/>
-      <c r="E17" s="66"/>
-      <c r="F17" s="66"/>
-      <c r="H17" s="54" t="s">
+      <c r="C17" s="50"/>
+      <c r="D17" s="50"/>
+      <c r="E17" s="50"/>
+      <c r="F17" s="50"/>
+      <c r="H17" s="42" t="s">
         <v>97</v>
       </c>
-      <c r="I17" s="55"/>
-      <c r="J17" s="56"/>
-      <c r="L17" s="63" t="s">
+      <c r="I17" s="57"/>
+      <c r="J17" s="43"/>
+      <c r="L17" s="52" t="s">
         <v>22</v>
       </c>
-      <c r="M17" s="63"/>
+      <c r="M17" s="52"/>
       <c r="O17" s="9" t="s">
         <v>67</v>
       </c>
-      <c r="P17" s="38"/>
+      <c r="P17" s="34"/>
     </row>
     <row r="18" spans="1:19" ht="48.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B18" s="3" t="s">
@@ -1955,12 +1935,12 @@
       <c r="J18" s="3" t="s">
         <v>95</v>
       </c>
-      <c r="L18" s="46">
+      <c r="L18" s="53">
         <f>SUM(B19:F19,H19:J19)</f>
         <v>85</v>
       </c>
-      <c r="M18" s="46"/>
-      <c r="O18" s="47">
+      <c r="M18" s="53"/>
+      <c r="O18" s="54">
         <v>4.5</v>
       </c>
     </row>
@@ -1989,9 +1969,9 @@
       <c r="J19" s="2">
         <v>19.5</v>
       </c>
-      <c r="L19" s="46"/>
-      <c r="M19" s="46"/>
-      <c r="O19" s="47"/>
+      <c r="L19" s="53"/>
+      <c r="M19" s="53"/>
+      <c r="O19" s="54"/>
     </row>
     <row r="21" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A21" s="6"/>
@@ -2016,62 +1996,62 @@
     </row>
     <row r="22" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="23" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B23" s="48" t="s">
+      <c r="B23" s="44" t="s">
         <v>79</v>
       </c>
-      <c r="C23" s="49"/>
-      <c r="D23" s="49"/>
-      <c r="E23" s="49"/>
-      <c r="F23" s="49"/>
-      <c r="G23" s="49"/>
-      <c r="H23" s="49"/>
-      <c r="I23" s="49"/>
-      <c r="J23" s="49"/>
-      <c r="K23" s="49"/>
-      <c r="L23" s="50"/>
-      <c r="N23" s="46" t="s">
+      <c r="C23" s="45"/>
+      <c r="D23" s="45"/>
+      <c r="E23" s="45"/>
+      <c r="F23" s="45"/>
+      <c r="G23" s="45"/>
+      <c r="H23" s="45"/>
+      <c r="I23" s="45"/>
+      <c r="J23" s="45"/>
+      <c r="K23" s="45"/>
+      <c r="L23" s="46"/>
+      <c r="N23" s="53" t="s">
         <v>120</v>
       </c>
-      <c r="O23" s="46"/>
+      <c r="O23" s="53"/>
       <c r="Q23" s="7"/>
       <c r="R23" s="7"/>
       <c r="S23" s="7"/>
     </row>
     <row r="24" spans="1:19" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B24" s="51"/>
-      <c r="C24" s="52"/>
-      <c r="D24" s="52"/>
-      <c r="E24" s="52"/>
-      <c r="F24" s="52"/>
-      <c r="G24" s="52"/>
-      <c r="H24" s="52"/>
-      <c r="I24" s="52"/>
-      <c r="J24" s="52"/>
-      <c r="K24" s="52"/>
-      <c r="L24" s="53"/>
-      <c r="N24" s="46"/>
-      <c r="O24" s="46"/>
+      <c r="B24" s="47"/>
+      <c r="C24" s="48"/>
+      <c r="D24" s="48"/>
+      <c r="E24" s="48"/>
+      <c r="F24" s="48"/>
+      <c r="G24" s="48"/>
+      <c r="H24" s="48"/>
+      <c r="I24" s="48"/>
+      <c r="J24" s="48"/>
+      <c r="K24" s="48"/>
+      <c r="L24" s="49"/>
+      <c r="N24" s="53"/>
+      <c r="O24" s="53"/>
       <c r="Q24" s="7"/>
       <c r="R24" s="7"/>
       <c r="S24" s="7"/>
     </row>
     <row r="26" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B26" s="66" t="s">
+      <c r="B26" s="50" t="s">
         <v>8</v>
       </c>
-      <c r="C26" s="66"/>
-      <c r="D26" s="66"/>
-      <c r="F26" s="66" t="s">
+      <c r="C26" s="50"/>
+      <c r="D26" s="50"/>
+      <c r="F26" s="50" t="s">
         <v>199</v>
       </c>
-      <c r="G26" s="66"/>
-      <c r="H26" s="66"/>
-      <c r="I26" s="66"/>
+      <c r="G26" s="50"/>
+      <c r="H26" s="50"/>
+      <c r="I26" s="50"/>
       <c r="J26" s="7"/>
-      <c r="K26" s="54" t="s">
+      <c r="K26" s="42" t="s">
         <v>119</v>
       </c>
-      <c r="L26" s="56"/>
+      <c r="L26" s="43"/>
       <c r="N26" s="9" t="s">
         <v>67</v>
       </c>
@@ -2104,9 +2084,9 @@
       <c r="L27" s="2" t="s">
         <v>118</v>
       </c>
-      <c r="N27" s="69">
+      <c r="N27" s="66">
         <f>(K29/30*0.4*5)+(B29/25*0.3*5)+(0.3*F29)</f>
-        <v>4.2133333333333329</v>
+        <v>4.2733333333333334</v>
       </c>
     </row>
     <row r="28" spans="1:19" x14ac:dyDescent="0.25">
@@ -2135,27 +2115,27 @@
         <v>20</v>
       </c>
       <c r="L28" s="2"/>
-      <c r="N28" s="70"/>
+      <c r="N28" s="67"/>
     </row>
     <row r="29" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B29" s="71">
-        <f>SUM(B28:C28)</f>
-        <v>23</v>
-      </c>
-      <c r="C29" s="71"/>
-      <c r="D29" s="71"/>
-      <c r="F29" s="71">
+      <c r="B29" s="51">
+        <f>SUM(B28:D28)</f>
+        <v>24</v>
+      </c>
+      <c r="C29" s="51"/>
+      <c r="D29" s="51"/>
+      <c r="F29" s="51">
         <v>5</v>
       </c>
-      <c r="G29" s="71"/>
-      <c r="H29" s="71"/>
-      <c r="I29" s="71"/>
-      <c r="K29" s="71">
+      <c r="G29" s="51"/>
+      <c r="H29" s="51"/>
+      <c r="I29" s="51"/>
+      <c r="K29" s="51">
         <f>SUM(K28:L28)</f>
         <v>20</v>
       </c>
-      <c r="L29" s="71"/>
-      <c r="N29" s="38"/>
+      <c r="L29" s="51"/>
+      <c r="N29" s="34"/>
     </row>
     <row r="31" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A31" s="6"/>
@@ -2180,39 +2160,39 @@
     </row>
     <row r="32" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="33" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B33" s="48" t="s">
+      <c r="B33" s="44" t="s">
         <v>78</v>
       </c>
-      <c r="C33" s="49"/>
-      <c r="D33" s="49"/>
-      <c r="E33" s="49"/>
-      <c r="F33" s="49"/>
-      <c r="G33" s="49"/>
-      <c r="H33" s="49"/>
-      <c r="I33" s="50"/>
+      <c r="C33" s="45"/>
+      <c r="D33" s="45"/>
+      <c r="E33" s="45"/>
+      <c r="F33" s="45"/>
+      <c r="G33" s="45"/>
+      <c r="H33" s="45"/>
+      <c r="I33" s="46"/>
     </row>
     <row r="34" spans="2:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B34" s="51"/>
-      <c r="C34" s="52"/>
-      <c r="D34" s="52"/>
-      <c r="E34" s="52"/>
-      <c r="F34" s="52"/>
-      <c r="G34" s="52"/>
-      <c r="H34" s="52"/>
-      <c r="I34" s="53"/>
+      <c r="B34" s="47"/>
+      <c r="C34" s="48"/>
+      <c r="D34" s="48"/>
+      <c r="E34" s="48"/>
+      <c r="F34" s="48"/>
+      <c r="G34" s="48"/>
+      <c r="H34" s="48"/>
+      <c r="I34" s="49"/>
     </row>
     <row r="36" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B36" s="66" t="s">
+      <c r="B36" s="50" t="s">
         <v>98</v>
       </c>
-      <c r="C36" s="66"/>
+      <c r="C36" s="50"/>
       <c r="D36" s="7"/>
-      <c r="E36" s="54" t="s">
+      <c r="E36" s="42" t="s">
         <v>135</v>
       </c>
-      <c r="F36" s="55"/>
-      <c r="G36" s="55"/>
-      <c r="H36" s="56"/>
+      <c r="F36" s="57"/>
+      <c r="G36" s="57"/>
+      <c r="H36" s="43"/>
     </row>
     <row r="37" spans="2:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B37" s="2" t="s">
@@ -2259,10 +2239,10 @@
         <v>117</v>
       </c>
       <c r="C41" s="65"/>
-      <c r="F41" s="46" t="s">
+      <c r="F41" s="53" t="s">
         <v>102</v>
       </c>
-      <c r="G41" s="46"/>
+      <c r="G41" s="53"/>
       <c r="I41" s="9" t="s">
         <v>22</v>
       </c>
@@ -2318,7 +2298,7 @@
       <c r="G44" s="2">
         <v>10</v>
       </c>
-      <c r="I44" s="63" t="s">
+      <c r="I44" s="52" t="s">
         <v>67</v>
       </c>
     </row>
@@ -2329,7 +2309,7 @@
       <c r="C45" s="2">
         <v>4</v>
       </c>
-      <c r="I45" s="63"/>
+      <c r="I45" s="52"/>
     </row>
     <row r="46" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B46" s="2" t="s">
@@ -2362,7 +2342,7 @@
       <c r="C48" s="2">
         <v>2</v>
       </c>
-      <c r="I48" s="38"/>
+      <c r="I48" s="34"/>
     </row>
     <row r="49" spans="1:19" x14ac:dyDescent="0.25">
       <c r="B49" s="2" t="s">
@@ -2426,70 +2406,70 @@
     </row>
     <row r="57" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="58" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B58" s="48" t="s">
+      <c r="B58" s="44" t="s">
         <v>80</v>
       </c>
-      <c r="C58" s="49"/>
-      <c r="D58" s="49"/>
-      <c r="E58" s="49"/>
-      <c r="F58" s="49"/>
-      <c r="G58" s="49"/>
-      <c r="H58" s="49"/>
-      <c r="I58" s="49"/>
-      <c r="J58" s="49"/>
-      <c r="K58" s="49"/>
-      <c r="L58" s="49"/>
-      <c r="M58" s="49"/>
-      <c r="N58" s="49"/>
-      <c r="O58" s="49"/>
-      <c r="P58" s="49"/>
-      <c r="Q58" s="49"/>
-      <c r="R58" s="49"/>
-      <c r="S58" s="50"/>
+      <c r="C58" s="45"/>
+      <c r="D58" s="45"/>
+      <c r="E58" s="45"/>
+      <c r="F58" s="45"/>
+      <c r="G58" s="45"/>
+      <c r="H58" s="45"/>
+      <c r="I58" s="45"/>
+      <c r="J58" s="45"/>
+      <c r="K58" s="45"/>
+      <c r="L58" s="45"/>
+      <c r="M58" s="45"/>
+      <c r="N58" s="45"/>
+      <c r="O58" s="45"/>
+      <c r="P58" s="45"/>
+      <c r="Q58" s="45"/>
+      <c r="R58" s="45"/>
+      <c r="S58" s="46"/>
     </row>
     <row r="59" spans="1:19" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B59" s="51"/>
-      <c r="C59" s="52"/>
-      <c r="D59" s="52"/>
-      <c r="E59" s="52"/>
-      <c r="F59" s="52"/>
-      <c r="G59" s="52"/>
-      <c r="H59" s="52"/>
-      <c r="I59" s="52"/>
-      <c r="J59" s="52"/>
-      <c r="K59" s="52"/>
-      <c r="L59" s="52"/>
-      <c r="M59" s="52"/>
-      <c r="N59" s="52"/>
-      <c r="O59" s="52"/>
-      <c r="P59" s="52"/>
-      <c r="Q59" s="52"/>
-      <c r="R59" s="52"/>
-      <c r="S59" s="53"/>
+      <c r="B59" s="47"/>
+      <c r="C59" s="48"/>
+      <c r="D59" s="48"/>
+      <c r="E59" s="48"/>
+      <c r="F59" s="48"/>
+      <c r="G59" s="48"/>
+      <c r="H59" s="48"/>
+      <c r="I59" s="48"/>
+      <c r="J59" s="48"/>
+      <c r="K59" s="48"/>
+      <c r="L59" s="48"/>
+      <c r="M59" s="48"/>
+      <c r="N59" s="48"/>
+      <c r="O59" s="48"/>
+      <c r="P59" s="48"/>
+      <c r="Q59" s="48"/>
+      <c r="R59" s="48"/>
+      <c r="S59" s="49"/>
     </row>
     <row r="61" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B61" s="66" t="s">
+      <c r="B61" s="50" t="s">
         <v>63</v>
       </c>
-      <c r="C61" s="66"/>
-      <c r="D61" s="66"/>
-      <c r="E61" s="66"/>
-      <c r="F61" s="66"/>
-      <c r="G61" s="66"/>
-      <c r="H61" s="66"/>
-      <c r="I61" s="66"/>
-      <c r="J61" s="66"/>
-      <c r="K61" s="66"/>
-      <c r="M61" s="66" t="s">
+      <c r="C61" s="50"/>
+      <c r="D61" s="50"/>
+      <c r="E61" s="50"/>
+      <c r="F61" s="50"/>
+      <c r="G61" s="50"/>
+      <c r="H61" s="50"/>
+      <c r="I61" s="50"/>
+      <c r="J61" s="50"/>
+      <c r="K61" s="50"/>
+      <c r="M61" s="50" t="s">
         <v>90</v>
       </c>
-      <c r="N61" s="66"/>
-      <c r="O61" s="66"/>
-      <c r="P61" s="66"/>
-      <c r="R61" s="66" t="s">
+      <c r="N61" s="50"/>
+      <c r="O61" s="50"/>
+      <c r="P61" s="50"/>
+      <c r="R61" s="50" t="s">
         <v>64</v>
       </c>
-      <c r="S61" s="66"/>
+      <c r="S61" s="50"/>
     </row>
     <row r="62" spans="1:19" x14ac:dyDescent="0.25">
       <c r="B62" s="2" t="s">
@@ -2584,66 +2564,49 @@
       <c r="P63" s="2">
         <v>20</v>
       </c>
-      <c r="R63" s="2"/>
-      <c r="S63" s="2"/>
+      <c r="R63" s="2">
+        <v>25</v>
+      </c>
+      <c r="S63" s="2">
+        <v>8</v>
+      </c>
     </row>
     <row r="66" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B66" s="63" t="s">
+      <c r="B66" s="52" t="s">
         <v>22</v>
       </c>
-      <c r="C66" s="63"/>
+      <c r="C66" s="52"/>
       <c r="E66" s="9" t="s">
         <v>67</v>
       </c>
-      <c r="G66" s="39" t="s">
+      <c r="G66" s="35" t="s">
         <v>214</v>
       </c>
-      <c r="H66" s="78"/>
+      <c r="H66" s="11"/>
     </row>
     <row r="67" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B67" s="46">
+      <c r="B67" s="53">
         <f>SUM(B63:K63,M63:P63,R63:S63,G67)</f>
-        <v>65</v>
-      </c>
-      <c r="C67" s="46"/>
-      <c r="E67" s="47"/>
-      <c r="G67" s="46">
+        <v>98</v>
+      </c>
+      <c r="C67" s="53"/>
+      <c r="E67" s="54">
+        <v>5</v>
+      </c>
+      <c r="G67" s="53">
         <v>9</v>
       </c>
-      <c r="H67" s="79"/>
+      <c r="H67" s="7"/>
     </row>
     <row r="68" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B68" s="46"/>
-      <c r="C68" s="46"/>
-      <c r="E68" s="47"/>
-      <c r="G68" s="46"/>
-      <c r="H68" s="79"/>
+      <c r="B68" s="53"/>
+      <c r="C68" s="53"/>
+      <c r="E68" s="54"/>
+      <c r="G68" s="53"/>
+      <c r="H68" s="7"/>
     </row>
   </sheetData>
   <mergeCells count="38">
-    <mergeCell ref="K29:L29"/>
-    <mergeCell ref="R61:S61"/>
-    <mergeCell ref="B33:I34"/>
-    <mergeCell ref="B61:K61"/>
-    <mergeCell ref="B58:S59"/>
-    <mergeCell ref="M61:P61"/>
-    <mergeCell ref="F29:I29"/>
-    <mergeCell ref="B29:D29"/>
-    <mergeCell ref="N27:N28"/>
-    <mergeCell ref="F26:I26"/>
-    <mergeCell ref="K26:L26"/>
-    <mergeCell ref="B23:L24"/>
-    <mergeCell ref="B26:D26"/>
-    <mergeCell ref="L17:M17"/>
-    <mergeCell ref="E10:E11"/>
-    <mergeCell ref="G10:H11"/>
-    <mergeCell ref="B17:F17"/>
-    <mergeCell ref="H17:J17"/>
-    <mergeCell ref="B66:C66"/>
-    <mergeCell ref="B67:C68"/>
-    <mergeCell ref="B9:C9"/>
-    <mergeCell ref="B10:C11"/>
-    <mergeCell ref="G67:G68"/>
     <mergeCell ref="O18:O19"/>
     <mergeCell ref="B14:H15"/>
     <mergeCell ref="K5:N5"/>
@@ -2658,7 +2621,30 @@
     <mergeCell ref="B36:C36"/>
     <mergeCell ref="E36:H36"/>
     <mergeCell ref="G9:H9"/>
+    <mergeCell ref="L17:M17"/>
+    <mergeCell ref="N27:N28"/>
+    <mergeCell ref="B66:C66"/>
+    <mergeCell ref="B67:C68"/>
+    <mergeCell ref="B9:C9"/>
+    <mergeCell ref="B10:C11"/>
+    <mergeCell ref="G67:G68"/>
     <mergeCell ref="E67:E68"/>
+    <mergeCell ref="E10:E11"/>
+    <mergeCell ref="G10:H11"/>
+    <mergeCell ref="B17:F17"/>
+    <mergeCell ref="H17:J17"/>
+    <mergeCell ref="F26:I26"/>
+    <mergeCell ref="K26:L26"/>
+    <mergeCell ref="B23:L24"/>
+    <mergeCell ref="B26:D26"/>
+    <mergeCell ref="K29:L29"/>
+    <mergeCell ref="R61:S61"/>
+    <mergeCell ref="B33:I34"/>
+    <mergeCell ref="B61:K61"/>
+    <mergeCell ref="B58:S59"/>
+    <mergeCell ref="M61:P61"/>
+    <mergeCell ref="F29:I29"/>
+    <mergeCell ref="B29:D29"/>
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2694,60 +2680,60 @@
   <sheetData>
     <row r="1" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="2" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B2" s="48" t="s">
+      <c r="B2" s="44" t="s">
         <v>121</v>
       </c>
-      <c r="C2" s="49"/>
-      <c r="D2" s="49"/>
-      <c r="E2" s="49"/>
-      <c r="F2" s="49"/>
-      <c r="G2" s="49"/>
-      <c r="H2" s="49"/>
-      <c r="I2" s="49"/>
-      <c r="J2" s="49"/>
-      <c r="K2" s="49"/>
-      <c r="L2" s="49"/>
-      <c r="M2" s="49"/>
-      <c r="N2" s="49"/>
-      <c r="O2" s="49"/>
-      <c r="P2" s="50"/>
+      <c r="C2" s="45"/>
+      <c r="D2" s="45"/>
+      <c r="E2" s="45"/>
+      <c r="F2" s="45"/>
+      <c r="G2" s="45"/>
+      <c r="H2" s="45"/>
+      <c r="I2" s="45"/>
+      <c r="J2" s="45"/>
+      <c r="K2" s="45"/>
+      <c r="L2" s="45"/>
+      <c r="M2" s="45"/>
+      <c r="N2" s="45"/>
+      <c r="O2" s="45"/>
+      <c r="P2" s="46"/>
     </row>
     <row r="3" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B3" s="51"/>
-      <c r="C3" s="52"/>
-      <c r="D3" s="52"/>
-      <c r="E3" s="52"/>
-      <c r="F3" s="52"/>
-      <c r="G3" s="52"/>
-      <c r="H3" s="52"/>
-      <c r="I3" s="52"/>
-      <c r="J3" s="52"/>
-      <c r="K3" s="52"/>
-      <c r="L3" s="52"/>
-      <c r="M3" s="52"/>
-      <c r="N3" s="52"/>
-      <c r="O3" s="52"/>
-      <c r="P3" s="53"/>
+      <c r="B3" s="47"/>
+      <c r="C3" s="48"/>
+      <c r="D3" s="48"/>
+      <c r="E3" s="48"/>
+      <c r="F3" s="48"/>
+      <c r="G3" s="48"/>
+      <c r="H3" s="48"/>
+      <c r="I3" s="48"/>
+      <c r="J3" s="48"/>
+      <c r="K3" s="48"/>
+      <c r="L3" s="48"/>
+      <c r="M3" s="48"/>
+      <c r="N3" s="48"/>
+      <c r="O3" s="48"/>
+      <c r="P3" s="49"/>
       <c r="R3" s="12"/>
     </row>
     <row r="5" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B5" s="66" t="s">
+      <c r="B5" s="50" t="s">
         <v>18</v>
       </c>
-      <c r="C5" s="66"/>
-      <c r="D5" s="66"/>
-      <c r="E5" s="66"/>
-      <c r="F5" s="66"/>
-      <c r="G5" s="66"/>
+      <c r="C5" s="50"/>
+      <c r="D5" s="50"/>
+      <c r="E5" s="50"/>
+      <c r="F5" s="50"/>
+      <c r="G5" s="50"/>
       <c r="I5" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="K5" s="54" t="s">
+      <c r="K5" s="42" t="s">
         <v>8</v>
       </c>
-      <c r="L5" s="55"/>
-      <c r="M5" s="55"/>
-      <c r="N5" s="56"/>
+      <c r="L5" s="57"/>
+      <c r="M5" s="57"/>
+      <c r="N5" s="43"/>
       <c r="P5" s="4" t="s">
         <v>74</v>
       </c>
@@ -2829,28 +2815,28 @@
       </c>
     </row>
     <row r="9" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B9" s="63" t="s">
+      <c r="B9" s="52" t="s">
         <v>22</v>
       </c>
-      <c r="C9" s="63"/>
+      <c r="C9" s="52"/>
       <c r="E9" s="9" t="s">
         <v>67</v>
       </c>
     </row>
     <row r="10" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B10" s="46">
+      <c r="B10" s="53">
         <f>_xlfn.CEILING.MATH(SUM(B7:G7,I7,K7:N7,P7),1,1)</f>
         <v>110</v>
       </c>
-      <c r="C10" s="46"/>
-      <c r="E10" s="67">
+      <c r="C10" s="53"/>
+      <c r="E10" s="55">
         <v>4</v>
       </c>
     </row>
     <row r="11" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B11" s="46"/>
-      <c r="C11" s="46"/>
-      <c r="E11" s="68"/>
+      <c r="B11" s="53"/>
+      <c r="C11" s="53"/>
+      <c r="E11" s="56"/>
     </row>
     <row r="12" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A12" s="6"/>
@@ -2875,40 +2861,40 @@
     </row>
     <row r="13" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="14" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B14" s="48" t="s">
+      <c r="B14" s="44" t="s">
         <v>122</v>
       </c>
-      <c r="C14" s="49"/>
-      <c r="D14" s="49"/>
-      <c r="E14" s="49"/>
-      <c r="F14" s="49"/>
-      <c r="G14" s="49"/>
-      <c r="H14" s="50"/>
+      <c r="C14" s="45"/>
+      <c r="D14" s="45"/>
+      <c r="E14" s="45"/>
+      <c r="F14" s="45"/>
+      <c r="G14" s="45"/>
+      <c r="H14" s="46"/>
     </row>
     <row r="15" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B15" s="51"/>
-      <c r="C15" s="52"/>
-      <c r="D15" s="52"/>
-      <c r="E15" s="52"/>
-      <c r="F15" s="52"/>
-      <c r="G15" s="52"/>
-      <c r="H15" s="53"/>
+      <c r="B15" s="47"/>
+      <c r="C15" s="48"/>
+      <c r="D15" s="48"/>
+      <c r="E15" s="48"/>
+      <c r="F15" s="48"/>
+      <c r="G15" s="48"/>
+      <c r="H15" s="49"/>
     </row>
     <row r="17" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B17" s="66" t="s">
+      <c r="B17" s="50" t="s">
         <v>12</v>
       </c>
-      <c r="C17" s="66"/>
-      <c r="D17" s="66"/>
-      <c r="F17" s="66" t="s">
+      <c r="C17" s="50"/>
+      <c r="D17" s="50"/>
+      <c r="F17" s="50" t="s">
         <v>8</v>
       </c>
-      <c r="G17" s="66"/>
-      <c r="H17" s="66"/>
-      <c r="J17" s="63" t="s">
+      <c r="G17" s="50"/>
+      <c r="H17" s="50"/>
+      <c r="J17" s="52" t="s">
         <v>22</v>
       </c>
-      <c r="K17" s="63"/>
+      <c r="K17" s="52"/>
       <c r="M17" s="9" t="s">
         <v>67</v>
       </c>
@@ -2932,12 +2918,12 @@
       <c r="H18" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="J18" s="46">
+      <c r="J18" s="53">
         <f>SUM(B19:D19,F19:H19)</f>
         <v>93</v>
       </c>
-      <c r="K18" s="46"/>
-      <c r="M18" s="47">
+      <c r="K18" s="53"/>
+      <c r="M18" s="54">
         <v>5</v>
       </c>
     </row>
@@ -2960,9 +2946,9 @@
       <c r="H19" s="2">
         <v>4</v>
       </c>
-      <c r="J19" s="46"/>
-      <c r="K19" s="46"/>
-      <c r="M19" s="47"/>
+      <c r="J19" s="53"/>
+      <c r="K19" s="53"/>
+      <c r="M19" s="54"/>
     </row>
     <row r="21" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A21" s="6"/>
@@ -2987,46 +2973,46 @@
     </row>
     <row r="22" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="23" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B23" s="48" t="s">
+      <c r="B23" s="44" t="s">
         <v>123</v>
       </c>
-      <c r="C23" s="49"/>
-      <c r="D23" s="49"/>
-      <c r="E23" s="49"/>
-      <c r="F23" s="49"/>
-      <c r="G23" s="49"/>
-      <c r="H23" s="49"/>
-      <c r="I23" s="49"/>
-      <c r="J23" s="49"/>
-      <c r="K23" s="50"/>
+      <c r="C23" s="45"/>
+      <c r="D23" s="45"/>
+      <c r="E23" s="45"/>
+      <c r="F23" s="45"/>
+      <c r="G23" s="45"/>
+      <c r="H23" s="45"/>
+      <c r="I23" s="45"/>
+      <c r="J23" s="45"/>
+      <c r="K23" s="46"/>
     </row>
     <row r="24" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B24" s="51"/>
-      <c r="C24" s="52"/>
-      <c r="D24" s="52"/>
-      <c r="E24" s="52"/>
-      <c r="F24" s="52"/>
-      <c r="G24" s="52"/>
-      <c r="H24" s="52"/>
-      <c r="I24" s="52"/>
-      <c r="J24" s="52"/>
-      <c r="K24" s="53"/>
+      <c r="B24" s="47"/>
+      <c r="C24" s="48"/>
+      <c r="D24" s="48"/>
+      <c r="E24" s="48"/>
+      <c r="F24" s="48"/>
+      <c r="G24" s="48"/>
+      <c r="H24" s="48"/>
+      <c r="I24" s="48"/>
+      <c r="J24" s="48"/>
+      <c r="K24" s="49"/>
     </row>
     <row r="26" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B26" s="66" t="s">
+      <c r="B26" s="50" t="s">
         <v>17</v>
       </c>
-      <c r="C26" s="66"/>
-      <c r="E26" s="54" t="s">
+      <c r="C26" s="50"/>
+      <c r="E26" s="42" t="s">
         <v>21</v>
       </c>
-      <c r="F26" s="55"/>
-      <c r="G26" s="56"/>
-      <c r="I26" s="66" t="s">
+      <c r="F26" s="57"/>
+      <c r="G26" s="43"/>
+      <c r="I26" s="50" t="s">
         <v>20</v>
       </c>
-      <c r="J26" s="66"/>
-      <c r="K26" s="66"/>
+      <c r="J26" s="50"/>
+      <c r="K26" s="50"/>
       <c r="M26" s="10" t="s">
         <v>22</v>
       </c>
@@ -3061,12 +3047,12 @@
       <c r="K27" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="M27" s="72">
+      <c r="M27" s="68">
         <f>SUM(B28:C28,E28:G28,I28:K28)</f>
         <v>36</v>
       </c>
       <c r="N27" s="7"/>
-      <c r="O27" s="47">
+      <c r="O27" s="54">
         <v>4</v>
       </c>
       <c r="P27" s="8"/>
@@ -3096,9 +3082,9 @@
       <c r="K28" s="2">
         <v>3.2</v>
       </c>
-      <c r="M28" s="72"/>
+      <c r="M28" s="68"/>
       <c r="N28" s="7"/>
-      <c r="O28" s="47"/>
+      <c r="O28" s="54"/>
       <c r="P28" s="8"/>
     </row>
     <row r="30" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -3124,39 +3110,39 @@
     </row>
     <row r="31" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="32" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B32" s="48" t="s">
+      <c r="B32" s="44" t="s">
         <v>124</v>
       </c>
-      <c r="C32" s="49"/>
-      <c r="D32" s="49"/>
-      <c r="E32" s="49"/>
-      <c r="F32" s="49"/>
-      <c r="G32" s="49"/>
-      <c r="H32" s="49"/>
-      <c r="I32" s="50"/>
+      <c r="C32" s="45"/>
+      <c r="D32" s="45"/>
+      <c r="E32" s="45"/>
+      <c r="F32" s="45"/>
+      <c r="G32" s="45"/>
+      <c r="H32" s="45"/>
+      <c r="I32" s="46"/>
     </row>
     <row r="33" spans="2:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B33" s="51"/>
-      <c r="C33" s="52"/>
-      <c r="D33" s="52"/>
-      <c r="E33" s="52"/>
-      <c r="F33" s="52"/>
-      <c r="G33" s="52"/>
-      <c r="H33" s="52"/>
-      <c r="I33" s="53"/>
+      <c r="B33" s="47"/>
+      <c r="C33" s="48"/>
+      <c r="D33" s="48"/>
+      <c r="E33" s="48"/>
+      <c r="F33" s="48"/>
+      <c r="G33" s="48"/>
+      <c r="H33" s="48"/>
+      <c r="I33" s="49"/>
     </row>
     <row r="35" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B35" s="66" t="s">
+      <c r="B35" s="50" t="s">
         <v>31</v>
       </c>
-      <c r="C35" s="66"/>
-      <c r="D35" s="66"/>
-      <c r="F35" s="66" t="s">
+      <c r="C35" s="50"/>
+      <c r="D35" s="50"/>
+      <c r="F35" s="50" t="s">
         <v>12</v>
       </c>
-      <c r="G35" s="66"/>
-      <c r="H35" s="66"/>
-      <c r="I35" s="66"/>
+      <c r="G35" s="50"/>
+      <c r="H35" s="50"/>
+      <c r="I35" s="50"/>
       <c r="N35" s="7"/>
       <c r="O35" s="7"/>
     </row>
@@ -3217,10 +3203,10 @@
         <v>35</v>
       </c>
       <c r="C40" s="65"/>
-      <c r="F40" s="46" t="s">
+      <c r="F40" s="53" t="s">
         <v>36</v>
       </c>
-      <c r="G40" s="46"/>
+      <c r="G40" s="53"/>
       <c r="I40" s="9" t="s">
         <v>22</v>
       </c>
@@ -3276,7 +3262,7 @@
       <c r="G43" s="2">
         <v>0.44</v>
       </c>
-      <c r="I43" s="63" t="s">
+      <c r="I43" s="52" t="s">
         <v>67</v>
       </c>
     </row>
@@ -3293,7 +3279,7 @@
       <c r="G44" s="2">
         <v>1</v>
       </c>
-      <c r="I44" s="63"/>
+      <c r="I44" s="52"/>
     </row>
     <row r="45" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B45" s="2" t="s">
@@ -3437,67 +3423,67 @@
     </row>
     <row r="57" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="58" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B58" s="48" t="s">
+      <c r="B58" s="44" t="s">
         <v>125</v>
       </c>
-      <c r="C58" s="49"/>
-      <c r="D58" s="49"/>
-      <c r="E58" s="49"/>
-      <c r="F58" s="49"/>
-      <c r="G58" s="49"/>
-      <c r="H58" s="49"/>
-      <c r="I58" s="49"/>
-      <c r="J58" s="49"/>
-      <c r="K58" s="49"/>
-      <c r="L58" s="49"/>
-      <c r="M58" s="49"/>
-      <c r="N58" s="49"/>
-      <c r="O58" s="49"/>
-      <c r="P58" s="49"/>
-      <c r="Q58" s="49"/>
-      <c r="R58" s="50"/>
+      <c r="C58" s="45"/>
+      <c r="D58" s="45"/>
+      <c r="E58" s="45"/>
+      <c r="F58" s="45"/>
+      <c r="G58" s="45"/>
+      <c r="H58" s="45"/>
+      <c r="I58" s="45"/>
+      <c r="J58" s="45"/>
+      <c r="K58" s="45"/>
+      <c r="L58" s="45"/>
+      <c r="M58" s="45"/>
+      <c r="N58" s="45"/>
+      <c r="O58" s="45"/>
+      <c r="P58" s="45"/>
+      <c r="Q58" s="45"/>
+      <c r="R58" s="46"/>
     </row>
     <row r="59" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B59" s="51"/>
-      <c r="C59" s="52"/>
-      <c r="D59" s="52"/>
-      <c r="E59" s="52"/>
-      <c r="F59" s="52"/>
-      <c r="G59" s="52"/>
-      <c r="H59" s="52"/>
-      <c r="I59" s="52"/>
-      <c r="J59" s="52"/>
-      <c r="K59" s="52"/>
-      <c r="L59" s="52"/>
-      <c r="M59" s="52"/>
-      <c r="N59" s="52"/>
-      <c r="O59" s="52"/>
-      <c r="P59" s="52"/>
-      <c r="Q59" s="52"/>
-      <c r="R59" s="53"/>
+      <c r="B59" s="47"/>
+      <c r="C59" s="48"/>
+      <c r="D59" s="48"/>
+      <c r="E59" s="48"/>
+      <c r="F59" s="48"/>
+      <c r="G59" s="48"/>
+      <c r="H59" s="48"/>
+      <c r="I59" s="48"/>
+      <c r="J59" s="48"/>
+      <c r="K59" s="48"/>
+      <c r="L59" s="48"/>
+      <c r="M59" s="48"/>
+      <c r="N59" s="48"/>
+      <c r="O59" s="48"/>
+      <c r="P59" s="48"/>
+      <c r="Q59" s="48"/>
+      <c r="R59" s="49"/>
     </row>
     <row r="61" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B61" s="66" t="s">
+      <c r="B61" s="50" t="s">
         <v>63</v>
       </c>
-      <c r="C61" s="66"/>
-      <c r="D61" s="66"/>
-      <c r="E61" s="66"/>
-      <c r="F61" s="66"/>
-      <c r="G61" s="66"/>
-      <c r="H61" s="66"/>
-      <c r="I61" s="66"/>
-      <c r="J61" s="66"/>
-      <c r="K61" s="66"/>
-      <c r="M61" s="66" t="s">
+      <c r="C61" s="50"/>
+      <c r="D61" s="50"/>
+      <c r="E61" s="50"/>
+      <c r="F61" s="50"/>
+      <c r="G61" s="50"/>
+      <c r="H61" s="50"/>
+      <c r="I61" s="50"/>
+      <c r="J61" s="50"/>
+      <c r="K61" s="50"/>
+      <c r="M61" s="50" t="s">
         <v>68</v>
       </c>
-      <c r="N61" s="66"/>
-      <c r="O61" s="66"/>
-      <c r="Q61" s="66" t="s">
+      <c r="N61" s="50"/>
+      <c r="O61" s="50"/>
+      <c r="Q61" s="50" t="s">
         <v>64</v>
       </c>
-      <c r="R61" s="66"/>
+      <c r="R61" s="50"/>
     </row>
     <row r="62" spans="1:19" x14ac:dyDescent="0.25">
       <c r="B62" s="2" t="s">
@@ -3594,28 +3580,28 @@
       </c>
     </row>
     <row r="66" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B66" s="63" t="s">
+      <c r="B66" s="52" t="s">
         <v>22</v>
       </c>
-      <c r="C66" s="63"/>
+      <c r="C66" s="52"/>
       <c r="E66" s="9" t="s">
         <v>67</v>
       </c>
     </row>
     <row r="67" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B67" s="46">
+      <c r="B67" s="53">
         <f xml:space="preserve"> SUM(B63:K63,M63:O63,Q63:R63)</f>
         <v>85.5</v>
       </c>
-      <c r="C67" s="46"/>
-      <c r="E67" s="47">
+      <c r="C67" s="53"/>
+      <c r="E67" s="54">
         <v>4.5</v>
       </c>
     </row>
     <row r="68" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B68" s="46"/>
-      <c r="C68" s="46"/>
-      <c r="E68" s="47"/>
+      <c r="B68" s="53"/>
+      <c r="C68" s="53"/>
+      <c r="E68" s="54"/>
     </row>
     <row r="70" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A70" s="6"/>
@@ -3640,26 +3626,26 @@
     </row>
     <row r="71" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="72" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B72" s="48" t="s">
+      <c r="B72" s="44" t="s">
         <v>126</v>
       </c>
-      <c r="C72" s="49"/>
-      <c r="D72" s="49"/>
-      <c r="E72" s="49"/>
-      <c r="F72" s="49"/>
-      <c r="G72" s="49"/>
-      <c r="H72" s="49"/>
-      <c r="I72" s="50"/>
+      <c r="C72" s="45"/>
+      <c r="D72" s="45"/>
+      <c r="E72" s="45"/>
+      <c r="F72" s="45"/>
+      <c r="G72" s="45"/>
+      <c r="H72" s="45"/>
+      <c r="I72" s="46"/>
     </row>
     <row r="73" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B73" s="51"/>
-      <c r="C73" s="52"/>
-      <c r="D73" s="52"/>
-      <c r="E73" s="52"/>
-      <c r="F73" s="52"/>
-      <c r="G73" s="52"/>
-      <c r="H73" s="52"/>
-      <c r="I73" s="53"/>
+      <c r="B73" s="47"/>
+      <c r="C73" s="48"/>
+      <c r="D73" s="48"/>
+      <c r="E73" s="48"/>
+      <c r="F73" s="48"/>
+      <c r="G73" s="48"/>
+      <c r="H73" s="48"/>
+      <c r="I73" s="49"/>
     </row>
     <row r="75" spans="1:19" x14ac:dyDescent="0.25">
       <c r="B75" s="4" t="s">
@@ -3686,10 +3672,10 @@
       <c r="I75" s="4" t="s">
         <v>134</v>
       </c>
-      <c r="K75" s="63" t="s">
+      <c r="K75" s="52" t="s">
         <v>22</v>
       </c>
-      <c r="L75" s="63"/>
+      <c r="L75" s="52"/>
       <c r="N75" s="9" t="s">
         <v>67</v>
       </c>
@@ -3719,11 +3705,11 @@
       <c r="I76" s="2">
         <v>5</v>
       </c>
-      <c r="K76" s="46">
+      <c r="K76" s="53">
         <f>SUM(B76:I76)</f>
         <v>96</v>
       </c>
-      <c r="L76" s="46"/>
+      <c r="L76" s="53"/>
       <c r="N76" s="13">
         <v>5</v>
       </c>
@@ -3751,6 +3737,30 @@
     </row>
   </sheetData>
   <mergeCells count="34">
+    <mergeCell ref="B2:P3"/>
+    <mergeCell ref="B5:G5"/>
+    <mergeCell ref="K5:N5"/>
+    <mergeCell ref="B9:C9"/>
+    <mergeCell ref="B10:C11"/>
+    <mergeCell ref="E10:E11"/>
+    <mergeCell ref="M27:M28"/>
+    <mergeCell ref="O27:O28"/>
+    <mergeCell ref="B14:H15"/>
+    <mergeCell ref="B17:D17"/>
+    <mergeCell ref="F17:H17"/>
+    <mergeCell ref="J17:K17"/>
+    <mergeCell ref="J18:K19"/>
+    <mergeCell ref="M18:M19"/>
+    <mergeCell ref="I43:I44"/>
+    <mergeCell ref="B23:K24"/>
+    <mergeCell ref="B26:C26"/>
+    <mergeCell ref="E26:G26"/>
+    <mergeCell ref="I26:K26"/>
+    <mergeCell ref="B32:I33"/>
+    <mergeCell ref="B35:D35"/>
+    <mergeCell ref="F35:I35"/>
+    <mergeCell ref="B40:C40"/>
+    <mergeCell ref="F40:G40"/>
     <mergeCell ref="B72:I73"/>
     <mergeCell ref="K75:L75"/>
     <mergeCell ref="K76:L76"/>
@@ -3761,30 +3771,6 @@
     <mergeCell ref="B66:C66"/>
     <mergeCell ref="B67:C68"/>
     <mergeCell ref="E67:E68"/>
-    <mergeCell ref="I43:I44"/>
-    <mergeCell ref="B23:K24"/>
-    <mergeCell ref="B26:C26"/>
-    <mergeCell ref="E26:G26"/>
-    <mergeCell ref="I26:K26"/>
-    <mergeCell ref="B32:I33"/>
-    <mergeCell ref="B35:D35"/>
-    <mergeCell ref="F35:I35"/>
-    <mergeCell ref="B40:C40"/>
-    <mergeCell ref="F40:G40"/>
-    <mergeCell ref="M27:M28"/>
-    <mergeCell ref="O27:O28"/>
-    <mergeCell ref="B14:H15"/>
-    <mergeCell ref="B17:D17"/>
-    <mergeCell ref="F17:H17"/>
-    <mergeCell ref="J17:K17"/>
-    <mergeCell ref="J18:K19"/>
-    <mergeCell ref="M18:M19"/>
-    <mergeCell ref="B2:P3"/>
-    <mergeCell ref="B5:G5"/>
-    <mergeCell ref="K5:N5"/>
-    <mergeCell ref="B9:C9"/>
-    <mergeCell ref="B10:C11"/>
-    <mergeCell ref="E10:E11"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
@@ -3818,551 +3804,551 @@
       </c>
     </row>
     <row r="3" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B3" s="22" t="b">
+      <c r="B3" s="18" t="b">
         <v>1</v>
       </c>
-      <c r="C3" s="29" t="s">
+      <c r="C3" s="25" t="s">
         <v>77</v>
       </c>
-      <c r="D3" s="24">
+      <c r="D3" s="20">
         <v>45763</v>
       </c>
-      <c r="E3" s="25" t="s">
+      <c r="E3" s="21" t="s">
         <v>138</v>
       </c>
-      <c r="F3" s="23" t="s">
+      <c r="F3" s="19" t="s">
         <v>172</v>
       </c>
     </row>
     <row r="4" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B4" s="22" t="b">
+      <c r="B4" s="18" t="b">
         <v>1</v>
       </c>
-      <c r="C4" s="28" t="s">
+      <c r="C4" s="24" t="s">
         <v>77</v>
       </c>
-      <c r="D4" s="27">
+      <c r="D4" s="23">
         <v>45812</v>
       </c>
-      <c r="E4" s="40" t="s">
+      <c r="E4" s="36" t="s">
         <v>139</v>
       </c>
-      <c r="F4" s="26" t="s">
+      <c r="F4" s="22" t="s">
         <v>173</v>
       </c>
     </row>
     <row r="5" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B5" s="41" t="b">
+      <c r="B5" s="37" t="b">
         <v>0</v>
       </c>
-      <c r="C5" s="42" t="s">
+      <c r="C5" s="38" t="s">
         <v>77</v>
       </c>
-      <c r="D5" s="43">
+      <c r="D5" s="39">
         <v>45817</v>
       </c>
-      <c r="E5" s="44" t="s">
+      <c r="E5" s="40" t="s">
         <v>140</v>
       </c>
-      <c r="F5" s="45" t="s">
+      <c r="F5" s="41" t="s">
         <v>141</v>
       </c>
     </row>
     <row r="6" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="C6" s="30"/>
+      <c r="C6" s="26"/>
     </row>
     <row r="7" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B7" s="22" t="b">
+      <c r="B7" s="18" t="b">
         <v>1</v>
       </c>
-      <c r="C7" s="28" t="s">
+      <c r="C7" s="24" t="s">
         <v>77</v>
       </c>
-      <c r="D7" s="27">
+      <c r="D7" s="23">
         <v>45729</v>
       </c>
-      <c r="E7" s="26" t="s">
+      <c r="E7" s="22" t="s">
         <v>103</v>
       </c>
-      <c r="F7" s="26" t="s">
+      <c r="F7" s="22" t="s">
         <v>142</v>
       </c>
     </row>
     <row r="8" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B8" s="22" t="b">
+      <c r="B8" s="18" t="b">
         <v>1</v>
       </c>
-      <c r="C8" s="28" t="s">
+      <c r="C8" s="24" t="s">
         <v>77</v>
       </c>
-      <c r="D8" s="27">
+      <c r="D8" s="23">
         <v>45743</v>
       </c>
-      <c r="E8" s="26" t="s">
+      <c r="E8" s="22" t="s">
         <v>104</v>
       </c>
-      <c r="F8" s="26" t="s">
+      <c r="F8" s="22" t="s">
         <v>143</v>
       </c>
     </row>
     <row r="9" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B9" s="22" t="b">
+      <c r="B9" s="18" t="b">
         <v>1</v>
       </c>
-      <c r="C9" s="28" t="s">
+      <c r="C9" s="24" t="s">
         <v>77</v>
       </c>
-      <c r="D9" s="27">
+      <c r="D9" s="23">
         <v>45757</v>
       </c>
-      <c r="E9" s="26" t="s">
+      <c r="E9" s="22" t="s">
         <v>105</v>
       </c>
-      <c r="F9" s="26" t="s">
+      <c r="F9" s="22" t="s">
         <v>144</v>
       </c>
     </row>
     <row r="10" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B10" s="22" t="b">
+      <c r="B10" s="18" t="b">
         <v>1</v>
       </c>
-      <c r="C10" s="28" t="s">
+      <c r="C10" s="24" t="s">
         <v>77</v>
       </c>
-      <c r="D10" s="27">
+      <c r="D10" s="23">
         <v>45785</v>
       </c>
-      <c r="E10" s="26" t="s">
+      <c r="E10" s="22" t="s">
         <v>106</v>
       </c>
-      <c r="F10" s="26" t="s">
+      <c r="F10" s="22" t="s">
         <v>145</v>
       </c>
     </row>
     <row r="11" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B11" s="22" t="b">
+      <c r="B11" s="18" t="b">
         <v>1</v>
       </c>
-      <c r="C11" s="28" t="s">
+      <c r="C11" s="24" t="s">
         <v>77</v>
       </c>
-      <c r="D11" s="27">
+      <c r="D11" s="23">
         <v>45799</v>
       </c>
-      <c r="E11" s="26" t="s">
+      <c r="E11" s="22" t="s">
         <v>107</v>
       </c>
-      <c r="F11" s="26" t="s">
+      <c r="F11" s="22" t="s">
         <v>146</v>
       </c>
     </row>
     <row r="12" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="C12" s="30"/>
+      <c r="C12" s="26"/>
     </row>
     <row r="13" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B13" s="22" t="b">
+      <c r="B13" s="18" t="b">
         <v>1</v>
       </c>
-      <c r="C13" s="28" t="s">
+      <c r="C13" s="24" t="s">
         <v>150</v>
       </c>
-      <c r="D13" s="27">
+      <c r="D13" s="23">
         <v>45728</v>
       </c>
-      <c r="E13" s="26" t="s">
+      <c r="E13" s="22" t="s">
         <v>84</v>
       </c>
-      <c r="F13" s="26" t="s">
+      <c r="F13" s="22" t="s">
         <v>151</v>
       </c>
     </row>
     <row r="14" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B14" s="22" t="b">
+      <c r="B14" s="18" t="b">
         <v>1</v>
       </c>
-      <c r="C14" s="28" t="s">
+      <c r="C14" s="24" t="s">
         <v>150</v>
       </c>
-      <c r="D14" s="27">
+      <c r="D14" s="23">
         <v>45747</v>
       </c>
-      <c r="E14" s="26" t="s">
+      <c r="E14" s="22" t="s">
         <v>152</v>
       </c>
-      <c r="F14" s="26" t="s">
+      <c r="F14" s="22" t="s">
         <v>156</v>
       </c>
     </row>
     <row r="15" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B15" s="22" t="b">
+      <c r="B15" s="18" t="b">
         <v>1</v>
       </c>
-      <c r="C15" s="28" t="s">
+      <c r="C15" s="24" t="s">
         <v>150</v>
       </c>
-      <c r="D15" s="27">
+      <c r="D15" s="23">
         <v>45784</v>
       </c>
-      <c r="E15" s="26" t="s">
+      <c r="E15" s="22" t="s">
         <v>153</v>
       </c>
-      <c r="F15" s="26" t="s">
+      <c r="F15" s="22" t="s">
         <v>154</v>
       </c>
     </row>
     <row r="16" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B16" s="22" t="b">
+      <c r="B16" s="18" t="b">
         <v>1</v>
       </c>
-      <c r="C16" s="28" t="s">
+      <c r="C16" s="24" t="s">
         <v>150</v>
       </c>
-      <c r="D16" s="27">
+      <c r="D16" s="23">
         <v>45806</v>
       </c>
-      <c r="E16" s="26" t="s">
+      <c r="E16" s="22" t="s">
         <v>85</v>
       </c>
-      <c r="F16" s="26" t="s">
+      <c r="F16" s="22" t="s">
         <v>155</v>
       </c>
     </row>
     <row r="17" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B17" s="22" t="b">
+      <c r="B17" s="18" t="b">
         <v>1</v>
       </c>
-      <c r="C17" s="28" t="s">
+      <c r="C17" s="24" t="s">
         <v>150</v>
       </c>
-      <c r="D17" s="27">
+      <c r="D17" s="23">
         <v>45817</v>
       </c>
-      <c r="E17" s="26" t="s">
+      <c r="E17" s="22" t="s">
         <v>158</v>
       </c>
-      <c r="F17" s="28" t="s">
+      <c r="F17" s="24" t="s">
         <v>157</v>
       </c>
     </row>
     <row r="18" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B18" s="22" t="b">
+      <c r="B18" s="18" t="b">
         <v>1</v>
       </c>
-      <c r="C18" s="28" t="s">
+      <c r="C18" s="24" t="s">
         <v>150</v>
       </c>
-      <c r="D18" s="27">
+      <c r="D18" s="23">
         <v>45819</v>
       </c>
-      <c r="E18" s="26" t="s">
+      <c r="E18" s="22" t="s">
         <v>160</v>
       </c>
-      <c r="F18" s="28" t="s">
+      <c r="F18" s="24" t="s">
         <v>159</v>
       </c>
     </row>
     <row r="19" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="C19" s="30"/>
-      <c r="D19" s="21"/>
+      <c r="C19" s="26"/>
+      <c r="D19" s="17"/>
     </row>
     <row r="20" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B20" s="18" t="b">
-        <v>0</v>
-      </c>
-      <c r="C20" s="20" t="s">
+        <v>1</v>
+      </c>
+      <c r="C20" s="24" t="s">
         <v>150</v>
       </c>
-      <c r="D20" s="19">
+      <c r="D20" s="23">
         <v>45820</v>
       </c>
-      <c r="E20" s="17" t="s">
+      <c r="E20" s="22" t="s">
         <v>161</v>
       </c>
     </row>
     <row r="21" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B21" s="18" t="b">
-        <v>0</v>
-      </c>
-      <c r="C21" s="20" t="s">
+        <v>1</v>
+      </c>
+      <c r="C21" s="24" t="s">
         <v>150</v>
       </c>
-      <c r="D21" s="19">
+      <c r="D21" s="23">
         <v>45820</v>
       </c>
-      <c r="E21" s="17" t="s">
+      <c r="E21" s="22" t="s">
         <v>162</v>
       </c>
     </row>
     <row r="22" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="C22" s="30"/>
-      <c r="D22" s="21"/>
+      <c r="C22" s="26"/>
+      <c r="D22" s="17"/>
     </row>
     <row r="23" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B23" s="22" t="b">
+      <c r="B23" s="18" t="b">
         <v>1</v>
       </c>
-      <c r="C23" s="28" t="s">
+      <c r="C23" s="24" t="s">
         <v>76</v>
       </c>
-      <c r="D23" s="27">
+      <c r="D23" s="23">
         <v>45728</v>
       </c>
-      <c r="E23" s="26" t="s">
+      <c r="E23" s="22" t="s">
         <v>169</v>
       </c>
-      <c r="F23" s="26" t="s">
+      <c r="F23" s="22" t="s">
         <v>174</v>
       </c>
     </row>
     <row r="24" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B24" s="22" t="b">
+      <c r="B24" s="18" t="b">
         <v>1</v>
       </c>
-      <c r="C24" s="28" t="s">
+      <c r="C24" s="24" t="s">
         <v>76</v>
       </c>
-      <c r="D24" s="27">
+      <c r="D24" s="23">
         <v>45742</v>
       </c>
-      <c r="E24" s="26" t="s">
+      <c r="E24" s="22" t="s">
         <v>169</v>
       </c>
-      <c r="F24" s="26" t="s">
+      <c r="F24" s="22" t="s">
         <v>175</v>
       </c>
     </row>
     <row r="25" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B25" s="22" t="b">
+      <c r="B25" s="18" t="b">
         <v>1</v>
       </c>
-      <c r="C25" s="28" t="s">
+      <c r="C25" s="24" t="s">
         <v>76</v>
       </c>
-      <c r="D25" s="27">
+      <c r="D25" s="23">
         <v>45756</v>
       </c>
-      <c r="E25" s="26" t="s">
+      <c r="E25" s="22" t="s">
         <v>169</v>
       </c>
-      <c r="F25" s="26" t="s">
+      <c r="F25" s="22" t="s">
         <v>176</v>
       </c>
     </row>
     <row r="26" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B26" s="22" t="b">
+      <c r="B26" s="18" t="b">
         <v>1</v>
       </c>
-      <c r="C26" s="28" t="s">
+      <c r="C26" s="24" t="s">
         <v>76</v>
       </c>
-      <c r="D26" s="27">
+      <c r="D26" s="23">
         <v>45770</v>
       </c>
-      <c r="E26" s="26" t="s">
+      <c r="E26" s="22" t="s">
         <v>168</v>
       </c>
-      <c r="F26" s="28" t="s">
+      <c r="F26" s="24" t="s">
         <v>180</v>
       </c>
     </row>
     <row r="27" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B27" s="22" t="b">
+      <c r="B27" s="18" t="b">
         <v>1</v>
       </c>
-      <c r="C27" s="28" t="s">
+      <c r="C27" s="24" t="s">
         <v>76</v>
       </c>
-      <c r="D27" s="27">
+      <c r="D27" s="23">
         <v>45784</v>
       </c>
-      <c r="E27" s="26" t="s">
+      <c r="E27" s="22" t="s">
         <v>169</v>
       </c>
-      <c r="F27" s="26" t="s">
+      <c r="F27" s="22" t="s">
         <v>177</v>
       </c>
     </row>
     <row r="28" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B28" s="22" t="b">
+      <c r="B28" s="18" t="b">
         <v>1</v>
       </c>
-      <c r="C28" s="28" t="s">
+      <c r="C28" s="24" t="s">
         <v>76</v>
       </c>
-      <c r="D28" s="27">
+      <c r="D28" s="23">
         <v>45798</v>
       </c>
-      <c r="E28" s="26" t="s">
+      <c r="E28" s="22" t="s">
         <v>169</v>
       </c>
-      <c r="F28" s="26" t="s">
+      <c r="F28" s="22" t="s">
         <v>178</v>
       </c>
     </row>
     <row r="29" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B29" s="22" t="b">
+      <c r="B29" s="18" t="b">
         <v>1</v>
       </c>
-      <c r="C29" s="28" t="s">
+      <c r="C29" s="24" t="s">
         <v>76</v>
       </c>
-      <c r="D29" s="27">
+      <c r="D29" s="23">
         <v>45812</v>
       </c>
-      <c r="E29" s="26" t="s">
+      <c r="E29" s="22" t="s">
         <v>168</v>
       </c>
-      <c r="F29" s="28" t="s">
+      <c r="F29" s="24" t="s">
         <v>206</v>
       </c>
     </row>
     <row r="30" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="C30" s="30"/>
+      <c r="C30" s="26"/>
     </row>
     <row r="31" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B31" s="22" t="b">
+      <c r="B31" s="18" t="b">
         <v>1</v>
       </c>
-      <c r="C31" s="28" t="s">
+      <c r="C31" s="24" t="s">
         <v>76</v>
       </c>
-      <c r="D31" s="27">
+      <c r="D31" s="23">
         <v>45764</v>
       </c>
-      <c r="E31" s="26" t="s">
+      <c r="E31" s="22" t="s">
         <v>138</v>
       </c>
-      <c r="F31" s="26" t="s">
+      <c r="F31" s="22" t="s">
         <v>181</v>
       </c>
     </row>
     <row r="32" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B32" s="22" t="b">
+      <c r="B32" s="18" t="b">
         <v>1</v>
       </c>
-      <c r="C32" s="28" t="s">
+      <c r="C32" s="24" t="s">
         <v>76</v>
       </c>
-      <c r="D32" s="27">
+      <c r="D32" s="23">
         <v>45815</v>
       </c>
-      <c r="E32" s="26" t="s">
+      <c r="E32" s="22" t="s">
         <v>207</v>
       </c>
     </row>
     <row r="33" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B33" s="22" t="b">
+      <c r="B33" s="18" t="b">
         <v>1</v>
       </c>
-      <c r="C33" s="28" t="s">
+      <c r="C33" s="24" t="s">
         <v>76</v>
       </c>
-      <c r="D33" s="27">
+      <c r="D33" s="23">
         <v>45814</v>
       </c>
-      <c r="E33" s="26" t="s">
+      <c r="E33" s="22" t="s">
         <v>139</v>
       </c>
-      <c r="F33" s="26" t="s">
+      <c r="F33" s="22" t="s">
         <v>212</v>
       </c>
     </row>
     <row r="35" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B35" s="22" t="b">
+      <c r="B35" s="18" t="b">
         <v>1</v>
       </c>
-      <c r="C35" s="28" t="s">
+      <c r="C35" s="24" t="s">
         <v>78</v>
       </c>
-      <c r="D35" s="27">
+      <c r="D35" s="23">
         <v>45767</v>
       </c>
-      <c r="E35" s="26" t="s">
+      <c r="E35" s="22" t="s">
         <v>170</v>
       </c>
-      <c r="F35" s="26" t="s">
+      <c r="F35" s="22" t="s">
         <v>179</v>
       </c>
     </row>
     <row r="36" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B36" s="22" t="b">
+      <c r="B36" s="18" t="b">
         <v>1</v>
       </c>
-      <c r="C36" s="28" t="s">
+      <c r="C36" s="24" t="s">
         <v>78</v>
       </c>
-      <c r="D36" s="27">
+      <c r="D36" s="23">
         <v>45775</v>
       </c>
-      <c r="E36" s="26" t="s">
+      <c r="E36" s="22" t="s">
         <v>138</v>
       </c>
     </row>
     <row r="37" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B37" s="22" t="b">
+      <c r="B37" s="18" t="b">
         <v>1</v>
       </c>
-      <c r="C37" s="28" t="s">
+      <c r="C37" s="24" t="s">
         <v>78</v>
       </c>
-      <c r="D37" s="27">
+      <c r="D37" s="23">
         <v>45794</v>
       </c>
-      <c r="E37" s="26" t="s">
+      <c r="E37" s="22" t="s">
         <v>203</v>
       </c>
-      <c r="F37" s="26" t="s">
+      <c r="F37" s="22" t="s">
         <v>202</v>
       </c>
     </row>
     <row r="39" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B39" s="22" t="b">
+      <c r="B39" s="18" t="b">
         <v>1</v>
       </c>
-      <c r="C39" s="28" t="s">
+      <c r="C39" s="24" t="s">
         <v>79</v>
       </c>
-      <c r="D39" s="27">
+      <c r="D39" s="23">
         <v>45784</v>
       </c>
-      <c r="E39" s="26" t="s">
+      <c r="E39" s="22" t="s">
         <v>213</v>
       </c>
-      <c r="F39" s="26" t="s">
+      <c r="F39" s="22" t="s">
         <v>209</v>
       </c>
     </row>
     <row r="40" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B40" s="22" t="b">
+      <c r="B40" s="18" t="b">
         <v>1</v>
       </c>
-      <c r="C40" s="28" t="s">
+      <c r="C40" s="24" t="s">
         <v>79</v>
       </c>
-      <c r="D40" s="27">
+      <c r="D40" s="23">
         <v>45798</v>
       </c>
-      <c r="E40" s="26" t="s">
+      <c r="E40" s="22" t="s">
         <v>208</v>
       </c>
-      <c r="F40" s="26" t="s">
+      <c r="F40" s="22" t="s">
         <v>209</v>
       </c>
     </row>
     <row r="41" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B41" s="22" t="b">
+      <c r="B41" s="18" t="b">
         <v>1</v>
       </c>
-      <c r="C41" s="28" t="s">
+      <c r="C41" s="24" t="s">
         <v>79</v>
       </c>
-      <c r="D41" s="27">
+      <c r="D41" s="23">
         <v>45805</v>
       </c>
-      <c r="E41" s="26" t="s">
+      <c r="E41" s="22" t="s">
         <v>211</v>
       </c>
-      <c r="F41" s="26" t="s">
+      <c r="F41" s="22" t="s">
         <v>210</v>
       </c>
     </row>
@@ -4391,53 +4377,53 @@
   <sheetData>
     <row r="1" spans="2:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="2" spans="2:12" ht="23.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B2" s="73" t="s">
+      <c r="B2" s="69" t="s">
         <v>192</v>
       </c>
-      <c r="C2" s="74"/>
-      <c r="D2" s="75"/>
-      <c r="F2" s="73" t="s">
+      <c r="C2" s="70"/>
+      <c r="D2" s="71"/>
+      <c r="F2" s="69" t="s">
         <v>193</v>
       </c>
-      <c r="G2" s="74"/>
-      <c r="H2" s="75"/>
-      <c r="J2" s="73" t="s">
+      <c r="G2" s="70"/>
+      <c r="H2" s="71"/>
+      <c r="J2" s="69" t="s">
         <v>194</v>
       </c>
-      <c r="K2" s="74"/>
-      <c r="L2" s="75"/>
+      <c r="K2" s="70"/>
+      <c r="L2" s="71"/>
     </row>
     <row r="3" spans="2:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B3" s="33" t="s">
+      <c r="B3" s="29" t="s">
         <v>136</v>
       </c>
-      <c r="C3" s="34" t="s">
+      <c r="C3" s="30" t="s">
         <v>185</v>
       </c>
-      <c r="D3" s="35" t="s">
+      <c r="D3" s="31" t="s">
         <v>184</v>
       </c>
-      <c r="F3" s="33" t="s">
+      <c r="F3" s="29" t="s">
         <v>136</v>
       </c>
-      <c r="G3" s="34" t="s">
+      <c r="G3" s="30" t="s">
         <v>185</v>
       </c>
-      <c r="H3" s="35" t="s">
+      <c r="H3" s="31" t="s">
         <v>184</v>
       </c>
-      <c r="J3" s="33" t="s">
+      <c r="J3" s="29" t="s">
         <v>136</v>
       </c>
-      <c r="K3" s="34" t="s">
+      <c r="K3" s="30" t="s">
         <v>185</v>
       </c>
-      <c r="L3" s="35" t="s">
+      <c r="L3" s="31" t="s">
         <v>184</v>
       </c>
     </row>
     <row r="4" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B4" s="36" t="s">
+      <c r="B4" s="32" t="s">
         <v>121</v>
       </c>
       <c r="C4" s="14">
@@ -4446,14 +4432,14 @@
       <c r="D4" s="14">
         <v>4</v>
       </c>
-      <c r="F4" s="36" t="s">
+      <c r="F4" s="32" t="s">
         <v>76</v>
       </c>
       <c r="G4" s="14">
         <v>5</v>
       </c>
       <c r="H4" s="14"/>
-      <c r="J4" s="36" t="s">
+      <c r="J4" s="32" t="s">
         <v>187</v>
       </c>
       <c r="K4" s="14">
@@ -4462,7 +4448,7 @@
       <c r="L4" s="14"/>
     </row>
     <row r="5" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B5" s="37" t="s">
+      <c r="B5" s="33" t="s">
         <v>122</v>
       </c>
       <c r="C5" s="2">
@@ -4471,14 +4457,14 @@
       <c r="D5" s="2">
         <v>5</v>
       </c>
-      <c r="F5" s="37" t="s">
+      <c r="F5" s="33" t="s">
         <v>79</v>
       </c>
       <c r="G5" s="2">
         <v>4</v>
       </c>
       <c r="H5" s="2"/>
-      <c r="J5" s="37" t="s">
+      <c r="J5" s="33" t="s">
         <v>188</v>
       </c>
       <c r="K5" s="2">
@@ -4487,7 +4473,7 @@
       <c r="L5" s="2"/>
     </row>
     <row r="6" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B6" s="37" t="s">
+      <c r="B6" s="33" t="s">
         <v>123</v>
       </c>
       <c r="C6" s="2">
@@ -4496,7 +4482,7 @@
       <c r="D6" s="2">
         <v>4</v>
       </c>
-      <c r="F6" s="37" t="s">
+      <c r="F6" s="33" t="s">
         <v>77</v>
       </c>
       <c r="G6" s="2">
@@ -4505,7 +4491,7 @@
       <c r="H6" s="2">
         <v>4.5</v>
       </c>
-      <c r="J6" s="37" t="s">
+      <c r="J6" s="33" t="s">
         <v>189</v>
       </c>
       <c r="K6" s="2">
@@ -4514,7 +4500,7 @@
       <c r="L6" s="2"/>
     </row>
     <row r="7" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B7" s="37" t="s">
+      <c r="B7" s="33" t="s">
         <v>124</v>
       </c>
       <c r="C7" s="2">
@@ -4523,7 +4509,7 @@
       <c r="D7" s="2">
         <v>4</v>
       </c>
-      <c r="F7" s="37" t="s">
+      <c r="F7" s="33" t="s">
         <v>78</v>
       </c>
       <c r="G7" s="2">
@@ -4532,7 +4518,7 @@
       <c r="H7" s="2">
         <v>5</v>
       </c>
-      <c r="J7" s="37" t="s">
+      <c r="J7" s="33" t="s">
         <v>190</v>
       </c>
       <c r="K7" s="2">
@@ -4541,7 +4527,7 @@
       <c r="L7" s="2"/>
     </row>
     <row r="8" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B8" s="37" t="s">
+      <c r="B8" s="33" t="s">
         <v>125</v>
       </c>
       <c r="C8" s="2">
@@ -4550,14 +4536,16 @@
       <c r="D8" s="2">
         <v>4.5</v>
       </c>
-      <c r="F8" s="37" t="s">
+      <c r="F8" s="33" t="s">
         <v>80</v>
       </c>
       <c r="G8" s="2">
         <v>11</v>
       </c>
-      <c r="H8" s="2"/>
-      <c r="J8" s="37" t="s">
+      <c r="H8" s="2">
+        <v>5</v>
+      </c>
+      <c r="J8" s="33" t="s">
         <v>191</v>
       </c>
       <c r="K8" s="2">
@@ -4566,7 +4554,7 @@
       <c r="L8" s="2"/>
     </row>
     <row r="9" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B9" s="37" t="s">
+      <c r="B9" s="33" t="s">
         <v>126</v>
       </c>
       <c r="C9" s="2">
@@ -4575,36 +4563,36 @@
       <c r="D9" s="2">
         <v>5</v>
       </c>
-      <c r="F9" s="31"/>
+      <c r="F9" s="27"/>
       <c r="G9" s="1"/>
       <c r="H9" s="1"/>
-      <c r="J9" s="31"/>
+      <c r="J9" s="27"/>
       <c r="K9" s="1"/>
       <c r="L9" s="1"/>
     </row>
     <row r="10" spans="2:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="11" spans="2:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B11" s="76" t="s">
+      <c r="B11" s="72" t="s">
         <v>186</v>
       </c>
-      <c r="C11" s="77"/>
-      <c r="D11" s="32">
+      <c r="C11" s="73"/>
+      <c r="D11" s="28">
         <f>(D4*C4+D5*C5+D6*C6+D7*C7+D8*C8+D9*C9)/30</f>
         <v>4.4333333333333336</v>
       </c>
-      <c r="F11" s="76" t="s">
+      <c r="F11" s="72" t="s">
         <v>186</v>
       </c>
-      <c r="G11" s="77"/>
-      <c r="H11" s="32">
+      <c r="G11" s="73"/>
+      <c r="H11" s="28">
         <f>(H4*G4+H5*G5+H6*G6+H7*G7+H8*G8)/30</f>
-        <v>1.5833333333333333</v>
-      </c>
-      <c r="J11" s="76" t="s">
+        <v>3.4166666666666665</v>
+      </c>
+      <c r="J11" s="72" t="s">
         <v>186</v>
       </c>
-      <c r="K11" s="77"/>
-      <c r="L11" s="32">
+      <c r="K11" s="73"/>
+      <c r="L11" s="28">
         <f>(L4*K4+L5*K5+L6*K6+L7*K7+L8*K8)/30</f>
         <v>0</v>
       </c>

</xml_diff>

<commit_message>
New points - MAT3 and FIZ1 exams -> everything passed and holidays!@
</commit_message>
<xml_diff>
--- a/IoT-points-schedule.xlsx
+++ b/IoT-points-schedule.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\dodo\Desktop\IoT-studies\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{69F574BF-2489-4E09-8598-D6F07679B0E8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{68C43C02-BBA6-40DA-B027-5612C705B080}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="25440" windowHeight="15390" xr2:uid="{F85F5544-1FE8-4920-A5D4-192A98B113BD}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="343" uniqueCount="216">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="342" uniqueCount="215">
   <si>
     <t>1. Krypto</t>
   </si>
@@ -302,9 +302,6 @@
     <t>Prez. końcowa</t>
   </si>
   <si>
-    <t>Do zdania brakuje:</t>
-  </si>
-  <si>
     <t>Ustny [30 pkt]</t>
   </si>
   <si>
@@ -338,12 +335,6 @@
     <t>Wykłady [20 + 20 pkt]</t>
   </si>
   <si>
-    <t>BONUS 1</t>
-  </si>
-  <si>
-    <t>BONUS 2</t>
-  </si>
-  <si>
     <t>Laby</t>
   </si>
   <si>
@@ -401,9 +392,6 @@
     <t>Egzamin [20+10 pkt]</t>
   </si>
   <si>
-    <t>W = 0,4E + 0,3C + 0,3L</t>
-  </si>
-  <si>
     <t>MAT1</t>
   </si>
   <si>
@@ -687,6 +675,15 @@
   </si>
   <si>
     <t>Mini-projekt [10 pkt]</t>
+  </si>
+  <si>
+    <t>Średnia:</t>
+  </si>
+  <si>
+    <t>Bonus</t>
+  </si>
+  <si>
+    <t>W = (E/30)*0,4*5 + (C/25)*0,3*5 + 0,3L</t>
   </si>
 </sst>
 </file>
@@ -769,7 +766,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="9">
+  <fills count="8">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -785,12 +782,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="3" tint="0.89999084444715716"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.59999389629810485"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1068,7 +1059,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="74">
+  <cellXfs count="70">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1121,32 +1112,32 @@
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1">
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1">
       <extLst>
         <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
           <xfpb:xfComplement i="0"/>
         </ext>
       </extLst>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="5" borderId="12" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="0" fillId="4" borderId="12" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="14" fontId="0" fillId="5" borderId="12" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="14" fontId="0" fillId="4" borderId="12" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="0" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -1156,47 +1147,47 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="19" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="14" fontId="0" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="14" fontId="0" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
       <extLst>
         <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
           <xfpb:xfComplement i="0"/>
         </ext>
       </extLst>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="165" fontId="7" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="7" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="14" fontId="7" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="14" fontId="7" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1205,28 +1196,28 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="6" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="6" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="6" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="6" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="6" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="6" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1247,24 +1238,6 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1280,13 +1253,13 @@
     <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1294,6 +1267,12 @@
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1673,7 +1652,7 @@
     <col min="12" max="12" width="10.85546875" style="1" customWidth="1"/>
     <col min="13" max="13" width="15.28515625" style="1" customWidth="1"/>
     <col min="14" max="14" width="15.7109375" style="1" customWidth="1"/>
-    <col min="15" max="15" width="14.28515625" style="1" customWidth="1"/>
+    <col min="15" max="15" width="17.28515625" style="1" customWidth="1"/>
     <col min="16" max="16" width="15.140625" style="1" customWidth="1"/>
     <col min="17" max="17" width="12.28515625" style="1" customWidth="1"/>
     <col min="18" max="18" width="13.85546875" style="1" customWidth="1"/>
@@ -1683,40 +1662,40 @@
   <sheetData>
     <row r="1" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="2" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B2" s="58" t="s">
+      <c r="B2" s="44" t="s">
         <v>76</v>
       </c>
-      <c r="C2" s="59"/>
-      <c r="D2" s="59"/>
-      <c r="E2" s="59"/>
-      <c r="F2" s="59"/>
-      <c r="G2" s="59"/>
-      <c r="H2" s="59"/>
-      <c r="I2" s="59"/>
-      <c r="J2" s="59"/>
-      <c r="K2" s="59"/>
-      <c r="L2" s="59"/>
-      <c r="M2" s="59"/>
-      <c r="N2" s="59"/>
-      <c r="O2" s="59"/>
-      <c r="P2" s="60"/>
+      <c r="C2" s="45"/>
+      <c r="D2" s="45"/>
+      <c r="E2" s="45"/>
+      <c r="F2" s="45"/>
+      <c r="G2" s="45"/>
+      <c r="H2" s="45"/>
+      <c r="I2" s="45"/>
+      <c r="J2" s="45"/>
+      <c r="K2" s="45"/>
+      <c r="L2" s="45"/>
+      <c r="M2" s="45"/>
+      <c r="N2" s="45"/>
+      <c r="O2" s="45"/>
+      <c r="P2" s="46"/>
     </row>
     <row r="3" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B3" s="61"/>
-      <c r="C3" s="62"/>
-      <c r="D3" s="62"/>
-      <c r="E3" s="62"/>
-      <c r="F3" s="62"/>
-      <c r="G3" s="62"/>
-      <c r="H3" s="62"/>
-      <c r="I3" s="62"/>
-      <c r="J3" s="62"/>
-      <c r="K3" s="62"/>
-      <c r="L3" s="62"/>
-      <c r="M3" s="62"/>
-      <c r="N3" s="62"/>
-      <c r="O3" s="62"/>
-      <c r="P3" s="63"/>
+      <c r="B3" s="47"/>
+      <c r="C3" s="48"/>
+      <c r="D3" s="48"/>
+      <c r="E3" s="48"/>
+      <c r="F3" s="48"/>
+      <c r="G3" s="48"/>
+      <c r="H3" s="48"/>
+      <c r="I3" s="48"/>
+      <c r="J3" s="48"/>
+      <c r="K3" s="48"/>
+      <c r="L3" s="48"/>
+      <c r="M3" s="48"/>
+      <c r="N3" s="48"/>
+      <c r="O3" s="48"/>
+      <c r="P3" s="49"/>
       <c r="R3" s="12"/>
     </row>
     <row r="5" spans="1:19" x14ac:dyDescent="0.25">
@@ -1743,25 +1722,25 @@
     </row>
     <row r="6" spans="1:19" ht="29.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B6" s="3" t="s">
+        <v>159</v>
+      </c>
+      <c r="C6" s="3" t="s">
+        <v>160</v>
+      </c>
+      <c r="D6" s="3" t="s">
+        <v>161</v>
+      </c>
+      <c r="E6" s="3" t="s">
+        <v>162</v>
+      </c>
+      <c r="F6" s="3" t="s">
         <v>163</v>
       </c>
-      <c r="C6" s="3" t="s">
-        <v>164</v>
-      </c>
-      <c r="D6" s="3" t="s">
-        <v>165</v>
-      </c>
-      <c r="E6" s="3" t="s">
-        <v>166</v>
-      </c>
-      <c r="F6" s="3" t="s">
-        <v>167</v>
-      </c>
       <c r="H6" s="2" t="s">
-        <v>201</v>
+        <v>197</v>
       </c>
       <c r="I6" s="2" t="s">
-        <v>204</v>
+        <v>200</v>
       </c>
       <c r="K6" s="2" t="s">
         <v>24</v>
@@ -1811,7 +1790,9 @@
       <c r="N7" s="2">
         <v>6</v>
       </c>
-      <c r="P7" s="2"/>
+      <c r="P7" s="2">
+        <v>39</v>
+      </c>
     </row>
     <row r="9" spans="1:19" x14ac:dyDescent="0.25">
       <c r="B9" s="52" t="s">
@@ -1821,30 +1802,27 @@
       <c r="E9" s="9" t="s">
         <v>67</v>
       </c>
-      <c r="G9" s="52" t="s">
-        <v>87</v>
-      </c>
-      <c r="H9" s="52"/>
+      <c r="G9" s="68"/>
+      <c r="H9" s="68"/>
     </row>
     <row r="10" spans="1:19" x14ac:dyDescent="0.25">
       <c r="B10" s="53">
         <f>SUM(B7:F7,H7:I7,K7:N7,P7)</f>
-        <v>55.1</v>
+        <v>94.1</v>
       </c>
       <c r="C10" s="53"/>
-      <c r="E10" s="55"/>
-      <c r="G10" s="53">
-        <f>66-SUM(B7:F7,H7:I7,K7:N7,P7)</f>
-        <v>10.899999999999999</v>
-      </c>
-      <c r="H10" s="53"/>
+      <c r="E10" s="55">
+        <v>4</v>
+      </c>
+      <c r="G10" s="69"/>
+      <c r="H10" s="69"/>
     </row>
     <row r="11" spans="1:19" x14ac:dyDescent="0.25">
       <c r="B11" s="53"/>
       <c r="C11" s="53"/>
       <c r="E11" s="56"/>
-      <c r="G11" s="53"/>
-      <c r="H11" s="53"/>
+      <c r="G11" s="69"/>
+      <c r="H11" s="69"/>
     </row>
     <row r="12" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A12" s="6"/>
@@ -1890,14 +1868,14 @@
     </row>
     <row r="17" spans="1:19" x14ac:dyDescent="0.25">
       <c r="B17" s="50" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C17" s="50"/>
       <c r="D17" s="50"/>
       <c r="E17" s="50"/>
       <c r="F17" s="50"/>
       <c r="H17" s="42" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="I17" s="57"/>
       <c r="J17" s="43"/>
@@ -1912,28 +1890,28 @@
     </row>
     <row r="18" spans="1:19" ht="48.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B18" s="3" t="s">
-        <v>147</v>
+        <v>143</v>
       </c>
       <c r="C18" s="3" t="s">
-        <v>148</v>
+        <v>144</v>
       </c>
       <c r="D18" s="3" t="s">
-        <v>149</v>
+        <v>145</v>
       </c>
       <c r="E18" s="3" t="s">
+        <v>91</v>
+      </c>
+      <c r="F18" s="3" t="s">
         <v>92</v>
       </c>
-      <c r="F18" s="3" t="s">
+      <c r="H18" s="3" t="s">
         <v>93</v>
       </c>
-      <c r="H18" s="3" t="s">
+      <c r="I18" s="2" t="s">
+        <v>95</v>
+      </c>
+      <c r="J18" s="3" t="s">
         <v>94</v>
-      </c>
-      <c r="I18" s="2" t="s">
-        <v>96</v>
-      </c>
-      <c r="J18" s="3" t="s">
-        <v>95</v>
       </c>
       <c r="L18" s="53">
         <f>SUM(B19:F19,H19:J19)</f>
@@ -2010,7 +1988,7 @@
       <c r="K23" s="45"/>
       <c r="L23" s="46"/>
       <c r="N23" s="53" t="s">
-        <v>120</v>
+        <v>214</v>
       </c>
       <c r="O23" s="53"/>
       <c r="Q23" s="7"/>
@@ -2042,51 +2020,57 @@
       <c r="C26" s="50"/>
       <c r="D26" s="50"/>
       <c r="F26" s="50" t="s">
-        <v>199</v>
+        <v>195</v>
       </c>
       <c r="G26" s="50"/>
       <c r="H26" s="50"/>
       <c r="I26" s="50"/>
       <c r="J26" s="7"/>
       <c r="K26" s="42" t="s">
-        <v>119</v>
+        <v>116</v>
       </c>
       <c r="L26" s="43"/>
       <c r="N26" s="9" t="s">
+        <v>212</v>
+      </c>
+      <c r="O26" s="9" t="s">
         <v>67</v>
       </c>
     </row>
     <row r="27" spans="1:19" x14ac:dyDescent="0.25">
       <c r="B27" s="14" t="s">
-        <v>205</v>
+        <v>201</v>
       </c>
       <c r="C27" s="14" t="s">
-        <v>215</v>
+        <v>211</v>
       </c>
       <c r="D27" s="2" t="s">
         <v>11</v>
       </c>
       <c r="F27" s="2" t="s">
-        <v>195</v>
+        <v>191</v>
       </c>
       <c r="G27" s="2" t="s">
-        <v>197</v>
+        <v>193</v>
       </c>
       <c r="H27" s="2" t="s">
-        <v>196</v>
+        <v>192</v>
       </c>
       <c r="I27" s="2" t="s">
-        <v>198</v>
+        <v>194</v>
       </c>
       <c r="K27" s="14" t="s">
         <v>73</v>
       </c>
       <c r="L27" s="2" t="s">
-        <v>118</v>
-      </c>
-      <c r="N27" s="66">
+        <v>115</v>
+      </c>
+      <c r="N27" s="60">
         <f>(K29/30*0.4*5)+(B29/25*0.3*5)+(0.3*F29)</f>
-        <v>4.2733333333333334</v>
+        <v>4.9399999999999995</v>
+      </c>
+      <c r="O27" s="54">
+        <v>5</v>
       </c>
     </row>
     <row r="28" spans="1:19" x14ac:dyDescent="0.25">
@@ -2114,8 +2098,11 @@
       <c r="K28" s="2">
         <v>20</v>
       </c>
-      <c r="L28" s="2"/>
-      <c r="N28" s="67"/>
+      <c r="L28" s="2">
+        <v>10</v>
+      </c>
+      <c r="N28" s="61"/>
+      <c r="O28" s="54"/>
     </row>
     <row r="29" spans="1:19" x14ac:dyDescent="0.25">
       <c r="B29" s="51">
@@ -2132,7 +2119,7 @@
       <c r="I29" s="51"/>
       <c r="K29" s="51">
         <f>SUM(K28:L28)</f>
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="L29" s="51"/>
       <c r="N29" s="34"/>
@@ -2183,16 +2170,16 @@
     </row>
     <row r="36" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B36" s="50" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="C36" s="50"/>
       <c r="D36" s="7"/>
-      <c r="E36" s="42" t="s">
-        <v>135</v>
-      </c>
-      <c r="F36" s="57"/>
-      <c r="G36" s="57"/>
-      <c r="H36" s="43"/>
+      <c r="E36" s="50" t="s">
+        <v>131</v>
+      </c>
+      <c r="F36" s="50"/>
+      <c r="G36" s="50"/>
+      <c r="H36" s="7"/>
     </row>
     <row r="37" spans="2:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B37" s="2" t="s">
@@ -2202,16 +2189,13 @@
         <v>7</v>
       </c>
       <c r="E37" s="3" t="s">
-        <v>101</v>
+        <v>98</v>
       </c>
       <c r="F37" s="3" t="s">
-        <v>102</v>
+        <v>99</v>
       </c>
       <c r="G37" s="2" t="s">
-        <v>99</v>
-      </c>
-      <c r="H37" s="2" t="s">
-        <v>100</v>
+        <v>213</v>
       </c>
       <c r="O37" s="7"/>
     </row>
@@ -2230,17 +2214,18 @@
         <f>G46</f>
         <v>29</v>
       </c>
-      <c r="G38" s="2"/>
-      <c r="H38" s="2"/>
+      <c r="G38" s="2">
+        <v>2</v>
+      </c>
       <c r="O38" s="7"/>
     </row>
     <row r="41" spans="2:15" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B41" s="64" t="s">
-        <v>117</v>
-      </c>
-      <c r="C41" s="65"/>
+      <c r="B41" s="58" t="s">
+        <v>114</v>
+      </c>
+      <c r="C41" s="59"/>
       <c r="F41" s="53" t="s">
-        <v>102</v>
+        <v>99</v>
       </c>
       <c r="G41" s="53"/>
       <c r="I41" s="9" t="s">
@@ -2251,33 +2236,33 @@
     </row>
     <row r="42" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B42" s="2" t="s">
-        <v>103</v>
+        <v>100</v>
       </c>
       <c r="C42" s="2">
         <v>2</v>
       </c>
       <c r="F42" s="2" t="s">
-        <v>114</v>
+        <v>111</v>
       </c>
       <c r="G42" s="2">
         <v>9</v>
       </c>
       <c r="I42" s="2">
-        <f>SUM(B38:C38,E38:H38)</f>
-        <v>91</v>
+        <f>SUM(B38:C38,E38:G38)</f>
+        <v>93</v>
       </c>
       <c r="J42" s="7"/>
       <c r="L42" s="7"/>
     </row>
     <row r="43" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B43" s="2" t="s">
-        <v>104</v>
+        <v>101</v>
       </c>
       <c r="C43" s="2">
         <v>2</v>
       </c>
       <c r="F43" s="2" t="s">
-        <v>115</v>
+        <v>112</v>
       </c>
       <c r="G43" s="2">
         <v>10</v>
@@ -2287,13 +2272,13 @@
     </row>
     <row r="44" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B44" s="2" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="C44" s="2">
         <v>3</v>
       </c>
       <c r="F44" s="2" t="s">
-        <v>116</v>
+        <v>113</v>
       </c>
       <c r="G44" s="2">
         <v>10</v>
@@ -2304,7 +2289,7 @@
     </row>
     <row r="45" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B45" s="2" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="C45" s="2">
         <v>4</v>
@@ -2313,7 +2298,7 @@
     </row>
     <row r="46" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B46" s="2" t="s">
-        <v>107</v>
+        <v>104</v>
       </c>
       <c r="C46" s="2">
         <v>4</v>
@@ -2331,13 +2316,13 @@
     </row>
     <row r="47" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B47" s="2" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="C47" s="2"/>
     </row>
     <row r="48" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B48" s="2" t="s">
-        <v>109</v>
+        <v>106</v>
       </c>
       <c r="C48" s="2">
         <v>2</v>
@@ -2346,7 +2331,7 @@
     </row>
     <row r="49" spans="1:19" x14ac:dyDescent="0.25">
       <c r="B49" s="2" t="s">
-        <v>110</v>
+        <v>107</v>
       </c>
       <c r="C49" s="2">
         <v>2</v>
@@ -2354,7 +2339,7 @@
     </row>
     <row r="50" spans="1:19" x14ac:dyDescent="0.25">
       <c r="B50" s="2" t="s">
-        <v>111</v>
+        <v>108</v>
       </c>
       <c r="C50" s="2">
         <v>2</v>
@@ -2362,7 +2347,7 @@
     </row>
     <row r="51" spans="1:19" x14ac:dyDescent="0.25">
       <c r="B51" s="2" t="s">
-        <v>112</v>
+        <v>109</v>
       </c>
       <c r="C51" s="2">
         <v>4</v>
@@ -2370,7 +2355,7 @@
     </row>
     <row r="52" spans="1:19" x14ac:dyDescent="0.25">
       <c r="B52" s="2" t="s">
-        <v>113</v>
+        <v>110</v>
       </c>
       <c r="C52" s="2"/>
     </row>
@@ -2461,7 +2446,7 @@
       <c r="J61" s="50"/>
       <c r="K61" s="50"/>
       <c r="M61" s="50" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="N61" s="50"/>
       <c r="O61" s="50"/>
@@ -2497,7 +2482,7 @@
         <v>81</v>
       </c>
       <c r="J62" s="2" t="s">
-        <v>200</v>
+        <v>196</v>
       </c>
       <c r="K62" s="2" t="s">
         <v>85</v>
@@ -2515,10 +2500,10 @@
         <v>71</v>
       </c>
       <c r="R62" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="S62" s="2" t="s">
         <v>88</v>
-      </c>
-      <c r="S62" s="2" t="s">
-        <v>89</v>
       </c>
     </row>
     <row r="63" spans="1:19" x14ac:dyDescent="0.25">
@@ -2535,10 +2520,10 @@
         <v>2</v>
       </c>
       <c r="F63" s="2" t="s">
-        <v>182</v>
+        <v>178</v>
       </c>
       <c r="G63" s="2" t="s">
-        <v>182</v>
+        <v>178</v>
       </c>
       <c r="H63" s="2">
         <v>2</v>
@@ -2568,7 +2553,7 @@
         <v>25</v>
       </c>
       <c r="S63" s="2">
-        <v>8</v>
+        <v>7.5</v>
       </c>
     </row>
     <row r="66" spans="2:8" x14ac:dyDescent="0.25">
@@ -2580,13 +2565,13 @@
         <v>67</v>
       </c>
       <c r="G66" s="35" t="s">
-        <v>214</v>
+        <v>210</v>
       </c>
       <c r="H66" s="11"/>
     </row>
     <row r="67" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B67" s="53">
-        <f>SUM(B63:K63,M63:P63,R63:S63,G67)</f>
+        <f>_xlfn.CEILING.MATH(SUM(B63:K63,M63:P63,R63:S63,G67))</f>
         <v>98</v>
       </c>
       <c r="C67" s="53"/>
@@ -2606,7 +2591,7 @@
       <c r="H68" s="7"/>
     </row>
   </sheetData>
-  <mergeCells count="38">
+  <mergeCells count="37">
     <mergeCell ref="O18:O19"/>
     <mergeCell ref="B14:H15"/>
     <mergeCell ref="K5:N5"/>
@@ -2619,10 +2604,9 @@
     <mergeCell ref="H5:I5"/>
     <mergeCell ref="N23:O24"/>
     <mergeCell ref="B36:C36"/>
-    <mergeCell ref="E36:H36"/>
-    <mergeCell ref="G9:H9"/>
     <mergeCell ref="L17:M17"/>
     <mergeCell ref="N27:N28"/>
+    <mergeCell ref="O27:O28"/>
     <mergeCell ref="B66:C66"/>
     <mergeCell ref="B67:C68"/>
     <mergeCell ref="B9:C9"/>
@@ -2630,7 +2614,6 @@
     <mergeCell ref="G67:G68"/>
     <mergeCell ref="E67:E68"/>
     <mergeCell ref="E10:E11"/>
-    <mergeCell ref="G10:H11"/>
     <mergeCell ref="B17:F17"/>
     <mergeCell ref="H17:J17"/>
     <mergeCell ref="F26:I26"/>
@@ -2645,6 +2628,7 @@
     <mergeCell ref="M61:P61"/>
     <mergeCell ref="F29:I29"/>
     <mergeCell ref="B29:D29"/>
+    <mergeCell ref="E36:G36"/>
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2681,7 +2665,7 @@
     <row r="1" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="2" spans="1:19" x14ac:dyDescent="0.25">
       <c r="B2" s="44" t="s">
-        <v>121</v>
+        <v>117</v>
       </c>
       <c r="C2" s="45"/>
       <c r="D2" s="45"/>
@@ -2862,7 +2846,7 @@
     <row r="13" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="14" spans="1:19" x14ac:dyDescent="0.25">
       <c r="B14" s="44" t="s">
-        <v>122</v>
+        <v>118</v>
       </c>
       <c r="C14" s="45"/>
       <c r="D14" s="45"/>
@@ -2974,7 +2958,7 @@
     <row r="22" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="23" spans="1:19" x14ac:dyDescent="0.25">
       <c r="B23" s="44" t="s">
-        <v>123</v>
+        <v>119</v>
       </c>
       <c r="C23" s="45"/>
       <c r="D23" s="45"/>
@@ -3047,7 +3031,7 @@
       <c r="K27" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="M27" s="68">
+      <c r="M27" s="62">
         <f>SUM(B28:C28,E28:G28,I28:K28)</f>
         <v>36</v>
       </c>
@@ -3082,7 +3066,7 @@
       <c r="K28" s="2">
         <v>3.2</v>
       </c>
-      <c r="M28" s="68"/>
+      <c r="M28" s="62"/>
       <c r="N28" s="7"/>
       <c r="O28" s="54"/>
       <c r="P28" s="8"/>
@@ -3111,7 +3095,7 @@
     <row r="31" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="32" spans="1:19" x14ac:dyDescent="0.25">
       <c r="B32" s="44" t="s">
-        <v>124</v>
+        <v>120</v>
       </c>
       <c r="C32" s="45"/>
       <c r="D32" s="45"/>
@@ -3199,10 +3183,10 @@
       <c r="O37" s="7"/>
     </row>
     <row r="40" spans="2:15" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B40" s="64" t="s">
+      <c r="B40" s="58" t="s">
         <v>35</v>
       </c>
-      <c r="C40" s="65"/>
+      <c r="C40" s="59"/>
       <c r="F40" s="53" t="s">
         <v>36</v>
       </c>
@@ -3424,7 +3408,7 @@
     <row r="57" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="58" spans="1:19" x14ac:dyDescent="0.25">
       <c r="B58" s="44" t="s">
-        <v>125</v>
+        <v>121</v>
       </c>
       <c r="C58" s="45"/>
       <c r="D58" s="45"/>
@@ -3627,7 +3611,7 @@
     <row r="71" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="72" spans="1:19" x14ac:dyDescent="0.25">
       <c r="B72" s="44" t="s">
-        <v>126</v>
+        <v>122</v>
       </c>
       <c r="C72" s="45"/>
       <c r="D72" s="45"/>
@@ -3649,28 +3633,28 @@
     </row>
     <row r="75" spans="1:19" x14ac:dyDescent="0.25">
       <c r="B75" s="4" t="s">
+        <v>123</v>
+      </c>
+      <c r="C75" s="4" t="s">
+        <v>124</v>
+      </c>
+      <c r="D75" s="4" t="s">
+        <v>125</v>
+      </c>
+      <c r="E75" s="4" t="s">
+        <v>126</v>
+      </c>
+      <c r="F75" s="4" t="s">
         <v>127</v>
       </c>
-      <c r="C75" s="4" t="s">
+      <c r="G75" s="4" t="s">
         <v>128</v>
       </c>
-      <c r="D75" s="4" t="s">
+      <c r="H75" s="4" t="s">
         <v>129</v>
       </c>
-      <c r="E75" s="4" t="s">
+      <c r="I75" s="4" t="s">
         <v>130</v>
-      </c>
-      <c r="F75" s="4" t="s">
-        <v>131</v>
-      </c>
-      <c r="G75" s="4" t="s">
-        <v>132</v>
-      </c>
-      <c r="H75" s="4" t="s">
-        <v>133</v>
-      </c>
-      <c r="I75" s="4" t="s">
-        <v>134</v>
       </c>
       <c r="K75" s="52" t="s">
         <v>22</v>
@@ -3791,16 +3775,16 @@
     <row r="1" spans="2:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="2" spans="2:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="C2" s="15" t="s">
-        <v>136</v>
+        <v>132</v>
       </c>
       <c r="D2" s="15" t="s">
-        <v>137</v>
+        <v>133</v>
       </c>
       <c r="E2" s="15" t="s">
-        <v>171</v>
+        <v>167</v>
       </c>
       <c r="F2" s="15" t="s">
-        <v>183</v>
+        <v>179</v>
       </c>
     </row>
     <row r="3" spans="2:6" x14ac:dyDescent="0.25">
@@ -3814,10 +3798,10 @@
         <v>45763</v>
       </c>
       <c r="E3" s="21" t="s">
-        <v>138</v>
+        <v>134</v>
       </c>
       <c r="F3" s="19" t="s">
-        <v>172</v>
+        <v>168</v>
       </c>
     </row>
     <row r="4" spans="2:6" x14ac:dyDescent="0.25">
@@ -3831,10 +3815,10 @@
         <v>45812</v>
       </c>
       <c r="E4" s="36" t="s">
-        <v>139</v>
+        <v>135</v>
       </c>
       <c r="F4" s="22" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
     </row>
     <row r="5" spans="2:6" x14ac:dyDescent="0.25">
@@ -3848,10 +3832,10 @@
         <v>45817</v>
       </c>
       <c r="E5" s="40" t="s">
-        <v>140</v>
+        <v>136</v>
       </c>
       <c r="F5" s="41" t="s">
-        <v>141</v>
+        <v>137</v>
       </c>
     </row>
     <row r="6" spans="2:6" x14ac:dyDescent="0.25">
@@ -3868,10 +3852,10 @@
         <v>45729</v>
       </c>
       <c r="E7" s="22" t="s">
-        <v>103</v>
+        <v>100</v>
       </c>
       <c r="F7" s="22" t="s">
-        <v>142</v>
+        <v>138</v>
       </c>
     </row>
     <row r="8" spans="2:6" x14ac:dyDescent="0.25">
@@ -3885,10 +3869,10 @@
         <v>45743</v>
       </c>
       <c r="E8" s="22" t="s">
-        <v>104</v>
+        <v>101</v>
       </c>
       <c r="F8" s="22" t="s">
-        <v>143</v>
+        <v>139</v>
       </c>
     </row>
     <row r="9" spans="2:6" x14ac:dyDescent="0.25">
@@ -3902,10 +3886,10 @@
         <v>45757</v>
       </c>
       <c r="E9" s="22" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="F9" s="22" t="s">
-        <v>144</v>
+        <v>140</v>
       </c>
     </row>
     <row r="10" spans="2:6" x14ac:dyDescent="0.25">
@@ -3919,10 +3903,10 @@
         <v>45785</v>
       </c>
       <c r="E10" s="22" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="F10" s="22" t="s">
-        <v>145</v>
+        <v>141</v>
       </c>
     </row>
     <row r="11" spans="2:6" x14ac:dyDescent="0.25">
@@ -3936,10 +3920,10 @@
         <v>45799</v>
       </c>
       <c r="E11" s="22" t="s">
-        <v>107</v>
+        <v>104</v>
       </c>
       <c r="F11" s="22" t="s">
-        <v>146</v>
+        <v>142</v>
       </c>
     </row>
     <row r="12" spans="2:6" x14ac:dyDescent="0.25">
@@ -3950,7 +3934,7 @@
         <v>1</v>
       </c>
       <c r="C13" s="24" t="s">
-        <v>150</v>
+        <v>146</v>
       </c>
       <c r="D13" s="23">
         <v>45728</v>
@@ -3959,7 +3943,7 @@
         <v>84</v>
       </c>
       <c r="F13" s="22" t="s">
-        <v>151</v>
+        <v>147</v>
       </c>
     </row>
     <row r="14" spans="2:6" x14ac:dyDescent="0.25">
@@ -3967,16 +3951,16 @@
         <v>1</v>
       </c>
       <c r="C14" s="24" t="s">
-        <v>150</v>
+        <v>146</v>
       </c>
       <c r="D14" s="23">
         <v>45747</v>
       </c>
       <c r="E14" s="22" t="s">
+        <v>148</v>
+      </c>
+      <c r="F14" s="22" t="s">
         <v>152</v>
-      </c>
-      <c r="F14" s="22" t="s">
-        <v>156</v>
       </c>
     </row>
     <row r="15" spans="2:6" x14ac:dyDescent="0.25">
@@ -3984,16 +3968,16 @@
         <v>1</v>
       </c>
       <c r="C15" s="24" t="s">
-        <v>150</v>
+        <v>146</v>
       </c>
       <c r="D15" s="23">
         <v>45784</v>
       </c>
       <c r="E15" s="22" t="s">
-        <v>153</v>
+        <v>149</v>
       </c>
       <c r="F15" s="22" t="s">
-        <v>154</v>
+        <v>150</v>
       </c>
     </row>
     <row r="16" spans="2:6" x14ac:dyDescent="0.25">
@@ -4001,7 +3985,7 @@
         <v>1</v>
       </c>
       <c r="C16" s="24" t="s">
-        <v>150</v>
+        <v>146</v>
       </c>
       <c r="D16" s="23">
         <v>45806</v>
@@ -4010,7 +3994,7 @@
         <v>85</v>
       </c>
       <c r="F16" s="22" t="s">
-        <v>155</v>
+        <v>151</v>
       </c>
     </row>
     <row r="17" spans="2:6" x14ac:dyDescent="0.25">
@@ -4018,16 +4002,16 @@
         <v>1</v>
       </c>
       <c r="C17" s="24" t="s">
-        <v>150</v>
+        <v>146</v>
       </c>
       <c r="D17" s="23">
         <v>45817</v>
       </c>
       <c r="E17" s="22" t="s">
-        <v>158</v>
+        <v>154</v>
       </c>
       <c r="F17" s="24" t="s">
-        <v>157</v>
+        <v>153</v>
       </c>
     </row>
     <row r="18" spans="2:6" x14ac:dyDescent="0.25">
@@ -4035,16 +4019,16 @@
         <v>1</v>
       </c>
       <c r="C18" s="24" t="s">
-        <v>150</v>
+        <v>146</v>
       </c>
       <c r="D18" s="23">
         <v>45819</v>
       </c>
       <c r="E18" s="22" t="s">
-        <v>160</v>
+        <v>156</v>
       </c>
       <c r="F18" s="24" t="s">
-        <v>159</v>
+        <v>155</v>
       </c>
     </row>
     <row r="19" spans="2:6" x14ac:dyDescent="0.25">
@@ -4056,13 +4040,13 @@
         <v>1</v>
       </c>
       <c r="C20" s="24" t="s">
-        <v>150</v>
+        <v>146</v>
       </c>
       <c r="D20" s="23">
         <v>45820</v>
       </c>
       <c r="E20" s="22" t="s">
-        <v>161</v>
+        <v>157</v>
       </c>
     </row>
     <row r="21" spans="2:6" x14ac:dyDescent="0.25">
@@ -4070,13 +4054,13 @@
         <v>1</v>
       </c>
       <c r="C21" s="24" t="s">
-        <v>150</v>
+        <v>146</v>
       </c>
       <c r="D21" s="23">
         <v>45820</v>
       </c>
       <c r="E21" s="22" t="s">
-        <v>162</v>
+        <v>158</v>
       </c>
     </row>
     <row r="22" spans="2:6" x14ac:dyDescent="0.25">
@@ -4094,10 +4078,10 @@
         <v>45728</v>
       </c>
       <c r="E23" s="22" t="s">
-        <v>169</v>
+        <v>165</v>
       </c>
       <c r="F23" s="22" t="s">
-        <v>174</v>
+        <v>170</v>
       </c>
     </row>
     <row r="24" spans="2:6" x14ac:dyDescent="0.25">
@@ -4111,10 +4095,10 @@
         <v>45742</v>
       </c>
       <c r="E24" s="22" t="s">
-        <v>169</v>
+        <v>165</v>
       </c>
       <c r="F24" s="22" t="s">
-        <v>175</v>
+        <v>171</v>
       </c>
     </row>
     <row r="25" spans="2:6" x14ac:dyDescent="0.25">
@@ -4128,10 +4112,10 @@
         <v>45756</v>
       </c>
       <c r="E25" s="22" t="s">
-        <v>169</v>
+        <v>165</v>
       </c>
       <c r="F25" s="22" t="s">
-        <v>176</v>
+        <v>172</v>
       </c>
     </row>
     <row r="26" spans="2:6" x14ac:dyDescent="0.25">
@@ -4145,10 +4129,10 @@
         <v>45770</v>
       </c>
       <c r="E26" s="22" t="s">
-        <v>168</v>
+        <v>164</v>
       </c>
       <c r="F26" s="24" t="s">
-        <v>180</v>
+        <v>176</v>
       </c>
     </row>
     <row r="27" spans="2:6" x14ac:dyDescent="0.25">
@@ -4162,10 +4146,10 @@
         <v>45784</v>
       </c>
       <c r="E27" s="22" t="s">
-        <v>169</v>
+        <v>165</v>
       </c>
       <c r="F27" s="22" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
     </row>
     <row r="28" spans="2:6" x14ac:dyDescent="0.25">
@@ -4179,10 +4163,10 @@
         <v>45798</v>
       </c>
       <c r="E28" s="22" t="s">
-        <v>169</v>
+        <v>165</v>
       </c>
       <c r="F28" s="22" t="s">
-        <v>178</v>
+        <v>174</v>
       </c>
     </row>
     <row r="29" spans="2:6" x14ac:dyDescent="0.25">
@@ -4196,10 +4180,10 @@
         <v>45812</v>
       </c>
       <c r="E29" s="22" t="s">
-        <v>168</v>
+        <v>164</v>
       </c>
       <c r="F29" s="24" t="s">
-        <v>206</v>
+        <v>202</v>
       </c>
     </row>
     <row r="30" spans="2:6" x14ac:dyDescent="0.25">
@@ -4216,10 +4200,10 @@
         <v>45764</v>
       </c>
       <c r="E31" s="22" t="s">
-        <v>138</v>
+        <v>134</v>
       </c>
       <c r="F31" s="22" t="s">
-        <v>181</v>
+        <v>177</v>
       </c>
     </row>
     <row r="32" spans="2:6" x14ac:dyDescent="0.25">
@@ -4233,7 +4217,7 @@
         <v>45815</v>
       </c>
       <c r="E32" s="22" t="s">
-        <v>207</v>
+        <v>203</v>
       </c>
     </row>
     <row r="33" spans="2:6" x14ac:dyDescent="0.25">
@@ -4247,10 +4231,10 @@
         <v>45814</v>
       </c>
       <c r="E33" s="22" t="s">
-        <v>139</v>
+        <v>135</v>
       </c>
       <c r="F33" s="22" t="s">
-        <v>212</v>
+        <v>208</v>
       </c>
     </row>
     <row r="35" spans="2:6" x14ac:dyDescent="0.25">
@@ -4264,10 +4248,10 @@
         <v>45767</v>
       </c>
       <c r="E35" s="22" t="s">
-        <v>170</v>
+        <v>166</v>
       </c>
       <c r="F35" s="22" t="s">
-        <v>179</v>
+        <v>175</v>
       </c>
     </row>
     <row r="36" spans="2:6" x14ac:dyDescent="0.25">
@@ -4281,7 +4265,7 @@
         <v>45775</v>
       </c>
       <c r="E36" s="22" t="s">
-        <v>138</v>
+        <v>134</v>
       </c>
     </row>
     <row r="37" spans="2:6" x14ac:dyDescent="0.25">
@@ -4295,10 +4279,10 @@
         <v>45794</v>
       </c>
       <c r="E37" s="22" t="s">
-        <v>203</v>
+        <v>199</v>
       </c>
       <c r="F37" s="22" t="s">
-        <v>202</v>
+        <v>198</v>
       </c>
     </row>
     <row r="39" spans="2:6" x14ac:dyDescent="0.25">
@@ -4312,10 +4296,10 @@
         <v>45784</v>
       </c>
       <c r="E39" s="22" t="s">
-        <v>213</v>
+        <v>209</v>
       </c>
       <c r="F39" s="22" t="s">
-        <v>209</v>
+        <v>205</v>
       </c>
     </row>
     <row r="40" spans="2:6" x14ac:dyDescent="0.25">
@@ -4329,10 +4313,10 @@
         <v>45798</v>
       </c>
       <c r="E40" s="22" t="s">
-        <v>208</v>
+        <v>204</v>
       </c>
       <c r="F40" s="22" t="s">
-        <v>209</v>
+        <v>205</v>
       </c>
     </row>
     <row r="41" spans="2:6" x14ac:dyDescent="0.25">
@@ -4346,10 +4330,10 @@
         <v>45805</v>
       </c>
       <c r="E41" s="22" t="s">
-        <v>211</v>
+        <v>207</v>
       </c>
       <c r="F41" s="22" t="s">
-        <v>210</v>
+        <v>206</v>
       </c>
     </row>
   </sheetData>
@@ -4377,54 +4361,54 @@
   <sheetData>
     <row r="1" spans="2:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="2" spans="2:12" ht="23.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B2" s="69" t="s">
-        <v>192</v>
-      </c>
-      <c r="C2" s="70"/>
-      <c r="D2" s="71"/>
-      <c r="F2" s="69" t="s">
-        <v>193</v>
-      </c>
-      <c r="G2" s="70"/>
-      <c r="H2" s="71"/>
-      <c r="J2" s="69" t="s">
-        <v>194</v>
-      </c>
-      <c r="K2" s="70"/>
-      <c r="L2" s="71"/>
+      <c r="B2" s="63" t="s">
+        <v>188</v>
+      </c>
+      <c r="C2" s="64"/>
+      <c r="D2" s="65"/>
+      <c r="F2" s="63" t="s">
+        <v>189</v>
+      </c>
+      <c r="G2" s="64"/>
+      <c r="H2" s="65"/>
+      <c r="J2" s="63" t="s">
+        <v>190</v>
+      </c>
+      <c r="K2" s="64"/>
+      <c r="L2" s="65"/>
     </row>
     <row r="3" spans="2:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B3" s="29" t="s">
-        <v>136</v>
+        <v>132</v>
       </c>
       <c r="C3" s="30" t="s">
-        <v>185</v>
+        <v>181</v>
       </c>
       <c r="D3" s="31" t="s">
-        <v>184</v>
+        <v>180</v>
       </c>
       <c r="F3" s="29" t="s">
-        <v>136</v>
+        <v>132</v>
       </c>
       <c r="G3" s="30" t="s">
-        <v>185</v>
+        <v>181</v>
       </c>
       <c r="H3" s="31" t="s">
-        <v>184</v>
+        <v>180</v>
       </c>
       <c r="J3" s="29" t="s">
-        <v>136</v>
+        <v>132</v>
       </c>
       <c r="K3" s="30" t="s">
-        <v>185</v>
+        <v>181</v>
       </c>
       <c r="L3" s="31" t="s">
-        <v>184</v>
+        <v>180</v>
       </c>
     </row>
     <row r="4" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B4" s="32" t="s">
-        <v>121</v>
+        <v>117</v>
       </c>
       <c r="C4" s="14">
         <v>4</v>
@@ -4438,9 +4422,11 @@
       <c r="G4" s="14">
         <v>5</v>
       </c>
-      <c r="H4" s="14"/>
+      <c r="H4" s="14">
+        <v>4</v>
+      </c>
       <c r="J4" s="32" t="s">
-        <v>187</v>
+        <v>183</v>
       </c>
       <c r="K4" s="14">
         <v>4</v>
@@ -4449,7 +4435,7 @@
     </row>
     <row r="5" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B5" s="33" t="s">
-        <v>122</v>
+        <v>118</v>
       </c>
       <c r="C5" s="2">
         <v>6</v>
@@ -4463,9 +4449,11 @@
       <c r="G5" s="2">
         <v>4</v>
       </c>
-      <c r="H5" s="2"/>
+      <c r="H5" s="2">
+        <v>5</v>
+      </c>
       <c r="J5" s="33" t="s">
-        <v>188</v>
+        <v>184</v>
       </c>
       <c r="K5" s="2">
         <v>4</v>
@@ -4474,7 +4462,7 @@
     </row>
     <row r="6" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B6" s="33" t="s">
-        <v>123</v>
+        <v>119</v>
       </c>
       <c r="C6" s="2">
         <v>4</v>
@@ -4492,7 +4480,7 @@
         <v>4.5</v>
       </c>
       <c r="J6" s="33" t="s">
-        <v>189</v>
+        <v>185</v>
       </c>
       <c r="K6" s="2">
         <v>5</v>
@@ -4501,7 +4489,7 @@
     </row>
     <row r="7" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B7" s="33" t="s">
-        <v>124</v>
+        <v>120</v>
       </c>
       <c r="C7" s="2">
         <v>4</v>
@@ -4519,7 +4507,7 @@
         <v>5</v>
       </c>
       <c r="J7" s="33" t="s">
-        <v>190</v>
+        <v>186</v>
       </c>
       <c r="K7" s="2">
         <v>5</v>
@@ -4528,7 +4516,7 @@
     </row>
     <row r="8" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B8" s="33" t="s">
-        <v>125</v>
+        <v>121</v>
       </c>
       <c r="C8" s="2">
         <v>10</v>
@@ -4546,7 +4534,7 @@
         <v>5</v>
       </c>
       <c r="J8" s="33" t="s">
-        <v>191</v>
+        <v>187</v>
       </c>
       <c r="K8" s="2">
         <v>12</v>
@@ -4555,7 +4543,7 @@
     </row>
     <row r="9" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B9" s="33" t="s">
-        <v>126</v>
+        <v>122</v>
       </c>
       <c r="C9" s="2">
         <v>2</v>
@@ -4572,26 +4560,26 @@
     </row>
     <row r="10" spans="2:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="11" spans="2:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B11" s="72" t="s">
-        <v>186</v>
-      </c>
-      <c r="C11" s="73"/>
+      <c r="B11" s="66" t="s">
+        <v>182</v>
+      </c>
+      <c r="C11" s="67"/>
       <c r="D11" s="28">
         <f>(D4*C4+D5*C5+D6*C6+D7*C7+D8*C8+D9*C9)/30</f>
         <v>4.4333333333333336</v>
       </c>
-      <c r="F11" s="72" t="s">
-        <v>186</v>
-      </c>
-      <c r="G11" s="73"/>
+      <c r="F11" s="66" t="s">
+        <v>182</v>
+      </c>
+      <c r="G11" s="67"/>
       <c r="H11" s="28">
         <f>(H4*G4+H5*G5+H6*G6+H7*G7+H8*G8)/30</f>
-        <v>3.4166666666666665</v>
-      </c>
-      <c r="J11" s="72" t="s">
-        <v>186</v>
-      </c>
-      <c r="K11" s="73"/>
+        <v>4.75</v>
+      </c>
+      <c r="J11" s="66" t="s">
+        <v>182</v>
+      </c>
+      <c r="K11" s="67"/>
       <c r="L11" s="28">
         <f>(L4*K4+L5*K5+L6*K6+L7*K7+L8*K8)/30</f>
         <v>0</v>

</xml_diff>

<commit_message>
2nd semester successfully ended - final points and marks
</commit_message>
<xml_diff>
--- a/IoT-points-schedule.xlsx
+++ b/IoT-points-schedule.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\dodo\Desktop\IoT-studies\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{68C43C02-BBA6-40DA-B027-5612C705B080}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8405FF14-EBBA-4923-9B6D-DAC24ED607FD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="25440" windowHeight="15390" xr2:uid="{F85F5544-1FE8-4920-A5D4-192A98B113BD}"/>
+    <workbookView xWindow="25080" yWindow="300" windowWidth="19440" windowHeight="15000" activeTab="2" xr2:uid="{F85F5544-1FE8-4920-A5D4-192A98B113BD}"/>
   </bookViews>
   <sheets>
     <sheet name="II-semestr-25L" sheetId="1" r:id="rId1"/>
@@ -1059,7 +1059,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="70">
+  <cellXfs count="68">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1267,12 +1267,6 @@
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1786,7 +1780,9 @@
       <c r="L7" s="2">
         <v>13.5</v>
       </c>
-      <c r="M7" s="2"/>
+      <c r="M7" s="2">
+        <v>5</v>
+      </c>
       <c r="N7" s="2">
         <v>6</v>
       </c>
@@ -1802,27 +1798,27 @@
       <c r="E9" s="9" t="s">
         <v>67</v>
       </c>
-      <c r="G9" s="68"/>
-      <c r="H9" s="68"/>
+      <c r="G9" s="11"/>
+      <c r="H9" s="11"/>
     </row>
     <row r="10" spans="1:19" x14ac:dyDescent="0.25">
       <c r="B10" s="53">
         <f>SUM(B7:F7,H7:I7,K7:N7,P7)</f>
-        <v>94.1</v>
+        <v>99.1</v>
       </c>
       <c r="C10" s="53"/>
       <c r="E10" s="55">
         <v>4</v>
       </c>
-      <c r="G10" s="69"/>
-      <c r="H10" s="69"/>
+      <c r="G10" s="7"/>
+      <c r="H10" s="7"/>
     </row>
     <row r="11" spans="1:19" x14ac:dyDescent="0.25">
       <c r="B11" s="53"/>
       <c r="C11" s="53"/>
       <c r="E11" s="56"/>
-      <c r="G11" s="69"/>
-      <c r="H11" s="69"/>
+      <c r="G11" s="7"/>
+      <c r="H11" s="7"/>
     </row>
     <row r="12" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A12" s="6"/>
@@ -2607,6 +2603,7 @@
     <mergeCell ref="L17:M17"/>
     <mergeCell ref="N27:N28"/>
     <mergeCell ref="O27:O28"/>
+    <mergeCell ref="H17:J17"/>
     <mergeCell ref="B66:C66"/>
     <mergeCell ref="B67:C68"/>
     <mergeCell ref="B9:C9"/>
@@ -2615,7 +2612,6 @@
     <mergeCell ref="E67:E68"/>
     <mergeCell ref="E10:E11"/>
     <mergeCell ref="B17:F17"/>
-    <mergeCell ref="H17:J17"/>
     <mergeCell ref="F26:I26"/>
     <mergeCell ref="K26:L26"/>
     <mergeCell ref="B23:L24"/>

</xml_diff>

<commit_message>
Updated schedule - 3rd sem
</commit_message>
<xml_diff>
--- a/IoT-points-schedule.xlsx
+++ b/IoT-points-schedule.xlsx
@@ -1,22 +1,24 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28827"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\dodo\Desktop\IoT-studies\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8405FF14-EBBA-4923-9B6D-DAC24ED607FD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0BB201D0-AF96-4BBA-AE1A-A92AE39289F6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="25080" yWindow="300" windowWidth="19440" windowHeight="15000" activeTab="2" xr2:uid="{F85F5544-1FE8-4920-A5D4-192A98B113BD}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="25440" windowHeight="15390" xr2:uid="{F85F5544-1FE8-4920-A5D4-192A98B113BD}"/>
   </bookViews>
   <sheets>
-    <sheet name="II-semestr-25L" sheetId="1" r:id="rId1"/>
-    <sheet name="I-semestr-24Z" sheetId="2" r:id="rId2"/>
-    <sheet name="Terminy" sheetId="3" r:id="rId3"/>
-    <sheet name="Ostateczne-oceny" sheetId="4" r:id="rId4"/>
+    <sheet name="III-semestr-25Z" sheetId="5" r:id="rId1"/>
+    <sheet name="II-semestr-25L" sheetId="1" r:id="rId2"/>
+    <sheet name="I-semestr-24Z" sheetId="2" r:id="rId3"/>
+    <sheet name="Terminy 25L" sheetId="3" state="hidden" r:id="rId4"/>
+    <sheet name="Terminy 25Z" sheetId="8" r:id="rId5"/>
+    <sheet name="Ostateczne-oceny" sheetId="4" r:id="rId6"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -39,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="342" uniqueCount="215">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="527" uniqueCount="316">
   <si>
     <t>1. Krypto</t>
   </si>
@@ -684,15 +686,319 @@
   </si>
   <si>
     <t>W = (E/30)*0,4*5 + (C/25)*0,3*5 + 0,3L</t>
+  </si>
+  <si>
+    <t>Lab1</t>
+  </si>
+  <si>
+    <t>Lab2</t>
+  </si>
+  <si>
+    <t>Lab3</t>
+  </si>
+  <si>
+    <t>Lab4</t>
+  </si>
+  <si>
+    <t>Lab5</t>
+  </si>
+  <si>
+    <t>Lab6</t>
+  </si>
+  <si>
+    <t>11 grudnia</t>
+  </si>
+  <si>
+    <t>6 listopada</t>
+  </si>
+  <si>
+    <t>19 listopada</t>
+  </si>
+  <si>
+    <t>3 grudnia</t>
+  </si>
+  <si>
+    <t>18 grudnia</t>
+  </si>
+  <si>
+    <t>15 stycznia</t>
+  </si>
+  <si>
+    <t>Badanie właściwości sygnałów z modulacjami cyfrowymi</t>
+  </si>
+  <si>
+    <t>Badanie kanału propagacyjnego</t>
+  </si>
+  <si>
+    <t>Badanie podstawowych elementów toru radiowego</t>
+  </si>
+  <si>
+    <t>Badanie anten</t>
+  </si>
+  <si>
+    <t>Badanie sygnałów CDMA</t>
+  </si>
+  <si>
+    <t>Badanie sygnałów OFDM</t>
+  </si>
+  <si>
+    <t>15 października</t>
+  </si>
+  <si>
+    <t>Ćwiczenia 1</t>
+  </si>
+  <si>
+    <t>22 października</t>
+  </si>
+  <si>
+    <t>29 października</t>
+  </si>
+  <si>
+    <t>17 grudnia</t>
+  </si>
+  <si>
+    <t>Ćwiczenia 4</t>
+  </si>
+  <si>
+    <t>Ćwiczenia 2</t>
+  </si>
+  <si>
+    <t>Ćwiczenia 3</t>
+  </si>
+  <si>
+    <t>Pomiary: obiekty i miary</t>
+  </si>
+  <si>
+    <t>Analiza sygnałów w dziedzinach czasu i częstotliwości</t>
+  </si>
+  <si>
+    <t>Generatory sygnałowe i analizatory obwodów</t>
+  </si>
+  <si>
+    <t>Pomiary sygnałów CDMA i OFDM. Przykład bilansu łącza radiowego</t>
+  </si>
+  <si>
+    <t>Godziny</t>
+  </si>
+  <si>
+    <t xml:space="preserve">14:15-16:10 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">14:15-16:50 </t>
+  </si>
+  <si>
+    <t>12:00-15:00</t>
+  </si>
+  <si>
+    <t>14:00-17:00</t>
+  </si>
+  <si>
+    <t>8:00-11:00</t>
+  </si>
+  <si>
+    <t>20 października</t>
+  </si>
+  <si>
+    <t>14:15-17:00</t>
+  </si>
+  <si>
+    <t>Sala</t>
+  </si>
+  <si>
+    <t>DS400</t>
+  </si>
+  <si>
+    <t>17 listopada</t>
+  </si>
+  <si>
+    <t>24 listopada</t>
+  </si>
+  <si>
+    <t>15 grudnia</t>
+  </si>
+  <si>
+    <t>12 stycznia</t>
+  </si>
+  <si>
+    <t>K1</t>
+  </si>
+  <si>
+    <t>K2</t>
+  </si>
+  <si>
+    <t>Kolokwia [2*25 pkt]</t>
+  </si>
+  <si>
+    <t>Laboratoria [5*5 pkt]</t>
+  </si>
+  <si>
+    <t>Projekty [25 pkt]</t>
+  </si>
+  <si>
+    <t>1. Kolosy: minimum 11 pkt z każdego</t>
+  </si>
+  <si>
+    <t>2. Labki: minimum 2 pkt z każdego</t>
+  </si>
+  <si>
+    <t>3. Labki: minimum 13 pkt łącznie</t>
+  </si>
+  <si>
+    <t>4. Projekty: minimum 13 pkt łącznie</t>
+  </si>
+  <si>
+    <t>ZALICZENIE</t>
+  </si>
+  <si>
+    <t>5. SUMA &gt; 51 pkt</t>
+  </si>
+  <si>
+    <t>Ćwiczenia [4*1,5 pkt]</t>
+  </si>
+  <si>
+    <t>C1</t>
+  </si>
+  <si>
+    <t>C2</t>
+  </si>
+  <si>
+    <t>C3</t>
+  </si>
+  <si>
+    <t>C4</t>
+  </si>
+  <si>
+    <t>Laboratoria [6*4 pkt]</t>
+  </si>
+  <si>
+    <t>Kolokwia [2*15 pkt]</t>
+  </si>
+  <si>
+    <t>Egzamin [40 pkt]</t>
+  </si>
+  <si>
+    <t>K1 [12 pkt]</t>
+  </si>
+  <si>
+    <t>K2 [12 pkt]</t>
+  </si>
+  <si>
+    <t>Aktywność [2 pkt]</t>
+  </si>
+  <si>
+    <t>Egzamin [30 + 20 pkt]</t>
+  </si>
+  <si>
+    <t>W1</t>
+  </si>
+  <si>
+    <t>Zad 1</t>
+  </si>
+  <si>
+    <t>Zad 2</t>
+  </si>
+  <si>
+    <t>Zad 3</t>
+  </si>
+  <si>
+    <t>Zad 4</t>
+  </si>
+  <si>
+    <t>Zad 5</t>
+  </si>
+  <si>
+    <t>Zad 6</t>
+  </si>
+  <si>
+    <t>Etap 1</t>
+  </si>
+  <si>
+    <t>Etap 2</t>
+  </si>
+  <si>
+    <t>Etap 3</t>
+  </si>
+  <si>
+    <t>Prezentacja</t>
+  </si>
+  <si>
+    <t>Etap 1 [3 + 2 pkt]</t>
+  </si>
+  <si>
+    <t>Etap 2 [6 + 4 pkt]</t>
+  </si>
+  <si>
+    <t>Etap 3 [6 + 4 pkt]</t>
+  </si>
+  <si>
+    <t>18/19 listopada</t>
+  </si>
+  <si>
+    <t>Projekt - etap 1</t>
+  </si>
+  <si>
+    <t>16/17 grudnia</t>
+  </si>
+  <si>
+    <t>Projekt - etap 2</t>
+  </si>
+  <si>
+    <t>30 stycznia</t>
+  </si>
+  <si>
+    <t>Projekt - prezentacja finalna</t>
+  </si>
+  <si>
+    <t>Warsztaty [15 * 3 pkt]</t>
+  </si>
+  <si>
+    <t>Egzamin [30 pkt]</t>
+  </si>
+  <si>
+    <t>Projekt [25 pkt]</t>
+  </si>
+  <si>
+    <t>ANG</t>
+  </si>
+  <si>
+    <t>Testy cząstkowe</t>
+  </si>
+  <si>
+    <t>Starter Unit</t>
+  </si>
+  <si>
+    <t>4+</t>
+  </si>
+  <si>
+    <t>1. Warsztaty: minimum 50 %</t>
+  </si>
+  <si>
+    <t>2. Projekt: minimum 50 %</t>
+  </si>
+  <si>
+    <t>3. Egzamin: minimum 50 %</t>
+  </si>
+  <si>
+    <t>1. Ćwiczenia: minimum 12 pkt</t>
+  </si>
+  <si>
+    <t>2. Egzamin: minimum 26 pkt</t>
+  </si>
+  <si>
+    <t>1. Całość: minimum 51 pkt</t>
+  </si>
+  <si>
+    <t>2. Egzamin: minimum 21 pkt</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="2">
+  <numFmts count="3">
     <numFmt numFmtId="164" formatCode="0.0"/>
     <numFmt numFmtId="165" formatCode="[$-415]d\ mmmm\ yyyy;@"/>
+    <numFmt numFmtId="166" formatCode="[$-F800]dddd\,\ mmmm\ dd\,\ yyyy"/>
   </numFmts>
   <fonts count="9" x14ac:knownFonts="1">
     <font>
@@ -766,7 +1072,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="8">
+  <fills count="10">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -806,6 +1112,18 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="2" tint="-9.9978637043366805E-2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFDEEDF4"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.79998168889431442"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1059,7 +1377,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="68">
+  <cellXfs count="98">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1190,51 +1508,102 @@
     <xf numFmtId="0" fontId="7" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1">
+      <extLst>
+        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
+          <xfpb:xfComplement i="0"/>
+        </ext>
+      </extLst>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="8" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1266,6 +1635,45 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="9" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="9" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="9" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="9" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="9" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="9" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1276,11 +1684,11 @@
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <mruColors>
+      <color rgb="FFDEEDF4"/>
       <color rgb="FFFF8585"/>
       <color rgb="FFFDBF8B"/>
       <color rgb="FFFDAF6F"/>
       <color rgb="FFFFCC66"/>
-      <color rgb="FFDEEDF4"/>
       <color rgb="FFE3EAEF"/>
     </mruColors>
   </colors>
@@ -1628,7 +2036,883 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9FFDB1E6-87C0-4917-B2B5-BFB3BFC54144}">
+  <sheetPr>
+    <tabColor theme="5" tint="0.79998168889431442"/>
+  </sheetPr>
+  <dimension ref="A1:V52"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="2" max="2" width="11.42578125" customWidth="1"/>
+    <col min="3" max="3" width="12.28515625" customWidth="1"/>
+    <col min="5" max="5" width="12.140625" customWidth="1"/>
+    <col min="7" max="7" width="12.28515625" customWidth="1"/>
+    <col min="8" max="8" width="11.42578125" customWidth="1"/>
+    <col min="9" max="9" width="9.140625" customWidth="1"/>
+    <col min="17" max="17" width="14.85546875" customWidth="1"/>
+    <col min="18" max="18" width="9.140625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="2" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="B2" s="85" t="s">
+        <v>185</v>
+      </c>
+      <c r="C2" s="86"/>
+      <c r="D2" s="86"/>
+      <c r="E2" s="86"/>
+      <c r="F2" s="86"/>
+      <c r="G2" s="86"/>
+      <c r="H2" s="86"/>
+      <c r="I2" s="86"/>
+      <c r="J2" s="86"/>
+      <c r="K2" s="86"/>
+      <c r="L2" s="86"/>
+      <c r="M2" s="86"/>
+      <c r="N2" s="86"/>
+      <c r="O2" s="86"/>
+      <c r="P2" s="87"/>
+      <c r="R2" s="69" t="s">
+        <v>268</v>
+      </c>
+      <c r="S2" s="69"/>
+      <c r="T2" s="69"/>
+      <c r="U2" s="69"/>
+    </row>
+    <row r="3" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B3" s="88"/>
+      <c r="C3" s="89"/>
+      <c r="D3" s="89"/>
+      <c r="E3" s="89"/>
+      <c r="F3" s="89"/>
+      <c r="G3" s="89"/>
+      <c r="H3" s="89"/>
+      <c r="I3" s="89"/>
+      <c r="J3" s="89"/>
+      <c r="K3" s="89"/>
+      <c r="L3" s="89"/>
+      <c r="M3" s="89"/>
+      <c r="N3" s="89"/>
+      <c r="O3" s="89"/>
+      <c r="P3" s="90"/>
+      <c r="R3" s="66" t="s">
+        <v>264</v>
+      </c>
+      <c r="S3" s="67"/>
+      <c r="T3" s="67"/>
+      <c r="U3" s="68"/>
+    </row>
+    <row r="4" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="R4" s="66" t="s">
+        <v>265</v>
+      </c>
+      <c r="S4" s="67"/>
+      <c r="T4" s="67"/>
+      <c r="U4" s="68"/>
+    </row>
+    <row r="5" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="B5" s="52" t="s">
+        <v>261</v>
+      </c>
+      <c r="C5" s="52"/>
+      <c r="E5" s="52" t="s">
+        <v>262</v>
+      </c>
+      <c r="F5" s="52"/>
+      <c r="G5" s="52"/>
+      <c r="H5" s="52"/>
+      <c r="I5" s="52"/>
+      <c r="K5" s="52" t="s">
+        <v>263</v>
+      </c>
+      <c r="L5" s="52"/>
+      <c r="M5" s="52"/>
+      <c r="N5" s="52"/>
+      <c r="O5" s="52"/>
+      <c r="P5" s="52"/>
+      <c r="R5" s="66" t="s">
+        <v>266</v>
+      </c>
+      <c r="S5" s="67"/>
+      <c r="T5" s="67"/>
+      <c r="U5" s="68"/>
+    </row>
+    <row r="6" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="B6" s="49" t="s">
+        <v>259</v>
+      </c>
+      <c r="C6" s="49" t="s">
+        <v>260</v>
+      </c>
+      <c r="E6" s="49" t="s">
+        <v>215</v>
+      </c>
+      <c r="F6" s="49" t="s">
+        <v>216</v>
+      </c>
+      <c r="G6" s="49" t="s">
+        <v>217</v>
+      </c>
+      <c r="H6" s="49" t="s">
+        <v>218</v>
+      </c>
+      <c r="I6" s="49" t="s">
+        <v>219</v>
+      </c>
+      <c r="K6" s="49" t="s">
+        <v>283</v>
+      </c>
+      <c r="L6" s="49" t="s">
+        <v>284</v>
+      </c>
+      <c r="M6" s="49" t="s">
+        <v>285</v>
+      </c>
+      <c r="N6" s="49" t="s">
+        <v>286</v>
+      </c>
+      <c r="O6" s="49" t="s">
+        <v>287</v>
+      </c>
+      <c r="P6" s="49" t="s">
+        <v>288</v>
+      </c>
+      <c r="R6" s="66" t="s">
+        <v>267</v>
+      </c>
+      <c r="S6" s="67"/>
+      <c r="T6" s="67"/>
+      <c r="U6" s="68"/>
+    </row>
+    <row r="7" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="B7" s="50"/>
+      <c r="C7" s="50"/>
+      <c r="E7" s="49"/>
+      <c r="F7" s="49"/>
+      <c r="G7" s="49"/>
+      <c r="H7" s="49"/>
+      <c r="I7" s="49"/>
+      <c r="K7" s="50"/>
+      <c r="L7" s="50"/>
+      <c r="M7" s="50"/>
+      <c r="N7" s="50"/>
+      <c r="O7" s="50"/>
+      <c r="P7" s="50"/>
+      <c r="R7" s="66" t="s">
+        <v>269</v>
+      </c>
+      <c r="S7" s="67"/>
+      <c r="T7" s="67"/>
+      <c r="U7" s="68"/>
+    </row>
+    <row r="9" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="B9" s="63" t="s">
+        <v>22</v>
+      </c>
+      <c r="C9" s="63"/>
+      <c r="D9" s="1"/>
+      <c r="E9" s="9" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="10" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="B10" s="53">
+        <f>SUM(B7:C7,E7:I7,K7:P7)</f>
+        <v>0</v>
+      </c>
+      <c r="C10" s="53"/>
+      <c r="D10" s="1"/>
+      <c r="E10" s="64"/>
+    </row>
+    <row r="11" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="B11" s="53"/>
+      <c r="C11" s="53"/>
+      <c r="D11" s="1"/>
+      <c r="E11" s="65"/>
+    </row>
+    <row r="12" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A12" s="6"/>
+      <c r="B12" s="6"/>
+      <c r="C12" s="6"/>
+      <c r="D12" s="6"/>
+      <c r="E12" s="6"/>
+      <c r="F12" s="6"/>
+      <c r="G12" s="6"/>
+      <c r="H12" s="6"/>
+      <c r="I12" s="6"/>
+      <c r="J12" s="6"/>
+      <c r="K12" s="6"/>
+      <c r="L12" s="6"/>
+      <c r="M12" s="6"/>
+      <c r="N12" s="6"/>
+      <c r="O12" s="6"/>
+      <c r="P12" s="6"/>
+      <c r="Q12" s="6"/>
+      <c r="R12" s="6"/>
+      <c r="S12" s="6"/>
+      <c r="T12" s="6"/>
+      <c r="U12" s="6"/>
+      <c r="V12" s="6"/>
+    </row>
+    <row r="13" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="14" spans="1:22" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B14" s="85" t="s">
+        <v>186</v>
+      </c>
+      <c r="C14" s="86"/>
+      <c r="D14" s="86"/>
+      <c r="E14" s="86"/>
+      <c r="F14" s="86"/>
+      <c r="G14" s="86"/>
+      <c r="H14" s="86"/>
+      <c r="I14" s="86"/>
+      <c r="J14" s="86"/>
+      <c r="K14" s="86"/>
+      <c r="L14" s="86"/>
+      <c r="M14" s="86"/>
+      <c r="N14" s="86"/>
+      <c r="O14" s="86"/>
+      <c r="P14" s="86"/>
+      <c r="Q14" s="87"/>
+      <c r="S14" s="69" t="s">
+        <v>268</v>
+      </c>
+      <c r="T14" s="69"/>
+      <c r="U14" s="69"/>
+      <c r="V14" s="69"/>
+    </row>
+    <row r="15" spans="1:22" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B15" s="88"/>
+      <c r="C15" s="89"/>
+      <c r="D15" s="89"/>
+      <c r="E15" s="89"/>
+      <c r="F15" s="89"/>
+      <c r="G15" s="89"/>
+      <c r="H15" s="89"/>
+      <c r="I15" s="89"/>
+      <c r="J15" s="89"/>
+      <c r="K15" s="89"/>
+      <c r="L15" s="89"/>
+      <c r="M15" s="89"/>
+      <c r="N15" s="89"/>
+      <c r="O15" s="89"/>
+      <c r="P15" s="89"/>
+      <c r="Q15" s="90"/>
+      <c r="S15" s="66" t="s">
+        <v>314</v>
+      </c>
+      <c r="T15" s="67"/>
+      <c r="U15" s="67"/>
+      <c r="V15" s="68"/>
+    </row>
+    <row r="16" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="S16" s="66" t="s">
+        <v>315</v>
+      </c>
+      <c r="T16" s="67"/>
+      <c r="U16" s="67"/>
+      <c r="V16" s="68"/>
+    </row>
+    <row r="17" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="B17" s="52" t="s">
+        <v>270</v>
+      </c>
+      <c r="C17" s="52"/>
+      <c r="D17" s="52"/>
+      <c r="E17" s="52"/>
+      <c r="G17" s="52" t="s">
+        <v>275</v>
+      </c>
+      <c r="H17" s="52"/>
+      <c r="I17" s="52"/>
+      <c r="J17" s="52"/>
+      <c r="K17" s="52"/>
+      <c r="L17" s="52"/>
+      <c r="N17" s="52" t="s">
+        <v>276</v>
+      </c>
+      <c r="O17" s="52"/>
+      <c r="Q17" s="51" t="s">
+        <v>277</v>
+      </c>
+    </row>
+    <row r="18" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="B18" s="49" t="s">
+        <v>271</v>
+      </c>
+      <c r="C18" s="49" t="s">
+        <v>272</v>
+      </c>
+      <c r="D18" s="49" t="s">
+        <v>273</v>
+      </c>
+      <c r="E18" s="49" t="s">
+        <v>274</v>
+      </c>
+      <c r="G18" s="49" t="s">
+        <v>215</v>
+      </c>
+      <c r="H18" s="49" t="s">
+        <v>216</v>
+      </c>
+      <c r="I18" s="49" t="s">
+        <v>217</v>
+      </c>
+      <c r="J18" s="49" t="s">
+        <v>218</v>
+      </c>
+      <c r="K18" s="49" t="s">
+        <v>219</v>
+      </c>
+      <c r="L18" s="49" t="s">
+        <v>220</v>
+      </c>
+      <c r="N18" s="49" t="s">
+        <v>259</v>
+      </c>
+      <c r="O18" s="49" t="s">
+        <v>260</v>
+      </c>
+      <c r="Q18" s="61"/>
+    </row>
+    <row r="19" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="B19" s="49"/>
+      <c r="C19" s="49"/>
+      <c r="D19" s="49"/>
+      <c r="E19" s="49"/>
+      <c r="G19" s="49"/>
+      <c r="H19" s="49"/>
+      <c r="I19" s="49"/>
+      <c r="J19" s="49"/>
+      <c r="K19" s="49"/>
+      <c r="L19" s="49"/>
+      <c r="N19" s="49"/>
+      <c r="O19" s="49"/>
+      <c r="Q19" s="62"/>
+    </row>
+    <row r="21" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="B21" s="63" t="s">
+        <v>22</v>
+      </c>
+      <c r="C21" s="63"/>
+      <c r="D21" s="1"/>
+      <c r="E21" s="9" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="22" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="B22" s="53">
+        <f>SUM(B19:E19,G19:L19,N19:O19,Q18)</f>
+        <v>0</v>
+      </c>
+      <c r="C22" s="53"/>
+      <c r="D22" s="1"/>
+      <c r="E22" s="64"/>
+    </row>
+    <row r="23" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="B23" s="53"/>
+      <c r="C23" s="53"/>
+      <c r="D23" s="1"/>
+      <c r="E23" s="65"/>
+    </row>
+    <row r="24" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A24" s="6"/>
+      <c r="B24" s="6"/>
+      <c r="C24" s="6"/>
+      <c r="D24" s="6"/>
+      <c r="E24" s="6"/>
+      <c r="F24" s="6"/>
+      <c r="G24" s="6"/>
+      <c r="H24" s="6"/>
+      <c r="I24" s="6"/>
+      <c r="J24" s="6"/>
+      <c r="K24" s="6"/>
+      <c r="L24" s="6"/>
+      <c r="M24" s="6"/>
+      <c r="N24" s="6"/>
+      <c r="O24" s="6"/>
+      <c r="P24" s="6"/>
+      <c r="Q24" s="6"/>
+      <c r="R24" s="6"/>
+      <c r="S24" s="6"/>
+      <c r="T24" s="6"/>
+      <c r="U24" s="6"/>
+      <c r="V24" s="6"/>
+    </row>
+    <row r="25" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="26" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="B26" s="85" t="s">
+        <v>184</v>
+      </c>
+      <c r="C26" s="86"/>
+      <c r="D26" s="86"/>
+      <c r="E26" s="86"/>
+      <c r="F26" s="86"/>
+      <c r="G26" s="86"/>
+      <c r="H26" s="86"/>
+      <c r="I26" s="86"/>
+      <c r="J26" s="86"/>
+      <c r="K26" s="86"/>
+      <c r="L26" s="86"/>
+      <c r="M26" s="86"/>
+      <c r="N26" s="86"/>
+      <c r="O26" s="86"/>
+      <c r="P26" s="86"/>
+      <c r="Q26" s="87"/>
+      <c r="S26" s="69" t="s">
+        <v>268</v>
+      </c>
+      <c r="T26" s="69"/>
+      <c r="U26" s="69"/>
+      <c r="V26" s="69"/>
+    </row>
+    <row r="27" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B27" s="88"/>
+      <c r="C27" s="89"/>
+      <c r="D27" s="89"/>
+      <c r="E27" s="89"/>
+      <c r="F27" s="89"/>
+      <c r="G27" s="89"/>
+      <c r="H27" s="89"/>
+      <c r="I27" s="89"/>
+      <c r="J27" s="89"/>
+      <c r="K27" s="89"/>
+      <c r="L27" s="89"/>
+      <c r="M27" s="89"/>
+      <c r="N27" s="89"/>
+      <c r="O27" s="89"/>
+      <c r="P27" s="89"/>
+      <c r="Q27" s="90"/>
+      <c r="S27" s="66" t="s">
+        <v>312</v>
+      </c>
+      <c r="T27" s="67"/>
+      <c r="U27" s="67"/>
+      <c r="V27" s="68"/>
+    </row>
+    <row r="28" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="S28" s="66" t="s">
+        <v>313</v>
+      </c>
+      <c r="T28" s="67"/>
+      <c r="U28" s="67"/>
+      <c r="V28" s="68"/>
+    </row>
+    <row r="29" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="B29" s="54" t="s">
+        <v>8</v>
+      </c>
+      <c r="C29" s="54"/>
+      <c r="D29" s="54"/>
+      <c r="E29" s="54"/>
+      <c r="G29" s="52" t="s">
+        <v>281</v>
+      </c>
+      <c r="H29" s="52"/>
+    </row>
+    <row r="30" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="B30" s="2" t="s">
+        <v>278</v>
+      </c>
+      <c r="C30" s="2" t="s">
+        <v>279</v>
+      </c>
+      <c r="D30" s="53" t="s">
+        <v>280</v>
+      </c>
+      <c r="E30" s="53"/>
+      <c r="G30" s="49" t="s">
+        <v>73</v>
+      </c>
+      <c r="H30" s="49" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="31" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="B31" s="2"/>
+      <c r="C31" s="2"/>
+      <c r="D31" s="53"/>
+      <c r="E31" s="53"/>
+      <c r="G31" s="49"/>
+      <c r="H31" s="49"/>
+    </row>
+    <row r="32" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A32" s="6"/>
+      <c r="B32" s="6"/>
+      <c r="C32" s="6"/>
+      <c r="D32" s="6"/>
+      <c r="E32" s="6"/>
+      <c r="F32" s="6"/>
+      <c r="G32" s="6"/>
+      <c r="H32" s="6"/>
+      <c r="I32" s="6"/>
+      <c r="J32" s="6"/>
+      <c r="K32" s="6"/>
+      <c r="L32" s="6"/>
+      <c r="M32" s="6"/>
+      <c r="N32" s="6"/>
+      <c r="O32" s="6"/>
+      <c r="P32" s="6"/>
+      <c r="Q32" s="6"/>
+      <c r="R32" s="6"/>
+      <c r="S32" s="6"/>
+      <c r="T32" s="6"/>
+      <c r="U32" s="6"/>
+      <c r="V32" s="6"/>
+    </row>
+    <row r="33" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="34" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="B34" s="85" t="s">
+        <v>187</v>
+      </c>
+      <c r="C34" s="86"/>
+      <c r="D34" s="86"/>
+      <c r="E34" s="86"/>
+      <c r="F34" s="86"/>
+      <c r="G34" s="86"/>
+      <c r="H34" s="86"/>
+      <c r="I34" s="86"/>
+      <c r="J34" s="86"/>
+      <c r="K34" s="86"/>
+      <c r="L34" s="86"/>
+      <c r="M34" s="86"/>
+      <c r="N34" s="86"/>
+      <c r="O34" s="86"/>
+      <c r="P34" s="86"/>
+      <c r="Q34" s="87"/>
+      <c r="S34" s="69" t="s">
+        <v>268</v>
+      </c>
+      <c r="T34" s="69"/>
+      <c r="U34" s="69"/>
+      <c r="V34" s="69"/>
+    </row>
+    <row r="35" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B35" s="88"/>
+      <c r="C35" s="89"/>
+      <c r="D35" s="89"/>
+      <c r="E35" s="89"/>
+      <c r="F35" s="89"/>
+      <c r="G35" s="89"/>
+      <c r="H35" s="89"/>
+      <c r="I35" s="89"/>
+      <c r="J35" s="89"/>
+      <c r="K35" s="89"/>
+      <c r="L35" s="89"/>
+      <c r="M35" s="89"/>
+      <c r="N35" s="89"/>
+      <c r="O35" s="89"/>
+      <c r="P35" s="89"/>
+      <c r="Q35" s="90"/>
+      <c r="S35" s="66" t="s">
+        <v>309</v>
+      </c>
+      <c r="T35" s="67"/>
+      <c r="U35" s="67"/>
+      <c r="V35" s="68"/>
+    </row>
+    <row r="36" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="S36" s="66" t="s">
+        <v>310</v>
+      </c>
+      <c r="T36" s="67"/>
+      <c r="U36" s="67"/>
+      <c r="V36" s="68"/>
+    </row>
+    <row r="37" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="B37" s="52" t="s">
+        <v>302</v>
+      </c>
+      <c r="C37" s="52"/>
+      <c r="D37" s="52"/>
+      <c r="E37" s="52"/>
+      <c r="F37" s="52"/>
+      <c r="G37" s="52"/>
+      <c r="H37" s="52"/>
+      <c r="I37" s="52"/>
+      <c r="J37" s="52"/>
+      <c r="K37" s="52"/>
+      <c r="L37" s="52"/>
+      <c r="M37" s="52"/>
+      <c r="N37" s="52"/>
+      <c r="O37" s="52"/>
+      <c r="P37" s="52"/>
+      <c r="S37" s="66" t="s">
+        <v>311</v>
+      </c>
+      <c r="T37" s="67"/>
+      <c r="U37" s="67"/>
+      <c r="V37" s="68"/>
+    </row>
+    <row r="38" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="B38" s="49" t="s">
+        <v>282</v>
+      </c>
+      <c r="C38" s="49" t="s">
+        <v>49</v>
+      </c>
+      <c r="D38" s="49" t="s">
+        <v>50</v>
+      </c>
+      <c r="E38" s="49" t="s">
+        <v>51</v>
+      </c>
+      <c r="F38" s="49" t="s">
+        <v>52</v>
+      </c>
+      <c r="G38" s="49" t="s">
+        <v>53</v>
+      </c>
+      <c r="H38" s="49" t="s">
+        <v>54</v>
+      </c>
+      <c r="I38" s="49" t="s">
+        <v>62</v>
+      </c>
+      <c r="J38" s="49" t="s">
+        <v>55</v>
+      </c>
+      <c r="K38" s="49" t="s">
+        <v>56</v>
+      </c>
+      <c r="L38" s="49" t="s">
+        <v>57</v>
+      </c>
+      <c r="M38" s="49" t="s">
+        <v>58</v>
+      </c>
+      <c r="N38" s="49" t="s">
+        <v>59</v>
+      </c>
+      <c r="O38" s="49" t="s">
+        <v>60</v>
+      </c>
+      <c r="P38" s="49" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="39" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="B39" s="49"/>
+      <c r="C39" s="49"/>
+      <c r="D39" s="49"/>
+      <c r="E39" s="49"/>
+      <c r="F39" s="49"/>
+      <c r="G39" s="49"/>
+      <c r="H39" s="49"/>
+      <c r="I39" s="49"/>
+      <c r="J39" s="49"/>
+      <c r="K39" s="49"/>
+      <c r="L39" s="49"/>
+      <c r="M39" s="49"/>
+      <c r="N39" s="49"/>
+      <c r="O39" s="49"/>
+      <c r="P39" s="49"/>
+    </row>
+    <row r="41" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="B41" s="52" t="s">
+        <v>304</v>
+      </c>
+      <c r="C41" s="52"/>
+      <c r="D41" s="52"/>
+      <c r="E41" s="52"/>
+      <c r="F41" s="52"/>
+      <c r="G41" s="52"/>
+      <c r="I41" s="52" t="s">
+        <v>303</v>
+      </c>
+      <c r="J41" s="52"/>
+    </row>
+    <row r="42" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="B42" s="91" t="s">
+        <v>293</v>
+      </c>
+      <c r="C42" s="91"/>
+      <c r="D42" s="91" t="s">
+        <v>294</v>
+      </c>
+      <c r="E42" s="91"/>
+      <c r="F42" s="91" t="s">
+        <v>295</v>
+      </c>
+      <c r="G42" s="91"/>
+      <c r="I42" s="91"/>
+      <c r="J42" s="91"/>
+    </row>
+    <row r="43" spans="1:22" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B43" s="2" t="s">
+        <v>154</v>
+      </c>
+      <c r="C43" s="2" t="s">
+        <v>292</v>
+      </c>
+      <c r="D43" s="2" t="s">
+        <v>154</v>
+      </c>
+      <c r="E43" s="2" t="s">
+        <v>292</v>
+      </c>
+      <c r="F43" s="2" t="s">
+        <v>154</v>
+      </c>
+      <c r="G43" s="2" t="s">
+        <v>292</v>
+      </c>
+      <c r="I43" s="91"/>
+      <c r="J43" s="91"/>
+    </row>
+    <row r="44" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="B44" s="50"/>
+      <c r="C44" s="50"/>
+      <c r="D44" s="50"/>
+      <c r="E44" s="50"/>
+      <c r="F44" s="50"/>
+      <c r="G44" s="50"/>
+      <c r="I44" s="91"/>
+      <c r="J44" s="91"/>
+    </row>
+    <row r="45" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A45" s="6"/>
+      <c r="B45" s="6"/>
+      <c r="C45" s="6"/>
+      <c r="D45" s="6"/>
+      <c r="E45" s="6"/>
+      <c r="F45" s="6"/>
+      <c r="G45" s="6"/>
+      <c r="H45" s="6"/>
+      <c r="I45" s="6"/>
+      <c r="J45" s="6"/>
+      <c r="K45" s="6"/>
+      <c r="L45" s="6"/>
+      <c r="M45" s="6"/>
+      <c r="N45" s="6"/>
+      <c r="O45" s="6"/>
+      <c r="P45" s="6"/>
+      <c r="Q45" s="6"/>
+      <c r="R45" s="6"/>
+      <c r="S45" s="6"/>
+      <c r="T45" s="6"/>
+      <c r="U45" s="6"/>
+      <c r="V45" s="6"/>
+    </row>
+    <row r="46" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="47" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="B47" s="85" t="s">
+        <v>305</v>
+      </c>
+      <c r="C47" s="86"/>
+      <c r="D47" s="86"/>
+      <c r="E47" s="86"/>
+      <c r="F47" s="86"/>
+      <c r="G47" s="86"/>
+      <c r="H47" s="86"/>
+      <c r="I47" s="86"/>
+      <c r="J47" s="86"/>
+      <c r="K47" s="86"/>
+      <c r="L47" s="86"/>
+      <c r="M47" s="86"/>
+      <c r="N47" s="86"/>
+      <c r="O47" s="86"/>
+      <c r="P47" s="86"/>
+      <c r="Q47" s="87"/>
+    </row>
+    <row r="48" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B48" s="88"/>
+      <c r="C48" s="89"/>
+      <c r="D48" s="89"/>
+      <c r="E48" s="89"/>
+      <c r="F48" s="89"/>
+      <c r="G48" s="89"/>
+      <c r="H48" s="89"/>
+      <c r="I48" s="89"/>
+      <c r="J48" s="89"/>
+      <c r="K48" s="89"/>
+      <c r="L48" s="89"/>
+      <c r="M48" s="89"/>
+      <c r="N48" s="89"/>
+      <c r="O48" s="89"/>
+      <c r="P48" s="89"/>
+      <c r="Q48" s="90"/>
+    </row>
+    <row r="50" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B50" s="52" t="s">
+        <v>306</v>
+      </c>
+      <c r="C50" s="52"/>
+      <c r="D50" s="52"/>
+      <c r="E50" s="52"/>
+      <c r="F50" s="52"/>
+      <c r="G50" s="52"/>
+      <c r="H50" s="52"/>
+    </row>
+    <row r="51" spans="2:8" s="16" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B51" s="49" t="s">
+        <v>307</v>
+      </c>
+    </row>
+    <row r="52" spans="2:8" s="16" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B52" s="49" t="s">
+        <v>308</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="46">
+    <mergeCell ref="B47:Q48"/>
+    <mergeCell ref="B50:H50"/>
+    <mergeCell ref="S34:V34"/>
+    <mergeCell ref="S35:V35"/>
+    <mergeCell ref="S36:V36"/>
+    <mergeCell ref="S37:V37"/>
+    <mergeCell ref="R2:U2"/>
+    <mergeCell ref="B42:C42"/>
+    <mergeCell ref="D42:E42"/>
+    <mergeCell ref="F42:G42"/>
+    <mergeCell ref="B41:G41"/>
+    <mergeCell ref="I41:J41"/>
+    <mergeCell ref="I42:J44"/>
+    <mergeCell ref="S26:V26"/>
+    <mergeCell ref="S27:V27"/>
+    <mergeCell ref="S28:V28"/>
+    <mergeCell ref="S14:V14"/>
+    <mergeCell ref="S15:V15"/>
+    <mergeCell ref="S16:V16"/>
+    <mergeCell ref="R6:U6"/>
+    <mergeCell ref="R5:U5"/>
+    <mergeCell ref="R4:U4"/>
+    <mergeCell ref="R3:U3"/>
+    <mergeCell ref="B17:E17"/>
+    <mergeCell ref="G17:L17"/>
+    <mergeCell ref="N17:O17"/>
+    <mergeCell ref="B14:Q15"/>
+    <mergeCell ref="B9:C9"/>
+    <mergeCell ref="B10:C11"/>
+    <mergeCell ref="E10:E11"/>
+    <mergeCell ref="R7:U7"/>
+    <mergeCell ref="B2:P3"/>
+    <mergeCell ref="B5:C5"/>
+    <mergeCell ref="E5:I5"/>
+    <mergeCell ref="K5:P5"/>
+    <mergeCell ref="Q18:Q19"/>
+    <mergeCell ref="B21:C21"/>
+    <mergeCell ref="B22:C23"/>
+    <mergeCell ref="E22:E23"/>
+    <mergeCell ref="B26:Q27"/>
+    <mergeCell ref="B37:P37"/>
+    <mergeCell ref="D30:E30"/>
+    <mergeCell ref="B29:E29"/>
+    <mergeCell ref="D31:E31"/>
+    <mergeCell ref="G29:H29"/>
+    <mergeCell ref="B34:Q35"/>
+  </mergeCells>
+  <phoneticPr fontId="1" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{03C86BD6-21E5-4E44-BF61-9A65607E6D85}">
+  <sheetPr>
+    <tabColor theme="9" tint="0.79998168889431442"/>
+  </sheetPr>
   <dimension ref="A1:S68"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -1656,60 +2940,60 @@
   <sheetData>
     <row r="1" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="2" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B2" s="44" t="s">
+      <c r="B2" s="55" t="s">
         <v>76</v>
       </c>
-      <c r="C2" s="45"/>
-      <c r="D2" s="45"/>
-      <c r="E2" s="45"/>
-      <c r="F2" s="45"/>
-      <c r="G2" s="45"/>
-      <c r="H2" s="45"/>
-      <c r="I2" s="45"/>
-      <c r="J2" s="45"/>
-      <c r="K2" s="45"/>
-      <c r="L2" s="45"/>
-      <c r="M2" s="45"/>
-      <c r="N2" s="45"/>
-      <c r="O2" s="45"/>
-      <c r="P2" s="46"/>
+      <c r="C2" s="56"/>
+      <c r="D2" s="56"/>
+      <c r="E2" s="56"/>
+      <c r="F2" s="56"/>
+      <c r="G2" s="56"/>
+      <c r="H2" s="56"/>
+      <c r="I2" s="56"/>
+      <c r="J2" s="56"/>
+      <c r="K2" s="56"/>
+      <c r="L2" s="56"/>
+      <c r="M2" s="56"/>
+      <c r="N2" s="56"/>
+      <c r="O2" s="56"/>
+      <c r="P2" s="57"/>
     </row>
     <row r="3" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B3" s="47"/>
-      <c r="C3" s="48"/>
-      <c r="D3" s="48"/>
-      <c r="E3" s="48"/>
-      <c r="F3" s="48"/>
-      <c r="G3" s="48"/>
-      <c r="H3" s="48"/>
-      <c r="I3" s="48"/>
-      <c r="J3" s="48"/>
-      <c r="K3" s="48"/>
-      <c r="L3" s="48"/>
-      <c r="M3" s="48"/>
-      <c r="N3" s="48"/>
-      <c r="O3" s="48"/>
-      <c r="P3" s="49"/>
+      <c r="B3" s="58"/>
+      <c r="C3" s="59"/>
+      <c r="D3" s="59"/>
+      <c r="E3" s="59"/>
+      <c r="F3" s="59"/>
+      <c r="G3" s="59"/>
+      <c r="H3" s="59"/>
+      <c r="I3" s="59"/>
+      <c r="J3" s="59"/>
+      <c r="K3" s="59"/>
+      <c r="L3" s="59"/>
+      <c r="M3" s="59"/>
+      <c r="N3" s="59"/>
+      <c r="O3" s="59"/>
+      <c r="P3" s="60"/>
       <c r="R3" s="12"/>
     </row>
     <row r="5" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B5" s="42" t="s">
+      <c r="B5" s="70" t="s">
         <v>83</v>
       </c>
-      <c r="C5" s="57"/>
-      <c r="D5" s="57"/>
-      <c r="E5" s="57"/>
-      <c r="F5" s="43"/>
-      <c r="H5" s="42" t="s">
+      <c r="C5" s="74"/>
+      <c r="D5" s="74"/>
+      <c r="E5" s="74"/>
+      <c r="F5" s="71"/>
+      <c r="H5" s="70" t="s">
         <v>82</v>
       </c>
-      <c r="I5" s="43"/>
-      <c r="K5" s="42" t="s">
+      <c r="I5" s="71"/>
+      <c r="K5" s="70" t="s">
         <v>8</v>
       </c>
-      <c r="L5" s="57"/>
-      <c r="M5" s="57"/>
-      <c r="N5" s="43"/>
+      <c r="L5" s="74"/>
+      <c r="M5" s="74"/>
+      <c r="N5" s="71"/>
       <c r="P5" s="4" t="s">
         <v>74</v>
       </c>
@@ -1791,10 +3075,10 @@
       </c>
     </row>
     <row r="9" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B9" s="52" t="s">
+      <c r="B9" s="63" t="s">
         <v>22</v>
       </c>
-      <c r="C9" s="52"/>
+      <c r="C9" s="63"/>
       <c r="E9" s="9" t="s">
         <v>67</v>
       </c>
@@ -1807,7 +3091,7 @@
         <v>99.1</v>
       </c>
       <c r="C10" s="53"/>
-      <c r="E10" s="55">
+      <c r="E10" s="64">
         <v>4</v>
       </c>
       <c r="G10" s="7"/>
@@ -1816,7 +3100,7 @@
     <row r="11" spans="1:19" x14ac:dyDescent="0.25">
       <c r="B11" s="53"/>
       <c r="C11" s="53"/>
-      <c r="E11" s="56"/>
+      <c r="E11" s="65"/>
       <c r="G11" s="7"/>
       <c r="H11" s="7"/>
     </row>
@@ -1843,42 +3127,42 @@
     </row>
     <row r="13" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="14" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B14" s="44" t="s">
+      <c r="B14" s="55" t="s">
         <v>77</v>
       </c>
-      <c r="C14" s="45"/>
-      <c r="D14" s="45"/>
-      <c r="E14" s="45"/>
-      <c r="F14" s="45"/>
-      <c r="G14" s="45"/>
-      <c r="H14" s="46"/>
+      <c r="C14" s="56"/>
+      <c r="D14" s="56"/>
+      <c r="E14" s="56"/>
+      <c r="F14" s="56"/>
+      <c r="G14" s="56"/>
+      <c r="H14" s="57"/>
     </row>
     <row r="15" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B15" s="47"/>
-      <c r="C15" s="48"/>
-      <c r="D15" s="48"/>
-      <c r="E15" s="48"/>
-      <c r="F15" s="48"/>
-      <c r="G15" s="48"/>
-      <c r="H15" s="49"/>
+      <c r="B15" s="58"/>
+      <c r="C15" s="59"/>
+      <c r="D15" s="59"/>
+      <c r="E15" s="59"/>
+      <c r="F15" s="59"/>
+      <c r="G15" s="59"/>
+      <c r="H15" s="60"/>
     </row>
     <row r="17" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B17" s="50" t="s">
+      <c r="B17" s="54" t="s">
         <v>90</v>
       </c>
-      <c r="C17" s="50"/>
-      <c r="D17" s="50"/>
-      <c r="E17" s="50"/>
-      <c r="F17" s="50"/>
-      <c r="H17" s="42" t="s">
+      <c r="C17" s="54"/>
+      <c r="D17" s="54"/>
+      <c r="E17" s="54"/>
+      <c r="F17" s="54"/>
+      <c r="H17" s="70" t="s">
         <v>96</v>
       </c>
-      <c r="I17" s="57"/>
-      <c r="J17" s="43"/>
-      <c r="L17" s="52" t="s">
+      <c r="I17" s="74"/>
+      <c r="J17" s="71"/>
+      <c r="L17" s="63" t="s">
         <v>22</v>
       </c>
-      <c r="M17" s="52"/>
+      <c r="M17" s="63"/>
       <c r="O17" s="9" t="s">
         <v>67</v>
       </c>
@@ -1914,7 +3198,7 @@
         <v>85</v>
       </c>
       <c r="M18" s="53"/>
-      <c r="O18" s="54">
+      <c r="O18" s="73">
         <v>4.5</v>
       </c>
     </row>
@@ -1945,7 +3229,7 @@
       </c>
       <c r="L19" s="53"/>
       <c r="M19" s="53"/>
-      <c r="O19" s="54"/>
+      <c r="O19" s="73"/>
     </row>
     <row r="21" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A21" s="6"/>
@@ -1970,19 +3254,19 @@
     </row>
     <row r="22" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="23" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B23" s="44" t="s">
+      <c r="B23" s="55" t="s">
         <v>79</v>
       </c>
-      <c r="C23" s="45"/>
-      <c r="D23" s="45"/>
-      <c r="E23" s="45"/>
-      <c r="F23" s="45"/>
-      <c r="G23" s="45"/>
-      <c r="H23" s="45"/>
-      <c r="I23" s="45"/>
-      <c r="J23" s="45"/>
-      <c r="K23" s="45"/>
-      <c r="L23" s="46"/>
+      <c r="C23" s="56"/>
+      <c r="D23" s="56"/>
+      <c r="E23" s="56"/>
+      <c r="F23" s="56"/>
+      <c r="G23" s="56"/>
+      <c r="H23" s="56"/>
+      <c r="I23" s="56"/>
+      <c r="J23" s="56"/>
+      <c r="K23" s="56"/>
+      <c r="L23" s="57"/>
       <c r="N23" s="53" t="s">
         <v>214</v>
       </c>
@@ -1992,17 +3276,17 @@
       <c r="S23" s="7"/>
     </row>
     <row r="24" spans="1:19" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B24" s="47"/>
-      <c r="C24" s="48"/>
-      <c r="D24" s="48"/>
-      <c r="E24" s="48"/>
-      <c r="F24" s="48"/>
-      <c r="G24" s="48"/>
-      <c r="H24" s="48"/>
-      <c r="I24" s="48"/>
-      <c r="J24" s="48"/>
-      <c r="K24" s="48"/>
-      <c r="L24" s="49"/>
+      <c r="B24" s="58"/>
+      <c r="C24" s="59"/>
+      <c r="D24" s="59"/>
+      <c r="E24" s="59"/>
+      <c r="F24" s="59"/>
+      <c r="G24" s="59"/>
+      <c r="H24" s="59"/>
+      <c r="I24" s="59"/>
+      <c r="J24" s="59"/>
+      <c r="K24" s="59"/>
+      <c r="L24" s="60"/>
       <c r="N24" s="53"/>
       <c r="O24" s="53"/>
       <c r="Q24" s="7"/>
@@ -2010,22 +3294,22 @@
       <c r="S24" s="7"/>
     </row>
     <row r="26" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B26" s="50" t="s">
+      <c r="B26" s="54" t="s">
         <v>8</v>
       </c>
-      <c r="C26" s="50"/>
-      <c r="D26" s="50"/>
-      <c r="F26" s="50" t="s">
+      <c r="C26" s="54"/>
+      <c r="D26" s="54"/>
+      <c r="F26" s="54" t="s">
         <v>195</v>
       </c>
-      <c r="G26" s="50"/>
-      <c r="H26" s="50"/>
-      <c r="I26" s="50"/>
+      <c r="G26" s="54"/>
+      <c r="H26" s="54"/>
+      <c r="I26" s="54"/>
       <c r="J26" s="7"/>
-      <c r="K26" s="42" t="s">
+      <c r="K26" s="70" t="s">
         <v>116</v>
       </c>
-      <c r="L26" s="43"/>
+      <c r="L26" s="71"/>
       <c r="N26" s="9" t="s">
         <v>212</v>
       </c>
@@ -2061,11 +3345,11 @@
       <c r="L27" s="2" t="s">
         <v>115</v>
       </c>
-      <c r="N27" s="60">
+      <c r="N27" s="77">
         <f>(K29/30*0.4*5)+(B29/25*0.3*5)+(0.3*F29)</f>
         <v>4.9399999999999995</v>
       </c>
-      <c r="O27" s="54">
+      <c r="O27" s="73">
         <v>5</v>
       </c>
     </row>
@@ -2097,27 +3381,27 @@
       <c r="L28" s="2">
         <v>10</v>
       </c>
-      <c r="N28" s="61"/>
-      <c r="O28" s="54"/>
+      <c r="N28" s="78"/>
+      <c r="O28" s="73"/>
     </row>
     <row r="29" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B29" s="51">
+      <c r="B29" s="72">
         <f>SUM(B28:D28)</f>
         <v>24</v>
       </c>
-      <c r="C29" s="51"/>
-      <c r="D29" s="51"/>
-      <c r="F29" s="51">
+      <c r="C29" s="72"/>
+      <c r="D29" s="72"/>
+      <c r="F29" s="72">
         <v>5</v>
       </c>
-      <c r="G29" s="51"/>
-      <c r="H29" s="51"/>
-      <c r="I29" s="51"/>
-      <c r="K29" s="51">
+      <c r="G29" s="72"/>
+      <c r="H29" s="72"/>
+      <c r="I29" s="72"/>
+      <c r="K29" s="72">
         <f>SUM(K28:L28)</f>
         <v>30</v>
       </c>
-      <c r="L29" s="51"/>
+      <c r="L29" s="72"/>
       <c r="N29" s="34"/>
     </row>
     <row r="31" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -2143,38 +3427,38 @@
     </row>
     <row r="32" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="33" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B33" s="44" t="s">
+      <c r="B33" s="55" t="s">
         <v>78</v>
       </c>
-      <c r="C33" s="45"/>
-      <c r="D33" s="45"/>
-      <c r="E33" s="45"/>
-      <c r="F33" s="45"/>
-      <c r="G33" s="45"/>
-      <c r="H33" s="45"/>
-      <c r="I33" s="46"/>
+      <c r="C33" s="56"/>
+      <c r="D33" s="56"/>
+      <c r="E33" s="56"/>
+      <c r="F33" s="56"/>
+      <c r="G33" s="56"/>
+      <c r="H33" s="56"/>
+      <c r="I33" s="57"/>
     </row>
     <row r="34" spans="2:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B34" s="47"/>
-      <c r="C34" s="48"/>
-      <c r="D34" s="48"/>
-      <c r="E34" s="48"/>
-      <c r="F34" s="48"/>
-      <c r="G34" s="48"/>
-      <c r="H34" s="48"/>
-      <c r="I34" s="49"/>
+      <c r="B34" s="58"/>
+      <c r="C34" s="59"/>
+      <c r="D34" s="59"/>
+      <c r="E34" s="59"/>
+      <c r="F34" s="59"/>
+      <c r="G34" s="59"/>
+      <c r="H34" s="59"/>
+      <c r="I34" s="60"/>
     </row>
     <row r="36" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B36" s="50" t="s">
+      <c r="B36" s="54" t="s">
         <v>97</v>
       </c>
-      <c r="C36" s="50"/>
+      <c r="C36" s="54"/>
       <c r="D36" s="7"/>
-      <c r="E36" s="50" t="s">
+      <c r="E36" s="54" t="s">
         <v>131</v>
       </c>
-      <c r="F36" s="50"/>
-      <c r="G36" s="50"/>
+      <c r="F36" s="54"/>
+      <c r="G36" s="54"/>
       <c r="H36" s="7"/>
     </row>
     <row r="37" spans="2:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -2216,10 +3500,10 @@
       <c r="O38" s="7"/>
     </row>
     <row r="41" spans="2:15" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B41" s="58" t="s">
+      <c r="B41" s="75" t="s">
         <v>114</v>
       </c>
-      <c r="C41" s="59"/>
+      <c r="C41" s="76"/>
       <c r="F41" s="53" t="s">
         <v>99</v>
       </c>
@@ -2279,7 +3563,7 @@
       <c r="G44" s="2">
         <v>10</v>
       </c>
-      <c r="I44" s="52" t="s">
+      <c r="I44" s="63" t="s">
         <v>67</v>
       </c>
     </row>
@@ -2290,7 +3574,7 @@
       <c r="C45" s="2">
         <v>4</v>
       </c>
-      <c r="I45" s="52"/>
+      <c r="I45" s="63"/>
     </row>
     <row r="46" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B46" s="2" t="s">
@@ -2387,70 +3671,70 @@
     </row>
     <row r="57" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="58" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B58" s="44" t="s">
+      <c r="B58" s="55" t="s">
         <v>80</v>
       </c>
-      <c r="C58" s="45"/>
-      <c r="D58" s="45"/>
-      <c r="E58" s="45"/>
-      <c r="F58" s="45"/>
-      <c r="G58" s="45"/>
-      <c r="H58" s="45"/>
-      <c r="I58" s="45"/>
-      <c r="J58" s="45"/>
-      <c r="K58" s="45"/>
-      <c r="L58" s="45"/>
-      <c r="M58" s="45"/>
-      <c r="N58" s="45"/>
-      <c r="O58" s="45"/>
-      <c r="P58" s="45"/>
-      <c r="Q58" s="45"/>
-      <c r="R58" s="45"/>
-      <c r="S58" s="46"/>
+      <c r="C58" s="56"/>
+      <c r="D58" s="56"/>
+      <c r="E58" s="56"/>
+      <c r="F58" s="56"/>
+      <c r="G58" s="56"/>
+      <c r="H58" s="56"/>
+      <c r="I58" s="56"/>
+      <c r="J58" s="56"/>
+      <c r="K58" s="56"/>
+      <c r="L58" s="56"/>
+      <c r="M58" s="56"/>
+      <c r="N58" s="56"/>
+      <c r="O58" s="56"/>
+      <c r="P58" s="56"/>
+      <c r="Q58" s="56"/>
+      <c r="R58" s="56"/>
+      <c r="S58" s="57"/>
     </row>
     <row r="59" spans="1:19" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B59" s="47"/>
-      <c r="C59" s="48"/>
-      <c r="D59" s="48"/>
-      <c r="E59" s="48"/>
-      <c r="F59" s="48"/>
-      <c r="G59" s="48"/>
-      <c r="H59" s="48"/>
-      <c r="I59" s="48"/>
-      <c r="J59" s="48"/>
-      <c r="K59" s="48"/>
-      <c r="L59" s="48"/>
-      <c r="M59" s="48"/>
-      <c r="N59" s="48"/>
-      <c r="O59" s="48"/>
-      <c r="P59" s="48"/>
-      <c r="Q59" s="48"/>
-      <c r="R59" s="48"/>
-      <c r="S59" s="49"/>
+      <c r="B59" s="58"/>
+      <c r="C59" s="59"/>
+      <c r="D59" s="59"/>
+      <c r="E59" s="59"/>
+      <c r="F59" s="59"/>
+      <c r="G59" s="59"/>
+      <c r="H59" s="59"/>
+      <c r="I59" s="59"/>
+      <c r="J59" s="59"/>
+      <c r="K59" s="59"/>
+      <c r="L59" s="59"/>
+      <c r="M59" s="59"/>
+      <c r="N59" s="59"/>
+      <c r="O59" s="59"/>
+      <c r="P59" s="59"/>
+      <c r="Q59" s="59"/>
+      <c r="R59" s="59"/>
+      <c r="S59" s="60"/>
     </row>
     <row r="61" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B61" s="50" t="s">
+      <c r="B61" s="54" t="s">
         <v>63</v>
       </c>
-      <c r="C61" s="50"/>
-      <c r="D61" s="50"/>
-      <c r="E61" s="50"/>
-      <c r="F61" s="50"/>
-      <c r="G61" s="50"/>
-      <c r="H61" s="50"/>
-      <c r="I61" s="50"/>
-      <c r="J61" s="50"/>
-      <c r="K61" s="50"/>
-      <c r="M61" s="50" t="s">
+      <c r="C61" s="54"/>
+      <c r="D61" s="54"/>
+      <c r="E61" s="54"/>
+      <c r="F61" s="54"/>
+      <c r="G61" s="54"/>
+      <c r="H61" s="54"/>
+      <c r="I61" s="54"/>
+      <c r="J61" s="54"/>
+      <c r="K61" s="54"/>
+      <c r="M61" s="54" t="s">
         <v>89</v>
       </c>
-      <c r="N61" s="50"/>
-      <c r="O61" s="50"/>
-      <c r="P61" s="50"/>
-      <c r="R61" s="50" t="s">
+      <c r="N61" s="54"/>
+      <c r="O61" s="54"/>
+      <c r="P61" s="54"/>
+      <c r="R61" s="54" t="s">
         <v>64</v>
       </c>
-      <c r="S61" s="50"/>
+      <c r="S61" s="54"/>
     </row>
     <row r="62" spans="1:19" x14ac:dyDescent="0.25">
       <c r="B62" s="2" t="s">
@@ -2553,10 +3837,10 @@
       </c>
     </row>
     <row r="66" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B66" s="52" t="s">
+      <c r="B66" s="63" t="s">
         <v>22</v>
       </c>
-      <c r="C66" s="52"/>
+      <c r="C66" s="63"/>
       <c r="E66" s="9" t="s">
         <v>67</v>
       </c>
@@ -2571,7 +3855,7 @@
         <v>98</v>
       </c>
       <c r="C67" s="53"/>
-      <c r="E67" s="54">
+      <c r="E67" s="73">
         <v>5</v>
       </c>
       <c r="G67" s="53">
@@ -2582,7 +3866,7 @@
     <row r="68" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B68" s="53"/>
       <c r="C68" s="53"/>
-      <c r="E68" s="54"/>
+      <c r="E68" s="73"/>
       <c r="G68" s="53"/>
       <c r="H68" s="7"/>
     </row>
@@ -2632,8 +3916,11 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C5356A30-E1AA-4069-A4C8-FC0BE8204C56}">
+  <sheetPr>
+    <tabColor theme="9" tint="0.79998168889431442"/>
+  </sheetPr>
   <dimension ref="A1:S78"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -2660,60 +3947,60 @@
   <sheetData>
     <row r="1" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="2" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B2" s="44" t="s">
+      <c r="B2" s="55" t="s">
         <v>117</v>
       </c>
-      <c r="C2" s="45"/>
-      <c r="D2" s="45"/>
-      <c r="E2" s="45"/>
-      <c r="F2" s="45"/>
-      <c r="G2" s="45"/>
-      <c r="H2" s="45"/>
-      <c r="I2" s="45"/>
-      <c r="J2" s="45"/>
-      <c r="K2" s="45"/>
-      <c r="L2" s="45"/>
-      <c r="M2" s="45"/>
-      <c r="N2" s="45"/>
-      <c r="O2" s="45"/>
-      <c r="P2" s="46"/>
+      <c r="C2" s="56"/>
+      <c r="D2" s="56"/>
+      <c r="E2" s="56"/>
+      <c r="F2" s="56"/>
+      <c r="G2" s="56"/>
+      <c r="H2" s="56"/>
+      <c r="I2" s="56"/>
+      <c r="J2" s="56"/>
+      <c r="K2" s="56"/>
+      <c r="L2" s="56"/>
+      <c r="M2" s="56"/>
+      <c r="N2" s="56"/>
+      <c r="O2" s="56"/>
+      <c r="P2" s="57"/>
     </row>
     <row r="3" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B3" s="47"/>
-      <c r="C3" s="48"/>
-      <c r="D3" s="48"/>
-      <c r="E3" s="48"/>
-      <c r="F3" s="48"/>
-      <c r="G3" s="48"/>
-      <c r="H3" s="48"/>
-      <c r="I3" s="48"/>
-      <c r="J3" s="48"/>
-      <c r="K3" s="48"/>
-      <c r="L3" s="48"/>
-      <c r="M3" s="48"/>
-      <c r="N3" s="48"/>
-      <c r="O3" s="48"/>
-      <c r="P3" s="49"/>
+      <c r="B3" s="58"/>
+      <c r="C3" s="59"/>
+      <c r="D3" s="59"/>
+      <c r="E3" s="59"/>
+      <c r="F3" s="59"/>
+      <c r="G3" s="59"/>
+      <c r="H3" s="59"/>
+      <c r="I3" s="59"/>
+      <c r="J3" s="59"/>
+      <c r="K3" s="59"/>
+      <c r="L3" s="59"/>
+      <c r="M3" s="59"/>
+      <c r="N3" s="59"/>
+      <c r="O3" s="59"/>
+      <c r="P3" s="60"/>
       <c r="R3" s="12"/>
     </row>
     <row r="5" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B5" s="50" t="s">
+      <c r="B5" s="54" t="s">
         <v>18</v>
       </c>
-      <c r="C5" s="50"/>
-      <c r="D5" s="50"/>
-      <c r="E5" s="50"/>
-      <c r="F5" s="50"/>
-      <c r="G5" s="50"/>
+      <c r="C5" s="54"/>
+      <c r="D5" s="54"/>
+      <c r="E5" s="54"/>
+      <c r="F5" s="54"/>
+      <c r="G5" s="54"/>
       <c r="I5" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="K5" s="42" t="s">
+      <c r="K5" s="70" t="s">
         <v>8</v>
       </c>
-      <c r="L5" s="57"/>
-      <c r="M5" s="57"/>
-      <c r="N5" s="43"/>
+      <c r="L5" s="74"/>
+      <c r="M5" s="74"/>
+      <c r="N5" s="71"/>
       <c r="P5" s="4" t="s">
         <v>74</v>
       </c>
@@ -2795,10 +4082,10 @@
       </c>
     </row>
     <row r="9" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B9" s="52" t="s">
+      <c r="B9" s="63" t="s">
         <v>22</v>
       </c>
-      <c r="C9" s="52"/>
+      <c r="C9" s="63"/>
       <c r="E9" s="9" t="s">
         <v>67</v>
       </c>
@@ -2809,14 +4096,14 @@
         <v>110</v>
       </c>
       <c r="C10" s="53"/>
-      <c r="E10" s="55">
+      <c r="E10" s="64">
         <v>4</v>
       </c>
     </row>
     <row r="11" spans="1:19" x14ac:dyDescent="0.25">
       <c r="B11" s="53"/>
       <c r="C11" s="53"/>
-      <c r="E11" s="56"/>
+      <c r="E11" s="65"/>
     </row>
     <row r="12" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A12" s="6"/>
@@ -2841,40 +4128,40 @@
     </row>
     <row r="13" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="14" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B14" s="44" t="s">
+      <c r="B14" s="55" t="s">
         <v>118</v>
       </c>
-      <c r="C14" s="45"/>
-      <c r="D14" s="45"/>
-      <c r="E14" s="45"/>
-      <c r="F14" s="45"/>
-      <c r="G14" s="45"/>
-      <c r="H14" s="46"/>
+      <c r="C14" s="56"/>
+      <c r="D14" s="56"/>
+      <c r="E14" s="56"/>
+      <c r="F14" s="56"/>
+      <c r="G14" s="56"/>
+      <c r="H14" s="57"/>
     </row>
     <row r="15" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B15" s="47"/>
-      <c r="C15" s="48"/>
-      <c r="D15" s="48"/>
-      <c r="E15" s="48"/>
-      <c r="F15" s="48"/>
-      <c r="G15" s="48"/>
-      <c r="H15" s="49"/>
+      <c r="B15" s="58"/>
+      <c r="C15" s="59"/>
+      <c r="D15" s="59"/>
+      <c r="E15" s="59"/>
+      <c r="F15" s="59"/>
+      <c r="G15" s="59"/>
+      <c r="H15" s="60"/>
     </row>
     <row r="17" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B17" s="50" t="s">
+      <c r="B17" s="54" t="s">
         <v>12</v>
       </c>
-      <c r="C17" s="50"/>
-      <c r="D17" s="50"/>
-      <c r="F17" s="50" t="s">
+      <c r="C17" s="54"/>
+      <c r="D17" s="54"/>
+      <c r="F17" s="54" t="s">
         <v>8</v>
       </c>
-      <c r="G17" s="50"/>
-      <c r="H17" s="50"/>
-      <c r="J17" s="52" t="s">
+      <c r="G17" s="54"/>
+      <c r="H17" s="54"/>
+      <c r="J17" s="63" t="s">
         <v>22</v>
       </c>
-      <c r="K17" s="52"/>
+      <c r="K17" s="63"/>
       <c r="M17" s="9" t="s">
         <v>67</v>
       </c>
@@ -2903,7 +4190,7 @@
         <v>93</v>
       </c>
       <c r="K18" s="53"/>
-      <c r="M18" s="54">
+      <c r="M18" s="73">
         <v>5</v>
       </c>
     </row>
@@ -2928,7 +4215,7 @@
       </c>
       <c r="J19" s="53"/>
       <c r="K19" s="53"/>
-      <c r="M19" s="54"/>
+      <c r="M19" s="73"/>
     </row>
     <row r="21" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A21" s="6"/>
@@ -2953,46 +4240,46 @@
     </row>
     <row r="22" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="23" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B23" s="44" t="s">
+      <c r="B23" s="55" t="s">
         <v>119</v>
       </c>
-      <c r="C23" s="45"/>
-      <c r="D23" s="45"/>
-      <c r="E23" s="45"/>
-      <c r="F23" s="45"/>
-      <c r="G23" s="45"/>
-      <c r="H23" s="45"/>
-      <c r="I23" s="45"/>
-      <c r="J23" s="45"/>
-      <c r="K23" s="46"/>
+      <c r="C23" s="56"/>
+      <c r="D23" s="56"/>
+      <c r="E23" s="56"/>
+      <c r="F23" s="56"/>
+      <c r="G23" s="56"/>
+      <c r="H23" s="56"/>
+      <c r="I23" s="56"/>
+      <c r="J23" s="56"/>
+      <c r="K23" s="57"/>
     </row>
     <row r="24" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B24" s="47"/>
-      <c r="C24" s="48"/>
-      <c r="D24" s="48"/>
-      <c r="E24" s="48"/>
-      <c r="F24" s="48"/>
-      <c r="G24" s="48"/>
-      <c r="H24" s="48"/>
-      <c r="I24" s="48"/>
-      <c r="J24" s="48"/>
-      <c r="K24" s="49"/>
+      <c r="B24" s="58"/>
+      <c r="C24" s="59"/>
+      <c r="D24" s="59"/>
+      <c r="E24" s="59"/>
+      <c r="F24" s="59"/>
+      <c r="G24" s="59"/>
+      <c r="H24" s="59"/>
+      <c r="I24" s="59"/>
+      <c r="J24" s="59"/>
+      <c r="K24" s="60"/>
     </row>
     <row r="26" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B26" s="50" t="s">
+      <c r="B26" s="54" t="s">
         <v>17</v>
       </c>
-      <c r="C26" s="50"/>
-      <c r="E26" s="42" t="s">
+      <c r="C26" s="54"/>
+      <c r="E26" s="70" t="s">
         <v>21</v>
       </c>
-      <c r="F26" s="57"/>
-      <c r="G26" s="43"/>
-      <c r="I26" s="50" t="s">
+      <c r="F26" s="74"/>
+      <c r="G26" s="71"/>
+      <c r="I26" s="54" t="s">
         <v>20</v>
       </c>
-      <c r="J26" s="50"/>
-      <c r="K26" s="50"/>
+      <c r="J26" s="54"/>
+      <c r="K26" s="54"/>
       <c r="M26" s="10" t="s">
         <v>22</v>
       </c>
@@ -3027,12 +4314,12 @@
       <c r="K27" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="M27" s="62">
+      <c r="M27" s="79">
         <f>SUM(B28:C28,E28:G28,I28:K28)</f>
         <v>36</v>
       </c>
       <c r="N27" s="7"/>
-      <c r="O27" s="54">
+      <c r="O27" s="73">
         <v>4</v>
       </c>
       <c r="P27" s="8"/>
@@ -3062,9 +4349,9 @@
       <c r="K28" s="2">
         <v>3.2</v>
       </c>
-      <c r="M28" s="62"/>
+      <c r="M28" s="79"/>
       <c r="N28" s="7"/>
-      <c r="O28" s="54"/>
+      <c r="O28" s="73"/>
       <c r="P28" s="8"/>
     </row>
     <row r="30" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -3090,39 +4377,39 @@
     </row>
     <row r="31" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="32" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B32" s="44" t="s">
+      <c r="B32" s="55" t="s">
         <v>120</v>
       </c>
-      <c r="C32" s="45"/>
-      <c r="D32" s="45"/>
-      <c r="E32" s="45"/>
-      <c r="F32" s="45"/>
-      <c r="G32" s="45"/>
-      <c r="H32" s="45"/>
-      <c r="I32" s="46"/>
+      <c r="C32" s="56"/>
+      <c r="D32" s="56"/>
+      <c r="E32" s="56"/>
+      <c r="F32" s="56"/>
+      <c r="G32" s="56"/>
+      <c r="H32" s="56"/>
+      <c r="I32" s="57"/>
     </row>
     <row r="33" spans="2:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B33" s="47"/>
-      <c r="C33" s="48"/>
-      <c r="D33" s="48"/>
-      <c r="E33" s="48"/>
-      <c r="F33" s="48"/>
-      <c r="G33" s="48"/>
-      <c r="H33" s="48"/>
-      <c r="I33" s="49"/>
+      <c r="B33" s="58"/>
+      <c r="C33" s="59"/>
+      <c r="D33" s="59"/>
+      <c r="E33" s="59"/>
+      <c r="F33" s="59"/>
+      <c r="G33" s="59"/>
+      <c r="H33" s="59"/>
+      <c r="I33" s="60"/>
     </row>
     <row r="35" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B35" s="50" t="s">
+      <c r="B35" s="54" t="s">
         <v>31</v>
       </c>
-      <c r="C35" s="50"/>
-      <c r="D35" s="50"/>
-      <c r="F35" s="50" t="s">
+      <c r="C35" s="54"/>
+      <c r="D35" s="54"/>
+      <c r="F35" s="54" t="s">
         <v>12</v>
       </c>
-      <c r="G35" s="50"/>
-      <c r="H35" s="50"/>
-      <c r="I35" s="50"/>
+      <c r="G35" s="54"/>
+      <c r="H35" s="54"/>
+      <c r="I35" s="54"/>
       <c r="N35" s="7"/>
       <c r="O35" s="7"/>
     </row>
@@ -3179,10 +4466,10 @@
       <c r="O37" s="7"/>
     </row>
     <row r="40" spans="2:15" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B40" s="58" t="s">
+      <c r="B40" s="75" t="s">
         <v>35</v>
       </c>
-      <c r="C40" s="59"/>
+      <c r="C40" s="76"/>
       <c r="F40" s="53" t="s">
         <v>36</v>
       </c>
@@ -3242,7 +4529,7 @@
       <c r="G43" s="2">
         <v>0.44</v>
       </c>
-      <c r="I43" s="52" t="s">
+      <c r="I43" s="63" t="s">
         <v>67</v>
       </c>
     </row>
@@ -3259,7 +4546,7 @@
       <c r="G44" s="2">
         <v>1</v>
       </c>
-      <c r="I44" s="52"/>
+      <c r="I44" s="63"/>
     </row>
     <row r="45" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B45" s="2" t="s">
@@ -3403,67 +4690,67 @@
     </row>
     <row r="57" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="58" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B58" s="44" t="s">
+      <c r="B58" s="55" t="s">
         <v>121</v>
       </c>
-      <c r="C58" s="45"/>
-      <c r="D58" s="45"/>
-      <c r="E58" s="45"/>
-      <c r="F58" s="45"/>
-      <c r="G58" s="45"/>
-      <c r="H58" s="45"/>
-      <c r="I58" s="45"/>
-      <c r="J58" s="45"/>
-      <c r="K58" s="45"/>
-      <c r="L58" s="45"/>
-      <c r="M58" s="45"/>
-      <c r="N58" s="45"/>
-      <c r="O58" s="45"/>
-      <c r="P58" s="45"/>
-      <c r="Q58" s="45"/>
-      <c r="R58" s="46"/>
+      <c r="C58" s="56"/>
+      <c r="D58" s="56"/>
+      <c r="E58" s="56"/>
+      <c r="F58" s="56"/>
+      <c r="G58" s="56"/>
+      <c r="H58" s="56"/>
+      <c r="I58" s="56"/>
+      <c r="J58" s="56"/>
+      <c r="K58" s="56"/>
+      <c r="L58" s="56"/>
+      <c r="M58" s="56"/>
+      <c r="N58" s="56"/>
+      <c r="O58" s="56"/>
+      <c r="P58" s="56"/>
+      <c r="Q58" s="56"/>
+      <c r="R58" s="57"/>
     </row>
     <row r="59" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B59" s="47"/>
-      <c r="C59" s="48"/>
-      <c r="D59" s="48"/>
-      <c r="E59" s="48"/>
-      <c r="F59" s="48"/>
-      <c r="G59" s="48"/>
-      <c r="H59" s="48"/>
-      <c r="I59" s="48"/>
-      <c r="J59" s="48"/>
-      <c r="K59" s="48"/>
-      <c r="L59" s="48"/>
-      <c r="M59" s="48"/>
-      <c r="N59" s="48"/>
-      <c r="O59" s="48"/>
-      <c r="P59" s="48"/>
-      <c r="Q59" s="48"/>
-      <c r="R59" s="49"/>
+      <c r="B59" s="58"/>
+      <c r="C59" s="59"/>
+      <c r="D59" s="59"/>
+      <c r="E59" s="59"/>
+      <c r="F59" s="59"/>
+      <c r="G59" s="59"/>
+      <c r="H59" s="59"/>
+      <c r="I59" s="59"/>
+      <c r="J59" s="59"/>
+      <c r="K59" s="59"/>
+      <c r="L59" s="59"/>
+      <c r="M59" s="59"/>
+      <c r="N59" s="59"/>
+      <c r="O59" s="59"/>
+      <c r="P59" s="59"/>
+      <c r="Q59" s="59"/>
+      <c r="R59" s="60"/>
     </row>
     <row r="61" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B61" s="50" t="s">
+      <c r="B61" s="54" t="s">
         <v>63</v>
       </c>
-      <c r="C61" s="50"/>
-      <c r="D61" s="50"/>
-      <c r="E61" s="50"/>
-      <c r="F61" s="50"/>
-      <c r="G61" s="50"/>
-      <c r="H61" s="50"/>
-      <c r="I61" s="50"/>
-      <c r="J61" s="50"/>
-      <c r="K61" s="50"/>
-      <c r="M61" s="50" t="s">
+      <c r="C61" s="54"/>
+      <c r="D61" s="54"/>
+      <c r="E61" s="54"/>
+      <c r="F61" s="54"/>
+      <c r="G61" s="54"/>
+      <c r="H61" s="54"/>
+      <c r="I61" s="54"/>
+      <c r="J61" s="54"/>
+      <c r="K61" s="54"/>
+      <c r="M61" s="54" t="s">
         <v>68</v>
       </c>
-      <c r="N61" s="50"/>
-      <c r="O61" s="50"/>
-      <c r="Q61" s="50" t="s">
+      <c r="N61" s="54"/>
+      <c r="O61" s="54"/>
+      <c r="Q61" s="54" t="s">
         <v>64</v>
       </c>
-      <c r="R61" s="50"/>
+      <c r="R61" s="54"/>
     </row>
     <row r="62" spans="1:19" x14ac:dyDescent="0.25">
       <c r="B62" s="2" t="s">
@@ -3560,10 +4847,10 @@
       </c>
     </row>
     <row r="66" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B66" s="52" t="s">
+      <c r="B66" s="63" t="s">
         <v>22</v>
       </c>
-      <c r="C66" s="52"/>
+      <c r="C66" s="63"/>
       <c r="E66" s="9" t="s">
         <v>67</v>
       </c>
@@ -3574,14 +4861,14 @@
         <v>85.5</v>
       </c>
       <c r="C67" s="53"/>
-      <c r="E67" s="54">
+      <c r="E67" s="73">
         <v>4.5</v>
       </c>
     </row>
     <row r="68" spans="1:19" x14ac:dyDescent="0.25">
       <c r="B68" s="53"/>
       <c r="C68" s="53"/>
-      <c r="E68" s="54"/>
+      <c r="E68" s="73"/>
     </row>
     <row r="70" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A70" s="6"/>
@@ -3606,26 +4893,26 @@
     </row>
     <row r="71" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="72" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B72" s="44" t="s">
+      <c r="B72" s="55" t="s">
         <v>122</v>
       </c>
-      <c r="C72" s="45"/>
-      <c r="D72" s="45"/>
-      <c r="E72" s="45"/>
-      <c r="F72" s="45"/>
-      <c r="G72" s="45"/>
-      <c r="H72" s="45"/>
-      <c r="I72" s="46"/>
+      <c r="C72" s="56"/>
+      <c r="D72" s="56"/>
+      <c r="E72" s="56"/>
+      <c r="F72" s="56"/>
+      <c r="G72" s="56"/>
+      <c r="H72" s="56"/>
+      <c r="I72" s="57"/>
     </row>
     <row r="73" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B73" s="47"/>
-      <c r="C73" s="48"/>
-      <c r="D73" s="48"/>
-      <c r="E73" s="48"/>
-      <c r="F73" s="48"/>
-      <c r="G73" s="48"/>
-      <c r="H73" s="48"/>
-      <c r="I73" s="49"/>
+      <c r="B73" s="58"/>
+      <c r="C73" s="59"/>
+      <c r="D73" s="59"/>
+      <c r="E73" s="59"/>
+      <c r="F73" s="59"/>
+      <c r="G73" s="59"/>
+      <c r="H73" s="59"/>
+      <c r="I73" s="60"/>
     </row>
     <row r="75" spans="1:19" x14ac:dyDescent="0.25">
       <c r="B75" s="4" t="s">
@@ -3652,10 +4939,10 @@
       <c r="I75" s="4" t="s">
         <v>130</v>
       </c>
-      <c r="K75" s="52" t="s">
+      <c r="K75" s="63" t="s">
         <v>22</v>
       </c>
-      <c r="L75" s="52"/>
+      <c r="L75" s="63"/>
       <c r="N75" s="9" t="s">
         <v>67</v>
       </c>
@@ -3757,8 +5044,11 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CEAA0BBB-B59A-4C0E-8304-D0FA810EECB4}">
+  <sheetPr>
+    <tabColor theme="0" tint="-0.14999847407452621"/>
+  </sheetPr>
   <dimension ref="B1:F41"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -4339,8 +5629,412 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5DD1FAA5-236E-4DD4-8E6C-D46CD3E83407}">
+  <sheetPr>
+    <tabColor theme="0" tint="-0.14999847407452621"/>
+  </sheetPr>
+  <dimension ref="B1:H22"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="3" max="3" width="10.140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="17.140625" style="1" customWidth="1"/>
+    <col min="5" max="5" width="12.28515625" style="1" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="63.85546875" style="1" customWidth="1"/>
+    <col min="7" max="7" width="12.140625" style="1" customWidth="1"/>
+    <col min="8" max="8" width="9.140625" style="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="2:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="2" spans="2:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="C2" s="15" t="s">
+        <v>132</v>
+      </c>
+      <c r="D2" s="97" t="s">
+        <v>133</v>
+      </c>
+      <c r="E2" s="97" t="s">
+        <v>167</v>
+      </c>
+      <c r="F2" s="97" t="s">
+        <v>179</v>
+      </c>
+      <c r="G2" s="97" t="s">
+        <v>245</v>
+      </c>
+      <c r="H2" s="97" t="s">
+        <v>253</v>
+      </c>
+    </row>
+    <row r="3" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B3" s="43" t="b">
+        <v>1</v>
+      </c>
+      <c r="C3" s="94" t="s">
+        <v>185</v>
+      </c>
+      <c r="D3" s="95" t="s">
+        <v>251</v>
+      </c>
+      <c r="E3" s="96" t="s">
+        <v>215</v>
+      </c>
+      <c r="F3" s="14"/>
+      <c r="G3" s="14" t="s">
+        <v>252</v>
+      </c>
+      <c r="H3" s="14" t="s">
+        <v>254</v>
+      </c>
+    </row>
+    <row r="4" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B4" s="43" t="b">
+        <v>0</v>
+      </c>
+      <c r="C4" s="46" t="s">
+        <v>185</v>
+      </c>
+      <c r="D4" s="44" t="s">
+        <v>255</v>
+      </c>
+      <c r="E4" s="45" t="s">
+        <v>216</v>
+      </c>
+      <c r="F4" s="2"/>
+      <c r="G4" s="2" t="s">
+        <v>252</v>
+      </c>
+      <c r="H4" s="2">
+        <v>536</v>
+      </c>
+    </row>
+    <row r="5" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B5" s="43" t="b">
+        <v>0</v>
+      </c>
+      <c r="C5" s="46" t="s">
+        <v>185</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>256</v>
+      </c>
+      <c r="E5" s="2" t="s">
+        <v>218</v>
+      </c>
+      <c r="F5" s="2"/>
+      <c r="G5" s="2" t="s">
+        <v>252</v>
+      </c>
+      <c r="H5" s="2" t="s">
+        <v>254</v>
+      </c>
+    </row>
+    <row r="6" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B6" s="43" t="b">
+        <v>0</v>
+      </c>
+      <c r="C6" s="46" t="s">
+        <v>185</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>257</v>
+      </c>
+      <c r="E6" s="2" t="s">
+        <v>217</v>
+      </c>
+      <c r="F6" s="2"/>
+      <c r="G6" s="2" t="s">
+        <v>252</v>
+      </c>
+      <c r="H6" s="2">
+        <v>536</v>
+      </c>
+    </row>
+    <row r="7" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B7" s="43" t="b">
+        <v>0</v>
+      </c>
+      <c r="C7" s="46" t="s">
+        <v>185</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>258</v>
+      </c>
+      <c r="E7" s="2" t="s">
+        <v>219</v>
+      </c>
+      <c r="F7" s="2"/>
+      <c r="G7" s="2" t="s">
+        <v>252</v>
+      </c>
+      <c r="H7" s="2" t="s">
+        <v>254</v>
+      </c>
+    </row>
+    <row r="9" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B9" s="43" t="b">
+        <v>1</v>
+      </c>
+      <c r="C9" s="46" t="s">
+        <v>186</v>
+      </c>
+      <c r="D9" s="2" t="s">
+        <v>233</v>
+      </c>
+      <c r="E9" s="42" t="s">
+        <v>234</v>
+      </c>
+      <c r="F9" s="2" t="s">
+        <v>241</v>
+      </c>
+      <c r="G9" s="2" t="s">
+        <v>246</v>
+      </c>
+    </row>
+    <row r="10" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B10" s="43" t="b">
+        <v>1</v>
+      </c>
+      <c r="C10" s="46" t="s">
+        <v>186</v>
+      </c>
+      <c r="D10" s="2" t="s">
+        <v>235</v>
+      </c>
+      <c r="E10" s="42" t="s">
+        <v>239</v>
+      </c>
+      <c r="F10" s="2" t="s">
+        <v>242</v>
+      </c>
+      <c r="G10" s="2" t="s">
+        <v>246</v>
+      </c>
+    </row>
+    <row r="11" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B11" s="43" t="b">
+        <v>0</v>
+      </c>
+      <c r="C11" s="46" t="s">
+        <v>186</v>
+      </c>
+      <c r="D11" s="2" t="s">
+        <v>236</v>
+      </c>
+      <c r="E11" s="42" t="s">
+        <v>240</v>
+      </c>
+      <c r="F11" s="2" t="s">
+        <v>243</v>
+      </c>
+      <c r="G11" s="2" t="s">
+        <v>246</v>
+      </c>
+    </row>
+    <row r="12" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B12" s="43" t="b">
+        <v>0</v>
+      </c>
+      <c r="C12" s="46" t="s">
+        <v>186</v>
+      </c>
+      <c r="D12" s="47" t="s">
+        <v>222</v>
+      </c>
+      <c r="E12" s="48" t="s">
+        <v>215</v>
+      </c>
+      <c r="F12" s="2" t="s">
+        <v>227</v>
+      </c>
+      <c r="G12" s="2" t="s">
+        <v>248</v>
+      </c>
+    </row>
+    <row r="13" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B13" s="43" t="b">
+        <v>0</v>
+      </c>
+      <c r="C13" s="46" t="s">
+        <v>186</v>
+      </c>
+      <c r="D13" s="44" t="s">
+        <v>223</v>
+      </c>
+      <c r="E13" s="48" t="s">
+        <v>217</v>
+      </c>
+      <c r="F13" s="2" t="s">
+        <v>229</v>
+      </c>
+      <c r="G13" s="2" t="s">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="14" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B14" s="43" t="b">
+        <v>0</v>
+      </c>
+      <c r="C14" s="46" t="s">
+        <v>186</v>
+      </c>
+      <c r="D14" s="44" t="s">
+        <v>224</v>
+      </c>
+      <c r="E14" s="48" t="s">
+        <v>216</v>
+      </c>
+      <c r="F14" s="2" t="s">
+        <v>228</v>
+      </c>
+      <c r="G14" s="2" t="s">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="15" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B15" s="43" t="b">
+        <v>0</v>
+      </c>
+      <c r="C15" s="46" t="s">
+        <v>186</v>
+      </c>
+      <c r="D15" s="44" t="s">
+        <v>221</v>
+      </c>
+      <c r="E15" s="48" t="s">
+        <v>218</v>
+      </c>
+      <c r="F15" s="2" t="s">
+        <v>230</v>
+      </c>
+      <c r="G15" s="2" t="s">
+        <v>248</v>
+      </c>
+    </row>
+    <row r="16" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B16" s="43" t="b">
+        <v>0</v>
+      </c>
+      <c r="C16" s="46" t="s">
+        <v>186</v>
+      </c>
+      <c r="D16" s="2" t="s">
+        <v>237</v>
+      </c>
+      <c r="E16" s="42" t="s">
+        <v>238</v>
+      </c>
+      <c r="F16" s="2" t="s">
+        <v>244</v>
+      </c>
+      <c r="G16" s="2" t="s">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="17" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B17" s="43" t="b">
+        <v>0</v>
+      </c>
+      <c r="C17" s="46" t="s">
+        <v>186</v>
+      </c>
+      <c r="D17" s="44" t="s">
+        <v>225</v>
+      </c>
+      <c r="E17" s="48" t="s">
+        <v>219</v>
+      </c>
+      <c r="F17" s="2" t="s">
+        <v>231</v>
+      </c>
+      <c r="G17" s="2" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="18" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B18" s="43" t="b">
+        <v>0</v>
+      </c>
+      <c r="C18" s="46" t="s">
+        <v>186</v>
+      </c>
+      <c r="D18" s="44" t="s">
+        <v>226</v>
+      </c>
+      <c r="E18" s="48" t="s">
+        <v>220</v>
+      </c>
+      <c r="F18" s="2" t="s">
+        <v>232</v>
+      </c>
+      <c r="G18" s="2" t="s">
+        <v>248</v>
+      </c>
+    </row>
+    <row r="20" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B20" s="43" t="b">
+        <v>0</v>
+      </c>
+      <c r="C20" s="46" t="s">
+        <v>187</v>
+      </c>
+      <c r="D20" s="44" t="s">
+        <v>296</v>
+      </c>
+      <c r="E20" s="93" t="s">
+        <v>289</v>
+      </c>
+      <c r="F20" s="2" t="s">
+        <v>297</v>
+      </c>
+      <c r="G20" s="92"/>
+      <c r="H20" s="92"/>
+    </row>
+    <row r="21" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B21" s="43" t="b">
+        <v>0</v>
+      </c>
+      <c r="C21" s="46" t="s">
+        <v>187</v>
+      </c>
+      <c r="D21" s="44" t="s">
+        <v>298</v>
+      </c>
+      <c r="E21" s="45" t="s">
+        <v>290</v>
+      </c>
+      <c r="F21" s="2" t="s">
+        <v>299</v>
+      </c>
+    </row>
+    <row r="22" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B22" s="43" t="b">
+        <v>0</v>
+      </c>
+      <c r="C22" s="46" t="s">
+        <v>187</v>
+      </c>
+      <c r="D22" s="2" t="s">
+        <v>300</v>
+      </c>
+      <c r="E22" s="2" t="s">
+        <v>291</v>
+      </c>
+      <c r="F22" s="2" t="s">
+        <v>301</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="1" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DBA352BE-3E69-4CCA-8EEB-A9094B74606F}">
+  <sheetPr>
+    <tabColor theme="7" tint="0.79998168889431442"/>
+  </sheetPr>
   <dimension ref="B1:L11"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -4357,21 +6051,21 @@
   <sheetData>
     <row r="1" spans="2:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="2" spans="2:12" ht="23.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B2" s="63" t="s">
+      <c r="B2" s="80" t="s">
         <v>188</v>
       </c>
-      <c r="C2" s="64"/>
-      <c r="D2" s="65"/>
-      <c r="F2" s="63" t="s">
+      <c r="C2" s="81"/>
+      <c r="D2" s="82"/>
+      <c r="F2" s="80" t="s">
         <v>189</v>
       </c>
-      <c r="G2" s="64"/>
-      <c r="H2" s="65"/>
-      <c r="J2" s="63" t="s">
+      <c r="G2" s="81"/>
+      <c r="H2" s="82"/>
+      <c r="J2" s="80" t="s">
         <v>190</v>
       </c>
-      <c r="K2" s="64"/>
-      <c r="L2" s="65"/>
+      <c r="K2" s="81"/>
+      <c r="L2" s="82"/>
     </row>
     <row r="3" spans="2:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B3" s="29" t="s">
@@ -4556,26 +6250,26 @@
     </row>
     <row r="10" spans="2:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="11" spans="2:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B11" s="66" t="s">
+      <c r="B11" s="83" t="s">
         <v>182</v>
       </c>
-      <c r="C11" s="67"/>
+      <c r="C11" s="84"/>
       <c r="D11" s="28">
         <f>(D4*C4+D5*C5+D6*C6+D7*C7+D8*C8+D9*C9)/30</f>
         <v>4.4333333333333336</v>
       </c>
-      <c r="F11" s="66" t="s">
+      <c r="F11" s="83" t="s">
         <v>182</v>
       </c>
-      <c r="G11" s="67"/>
+      <c r="G11" s="84"/>
       <c r="H11" s="28">
         <f>(H4*G4+H5*G5+H6*G6+H7*G7+H8*G8)/30</f>
         <v>4.75</v>
       </c>
-      <c r="J11" s="66" t="s">
+      <c r="J11" s="83" t="s">
         <v>182</v>
       </c>
-      <c r="K11" s="67"/>
+      <c r="K11" s="84"/>
       <c r="L11" s="28">
         <f>(L4*K4+L5*K5+L6*K6+L7*K7+L8*K8)/30</f>
         <v>0</v>

</xml_diff>

<commit_message>
Updated schedule - FIZ2 colloquium
</commit_message>
<xml_diff>
--- a/IoT-points-schedule.xlsx
+++ b/IoT-points-schedule.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\dodo\Desktop\IoT-studies\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0BB201D0-AF96-4BBA-AE1A-A92AE39289F6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{68A983F3-682A-4E4A-8C85-CD5E131CE62F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="25440" windowHeight="15390" xr2:uid="{F85F5544-1FE8-4920-A5D4-192A98B113BD}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="25440" windowHeight="15390" activeTab="4" xr2:uid="{F85F5544-1FE8-4920-A5D4-192A98B113BD}"/>
   </bookViews>
   <sheets>
     <sheet name="III-semestr-25Z" sheetId="5" r:id="rId1"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="527" uniqueCount="316">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="531" uniqueCount="318">
   <si>
     <t>1. Krypto</t>
   </si>
@@ -989,6 +989,12 @@
   </si>
   <si>
     <t>2. Egzamin: minimum 21 pkt</t>
+  </si>
+  <si>
+    <t>14 listopada</t>
+  </si>
+  <si>
+    <t>Kolos 1</t>
   </si>
 </sst>
 </file>
@@ -1377,7 +1383,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="98">
+  <cellXfs count="97">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1538,15 +1544,81 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="9" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="9" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="9" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="9" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="9" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="9" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1565,60 +1637,30 @@
     <xf numFmtId="0" fontId="5" fillId="5" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="2" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="2" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="2" fontId="2" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="2" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1635,45 +1677,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="9" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="9" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="9" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="9" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="9" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="9" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -2055,87 +2058,87 @@
   <sheetData>
     <row r="1" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="2" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="B2" s="85" t="s">
+      <c r="B2" s="57" t="s">
         <v>185</v>
       </c>
-      <c r="C2" s="86"/>
-      <c r="D2" s="86"/>
-      <c r="E2" s="86"/>
-      <c r="F2" s="86"/>
-      <c r="G2" s="86"/>
-      <c r="H2" s="86"/>
-      <c r="I2" s="86"/>
-      <c r="J2" s="86"/>
-      <c r="K2" s="86"/>
-      <c r="L2" s="86"/>
-      <c r="M2" s="86"/>
-      <c r="N2" s="86"/>
-      <c r="O2" s="86"/>
-      <c r="P2" s="87"/>
-      <c r="R2" s="69" t="s">
+      <c r="C2" s="58"/>
+      <c r="D2" s="58"/>
+      <c r="E2" s="58"/>
+      <c r="F2" s="58"/>
+      <c r="G2" s="58"/>
+      <c r="H2" s="58"/>
+      <c r="I2" s="58"/>
+      <c r="J2" s="58"/>
+      <c r="K2" s="58"/>
+      <c r="L2" s="58"/>
+      <c r="M2" s="58"/>
+      <c r="N2" s="58"/>
+      <c r="O2" s="58"/>
+      <c r="P2" s="59"/>
+      <c r="R2" s="64" t="s">
         <v>268</v>
       </c>
-      <c r="S2" s="69"/>
-      <c r="T2" s="69"/>
-      <c r="U2" s="69"/>
+      <c r="S2" s="64"/>
+      <c r="T2" s="64"/>
+      <c r="U2" s="64"/>
     </row>
     <row r="3" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B3" s="88"/>
-      <c r="C3" s="89"/>
-      <c r="D3" s="89"/>
-      <c r="E3" s="89"/>
-      <c r="F3" s="89"/>
-      <c r="G3" s="89"/>
-      <c r="H3" s="89"/>
-      <c r="I3" s="89"/>
-      <c r="J3" s="89"/>
-      <c r="K3" s="89"/>
-      <c r="L3" s="89"/>
-      <c r="M3" s="89"/>
-      <c r="N3" s="89"/>
-      <c r="O3" s="89"/>
-      <c r="P3" s="90"/>
-      <c r="R3" s="66" t="s">
+      <c r="B3" s="60"/>
+      <c r="C3" s="61"/>
+      <c r="D3" s="61"/>
+      <c r="E3" s="61"/>
+      <c r="F3" s="61"/>
+      <c r="G3" s="61"/>
+      <c r="H3" s="61"/>
+      <c r="I3" s="61"/>
+      <c r="J3" s="61"/>
+      <c r="K3" s="61"/>
+      <c r="L3" s="61"/>
+      <c r="M3" s="61"/>
+      <c r="N3" s="61"/>
+      <c r="O3" s="61"/>
+      <c r="P3" s="62"/>
+      <c r="R3" s="65" t="s">
         <v>264</v>
       </c>
-      <c r="S3" s="67"/>
-      <c r="T3" s="67"/>
-      <c r="U3" s="68"/>
+      <c r="S3" s="66"/>
+      <c r="T3" s="66"/>
+      <c r="U3" s="67"/>
     </row>
     <row r="4" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="R4" s="66" t="s">
+      <c r="R4" s="65" t="s">
         <v>265</v>
       </c>
-      <c r="S4" s="67"/>
-      <c r="T4" s="67"/>
-      <c r="U4" s="68"/>
+      <c r="S4" s="66"/>
+      <c r="T4" s="66"/>
+      <c r="U4" s="67"/>
     </row>
     <row r="5" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="B5" s="52" t="s">
+      <c r="B5" s="63" t="s">
         <v>261</v>
       </c>
-      <c r="C5" s="52"/>
-      <c r="E5" s="52" t="s">
+      <c r="C5" s="63"/>
+      <c r="E5" s="63" t="s">
         <v>262</v>
       </c>
-      <c r="F5" s="52"/>
-      <c r="G5" s="52"/>
-      <c r="H5" s="52"/>
-      <c r="I5" s="52"/>
-      <c r="K5" s="52" t="s">
+      <c r="F5" s="63"/>
+      <c r="G5" s="63"/>
+      <c r="H5" s="63"/>
+      <c r="I5" s="63"/>
+      <c r="K5" s="63" t="s">
         <v>263</v>
       </c>
-      <c r="L5" s="52"/>
-      <c r="M5" s="52"/>
-      <c r="N5" s="52"/>
-      <c r="O5" s="52"/>
-      <c r="P5" s="52"/>
-      <c r="R5" s="66" t="s">
+      <c r="L5" s="63"/>
+      <c r="M5" s="63"/>
+      <c r="N5" s="63"/>
+      <c r="O5" s="63"/>
+      <c r="P5" s="63"/>
+      <c r="R5" s="65" t="s">
         <v>266</v>
       </c>
-      <c r="S5" s="67"/>
-      <c r="T5" s="67"/>
-      <c r="U5" s="68"/>
+      <c r="S5" s="66"/>
+      <c r="T5" s="66"/>
+      <c r="U5" s="67"/>
     </row>
     <row r="6" spans="1:22" x14ac:dyDescent="0.25">
       <c r="B6" s="49" t="s">
@@ -2177,12 +2180,12 @@
       <c r="P6" s="49" t="s">
         <v>288</v>
       </c>
-      <c r="R6" s="66" t="s">
+      <c r="R6" s="65" t="s">
         <v>267</v>
       </c>
-      <c r="S6" s="67"/>
-      <c r="T6" s="67"/>
-      <c r="U6" s="68"/>
+      <c r="S6" s="66"/>
+      <c r="T6" s="66"/>
+      <c r="U6" s="67"/>
     </row>
     <row r="7" spans="1:22" x14ac:dyDescent="0.25">
       <c r="B7" s="50"/>
@@ -2198,37 +2201,37 @@
       <c r="N7" s="50"/>
       <c r="O7" s="50"/>
       <c r="P7" s="50"/>
-      <c r="R7" s="66" t="s">
+      <c r="R7" s="65" t="s">
         <v>269</v>
       </c>
-      <c r="S7" s="67"/>
-      <c r="T7" s="67"/>
-      <c r="U7" s="68"/>
+      <c r="S7" s="66"/>
+      <c r="T7" s="66"/>
+      <c r="U7" s="67"/>
     </row>
     <row r="9" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="B9" s="63" t="s">
+      <c r="B9" s="69" t="s">
         <v>22</v>
       </c>
-      <c r="C9" s="63"/>
+      <c r="C9" s="69"/>
       <c r="D9" s="1"/>
       <c r="E9" s="9" t="s">
         <v>67</v>
       </c>
     </row>
     <row r="10" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="B10" s="53">
+      <c r="B10" s="70">
         <f>SUM(B7:C7,E7:I7,K7:P7)</f>
         <v>0</v>
       </c>
-      <c r="C10" s="53"/>
+      <c r="C10" s="70"/>
       <c r="D10" s="1"/>
-      <c r="E10" s="64"/>
+      <c r="E10" s="71"/>
     </row>
     <row r="11" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="B11" s="53"/>
-      <c r="C11" s="53"/>
+      <c r="B11" s="70"/>
+      <c r="C11" s="70"/>
       <c r="D11" s="1"/>
-      <c r="E11" s="65"/>
+      <c r="E11" s="72"/>
     </row>
     <row r="12" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A12" s="6"/>
@@ -2256,82 +2259,82 @@
     </row>
     <row r="13" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="14" spans="1:22" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B14" s="85" t="s">
+      <c r="B14" s="57" t="s">
         <v>186</v>
       </c>
-      <c r="C14" s="86"/>
-      <c r="D14" s="86"/>
-      <c r="E14" s="86"/>
-      <c r="F14" s="86"/>
-      <c r="G14" s="86"/>
-      <c r="H14" s="86"/>
-      <c r="I14" s="86"/>
-      <c r="J14" s="86"/>
-      <c r="K14" s="86"/>
-      <c r="L14" s="86"/>
-      <c r="M14" s="86"/>
-      <c r="N14" s="86"/>
-      <c r="O14" s="86"/>
-      <c r="P14" s="86"/>
-      <c r="Q14" s="87"/>
-      <c r="S14" s="69" t="s">
+      <c r="C14" s="58"/>
+      <c r="D14" s="58"/>
+      <c r="E14" s="58"/>
+      <c r="F14" s="58"/>
+      <c r="G14" s="58"/>
+      <c r="H14" s="58"/>
+      <c r="I14" s="58"/>
+      <c r="J14" s="58"/>
+      <c r="K14" s="58"/>
+      <c r="L14" s="58"/>
+      <c r="M14" s="58"/>
+      <c r="N14" s="58"/>
+      <c r="O14" s="58"/>
+      <c r="P14" s="58"/>
+      <c r="Q14" s="59"/>
+      <c r="S14" s="64" t="s">
         <v>268</v>
       </c>
-      <c r="T14" s="69"/>
-      <c r="U14" s="69"/>
-      <c r="V14" s="69"/>
+      <c r="T14" s="64"/>
+      <c r="U14" s="64"/>
+      <c r="V14" s="64"/>
     </row>
     <row r="15" spans="1:22" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B15" s="88"/>
-      <c r="C15" s="89"/>
-      <c r="D15" s="89"/>
-      <c r="E15" s="89"/>
-      <c r="F15" s="89"/>
-      <c r="G15" s="89"/>
-      <c r="H15" s="89"/>
-      <c r="I15" s="89"/>
-      <c r="J15" s="89"/>
-      <c r="K15" s="89"/>
-      <c r="L15" s="89"/>
-      <c r="M15" s="89"/>
-      <c r="N15" s="89"/>
-      <c r="O15" s="89"/>
-      <c r="P15" s="89"/>
-      <c r="Q15" s="90"/>
-      <c r="S15" s="66" t="s">
+      <c r="B15" s="60"/>
+      <c r="C15" s="61"/>
+      <c r="D15" s="61"/>
+      <c r="E15" s="61"/>
+      <c r="F15" s="61"/>
+      <c r="G15" s="61"/>
+      <c r="H15" s="61"/>
+      <c r="I15" s="61"/>
+      <c r="J15" s="61"/>
+      <c r="K15" s="61"/>
+      <c r="L15" s="61"/>
+      <c r="M15" s="61"/>
+      <c r="N15" s="61"/>
+      <c r="O15" s="61"/>
+      <c r="P15" s="61"/>
+      <c r="Q15" s="62"/>
+      <c r="S15" s="65" t="s">
         <v>314</v>
       </c>
-      <c r="T15" s="67"/>
-      <c r="U15" s="67"/>
-      <c r="V15" s="68"/>
+      <c r="T15" s="66"/>
+      <c r="U15" s="66"/>
+      <c r="V15" s="67"/>
     </row>
     <row r="16" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="S16" s="66" t="s">
+      <c r="S16" s="65" t="s">
         <v>315</v>
       </c>
-      <c r="T16" s="67"/>
-      <c r="U16" s="67"/>
-      <c r="V16" s="68"/>
+      <c r="T16" s="66"/>
+      <c r="U16" s="66"/>
+      <c r="V16" s="67"/>
     </row>
     <row r="17" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="B17" s="52" t="s">
+      <c r="B17" s="63" t="s">
         <v>270</v>
       </c>
-      <c r="C17" s="52"/>
-      <c r="D17" s="52"/>
-      <c r="E17" s="52"/>
-      <c r="G17" s="52" t="s">
+      <c r="C17" s="63"/>
+      <c r="D17" s="63"/>
+      <c r="E17" s="63"/>
+      <c r="G17" s="63" t="s">
         <v>275</v>
       </c>
-      <c r="H17" s="52"/>
-      <c r="I17" s="52"/>
-      <c r="J17" s="52"/>
-      <c r="K17" s="52"/>
-      <c r="L17" s="52"/>
-      <c r="N17" s="52" t="s">
+      <c r="H17" s="63"/>
+      <c r="I17" s="63"/>
+      <c r="J17" s="63"/>
+      <c r="K17" s="63"/>
+      <c r="L17" s="63"/>
+      <c r="N17" s="63" t="s">
         <v>276</v>
       </c>
-      <c r="O17" s="52"/>
+      <c r="O17" s="63"/>
       <c r="Q17" s="51" t="s">
         <v>277</v>
       </c>
@@ -2373,7 +2376,7 @@
       <c r="O18" s="49" t="s">
         <v>260</v>
       </c>
-      <c r="Q18" s="61"/>
+      <c r="Q18" s="73"/>
     </row>
     <row r="19" spans="1:22" x14ac:dyDescent="0.25">
       <c r="B19" s="49"/>
@@ -2388,32 +2391,32 @@
       <c r="L19" s="49"/>
       <c r="N19" s="49"/>
       <c r="O19" s="49"/>
-      <c r="Q19" s="62"/>
+      <c r="Q19" s="74"/>
     </row>
     <row r="21" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="B21" s="63" t="s">
+      <c r="B21" s="69" t="s">
         <v>22</v>
       </c>
-      <c r="C21" s="63"/>
+      <c r="C21" s="69"/>
       <c r="D21" s="1"/>
       <c r="E21" s="9" t="s">
         <v>67</v>
       </c>
     </row>
     <row r="22" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="B22" s="53">
+      <c r="B22" s="70">
         <f>SUM(B19:E19,G19:L19,N19:O19,Q18)</f>
         <v>0</v>
       </c>
-      <c r="C22" s="53"/>
+      <c r="C22" s="70"/>
       <c r="D22" s="1"/>
-      <c r="E22" s="64"/>
+      <c r="E22" s="71"/>
     </row>
     <row r="23" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="B23" s="53"/>
-      <c r="C23" s="53"/>
+      <c r="B23" s="70"/>
+      <c r="C23" s="70"/>
       <c r="D23" s="1"/>
-      <c r="E23" s="65"/>
+      <c r="E23" s="72"/>
     </row>
     <row r="24" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A24" s="6"/>
@@ -2441,74 +2444,74 @@
     </row>
     <row r="25" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="26" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="B26" s="85" t="s">
+      <c r="B26" s="57" t="s">
         <v>184</v>
       </c>
-      <c r="C26" s="86"/>
-      <c r="D26" s="86"/>
-      <c r="E26" s="86"/>
-      <c r="F26" s="86"/>
-      <c r="G26" s="86"/>
-      <c r="H26" s="86"/>
-      <c r="I26" s="86"/>
-      <c r="J26" s="86"/>
-      <c r="K26" s="86"/>
-      <c r="L26" s="86"/>
-      <c r="M26" s="86"/>
-      <c r="N26" s="86"/>
-      <c r="O26" s="86"/>
-      <c r="P26" s="86"/>
-      <c r="Q26" s="87"/>
-      <c r="S26" s="69" t="s">
+      <c r="C26" s="58"/>
+      <c r="D26" s="58"/>
+      <c r="E26" s="58"/>
+      <c r="F26" s="58"/>
+      <c r="G26" s="58"/>
+      <c r="H26" s="58"/>
+      <c r="I26" s="58"/>
+      <c r="J26" s="58"/>
+      <c r="K26" s="58"/>
+      <c r="L26" s="58"/>
+      <c r="M26" s="58"/>
+      <c r="N26" s="58"/>
+      <c r="O26" s="58"/>
+      <c r="P26" s="58"/>
+      <c r="Q26" s="59"/>
+      <c r="S26" s="64" t="s">
         <v>268</v>
       </c>
-      <c r="T26" s="69"/>
-      <c r="U26" s="69"/>
-      <c r="V26" s="69"/>
+      <c r="T26" s="64"/>
+      <c r="U26" s="64"/>
+      <c r="V26" s="64"/>
     </row>
     <row r="27" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B27" s="88"/>
-      <c r="C27" s="89"/>
-      <c r="D27" s="89"/>
-      <c r="E27" s="89"/>
-      <c r="F27" s="89"/>
-      <c r="G27" s="89"/>
-      <c r="H27" s="89"/>
-      <c r="I27" s="89"/>
-      <c r="J27" s="89"/>
-      <c r="K27" s="89"/>
-      <c r="L27" s="89"/>
-      <c r="M27" s="89"/>
-      <c r="N27" s="89"/>
-      <c r="O27" s="89"/>
-      <c r="P27" s="89"/>
-      <c r="Q27" s="90"/>
-      <c r="S27" s="66" t="s">
+      <c r="B27" s="60"/>
+      <c r="C27" s="61"/>
+      <c r="D27" s="61"/>
+      <c r="E27" s="61"/>
+      <c r="F27" s="61"/>
+      <c r="G27" s="61"/>
+      <c r="H27" s="61"/>
+      <c r="I27" s="61"/>
+      <c r="J27" s="61"/>
+      <c r="K27" s="61"/>
+      <c r="L27" s="61"/>
+      <c r="M27" s="61"/>
+      <c r="N27" s="61"/>
+      <c r="O27" s="61"/>
+      <c r="P27" s="61"/>
+      <c r="Q27" s="62"/>
+      <c r="S27" s="65" t="s">
         <v>312</v>
       </c>
-      <c r="T27" s="67"/>
-      <c r="U27" s="67"/>
-      <c r="V27" s="68"/>
+      <c r="T27" s="66"/>
+      <c r="U27" s="66"/>
+      <c r="V27" s="67"/>
     </row>
     <row r="28" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="S28" s="66" t="s">
+      <c r="S28" s="65" t="s">
         <v>313</v>
       </c>
-      <c r="T28" s="67"/>
-      <c r="U28" s="67"/>
-      <c r="V28" s="68"/>
+      <c r="T28" s="66"/>
+      <c r="U28" s="66"/>
+      <c r="V28" s="67"/>
     </row>
     <row r="29" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="B29" s="54" t="s">
+      <c r="B29" s="75" t="s">
         <v>8</v>
       </c>
-      <c r="C29" s="54"/>
-      <c r="D29" s="54"/>
-      <c r="E29" s="54"/>
-      <c r="G29" s="52" t="s">
+      <c r="C29" s="75"/>
+      <c r="D29" s="75"/>
+      <c r="E29" s="75"/>
+      <c r="G29" s="63" t="s">
         <v>281</v>
       </c>
-      <c r="H29" s="52"/>
+      <c r="H29" s="63"/>
     </row>
     <row r="30" spans="1:22" x14ac:dyDescent="0.25">
       <c r="B30" s="2" t="s">
@@ -2517,10 +2520,10 @@
       <c r="C30" s="2" t="s">
         <v>279</v>
       </c>
-      <c r="D30" s="53" t="s">
+      <c r="D30" s="70" t="s">
         <v>280</v>
       </c>
-      <c r="E30" s="53"/>
+      <c r="E30" s="70"/>
       <c r="G30" s="49" t="s">
         <v>73</v>
       </c>
@@ -2531,8 +2534,8 @@
     <row r="31" spans="1:22" x14ac:dyDescent="0.25">
       <c r="B31" s="2"/>
       <c r="C31" s="2"/>
-      <c r="D31" s="53"/>
-      <c r="E31" s="53"/>
+      <c r="D31" s="70"/>
+      <c r="E31" s="70"/>
       <c r="G31" s="49"/>
       <c r="H31" s="49"/>
     </row>
@@ -2562,87 +2565,87 @@
     </row>
     <row r="33" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="34" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="B34" s="85" t="s">
+      <c r="B34" s="57" t="s">
         <v>187</v>
       </c>
-      <c r="C34" s="86"/>
-      <c r="D34" s="86"/>
-      <c r="E34" s="86"/>
-      <c r="F34" s="86"/>
-      <c r="G34" s="86"/>
-      <c r="H34" s="86"/>
-      <c r="I34" s="86"/>
-      <c r="J34" s="86"/>
-      <c r="K34" s="86"/>
-      <c r="L34" s="86"/>
-      <c r="M34" s="86"/>
-      <c r="N34" s="86"/>
-      <c r="O34" s="86"/>
-      <c r="P34" s="86"/>
-      <c r="Q34" s="87"/>
-      <c r="S34" s="69" t="s">
+      <c r="C34" s="58"/>
+      <c r="D34" s="58"/>
+      <c r="E34" s="58"/>
+      <c r="F34" s="58"/>
+      <c r="G34" s="58"/>
+      <c r="H34" s="58"/>
+      <c r="I34" s="58"/>
+      <c r="J34" s="58"/>
+      <c r="K34" s="58"/>
+      <c r="L34" s="58"/>
+      <c r="M34" s="58"/>
+      <c r="N34" s="58"/>
+      <c r="O34" s="58"/>
+      <c r="P34" s="58"/>
+      <c r="Q34" s="59"/>
+      <c r="S34" s="64" t="s">
         <v>268</v>
       </c>
-      <c r="T34" s="69"/>
-      <c r="U34" s="69"/>
-      <c r="V34" s="69"/>
+      <c r="T34" s="64"/>
+      <c r="U34" s="64"/>
+      <c r="V34" s="64"/>
     </row>
     <row r="35" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B35" s="88"/>
-      <c r="C35" s="89"/>
-      <c r="D35" s="89"/>
-      <c r="E35" s="89"/>
-      <c r="F35" s="89"/>
-      <c r="G35" s="89"/>
-      <c r="H35" s="89"/>
-      <c r="I35" s="89"/>
-      <c r="J35" s="89"/>
-      <c r="K35" s="89"/>
-      <c r="L35" s="89"/>
-      <c r="M35" s="89"/>
-      <c r="N35" s="89"/>
-      <c r="O35" s="89"/>
-      <c r="P35" s="89"/>
-      <c r="Q35" s="90"/>
-      <c r="S35" s="66" t="s">
+      <c r="B35" s="60"/>
+      <c r="C35" s="61"/>
+      <c r="D35" s="61"/>
+      <c r="E35" s="61"/>
+      <c r="F35" s="61"/>
+      <c r="G35" s="61"/>
+      <c r="H35" s="61"/>
+      <c r="I35" s="61"/>
+      <c r="J35" s="61"/>
+      <c r="K35" s="61"/>
+      <c r="L35" s="61"/>
+      <c r="M35" s="61"/>
+      <c r="N35" s="61"/>
+      <c r="O35" s="61"/>
+      <c r="P35" s="61"/>
+      <c r="Q35" s="62"/>
+      <c r="S35" s="65" t="s">
         <v>309</v>
       </c>
-      <c r="T35" s="67"/>
-      <c r="U35" s="67"/>
-      <c r="V35" s="68"/>
+      <c r="T35" s="66"/>
+      <c r="U35" s="66"/>
+      <c r="V35" s="67"/>
     </row>
     <row r="36" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="S36" s="66" t="s">
+      <c r="S36" s="65" t="s">
         <v>310</v>
       </c>
-      <c r="T36" s="67"/>
-      <c r="U36" s="67"/>
-      <c r="V36" s="68"/>
+      <c r="T36" s="66"/>
+      <c r="U36" s="66"/>
+      <c r="V36" s="67"/>
     </row>
     <row r="37" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="B37" s="52" t="s">
+      <c r="B37" s="63" t="s">
         <v>302</v>
       </c>
-      <c r="C37" s="52"/>
-      <c r="D37" s="52"/>
-      <c r="E37" s="52"/>
-      <c r="F37" s="52"/>
-      <c r="G37" s="52"/>
-      <c r="H37" s="52"/>
-      <c r="I37" s="52"/>
-      <c r="J37" s="52"/>
-      <c r="K37" s="52"/>
-      <c r="L37" s="52"/>
-      <c r="M37" s="52"/>
-      <c r="N37" s="52"/>
-      <c r="O37" s="52"/>
-      <c r="P37" s="52"/>
-      <c r="S37" s="66" t="s">
+      <c r="C37" s="63"/>
+      <c r="D37" s="63"/>
+      <c r="E37" s="63"/>
+      <c r="F37" s="63"/>
+      <c r="G37" s="63"/>
+      <c r="H37" s="63"/>
+      <c r="I37" s="63"/>
+      <c r="J37" s="63"/>
+      <c r="K37" s="63"/>
+      <c r="L37" s="63"/>
+      <c r="M37" s="63"/>
+      <c r="N37" s="63"/>
+      <c r="O37" s="63"/>
+      <c r="P37" s="63"/>
+      <c r="S37" s="65" t="s">
         <v>311</v>
       </c>
-      <c r="T37" s="67"/>
-      <c r="U37" s="67"/>
-      <c r="V37" s="68"/>
+      <c r="T37" s="66"/>
+      <c r="U37" s="66"/>
+      <c r="V37" s="67"/>
     </row>
     <row r="38" spans="1:22" x14ac:dyDescent="0.25">
       <c r="B38" s="49" t="s">
@@ -2709,34 +2712,34 @@
       <c r="P39" s="49"/>
     </row>
     <row r="41" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="B41" s="52" t="s">
+      <c r="B41" s="63" t="s">
         <v>304</v>
       </c>
-      <c r="C41" s="52"/>
-      <c r="D41" s="52"/>
-      <c r="E41" s="52"/>
-      <c r="F41" s="52"/>
-      <c r="G41" s="52"/>
-      <c r="I41" s="52" t="s">
+      <c r="C41" s="63"/>
+      <c r="D41" s="63"/>
+      <c r="E41" s="63"/>
+      <c r="F41" s="63"/>
+      <c r="G41" s="63"/>
+      <c r="I41" s="63" t="s">
         <v>303</v>
       </c>
-      <c r="J41" s="52"/>
+      <c r="J41" s="63"/>
     </row>
     <row r="42" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="B42" s="91" t="s">
+      <c r="B42" s="68" t="s">
         <v>293</v>
       </c>
-      <c r="C42" s="91"/>
-      <c r="D42" s="91" t="s">
+      <c r="C42" s="68"/>
+      <c r="D42" s="68" t="s">
         <v>294</v>
       </c>
-      <c r="E42" s="91"/>
-      <c r="F42" s="91" t="s">
+      <c r="E42" s="68"/>
+      <c r="F42" s="68" t="s">
         <v>295</v>
       </c>
-      <c r="G42" s="91"/>
-      <c r="I42" s="91"/>
-      <c r="J42" s="91"/>
+      <c r="G42" s="68"/>
+      <c r="I42" s="68"/>
+      <c r="J42" s="68"/>
     </row>
     <row r="43" spans="1:22" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B43" s="2" t="s">
@@ -2757,8 +2760,8 @@
       <c r="G43" s="2" t="s">
         <v>292</v>
       </c>
-      <c r="I43" s="91"/>
-      <c r="J43" s="91"/>
+      <c r="I43" s="68"/>
+      <c r="J43" s="68"/>
     </row>
     <row r="44" spans="1:22" x14ac:dyDescent="0.25">
       <c r="B44" s="50"/>
@@ -2767,8 +2770,8 @@
       <c r="E44" s="50"/>
       <c r="F44" s="50"/>
       <c r="G44" s="50"/>
-      <c r="I44" s="91"/>
-      <c r="J44" s="91"/>
+      <c r="I44" s="68"/>
+      <c r="J44" s="68"/>
     </row>
     <row r="45" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A45" s="6"/>
@@ -2796,53 +2799,53 @@
     </row>
     <row r="46" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="47" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="B47" s="85" t="s">
+      <c r="B47" s="57" t="s">
         <v>305</v>
       </c>
-      <c r="C47" s="86"/>
-      <c r="D47" s="86"/>
-      <c r="E47" s="86"/>
-      <c r="F47" s="86"/>
-      <c r="G47" s="86"/>
-      <c r="H47" s="86"/>
-      <c r="I47" s="86"/>
-      <c r="J47" s="86"/>
-      <c r="K47" s="86"/>
-      <c r="L47" s="86"/>
-      <c r="M47" s="86"/>
-      <c r="N47" s="86"/>
-      <c r="O47" s="86"/>
-      <c r="P47" s="86"/>
-      <c r="Q47" s="87"/>
+      <c r="C47" s="58"/>
+      <c r="D47" s="58"/>
+      <c r="E47" s="58"/>
+      <c r="F47" s="58"/>
+      <c r="G47" s="58"/>
+      <c r="H47" s="58"/>
+      <c r="I47" s="58"/>
+      <c r="J47" s="58"/>
+      <c r="K47" s="58"/>
+      <c r="L47" s="58"/>
+      <c r="M47" s="58"/>
+      <c r="N47" s="58"/>
+      <c r="O47" s="58"/>
+      <c r="P47" s="58"/>
+      <c r="Q47" s="59"/>
     </row>
     <row r="48" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B48" s="88"/>
-      <c r="C48" s="89"/>
-      <c r="D48" s="89"/>
-      <c r="E48" s="89"/>
-      <c r="F48" s="89"/>
-      <c r="G48" s="89"/>
-      <c r="H48" s="89"/>
-      <c r="I48" s="89"/>
-      <c r="J48" s="89"/>
-      <c r="K48" s="89"/>
-      <c r="L48" s="89"/>
-      <c r="M48" s="89"/>
-      <c r="N48" s="89"/>
-      <c r="O48" s="89"/>
-      <c r="P48" s="89"/>
-      <c r="Q48" s="90"/>
+      <c r="B48" s="60"/>
+      <c r="C48" s="61"/>
+      <c r="D48" s="61"/>
+      <c r="E48" s="61"/>
+      <c r="F48" s="61"/>
+      <c r="G48" s="61"/>
+      <c r="H48" s="61"/>
+      <c r="I48" s="61"/>
+      <c r="J48" s="61"/>
+      <c r="K48" s="61"/>
+      <c r="L48" s="61"/>
+      <c r="M48" s="61"/>
+      <c r="N48" s="61"/>
+      <c r="O48" s="61"/>
+      <c r="P48" s="61"/>
+      <c r="Q48" s="62"/>
     </row>
     <row r="50" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B50" s="52" t="s">
+      <c r="B50" s="63" t="s">
         <v>306</v>
       </c>
-      <c r="C50" s="52"/>
-      <c r="D50" s="52"/>
-      <c r="E50" s="52"/>
-      <c r="F50" s="52"/>
-      <c r="G50" s="52"/>
-      <c r="H50" s="52"/>
+      <c r="C50" s="63"/>
+      <c r="D50" s="63"/>
+      <c r="E50" s="63"/>
+      <c r="F50" s="63"/>
+      <c r="G50" s="63"/>
+      <c r="H50" s="63"/>
     </row>
     <row r="51" spans="2:8" s="16" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B51" s="49" t="s">
@@ -2856,12 +2859,29 @@
     </row>
   </sheetData>
   <mergeCells count="46">
-    <mergeCell ref="B47:Q48"/>
-    <mergeCell ref="B50:H50"/>
-    <mergeCell ref="S34:V34"/>
-    <mergeCell ref="S35:V35"/>
-    <mergeCell ref="S36:V36"/>
-    <mergeCell ref="S37:V37"/>
+    <mergeCell ref="D30:E30"/>
+    <mergeCell ref="B29:E29"/>
+    <mergeCell ref="D31:E31"/>
+    <mergeCell ref="G29:H29"/>
+    <mergeCell ref="B34:Q35"/>
+    <mergeCell ref="Q18:Q19"/>
+    <mergeCell ref="B21:C21"/>
+    <mergeCell ref="B22:C23"/>
+    <mergeCell ref="E22:E23"/>
+    <mergeCell ref="B26:Q27"/>
+    <mergeCell ref="R3:U3"/>
+    <mergeCell ref="B17:E17"/>
+    <mergeCell ref="G17:L17"/>
+    <mergeCell ref="N17:O17"/>
+    <mergeCell ref="B14:Q15"/>
+    <mergeCell ref="B9:C9"/>
+    <mergeCell ref="B10:C11"/>
+    <mergeCell ref="E10:E11"/>
+    <mergeCell ref="R7:U7"/>
+    <mergeCell ref="B2:P3"/>
+    <mergeCell ref="B5:C5"/>
+    <mergeCell ref="E5:I5"/>
+    <mergeCell ref="K5:P5"/>
     <mergeCell ref="R2:U2"/>
     <mergeCell ref="B42:C42"/>
     <mergeCell ref="D42:E42"/>
@@ -2878,30 +2898,13 @@
     <mergeCell ref="R6:U6"/>
     <mergeCell ref="R5:U5"/>
     <mergeCell ref="R4:U4"/>
-    <mergeCell ref="R3:U3"/>
-    <mergeCell ref="B17:E17"/>
-    <mergeCell ref="G17:L17"/>
-    <mergeCell ref="N17:O17"/>
-    <mergeCell ref="B14:Q15"/>
-    <mergeCell ref="B9:C9"/>
-    <mergeCell ref="B10:C11"/>
-    <mergeCell ref="E10:E11"/>
-    <mergeCell ref="R7:U7"/>
-    <mergeCell ref="B2:P3"/>
-    <mergeCell ref="B5:C5"/>
-    <mergeCell ref="E5:I5"/>
-    <mergeCell ref="K5:P5"/>
-    <mergeCell ref="Q18:Q19"/>
-    <mergeCell ref="B21:C21"/>
-    <mergeCell ref="B22:C23"/>
-    <mergeCell ref="E22:E23"/>
-    <mergeCell ref="B26:Q27"/>
+    <mergeCell ref="B47:Q48"/>
+    <mergeCell ref="B50:H50"/>
+    <mergeCell ref="S34:V34"/>
+    <mergeCell ref="S35:V35"/>
+    <mergeCell ref="S36:V36"/>
+    <mergeCell ref="S37:V37"/>
     <mergeCell ref="B37:P37"/>
-    <mergeCell ref="D30:E30"/>
-    <mergeCell ref="B29:E29"/>
-    <mergeCell ref="D31:E31"/>
-    <mergeCell ref="G29:H29"/>
-    <mergeCell ref="B34:Q35"/>
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2940,60 +2943,60 @@
   <sheetData>
     <row r="1" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="2" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B2" s="55" t="s">
+      <c r="B2" s="77" t="s">
         <v>76</v>
       </c>
-      <c r="C2" s="56"/>
-      <c r="D2" s="56"/>
-      <c r="E2" s="56"/>
-      <c r="F2" s="56"/>
-      <c r="G2" s="56"/>
-      <c r="H2" s="56"/>
-      <c r="I2" s="56"/>
-      <c r="J2" s="56"/>
-      <c r="K2" s="56"/>
-      <c r="L2" s="56"/>
-      <c r="M2" s="56"/>
-      <c r="N2" s="56"/>
-      <c r="O2" s="56"/>
-      <c r="P2" s="57"/>
+      <c r="C2" s="78"/>
+      <c r="D2" s="78"/>
+      <c r="E2" s="78"/>
+      <c r="F2" s="78"/>
+      <c r="G2" s="78"/>
+      <c r="H2" s="78"/>
+      <c r="I2" s="78"/>
+      <c r="J2" s="78"/>
+      <c r="K2" s="78"/>
+      <c r="L2" s="78"/>
+      <c r="M2" s="78"/>
+      <c r="N2" s="78"/>
+      <c r="O2" s="78"/>
+      <c r="P2" s="79"/>
     </row>
     <row r="3" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B3" s="58"/>
-      <c r="C3" s="59"/>
-      <c r="D3" s="59"/>
-      <c r="E3" s="59"/>
-      <c r="F3" s="59"/>
-      <c r="G3" s="59"/>
-      <c r="H3" s="59"/>
-      <c r="I3" s="59"/>
-      <c r="J3" s="59"/>
-      <c r="K3" s="59"/>
-      <c r="L3" s="59"/>
-      <c r="M3" s="59"/>
-      <c r="N3" s="59"/>
-      <c r="O3" s="59"/>
-      <c r="P3" s="60"/>
+      <c r="B3" s="80"/>
+      <c r="C3" s="81"/>
+      <c r="D3" s="81"/>
+      <c r="E3" s="81"/>
+      <c r="F3" s="81"/>
+      <c r="G3" s="81"/>
+      <c r="H3" s="81"/>
+      <c r="I3" s="81"/>
+      <c r="J3" s="81"/>
+      <c r="K3" s="81"/>
+      <c r="L3" s="81"/>
+      <c r="M3" s="81"/>
+      <c r="N3" s="81"/>
+      <c r="O3" s="81"/>
+      <c r="P3" s="82"/>
       <c r="R3" s="12"/>
     </row>
     <row r="5" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B5" s="70" t="s">
+      <c r="B5" s="83" t="s">
         <v>83</v>
       </c>
-      <c r="C5" s="74"/>
-      <c r="D5" s="74"/>
-      <c r="E5" s="74"/>
-      <c r="F5" s="71"/>
-      <c r="H5" s="70" t="s">
+      <c r="C5" s="84"/>
+      <c r="D5" s="84"/>
+      <c r="E5" s="84"/>
+      <c r="F5" s="85"/>
+      <c r="H5" s="83" t="s">
         <v>82</v>
       </c>
-      <c r="I5" s="71"/>
-      <c r="K5" s="70" t="s">
+      <c r="I5" s="85"/>
+      <c r="K5" s="83" t="s">
         <v>8</v>
       </c>
-      <c r="L5" s="74"/>
-      <c r="M5" s="74"/>
-      <c r="N5" s="71"/>
+      <c r="L5" s="84"/>
+      <c r="M5" s="84"/>
+      <c r="N5" s="85"/>
       <c r="P5" s="4" t="s">
         <v>74</v>
       </c>
@@ -3075,10 +3078,10 @@
       </c>
     </row>
     <row r="9" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B9" s="63" t="s">
+      <c r="B9" s="69" t="s">
         <v>22</v>
       </c>
-      <c r="C9" s="63"/>
+      <c r="C9" s="69"/>
       <c r="E9" s="9" t="s">
         <v>67</v>
       </c>
@@ -3086,21 +3089,21 @@
       <c r="H9" s="11"/>
     </row>
     <row r="10" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B10" s="53">
+      <c r="B10" s="70">
         <f>SUM(B7:F7,H7:I7,K7:N7,P7)</f>
         <v>99.1</v>
       </c>
-      <c r="C10" s="53"/>
-      <c r="E10" s="64">
+      <c r="C10" s="70"/>
+      <c r="E10" s="71">
         <v>4</v>
       </c>
       <c r="G10" s="7"/>
       <c r="H10" s="7"/>
     </row>
     <row r="11" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B11" s="53"/>
-      <c r="C11" s="53"/>
-      <c r="E11" s="65"/>
+      <c r="B11" s="70"/>
+      <c r="C11" s="70"/>
+      <c r="E11" s="72"/>
       <c r="G11" s="7"/>
       <c r="H11" s="7"/>
     </row>
@@ -3127,42 +3130,42 @@
     </row>
     <row r="13" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="14" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B14" s="55" t="s">
+      <c r="B14" s="77" t="s">
         <v>77</v>
       </c>
-      <c r="C14" s="56"/>
-      <c r="D14" s="56"/>
-      <c r="E14" s="56"/>
-      <c r="F14" s="56"/>
-      <c r="G14" s="56"/>
-      <c r="H14" s="57"/>
+      <c r="C14" s="78"/>
+      <c r="D14" s="78"/>
+      <c r="E14" s="78"/>
+      <c r="F14" s="78"/>
+      <c r="G14" s="78"/>
+      <c r="H14" s="79"/>
     </row>
     <row r="15" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B15" s="58"/>
-      <c r="C15" s="59"/>
-      <c r="D15" s="59"/>
-      <c r="E15" s="59"/>
-      <c r="F15" s="59"/>
-      <c r="G15" s="59"/>
-      <c r="H15" s="60"/>
+      <c r="B15" s="80"/>
+      <c r="C15" s="81"/>
+      <c r="D15" s="81"/>
+      <c r="E15" s="81"/>
+      <c r="F15" s="81"/>
+      <c r="G15" s="81"/>
+      <c r="H15" s="82"/>
     </row>
     <row r="17" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B17" s="54" t="s">
+      <c r="B17" s="75" t="s">
         <v>90</v>
       </c>
-      <c r="C17" s="54"/>
-      <c r="D17" s="54"/>
-      <c r="E17" s="54"/>
-      <c r="F17" s="54"/>
-      <c r="H17" s="70" t="s">
+      <c r="C17" s="75"/>
+      <c r="D17" s="75"/>
+      <c r="E17" s="75"/>
+      <c r="F17" s="75"/>
+      <c r="H17" s="83" t="s">
         <v>96</v>
       </c>
-      <c r="I17" s="74"/>
-      <c r="J17" s="71"/>
-      <c r="L17" s="63" t="s">
+      <c r="I17" s="84"/>
+      <c r="J17" s="85"/>
+      <c r="L17" s="69" t="s">
         <v>22</v>
       </c>
-      <c r="M17" s="63"/>
+      <c r="M17" s="69"/>
       <c r="O17" s="9" t="s">
         <v>67</v>
       </c>
@@ -3193,12 +3196,12 @@
       <c r="J18" s="3" t="s">
         <v>94</v>
       </c>
-      <c r="L18" s="53">
+      <c r="L18" s="70">
         <f>SUM(B19:F19,H19:J19)</f>
         <v>85</v>
       </c>
-      <c r="M18" s="53"/>
-      <c r="O18" s="73">
+      <c r="M18" s="70"/>
+      <c r="O18" s="76">
         <v>4.5</v>
       </c>
     </row>
@@ -3227,9 +3230,9 @@
       <c r="J19" s="2">
         <v>19.5</v>
       </c>
-      <c r="L19" s="53"/>
-      <c r="M19" s="53"/>
-      <c r="O19" s="73"/>
+      <c r="L19" s="70"/>
+      <c r="M19" s="70"/>
+      <c r="O19" s="76"/>
     </row>
     <row r="21" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A21" s="6"/>
@@ -3254,62 +3257,62 @@
     </row>
     <row r="22" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="23" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B23" s="55" t="s">
+      <c r="B23" s="77" t="s">
         <v>79</v>
       </c>
-      <c r="C23" s="56"/>
-      <c r="D23" s="56"/>
-      <c r="E23" s="56"/>
-      <c r="F23" s="56"/>
-      <c r="G23" s="56"/>
-      <c r="H23" s="56"/>
-      <c r="I23" s="56"/>
-      <c r="J23" s="56"/>
-      <c r="K23" s="56"/>
-      <c r="L23" s="57"/>
-      <c r="N23" s="53" t="s">
+      <c r="C23" s="78"/>
+      <c r="D23" s="78"/>
+      <c r="E23" s="78"/>
+      <c r="F23" s="78"/>
+      <c r="G23" s="78"/>
+      <c r="H23" s="78"/>
+      <c r="I23" s="78"/>
+      <c r="J23" s="78"/>
+      <c r="K23" s="78"/>
+      <c r="L23" s="79"/>
+      <c r="N23" s="70" t="s">
         <v>214</v>
       </c>
-      <c r="O23" s="53"/>
+      <c r="O23" s="70"/>
       <c r="Q23" s="7"/>
       <c r="R23" s="7"/>
       <c r="S23" s="7"/>
     </row>
     <row r="24" spans="1:19" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B24" s="58"/>
-      <c r="C24" s="59"/>
-      <c r="D24" s="59"/>
-      <c r="E24" s="59"/>
-      <c r="F24" s="59"/>
-      <c r="G24" s="59"/>
-      <c r="H24" s="59"/>
-      <c r="I24" s="59"/>
-      <c r="J24" s="59"/>
-      <c r="K24" s="59"/>
-      <c r="L24" s="60"/>
-      <c r="N24" s="53"/>
-      <c r="O24" s="53"/>
+      <c r="B24" s="80"/>
+      <c r="C24" s="81"/>
+      <c r="D24" s="81"/>
+      <c r="E24" s="81"/>
+      <c r="F24" s="81"/>
+      <c r="G24" s="81"/>
+      <c r="H24" s="81"/>
+      <c r="I24" s="81"/>
+      <c r="J24" s="81"/>
+      <c r="K24" s="81"/>
+      <c r="L24" s="82"/>
+      <c r="N24" s="70"/>
+      <c r="O24" s="70"/>
       <c r="Q24" s="7"/>
       <c r="R24" s="7"/>
       <c r="S24" s="7"/>
     </row>
     <row r="26" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B26" s="54" t="s">
+      <c r="B26" s="75" t="s">
         <v>8</v>
       </c>
-      <c r="C26" s="54"/>
-      <c r="D26" s="54"/>
-      <c r="F26" s="54" t="s">
+      <c r="C26" s="75"/>
+      <c r="D26" s="75"/>
+      <c r="F26" s="75" t="s">
         <v>195</v>
       </c>
-      <c r="G26" s="54"/>
-      <c r="H26" s="54"/>
-      <c r="I26" s="54"/>
+      <c r="G26" s="75"/>
+      <c r="H26" s="75"/>
+      <c r="I26" s="75"/>
       <c r="J26" s="7"/>
-      <c r="K26" s="70" t="s">
+      <c r="K26" s="83" t="s">
         <v>116</v>
       </c>
-      <c r="L26" s="71"/>
+      <c r="L26" s="85"/>
       <c r="N26" s="9" t="s">
         <v>212</v>
       </c>
@@ -3345,11 +3348,11 @@
       <c r="L27" s="2" t="s">
         <v>115</v>
       </c>
-      <c r="N27" s="77">
+      <c r="N27" s="88">
         <f>(K29/30*0.4*5)+(B29/25*0.3*5)+(0.3*F29)</f>
         <v>4.9399999999999995</v>
       </c>
-      <c r="O27" s="73">
+      <c r="O27" s="76">
         <v>5</v>
       </c>
     </row>
@@ -3381,27 +3384,27 @@
       <c r="L28" s="2">
         <v>10</v>
       </c>
-      <c r="N28" s="78"/>
-      <c r="O28" s="73"/>
+      <c r="N28" s="89"/>
+      <c r="O28" s="76"/>
     </row>
     <row r="29" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B29" s="72">
+      <c r="B29" s="90">
         <f>SUM(B28:D28)</f>
         <v>24</v>
       </c>
-      <c r="C29" s="72"/>
-      <c r="D29" s="72"/>
-      <c r="F29" s="72">
+      <c r="C29" s="90"/>
+      <c r="D29" s="90"/>
+      <c r="F29" s="90">
         <v>5</v>
       </c>
-      <c r="G29" s="72"/>
-      <c r="H29" s="72"/>
-      <c r="I29" s="72"/>
-      <c r="K29" s="72">
+      <c r="G29" s="90"/>
+      <c r="H29" s="90"/>
+      <c r="I29" s="90"/>
+      <c r="K29" s="90">
         <f>SUM(K28:L28)</f>
         <v>30</v>
       </c>
-      <c r="L29" s="72"/>
+      <c r="L29" s="90"/>
       <c r="N29" s="34"/>
     </row>
     <row r="31" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -3427,38 +3430,38 @@
     </row>
     <row r="32" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="33" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B33" s="55" t="s">
+      <c r="B33" s="77" t="s">
         <v>78</v>
       </c>
-      <c r="C33" s="56"/>
-      <c r="D33" s="56"/>
-      <c r="E33" s="56"/>
-      <c r="F33" s="56"/>
-      <c r="G33" s="56"/>
-      <c r="H33" s="56"/>
-      <c r="I33" s="57"/>
+      <c r="C33" s="78"/>
+      <c r="D33" s="78"/>
+      <c r="E33" s="78"/>
+      <c r="F33" s="78"/>
+      <c r="G33" s="78"/>
+      <c r="H33" s="78"/>
+      <c r="I33" s="79"/>
     </row>
     <row r="34" spans="2:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B34" s="58"/>
-      <c r="C34" s="59"/>
-      <c r="D34" s="59"/>
-      <c r="E34" s="59"/>
-      <c r="F34" s="59"/>
-      <c r="G34" s="59"/>
-      <c r="H34" s="59"/>
-      <c r="I34" s="60"/>
+      <c r="B34" s="80"/>
+      <c r="C34" s="81"/>
+      <c r="D34" s="81"/>
+      <c r="E34" s="81"/>
+      <c r="F34" s="81"/>
+      <c r="G34" s="81"/>
+      <c r="H34" s="81"/>
+      <c r="I34" s="82"/>
     </row>
     <row r="36" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B36" s="54" t="s">
+      <c r="B36" s="75" t="s">
         <v>97</v>
       </c>
-      <c r="C36" s="54"/>
+      <c r="C36" s="75"/>
       <c r="D36" s="7"/>
-      <c r="E36" s="54" t="s">
+      <c r="E36" s="75" t="s">
         <v>131</v>
       </c>
-      <c r="F36" s="54"/>
-      <c r="G36" s="54"/>
+      <c r="F36" s="75"/>
+      <c r="G36" s="75"/>
       <c r="H36" s="7"/>
     </row>
     <row r="37" spans="2:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -3500,14 +3503,14 @@
       <c r="O38" s="7"/>
     </row>
     <row r="41" spans="2:15" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B41" s="75" t="s">
+      <c r="B41" s="86" t="s">
         <v>114</v>
       </c>
-      <c r="C41" s="76"/>
-      <c r="F41" s="53" t="s">
+      <c r="C41" s="87"/>
+      <c r="F41" s="70" t="s">
         <v>99</v>
       </c>
-      <c r="G41" s="53"/>
+      <c r="G41" s="70"/>
       <c r="I41" s="9" t="s">
         <v>22</v>
       </c>
@@ -3563,7 +3566,7 @@
       <c r="G44" s="2">
         <v>10</v>
       </c>
-      <c r="I44" s="63" t="s">
+      <c r="I44" s="69" t="s">
         <v>67</v>
       </c>
     </row>
@@ -3574,7 +3577,7 @@
       <c r="C45" s="2">
         <v>4</v>
       </c>
-      <c r="I45" s="63"/>
+      <c r="I45" s="69"/>
     </row>
     <row r="46" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B46" s="2" t="s">
@@ -3671,70 +3674,70 @@
     </row>
     <row r="57" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="58" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B58" s="55" t="s">
+      <c r="B58" s="77" t="s">
         <v>80</v>
       </c>
-      <c r="C58" s="56"/>
-      <c r="D58" s="56"/>
-      <c r="E58" s="56"/>
-      <c r="F58" s="56"/>
-      <c r="G58" s="56"/>
-      <c r="H58" s="56"/>
-      <c r="I58" s="56"/>
-      <c r="J58" s="56"/>
-      <c r="K58" s="56"/>
-      <c r="L58" s="56"/>
-      <c r="M58" s="56"/>
-      <c r="N58" s="56"/>
-      <c r="O58" s="56"/>
-      <c r="P58" s="56"/>
-      <c r="Q58" s="56"/>
-      <c r="R58" s="56"/>
-      <c r="S58" s="57"/>
+      <c r="C58" s="78"/>
+      <c r="D58" s="78"/>
+      <c r="E58" s="78"/>
+      <c r="F58" s="78"/>
+      <c r="G58" s="78"/>
+      <c r="H58" s="78"/>
+      <c r="I58" s="78"/>
+      <c r="J58" s="78"/>
+      <c r="K58" s="78"/>
+      <c r="L58" s="78"/>
+      <c r="M58" s="78"/>
+      <c r="N58" s="78"/>
+      <c r="O58" s="78"/>
+      <c r="P58" s="78"/>
+      <c r="Q58" s="78"/>
+      <c r="R58" s="78"/>
+      <c r="S58" s="79"/>
     </row>
     <row r="59" spans="1:19" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B59" s="58"/>
-      <c r="C59" s="59"/>
-      <c r="D59" s="59"/>
-      <c r="E59" s="59"/>
-      <c r="F59" s="59"/>
-      <c r="G59" s="59"/>
-      <c r="H59" s="59"/>
-      <c r="I59" s="59"/>
-      <c r="J59" s="59"/>
-      <c r="K59" s="59"/>
-      <c r="L59" s="59"/>
-      <c r="M59" s="59"/>
-      <c r="N59" s="59"/>
-      <c r="O59" s="59"/>
-      <c r="P59" s="59"/>
-      <c r="Q59" s="59"/>
-      <c r="R59" s="59"/>
-      <c r="S59" s="60"/>
+      <c r="B59" s="80"/>
+      <c r="C59" s="81"/>
+      <c r="D59" s="81"/>
+      <c r="E59" s="81"/>
+      <c r="F59" s="81"/>
+      <c r="G59" s="81"/>
+      <c r="H59" s="81"/>
+      <c r="I59" s="81"/>
+      <c r="J59" s="81"/>
+      <c r="K59" s="81"/>
+      <c r="L59" s="81"/>
+      <c r="M59" s="81"/>
+      <c r="N59" s="81"/>
+      <c r="O59" s="81"/>
+      <c r="P59" s="81"/>
+      <c r="Q59" s="81"/>
+      <c r="R59" s="81"/>
+      <c r="S59" s="82"/>
     </row>
     <row r="61" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B61" s="54" t="s">
+      <c r="B61" s="75" t="s">
         <v>63</v>
       </c>
-      <c r="C61" s="54"/>
-      <c r="D61" s="54"/>
-      <c r="E61" s="54"/>
-      <c r="F61" s="54"/>
-      <c r="G61" s="54"/>
-      <c r="H61" s="54"/>
-      <c r="I61" s="54"/>
-      <c r="J61" s="54"/>
-      <c r="K61" s="54"/>
-      <c r="M61" s="54" t="s">
+      <c r="C61" s="75"/>
+      <c r="D61" s="75"/>
+      <c r="E61" s="75"/>
+      <c r="F61" s="75"/>
+      <c r="G61" s="75"/>
+      <c r="H61" s="75"/>
+      <c r="I61" s="75"/>
+      <c r="J61" s="75"/>
+      <c r="K61" s="75"/>
+      <c r="M61" s="75" t="s">
         <v>89</v>
       </c>
-      <c r="N61" s="54"/>
-      <c r="O61" s="54"/>
-      <c r="P61" s="54"/>
-      <c r="R61" s="54" t="s">
+      <c r="N61" s="75"/>
+      <c r="O61" s="75"/>
+      <c r="P61" s="75"/>
+      <c r="R61" s="75" t="s">
         <v>64</v>
       </c>
-      <c r="S61" s="54"/>
+      <c r="S61" s="75"/>
     </row>
     <row r="62" spans="1:19" x14ac:dyDescent="0.25">
       <c r="B62" s="2" t="s">
@@ -3837,10 +3840,10 @@
       </c>
     </row>
     <row r="66" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B66" s="63" t="s">
+      <c r="B66" s="69" t="s">
         <v>22</v>
       </c>
-      <c r="C66" s="63"/>
+      <c r="C66" s="69"/>
       <c r="E66" s="9" t="s">
         <v>67</v>
       </c>
@@ -3850,28 +3853,49 @@
       <c r="H66" s="11"/>
     </row>
     <row r="67" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B67" s="53">
+      <c r="B67" s="70">
         <f>_xlfn.CEILING.MATH(SUM(B63:K63,M63:P63,R63:S63,G67))</f>
         <v>98</v>
       </c>
-      <c r="C67" s="53"/>
-      <c r="E67" s="73">
+      <c r="C67" s="70"/>
+      <c r="E67" s="76">
         <v>5</v>
       </c>
-      <c r="G67" s="53">
+      <c r="G67" s="70">
         <v>9</v>
       </c>
       <c r="H67" s="7"/>
     </row>
     <row r="68" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B68" s="53"/>
-      <c r="C68" s="53"/>
-      <c r="E68" s="73"/>
-      <c r="G68" s="53"/>
+      <c r="B68" s="70"/>
+      <c r="C68" s="70"/>
+      <c r="E68" s="76"/>
+      <c r="G68" s="70"/>
       <c r="H68" s="7"/>
     </row>
   </sheetData>
   <mergeCells count="37">
+    <mergeCell ref="K26:L26"/>
+    <mergeCell ref="B23:L24"/>
+    <mergeCell ref="B26:D26"/>
+    <mergeCell ref="K29:L29"/>
+    <mergeCell ref="R61:S61"/>
+    <mergeCell ref="B33:I34"/>
+    <mergeCell ref="B61:K61"/>
+    <mergeCell ref="B58:S59"/>
+    <mergeCell ref="M61:P61"/>
+    <mergeCell ref="F29:I29"/>
+    <mergeCell ref="B29:D29"/>
+    <mergeCell ref="E36:G36"/>
+    <mergeCell ref="B66:C66"/>
+    <mergeCell ref="B67:C68"/>
+    <mergeCell ref="B9:C9"/>
+    <mergeCell ref="B10:C11"/>
+    <mergeCell ref="G67:G68"/>
+    <mergeCell ref="E67:E68"/>
+    <mergeCell ref="E10:E11"/>
+    <mergeCell ref="B17:F17"/>
+    <mergeCell ref="F26:I26"/>
     <mergeCell ref="O18:O19"/>
     <mergeCell ref="B14:H15"/>
     <mergeCell ref="K5:N5"/>
@@ -3888,27 +3912,6 @@
     <mergeCell ref="N27:N28"/>
     <mergeCell ref="O27:O28"/>
     <mergeCell ref="H17:J17"/>
-    <mergeCell ref="B66:C66"/>
-    <mergeCell ref="B67:C68"/>
-    <mergeCell ref="B9:C9"/>
-    <mergeCell ref="B10:C11"/>
-    <mergeCell ref="G67:G68"/>
-    <mergeCell ref="E67:E68"/>
-    <mergeCell ref="E10:E11"/>
-    <mergeCell ref="B17:F17"/>
-    <mergeCell ref="F26:I26"/>
-    <mergeCell ref="K26:L26"/>
-    <mergeCell ref="B23:L24"/>
-    <mergeCell ref="B26:D26"/>
-    <mergeCell ref="K29:L29"/>
-    <mergeCell ref="R61:S61"/>
-    <mergeCell ref="B33:I34"/>
-    <mergeCell ref="B61:K61"/>
-    <mergeCell ref="B58:S59"/>
-    <mergeCell ref="M61:P61"/>
-    <mergeCell ref="F29:I29"/>
-    <mergeCell ref="B29:D29"/>
-    <mergeCell ref="E36:G36"/>
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -3947,60 +3950,60 @@
   <sheetData>
     <row r="1" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="2" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B2" s="55" t="s">
+      <c r="B2" s="77" t="s">
         <v>117</v>
       </c>
-      <c r="C2" s="56"/>
-      <c r="D2" s="56"/>
-      <c r="E2" s="56"/>
-      <c r="F2" s="56"/>
-      <c r="G2" s="56"/>
-      <c r="H2" s="56"/>
-      <c r="I2" s="56"/>
-      <c r="J2" s="56"/>
-      <c r="K2" s="56"/>
-      <c r="L2" s="56"/>
-      <c r="M2" s="56"/>
-      <c r="N2" s="56"/>
-      <c r="O2" s="56"/>
-      <c r="P2" s="57"/>
+      <c r="C2" s="78"/>
+      <c r="D2" s="78"/>
+      <c r="E2" s="78"/>
+      <c r="F2" s="78"/>
+      <c r="G2" s="78"/>
+      <c r="H2" s="78"/>
+      <c r="I2" s="78"/>
+      <c r="J2" s="78"/>
+      <c r="K2" s="78"/>
+      <c r="L2" s="78"/>
+      <c r="M2" s="78"/>
+      <c r="N2" s="78"/>
+      <c r="O2" s="78"/>
+      <c r="P2" s="79"/>
     </row>
     <row r="3" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B3" s="58"/>
-      <c r="C3" s="59"/>
-      <c r="D3" s="59"/>
-      <c r="E3" s="59"/>
-      <c r="F3" s="59"/>
-      <c r="G3" s="59"/>
-      <c r="H3" s="59"/>
-      <c r="I3" s="59"/>
-      <c r="J3" s="59"/>
-      <c r="K3" s="59"/>
-      <c r="L3" s="59"/>
-      <c r="M3" s="59"/>
-      <c r="N3" s="59"/>
-      <c r="O3" s="59"/>
-      <c r="P3" s="60"/>
+      <c r="B3" s="80"/>
+      <c r="C3" s="81"/>
+      <c r="D3" s="81"/>
+      <c r="E3" s="81"/>
+      <c r="F3" s="81"/>
+      <c r="G3" s="81"/>
+      <c r="H3" s="81"/>
+      <c r="I3" s="81"/>
+      <c r="J3" s="81"/>
+      <c r="K3" s="81"/>
+      <c r="L3" s="81"/>
+      <c r="M3" s="81"/>
+      <c r="N3" s="81"/>
+      <c r="O3" s="81"/>
+      <c r="P3" s="82"/>
       <c r="R3" s="12"/>
     </row>
     <row r="5" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B5" s="54" t="s">
+      <c r="B5" s="75" t="s">
         <v>18</v>
       </c>
-      <c r="C5" s="54"/>
-      <c r="D5" s="54"/>
-      <c r="E5" s="54"/>
-      <c r="F5" s="54"/>
-      <c r="G5" s="54"/>
+      <c r="C5" s="75"/>
+      <c r="D5" s="75"/>
+      <c r="E5" s="75"/>
+      <c r="F5" s="75"/>
+      <c r="G5" s="75"/>
       <c r="I5" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="K5" s="70" t="s">
+      <c r="K5" s="83" t="s">
         <v>8</v>
       </c>
-      <c r="L5" s="74"/>
-      <c r="M5" s="74"/>
-      <c r="N5" s="71"/>
+      <c r="L5" s="84"/>
+      <c r="M5" s="84"/>
+      <c r="N5" s="85"/>
       <c r="P5" s="4" t="s">
         <v>74</v>
       </c>
@@ -4082,28 +4085,28 @@
       </c>
     </row>
     <row r="9" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B9" s="63" t="s">
+      <c r="B9" s="69" t="s">
         <v>22</v>
       </c>
-      <c r="C9" s="63"/>
+      <c r="C9" s="69"/>
       <c r="E9" s="9" t="s">
         <v>67</v>
       </c>
     </row>
     <row r="10" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B10" s="53">
+      <c r="B10" s="70">
         <f>_xlfn.CEILING.MATH(SUM(B7:G7,I7,K7:N7,P7),1,1)</f>
         <v>110</v>
       </c>
-      <c r="C10" s="53"/>
-      <c r="E10" s="64">
+      <c r="C10" s="70"/>
+      <c r="E10" s="71">
         <v>4</v>
       </c>
     </row>
     <row r="11" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B11" s="53"/>
-      <c r="C11" s="53"/>
-      <c r="E11" s="65"/>
+      <c r="B11" s="70"/>
+      <c r="C11" s="70"/>
+      <c r="E11" s="72"/>
     </row>
     <row r="12" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A12" s="6"/>
@@ -4128,40 +4131,40 @@
     </row>
     <row r="13" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="14" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B14" s="55" t="s">
+      <c r="B14" s="77" t="s">
         <v>118</v>
       </c>
-      <c r="C14" s="56"/>
-      <c r="D14" s="56"/>
-      <c r="E14" s="56"/>
-      <c r="F14" s="56"/>
-      <c r="G14" s="56"/>
-      <c r="H14" s="57"/>
+      <c r="C14" s="78"/>
+      <c r="D14" s="78"/>
+      <c r="E14" s="78"/>
+      <c r="F14" s="78"/>
+      <c r="G14" s="78"/>
+      <c r="H14" s="79"/>
     </row>
     <row r="15" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B15" s="58"/>
-      <c r="C15" s="59"/>
-      <c r="D15" s="59"/>
-      <c r="E15" s="59"/>
-      <c r="F15" s="59"/>
-      <c r="G15" s="59"/>
-      <c r="H15" s="60"/>
+      <c r="B15" s="80"/>
+      <c r="C15" s="81"/>
+      <c r="D15" s="81"/>
+      <c r="E15" s="81"/>
+      <c r="F15" s="81"/>
+      <c r="G15" s="81"/>
+      <c r="H15" s="82"/>
     </row>
     <row r="17" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B17" s="54" t="s">
+      <c r="B17" s="75" t="s">
         <v>12</v>
       </c>
-      <c r="C17" s="54"/>
-      <c r="D17" s="54"/>
-      <c r="F17" s="54" t="s">
+      <c r="C17" s="75"/>
+      <c r="D17" s="75"/>
+      <c r="F17" s="75" t="s">
         <v>8</v>
       </c>
-      <c r="G17" s="54"/>
-      <c r="H17" s="54"/>
-      <c r="J17" s="63" t="s">
+      <c r="G17" s="75"/>
+      <c r="H17" s="75"/>
+      <c r="J17" s="69" t="s">
         <v>22</v>
       </c>
-      <c r="K17" s="63"/>
+      <c r="K17" s="69"/>
       <c r="M17" s="9" t="s">
         <v>67</v>
       </c>
@@ -4185,12 +4188,12 @@
       <c r="H18" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="J18" s="53">
+      <c r="J18" s="70">
         <f>SUM(B19:D19,F19:H19)</f>
         <v>93</v>
       </c>
-      <c r="K18" s="53"/>
-      <c r="M18" s="73">
+      <c r="K18" s="70"/>
+      <c r="M18" s="76">
         <v>5</v>
       </c>
     </row>
@@ -4213,9 +4216,9 @@
       <c r="H19" s="2">
         <v>4</v>
       </c>
-      <c r="J19" s="53"/>
-      <c r="K19" s="53"/>
-      <c r="M19" s="73"/>
+      <c r="J19" s="70"/>
+      <c r="K19" s="70"/>
+      <c r="M19" s="76"/>
     </row>
     <row r="21" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A21" s="6"/>
@@ -4240,46 +4243,46 @@
     </row>
     <row r="22" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="23" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B23" s="55" t="s">
+      <c r="B23" s="77" t="s">
         <v>119</v>
       </c>
-      <c r="C23" s="56"/>
-      <c r="D23" s="56"/>
-      <c r="E23" s="56"/>
-      <c r="F23" s="56"/>
-      <c r="G23" s="56"/>
-      <c r="H23" s="56"/>
-      <c r="I23" s="56"/>
-      <c r="J23" s="56"/>
-      <c r="K23" s="57"/>
+      <c r="C23" s="78"/>
+      <c r="D23" s="78"/>
+      <c r="E23" s="78"/>
+      <c r="F23" s="78"/>
+      <c r="G23" s="78"/>
+      <c r="H23" s="78"/>
+      <c r="I23" s="78"/>
+      <c r="J23" s="78"/>
+      <c r="K23" s="79"/>
     </row>
     <row r="24" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B24" s="58"/>
-      <c r="C24" s="59"/>
-      <c r="D24" s="59"/>
-      <c r="E24" s="59"/>
-      <c r="F24" s="59"/>
-      <c r="G24" s="59"/>
-      <c r="H24" s="59"/>
-      <c r="I24" s="59"/>
-      <c r="J24" s="59"/>
-      <c r="K24" s="60"/>
+      <c r="B24" s="80"/>
+      <c r="C24" s="81"/>
+      <c r="D24" s="81"/>
+      <c r="E24" s="81"/>
+      <c r="F24" s="81"/>
+      <c r="G24" s="81"/>
+      <c r="H24" s="81"/>
+      <c r="I24" s="81"/>
+      <c r="J24" s="81"/>
+      <c r="K24" s="82"/>
     </row>
     <row r="26" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B26" s="54" t="s">
+      <c r="B26" s="75" t="s">
         <v>17</v>
       </c>
-      <c r="C26" s="54"/>
-      <c r="E26" s="70" t="s">
+      <c r="C26" s="75"/>
+      <c r="E26" s="83" t="s">
         <v>21</v>
       </c>
-      <c r="F26" s="74"/>
-      <c r="G26" s="71"/>
-      <c r="I26" s="54" t="s">
+      <c r="F26" s="84"/>
+      <c r="G26" s="85"/>
+      <c r="I26" s="75" t="s">
         <v>20</v>
       </c>
-      <c r="J26" s="54"/>
-      <c r="K26" s="54"/>
+      <c r="J26" s="75"/>
+      <c r="K26" s="75"/>
       <c r="M26" s="10" t="s">
         <v>22</v>
       </c>
@@ -4314,12 +4317,12 @@
       <c r="K27" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="M27" s="79">
+      <c r="M27" s="91">
         <f>SUM(B28:C28,E28:G28,I28:K28)</f>
         <v>36</v>
       </c>
       <c r="N27" s="7"/>
-      <c r="O27" s="73">
+      <c r="O27" s="76">
         <v>4</v>
       </c>
       <c r="P27" s="8"/>
@@ -4349,9 +4352,9 @@
       <c r="K28" s="2">
         <v>3.2</v>
       </c>
-      <c r="M28" s="79"/>
+      <c r="M28" s="91"/>
       <c r="N28" s="7"/>
-      <c r="O28" s="73"/>
+      <c r="O28" s="76"/>
       <c r="P28" s="8"/>
     </row>
     <row r="30" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -4377,39 +4380,39 @@
     </row>
     <row r="31" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="32" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B32" s="55" t="s">
+      <c r="B32" s="77" t="s">
         <v>120</v>
       </c>
-      <c r="C32" s="56"/>
-      <c r="D32" s="56"/>
-      <c r="E32" s="56"/>
-      <c r="F32" s="56"/>
-      <c r="G32" s="56"/>
-      <c r="H32" s="56"/>
-      <c r="I32" s="57"/>
+      <c r="C32" s="78"/>
+      <c r="D32" s="78"/>
+      <c r="E32" s="78"/>
+      <c r="F32" s="78"/>
+      <c r="G32" s="78"/>
+      <c r="H32" s="78"/>
+      <c r="I32" s="79"/>
     </row>
     <row r="33" spans="2:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B33" s="58"/>
-      <c r="C33" s="59"/>
-      <c r="D33" s="59"/>
-      <c r="E33" s="59"/>
-      <c r="F33" s="59"/>
-      <c r="G33" s="59"/>
-      <c r="H33" s="59"/>
-      <c r="I33" s="60"/>
+      <c r="B33" s="80"/>
+      <c r="C33" s="81"/>
+      <c r="D33" s="81"/>
+      <c r="E33" s="81"/>
+      <c r="F33" s="81"/>
+      <c r="G33" s="81"/>
+      <c r="H33" s="81"/>
+      <c r="I33" s="82"/>
     </row>
     <row r="35" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B35" s="54" t="s">
+      <c r="B35" s="75" t="s">
         <v>31</v>
       </c>
-      <c r="C35" s="54"/>
-      <c r="D35" s="54"/>
-      <c r="F35" s="54" t="s">
+      <c r="C35" s="75"/>
+      <c r="D35" s="75"/>
+      <c r="F35" s="75" t="s">
         <v>12</v>
       </c>
-      <c r="G35" s="54"/>
-      <c r="H35" s="54"/>
-      <c r="I35" s="54"/>
+      <c r="G35" s="75"/>
+      <c r="H35" s="75"/>
+      <c r="I35" s="75"/>
       <c r="N35" s="7"/>
       <c r="O35" s="7"/>
     </row>
@@ -4466,14 +4469,14 @@
       <c r="O37" s="7"/>
     </row>
     <row r="40" spans="2:15" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B40" s="75" t="s">
+      <c r="B40" s="86" t="s">
         <v>35</v>
       </c>
-      <c r="C40" s="76"/>
-      <c r="F40" s="53" t="s">
+      <c r="C40" s="87"/>
+      <c r="F40" s="70" t="s">
         <v>36</v>
       </c>
-      <c r="G40" s="53"/>
+      <c r="G40" s="70"/>
       <c r="I40" s="9" t="s">
         <v>22</v>
       </c>
@@ -4529,7 +4532,7 @@
       <c r="G43" s="2">
         <v>0.44</v>
       </c>
-      <c r="I43" s="63" t="s">
+      <c r="I43" s="69" t="s">
         <v>67</v>
       </c>
     </row>
@@ -4546,7 +4549,7 @@
       <c r="G44" s="2">
         <v>1</v>
       </c>
-      <c r="I44" s="63"/>
+      <c r="I44" s="69"/>
     </row>
     <row r="45" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B45" s="2" t="s">
@@ -4690,67 +4693,67 @@
     </row>
     <row r="57" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="58" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B58" s="55" t="s">
+      <c r="B58" s="77" t="s">
         <v>121</v>
       </c>
-      <c r="C58" s="56"/>
-      <c r="D58" s="56"/>
-      <c r="E58" s="56"/>
-      <c r="F58" s="56"/>
-      <c r="G58" s="56"/>
-      <c r="H58" s="56"/>
-      <c r="I58" s="56"/>
-      <c r="J58" s="56"/>
-      <c r="K58" s="56"/>
-      <c r="L58" s="56"/>
-      <c r="M58" s="56"/>
-      <c r="N58" s="56"/>
-      <c r="O58" s="56"/>
-      <c r="P58" s="56"/>
-      <c r="Q58" s="56"/>
-      <c r="R58" s="57"/>
+      <c r="C58" s="78"/>
+      <c r="D58" s="78"/>
+      <c r="E58" s="78"/>
+      <c r="F58" s="78"/>
+      <c r="G58" s="78"/>
+      <c r="H58" s="78"/>
+      <c r="I58" s="78"/>
+      <c r="J58" s="78"/>
+      <c r="K58" s="78"/>
+      <c r="L58" s="78"/>
+      <c r="M58" s="78"/>
+      <c r="N58" s="78"/>
+      <c r="O58" s="78"/>
+      <c r="P58" s="78"/>
+      <c r="Q58" s="78"/>
+      <c r="R58" s="79"/>
     </row>
     <row r="59" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B59" s="58"/>
-      <c r="C59" s="59"/>
-      <c r="D59" s="59"/>
-      <c r="E59" s="59"/>
-      <c r="F59" s="59"/>
-      <c r="G59" s="59"/>
-      <c r="H59" s="59"/>
-      <c r="I59" s="59"/>
-      <c r="J59" s="59"/>
-      <c r="K59" s="59"/>
-      <c r="L59" s="59"/>
-      <c r="M59" s="59"/>
-      <c r="N59" s="59"/>
-      <c r="O59" s="59"/>
-      <c r="P59" s="59"/>
-      <c r="Q59" s="59"/>
-      <c r="R59" s="60"/>
+      <c r="B59" s="80"/>
+      <c r="C59" s="81"/>
+      <c r="D59" s="81"/>
+      <c r="E59" s="81"/>
+      <c r="F59" s="81"/>
+      <c r="G59" s="81"/>
+      <c r="H59" s="81"/>
+      <c r="I59" s="81"/>
+      <c r="J59" s="81"/>
+      <c r="K59" s="81"/>
+      <c r="L59" s="81"/>
+      <c r="M59" s="81"/>
+      <c r="N59" s="81"/>
+      <c r="O59" s="81"/>
+      <c r="P59" s="81"/>
+      <c r="Q59" s="81"/>
+      <c r="R59" s="82"/>
     </row>
     <row r="61" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B61" s="54" t="s">
+      <c r="B61" s="75" t="s">
         <v>63</v>
       </c>
-      <c r="C61" s="54"/>
-      <c r="D61" s="54"/>
-      <c r="E61" s="54"/>
-      <c r="F61" s="54"/>
-      <c r="G61" s="54"/>
-      <c r="H61" s="54"/>
-      <c r="I61" s="54"/>
-      <c r="J61" s="54"/>
-      <c r="K61" s="54"/>
-      <c r="M61" s="54" t="s">
+      <c r="C61" s="75"/>
+      <c r="D61" s="75"/>
+      <c r="E61" s="75"/>
+      <c r="F61" s="75"/>
+      <c r="G61" s="75"/>
+      <c r="H61" s="75"/>
+      <c r="I61" s="75"/>
+      <c r="J61" s="75"/>
+      <c r="K61" s="75"/>
+      <c r="M61" s="75" t="s">
         <v>68</v>
       </c>
-      <c r="N61" s="54"/>
-      <c r="O61" s="54"/>
-      <c r="Q61" s="54" t="s">
+      <c r="N61" s="75"/>
+      <c r="O61" s="75"/>
+      <c r="Q61" s="75" t="s">
         <v>64</v>
       </c>
-      <c r="R61" s="54"/>
+      <c r="R61" s="75"/>
     </row>
     <row r="62" spans="1:19" x14ac:dyDescent="0.25">
       <c r="B62" s="2" t="s">
@@ -4847,28 +4850,28 @@
       </c>
     </row>
     <row r="66" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B66" s="63" t="s">
+      <c r="B66" s="69" t="s">
         <v>22</v>
       </c>
-      <c r="C66" s="63"/>
+      <c r="C66" s="69"/>
       <c r="E66" s="9" t="s">
         <v>67</v>
       </c>
     </row>
     <row r="67" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B67" s="53">
+      <c r="B67" s="70">
         <f xml:space="preserve"> SUM(B63:K63,M63:O63,Q63:R63)</f>
         <v>85.5</v>
       </c>
-      <c r="C67" s="53"/>
-      <c r="E67" s="73">
+      <c r="C67" s="70"/>
+      <c r="E67" s="76">
         <v>4.5</v>
       </c>
     </row>
     <row r="68" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B68" s="53"/>
-      <c r="C68" s="53"/>
-      <c r="E68" s="73"/>
+      <c r="B68" s="70"/>
+      <c r="C68" s="70"/>
+      <c r="E68" s="76"/>
     </row>
     <row r="70" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A70" s="6"/>
@@ -4893,26 +4896,26 @@
     </row>
     <row r="71" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="72" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B72" s="55" t="s">
+      <c r="B72" s="77" t="s">
         <v>122</v>
       </c>
-      <c r="C72" s="56"/>
-      <c r="D72" s="56"/>
-      <c r="E72" s="56"/>
-      <c r="F72" s="56"/>
-      <c r="G72" s="56"/>
-      <c r="H72" s="56"/>
-      <c r="I72" s="57"/>
+      <c r="C72" s="78"/>
+      <c r="D72" s="78"/>
+      <c r="E72" s="78"/>
+      <c r="F72" s="78"/>
+      <c r="G72" s="78"/>
+      <c r="H72" s="78"/>
+      <c r="I72" s="79"/>
     </row>
     <row r="73" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B73" s="58"/>
-      <c r="C73" s="59"/>
-      <c r="D73" s="59"/>
-      <c r="E73" s="59"/>
-      <c r="F73" s="59"/>
-      <c r="G73" s="59"/>
-      <c r="H73" s="59"/>
-      <c r="I73" s="60"/>
+      <c r="B73" s="80"/>
+      <c r="C73" s="81"/>
+      <c r="D73" s="81"/>
+      <c r="E73" s="81"/>
+      <c r="F73" s="81"/>
+      <c r="G73" s="81"/>
+      <c r="H73" s="81"/>
+      <c r="I73" s="82"/>
     </row>
     <row r="75" spans="1:19" x14ac:dyDescent="0.25">
       <c r="B75" s="4" t="s">
@@ -4939,10 +4942,10 @@
       <c r="I75" s="4" t="s">
         <v>130</v>
       </c>
-      <c r="K75" s="63" t="s">
+      <c r="K75" s="69" t="s">
         <v>22</v>
       </c>
-      <c r="L75" s="63"/>
+      <c r="L75" s="69"/>
       <c r="N75" s="9" t="s">
         <v>67</v>
       </c>
@@ -4972,11 +4975,11 @@
       <c r="I76" s="2">
         <v>5</v>
       </c>
-      <c r="K76" s="53">
+      <c r="K76" s="70">
         <f>SUM(B76:I76)</f>
         <v>96</v>
       </c>
-      <c r="L76" s="53"/>
+      <c r="L76" s="70"/>
       <c r="N76" s="13">
         <v>5</v>
       </c>
@@ -5004,20 +5007,16 @@
     </row>
   </sheetData>
   <mergeCells count="34">
-    <mergeCell ref="B2:P3"/>
-    <mergeCell ref="B5:G5"/>
-    <mergeCell ref="K5:N5"/>
-    <mergeCell ref="B9:C9"/>
-    <mergeCell ref="B10:C11"/>
-    <mergeCell ref="E10:E11"/>
-    <mergeCell ref="M27:M28"/>
-    <mergeCell ref="O27:O28"/>
-    <mergeCell ref="B14:H15"/>
-    <mergeCell ref="B17:D17"/>
-    <mergeCell ref="F17:H17"/>
-    <mergeCell ref="J17:K17"/>
-    <mergeCell ref="J18:K19"/>
-    <mergeCell ref="M18:M19"/>
+    <mergeCell ref="B72:I73"/>
+    <mergeCell ref="K75:L75"/>
+    <mergeCell ref="K76:L76"/>
+    <mergeCell ref="B58:R59"/>
+    <mergeCell ref="B61:K61"/>
+    <mergeCell ref="M61:O61"/>
+    <mergeCell ref="Q61:R61"/>
+    <mergeCell ref="B66:C66"/>
+    <mergeCell ref="B67:C68"/>
+    <mergeCell ref="E67:E68"/>
     <mergeCell ref="I43:I44"/>
     <mergeCell ref="B23:K24"/>
     <mergeCell ref="B26:C26"/>
@@ -5028,16 +5027,20 @@
     <mergeCell ref="F35:I35"/>
     <mergeCell ref="B40:C40"/>
     <mergeCell ref="F40:G40"/>
-    <mergeCell ref="B72:I73"/>
-    <mergeCell ref="K75:L75"/>
-    <mergeCell ref="K76:L76"/>
-    <mergeCell ref="B58:R59"/>
-    <mergeCell ref="B61:K61"/>
-    <mergeCell ref="M61:O61"/>
-    <mergeCell ref="Q61:R61"/>
-    <mergeCell ref="B66:C66"/>
-    <mergeCell ref="B67:C68"/>
-    <mergeCell ref="E67:E68"/>
+    <mergeCell ref="M27:M28"/>
+    <mergeCell ref="O27:O28"/>
+    <mergeCell ref="B14:H15"/>
+    <mergeCell ref="B17:D17"/>
+    <mergeCell ref="F17:H17"/>
+    <mergeCell ref="J17:K17"/>
+    <mergeCell ref="J18:K19"/>
+    <mergeCell ref="M18:M19"/>
+    <mergeCell ref="B2:P3"/>
+    <mergeCell ref="B5:G5"/>
+    <mergeCell ref="K5:N5"/>
+    <mergeCell ref="B9:C9"/>
+    <mergeCell ref="B10:C11"/>
+    <mergeCell ref="E10:E11"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
@@ -5634,7 +5637,7 @@
   <sheetPr>
     <tabColor theme="0" tint="-0.14999847407452621"/>
   </sheetPr>
-  <dimension ref="B1:H22"/>
+  <dimension ref="B1:H24"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="3" max="3" width="10.140625" bestFit="1" customWidth="1"/>
@@ -5650,19 +5653,19 @@
       <c r="C2" s="15" t="s">
         <v>132</v>
       </c>
-      <c r="D2" s="97" t="s">
+      <c r="D2" s="56" t="s">
         <v>133</v>
       </c>
-      <c r="E2" s="97" t="s">
+      <c r="E2" s="56" t="s">
         <v>167</v>
       </c>
-      <c r="F2" s="97" t="s">
+      <c r="F2" s="56" t="s">
         <v>179</v>
       </c>
-      <c r="G2" s="97" t="s">
+      <c r="G2" s="56" t="s">
         <v>245</v>
       </c>
-      <c r="H2" s="97" t="s">
+      <c r="H2" s="56" t="s">
         <v>253</v>
       </c>
     </row>
@@ -5670,13 +5673,13 @@
       <c r="B3" s="43" t="b">
         <v>1</v>
       </c>
-      <c r="C3" s="94" t="s">
+      <c r="C3" s="53" t="s">
         <v>185</v>
       </c>
-      <c r="D3" s="95" t="s">
+      <c r="D3" s="54" t="s">
         <v>251</v>
       </c>
-      <c r="E3" s="96" t="s">
+      <c r="E3" s="55" t="s">
         <v>215</v>
       </c>
       <c r="F3" s="14"/>
@@ -5931,7 +5934,7 @@
         <v>247</v>
       </c>
     </row>
-    <row r="17" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="17" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B17" s="43" t="b">
         <v>0</v>
       </c>
@@ -5951,7 +5954,7 @@
         <v>250</v>
       </c>
     </row>
-    <row r="18" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="18" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B18" s="43" t="b">
         <v>0</v>
       </c>
@@ -5971,7 +5974,7 @@
         <v>248</v>
       </c>
     </row>
-    <row r="20" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="20" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B20" s="43" t="b">
         <v>0</v>
       </c>
@@ -5981,16 +5984,14 @@
       <c r="D20" s="44" t="s">
         <v>296</v>
       </c>
-      <c r="E20" s="93" t="s">
+      <c r="E20" s="52" t="s">
         <v>289</v>
       </c>
       <c r="F20" s="2" t="s">
         <v>297</v>
       </c>
-      <c r="G20" s="92"/>
-      <c r="H20" s="92"/>
-    </row>
-    <row r="21" spans="2:8" x14ac:dyDescent="0.25">
+    </row>
+    <row r="21" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B21" s="43" t="b">
         <v>0</v>
       </c>
@@ -6007,7 +6008,7 @@
         <v>299</v>
       </c>
     </row>
-    <row r="22" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="22" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B22" s="43" t="b">
         <v>0</v>
       </c>
@@ -6022,6 +6023,23 @@
       </c>
       <c r="F22" s="2" t="s">
         <v>301</v>
+      </c>
+    </row>
+    <row r="24" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B24" s="43" t="b">
+        <v>0</v>
+      </c>
+      <c r="C24" s="46" t="s">
+        <v>184</v>
+      </c>
+      <c r="D24" s="2" t="s">
+        <v>316</v>
+      </c>
+      <c r="E24" s="2" t="s">
+        <v>317</v>
+      </c>
+      <c r="F24" s="2" t="s">
+        <v>134</v>
       </c>
     </row>
   </sheetData>
@@ -6051,21 +6069,21 @@
   <sheetData>
     <row r="1" spans="2:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="2" spans="2:12" ht="23.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B2" s="80" t="s">
+      <c r="B2" s="92" t="s">
         <v>188</v>
       </c>
-      <c r="C2" s="81"/>
-      <c r="D2" s="82"/>
-      <c r="F2" s="80" t="s">
+      <c r="C2" s="93"/>
+      <c r="D2" s="94"/>
+      <c r="F2" s="92" t="s">
         <v>189</v>
       </c>
-      <c r="G2" s="81"/>
-      <c r="H2" s="82"/>
-      <c r="J2" s="80" t="s">
+      <c r="G2" s="93"/>
+      <c r="H2" s="94"/>
+      <c r="J2" s="92" t="s">
         <v>190</v>
       </c>
-      <c r="K2" s="81"/>
-      <c r="L2" s="82"/>
+      <c r="K2" s="93"/>
+      <c r="L2" s="94"/>
     </row>
     <row r="3" spans="2:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B3" s="29" t="s">
@@ -6250,26 +6268,26 @@
     </row>
     <row r="10" spans="2:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="11" spans="2:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B11" s="83" t="s">
+      <c r="B11" s="95" t="s">
         <v>182</v>
       </c>
-      <c r="C11" s="84"/>
+      <c r="C11" s="96"/>
       <c r="D11" s="28">
         <f>(D4*C4+D5*C5+D6*C6+D7*C7+D8*C8+D9*C9)/30</f>
         <v>4.4333333333333336</v>
       </c>
-      <c r="F11" s="83" t="s">
+      <c r="F11" s="95" t="s">
         <v>182</v>
       </c>
-      <c r="G11" s="84"/>
+      <c r="G11" s="96"/>
       <c r="H11" s="28">
         <f>(H4*G4+H5*G5+H6*G6+H7*G7+H8*G8)/30</f>
         <v>4.75</v>
       </c>
-      <c r="J11" s="83" t="s">
+      <c r="J11" s="95" t="s">
         <v>182</v>
       </c>
-      <c r="K11" s="84"/>
+      <c r="K11" s="96"/>
       <c r="L11" s="28">
         <f>(L4*K4+L5*K5+L6*K6+L7*K7+L8*K8)/30</f>
         <v>0</v>

</xml_diff>